<commit_message>
Actualizar formatos: bitacoras, visitas y agregar nuevos formatos (carta intención, acta certificación)
</commit_message>
<xml_diff>
--- a/Formatos/BITACORAS GFPI-F-147V4.xlsx
+++ b/Formatos/BITACORAS GFPI-F-147V4.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SEANT\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SEANT\OneDrive\Documents\Seto 2026\sena\Manual SENA Etapa Productiva\manual-aprendiz-sena\Formatos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{324AC6E9-AFFB-4C03-A5D0-79D396FF8B1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9F1B76D-61E2-469A-AE3E-0093C7EEB615}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instrucciones" sheetId="5" r:id="rId1"/>
@@ -2610,300 +2610,6 @@
     <xf numFmtId="0" fontId="14" fillId="2" borderId="82" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="6" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="6" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="6" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="6" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="75" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="53" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="73" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="59" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="69" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="65" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="66" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="67" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="35" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center"/>
       <protection locked="0"/>
@@ -2944,37 +2650,251 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="74" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="2" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="2" borderId="53" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="76" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="55" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="6" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="6" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="6" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="6" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="85" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="70" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="74" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="85" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="70" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -2984,65 +2904,34 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="74" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="75" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="39" fillId="2" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="2" borderId="53" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="76" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="55" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment wrapText="1"/>
-      <protection locked="0"/>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="53" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="75" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="65" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="66" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="67" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -3052,38 +2941,30 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="59" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="57" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="59" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="55" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="86" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -3092,9 +2973,24 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -3104,21 +3000,125 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="73" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="59" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="69" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -4020,56 +4020,56 @@
       <c r="H2" s="7"/>
     </row>
     <row r="3" spans="2:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="137" t="s">
+      <c r="B3" s="188" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="138"/>
-      <c r="D3" s="138"/>
-      <c r="E3" s="139"/>
+      <c r="C3" s="189"/>
+      <c r="D3" s="189"/>
+      <c r="E3" s="190"/>
       <c r="F3" s="7"/>
       <c r="G3" s="7"/>
       <c r="H3" s="7"/>
     </row>
     <row r="4" spans="2:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="140" t="s">
+      <c r="B4" s="191" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="141"/>
-      <c r="D4" s="141"/>
-      <c r="E4" s="142"/>
+      <c r="C4" s="192"/>
+      <c r="D4" s="192"/>
+      <c r="E4" s="193"/>
       <c r="F4" s="7"/>
       <c r="G4" s="7"/>
       <c r="H4" s="7"/>
     </row>
     <row r="5" spans="2:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="143" t="s">
+      <c r="B5" s="194" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="144"/>
-      <c r="D5" s="144"/>
-      <c r="E5" s="145"/>
+      <c r="C5" s="195"/>
+      <c r="D5" s="195"/>
+      <c r="E5" s="196"/>
       <c r="F5" s="7"/>
       <c r="G5" s="7"/>
       <c r="H5" s="7"/>
     </row>
     <row r="6" spans="2:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="140" t="s">
+      <c r="B6" s="191" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="141"/>
-      <c r="D6" s="141"/>
-      <c r="E6" s="142"/>
+      <c r="C6" s="192"/>
+      <c r="D6" s="192"/>
+      <c r="E6" s="193"/>
       <c r="F6" s="7"/>
       <c r="G6" s="7"/>
       <c r="H6" s="7"/>
     </row>
     <row r="7" spans="2:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="137" t="s">
+      <c r="B7" s="188" t="s">
         <v>6</v>
       </c>
-      <c r="C7" s="138"/>
-      <c r="D7" s="138"/>
-      <c r="E7" s="139"/>
+      <c r="C7" s="189"/>
+      <c r="D7" s="189"/>
+      <c r="E7" s="190"/>
       <c r="F7" s="7"/>
       <c r="G7" s="7"/>
       <c r="H7" s="7"/>
@@ -4081,45 +4081,45 @@
       <c r="C8" s="54" t="s">
         <v>8</v>
       </c>
-      <c r="D8" s="146" t="s">
+      <c r="D8" s="197" t="s">
         <v>9</v>
       </c>
-      <c r="E8" s="147"/>
+      <c r="E8" s="198"/>
       <c r="H8" s="7"/>
     </row>
     <row r="9" spans="2:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="148" t="s">
+      <c r="B9" s="199" t="s">
         <v>10</v>
       </c>
-      <c r="C9" s="149"/>
-      <c r="D9" s="149"/>
-      <c r="E9" s="150"/>
+      <c r="C9" s="200"/>
+      <c r="D9" s="200"/>
+      <c r="E9" s="201"/>
       <c r="G9" s="7"/>
       <c r="H9" s="7"/>
     </row>
     <row r="10" spans="2:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="151" t="s">
+      <c r="B10" s="202" t="s">
         <v>11</v>
       </c>
-      <c r="C10" s="152"/>
-      <c r="D10" s="152"/>
-      <c r="E10" s="153"/>
+      <c r="C10" s="203"/>
+      <c r="D10" s="203"/>
+      <c r="E10" s="204"/>
     </row>
     <row r="11" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B11" s="154" t="s">
+      <c r="B11" s="180" t="s">
         <v>12</v>
       </c>
-      <c r="C11" s="155"/>
-      <c r="D11" s="155"/>
-      <c r="E11" s="156"/>
+      <c r="C11" s="181"/>
+      <c r="D11" s="181"/>
+      <c r="E11" s="182"/>
     </row>
     <row r="12" spans="2:8" ht="51" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="133" t="s">
+      <c r="B12" s="171" t="s">
         <v>13</v>
       </c>
-      <c r="C12" s="134"/>
-      <c r="D12" s="135"/>
-      <c r="E12" s="136"/>
+      <c r="C12" s="172"/>
+      <c r="D12" s="173"/>
+      <c r="E12" s="174"/>
       <c r="F12" s="1"/>
       <c r="G12" s="34"/>
     </row>
@@ -4130,28 +4130,28 @@
       <c r="E13" s="75"/>
     </row>
     <row r="14" spans="2:8" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="166" t="s">
+      <c r="B14" s="162" t="s">
         <v>14</v>
       </c>
-      <c r="C14" s="167"/>
-      <c r="D14" s="167"/>
-      <c r="E14" s="168"/>
+      <c r="C14" s="163"/>
+      <c r="D14" s="163"/>
+      <c r="E14" s="164"/>
     </row>
     <row r="15" spans="2:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="169" t="s">
+      <c r="B15" s="165" t="s">
         <v>15</v>
       </c>
-      <c r="C15" s="170"/>
-      <c r="D15" s="170"/>
-      <c r="E15" s="171"/>
+      <c r="C15" s="166"/>
+      <c r="D15" s="166"/>
+      <c r="E15" s="167"/>
     </row>
     <row r="16" spans="2:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="169" t="s">
+      <c r="B16" s="165" t="s">
         <v>16</v>
       </c>
-      <c r="C16" s="170"/>
-      <c r="D16" s="170"/>
-      <c r="E16" s="171"/>
+      <c r="C16" s="166"/>
+      <c r="D16" s="166"/>
+      <c r="E16" s="167"/>
     </row>
     <row r="17" spans="2:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="175" t="s">
@@ -4162,52 +4162,52 @@
       <c r="E17" s="177"/>
     </row>
     <row r="18" spans="2:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="169" t="s">
+      <c r="B18" s="165" t="s">
         <v>18</v>
       </c>
-      <c r="C18" s="170"/>
-      <c r="D18" s="170"/>
-      <c r="E18" s="171"/>
+      <c r="C18" s="166"/>
+      <c r="D18" s="166"/>
+      <c r="E18" s="167"/>
     </row>
     <row r="19" spans="2:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="169" t="s">
+      <c r="B19" s="165" t="s">
         <v>19</v>
       </c>
-      <c r="C19" s="170"/>
-      <c r="D19" s="170"/>
-      <c r="E19" s="171"/>
+      <c r="C19" s="166"/>
+      <c r="D19" s="166"/>
+      <c r="E19" s="167"/>
     </row>
     <row r="20" spans="2:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="172" t="s">
+      <c r="B20" s="168" t="s">
         <v>20</v>
       </c>
-      <c r="C20" s="173"/>
-      <c r="D20" s="173"/>
-      <c r="E20" s="174"/>
+      <c r="C20" s="169"/>
+      <c r="D20" s="169"/>
+      <c r="E20" s="170"/>
     </row>
     <row r="21" spans="2:6" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="133" t="s">
+      <c r="B21" s="171" t="s">
         <v>21</v>
       </c>
-      <c r="C21" s="134"/>
-      <c r="D21" s="135"/>
-      <c r="E21" s="136"/>
+      <c r="C21" s="172"/>
+      <c r="D21" s="173"/>
+      <c r="E21" s="174"/>
     </row>
     <row r="22" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="154" t="s">
+      <c r="B22" s="180" t="s">
         <v>22</v>
       </c>
-      <c r="C22" s="155"/>
-      <c r="D22" s="155" t="s">
+      <c r="C22" s="181"/>
+      <c r="D22" s="181" t="s">
         <v>22</v>
       </c>
-      <c r="E22" s="156"/>
+      <c r="E22" s="182"/>
     </row>
     <row r="23" spans="2:6" ht="5.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="157"/>
-      <c r="C23" s="158"/>
-      <c r="D23" s="158"/>
-      <c r="E23" s="159"/>
+      <c r="B23" s="183"/>
+      <c r="C23" s="184"/>
+      <c r="D23" s="184"/>
+      <c r="E23" s="185"/>
     </row>
     <row r="24" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B24" s="68" t="s">
@@ -4216,10 +4216,10 @@
       <c r="C24" s="55" t="s">
         <v>24</v>
       </c>
-      <c r="D24" s="160" t="s">
+      <c r="D24" s="186" t="s">
         <v>25</v>
       </c>
-      <c r="E24" s="161"/>
+      <c r="E24" s="187"/>
       <c r="F24" s="8"/>
     </row>
     <row r="25" spans="2:6" x14ac:dyDescent="0.25">
@@ -4229,8 +4229,8 @@
       <c r="C25" s="56" t="s">
         <v>27</v>
       </c>
-      <c r="D25" s="162"/>
-      <c r="E25" s="163"/>
+      <c r="D25" s="178"/>
+      <c r="E25" s="179"/>
     </row>
     <row r="26" spans="2:6" ht="31.5" x14ac:dyDescent="0.25">
       <c r="B26" s="57" t="s">
@@ -4239,8 +4239,8 @@
       <c r="C26" s="58" t="s">
         <v>29</v>
       </c>
-      <c r="D26" s="162"/>
-      <c r="E26" s="163"/>
+      <c r="D26" s="178"/>
+      <c r="E26" s="179"/>
     </row>
     <row r="27" spans="2:6" ht="45" x14ac:dyDescent="0.25">
       <c r="B27" s="59" t="s">
@@ -4249,8 +4249,8 @@
       <c r="C27" s="56" t="s">
         <v>31</v>
       </c>
-      <c r="D27" s="162"/>
-      <c r="E27" s="163"/>
+      <c r="D27" s="178"/>
+      <c r="E27" s="179"/>
     </row>
     <row r="28" spans="2:6" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B28" s="69" t="s">
@@ -4259,8 +4259,8 @@
       <c r="C28" s="56" t="s">
         <v>33</v>
       </c>
-      <c r="D28" s="162"/>
-      <c r="E28" s="163"/>
+      <c r="D28" s="178"/>
+      <c r="E28" s="179"/>
     </row>
     <row r="29" spans="2:6" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B29" s="69" t="s">
@@ -4269,10 +4269,10 @@
       <c r="C29" s="56" t="s">
         <v>35</v>
       </c>
-      <c r="D29" s="162" t="s">
+      <c r="D29" s="178" t="s">
         <v>36</v>
       </c>
-      <c r="E29" s="163" t="s">
+      <c r="E29" s="179" t="s">
         <v>36</v>
       </c>
     </row>
@@ -4283,10 +4283,10 @@
       <c r="C30" s="56" t="s">
         <v>38</v>
       </c>
-      <c r="D30" s="162" t="s">
+      <c r="D30" s="178" t="s">
         <v>39</v>
       </c>
-      <c r="E30" s="163" t="s">
+      <c r="E30" s="179" t="s">
         <v>39</v>
       </c>
     </row>
@@ -4297,8 +4297,8 @@
       <c r="C31" s="56" t="s">
         <v>41</v>
       </c>
-      <c r="D31" s="162"/>
-      <c r="E31" s="163"/>
+      <c r="D31" s="178"/>
+      <c r="E31" s="179"/>
     </row>
     <row r="32" spans="2:6" ht="65.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B32" s="69" t="s">
@@ -4307,10 +4307,10 @@
       <c r="C32" s="56" t="s">
         <v>43</v>
       </c>
-      <c r="D32" s="162" t="s">
+      <c r="D32" s="178" t="s">
         <v>44</v>
       </c>
-      <c r="E32" s="163" t="s">
+      <c r="E32" s="179" t="s">
         <v>44</v>
       </c>
     </row>
@@ -4321,8 +4321,8 @@
       <c r="C33" s="56" t="s">
         <v>46</v>
       </c>
-      <c r="D33" s="162"/>
-      <c r="E33" s="163"/>
+      <c r="D33" s="178"/>
+      <c r="E33" s="179"/>
     </row>
     <row r="34" spans="2:5" ht="60" x14ac:dyDescent="0.25">
       <c r="B34" s="69" t="s">
@@ -4331,8 +4331,8 @@
       <c r="C34" s="56" t="s">
         <v>48</v>
       </c>
-      <c r="D34" s="162"/>
-      <c r="E34" s="163"/>
+      <c r="D34" s="178"/>
+      <c r="E34" s="179"/>
     </row>
     <row r="35" spans="2:5" ht="60" x14ac:dyDescent="0.25">
       <c r="B35" s="69" t="s">
@@ -4341,8 +4341,8 @@
       <c r="C35" s="56" t="s">
         <v>50</v>
       </c>
-      <c r="D35" s="162"/>
-      <c r="E35" s="163"/>
+      <c r="D35" s="178"/>
+      <c r="E35" s="179"/>
     </row>
     <row r="36" spans="2:5" ht="45" x14ac:dyDescent="0.25">
       <c r="B36" s="69" t="s">
@@ -4351,8 +4351,8 @@
       <c r="C36" s="56" t="s">
         <v>52</v>
       </c>
-      <c r="D36" s="162"/>
-      <c r="E36" s="163"/>
+      <c r="D36" s="178"/>
+      <c r="E36" s="179"/>
     </row>
     <row r="37" spans="2:5" ht="60" x14ac:dyDescent="0.25">
       <c r="B37" s="69" t="s">
@@ -4361,8 +4361,8 @@
       <c r="C37" s="56" t="s">
         <v>54</v>
       </c>
-      <c r="D37" s="162"/>
-      <c r="E37" s="163"/>
+      <c r="D37" s="178"/>
+      <c r="E37" s="179"/>
     </row>
     <row r="38" spans="2:5" ht="60" x14ac:dyDescent="0.25">
       <c r="B38" s="69" t="s">
@@ -4371,8 +4371,8 @@
       <c r="C38" s="56" t="s">
         <v>56</v>
       </c>
-      <c r="D38" s="162"/>
-      <c r="E38" s="163"/>
+      <c r="D38" s="178"/>
+      <c r="E38" s="179"/>
     </row>
     <row r="39" spans="2:5" ht="60" x14ac:dyDescent="0.25">
       <c r="B39" s="69" t="s">
@@ -4381,8 +4381,8 @@
       <c r="C39" s="56" t="s">
         <v>57</v>
       </c>
-      <c r="D39" s="162"/>
-      <c r="E39" s="163"/>
+      <c r="D39" s="178"/>
+      <c r="E39" s="179"/>
     </row>
     <row r="40" spans="2:5" ht="60" x14ac:dyDescent="0.25">
       <c r="B40" s="69" t="s">
@@ -4391,8 +4391,8 @@
       <c r="C40" s="56" t="s">
         <v>59</v>
       </c>
-      <c r="D40" s="162"/>
-      <c r="E40" s="163"/>
+      <c r="D40" s="178"/>
+      <c r="E40" s="179"/>
     </row>
     <row r="41" spans="2:5" ht="60" x14ac:dyDescent="0.25">
       <c r="B41" s="69" t="s">
@@ -4401,8 +4401,8 @@
       <c r="C41" s="56" t="s">
         <v>61</v>
       </c>
-      <c r="D41" s="162"/>
-      <c r="E41" s="163"/>
+      <c r="D41" s="178"/>
+      <c r="E41" s="179"/>
     </row>
     <row r="42" spans="2:5" ht="60" x14ac:dyDescent="0.25">
       <c r="B42" s="69" t="s">
@@ -4411,8 +4411,8 @@
       <c r="C42" s="56" t="s">
         <v>62</v>
       </c>
-      <c r="D42" s="162"/>
-      <c r="E42" s="163"/>
+      <c r="D42" s="178"/>
+      <c r="E42" s="179"/>
     </row>
     <row r="43" spans="2:5" ht="409.5" x14ac:dyDescent="0.25">
       <c r="B43" s="69" t="s">
@@ -4421,10 +4421,10 @@
       <c r="C43" s="60" t="s">
         <v>64</v>
       </c>
-      <c r="D43" s="162" t="s">
+      <c r="D43" s="178" t="s">
         <v>65</v>
       </c>
-      <c r="E43" s="163" t="s">
+      <c r="E43" s="179" t="s">
         <v>65</v>
       </c>
     </row>
@@ -4435,8 +4435,8 @@
       <c r="C44" s="56" t="s">
         <v>67</v>
       </c>
-      <c r="D44" s="162"/>
-      <c r="E44" s="163"/>
+      <c r="D44" s="178"/>
+      <c r="E44" s="179"/>
     </row>
     <row r="45" spans="2:5" ht="30" x14ac:dyDescent="0.25">
       <c r="B45" s="69" t="s">
@@ -4445,8 +4445,8 @@
       <c r="C45" s="56" t="s">
         <v>69</v>
       </c>
-      <c r="D45" s="162"/>
-      <c r="E45" s="163"/>
+      <c r="D45" s="178"/>
+      <c r="E45" s="179"/>
     </row>
     <row r="46" spans="2:5" ht="30" x14ac:dyDescent="0.25">
       <c r="B46" s="69" t="s">
@@ -4455,8 +4455,8 @@
       <c r="C46" s="56" t="s">
         <v>71</v>
       </c>
-      <c r="D46" s="162"/>
-      <c r="E46" s="163"/>
+      <c r="D46" s="178"/>
+      <c r="E46" s="179"/>
     </row>
     <row r="47" spans="2:5" ht="127.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B47" s="69" t="s">
@@ -4465,10 +4465,10 @@
       <c r="C47" s="56" t="s">
         <v>73</v>
       </c>
-      <c r="D47" s="162" t="s">
+      <c r="D47" s="178" t="s">
         <v>74</v>
       </c>
-      <c r="E47" s="163" t="s">
+      <c r="E47" s="179" t="s">
         <v>74</v>
       </c>
     </row>
@@ -4479,8 +4479,8 @@
       <c r="C48" s="56" t="s">
         <v>76</v>
       </c>
-      <c r="D48" s="162"/>
-      <c r="E48" s="163"/>
+      <c r="D48" s="178"/>
+      <c r="E48" s="179"/>
     </row>
     <row r="49" spans="2:5" ht="146.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B49" s="69" t="s">
@@ -4489,10 +4489,10 @@
       <c r="C49" s="56" t="s">
         <v>78</v>
       </c>
-      <c r="D49" s="162" t="s">
+      <c r="D49" s="178" t="s">
         <v>79</v>
       </c>
-      <c r="E49" s="163" t="s">
+      <c r="E49" s="179" t="s">
         <v>79</v>
       </c>
     </row>
@@ -4503,10 +4503,10 @@
       <c r="C50" s="61" t="s">
         <v>81</v>
       </c>
-      <c r="D50" s="162" t="s">
+      <c r="D50" s="178" t="s">
         <v>82</v>
       </c>
-      <c r="E50" s="163" t="s">
+      <c r="E50" s="179" t="s">
         <v>83</v>
       </c>
     </row>
@@ -4517,10 +4517,10 @@
       <c r="C51" s="61" t="s">
         <v>85</v>
       </c>
-      <c r="D51" s="162" t="s">
+      <c r="D51" s="178" t="s">
         <v>86</v>
       </c>
-      <c r="E51" s="163" t="s">
+      <c r="E51" s="179" t="s">
         <v>86</v>
       </c>
     </row>
@@ -4531,8 +4531,8 @@
       <c r="C52" s="56" t="s">
         <v>88</v>
       </c>
-      <c r="D52" s="162"/>
-      <c r="E52" s="163"/>
+      <c r="D52" s="178"/>
+      <c r="E52" s="179"/>
     </row>
     <row r="53" spans="2:5" ht="75" x14ac:dyDescent="0.25">
       <c r="B53" s="69" t="s">
@@ -4541,8 +4541,8 @@
       <c r="C53" s="61" t="s">
         <v>90</v>
       </c>
-      <c r="D53" s="162"/>
-      <c r="E53" s="163"/>
+      <c r="D53" s="178"/>
+      <c r="E53" s="179"/>
     </row>
     <row r="54" spans="2:5" ht="45" x14ac:dyDescent="0.25">
       <c r="B54" s="69" t="s">
@@ -4551,8 +4551,8 @@
       <c r="C54" s="61" t="s">
         <v>92</v>
       </c>
-      <c r="D54" s="162"/>
-      <c r="E54" s="163"/>
+      <c r="D54" s="178"/>
+      <c r="E54" s="179"/>
     </row>
     <row r="55" spans="2:5" ht="75" x14ac:dyDescent="0.25">
       <c r="B55" s="69" t="s">
@@ -4561,8 +4561,8 @@
       <c r="C55" s="56" t="s">
         <v>94</v>
       </c>
-      <c r="D55" s="162"/>
-      <c r="E55" s="163"/>
+      <c r="D55" s="178"/>
+      <c r="E55" s="179"/>
     </row>
     <row r="56" spans="2:5" ht="75" x14ac:dyDescent="0.25">
       <c r="B56" s="70" t="s">
@@ -4571,8 +4571,8 @@
       <c r="C56" s="56" t="s">
         <v>94</v>
       </c>
-      <c r="D56" s="162"/>
-      <c r="E56" s="163"/>
+      <c r="D56" s="178"/>
+      <c r="E56" s="179"/>
     </row>
     <row r="57" spans="2:5" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B57" s="71" t="s">
@@ -4581,10 +4581,10 @@
       <c r="C57" s="72" t="s">
         <v>97</v>
       </c>
-      <c r="D57" s="164" t="s">
+      <c r="D57" s="160" t="s">
         <v>98</v>
       </c>
-      <c r="E57" s="165" t="s">
+      <c r="E57" s="161" t="s">
         <v>98</v>
       </c>
     </row>
@@ -4602,6 +4602,44 @@
     </row>
   </sheetData>
   <mergeCells count="54">
+    <mergeCell ref="B12:E12"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="B4:E4"/>
+    <mergeCell ref="B5:E5"/>
+    <mergeCell ref="B6:E6"/>
+    <mergeCell ref="B7:E7"/>
+    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="B9:E9"/>
+    <mergeCell ref="B10:E10"/>
+    <mergeCell ref="B11:E11"/>
+    <mergeCell ref="B22:E22"/>
+    <mergeCell ref="B23:E23"/>
+    <mergeCell ref="D24:E24"/>
+    <mergeCell ref="D25:E25"/>
+    <mergeCell ref="D26:E26"/>
+    <mergeCell ref="D27:E27"/>
+    <mergeCell ref="D28:E28"/>
+    <mergeCell ref="D29:E29"/>
+    <mergeCell ref="D30:E30"/>
+    <mergeCell ref="D31:E31"/>
+    <mergeCell ref="D32:E32"/>
+    <mergeCell ref="D33:E33"/>
+    <mergeCell ref="D34:E34"/>
+    <mergeCell ref="D35:E35"/>
+    <mergeCell ref="D36:E36"/>
+    <mergeCell ref="D37:E37"/>
+    <mergeCell ref="D38:E38"/>
+    <mergeCell ref="D39:E39"/>
+    <mergeCell ref="D40:E40"/>
+    <mergeCell ref="D41:E41"/>
+    <mergeCell ref="D49:E49"/>
+    <mergeCell ref="D50:E50"/>
+    <mergeCell ref="D51:E51"/>
+    <mergeCell ref="D42:E42"/>
+    <mergeCell ref="D43:E43"/>
+    <mergeCell ref="D44:E44"/>
+    <mergeCell ref="D45:E45"/>
+    <mergeCell ref="D46:E46"/>
     <mergeCell ref="D57:E57"/>
     <mergeCell ref="B14:E14"/>
     <mergeCell ref="B19:E19"/>
@@ -4618,44 +4656,6 @@
     <mergeCell ref="D56:E56"/>
     <mergeCell ref="D47:E47"/>
     <mergeCell ref="D48:E48"/>
-    <mergeCell ref="D49:E49"/>
-    <mergeCell ref="D50:E50"/>
-    <mergeCell ref="D51:E51"/>
-    <mergeCell ref="D42:E42"/>
-    <mergeCell ref="D43:E43"/>
-    <mergeCell ref="D44:E44"/>
-    <mergeCell ref="D45:E45"/>
-    <mergeCell ref="D46:E46"/>
-    <mergeCell ref="D37:E37"/>
-    <mergeCell ref="D38:E38"/>
-    <mergeCell ref="D39:E39"/>
-    <mergeCell ref="D40:E40"/>
-    <mergeCell ref="D41:E41"/>
-    <mergeCell ref="D32:E32"/>
-    <mergeCell ref="D33:E33"/>
-    <mergeCell ref="D34:E34"/>
-    <mergeCell ref="D35:E35"/>
-    <mergeCell ref="D36:E36"/>
-    <mergeCell ref="D27:E27"/>
-    <mergeCell ref="D28:E28"/>
-    <mergeCell ref="D29:E29"/>
-    <mergeCell ref="D30:E30"/>
-    <mergeCell ref="D31:E31"/>
-    <mergeCell ref="B22:E22"/>
-    <mergeCell ref="B23:E23"/>
-    <mergeCell ref="D24:E24"/>
-    <mergeCell ref="D25:E25"/>
-    <mergeCell ref="D26:E26"/>
-    <mergeCell ref="B12:E12"/>
-    <mergeCell ref="B3:E3"/>
-    <mergeCell ref="B4:E4"/>
-    <mergeCell ref="B5:E5"/>
-    <mergeCell ref="B6:E6"/>
-    <mergeCell ref="B7:E7"/>
-    <mergeCell ref="D8:E8"/>
-    <mergeCell ref="B9:E9"/>
-    <mergeCell ref="B10:E10"/>
-    <mergeCell ref="B11:E11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -4670,23 +4670,23 @@
   <cols>
     <col min="1" max="1" width="2.28515625" style="9" customWidth="1"/>
     <col min="2" max="7" width="32.7109375" style="11" customWidth="1"/>
-    <col min="8" max="8" width="8.42578125" style="11" customWidth="1"/>
-    <col min="9" max="9" width="6.42578125" style="11" hidden="1" customWidth="1"/>
-    <col min="10" max="15" width="5.7109375" style="11" hidden="1" customWidth="1"/>
-    <col min="16" max="16" width="4.7109375" style="11" hidden="1" customWidth="1"/>
-    <col min="17" max="17" width="5.85546875" style="11" hidden="1" customWidth="1"/>
-    <col min="18" max="18" width="7.42578125" style="11" hidden="1" customWidth="1"/>
-    <col min="19" max="19" width="7.140625" style="11" hidden="1" customWidth="1"/>
-    <col min="20" max="21" width="5.7109375" style="11" hidden="1" customWidth="1"/>
-    <col min="22" max="22" width="5" style="11" hidden="1" customWidth="1"/>
-    <col min="23" max="23" width="6.42578125" style="11" hidden="1" customWidth="1"/>
-    <col min="24" max="24" width="8.140625" style="11" hidden="1" customWidth="1"/>
-    <col min="25" max="25" width="5.140625" style="11" hidden="1" customWidth="1"/>
-    <col min="26" max="26" width="24.42578125" style="10" hidden="1" customWidth="1"/>
+    <col min="8" max="8" width="6.42578125" style="11" hidden="1" customWidth="1"/>
+    <col min="9" max="14" width="5.7109375" style="11" hidden="1" customWidth="1"/>
+    <col min="15" max="15" width="4.7109375" style="11" hidden="1" customWidth="1"/>
+    <col min="16" max="16" width="5.85546875" style="11" hidden="1" customWidth="1"/>
+    <col min="17" max="17" width="7.42578125" style="11" hidden="1" customWidth="1"/>
+    <col min="18" max="18" width="7.140625" style="11" hidden="1" customWidth="1"/>
+    <col min="19" max="20" width="5.7109375" style="11" hidden="1" customWidth="1"/>
+    <col min="21" max="21" width="5" style="11" hidden="1" customWidth="1"/>
+    <col min="22" max="22" width="6.42578125" style="11" hidden="1" customWidth="1"/>
+    <col min="23" max="23" width="8.140625" style="11" hidden="1" customWidth="1"/>
+    <col min="24" max="24" width="5.140625" style="11" hidden="1" customWidth="1"/>
+    <col min="25" max="25" width="24.42578125" style="10" hidden="1" customWidth="1"/>
+    <col min="26" max="26" width="24.42578125" style="9" hidden="1"/>
     <col min="27" max="16384" width="11.42578125" style="9" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:26" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:25" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B1" s="107"/>
       <c r="C1" s="127"/>
       <c r="D1" s="127"/>
@@ -4695,7 +4695,7 @@
       <c r="G1" s="128" t="s">
         <v>0</v>
       </c>
-      <c r="H1" s="10"/>
+      <c r="H1" s="9"/>
       <c r="I1" s="9"/>
       <c r="J1" s="9"/>
       <c r="K1" s="9"/>
@@ -4713,9 +4713,8 @@
       <c r="W1" s="9"/>
       <c r="X1" s="9"/>
       <c r="Y1" s="9"/>
-      <c r="Z1" s="9"/>
-    </row>
-    <row r="2" spans="2:26" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="2:25" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="129"/>
       <c r="C2" s="18"/>
       <c r="D2" s="18"/>
@@ -4724,7 +4723,7 @@
       <c r="G2" s="130" t="s">
         <v>1</v>
       </c>
-      <c r="H2" s="10"/>
+      <c r="H2" s="9"/>
       <c r="I2" s="9"/>
       <c r="J2" s="9"/>
       <c r="K2" s="9"/>
@@ -4742,18 +4741,17 @@
       <c r="W2" s="9"/>
       <c r="X2" s="9"/>
       <c r="Y2" s="9"/>
-      <c r="Z2" s="9"/>
-    </row>
-    <row r="3" spans="2:26" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="137" t="s">
+    </row>
+    <row r="3" spans="2:25" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B3" s="188" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="138"/>
-      <c r="D3" s="138"/>
-      <c r="E3" s="138"/>
-      <c r="F3" s="138"/>
-      <c r="G3" s="139"/>
-      <c r="H3" s="10"/>
+      <c r="C3" s="189"/>
+      <c r="D3" s="189"/>
+      <c r="E3" s="189"/>
+      <c r="F3" s="189"/>
+      <c r="G3" s="190"/>
+      <c r="H3" s="9"/>
       <c r="I3" s="9"/>
       <c r="J3" s="9"/>
       <c r="K3" s="9"/>
@@ -4771,18 +4769,17 @@
       <c r="W3" s="9"/>
       <c r="X3" s="9"/>
       <c r="Y3" s="9"/>
-      <c r="Z3" s="9"/>
-    </row>
-    <row r="4" spans="2:26" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="140" t="s">
+    </row>
+    <row r="4" spans="2:25" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="191" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="141"/>
-      <c r="D4" s="141"/>
-      <c r="E4" s="141"/>
-      <c r="F4" s="141"/>
-      <c r="G4" s="142"/>
-      <c r="H4" s="10"/>
+      <c r="C4" s="192"/>
+      <c r="D4" s="192"/>
+      <c r="E4" s="192"/>
+      <c r="F4" s="192"/>
+      <c r="G4" s="193"/>
+      <c r="H4" s="9"/>
       <c r="I4" s="9"/>
       <c r="J4" s="9"/>
       <c r="K4" s="9"/>
@@ -4800,19 +4797,18 @@
       <c r="W4" s="9"/>
       <c r="X4" s="9"/>
       <c r="Y4" s="9"/>
-      <c r="Z4" s="9"/>
-    </row>
-    <row r="5" spans="2:26" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="137" t="s">
+    </row>
+    <row r="5" spans="2:25" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="188" t="s">
         <v>99</v>
       </c>
-      <c r="C5" s="138"/>
-      <c r="D5" s="138"/>
-      <c r="E5" s="138"/>
-      <c r="F5" s="138"/>
-      <c r="G5" s="139"/>
+      <c r="C5" s="189"/>
+      <c r="D5" s="189"/>
+      <c r="E5" s="189"/>
+      <c r="F5" s="189"/>
+      <c r="G5" s="190"/>
       <c r="H5" s="10"/>
-      <c r="I5" s="10"/>
+      <c r="I5" s="9"/>
       <c r="J5" s="9"/>
       <c r="K5" s="9"/>
       <c r="L5" s="9"/>
@@ -4829,19 +4825,18 @@
       <c r="W5" s="9"/>
       <c r="X5" s="9"/>
       <c r="Y5" s="9"/>
-      <c r="Z5" s="9"/>
-    </row>
-    <row r="6" spans="2:26" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="140" t="s">
+    </row>
+    <row r="6" spans="2:25" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B6" s="191" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="141"/>
-      <c r="D6" s="141"/>
-      <c r="E6" s="141"/>
-      <c r="F6" s="141"/>
-      <c r="G6" s="142"/>
+      <c r="C6" s="192"/>
+      <c r="D6" s="192"/>
+      <c r="E6" s="192"/>
+      <c r="F6" s="192"/>
+      <c r="G6" s="193"/>
       <c r="H6" s="10"/>
-      <c r="I6" s="10"/>
+      <c r="I6" s="9"/>
       <c r="J6" s="9"/>
       <c r="K6" s="9"/>
       <c r="L6" s="9"/>
@@ -4858,17 +4853,16 @@
       <c r="W6" s="9"/>
       <c r="X6" s="9"/>
       <c r="Y6" s="9"/>
-      <c r="Z6" s="9"/>
-    </row>
-    <row r="7" spans="2:26" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="137" t="s">
+    </row>
+    <row r="7" spans="2:25" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B7" s="188" t="s">
         <v>6</v>
       </c>
-      <c r="C7" s="138"/>
-      <c r="D7" s="138"/>
-      <c r="E7" s="138"/>
-      <c r="F7" s="138"/>
-      <c r="G7" s="139"/>
+      <c r="C7" s="189"/>
+      <c r="D7" s="189"/>
+      <c r="E7" s="189"/>
+      <c r="F7" s="189"/>
+      <c r="G7" s="190"/>
       <c r="H7" s="9"/>
       <c r="I7" s="9"/>
       <c r="J7" s="9"/>
@@ -4887,21 +4881,20 @@
       <c r="W7" s="9"/>
       <c r="X7" s="9"/>
       <c r="Y7" s="9"/>
-      <c r="Z7" s="9"/>
-    </row>
-    <row r="8" spans="2:26" ht="36.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="231" t="s">
+    </row>
+    <row r="8" spans="2:25" ht="36.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B8" s="133" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="232"/>
-      <c r="D8" s="233" t="s">
+      <c r="C8" s="134"/>
+      <c r="D8" s="135" t="s">
         <v>8</v>
       </c>
-      <c r="E8" s="232"/>
-      <c r="F8" s="233" t="s">
+      <c r="E8" s="134"/>
+      <c r="F8" s="135" t="s">
         <v>9</v>
       </c>
-      <c r="G8" s="234"/>
+      <c r="G8" s="136"/>
       <c r="H8" s="9"/>
       <c r="I8" s="9"/>
       <c r="J8" s="9"/>
@@ -4920,9 +4913,8 @@
       <c r="W8" s="9"/>
       <c r="X8" s="9"/>
       <c r="Y8" s="9"/>
-      <c r="Z8" s="9"/>
-    </row>
-    <row r="9" spans="2:26" ht="9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="9" spans="2:25" ht="9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B9" s="18"/>
       <c r="C9" s="20"/>
       <c r="D9" s="20"/>
@@ -4947,9 +4939,8 @@
       <c r="W9" s="9"/>
       <c r="X9" s="9"/>
       <c r="Y9" s="9"/>
-      <c r="Z9" s="9"/>
-    </row>
-    <row r="10" spans="2:26" s="11" customFormat="1" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="10" spans="2:25" s="11" customFormat="1" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="107" t="s">
         <v>100</v>
       </c>
@@ -4969,13 +4960,13 @@
         <v>37</v>
       </c>
     </row>
-    <row r="11" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="235"/>
-      <c r="C11" s="236"/>
-      <c r="D11" s="237"/>
-      <c r="E11" s="238"/>
-      <c r="F11" s="239"/>
-      <c r="G11" s="240"/>
+    <row r="11" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B11" s="137"/>
+      <c r="C11" s="138"/>
+      <c r="D11" s="139"/>
+      <c r="E11" s="140"/>
+      <c r="F11" s="141"/>
+      <c r="G11" s="142"/>
       <c r="H11" s="9"/>
       <c r="I11" s="9"/>
       <c r="J11" s="9"/>
@@ -4994,9 +4985,8 @@
       <c r="W11" s="9"/>
       <c r="X11" s="9"/>
       <c r="Y11" s="9"/>
-      <c r="Z11" s="9"/>
-    </row>
-    <row r="12" spans="2:26" ht="9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="12" spans="2:25" ht="9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B12" s="20"/>
       <c r="D12" s="20"/>
       <c r="E12" s="18"/>
@@ -5020,9 +5010,8 @@
       <c r="W12" s="9"/>
       <c r="X12" s="9"/>
       <c r="Y12" s="9"/>
-      <c r="Z12" s="9"/>
-    </row>
-    <row r="13" spans="2:26" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="13" spans="2:25" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="114" t="s">
         <v>102</v>
       </c>
@@ -5035,7 +5024,7 @@
       <c r="G13" s="106"/>
       <c r="H13" s="18"/>
       <c r="I13" s="18"/>
-      <c r="J13" s="18"/>
+      <c r="K13" s="18"/>
       <c r="L13" s="18"/>
       <c r="M13" s="18"/>
       <c r="N13" s="18"/>
@@ -5049,18 +5038,17 @@
       <c r="V13" s="18"/>
       <c r="W13" s="18"/>
       <c r="X13" s="18"/>
-      <c r="Y13" s="18"/>
-    </row>
-    <row r="14" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="241"/>
-      <c r="C14" s="242"/>
-      <c r="D14" s="243"/>
-      <c r="E14" s="244"/>
-      <c r="F14" s="245"/>
-      <c r="G14" s="246"/>
+    </row>
+    <row r="14" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B14" s="208"/>
+      <c r="C14" s="210"/>
+      <c r="D14" s="209"/>
+      <c r="E14" s="205"/>
+      <c r="F14" s="206"/>
+      <c r="G14" s="207"/>
       <c r="H14" s="20"/>
       <c r="I14" s="20"/>
-      <c r="J14" s="20"/>
+      <c r="K14" s="20"/>
       <c r="L14" s="20"/>
       <c r="M14" s="20"/>
       <c r="N14" s="20"/>
@@ -5074,9 +5062,8 @@
       <c r="V14" s="20"/>
       <c r="W14" s="20"/>
       <c r="X14" s="20"/>
-      <c r="Y14" s="20"/>
-    </row>
-    <row r="15" spans="2:26" ht="9.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="15" spans="2:25" ht="9.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B15" s="15"/>
       <c r="C15" s="15"/>
       <c r="D15" s="15"/>
@@ -5100,9 +5087,8 @@
       <c r="V15" s="15"/>
       <c r="W15" s="15"/>
       <c r="X15" s="15"/>
-      <c r="Y15" s="15"/>
-    </row>
-    <row r="16" spans="2:26" s="11" customFormat="1" ht="50.25" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="16" spans="2:25" s="11" customFormat="1" ht="50.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="107" t="s">
         <v>103</v>
       </c>
@@ -5118,34 +5104,32 @@
       </c>
       <c r="G16" s="113"/>
       <c r="H16" s="20"/>
-      <c r="I16" s="20"/>
+      <c r="J16" s="18"/>
       <c r="K16" s="18"/>
-      <c r="L16" s="18"/>
+      <c r="T16" s="18"/>
       <c r="U16" s="18"/>
       <c r="V16" s="18"/>
       <c r="W16" s="18"/>
       <c r="X16" s="18"/>
-      <c r="Y16" s="18"/>
-      <c r="Z16" s="12"/>
-    </row>
-    <row r="17" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="241"/>
-      <c r="C17" s="243"/>
-      <c r="D17" s="247"/>
-      <c r="E17" s="248"/>
-      <c r="F17" s="249"/>
-      <c r="G17" s="250"/>
+      <c r="Y16" s="12"/>
+    </row>
+    <row r="17" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B17" s="208"/>
+      <c r="C17" s="209"/>
+      <c r="D17" s="144"/>
+      <c r="E17" s="145"/>
+      <c r="F17" s="217"/>
+      <c r="G17" s="218"/>
       <c r="H17" s="20"/>
-      <c r="I17" s="20"/>
+      <c r="J17" s="20"/>
       <c r="K17" s="20"/>
-      <c r="L17" s="20"/>
+      <c r="T17" s="20"/>
       <c r="U17" s="20"/>
       <c r="V17" s="20"/>
       <c r="W17" s="20"/>
       <c r="X17" s="20"/>
-      <c r="Y17" s="20"/>
-    </row>
-    <row r="18" spans="2:26" ht="9.9499999999999993" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="18" spans="2:25" ht="9.9499999999999993" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B18" s="15"/>
       <c r="C18" s="15"/>
       <c r="D18" s="15"/>
@@ -5169,9 +5153,8 @@
       <c r="V18" s="15"/>
       <c r="W18" s="15"/>
       <c r="X18" s="15"/>
-      <c r="Y18" s="15"/>
-    </row>
-    <row r="19" spans="2:26" s="11" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+    </row>
+    <row r="19" spans="2:25" s="11" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="B19" s="107" t="s">
         <v>53</v>
       </c>
@@ -5186,43 +5169,41 @@
         <v>58</v>
       </c>
       <c r="G19" s="106"/>
-      <c r="H19" s="18"/>
+      <c r="K19" s="18"/>
       <c r="L19" s="18"/>
-      <c r="M19" s="18"/>
+      <c r="N19" s="18"/>
       <c r="O19" s="18"/>
       <c r="P19" s="18"/>
       <c r="Q19" s="18"/>
-      <c r="R19" s="18"/>
+      <c r="S19" s="18"/>
       <c r="T19" s="18"/>
       <c r="U19" s="18"/>
       <c r="V19" s="18"/>
       <c r="W19" s="18"/>
       <c r="X19" s="18"/>
-      <c r="Y19" s="18"/>
-      <c r="Z19" s="12"/>
-    </row>
-    <row r="20" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="241"/>
-      <c r="C20" s="243"/>
-      <c r="D20" s="251"/>
-      <c r="E20" s="252"/>
-      <c r="F20" s="253"/>
-      <c r="G20" s="254"/>
-      <c r="H20" s="20"/>
+      <c r="Y19" s="12"/>
+    </row>
+    <row r="20" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B20" s="208"/>
+      <c r="C20" s="209"/>
+      <c r="D20" s="143"/>
+      <c r="E20" s="146"/>
+      <c r="F20" s="219"/>
+      <c r="G20" s="220"/>
+      <c r="K20" s="20"/>
       <c r="L20" s="20"/>
-      <c r="M20" s="20"/>
+      <c r="N20" s="20"/>
       <c r="O20" s="20"/>
       <c r="P20" s="20"/>
       <c r="Q20" s="20"/>
-      <c r="R20" s="20"/>
+      <c r="S20" s="20"/>
       <c r="T20" s="20"/>
       <c r="U20" s="20"/>
       <c r="V20" s="20"/>
       <c r="W20" s="20"/>
       <c r="X20" s="20"/>
-      <c r="Y20" s="20"/>
-    </row>
-    <row r="21" spans="2:26" ht="8.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="21" spans="2:25" ht="8.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B21" s="15"/>
       <c r="C21" s="15"/>
       <c r="D21" s="15"/>
@@ -5246,17 +5227,16 @@
       <c r="V21" s="15"/>
       <c r="W21" s="15"/>
       <c r="X21" s="15"/>
-      <c r="Y21" s="15"/>
-    </row>
-    <row r="22" spans="2:26" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="189" t="s">
+    </row>
+    <row r="22" spans="2:25" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B22" s="225" t="s">
         <v>105</v>
       </c>
-      <c r="C22" s="190"/>
-      <c r="D22" s="190"/>
-      <c r="E22" s="190"/>
-      <c r="F22" s="190"/>
-      <c r="G22" s="191"/>
+      <c r="C22" s="226"/>
+      <c r="D22" s="226"/>
+      <c r="E22" s="226"/>
+      <c r="F22" s="226"/>
+      <c r="G22" s="227"/>
       <c r="H22" s="9"/>
       <c r="I22" s="9"/>
       <c r="J22" s="9"/>
@@ -5275,23 +5255,22 @@
       <c r="W22" s="9"/>
       <c r="X22" s="9"/>
       <c r="Y22" s="9"/>
-      <c r="Z22" s="9"/>
-    </row>
-    <row r="23" spans="2:26" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="23" spans="2:25" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B23" s="131" t="s">
         <v>106</v>
       </c>
-      <c r="C23" s="181" t="s">
+      <c r="C23" s="221" t="s">
         <v>189</v>
       </c>
-      <c r="D23" s="182"/>
+      <c r="D23" s="222"/>
       <c r="E23" s="132" t="s">
         <v>107</v>
       </c>
-      <c r="F23" s="180" t="s">
+      <c r="F23" s="223" t="s">
         <v>188</v>
       </c>
-      <c r="G23" s="178"/>
+      <c r="G23" s="224"/>
       <c r="H23" s="9"/>
       <c r="I23" s="9"/>
       <c r="J23" s="9"/>
@@ -5310,9 +5289,8 @@
       <c r="W23" s="9"/>
       <c r="X23" s="9"/>
       <c r="Y23" s="9"/>
-      <c r="Z23" s="9"/>
-    </row>
-    <row r="24" spans="2:26" ht="9.9499999999999993" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="24" spans="2:25" ht="9.9499999999999993" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B24" s="15"/>
       <c r="C24" s="15"/>
       <c r="D24" s="15"/>
@@ -5336,9 +5314,8 @@
       <c r="V24" s="15"/>
       <c r="W24" s="15"/>
       <c r="X24" s="15"/>
-      <c r="Y24" s="15"/>
-    </row>
-    <row r="25" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="25" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B25" s="36"/>
       <c r="C25" s="25" t="s">
         <v>108</v>
@@ -5349,7 +5326,7 @@
       <c r="G25" s="26"/>
       <c r="H25" s="22"/>
       <c r="I25" s="22"/>
-      <c r="J25" s="22"/>
+      <c r="J25" s="23"/>
       <c r="K25" s="23"/>
       <c r="L25" s="23"/>
       <c r="M25" s="23"/>
@@ -5364,9 +5341,8 @@
       <c r="V25" s="23"/>
       <c r="W25" s="23"/>
       <c r="X25" s="23"/>
-      <c r="Y25" s="23"/>
-    </row>
-    <row r="26" spans="2:26" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="26" spans="2:25" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B26" s="121" t="s">
         <v>109</v>
       </c>
@@ -5383,7 +5359,7 @@
       <c r="G26" s="122"/>
       <c r="H26" s="22"/>
       <c r="I26" s="22"/>
-      <c r="J26" s="22"/>
+      <c r="J26" s="23"/>
       <c r="K26" s="23"/>
       <c r="L26" s="23"/>
       <c r="M26" s="23"/>
@@ -5398,338 +5374,326 @@
       <c r="V26" s="23"/>
       <c r="W26" s="23"/>
       <c r="X26" s="23"/>
-      <c r="Y26" s="23"/>
-    </row>
-    <row r="27" spans="2:26" s="13" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.35">
+    </row>
+    <row r="27" spans="2:25" s="13" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B27" s="39"/>
       <c r="C27" s="76" t="s">
         <v>111</v>
       </c>
-      <c r="D27" s="255"/>
+      <c r="D27" s="147"/>
       <c r="E27" s="45"/>
       <c r="F27" s="76" t="s">
         <v>112</v>
       </c>
-      <c r="G27" s="262"/>
+      <c r="G27" s="154"/>
       <c r="H27" s="18"/>
-      <c r="I27" s="18"/>
+      <c r="I27" s="20"/>
       <c r="J27" s="20"/>
       <c r="K27" s="20"/>
       <c r="L27" s="20"/>
       <c r="M27" s="20"/>
       <c r="N27" s="20"/>
       <c r="O27" s="20"/>
-      <c r="P27" s="20"/>
+      <c r="P27" s="18"/>
       <c r="Q27" s="18"/>
-      <c r="R27" s="18"/>
+      <c r="R27" s="20"/>
       <c r="S27" s="20"/>
       <c r="T27" s="20"/>
       <c r="U27" s="20"/>
-      <c r="V27" s="20"/>
-      <c r="Z27" s="14"/>
-    </row>
-    <row r="28" spans="2:26" s="13" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="Y27" s="14"/>
+    </row>
+    <row r="28" spans="2:25" s="13" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B28" s="40"/>
       <c r="C28" s="21" t="s">
         <v>113</v>
       </c>
-      <c r="D28" s="256"/>
+      <c r="D28" s="148"/>
       <c r="E28" s="46"/>
-      <c r="F28" s="192" t="s">
+      <c r="F28" s="211" t="s">
         <v>114</v>
       </c>
-      <c r="G28" s="263"/>
+      <c r="G28" s="212"/>
       <c r="H28" s="18"/>
-      <c r="I28" s="18"/>
+      <c r="I28" s="20"/>
       <c r="J28" s="20"/>
       <c r="K28" s="20"/>
       <c r="L28" s="20"/>
       <c r="M28" s="20"/>
       <c r="N28" s="20"/>
       <c r="O28" s="20"/>
-      <c r="P28" s="20"/>
+      <c r="P28" s="18"/>
       <c r="Q28" s="18"/>
-      <c r="R28" s="18"/>
+      <c r="R28" s="20"/>
       <c r="S28" s="20"/>
       <c r="T28" s="20"/>
       <c r="U28" s="20"/>
-      <c r="V28" s="20"/>
-      <c r="Z28" s="14"/>
-    </row>
-    <row r="29" spans="2:26" s="13" customFormat="1" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="Y28" s="14"/>
+    </row>
+    <row r="29" spans="2:25" s="13" customFormat="1" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B29" s="41"/>
       <c r="C29" s="21" t="s">
         <v>115</v>
       </c>
-      <c r="D29" s="256"/>
+      <c r="D29" s="148"/>
       <c r="E29" s="41" t="s">
         <v>116</v>
       </c>
-      <c r="F29" s="192"/>
-      <c r="G29" s="263"/>
+      <c r="F29" s="211"/>
+      <c r="G29" s="212"/>
       <c r="H29" s="18"/>
-      <c r="I29" s="18"/>
+      <c r="I29" s="20"/>
       <c r="J29" s="20"/>
       <c r="K29" s="20"/>
       <c r="L29" s="20"/>
       <c r="M29" s="20"/>
       <c r="N29" s="20"/>
       <c r="O29" s="20"/>
-      <c r="P29" s="20"/>
+      <c r="P29" s="18"/>
       <c r="Q29" s="18"/>
-      <c r="R29" s="18"/>
+      <c r="R29" s="20"/>
       <c r="S29" s="20"/>
       <c r="T29" s="20"/>
       <c r="U29" s="20"/>
-      <c r="V29" s="20"/>
-      <c r="Z29" s="14"/>
-    </row>
-    <row r="30" spans="2:26" s="13" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="Y29" s="14"/>
+    </row>
+    <row r="30" spans="2:25" s="13" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B30" s="126" t="s">
         <v>117</v>
       </c>
       <c r="C30" s="38" t="s">
         <v>118</v>
       </c>
-      <c r="D30" s="256"/>
+      <c r="D30" s="148"/>
       <c r="E30" s="47" t="s">
         <v>119</v>
       </c>
       <c r="F30" s="21" t="s">
         <v>120</v>
       </c>
-      <c r="G30" s="256"/>
+      <c r="G30" s="148"/>
       <c r="H30" s="18"/>
-      <c r="I30" s="18"/>
+      <c r="I30" s="20"/>
       <c r="J30" s="20"/>
       <c r="K30" s="20"/>
       <c r="L30" s="20"/>
       <c r="M30" s="20"/>
       <c r="N30" s="20"/>
       <c r="O30" s="20"/>
-      <c r="P30" s="20"/>
+      <c r="P30" s="18"/>
       <c r="Q30" s="18"/>
-      <c r="R30" s="18"/>
+      <c r="R30" s="20"/>
       <c r="S30" s="20"/>
       <c r="T30" s="20"/>
       <c r="U30" s="20"/>
-      <c r="V30" s="20"/>
-      <c r="Z30" s="14"/>
-    </row>
-    <row r="31" spans="2:26" s="13" customFormat="1" ht="45" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="Y30" s="14"/>
+    </row>
+    <row r="31" spans="2:25" s="13" customFormat="1" ht="45" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B31" s="42"/>
       <c r="C31" s="21" t="s">
         <v>121</v>
       </c>
-      <c r="D31" s="257"/>
+      <c r="D31" s="149"/>
       <c r="E31" s="40"/>
       <c r="F31" s="83" t="s">
         <v>122</v>
       </c>
-      <c r="G31" s="261"/>
+      <c r="G31" s="153"/>
       <c r="H31" s="18"/>
-      <c r="I31" s="18"/>
-      <c r="J31" s="19"/>
+      <c r="I31" s="19"/>
+      <c r="J31" s="16"/>
       <c r="K31" s="16"/>
       <c r="L31" s="16"/>
       <c r="M31" s="16"/>
       <c r="N31" s="16"/>
-      <c r="O31" s="16"/>
-      <c r="P31" s="20"/>
+      <c r="O31" s="20"/>
+      <c r="P31" s="19"/>
       <c r="Q31" s="19"/>
-      <c r="R31" s="19"/>
+      <c r="R31" s="16"/>
       <c r="S31" s="16"/>
       <c r="T31" s="16"/>
-      <c r="U31" s="16"/>
-      <c r="V31" s="20"/>
+      <c r="U31" s="20"/>
+      <c r="V31" s="19"/>
       <c r="W31" s="19"/>
-      <c r="X31" s="19"/>
-      <c r="Y31" s="15"/>
-      <c r="Z31" s="14"/>
-    </row>
-    <row r="32" spans="2:26" s="13" customFormat="1" ht="44.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="X31" s="15"/>
+      <c r="Y31" s="14"/>
+    </row>
+    <row r="32" spans="2:25" s="13" customFormat="1" ht="44.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B32" s="42"/>
       <c r="C32" s="21" t="s">
         <v>123</v>
       </c>
-      <c r="D32" s="258"/>
+      <c r="D32" s="150"/>
       <c r="E32" s="44"/>
       <c r="F32" s="82" t="s">
         <v>124</v>
       </c>
-      <c r="G32" s="255"/>
+      <c r="G32" s="147"/>
       <c r="H32" s="18"/>
-      <c r="I32" s="18"/>
-      <c r="J32" s="19"/>
+      <c r="I32" s="19"/>
+      <c r="J32" s="16"/>
       <c r="K32" s="16"/>
       <c r="L32" s="16"/>
       <c r="M32" s="16"/>
       <c r="N32" s="16"/>
-      <c r="O32" s="16"/>
-      <c r="P32" s="20"/>
+      <c r="O32" s="20"/>
+      <c r="P32" s="19"/>
       <c r="Q32" s="19"/>
-      <c r="R32" s="19"/>
+      <c r="R32" s="16"/>
       <c r="S32" s="16"/>
       <c r="T32" s="16"/>
-      <c r="U32" s="16"/>
-      <c r="V32" s="20"/>
+      <c r="U32" s="20"/>
+      <c r="V32" s="19"/>
       <c r="W32" s="19"/>
-      <c r="X32" s="19"/>
-      <c r="Y32" s="15"/>
-      <c r="Z32" s="14"/>
-    </row>
-    <row r="33" spans="2:26" s="13" customFormat="1" ht="35.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="X32" s="15"/>
+      <c r="Y32" s="14"/>
+    </row>
+    <row r="33" spans="2:25" s="13" customFormat="1" ht="35.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B33" s="43"/>
       <c r="C33" s="81" t="s">
         <v>125</v>
       </c>
-      <c r="D33" s="259"/>
+      <c r="D33" s="151"/>
       <c r="E33" s="79" t="s">
         <v>126</v>
       </c>
       <c r="F33" s="37" t="s">
         <v>127</v>
       </c>
-      <c r="G33" s="264"/>
+      <c r="G33" s="155"/>
       <c r="H33" s="18"/>
-      <c r="I33" s="18"/>
-      <c r="J33" s="19"/>
+      <c r="I33" s="19"/>
+      <c r="J33" s="16"/>
       <c r="K33" s="16"/>
       <c r="L33" s="16"/>
       <c r="M33" s="16"/>
       <c r="N33" s="16"/>
-      <c r="O33" s="16"/>
-      <c r="P33" s="20"/>
+      <c r="O33" s="20"/>
+      <c r="P33" s="19"/>
       <c r="Q33" s="19"/>
-      <c r="R33" s="19"/>
+      <c r="R33" s="16"/>
       <c r="S33" s="16"/>
       <c r="T33" s="16"/>
-      <c r="U33" s="16"/>
-      <c r="V33" s="20"/>
+      <c r="U33" s="20"/>
+      <c r="V33" s="19"/>
       <c r="W33" s="19"/>
-      <c r="X33" s="19"/>
-      <c r="Y33" s="15"/>
-      <c r="Z33" s="14"/>
-    </row>
-    <row r="34" spans="2:26" s="13" customFormat="1" ht="45.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="X33" s="15"/>
+      <c r="Y33" s="14"/>
+    </row>
+    <row r="34" spans="2:25" s="13" customFormat="1" ht="45.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B34" s="44"/>
       <c r="C34" s="82" t="s">
         <v>128</v>
       </c>
-      <c r="D34" s="260"/>
+      <c r="D34" s="152"/>
       <c r="E34" s="48"/>
       <c r="F34" s="78" t="s">
         <v>129</v>
       </c>
-      <c r="G34" s="261"/>
+      <c r="G34" s="153"/>
       <c r="H34" s="18"/>
-      <c r="I34" s="18"/>
-      <c r="J34" s="19"/>
+      <c r="I34" s="19"/>
+      <c r="J34" s="16"/>
       <c r="K34" s="16"/>
       <c r="L34" s="16"/>
       <c r="M34" s="16"/>
       <c r="N34" s="16"/>
-      <c r="O34" s="16"/>
-      <c r="P34" s="20"/>
+      <c r="O34" s="20"/>
+      <c r="P34" s="19"/>
       <c r="Q34" s="19"/>
-      <c r="R34" s="19"/>
+      <c r="R34" s="16"/>
       <c r="S34" s="16"/>
       <c r="T34" s="16"/>
-      <c r="U34" s="16"/>
-      <c r="V34" s="20"/>
+      <c r="U34" s="20"/>
+      <c r="V34" s="19"/>
       <c r="W34" s="19"/>
-      <c r="X34" s="19"/>
-      <c r="Y34" s="15"/>
-      <c r="Z34" s="14"/>
-    </row>
-    <row r="35" spans="2:26" s="13" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="X34" s="15"/>
+      <c r="Y34" s="14"/>
+    </row>
+    <row r="35" spans="2:25" s="13" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B35" s="41" t="s">
         <v>130</v>
       </c>
       <c r="C35" s="37" t="s">
         <v>131</v>
       </c>
-      <c r="D35" s="256"/>
+      <c r="D35" s="148"/>
       <c r="E35" s="79" t="s">
         <v>132</v>
       </c>
       <c r="F35" s="80" t="s">
         <v>133</v>
       </c>
-      <c r="G35" s="265"/>
+      <c r="G35" s="156"/>
       <c r="H35" s="18"/>
-      <c r="I35" s="18"/>
-      <c r="J35" s="19"/>
+      <c r="I35" s="19"/>
+      <c r="J35" s="16"/>
       <c r="K35" s="16"/>
       <c r="L35" s="16"/>
       <c r="M35" s="16"/>
       <c r="N35" s="16"/>
-      <c r="O35" s="16"/>
-      <c r="P35" s="20"/>
+      <c r="O35" s="20"/>
+      <c r="P35" s="19"/>
       <c r="Q35" s="19"/>
-      <c r="R35" s="19"/>
+      <c r="R35" s="16"/>
       <c r="S35" s="16"/>
       <c r="T35" s="16"/>
-      <c r="U35" s="16"/>
-      <c r="V35" s="20"/>
+      <c r="U35" s="20"/>
+      <c r="V35" s="19"/>
       <c r="W35" s="19"/>
-      <c r="X35" s="19"/>
-      <c r="Y35" s="15"/>
-      <c r="Z35" s="14"/>
-    </row>
-    <row r="36" spans="2:26" s="13" customFormat="1" ht="46.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="X35" s="15"/>
+      <c r="Y35" s="14"/>
+    </row>
+    <row r="36" spans="2:25" s="13" customFormat="1" ht="46.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B36" s="43"/>
       <c r="C36" s="77" t="s">
         <v>134</v>
       </c>
-      <c r="D36" s="261"/>
+      <c r="D36" s="153"/>
       <c r="E36" s="125"/>
       <c r="F36" s="78" t="s">
         <v>135</v>
       </c>
-      <c r="G36" s="261"/>
+      <c r="G36" s="153"/>
       <c r="H36" s="18"/>
-      <c r="I36" s="18"/>
-      <c r="J36" s="19"/>
+      <c r="I36" s="19"/>
+      <c r="J36" s="16"/>
       <c r="K36" s="16"/>
       <c r="L36" s="16"/>
       <c r="M36" s="16"/>
       <c r="N36" s="16"/>
-      <c r="O36" s="16"/>
-      <c r="P36" s="20"/>
+      <c r="O36" s="20"/>
+      <c r="P36" s="19"/>
       <c r="Q36" s="19"/>
-      <c r="R36" s="19"/>
+      <c r="R36" s="16"/>
       <c r="S36" s="16"/>
       <c r="T36" s="16"/>
-      <c r="U36" s="16"/>
-      <c r="V36" s="20"/>
+      <c r="U36" s="20"/>
+      <c r="V36" s="19"/>
       <c r="W36" s="19"/>
-      <c r="X36" s="19"/>
-      <c r="Y36" s="15"/>
-      <c r="Z36" s="14"/>
-    </row>
-    <row r="37" spans="2:26" s="13" customFormat="1" ht="9.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="X36" s="15"/>
+      <c r="Y36" s="14"/>
+    </row>
+    <row r="37" spans="2:25" s="13" customFormat="1" ht="9.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="H37" s="18"/>
-      <c r="I37" s="18"/>
-      <c r="J37" s="19"/>
+      <c r="I37" s="19"/>
+      <c r="J37" s="16"/>
       <c r="K37" s="16"/>
       <c r="L37" s="16"/>
       <c r="M37" s="16"/>
       <c r="N37" s="16"/>
-      <c r="O37" s="16"/>
-      <c r="P37" s="20"/>
+      <c r="O37" s="20"/>
+      <c r="P37" s="19"/>
       <c r="Q37" s="19"/>
-      <c r="R37" s="19"/>
+      <c r="R37" s="16"/>
       <c r="S37" s="16"/>
       <c r="T37" s="16"/>
-      <c r="U37" s="16"/>
-      <c r="V37" s="20"/>
+      <c r="U37" s="20"/>
+      <c r="V37" s="19"/>
       <c r="W37" s="19"/>
-      <c r="X37" s="19"/>
-      <c r="Y37" s="15"/>
-      <c r="Z37" s="14"/>
-    </row>
-    <row r="38" spans="2:26" ht="68.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="X37" s="15"/>
+      <c r="Y37" s="14"/>
+    </row>
+    <row r="38" spans="2:25" ht="68.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B38" s="84" t="s">
         <v>136</v>
       </c>
@@ -5765,9 +5729,8 @@
       <c r="V38" s="18"/>
       <c r="W38" s="18"/>
       <c r="X38" s="18"/>
-      <c r="Y38" s="18"/>
-    </row>
-    <row r="39" spans="2:26" ht="52.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="39" spans="2:25" ht="52.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B39" s="91" t="s">
         <v>142</v>
       </c>
@@ -5799,16 +5762,15 @@
       <c r="V39" s="18"/>
       <c r="W39" s="18"/>
       <c r="X39" s="18"/>
-      <c r="Y39" s="18"/>
-    </row>
-    <row r="40" spans="2:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B40" s="266"/>
-      <c r="C40" s="267"/>
-      <c r="D40" s="268"/>
-      <c r="E40" s="268"/>
-      <c r="F40" s="268"/>
-      <c r="G40" s="269"/>
-      <c r="H40" s="20"/>
+    </row>
+    <row r="40" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B40" s="228"/>
+      <c r="C40" s="229"/>
+      <c r="D40" s="232"/>
+      <c r="E40" s="232"/>
+      <c r="F40" s="232"/>
+      <c r="G40" s="234"/>
+      <c r="H40" s="18"/>
       <c r="I40" s="18"/>
       <c r="J40" s="18"/>
       <c r="K40" s="18"/>
@@ -5825,16 +5787,15 @@
       <c r="V40" s="18"/>
       <c r="W40" s="18"/>
       <c r="X40" s="18"/>
-      <c r="Y40" s="18"/>
-    </row>
-    <row r="41" spans="2:26" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B41" s="270"/>
-      <c r="C41" s="271"/>
-      <c r="D41" s="272"/>
-      <c r="E41" s="272"/>
-      <c r="F41" s="272"/>
-      <c r="G41" s="273"/>
-      <c r="H41" s="20"/>
+    </row>
+    <row r="41" spans="2:25" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B41" s="230"/>
+      <c r="C41" s="231"/>
+      <c r="D41" s="233"/>
+      <c r="E41" s="233"/>
+      <c r="F41" s="233"/>
+      <c r="G41" s="235"/>
+      <c r="H41" s="18"/>
       <c r="I41" s="18"/>
       <c r="J41" s="18"/>
       <c r="K41" s="18"/>
@@ -5851,16 +5812,15 @@
       <c r="V41" s="18"/>
       <c r="W41" s="18"/>
       <c r="X41" s="18"/>
-      <c r="Y41" s="18"/>
-    </row>
-    <row r="42" spans="2:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B42" s="266"/>
-      <c r="C42" s="267"/>
-      <c r="D42" s="268"/>
-      <c r="E42" s="268"/>
-      <c r="F42" s="268"/>
-      <c r="G42" s="269"/>
-      <c r="H42" s="20"/>
+    </row>
+    <row r="42" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B42" s="228"/>
+      <c r="C42" s="229"/>
+      <c r="D42" s="232"/>
+      <c r="E42" s="232"/>
+      <c r="F42" s="232"/>
+      <c r="G42" s="234"/>
+      <c r="H42" s="18"/>
       <c r="I42" s="18"/>
       <c r="J42" s="18"/>
       <c r="K42" s="18"/>
@@ -5877,16 +5837,15 @@
       <c r="V42" s="18"/>
       <c r="W42" s="18"/>
       <c r="X42" s="18"/>
-      <c r="Y42" s="18"/>
-    </row>
-    <row r="43" spans="2:26" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B43" s="270"/>
-      <c r="C43" s="271"/>
-      <c r="D43" s="272"/>
-      <c r="E43" s="272"/>
-      <c r="F43" s="272"/>
-      <c r="G43" s="273"/>
-      <c r="H43" s="20"/>
+    </row>
+    <row r="43" spans="2:25" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B43" s="230"/>
+      <c r="C43" s="231"/>
+      <c r="D43" s="233"/>
+      <c r="E43" s="233"/>
+      <c r="F43" s="233"/>
+      <c r="G43" s="235"/>
+      <c r="H43" s="18"/>
       <c r="I43" s="18"/>
       <c r="J43" s="18"/>
       <c r="K43" s="18"/>
@@ -5903,16 +5862,15 @@
       <c r="V43" s="18"/>
       <c r="W43" s="18"/>
       <c r="X43" s="18"/>
-      <c r="Y43" s="18"/>
-    </row>
-    <row r="44" spans="2:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B44" s="266"/>
-      <c r="C44" s="267"/>
-      <c r="D44" s="268"/>
-      <c r="E44" s="268"/>
-      <c r="F44" s="268"/>
-      <c r="G44" s="269"/>
-      <c r="H44" s="20"/>
+    </row>
+    <row r="44" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B44" s="228"/>
+      <c r="C44" s="229"/>
+      <c r="D44" s="232"/>
+      <c r="E44" s="232"/>
+      <c r="F44" s="232"/>
+      <c r="G44" s="234"/>
+      <c r="H44" s="18"/>
       <c r="I44" s="18"/>
       <c r="J44" s="18"/>
       <c r="K44" s="18"/>
@@ -5929,16 +5887,15 @@
       <c r="V44" s="18"/>
       <c r="W44" s="18"/>
       <c r="X44" s="18"/>
-      <c r="Y44" s="18"/>
-    </row>
-    <row r="45" spans="2:26" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B45" s="270"/>
-      <c r="C45" s="271"/>
-      <c r="D45" s="272"/>
-      <c r="E45" s="272"/>
-      <c r="F45" s="272"/>
-      <c r="G45" s="273"/>
-      <c r="H45" s="20"/>
+    </row>
+    <row r="45" spans="2:25" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B45" s="230"/>
+      <c r="C45" s="231"/>
+      <c r="D45" s="233"/>
+      <c r="E45" s="233"/>
+      <c r="F45" s="233"/>
+      <c r="G45" s="235"/>
+      <c r="H45" s="18"/>
       <c r="I45" s="18"/>
       <c r="J45" s="18"/>
       <c r="K45" s="18"/>
@@ -5955,16 +5912,15 @@
       <c r="V45" s="18"/>
       <c r="W45" s="18"/>
       <c r="X45" s="18"/>
-      <c r="Y45" s="18"/>
-    </row>
-    <row r="46" spans="2:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B46" s="266"/>
-      <c r="C46" s="267"/>
-      <c r="D46" s="268"/>
-      <c r="E46" s="268"/>
-      <c r="F46" s="268"/>
-      <c r="G46" s="269"/>
-      <c r="H46" s="20"/>
+    </row>
+    <row r="46" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B46" s="228"/>
+      <c r="C46" s="229"/>
+      <c r="D46" s="232"/>
+      <c r="E46" s="232"/>
+      <c r="F46" s="232"/>
+      <c r="G46" s="234"/>
+      <c r="H46" s="18"/>
       <c r="I46" s="18"/>
       <c r="J46" s="18"/>
       <c r="K46" s="18"/>
@@ -5981,16 +5937,15 @@
       <c r="V46" s="18"/>
       <c r="W46" s="18"/>
       <c r="X46" s="18"/>
-      <c r="Y46" s="18"/>
-    </row>
-    <row r="47" spans="2:26" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B47" s="270"/>
-      <c r="C47" s="271"/>
-      <c r="D47" s="272"/>
-      <c r="E47" s="272"/>
-      <c r="F47" s="272"/>
-      <c r="G47" s="273"/>
-      <c r="H47" s="20"/>
+    </row>
+    <row r="47" spans="2:25" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B47" s="230"/>
+      <c r="C47" s="231"/>
+      <c r="D47" s="233"/>
+      <c r="E47" s="233"/>
+      <c r="F47" s="233"/>
+      <c r="G47" s="235"/>
+      <c r="H47" s="18"/>
       <c r="I47" s="18"/>
       <c r="J47" s="18"/>
       <c r="K47" s="18"/>
@@ -6007,16 +5962,15 @@
       <c r="V47" s="18"/>
       <c r="W47" s="18"/>
       <c r="X47" s="18"/>
-      <c r="Y47" s="18"/>
-    </row>
-    <row r="48" spans="2:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B48" s="266"/>
-      <c r="C48" s="267"/>
-      <c r="D48" s="268"/>
-      <c r="E48" s="268"/>
-      <c r="F48" s="268"/>
-      <c r="G48" s="269"/>
-      <c r="H48" s="20"/>
+    </row>
+    <row r="48" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B48" s="228"/>
+      <c r="C48" s="229"/>
+      <c r="D48" s="232"/>
+      <c r="E48" s="232"/>
+      <c r="F48" s="232"/>
+      <c r="G48" s="234"/>
+      <c r="H48" s="18"/>
       <c r="I48" s="18"/>
       <c r="J48" s="18"/>
       <c r="K48" s="18"/>
@@ -6033,16 +5987,15 @@
       <c r="V48" s="18"/>
       <c r="W48" s="18"/>
       <c r="X48" s="18"/>
-      <c r="Y48" s="18"/>
-    </row>
-    <row r="49" spans="2:26" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B49" s="270"/>
-      <c r="C49" s="271"/>
-      <c r="D49" s="272"/>
-      <c r="E49" s="272"/>
-      <c r="F49" s="272"/>
-      <c r="G49" s="273"/>
-      <c r="H49" s="20"/>
+    </row>
+    <row r="49" spans="2:25" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B49" s="230"/>
+      <c r="C49" s="231"/>
+      <c r="D49" s="233"/>
+      <c r="E49" s="233"/>
+      <c r="F49" s="233"/>
+      <c r="G49" s="235"/>
+      <c r="H49" s="18"/>
       <c r="I49" s="18"/>
       <c r="J49" s="18"/>
       <c r="K49" s="18"/>
@@ -6059,16 +6012,15 @@
       <c r="V49" s="18"/>
       <c r="W49" s="18"/>
       <c r="X49" s="18"/>
-      <c r="Y49" s="18"/>
-    </row>
-    <row r="50" spans="2:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B50" s="266"/>
-      <c r="C50" s="267"/>
-      <c r="D50" s="268"/>
-      <c r="E50" s="268"/>
-      <c r="F50" s="268"/>
-      <c r="G50" s="269"/>
-      <c r="H50" s="20"/>
+    </row>
+    <row r="50" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B50" s="228"/>
+      <c r="C50" s="229"/>
+      <c r="D50" s="232"/>
+      <c r="E50" s="232"/>
+      <c r="F50" s="232"/>
+      <c r="G50" s="234"/>
+      <c r="H50" s="18"/>
       <c r="I50" s="18"/>
       <c r="J50" s="18"/>
       <c r="K50" s="18"/>
@@ -6085,16 +6037,15 @@
       <c r="V50" s="18"/>
       <c r="W50" s="18"/>
       <c r="X50" s="18"/>
-      <c r="Y50" s="18"/>
-    </row>
-    <row r="51" spans="2:26" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B51" s="270"/>
-      <c r="C51" s="271"/>
-      <c r="D51" s="272"/>
-      <c r="E51" s="272"/>
-      <c r="F51" s="272"/>
-      <c r="G51" s="273"/>
-      <c r="H51" s="20"/>
+    </row>
+    <row r="51" spans="2:25" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B51" s="230"/>
+      <c r="C51" s="231"/>
+      <c r="D51" s="233"/>
+      <c r="E51" s="233"/>
+      <c r="F51" s="233"/>
+      <c r="G51" s="235"/>
+      <c r="H51" s="18"/>
       <c r="I51" s="18"/>
       <c r="J51" s="18"/>
       <c r="K51" s="18"/>
@@ -6111,16 +6062,15 @@
       <c r="V51" s="18"/>
       <c r="W51" s="18"/>
       <c r="X51" s="18"/>
-      <c r="Y51" s="18"/>
-    </row>
-    <row r="52" spans="2:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B52" s="266"/>
-      <c r="C52" s="267"/>
-      <c r="D52" s="268"/>
-      <c r="E52" s="268"/>
-      <c r="F52" s="268"/>
-      <c r="G52" s="269"/>
-      <c r="H52" s="20"/>
+    </row>
+    <row r="52" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B52" s="228"/>
+      <c r="C52" s="229"/>
+      <c r="D52" s="232"/>
+      <c r="E52" s="232"/>
+      <c r="F52" s="232"/>
+      <c r="G52" s="234"/>
+      <c r="H52" s="18"/>
       <c r="I52" s="18"/>
       <c r="J52" s="18"/>
       <c r="K52" s="18"/>
@@ -6137,16 +6087,15 @@
       <c r="V52" s="18"/>
       <c r="W52" s="18"/>
       <c r="X52" s="18"/>
-      <c r="Y52" s="18"/>
-    </row>
-    <row r="53" spans="2:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B53" s="270"/>
-      <c r="C53" s="271"/>
-      <c r="D53" s="272"/>
-      <c r="E53" s="272"/>
-      <c r="F53" s="272"/>
-      <c r="G53" s="273"/>
-      <c r="H53" s="20"/>
+    </row>
+    <row r="53" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B53" s="230"/>
+      <c r="C53" s="231"/>
+      <c r="D53" s="233"/>
+      <c r="E53" s="233"/>
+      <c r="F53" s="233"/>
+      <c r="G53" s="235"/>
+      <c r="H53" s="18"/>
       <c r="I53" s="18"/>
       <c r="J53" s="18"/>
       <c r="K53" s="18"/>
@@ -6163,16 +6112,15 @@
       <c r="V53" s="18"/>
       <c r="W53" s="18"/>
       <c r="X53" s="18"/>
-      <c r="Y53" s="18"/>
-    </row>
-    <row r="54" spans="2:26" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="54" spans="2:25" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B54" s="27"/>
       <c r="C54" s="20"/>
       <c r="D54" s="20"/>
       <c r="E54" s="20"/>
       <c r="F54" s="20"/>
       <c r="G54" s="20"/>
-      <c r="H54" s="20"/>
+      <c r="H54" s="18"/>
       <c r="I54" s="18"/>
       <c r="J54" s="18"/>
       <c r="K54" s="18"/>
@@ -6189,9 +6137,8 @@
       <c r="V54" s="18"/>
       <c r="W54" s="18"/>
       <c r="X54" s="18"/>
-      <c r="Y54" s="18"/>
-    </row>
-    <row r="55" spans="2:26" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="55" spans="2:25" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B55" s="93"/>
       <c r="C55" s="94" t="s">
         <v>146</v>
@@ -6217,17 +6164,16 @@
       <c r="V55" s="22"/>
       <c r="W55" s="22"/>
       <c r="X55" s="22"/>
-      <c r="Y55" s="22"/>
-    </row>
-    <row r="56" spans="2:26" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B56" s="194" t="s">
+    </row>
+    <row r="56" spans="2:25" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B56" s="214" t="s">
         <v>147</v>
       </c>
-      <c r="C56" s="195"/>
-      <c r="D56" s="195"/>
-      <c r="E56" s="195"/>
-      <c r="F56" s="195"/>
-      <c r="G56" s="196"/>
+      <c r="C56" s="215"/>
+      <c r="D56" s="215"/>
+      <c r="E56" s="215"/>
+      <c r="F56" s="215"/>
+      <c r="G56" s="216"/>
       <c r="H56" s="22"/>
       <c r="I56" s="22"/>
       <c r="J56" s="22"/>
@@ -6245,9 +6191,8 @@
       <c r="V56" s="22"/>
       <c r="W56" s="22"/>
       <c r="X56" s="22"/>
-      <c r="Y56" s="22"/>
-    </row>
-    <row r="57" spans="2:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="57" spans="2:25" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B57" s="97" t="s">
         <v>148</v>
       </c>
@@ -6273,9 +6218,8 @@
       <c r="V57" s="29"/>
       <c r="W57" s="29"/>
       <c r="X57" s="29"/>
-      <c r="Y57" s="29"/>
-    </row>
-    <row r="58" spans="2:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="58" spans="2:25" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B58" s="99" t="s">
         <v>149</v>
       </c>
@@ -6301,9 +6245,8 @@
       <c r="V58" s="29"/>
       <c r="W58" s="29"/>
       <c r="X58" s="29"/>
-      <c r="Y58" s="29"/>
-    </row>
-    <row r="59" spans="2:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="59" spans="2:25" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B59" s="99" t="s">
         <v>150</v>
       </c>
@@ -6329,9 +6272,8 @@
       <c r="V59" s="29"/>
       <c r="W59" s="29"/>
       <c r="X59" s="29"/>
-      <c r="Y59" s="29"/>
-    </row>
-    <row r="60" spans="2:26" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="60" spans="2:25" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B60" s="99" t="s">
         <v>151</v>
       </c>
@@ -6357,9 +6299,8 @@
       <c r="V60" s="29"/>
       <c r="W60" s="29"/>
       <c r="X60" s="29"/>
-      <c r="Y60" s="29"/>
-    </row>
-    <row r="61" spans="2:26" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="61" spans="2:25" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B61" s="102" t="s">
         <v>77</v>
       </c>
@@ -6369,11 +6310,11 @@
       <c r="D61" s="104" t="s">
         <v>84</v>
       </c>
-      <c r="E61" s="276"/>
+      <c r="E61" s="236"/>
       <c r="F61" s="104" t="s">
         <v>152</v>
       </c>
-      <c r="G61" s="276"/>
+      <c r="G61" s="236"/>
       <c r="H61" s="18"/>
       <c r="I61" s="18"/>
       <c r="J61" s="18"/>
@@ -6392,15 +6333,14 @@
       <c r="W61" s="18"/>
       <c r="X61" s="18"/>
       <c r="Y61" s="18"/>
-      <c r="Z61" s="18"/>
-    </row>
-    <row r="62" spans="2:26" ht="32.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B62" s="274"/>
-      <c r="C62" s="275"/>
+    </row>
+    <row r="62" spans="2:25" ht="32.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B62" s="157"/>
+      <c r="C62" s="158"/>
       <c r="D62" s="101"/>
-      <c r="E62" s="277"/>
+      <c r="E62" s="237"/>
       <c r="F62" s="101"/>
-      <c r="G62" s="277"/>
+      <c r="G62" s="237"/>
       <c r="H62" s="18"/>
       <c r="I62" s="18"/>
       <c r="J62" s="18"/>
@@ -6419,9 +6359,8 @@
       <c r="W62" s="18"/>
       <c r="X62" s="18"/>
       <c r="Y62" s="18"/>
-      <c r="Z62" s="18"/>
-    </row>
-    <row r="63" spans="2:26" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="63" spans="2:25" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B63" s="19"/>
       <c r="C63" s="19"/>
       <c r="D63" s="19"/>
@@ -6446,9 +6385,8 @@
       <c r="W63" s="18"/>
       <c r="X63" s="18"/>
       <c r="Y63" s="18"/>
-      <c r="Z63" s="18"/>
-    </row>
-    <row r="64" spans="2:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="64" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C64" s="30"/>
       <c r="D64" s="33" t="s">
         <v>153</v>
@@ -6474,12 +6412,11 @@
       <c r="W64" s="18"/>
       <c r="X64" s="18"/>
       <c r="Y64" s="18"/>
-      <c r="Z64" s="18"/>
-    </row>
-    <row r="65" spans="2:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B65" s="283"/>
-      <c r="C65" s="283"/>
-      <c r="D65" s="283"/>
+    </row>
+    <row r="65" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B65" s="238"/>
+      <c r="C65" s="238"/>
+      <c r="D65" s="238"/>
       <c r="E65" s="17"/>
       <c r="F65" s="17"/>
       <c r="G65" s="17"/>
@@ -6501,12 +6438,11 @@
       <c r="W65" s="18"/>
       <c r="X65" s="18"/>
       <c r="Y65" s="18"/>
-      <c r="Z65" s="18"/>
-    </row>
-    <row r="66" spans="2:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B66" s="283"/>
-      <c r="C66" s="283"/>
-      <c r="D66" s="283"/>
+    </row>
+    <row r="66" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B66" s="238"/>
+      <c r="C66" s="238"/>
+      <c r="D66" s="238"/>
       <c r="E66" s="17"/>
       <c r="F66" s="17"/>
       <c r="G66" s="17"/>
@@ -6528,13 +6464,12 @@
       <c r="W66" s="18"/>
       <c r="X66" s="18"/>
       <c r="Y66" s="18"/>
-      <c r="Z66" s="18"/>
-    </row>
-    <row r="67" spans="2:26" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B67" s="284"/>
-      <c r="C67" s="284"/>
-      <c r="D67" s="284"/>
-      <c r="F67" s="278"/>
+    </row>
+    <row r="67" spans="2:25" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B67" s="239"/>
+      <c r="C67" s="239"/>
+      <c r="D67" s="239"/>
+      <c r="F67" s="159"/>
       <c r="G67" s="18"/>
       <c r="H67" s="18"/>
       <c r="I67" s="18"/>
@@ -6554,14 +6489,13 @@
       <c r="W67" s="18"/>
       <c r="X67" s="18"/>
       <c r="Y67" s="18"/>
-      <c r="Z67" s="18"/>
-    </row>
-    <row r="68" spans="2:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B68" s="193" t="s">
+    </row>
+    <row r="68" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B68" s="213" t="s">
         <v>89</v>
       </c>
-      <c r="C68" s="193"/>
-      <c r="D68" s="193"/>
+      <c r="C68" s="213"/>
+      <c r="D68" s="213"/>
       <c r="F68" s="19" t="s">
         <v>91</v>
       </c>
@@ -6584,14 +6518,13 @@
       <c r="W68" s="18"/>
       <c r="X68" s="18"/>
       <c r="Y68" s="18"/>
-      <c r="Z68" s="18"/>
-    </row>
-    <row r="69" spans="2:26" x14ac:dyDescent="0.25">
-      <c r="B69" s="281"/>
-      <c r="C69" s="281"/>
-      <c r="D69" s="281"/>
-      <c r="F69" s="279"/>
-      <c r="G69" s="279"/>
+    </row>
+    <row r="69" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="B69" s="240"/>
+      <c r="C69" s="240"/>
+      <c r="D69" s="240"/>
+      <c r="F69" s="243"/>
+      <c r="G69" s="243"/>
       <c r="H69" s="18"/>
       <c r="I69" s="18"/>
       <c r="J69" s="18"/>
@@ -6610,14 +6543,13 @@
       <c r="W69" s="18"/>
       <c r="X69" s="18"/>
       <c r="Y69" s="18"/>
-      <c r="Z69" s="18"/>
-    </row>
-    <row r="70" spans="2:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B70" s="281"/>
-      <c r="C70" s="281"/>
-      <c r="D70" s="281"/>
-      <c r="F70" s="279"/>
-      <c r="G70" s="279"/>
+    </row>
+    <row r="70" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B70" s="240"/>
+      <c r="C70" s="240"/>
+      <c r="D70" s="240"/>
+      <c r="F70" s="243"/>
+      <c r="G70" s="243"/>
       <c r="H70" s="18"/>
       <c r="I70" s="18"/>
       <c r="J70" s="18"/>
@@ -6636,14 +6568,13 @@
       <c r="W70" s="18"/>
       <c r="X70" s="18"/>
       <c r="Y70" s="18"/>
-      <c r="Z70" s="18"/>
-    </row>
-    <row r="71" spans="2:26" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B71" s="282"/>
-      <c r="C71" s="282"/>
-      <c r="D71" s="282"/>
-      <c r="F71" s="280"/>
-      <c r="G71" s="280"/>
+    </row>
+    <row r="71" spans="2:25" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B71" s="241"/>
+      <c r="C71" s="241"/>
+      <c r="D71" s="241"/>
+      <c r="F71" s="244"/>
+      <c r="G71" s="244"/>
       <c r="H71" s="18"/>
       <c r="I71" s="18"/>
       <c r="J71" s="18"/>
@@ -6662,18 +6593,17 @@
       <c r="W71" s="18"/>
       <c r="X71" s="18"/>
       <c r="Y71" s="18"/>
-      <c r="Z71" s="18"/>
-    </row>
-    <row r="72" spans="2:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B72" s="179" t="s">
+    </row>
+    <row r="72" spans="2:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B72" s="242" t="s">
         <v>93</v>
       </c>
-      <c r="C72" s="179"/>
-      <c r="D72" s="179"/>
-      <c r="F72" s="193" t="s">
+      <c r="C72" s="242"/>
+      <c r="D72" s="242"/>
+      <c r="F72" s="213" t="s">
         <v>154</v>
       </c>
-      <c r="G72" s="193"/>
+      <c r="G72" s="213"/>
       <c r="H72" s="18"/>
       <c r="I72" s="18"/>
       <c r="J72" s="18"/>
@@ -6692,9 +6622,8 @@
       <c r="W72" s="18"/>
       <c r="X72" s="18"/>
       <c r="Y72" s="18"/>
-      <c r="Z72" s="18"/>
-    </row>
-    <row r="73" spans="2:26" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="73" spans="2:25" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B73" s="31" t="s">
         <v>155</v>
       </c>
@@ -6721,9 +6650,8 @@
       <c r="W73" s="18"/>
       <c r="X73" s="18"/>
       <c r="Y73" s="18"/>
-      <c r="Z73" s="18"/>
-    </row>
-    <row r="74" spans="2:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="74" spans="2:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B74" s="32"/>
       <c r="C74" s="32"/>
       <c r="D74" s="32"/>
@@ -6748,18 +6676,17 @@
       <c r="W74" s="18"/>
       <c r="X74" s="18"/>
       <c r="Y74" s="18"/>
-      <c r="Z74" s="18"/>
-    </row>
-    <row r="75" spans="2:26" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B75" s="183" t="s">
+    </row>
+    <row r="75" spans="2:25" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B75" s="245" t="s">
         <v>156</v>
       </c>
-      <c r="C75" s="184"/>
-      <c r="D75" s="184"/>
-      <c r="E75" s="184"/>
-      <c r="F75" s="184"/>
-      <c r="G75" s="185"/>
-      <c r="H75" s="10"/>
+      <c r="C75" s="246"/>
+      <c r="D75" s="246"/>
+      <c r="E75" s="246"/>
+      <c r="F75" s="246"/>
+      <c r="G75" s="247"/>
+      <c r="H75" s="9"/>
       <c r="I75" s="9"/>
       <c r="J75" s="9"/>
       <c r="K75" s="9"/>
@@ -6777,19 +6704,18 @@
       <c r="W75" s="9"/>
       <c r="X75" s="9"/>
       <c r="Y75" s="9"/>
-      <c r="Z75" s="9"/>
-    </row>
-    <row r="76" spans="2:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B76" s="186" t="s">
+    </row>
+    <row r="76" spans="2:25" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B76" s="248" t="s">
         <v>157</v>
       </c>
-      <c r="C76" s="187"/>
-      <c r="D76" s="187"/>
-      <c r="E76" s="187"/>
-      <c r="F76" s="187"/>
-      <c r="G76" s="188"/>
-      <c r="H76" s="10"/>
-      <c r="I76" s="35"/>
+      <c r="C76" s="249"/>
+      <c r="D76" s="249"/>
+      <c r="E76" s="249"/>
+      <c r="F76" s="249"/>
+      <c r="G76" s="250"/>
+      <c r="H76" s="35"/>
+      <c r="I76" s="9"/>
       <c r="J76" s="9"/>
       <c r="K76" s="9"/>
       <c r="L76" s="9"/>
@@ -6806,20 +6732,19 @@
       <c r="W76" s="9"/>
       <c r="X76" s="9"/>
       <c r="Y76" s="9"/>
-      <c r="Z76" s="9"/>
-    </row>
-    <row r="77" spans="2:26" s="10" customFormat="1" ht="63" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B77" s="241" t="s">
+    </row>
+    <row r="77" spans="2:25" s="10" customFormat="1" ht="63" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B77" s="208" t="s">
         <v>190</v>
       </c>
-      <c r="C77" s="242"/>
-      <c r="D77" s="242"/>
-      <c r="E77" s="242"/>
-      <c r="F77" s="242"/>
-      <c r="G77" s="254"/>
-    </row>
-    <row r="78" spans="2:26" x14ac:dyDescent="0.25">
-      <c r="H78" s="10"/>
+      <c r="C77" s="210"/>
+      <c r="D77" s="210"/>
+      <c r="E77" s="210"/>
+      <c r="F77" s="210"/>
+      <c r="G77" s="220"/>
+    </row>
+    <row r="78" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="H78" s="9"/>
       <c r="I78" s="9"/>
       <c r="J78" s="9"/>
       <c r="K78" s="9"/>
@@ -6837,17 +6762,52 @@
       <c r="W78" s="9"/>
       <c r="X78" s="9"/>
       <c r="Y78" s="9"/>
-      <c r="Z78" s="9"/>
-    </row>
-    <row r="79" spans="2:26" x14ac:dyDescent="0.25"/>
+    </row>
+    <row r="79" spans="2:25" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="h74j79N81pE9k28tS1hEwUnpWaq69PEBI419soBWgitnMz2Gg7k5LLyOyhb9pf6OY+cnVsCY9sIu412olw5/uQ==" saltValue="lqfSFUpefv9aiStoeeQPzg==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="63">
-    <mergeCell ref="E14:G14"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="B14:D14"/>
-    <mergeCell ref="F28:F29"/>
-    <mergeCell ref="G28:G29"/>
+    <mergeCell ref="B77:G77"/>
+    <mergeCell ref="E61:E62"/>
+    <mergeCell ref="G61:G62"/>
+    <mergeCell ref="B65:D67"/>
+    <mergeCell ref="B69:D71"/>
+    <mergeCell ref="B72:D72"/>
+    <mergeCell ref="F69:G71"/>
+    <mergeCell ref="B75:G75"/>
+    <mergeCell ref="B76:G76"/>
+    <mergeCell ref="B52:C53"/>
+    <mergeCell ref="D52:D53"/>
+    <mergeCell ref="E52:E53"/>
+    <mergeCell ref="F52:F53"/>
+    <mergeCell ref="G52:G53"/>
+    <mergeCell ref="B50:C51"/>
+    <mergeCell ref="D50:D51"/>
+    <mergeCell ref="E50:E51"/>
+    <mergeCell ref="F50:F51"/>
+    <mergeCell ref="G50:G51"/>
+    <mergeCell ref="B48:C49"/>
+    <mergeCell ref="D48:D49"/>
+    <mergeCell ref="E48:E49"/>
+    <mergeCell ref="F48:F49"/>
+    <mergeCell ref="G48:G49"/>
+    <mergeCell ref="B46:C47"/>
+    <mergeCell ref="D46:D47"/>
+    <mergeCell ref="E46:E47"/>
+    <mergeCell ref="F46:F47"/>
+    <mergeCell ref="G46:G47"/>
+    <mergeCell ref="B44:C45"/>
+    <mergeCell ref="D44:D45"/>
+    <mergeCell ref="E44:E45"/>
+    <mergeCell ref="F44:F45"/>
+    <mergeCell ref="G44:G45"/>
+    <mergeCell ref="E40:E41"/>
+    <mergeCell ref="F40:F41"/>
+    <mergeCell ref="G40:G41"/>
+    <mergeCell ref="B42:C43"/>
+    <mergeCell ref="D42:D43"/>
+    <mergeCell ref="E42:E43"/>
+    <mergeCell ref="F42:F43"/>
+    <mergeCell ref="G42:G43"/>
     <mergeCell ref="F72:G72"/>
     <mergeCell ref="B68:D68"/>
     <mergeCell ref="B56:G56"/>
@@ -6864,48 +6824,11 @@
     <mergeCell ref="B22:G22"/>
     <mergeCell ref="B40:C41"/>
     <mergeCell ref="D40:D41"/>
-    <mergeCell ref="E40:E41"/>
-    <mergeCell ref="F40:F41"/>
-    <mergeCell ref="G40:G41"/>
-    <mergeCell ref="B42:C43"/>
-    <mergeCell ref="D42:D43"/>
-    <mergeCell ref="E42:E43"/>
-    <mergeCell ref="F42:F43"/>
-    <mergeCell ref="G42:G43"/>
-    <mergeCell ref="B44:C45"/>
-    <mergeCell ref="D44:D45"/>
-    <mergeCell ref="E44:E45"/>
-    <mergeCell ref="F44:F45"/>
-    <mergeCell ref="G44:G45"/>
-    <mergeCell ref="B46:C47"/>
-    <mergeCell ref="D46:D47"/>
-    <mergeCell ref="E46:E47"/>
-    <mergeCell ref="F46:F47"/>
-    <mergeCell ref="G46:G47"/>
-    <mergeCell ref="B48:C49"/>
-    <mergeCell ref="D48:D49"/>
-    <mergeCell ref="E48:E49"/>
-    <mergeCell ref="F48:F49"/>
-    <mergeCell ref="G48:G49"/>
-    <mergeCell ref="B50:C51"/>
-    <mergeCell ref="D50:D51"/>
-    <mergeCell ref="E50:E51"/>
-    <mergeCell ref="F50:F51"/>
-    <mergeCell ref="G50:G51"/>
-    <mergeCell ref="B52:C53"/>
-    <mergeCell ref="D52:D53"/>
-    <mergeCell ref="E52:E53"/>
-    <mergeCell ref="F52:F53"/>
-    <mergeCell ref="G52:G53"/>
-    <mergeCell ref="B77:G77"/>
-    <mergeCell ref="E61:E62"/>
-    <mergeCell ref="G61:G62"/>
-    <mergeCell ref="B65:D67"/>
-    <mergeCell ref="B69:D71"/>
-    <mergeCell ref="B72:D72"/>
-    <mergeCell ref="F69:G71"/>
-    <mergeCell ref="B75:G75"/>
-    <mergeCell ref="B76:G76"/>
+    <mergeCell ref="E14:G14"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="B14:D14"/>
+    <mergeCell ref="F28:F29"/>
+    <mergeCell ref="G28:G29"/>
   </mergeCells>
   <conditionalFormatting sqref="B11:G11 B14:G14 B17:G17 B20:G20 C23:D23 F23:G23 B40:G53 E61 G61 B62:C62 B65:D71 F67 F69:G72 B77:G77">
     <cfRule type="containsBlanks" dxfId="0" priority="1">
@@ -7040,124 +6963,124 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:24" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A1" s="197" t="s">
+      <c r="A1" s="277" t="s">
         <v>158</v>
       </c>
-      <c r="B1" s="197"/>
-      <c r="C1" s="197"/>
-      <c r="D1" s="197"/>
-      <c r="E1" s="197"/>
-      <c r="F1" s="197"/>
-      <c r="G1" s="197"/>
-      <c r="H1" s="197"/>
-      <c r="I1" s="197"/>
-      <c r="J1" s="197"/>
-      <c r="K1" s="197"/>
-      <c r="L1" s="197"/>
-      <c r="M1" s="197"/>
-      <c r="N1" s="197"/>
-      <c r="O1" s="197"/>
-      <c r="P1" s="197"/>
-      <c r="Q1" s="197"/>
-      <c r="R1" s="197"/>
-      <c r="S1" s="197"/>
-      <c r="T1" s="197"/>
-      <c r="U1" s="197" t="s">
+      <c r="B1" s="277"/>
+      <c r="C1" s="277"/>
+      <c r="D1" s="277"/>
+      <c r="E1" s="277"/>
+      <c r="F1" s="277"/>
+      <c r="G1" s="277"/>
+      <c r="H1" s="277"/>
+      <c r="I1" s="277"/>
+      <c r="J1" s="277"/>
+      <c r="K1" s="277"/>
+      <c r="L1" s="277"/>
+      <c r="M1" s="277"/>
+      <c r="N1" s="277"/>
+      <c r="O1" s="277"/>
+      <c r="P1" s="277"/>
+      <c r="Q1" s="277"/>
+      <c r="R1" s="277"/>
+      <c r="S1" s="277"/>
+      <c r="T1" s="277"/>
+      <c r="U1" s="277" t="s">
         <v>159</v>
       </c>
-      <c r="V1" s="197"/>
-      <c r="W1" s="197"/>
-      <c r="X1" s="197"/>
+      <c r="V1" s="277"/>
+      <c r="W1" s="277"/>
+      <c r="X1" s="277"/>
     </row>
     <row r="2" spans="1:24" ht="33" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="197"/>
-      <c r="B2" s="197"/>
-      <c r="C2" s="197"/>
-      <c r="D2" s="197"/>
-      <c r="E2" s="197"/>
-      <c r="F2" s="197"/>
-      <c r="G2" s="197"/>
-      <c r="H2" s="197"/>
-      <c r="I2" s="197"/>
-      <c r="J2" s="197"/>
-      <c r="K2" s="197"/>
-      <c r="L2" s="197"/>
-      <c r="M2" s="197"/>
-      <c r="N2" s="197"/>
-      <c r="O2" s="197"/>
-      <c r="P2" s="197"/>
-      <c r="Q2" s="197"/>
-      <c r="R2" s="197"/>
-      <c r="S2" s="197"/>
-      <c r="T2" s="197"/>
-      <c r="U2" s="205" t="s">
+      <c r="A2" s="277"/>
+      <c r="B2" s="277"/>
+      <c r="C2" s="277"/>
+      <c r="D2" s="277"/>
+      <c r="E2" s="277"/>
+      <c r="F2" s="277"/>
+      <c r="G2" s="277"/>
+      <c r="H2" s="277"/>
+      <c r="I2" s="277"/>
+      <c r="J2" s="277"/>
+      <c r="K2" s="277"/>
+      <c r="L2" s="277"/>
+      <c r="M2" s="277"/>
+      <c r="N2" s="277"/>
+      <c r="O2" s="277"/>
+      <c r="P2" s="277"/>
+      <c r="Q2" s="277"/>
+      <c r="R2" s="277"/>
+      <c r="S2" s="277"/>
+      <c r="T2" s="277"/>
+      <c r="U2" s="257" t="s">
         <v>160</v>
       </c>
-      <c r="V2" s="205"/>
-      <c r="W2" s="205"/>
-      <c r="X2" s="205"/>
+      <c r="V2" s="257"/>
+      <c r="W2" s="257"/>
+      <c r="X2" s="257"/>
     </row>
     <row r="3" spans="1:24" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="U3" s="206"/>
-      <c r="V3" s="206"/>
-      <c r="W3" s="206"/>
-      <c r="X3" s="206"/>
+      <c r="U3" s="284"/>
+      <c r="V3" s="284"/>
+      <c r="W3" s="284"/>
+      <c r="X3" s="284"/>
     </row>
     <row r="4" spans="1:24" s="2" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="202" t="s">
+      <c r="A4" s="281" t="s">
         <v>161</v>
       </c>
-      <c r="B4" s="203"/>
-      <c r="C4" s="203"/>
-      <c r="D4" s="203"/>
-      <c r="E4" s="203"/>
-      <c r="F4" s="203"/>
-      <c r="G4" s="203"/>
-      <c r="H4" s="203"/>
-      <c r="I4" s="203"/>
-      <c r="J4" s="203"/>
-      <c r="K4" s="203"/>
-      <c r="L4" s="203"/>
-      <c r="M4" s="204"/>
-      <c r="N4" s="202" t="s">
+      <c r="B4" s="282"/>
+      <c r="C4" s="282"/>
+      <c r="D4" s="282"/>
+      <c r="E4" s="282"/>
+      <c r="F4" s="282"/>
+      <c r="G4" s="282"/>
+      <c r="H4" s="282"/>
+      <c r="I4" s="282"/>
+      <c r="J4" s="282"/>
+      <c r="K4" s="282"/>
+      <c r="L4" s="282"/>
+      <c r="M4" s="283"/>
+      <c r="N4" s="281" t="s">
         <v>162</v>
       </c>
-      <c r="O4" s="203"/>
-      <c r="P4" s="203"/>
-      <c r="Q4" s="203"/>
-      <c r="R4" s="203"/>
-      <c r="S4" s="203"/>
-      <c r="T4" s="203"/>
-      <c r="U4" s="203"/>
-      <c r="V4" s="203"/>
-      <c r="W4" s="203"/>
-      <c r="X4" s="204"/>
+      <c r="O4" s="282"/>
+      <c r="P4" s="282"/>
+      <c r="Q4" s="282"/>
+      <c r="R4" s="282"/>
+      <c r="S4" s="282"/>
+      <c r="T4" s="282"/>
+      <c r="U4" s="282"/>
+      <c r="V4" s="282"/>
+      <c r="W4" s="282"/>
+      <c r="X4" s="283"/>
     </row>
     <row r="5" spans="1:24" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="199"/>
-      <c r="B5" s="200"/>
-      <c r="C5" s="200"/>
-      <c r="D5" s="200"/>
-      <c r="E5" s="200"/>
-      <c r="F5" s="200"/>
-      <c r="G5" s="200"/>
-      <c r="H5" s="200"/>
-      <c r="I5" s="200"/>
-      <c r="J5" s="200"/>
-      <c r="K5" s="200"/>
-      <c r="L5" s="200"/>
-      <c r="M5" s="201"/>
-      <c r="N5" s="199"/>
-      <c r="O5" s="200"/>
-      <c r="P5" s="200"/>
-      <c r="Q5" s="200"/>
-      <c r="R5" s="200"/>
-      <c r="S5" s="200"/>
-      <c r="T5" s="200"/>
-      <c r="U5" s="200"/>
-      <c r="V5" s="200"/>
-      <c r="W5" s="200"/>
-      <c r="X5" s="201"/>
+      <c r="A5" s="278"/>
+      <c r="B5" s="279"/>
+      <c r="C5" s="279"/>
+      <c r="D5" s="279"/>
+      <c r="E5" s="279"/>
+      <c r="F5" s="279"/>
+      <c r="G5" s="279"/>
+      <c r="H5" s="279"/>
+      <c r="I5" s="279"/>
+      <c r="J5" s="279"/>
+      <c r="K5" s="279"/>
+      <c r="L5" s="279"/>
+      <c r="M5" s="280"/>
+      <c r="N5" s="278"/>
+      <c r="O5" s="279"/>
+      <c r="P5" s="279"/>
+      <c r="Q5" s="279"/>
+      <c r="R5" s="279"/>
+      <c r="S5" s="279"/>
+      <c r="T5" s="279"/>
+      <c r="U5" s="279"/>
+      <c r="V5" s="279"/>
+      <c r="W5" s="279"/>
+      <c r="X5" s="280"/>
     </row>
     <row r="6" spans="1:24" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3"/>
@@ -7186,66 +7109,66 @@
       <c r="X6" s="3"/>
     </row>
     <row r="7" spans="1:24" s="2" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="198" t="s">
+      <c r="A7" s="255" t="s">
         <v>163</v>
       </c>
-      <c r="B7" s="198"/>
-      <c r="C7" s="198"/>
-      <c r="D7" s="198"/>
-      <c r="E7" s="198"/>
-      <c r="F7" s="198"/>
-      <c r="G7" s="198"/>
-      <c r="H7" s="198"/>
-      <c r="I7" s="198"/>
-      <c r="J7" s="198" t="s">
+      <c r="B7" s="255"/>
+      <c r="C7" s="255"/>
+      <c r="D7" s="255"/>
+      <c r="E7" s="255"/>
+      <c r="F7" s="255"/>
+      <c r="G7" s="255"/>
+      <c r="H7" s="255"/>
+      <c r="I7" s="255"/>
+      <c r="J7" s="255" t="s">
         <v>32</v>
       </c>
-      <c r="K7" s="198"/>
-      <c r="L7" s="198"/>
-      <c r="M7" s="198"/>
-      <c r="N7" s="198"/>
-      <c r="O7" s="198"/>
-      <c r="P7" s="198" t="s">
+      <c r="K7" s="255"/>
+      <c r="L7" s="255"/>
+      <c r="M7" s="255"/>
+      <c r="N7" s="255"/>
+      <c r="O7" s="255"/>
+      <c r="P7" s="255" t="s">
         <v>58</v>
       </c>
-      <c r="Q7" s="198"/>
-      <c r="R7" s="198"/>
-      <c r="S7" s="198"/>
-      <c r="T7" s="198"/>
-      <c r="U7" s="198"/>
-      <c r="V7" s="198"/>
-      <c r="W7" s="198"/>
-      <c r="X7" s="198"/>
+      <c r="Q7" s="255"/>
+      <c r="R7" s="255"/>
+      <c r="S7" s="255"/>
+      <c r="T7" s="255"/>
+      <c r="U7" s="255"/>
+      <c r="V7" s="255"/>
+      <c r="W7" s="255"/>
+      <c r="X7" s="255"/>
     </row>
     <row r="8" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="207"/>
-      <c r="B8" s="207"/>
-      <c r="C8" s="207"/>
-      <c r="D8" s="207"/>
-      <c r="E8" s="207"/>
-      <c r="F8" s="207"/>
-      <c r="G8" s="207"/>
-      <c r="H8" s="207"/>
-      <c r="I8" s="207"/>
-      <c r="J8" s="208" t="s">
+      <c r="A8" s="262"/>
+      <c r="B8" s="262"/>
+      <c r="C8" s="262"/>
+      <c r="D8" s="262"/>
+      <c r="E8" s="262"/>
+      <c r="F8" s="262"/>
+      <c r="G8" s="262"/>
+      <c r="H8" s="262"/>
+      <c r="I8" s="262"/>
+      <c r="J8" s="263" t="s">
         <v>164</v>
       </c>
-      <c r="K8" s="209"/>
-      <c r="L8" s="209"/>
-      <c r="M8" s="209"/>
-      <c r="N8" s="209"/>
-      <c r="O8" s="210"/>
-      <c r="P8" s="208" t="s">
+      <c r="K8" s="264"/>
+      <c r="L8" s="264"/>
+      <c r="M8" s="264"/>
+      <c r="N8" s="264"/>
+      <c r="O8" s="265"/>
+      <c r="P8" s="263" t="s">
         <v>165</v>
       </c>
-      <c r="Q8" s="209"/>
-      <c r="R8" s="209"/>
-      <c r="S8" s="209"/>
-      <c r="T8" s="209"/>
-      <c r="U8" s="209"/>
-      <c r="V8" s="209"/>
-      <c r="W8" s="209"/>
-      <c r="X8" s="210"/>
+      <c r="Q8" s="264"/>
+      <c r="R8" s="264"/>
+      <c r="S8" s="264"/>
+      <c r="T8" s="264"/>
+      <c r="U8" s="264"/>
+      <c r="V8" s="264"/>
+      <c r="W8" s="264"/>
+      <c r="X8" s="265"/>
     </row>
     <row r="9" spans="1:24" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3"/>
@@ -7274,66 +7197,66 @@
       <c r="X9" s="3"/>
     </row>
     <row r="10" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="211" t="s">
+      <c r="A10" s="275" t="s">
         <v>166</v>
       </c>
-      <c r="B10" s="211"/>
-      <c r="C10" s="211"/>
-      <c r="D10" s="211"/>
-      <c r="E10" s="211"/>
-      <c r="F10" s="211"/>
-      <c r="G10" s="211"/>
-      <c r="H10" s="211"/>
-      <c r="I10" s="211"/>
-      <c r="J10" s="211"/>
-      <c r="K10" s="211"/>
-      <c r="L10" s="211"/>
-      <c r="M10" s="211"/>
-      <c r="N10" s="211"/>
-      <c r="O10" s="211"/>
-      <c r="P10" s="211"/>
-      <c r="Q10" s="211"/>
-      <c r="R10" s="211"/>
-      <c r="S10" s="211"/>
-      <c r="T10" s="211"/>
-      <c r="U10" s="211"/>
-      <c r="V10" s="211"/>
-      <c r="W10" s="211"/>
-      <c r="X10" s="211"/>
+      <c r="B10" s="275"/>
+      <c r="C10" s="275"/>
+      <c r="D10" s="275"/>
+      <c r="E10" s="275"/>
+      <c r="F10" s="275"/>
+      <c r="G10" s="275"/>
+      <c r="H10" s="275"/>
+      <c r="I10" s="275"/>
+      <c r="J10" s="275"/>
+      <c r="K10" s="275"/>
+      <c r="L10" s="275"/>
+      <c r="M10" s="275"/>
+      <c r="N10" s="275"/>
+      <c r="O10" s="275"/>
+      <c r="P10" s="275"/>
+      <c r="Q10" s="275"/>
+      <c r="R10" s="275"/>
+      <c r="S10" s="275"/>
+      <c r="T10" s="275"/>
+      <c r="U10" s="275"/>
+      <c r="V10" s="275"/>
+      <c r="W10" s="275"/>
+      <c r="X10" s="275"/>
     </row>
     <row r="11" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="212" t="s">
+      <c r="A11" s="276" t="s">
         <v>126</v>
       </c>
-      <c r="B11" s="212"/>
-      <c r="C11" s="212"/>
-      <c r="D11" s="212"/>
-      <c r="E11" s="212"/>
-      <c r="F11" s="212"/>
-      <c r="G11" s="212" t="s">
+      <c r="B11" s="276"/>
+      <c r="C11" s="276"/>
+      <c r="D11" s="276"/>
+      <c r="E11" s="276"/>
+      <c r="F11" s="276"/>
+      <c r="G11" s="276" t="s">
         <v>167</v>
       </c>
-      <c r="H11" s="212"/>
-      <c r="I11" s="212"/>
-      <c r="J11" s="212"/>
-      <c r="K11" s="212"/>
-      <c r="L11" s="212"/>
-      <c r="M11" s="212" t="s">
+      <c r="H11" s="276"/>
+      <c r="I11" s="276"/>
+      <c r="J11" s="276"/>
+      <c r="K11" s="276"/>
+      <c r="L11" s="276"/>
+      <c r="M11" s="276" t="s">
         <v>168</v>
       </c>
-      <c r="N11" s="212"/>
-      <c r="O11" s="212"/>
-      <c r="P11" s="212"/>
-      <c r="Q11" s="212"/>
-      <c r="R11" s="212"/>
-      <c r="S11" s="212" t="s">
+      <c r="N11" s="276"/>
+      <c r="O11" s="276"/>
+      <c r="P11" s="276"/>
+      <c r="Q11" s="276"/>
+      <c r="R11" s="276"/>
+      <c r="S11" s="276" t="s">
         <v>169</v>
       </c>
-      <c r="T11" s="212"/>
-      <c r="U11" s="212"/>
-      <c r="V11" s="212"/>
-      <c r="W11" s="212"/>
-      <c r="X11" s="212"/>
+      <c r="T11" s="276"/>
+      <c r="U11" s="276"/>
+      <c r="V11" s="276"/>
+      <c r="W11" s="276"/>
+      <c r="X11" s="276"/>
     </row>
     <row r="12" spans="1:24" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3"/>
@@ -7362,66 +7285,66 @@
       <c r="X12" s="3"/>
     </row>
     <row r="13" spans="1:24" s="2" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="198" t="s">
+      <c r="A13" s="255" t="s">
         <v>170</v>
       </c>
-      <c r="B13" s="198"/>
-      <c r="C13" s="198"/>
-      <c r="D13" s="198"/>
-      <c r="E13" s="198"/>
-      <c r="F13" s="198"/>
-      <c r="G13" s="198"/>
-      <c r="H13" s="198"/>
-      <c r="I13" s="198"/>
-      <c r="J13" s="198" t="s">
+      <c r="B13" s="255"/>
+      <c r="C13" s="255"/>
+      <c r="D13" s="255"/>
+      <c r="E13" s="255"/>
+      <c r="F13" s="255"/>
+      <c r="G13" s="255"/>
+      <c r="H13" s="255"/>
+      <c r="I13" s="255"/>
+      <c r="J13" s="255" t="s">
         <v>32</v>
       </c>
-      <c r="K13" s="198"/>
-      <c r="L13" s="198"/>
-      <c r="M13" s="198"/>
-      <c r="N13" s="198"/>
-      <c r="O13" s="198"/>
-      <c r="P13" s="198" t="s">
+      <c r="K13" s="255"/>
+      <c r="L13" s="255"/>
+      <c r="M13" s="255"/>
+      <c r="N13" s="255"/>
+      <c r="O13" s="255"/>
+      <c r="P13" s="255" t="s">
         <v>58</v>
       </c>
-      <c r="Q13" s="198"/>
-      <c r="R13" s="198"/>
-      <c r="S13" s="198"/>
-      <c r="T13" s="198"/>
-      <c r="U13" s="198"/>
-      <c r="V13" s="198"/>
-      <c r="W13" s="198"/>
-      <c r="X13" s="198"/>
+      <c r="Q13" s="255"/>
+      <c r="R13" s="255"/>
+      <c r="S13" s="255"/>
+      <c r="T13" s="255"/>
+      <c r="U13" s="255"/>
+      <c r="V13" s="255"/>
+      <c r="W13" s="255"/>
+      <c r="X13" s="255"/>
     </row>
     <row r="14" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="207"/>
-      <c r="B14" s="207"/>
-      <c r="C14" s="207"/>
-      <c r="D14" s="207"/>
-      <c r="E14" s="207"/>
-      <c r="F14" s="207"/>
-      <c r="G14" s="207"/>
-      <c r="H14" s="207"/>
-      <c r="I14" s="207"/>
-      <c r="J14" s="208" t="s">
+      <c r="A14" s="262"/>
+      <c r="B14" s="262"/>
+      <c r="C14" s="262"/>
+      <c r="D14" s="262"/>
+      <c r="E14" s="262"/>
+      <c r="F14" s="262"/>
+      <c r="G14" s="262"/>
+      <c r="H14" s="262"/>
+      <c r="I14" s="262"/>
+      <c r="J14" s="263" t="s">
         <v>171</v>
       </c>
-      <c r="K14" s="209"/>
-      <c r="L14" s="209"/>
-      <c r="M14" s="209"/>
-      <c r="N14" s="209"/>
-      <c r="O14" s="210"/>
-      <c r="P14" s="208" t="s">
+      <c r="K14" s="264"/>
+      <c r="L14" s="264"/>
+      <c r="M14" s="264"/>
+      <c r="N14" s="264"/>
+      <c r="O14" s="265"/>
+      <c r="P14" s="263" t="s">
         <v>172</v>
       </c>
-      <c r="Q14" s="209"/>
-      <c r="R14" s="209"/>
-      <c r="S14" s="209"/>
-      <c r="T14" s="209"/>
-      <c r="U14" s="209"/>
-      <c r="V14" s="209"/>
-      <c r="W14" s="209"/>
-      <c r="X14" s="210"/>
+      <c r="Q14" s="264"/>
+      <c r="R14" s="264"/>
+      <c r="S14" s="264"/>
+      <c r="T14" s="264"/>
+      <c r="U14" s="264"/>
+      <c r="V14" s="264"/>
+      <c r="W14" s="264"/>
+      <c r="X14" s="265"/>
     </row>
     <row r="15" spans="1:24" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3"/>
@@ -7450,172 +7373,184 @@
       <c r="X15" s="3"/>
     </row>
     <row r="16" spans="1:24" s="4" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="218" t="s">
+      <c r="A16" s="266" t="s">
         <v>173</v>
       </c>
-      <c r="B16" s="218"/>
-      <c r="C16" s="218"/>
-      <c r="D16" s="218"/>
-      <c r="E16" s="218"/>
-      <c r="F16" s="218"/>
-      <c r="G16" s="218"/>
-      <c r="H16" s="218"/>
-      <c r="I16" s="218"/>
-      <c r="J16" s="219" t="s">
+      <c r="B16" s="266"/>
+      <c r="C16" s="266"/>
+      <c r="D16" s="266"/>
+      <c r="E16" s="266"/>
+      <c r="F16" s="266"/>
+      <c r="G16" s="266"/>
+      <c r="H16" s="266"/>
+      <c r="I16" s="266"/>
+      <c r="J16" s="267" t="s">
         <v>174</v>
       </c>
-      <c r="K16" s="219"/>
-      <c r="L16" s="219"/>
-      <c r="M16" s="219"/>
-      <c r="N16" s="218" t="s">
+      <c r="K16" s="267"/>
+      <c r="L16" s="267"/>
+      <c r="M16" s="267"/>
+      <c r="N16" s="266" t="s">
         <v>175</v>
       </c>
-      <c r="O16" s="218"/>
-      <c r="P16" s="218"/>
-      <c r="Q16" s="218"/>
-      <c r="R16" s="218"/>
-      <c r="S16" s="218"/>
-      <c r="T16" s="220" t="s">
+      <c r="O16" s="266"/>
+      <c r="P16" s="266"/>
+      <c r="Q16" s="266"/>
+      <c r="R16" s="266"/>
+      <c r="S16" s="266"/>
+      <c r="T16" s="268" t="s">
         <v>176</v>
       </c>
-      <c r="U16" s="220"/>
-      <c r="V16" s="220"/>
-      <c r="W16" s="220"/>
-      <c r="X16" s="220"/>
+      <c r="U16" s="268"/>
+      <c r="V16" s="268"/>
+      <c r="W16" s="268"/>
+      <c r="X16" s="268"/>
     </row>
     <row r="17" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="213" t="s">
+      <c r="A17" s="256" t="s">
         <v>177</v>
       </c>
-      <c r="B17" s="205"/>
-      <c r="C17" s="205"/>
-      <c r="D17" s="205"/>
-      <c r="E17" s="205"/>
-      <c r="F17" s="205"/>
-      <c r="G17" s="205"/>
-      <c r="H17" s="205"/>
-      <c r="I17" s="214"/>
-      <c r="J17" s="221" t="s">
+      <c r="B17" s="257"/>
+      <c r="C17" s="257"/>
+      <c r="D17" s="257"/>
+      <c r="E17" s="257"/>
+      <c r="F17" s="257"/>
+      <c r="G17" s="257"/>
+      <c r="H17" s="257"/>
+      <c r="I17" s="258"/>
+      <c r="J17" s="269" t="s">
         <v>178</v>
       </c>
-      <c r="K17" s="222"/>
-      <c r="L17" s="222"/>
-      <c r="M17" s="223"/>
-      <c r="N17" s="213" t="s">
+      <c r="K17" s="270"/>
+      <c r="L17" s="270"/>
+      <c r="M17" s="271"/>
+      <c r="N17" s="256" t="s">
         <v>179</v>
       </c>
-      <c r="O17" s="205"/>
-      <c r="P17" s="205"/>
-      <c r="Q17" s="205"/>
-      <c r="R17" s="205"/>
-      <c r="S17" s="214"/>
-      <c r="T17" s="213" t="s">
+      <c r="O17" s="257"/>
+      <c r="P17" s="257"/>
+      <c r="Q17" s="257"/>
+      <c r="R17" s="257"/>
+      <c r="S17" s="258"/>
+      <c r="T17" s="256" t="s">
         <v>180</v>
       </c>
-      <c r="U17" s="205"/>
-      <c r="V17" s="205"/>
-      <c r="W17" s="205"/>
-      <c r="X17" s="214"/>
+      <c r="U17" s="257"/>
+      <c r="V17" s="257"/>
+      <c r="W17" s="257"/>
+      <c r="X17" s="258"/>
     </row>
     <row r="18" spans="1:24" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="215"/>
-      <c r="B18" s="216"/>
-      <c r="C18" s="216"/>
-      <c r="D18" s="216"/>
-      <c r="E18" s="216"/>
-      <c r="F18" s="216"/>
-      <c r="G18" s="216"/>
-      <c r="H18" s="216"/>
-      <c r="I18" s="217"/>
-      <c r="J18" s="224"/>
-      <c r="K18" s="225"/>
-      <c r="L18" s="225"/>
-      <c r="M18" s="226"/>
-      <c r="N18" s="215"/>
-      <c r="O18" s="216"/>
-      <c r="P18" s="216"/>
-      <c r="Q18" s="216"/>
-      <c r="R18" s="216"/>
-      <c r="S18" s="217"/>
-      <c r="T18" s="215"/>
-      <c r="U18" s="216"/>
-      <c r="V18" s="216"/>
-      <c r="W18" s="216"/>
-      <c r="X18" s="217"/>
+      <c r="A18" s="259"/>
+      <c r="B18" s="260"/>
+      <c r="C18" s="260"/>
+      <c r="D18" s="260"/>
+      <c r="E18" s="260"/>
+      <c r="F18" s="260"/>
+      <c r="G18" s="260"/>
+      <c r="H18" s="260"/>
+      <c r="I18" s="261"/>
+      <c r="J18" s="272"/>
+      <c r="K18" s="273"/>
+      <c r="L18" s="273"/>
+      <c r="M18" s="274"/>
+      <c r="N18" s="259"/>
+      <c r="O18" s="260"/>
+      <c r="P18" s="260"/>
+      <c r="Q18" s="260"/>
+      <c r="R18" s="260"/>
+      <c r="S18" s="261"/>
+      <c r="T18" s="259"/>
+      <c r="U18" s="260"/>
+      <c r="V18" s="260"/>
+      <c r="W18" s="260"/>
+      <c r="X18" s="261"/>
     </row>
     <row r="19" spans="1:24" ht="39" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="20" spans="1:24" ht="39" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="21" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A21" s="230" t="s">
+      <c r="A21" s="254" t="s">
         <v>181</v>
       </c>
-      <c r="B21" s="230"/>
-      <c r="C21" s="230"/>
-      <c r="D21" s="230"/>
-      <c r="E21" s="230"/>
-      <c r="F21" s="230"/>
-      <c r="G21" s="230"/>
-      <c r="H21" s="230"/>
+      <c r="B21" s="254"/>
+      <c r="C21" s="254"/>
+      <c r="D21" s="254"/>
+      <c r="E21" s="254"/>
+      <c r="F21" s="254"/>
+      <c r="G21" s="254"/>
+      <c r="H21" s="254"/>
       <c r="I21" s="5"/>
-      <c r="J21" s="230" t="s">
+      <c r="J21" s="254" t="s">
         <v>182</v>
       </c>
-      <c r="K21" s="230"/>
-      <c r="L21" s="230"/>
-      <c r="M21" s="230"/>
-      <c r="N21" s="230"/>
-      <c r="O21" s="230"/>
-      <c r="P21" s="230"/>
+      <c r="K21" s="254"/>
+      <c r="L21" s="254"/>
+      <c r="M21" s="254"/>
+      <c r="N21" s="254"/>
+      <c r="O21" s="254"/>
+      <c r="P21" s="254"/>
       <c r="Q21" s="6"/>
-      <c r="R21" s="230" t="s">
+      <c r="R21" s="254" t="s">
         <v>183</v>
       </c>
-      <c r="S21" s="230"/>
-      <c r="T21" s="230"/>
-      <c r="U21" s="230"/>
-      <c r="V21" s="230"/>
-      <c r="W21" s="230"/>
-      <c r="X21" s="230"/>
+      <c r="S21" s="254"/>
+      <c r="T21" s="254"/>
+      <c r="U21" s="254"/>
+      <c r="V21" s="254"/>
+      <c r="W21" s="254"/>
+      <c r="X21" s="254"/>
     </row>
     <row r="23" spans="1:24" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="P23" s="227" t="s">
+      <c r="P23" s="251" t="s">
         <v>184</v>
       </c>
-      <c r="Q23" s="227"/>
-      <c r="R23" s="227"/>
-      <c r="S23" s="227"/>
-      <c r="T23" s="227"/>
-      <c r="U23" s="228" t="s">
+      <c r="Q23" s="251"/>
+      <c r="R23" s="251"/>
+      <c r="S23" s="251"/>
+      <c r="T23" s="251"/>
+      <c r="U23" s="252" t="s">
         <v>185</v>
       </c>
-      <c r="V23" s="228"/>
-      <c r="W23" s="228"/>
-      <c r="X23" s="228"/>
+      <c r="V23" s="252"/>
+      <c r="W23" s="252"/>
+      <c r="X23" s="252"/>
     </row>
     <row r="24" spans="1:24" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="P24" s="227" t="s">
+      <c r="P24" s="251" t="s">
         <v>186</v>
       </c>
-      <c r="Q24" s="227"/>
-      <c r="R24" s="227"/>
-      <c r="S24" s="227"/>
-      <c r="T24" s="227"/>
-      <c r="U24" s="229" t="s">
+      <c r="Q24" s="251"/>
+      <c r="R24" s="251"/>
+      <c r="S24" s="251"/>
+      <c r="T24" s="251"/>
+      <c r="U24" s="253" t="s">
         <v>187</v>
       </c>
-      <c r="V24" s="229"/>
-      <c r="W24" s="229"/>
-      <c r="X24" s="229"/>
+      <c r="V24" s="253"/>
+      <c r="W24" s="253"/>
+      <c r="X24" s="253"/>
     </row>
   </sheetData>
   <mergeCells count="40">
-    <mergeCell ref="P23:T23"/>
-    <mergeCell ref="U23:X23"/>
-    <mergeCell ref="P24:T24"/>
-    <mergeCell ref="U24:X24"/>
-    <mergeCell ref="A21:H21"/>
-    <mergeCell ref="J21:P21"/>
-    <mergeCell ref="R21:X21"/>
+    <mergeCell ref="A1:T1"/>
+    <mergeCell ref="U1:X1"/>
+    <mergeCell ref="A2:T2"/>
+    <mergeCell ref="A7:I7"/>
+    <mergeCell ref="J7:O7"/>
+    <mergeCell ref="P7:X7"/>
+    <mergeCell ref="A5:M5"/>
+    <mergeCell ref="A4:M4"/>
+    <mergeCell ref="N4:X4"/>
+    <mergeCell ref="N5:X5"/>
+    <mergeCell ref="U2:X3"/>
+    <mergeCell ref="A8:I8"/>
+    <mergeCell ref="J8:O8"/>
+    <mergeCell ref="P8:X8"/>
+    <mergeCell ref="A10:X10"/>
+    <mergeCell ref="A11:F11"/>
+    <mergeCell ref="G11:L11"/>
+    <mergeCell ref="M11:R11"/>
+    <mergeCell ref="S11:X11"/>
     <mergeCell ref="A13:I13"/>
     <mergeCell ref="J13:O13"/>
     <mergeCell ref="P13:X13"/>
@@ -7630,25 +7565,13 @@
     <mergeCell ref="T16:X16"/>
     <mergeCell ref="A17:I18"/>
     <mergeCell ref="J17:M18"/>
-    <mergeCell ref="A8:I8"/>
-    <mergeCell ref="J8:O8"/>
-    <mergeCell ref="P8:X8"/>
-    <mergeCell ref="A10:X10"/>
-    <mergeCell ref="A11:F11"/>
-    <mergeCell ref="G11:L11"/>
-    <mergeCell ref="M11:R11"/>
-    <mergeCell ref="S11:X11"/>
-    <mergeCell ref="A1:T1"/>
-    <mergeCell ref="U1:X1"/>
-    <mergeCell ref="A2:T2"/>
-    <mergeCell ref="A7:I7"/>
-    <mergeCell ref="J7:O7"/>
-    <mergeCell ref="P7:X7"/>
-    <mergeCell ref="A5:M5"/>
-    <mergeCell ref="A4:M4"/>
-    <mergeCell ref="N4:X4"/>
-    <mergeCell ref="N5:X5"/>
-    <mergeCell ref="U2:X3"/>
+    <mergeCell ref="P23:T23"/>
+    <mergeCell ref="U23:X23"/>
+    <mergeCell ref="P24:T24"/>
+    <mergeCell ref="U24:X24"/>
+    <mergeCell ref="A21:H21"/>
+    <mergeCell ref="J21:P21"/>
+    <mergeCell ref="R21:X21"/>
   </mergeCells>
   <pageMargins left="0.51181102362204722" right="0.51181102362204722" top="0.35433070866141736" bottom="0.35433070866141736" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup scale="95" orientation="landscape" horizontalDpi="4294967294" verticalDpi="200" r:id="rId1"/>
@@ -7657,18 +7580,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <TaxCatchAll xmlns="41dd0a9e-964d-48c8-9389-7445c2a187f7" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="edbb1c21-1b45-407e-8894-c97732534993">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <_Flow_SignoffStatus xmlns="edbb1c21-1b45-407e-8894-c97732534993" xsi:nil="true"/>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <FechayHora xmlns="edbb1c21-1b45-407e-8894-c97732534993" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -7962,22 +7879,24 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <TaxCatchAll xmlns="41dd0a9e-964d-48c8-9389-7445c2a187f7" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="edbb1c21-1b45-407e-8894-c97732534993">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <_Flow_SignoffStatus xmlns="edbb1c21-1b45-407e-8894-c97732534993" xsi:nil="true"/>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <FechayHora xmlns="edbb1c21-1b45-407e-8894-c97732534993" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBE5A30C-34BC-4387-870E-CFF8B53C216A}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7CCE7917-804F-4951-9FEA-F53AEA82B8BE}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="41dd0a9e-964d-48c8-9389-7445c2a187f7"/>
-    <ds:schemaRef ds:uri="edbb1c21-1b45-407e-8894-c97732534993"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -8003,9 +7922,13 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7CCE7917-804F-4951-9FEA-F53AEA82B8BE}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBE5A30C-34BC-4387-870E-CFF8B53C216A}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="41dd0a9e-964d-48c8-9389-7445c2a187f7"/>
+    <ds:schemaRef ds:uri="edbb1c21-1b45-407e-8894-c97732534993"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Actualizacion de formatos: Bitacoras y Visitas
</commit_message>
<xml_diff>
--- a/Formatos/BITACORAS GFPI-F-147V4.xlsx
+++ b/Formatos/BITACORAS GFPI-F-147V4.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SEANT\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SEANT\OneDrive\Documents\Seto 2026\sena\Manual SENA Etapa Productiva\manual-general-aprendiz\Formatos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{324AC6E9-AFFB-4C03-A5D0-79D396FF8B1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10657848-F8CF-4322-822C-D0FE44C062DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="191">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="189">
   <si>
     <t>Código: 
 GFPI-F-147</t>
@@ -800,12 +800,6 @@
   </si>
   <si>
     <t>firma el instructor que recibe la bitácora</t>
-  </si>
-  <si>
-    <t>Satorres@sena.edu.co / Storres@timespanish.com</t>
-  </si>
-  <si>
-    <t>Sergio Andres Torres Martinez</t>
   </si>
   <si>
     <t>.</t>
@@ -2610,522 +2604,539 @@
     <xf numFmtId="0" fontId="14" fillId="2" borderId="82" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="6" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="6" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="6" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="6" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="75" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="53" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="73" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="59" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="69" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="65" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="66" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="67" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="35" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="82" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="82" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="83" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="74" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="2" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="2" borderId="53" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="76" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="55" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="85" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="70" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="74" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="6" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="6" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="75" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="75" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="53" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="75" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="65" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="66" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="67" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="56" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="59" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="57" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="55" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="86" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="63" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="73" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="59" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="69" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="6" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="6" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="35" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center"/>
       <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement i="0"/>
+        </ext>
+      </extLst>
     </xf>
     <xf numFmtId="0" fontId="35" fillId="0" borderId="75" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center"/>
       <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="82" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="82" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="83" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="74" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="85" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="70" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="75" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="74" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="75" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="2" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="2" borderId="53" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="76" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="55" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="56" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="57" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="59" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="55" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="86" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="63" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement i="0"/>
+        </ext>
+      </extLst>
     </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="2">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFDCFD71"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -3434,189 +3445,6 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>127000</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>127000</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>393700</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>384175</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Imagen 2">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9F5D1716-4E29-4788-B4AD-A5F6CB5F894F}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="2455333" y="2402417"/>
-          <a:ext cx="266700" cy="257175"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-        </a:extLst>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>321733</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>120650</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>588433</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>377825</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="5" name="Imagen 4">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{52642EA2-F24B-4131-A26C-FAE133CEDF2B}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="7010400" y="2396067"/>
-          <a:ext cx="266700" cy="257175"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-        </a:extLst>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>31751</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>126999</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>298451</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>384174</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="6" name="Imagen 5">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5FB48459-C783-4906-B92C-63C121B01FCA}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="11080751" y="2402416"/>
-          <a:ext cx="266700" cy="257175"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-        </a:extLst>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -3697,6 +3525,23 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
+</file>
+
+<file path=xl/featurePropertyBag/featurePropertyBag.xml><?xml version="1.0" encoding="utf-8"?>
+<FeaturePropertyBags xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag">
+  <bag type="Checkbox"/>
+  <bag type="XFControls">
+    <bagId k="CellControl">0</bagId>
+  </bag>
+  <bag type="XFComplement">
+    <bagId k="XFControls">1</bagId>
+  </bag>
+  <bag type="XFComplements" extRef="XFComplementsMapperExtRef">
+    <a k="MappedFeaturePropertyBags">
+      <bagId>2</bagId>
+    </a>
+  </bag>
+</FeaturePropertyBags>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4020,56 +3865,56 @@
       <c r="H2" s="7"/>
     </row>
     <row r="3" spans="2:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="137" t="s">
+      <c r="B3" s="170" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="138"/>
-      <c r="D3" s="138"/>
-      <c r="E3" s="139"/>
+      <c r="C3" s="171"/>
+      <c r="D3" s="171"/>
+      <c r="E3" s="172"/>
       <c r="F3" s="7"/>
       <c r="G3" s="7"/>
       <c r="H3" s="7"/>
     </row>
     <row r="4" spans="2:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="140" t="s">
+      <c r="B4" s="173" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="141"/>
-      <c r="D4" s="141"/>
-      <c r="E4" s="142"/>
+      <c r="C4" s="174"/>
+      <c r="D4" s="174"/>
+      <c r="E4" s="175"/>
       <c r="F4" s="7"/>
       <c r="G4" s="7"/>
       <c r="H4" s="7"/>
     </row>
     <row r="5" spans="2:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="143" t="s">
+      <c r="B5" s="238" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="144"/>
-      <c r="D5" s="144"/>
-      <c r="E5" s="145"/>
+      <c r="C5" s="239"/>
+      <c r="D5" s="239"/>
+      <c r="E5" s="240"/>
       <c r="F5" s="7"/>
       <c r="G5" s="7"/>
       <c r="H5" s="7"/>
     </row>
     <row r="6" spans="2:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="140" t="s">
+      <c r="B6" s="173" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="141"/>
-      <c r="D6" s="141"/>
-      <c r="E6" s="142"/>
+      <c r="C6" s="174"/>
+      <c r="D6" s="174"/>
+      <c r="E6" s="175"/>
       <c r="F6" s="7"/>
       <c r="G6" s="7"/>
       <c r="H6" s="7"/>
     </row>
     <row r="7" spans="2:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="137" t="s">
+      <c r="B7" s="170" t="s">
         <v>6</v>
       </c>
-      <c r="C7" s="138"/>
-      <c r="D7" s="138"/>
-      <c r="E7" s="139"/>
+      <c r="C7" s="171"/>
+      <c r="D7" s="171"/>
+      <c r="E7" s="172"/>
       <c r="F7" s="7"/>
       <c r="G7" s="7"/>
       <c r="H7" s="7"/>
@@ -4081,45 +3926,45 @@
       <c r="C8" s="54" t="s">
         <v>8</v>
       </c>
-      <c r="D8" s="146" t="s">
+      <c r="D8" s="241" t="s">
         <v>9</v>
       </c>
-      <c r="E8" s="147"/>
+      <c r="E8" s="242"/>
       <c r="H8" s="7"/>
     </row>
     <row r="9" spans="2:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="148" t="s">
+      <c r="B9" s="243" t="s">
         <v>10</v>
       </c>
-      <c r="C9" s="149"/>
-      <c r="D9" s="149"/>
-      <c r="E9" s="150"/>
+      <c r="C9" s="244"/>
+      <c r="D9" s="244"/>
+      <c r="E9" s="245"/>
       <c r="G9" s="7"/>
       <c r="H9" s="7"/>
     </row>
     <row r="10" spans="2:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="151" t="s">
+      <c r="B10" s="246" t="s">
         <v>11</v>
       </c>
-      <c r="C10" s="152"/>
-      <c r="D10" s="152"/>
-      <c r="E10" s="153"/>
+      <c r="C10" s="247"/>
+      <c r="D10" s="247"/>
+      <c r="E10" s="248"/>
     </row>
     <row r="11" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B11" s="154" t="s">
+      <c r="B11" s="230" t="s">
         <v>12</v>
       </c>
-      <c r="C11" s="155"/>
-      <c r="D11" s="155"/>
-      <c r="E11" s="156"/>
+      <c r="C11" s="231"/>
+      <c r="D11" s="231"/>
+      <c r="E11" s="232"/>
     </row>
     <row r="12" spans="2:8" ht="51" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="133" t="s">
+      <c r="B12" s="221" t="s">
         <v>13</v>
       </c>
-      <c r="C12" s="134"/>
-      <c r="D12" s="135"/>
-      <c r="E12" s="136"/>
+      <c r="C12" s="222"/>
+      <c r="D12" s="223"/>
+      <c r="E12" s="224"/>
       <c r="F12" s="1"/>
       <c r="G12" s="34"/>
     </row>
@@ -4130,84 +3975,84 @@
       <c r="E13" s="75"/>
     </row>
     <row r="14" spans="2:8" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="166" t="s">
+      <c r="B14" s="212" t="s">
         <v>14</v>
       </c>
-      <c r="C14" s="167"/>
-      <c r="D14" s="167"/>
-      <c r="E14" s="168"/>
+      <c r="C14" s="213"/>
+      <c r="D14" s="213"/>
+      <c r="E14" s="214"/>
     </row>
     <row r="15" spans="2:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="169" t="s">
+      <c r="B15" s="215" t="s">
         <v>15</v>
       </c>
-      <c r="C15" s="170"/>
-      <c r="D15" s="170"/>
-      <c r="E15" s="171"/>
+      <c r="C15" s="216"/>
+      <c r="D15" s="216"/>
+      <c r="E15" s="217"/>
     </row>
     <row r="16" spans="2:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="169" t="s">
+      <c r="B16" s="215" t="s">
         <v>16</v>
       </c>
-      <c r="C16" s="170"/>
-      <c r="D16" s="170"/>
-      <c r="E16" s="171"/>
+      <c r="C16" s="216"/>
+      <c r="D16" s="216"/>
+      <c r="E16" s="217"/>
     </row>
     <row r="17" spans="2:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="175" t="s">
+      <c r="B17" s="225" t="s">
         <v>17</v>
       </c>
-      <c r="C17" s="176"/>
-      <c r="D17" s="176"/>
-      <c r="E17" s="177"/>
+      <c r="C17" s="226"/>
+      <c r="D17" s="226"/>
+      <c r="E17" s="227"/>
     </row>
     <row r="18" spans="2:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="169" t="s">
+      <c r="B18" s="215" t="s">
         <v>18</v>
       </c>
-      <c r="C18" s="170"/>
-      <c r="D18" s="170"/>
-      <c r="E18" s="171"/>
+      <c r="C18" s="216"/>
+      <c r="D18" s="216"/>
+      <c r="E18" s="217"/>
     </row>
     <row r="19" spans="2:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="169" t="s">
+      <c r="B19" s="215" t="s">
         <v>19</v>
       </c>
-      <c r="C19" s="170"/>
-      <c r="D19" s="170"/>
-      <c r="E19" s="171"/>
+      <c r="C19" s="216"/>
+      <c r="D19" s="216"/>
+      <c r="E19" s="217"/>
     </row>
     <row r="20" spans="2:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="172" t="s">
+      <c r="B20" s="218" t="s">
         <v>20</v>
       </c>
-      <c r="C20" s="173"/>
-      <c r="D20" s="173"/>
-      <c r="E20" s="174"/>
+      <c r="C20" s="219"/>
+      <c r="D20" s="219"/>
+      <c r="E20" s="220"/>
     </row>
     <row r="21" spans="2:6" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="133" t="s">
+      <c r="B21" s="221" t="s">
         <v>21</v>
       </c>
-      <c r="C21" s="134"/>
-      <c r="D21" s="135"/>
-      <c r="E21" s="136"/>
+      <c r="C21" s="222"/>
+      <c r="D21" s="223"/>
+      <c r="E21" s="224"/>
     </row>
     <row r="22" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="154" t="s">
+      <c r="B22" s="230" t="s">
         <v>22</v>
       </c>
-      <c r="C22" s="155"/>
-      <c r="D22" s="155" t="s">
+      <c r="C22" s="231"/>
+      <c r="D22" s="231" t="s">
         <v>22</v>
       </c>
-      <c r="E22" s="156"/>
+      <c r="E22" s="232"/>
     </row>
     <row r="23" spans="2:6" ht="5.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="157"/>
-      <c r="C23" s="158"/>
-      <c r="D23" s="158"/>
-      <c r="E23" s="159"/>
+      <c r="B23" s="233"/>
+      <c r="C23" s="234"/>
+      <c r="D23" s="234"/>
+      <c r="E23" s="235"/>
     </row>
     <row r="24" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B24" s="68" t="s">
@@ -4216,10 +4061,10 @@
       <c r="C24" s="55" t="s">
         <v>24</v>
       </c>
-      <c r="D24" s="160" t="s">
+      <c r="D24" s="236" t="s">
         <v>25</v>
       </c>
-      <c r="E24" s="161"/>
+      <c r="E24" s="237"/>
       <c r="F24" s="8"/>
     </row>
     <row r="25" spans="2:6" x14ac:dyDescent="0.25">
@@ -4229,8 +4074,8 @@
       <c r="C25" s="56" t="s">
         <v>27</v>
       </c>
-      <c r="D25" s="162"/>
-      <c r="E25" s="163"/>
+      <c r="D25" s="228"/>
+      <c r="E25" s="229"/>
     </row>
     <row r="26" spans="2:6" ht="31.5" x14ac:dyDescent="0.25">
       <c r="B26" s="57" t="s">
@@ -4239,8 +4084,8 @@
       <c r="C26" s="58" t="s">
         <v>29</v>
       </c>
-      <c r="D26" s="162"/>
-      <c r="E26" s="163"/>
+      <c r="D26" s="228"/>
+      <c r="E26" s="229"/>
     </row>
     <row r="27" spans="2:6" ht="45" x14ac:dyDescent="0.25">
       <c r="B27" s="59" t="s">
@@ -4249,8 +4094,8 @@
       <c r="C27" s="56" t="s">
         <v>31</v>
       </c>
-      <c r="D27" s="162"/>
-      <c r="E27" s="163"/>
+      <c r="D27" s="228"/>
+      <c r="E27" s="229"/>
     </row>
     <row r="28" spans="2:6" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B28" s="69" t="s">
@@ -4259,8 +4104,8 @@
       <c r="C28" s="56" t="s">
         <v>33</v>
       </c>
-      <c r="D28" s="162"/>
-      <c r="E28" s="163"/>
+      <c r="D28" s="228"/>
+      <c r="E28" s="229"/>
     </row>
     <row r="29" spans="2:6" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B29" s="69" t="s">
@@ -4269,10 +4114,10 @@
       <c r="C29" s="56" t="s">
         <v>35</v>
       </c>
-      <c r="D29" s="162" t="s">
+      <c r="D29" s="228" t="s">
         <v>36</v>
       </c>
-      <c r="E29" s="163" t="s">
+      <c r="E29" s="229" t="s">
         <v>36</v>
       </c>
     </row>
@@ -4283,10 +4128,10 @@
       <c r="C30" s="56" t="s">
         <v>38</v>
       </c>
-      <c r="D30" s="162" t="s">
+      <c r="D30" s="228" t="s">
         <v>39</v>
       </c>
-      <c r="E30" s="163" t="s">
+      <c r="E30" s="229" t="s">
         <v>39</v>
       </c>
     </row>
@@ -4297,8 +4142,8 @@
       <c r="C31" s="56" t="s">
         <v>41</v>
       </c>
-      <c r="D31" s="162"/>
-      <c r="E31" s="163"/>
+      <c r="D31" s="228"/>
+      <c r="E31" s="229"/>
     </row>
     <row r="32" spans="2:6" ht="65.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B32" s="69" t="s">
@@ -4307,10 +4152,10 @@
       <c r="C32" s="56" t="s">
         <v>43</v>
       </c>
-      <c r="D32" s="162" t="s">
+      <c r="D32" s="228" t="s">
         <v>44</v>
       </c>
-      <c r="E32" s="163" t="s">
+      <c r="E32" s="229" t="s">
         <v>44</v>
       </c>
     </row>
@@ -4321,8 +4166,8 @@
       <c r="C33" s="56" t="s">
         <v>46</v>
       </c>
-      <c r="D33" s="162"/>
-      <c r="E33" s="163"/>
+      <c r="D33" s="228"/>
+      <c r="E33" s="229"/>
     </row>
     <row r="34" spans="2:5" ht="60" x14ac:dyDescent="0.25">
       <c r="B34" s="69" t="s">
@@ -4331,8 +4176,8 @@
       <c r="C34" s="56" t="s">
         <v>48</v>
       </c>
-      <c r="D34" s="162"/>
-      <c r="E34" s="163"/>
+      <c r="D34" s="228"/>
+      <c r="E34" s="229"/>
     </row>
     <row r="35" spans="2:5" ht="60" x14ac:dyDescent="0.25">
       <c r="B35" s="69" t="s">
@@ -4341,8 +4186,8 @@
       <c r="C35" s="56" t="s">
         <v>50</v>
       </c>
-      <c r="D35" s="162"/>
-      <c r="E35" s="163"/>
+      <c r="D35" s="228"/>
+      <c r="E35" s="229"/>
     </row>
     <row r="36" spans="2:5" ht="45" x14ac:dyDescent="0.25">
       <c r="B36" s="69" t="s">
@@ -4351,8 +4196,8 @@
       <c r="C36" s="56" t="s">
         <v>52</v>
       </c>
-      <c r="D36" s="162"/>
-      <c r="E36" s="163"/>
+      <c r="D36" s="228"/>
+      <c r="E36" s="229"/>
     </row>
     <row r="37" spans="2:5" ht="60" x14ac:dyDescent="0.25">
       <c r="B37" s="69" t="s">
@@ -4361,8 +4206,8 @@
       <c r="C37" s="56" t="s">
         <v>54</v>
       </c>
-      <c r="D37" s="162"/>
-      <c r="E37" s="163"/>
+      <c r="D37" s="228"/>
+      <c r="E37" s="229"/>
     </row>
     <row r="38" spans="2:5" ht="60" x14ac:dyDescent="0.25">
       <c r="B38" s="69" t="s">
@@ -4371,8 +4216,8 @@
       <c r="C38" s="56" t="s">
         <v>56</v>
       </c>
-      <c r="D38" s="162"/>
-      <c r="E38" s="163"/>
+      <c r="D38" s="228"/>
+      <c r="E38" s="229"/>
     </row>
     <row r="39" spans="2:5" ht="60" x14ac:dyDescent="0.25">
       <c r="B39" s="69" t="s">
@@ -4381,8 +4226,8 @@
       <c r="C39" s="56" t="s">
         <v>57</v>
       </c>
-      <c r="D39" s="162"/>
-      <c r="E39" s="163"/>
+      <c r="D39" s="228"/>
+      <c r="E39" s="229"/>
     </row>
     <row r="40" spans="2:5" ht="60" x14ac:dyDescent="0.25">
       <c r="B40" s="69" t="s">
@@ -4391,8 +4236,8 @@
       <c r="C40" s="56" t="s">
         <v>59</v>
       </c>
-      <c r="D40" s="162"/>
-      <c r="E40" s="163"/>
+      <c r="D40" s="228"/>
+      <c r="E40" s="229"/>
     </row>
     <row r="41" spans="2:5" ht="60" x14ac:dyDescent="0.25">
       <c r="B41" s="69" t="s">
@@ -4401,8 +4246,8 @@
       <c r="C41" s="56" t="s">
         <v>61</v>
       </c>
-      <c r="D41" s="162"/>
-      <c r="E41" s="163"/>
+      <c r="D41" s="228"/>
+      <c r="E41" s="229"/>
     </row>
     <row r="42" spans="2:5" ht="60" x14ac:dyDescent="0.25">
       <c r="B42" s="69" t="s">
@@ -4411,8 +4256,8 @@
       <c r="C42" s="56" t="s">
         <v>62</v>
       </c>
-      <c r="D42" s="162"/>
-      <c r="E42" s="163"/>
+      <c r="D42" s="228"/>
+      <c r="E42" s="229"/>
     </row>
     <row r="43" spans="2:5" ht="409.5" x14ac:dyDescent="0.25">
       <c r="B43" s="69" t="s">
@@ -4421,10 +4266,10 @@
       <c r="C43" s="60" t="s">
         <v>64</v>
       </c>
-      <c r="D43" s="162" t="s">
+      <c r="D43" s="228" t="s">
         <v>65</v>
       </c>
-      <c r="E43" s="163" t="s">
+      <c r="E43" s="229" t="s">
         <v>65</v>
       </c>
     </row>
@@ -4435,8 +4280,8 @@
       <c r="C44" s="56" t="s">
         <v>67</v>
       </c>
-      <c r="D44" s="162"/>
-      <c r="E44" s="163"/>
+      <c r="D44" s="228"/>
+      <c r="E44" s="229"/>
     </row>
     <row r="45" spans="2:5" ht="30" x14ac:dyDescent="0.25">
       <c r="B45" s="69" t="s">
@@ -4445,8 +4290,8 @@
       <c r="C45" s="56" t="s">
         <v>69</v>
       </c>
-      <c r="D45" s="162"/>
-      <c r="E45" s="163"/>
+      <c r="D45" s="228"/>
+      <c r="E45" s="229"/>
     </row>
     <row r="46" spans="2:5" ht="30" x14ac:dyDescent="0.25">
       <c r="B46" s="69" t="s">
@@ -4455,8 +4300,8 @@
       <c r="C46" s="56" t="s">
         <v>71</v>
       </c>
-      <c r="D46" s="162"/>
-      <c r="E46" s="163"/>
+      <c r="D46" s="228"/>
+      <c r="E46" s="229"/>
     </row>
     <row r="47" spans="2:5" ht="127.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B47" s="69" t="s">
@@ -4465,10 +4310,10 @@
       <c r="C47" s="56" t="s">
         <v>73</v>
       </c>
-      <c r="D47" s="162" t="s">
+      <c r="D47" s="228" t="s">
         <v>74</v>
       </c>
-      <c r="E47" s="163" t="s">
+      <c r="E47" s="229" t="s">
         <v>74</v>
       </c>
     </row>
@@ -4479,8 +4324,8 @@
       <c r="C48" s="56" t="s">
         <v>76</v>
       </c>
-      <c r="D48" s="162"/>
-      <c r="E48" s="163"/>
+      <c r="D48" s="228"/>
+      <c r="E48" s="229"/>
     </row>
     <row r="49" spans="2:5" ht="146.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B49" s="69" t="s">
@@ -4489,10 +4334,10 @@
       <c r="C49" s="56" t="s">
         <v>78</v>
       </c>
-      <c r="D49" s="162" t="s">
+      <c r="D49" s="228" t="s">
         <v>79</v>
       </c>
-      <c r="E49" s="163" t="s">
+      <c r="E49" s="229" t="s">
         <v>79</v>
       </c>
     </row>
@@ -4503,10 +4348,10 @@
       <c r="C50" s="61" t="s">
         <v>81</v>
       </c>
-      <c r="D50" s="162" t="s">
+      <c r="D50" s="228" t="s">
         <v>82</v>
       </c>
-      <c r="E50" s="163" t="s">
+      <c r="E50" s="229" t="s">
         <v>83</v>
       </c>
     </row>
@@ -4517,10 +4362,10 @@
       <c r="C51" s="61" t="s">
         <v>85</v>
       </c>
-      <c r="D51" s="162" t="s">
+      <c r="D51" s="228" t="s">
         <v>86</v>
       </c>
-      <c r="E51" s="163" t="s">
+      <c r="E51" s="229" t="s">
         <v>86</v>
       </c>
     </row>
@@ -4531,8 +4376,8 @@
       <c r="C52" s="56" t="s">
         <v>88</v>
       </c>
-      <c r="D52" s="162"/>
-      <c r="E52" s="163"/>
+      <c r="D52" s="228"/>
+      <c r="E52" s="229"/>
     </row>
     <row r="53" spans="2:5" ht="75" x14ac:dyDescent="0.25">
       <c r="B53" s="69" t="s">
@@ -4541,8 +4386,8 @@
       <c r="C53" s="61" t="s">
         <v>90</v>
       </c>
-      <c r="D53" s="162"/>
-      <c r="E53" s="163"/>
+      <c r="D53" s="228"/>
+      <c r="E53" s="229"/>
     </row>
     <row r="54" spans="2:5" ht="45" x14ac:dyDescent="0.25">
       <c r="B54" s="69" t="s">
@@ -4551,8 +4396,8 @@
       <c r="C54" s="61" t="s">
         <v>92</v>
       </c>
-      <c r="D54" s="162"/>
-      <c r="E54" s="163"/>
+      <c r="D54" s="228"/>
+      <c r="E54" s="229"/>
     </row>
     <row r="55" spans="2:5" ht="75" x14ac:dyDescent="0.25">
       <c r="B55" s="69" t="s">
@@ -4561,8 +4406,8 @@
       <c r="C55" s="56" t="s">
         <v>94</v>
       </c>
-      <c r="D55" s="162"/>
-      <c r="E55" s="163"/>
+      <c r="D55" s="228"/>
+      <c r="E55" s="229"/>
     </row>
     <row r="56" spans="2:5" ht="75" x14ac:dyDescent="0.25">
       <c r="B56" s="70" t="s">
@@ -4571,8 +4416,8 @@
       <c r="C56" s="56" t="s">
         <v>94</v>
       </c>
-      <c r="D56" s="162"/>
-      <c r="E56" s="163"/>
+      <c r="D56" s="228"/>
+      <c r="E56" s="229"/>
     </row>
     <row r="57" spans="2:5" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B57" s="71" t="s">
@@ -4581,10 +4426,10 @@
       <c r="C57" s="72" t="s">
         <v>97</v>
       </c>
-      <c r="D57" s="164" t="s">
+      <c r="D57" s="210" t="s">
         <v>98</v>
       </c>
-      <c r="E57" s="165" t="s">
+      <c r="E57" s="211" t="s">
         <v>98</v>
       </c>
     </row>
@@ -4602,6 +4447,44 @@
     </row>
   </sheetData>
   <mergeCells count="54">
+    <mergeCell ref="B12:E12"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="B4:E4"/>
+    <mergeCell ref="B5:E5"/>
+    <mergeCell ref="B6:E6"/>
+    <mergeCell ref="B7:E7"/>
+    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="B9:E9"/>
+    <mergeCell ref="B10:E10"/>
+    <mergeCell ref="B11:E11"/>
+    <mergeCell ref="B22:E22"/>
+    <mergeCell ref="B23:E23"/>
+    <mergeCell ref="D24:E24"/>
+    <mergeCell ref="D25:E25"/>
+    <mergeCell ref="D26:E26"/>
+    <mergeCell ref="D27:E27"/>
+    <mergeCell ref="D28:E28"/>
+    <mergeCell ref="D29:E29"/>
+    <mergeCell ref="D30:E30"/>
+    <mergeCell ref="D31:E31"/>
+    <mergeCell ref="D32:E32"/>
+    <mergeCell ref="D33:E33"/>
+    <mergeCell ref="D34:E34"/>
+    <mergeCell ref="D35:E35"/>
+    <mergeCell ref="D36:E36"/>
+    <mergeCell ref="D37:E37"/>
+    <mergeCell ref="D38:E38"/>
+    <mergeCell ref="D39:E39"/>
+    <mergeCell ref="D40:E40"/>
+    <mergeCell ref="D41:E41"/>
+    <mergeCell ref="D49:E49"/>
+    <mergeCell ref="D50:E50"/>
+    <mergeCell ref="D51:E51"/>
+    <mergeCell ref="D42:E42"/>
+    <mergeCell ref="D43:E43"/>
+    <mergeCell ref="D44:E44"/>
+    <mergeCell ref="D45:E45"/>
+    <mergeCell ref="D46:E46"/>
     <mergeCell ref="D57:E57"/>
     <mergeCell ref="B14:E14"/>
     <mergeCell ref="B19:E19"/>
@@ -4618,44 +4501,6 @@
     <mergeCell ref="D56:E56"/>
     <mergeCell ref="D47:E47"/>
     <mergeCell ref="D48:E48"/>
-    <mergeCell ref="D49:E49"/>
-    <mergeCell ref="D50:E50"/>
-    <mergeCell ref="D51:E51"/>
-    <mergeCell ref="D42:E42"/>
-    <mergeCell ref="D43:E43"/>
-    <mergeCell ref="D44:E44"/>
-    <mergeCell ref="D45:E45"/>
-    <mergeCell ref="D46:E46"/>
-    <mergeCell ref="D37:E37"/>
-    <mergeCell ref="D38:E38"/>
-    <mergeCell ref="D39:E39"/>
-    <mergeCell ref="D40:E40"/>
-    <mergeCell ref="D41:E41"/>
-    <mergeCell ref="D32:E32"/>
-    <mergeCell ref="D33:E33"/>
-    <mergeCell ref="D34:E34"/>
-    <mergeCell ref="D35:E35"/>
-    <mergeCell ref="D36:E36"/>
-    <mergeCell ref="D27:E27"/>
-    <mergeCell ref="D28:E28"/>
-    <mergeCell ref="D29:E29"/>
-    <mergeCell ref="D30:E30"/>
-    <mergeCell ref="D31:E31"/>
-    <mergeCell ref="B22:E22"/>
-    <mergeCell ref="B23:E23"/>
-    <mergeCell ref="D24:E24"/>
-    <mergeCell ref="D25:E25"/>
-    <mergeCell ref="D26:E26"/>
-    <mergeCell ref="B12:E12"/>
-    <mergeCell ref="B3:E3"/>
-    <mergeCell ref="B4:E4"/>
-    <mergeCell ref="B5:E5"/>
-    <mergeCell ref="B6:E6"/>
-    <mergeCell ref="B7:E7"/>
-    <mergeCell ref="D8:E8"/>
-    <mergeCell ref="B9:E9"/>
-    <mergeCell ref="B10:E10"/>
-    <mergeCell ref="B11:E11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -4745,14 +4590,14 @@
       <c r="Z2" s="9"/>
     </row>
     <row r="3" spans="2:26" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="137" t="s">
+      <c r="B3" s="170" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="138"/>
-      <c r="D3" s="138"/>
-      <c r="E3" s="138"/>
-      <c r="F3" s="138"/>
-      <c r="G3" s="139"/>
+      <c r="C3" s="171"/>
+      <c r="D3" s="171"/>
+      <c r="E3" s="171"/>
+      <c r="F3" s="171"/>
+      <c r="G3" s="172"/>
       <c r="H3" s="10"/>
       <c r="I3" s="9"/>
       <c r="J3" s="9"/>
@@ -4774,14 +4619,14 @@
       <c r="Z3" s="9"/>
     </row>
     <row r="4" spans="2:26" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="140" t="s">
+      <c r="B4" s="173" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="141"/>
-      <c r="D4" s="141"/>
-      <c r="E4" s="141"/>
-      <c r="F4" s="141"/>
-      <c r="G4" s="142"/>
+      <c r="C4" s="174"/>
+      <c r="D4" s="174"/>
+      <c r="E4" s="174"/>
+      <c r="F4" s="174"/>
+      <c r="G4" s="175"/>
       <c r="H4" s="10"/>
       <c r="I4" s="9"/>
       <c r="J4" s="9"/>
@@ -4803,14 +4648,14 @@
       <c r="Z4" s="9"/>
     </row>
     <row r="5" spans="2:26" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="137" t="s">
+      <c r="B5" s="170" t="s">
         <v>99</v>
       </c>
-      <c r="C5" s="138"/>
-      <c r="D5" s="138"/>
-      <c r="E5" s="138"/>
-      <c r="F5" s="138"/>
-      <c r="G5" s="139"/>
+      <c r="C5" s="171"/>
+      <c r="D5" s="171"/>
+      <c r="E5" s="171"/>
+      <c r="F5" s="171"/>
+      <c r="G5" s="172"/>
       <c r="H5" s="10"/>
       <c r="I5" s="10"/>
       <c r="J5" s="9"/>
@@ -4832,14 +4677,14 @@
       <c r="Z5" s="9"/>
     </row>
     <row r="6" spans="2:26" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="140" t="s">
+      <c r="B6" s="173" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="141"/>
-      <c r="D6" s="141"/>
-      <c r="E6" s="141"/>
-      <c r="F6" s="141"/>
-      <c r="G6" s="142"/>
+      <c r="C6" s="174"/>
+      <c r="D6" s="174"/>
+      <c r="E6" s="174"/>
+      <c r="F6" s="174"/>
+      <c r="G6" s="175"/>
       <c r="H6" s="10"/>
       <c r="I6" s="10"/>
       <c r="J6" s="9"/>
@@ -4861,14 +4706,14 @@
       <c r="Z6" s="9"/>
     </row>
     <row r="7" spans="2:26" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="137" t="s">
+      <c r="B7" s="170" t="s">
         <v>6</v>
       </c>
-      <c r="C7" s="138"/>
-      <c r="D7" s="138"/>
-      <c r="E7" s="138"/>
-      <c r="F7" s="138"/>
-      <c r="G7" s="139"/>
+      <c r="C7" s="171"/>
+      <c r="D7" s="171"/>
+      <c r="E7" s="171"/>
+      <c r="F7" s="171"/>
+      <c r="G7" s="172"/>
       <c r="H7" s="9"/>
       <c r="I7" s="9"/>
       <c r="J7" s="9"/>
@@ -4890,18 +4735,24 @@
       <c r="Z7" s="9"/>
     </row>
     <row r="8" spans="2:26" ht="36.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="231" t="s">
+      <c r="B8" s="133" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="232"/>
-      <c r="D8" s="233" t="s">
+      <c r="C8" s="283" t="b">
+        <v>0</v>
+      </c>
+      <c r="D8" s="134" t="s">
         <v>8</v>
       </c>
-      <c r="E8" s="232"/>
-      <c r="F8" s="233" t="s">
+      <c r="E8" s="283" t="b">
+        <v>0</v>
+      </c>
+      <c r="F8" s="134" t="s">
         <v>9</v>
       </c>
-      <c r="G8" s="234"/>
+      <c r="G8" s="284" t="b">
+        <v>0</v>
+      </c>
       <c r="H8" s="9"/>
       <c r="I8" s="9"/>
       <c r="J8" s="9"/>
@@ -4970,12 +4821,12 @@
       </c>
     </row>
     <row r="11" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="235"/>
-      <c r="C11" s="236"/>
-      <c r="D11" s="237"/>
-      <c r="E11" s="238"/>
-      <c r="F11" s="239"/>
-      <c r="G11" s="240"/>
+      <c r="B11" s="135"/>
+      <c r="C11" s="136"/>
+      <c r="D11" s="137"/>
+      <c r="E11" s="138"/>
+      <c r="F11" s="139"/>
+      <c r="G11" s="140"/>
       <c r="H11" s="9"/>
       <c r="I11" s="9"/>
       <c r="J11" s="9"/>
@@ -5052,12 +4903,12 @@
       <c r="Y13" s="18"/>
     </row>
     <row r="14" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="241"/>
-      <c r="C14" s="242"/>
-      <c r="D14" s="243"/>
-      <c r="E14" s="244"/>
-      <c r="F14" s="245"/>
-      <c r="G14" s="246"/>
+      <c r="B14" s="161"/>
+      <c r="C14" s="163"/>
+      <c r="D14" s="162"/>
+      <c r="E14" s="158"/>
+      <c r="F14" s="159"/>
+      <c r="G14" s="160"/>
       <c r="H14" s="20"/>
       <c r="I14" s="20"/>
       <c r="J14" s="20"/>
@@ -5129,12 +4980,12 @@
       <c r="Z16" s="12"/>
     </row>
     <row r="17" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="241"/>
-      <c r="C17" s="243"/>
-      <c r="D17" s="247"/>
-      <c r="E17" s="248"/>
-      <c r="F17" s="249"/>
-      <c r="G17" s="250"/>
+      <c r="B17" s="161"/>
+      <c r="C17" s="162"/>
+      <c r="D17" s="142"/>
+      <c r="E17" s="143"/>
+      <c r="F17" s="176"/>
+      <c r="G17" s="177"/>
       <c r="H17" s="20"/>
       <c r="I17" s="20"/>
       <c r="K17" s="20"/>
@@ -5202,12 +5053,12 @@
       <c r="Z19" s="12"/>
     </row>
     <row r="20" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="241"/>
-      <c r="C20" s="243"/>
-      <c r="D20" s="251"/>
-      <c r="E20" s="252"/>
-      <c r="F20" s="253"/>
-      <c r="G20" s="254"/>
+      <c r="B20" s="161"/>
+      <c r="C20" s="162"/>
+      <c r="D20" s="141"/>
+      <c r="E20" s="144"/>
+      <c r="F20" s="178"/>
+      <c r="G20" s="179"/>
       <c r="H20" s="20"/>
       <c r="L20" s="20"/>
       <c r="M20" s="20"/>
@@ -5249,14 +5100,14 @@
       <c r="Y21" s="15"/>
     </row>
     <row r="22" spans="2:26" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="189" t="s">
+      <c r="B22" s="184" t="s">
         <v>105</v>
       </c>
-      <c r="C22" s="190"/>
-      <c r="D22" s="190"/>
-      <c r="E22" s="190"/>
-      <c r="F22" s="190"/>
-      <c r="G22" s="191"/>
+      <c r="C22" s="185"/>
+      <c r="D22" s="185"/>
+      <c r="E22" s="185"/>
+      <c r="F22" s="185"/>
+      <c r="G22" s="186"/>
       <c r="H22" s="9"/>
       <c r="I22" s="9"/>
       <c r="J22" s="9"/>
@@ -5281,17 +5132,13 @@
       <c r="B23" s="131" t="s">
         <v>106</v>
       </c>
-      <c r="C23" s="181" t="s">
-        <v>189</v>
-      </c>
-      <c r="D23" s="182"/>
+      <c r="C23" s="180"/>
+      <c r="D23" s="181"/>
       <c r="E23" s="132" t="s">
         <v>107</v>
       </c>
-      <c r="F23" s="180" t="s">
-        <v>188</v>
-      </c>
-      <c r="G23" s="178"/>
+      <c r="F23" s="182"/>
+      <c r="G23" s="183"/>
       <c r="H23" s="9"/>
       <c r="I23" s="9"/>
       <c r="J23" s="9"/>
@@ -5405,12 +5252,12 @@
       <c r="C27" s="76" t="s">
         <v>111</v>
       </c>
-      <c r="D27" s="255"/>
+      <c r="D27" s="145"/>
       <c r="E27" s="45"/>
       <c r="F27" s="76" t="s">
         <v>112</v>
       </c>
-      <c r="G27" s="262"/>
+      <c r="G27" s="152"/>
       <c r="H27" s="18"/>
       <c r="I27" s="18"/>
       <c r="J27" s="20"/>
@@ -5433,12 +5280,12 @@
       <c r="C28" s="21" t="s">
         <v>113</v>
       </c>
-      <c r="D28" s="256"/>
+      <c r="D28" s="146"/>
       <c r="E28" s="46"/>
-      <c r="F28" s="192" t="s">
+      <c r="F28" s="164" t="s">
         <v>114</v>
       </c>
-      <c r="G28" s="263"/>
+      <c r="G28" s="165"/>
       <c r="H28" s="18"/>
       <c r="I28" s="18"/>
       <c r="J28" s="20"/>
@@ -5461,12 +5308,12 @@
       <c r="C29" s="21" t="s">
         <v>115</v>
       </c>
-      <c r="D29" s="256"/>
+      <c r="D29" s="146"/>
       <c r="E29" s="41" t="s">
         <v>116</v>
       </c>
-      <c r="F29" s="192"/>
-      <c r="G29" s="263"/>
+      <c r="F29" s="164"/>
+      <c r="G29" s="165"/>
       <c r="H29" s="18"/>
       <c r="I29" s="18"/>
       <c r="J29" s="20"/>
@@ -5491,14 +5338,14 @@
       <c r="C30" s="38" t="s">
         <v>118</v>
       </c>
-      <c r="D30" s="256"/>
+      <c r="D30" s="146"/>
       <c r="E30" s="47" t="s">
         <v>119</v>
       </c>
       <c r="F30" s="21" t="s">
         <v>120</v>
       </c>
-      <c r="G30" s="256"/>
+      <c r="G30" s="146"/>
       <c r="H30" s="18"/>
       <c r="I30" s="18"/>
       <c r="J30" s="20"/>
@@ -5521,12 +5368,12 @@
       <c r="C31" s="21" t="s">
         <v>121</v>
       </c>
-      <c r="D31" s="257"/>
+      <c r="D31" s="147"/>
       <c r="E31" s="40"/>
       <c r="F31" s="83" t="s">
         <v>122</v>
       </c>
-      <c r="G31" s="261"/>
+      <c r="G31" s="151"/>
       <c r="H31" s="18"/>
       <c r="I31" s="18"/>
       <c r="J31" s="19"/>
@@ -5552,12 +5399,12 @@
       <c r="C32" s="21" t="s">
         <v>123</v>
       </c>
-      <c r="D32" s="258"/>
+      <c r="D32" s="148"/>
       <c r="E32" s="44"/>
       <c r="F32" s="82" t="s">
         <v>124</v>
       </c>
-      <c r="G32" s="255"/>
+      <c r="G32" s="145"/>
       <c r="H32" s="18"/>
       <c r="I32" s="18"/>
       <c r="J32" s="19"/>
@@ -5583,14 +5430,14 @@
       <c r="C33" s="81" t="s">
         <v>125</v>
       </c>
-      <c r="D33" s="259"/>
+      <c r="D33" s="149"/>
       <c r="E33" s="79" t="s">
         <v>126</v>
       </c>
       <c r="F33" s="37" t="s">
         <v>127</v>
       </c>
-      <c r="G33" s="264"/>
+      <c r="G33" s="153"/>
       <c r="H33" s="18"/>
       <c r="I33" s="18"/>
       <c r="J33" s="19"/>
@@ -5616,12 +5463,12 @@
       <c r="C34" s="82" t="s">
         <v>128</v>
       </c>
-      <c r="D34" s="260"/>
+      <c r="D34" s="150"/>
       <c r="E34" s="48"/>
       <c r="F34" s="78" t="s">
         <v>129</v>
       </c>
-      <c r="G34" s="261"/>
+      <c r="G34" s="151"/>
       <c r="H34" s="18"/>
       <c r="I34" s="18"/>
       <c r="J34" s="19"/>
@@ -5649,14 +5496,14 @@
       <c r="C35" s="37" t="s">
         <v>131</v>
       </c>
-      <c r="D35" s="256"/>
+      <c r="D35" s="146"/>
       <c r="E35" s="79" t="s">
         <v>132</v>
       </c>
       <c r="F35" s="80" t="s">
         <v>133</v>
       </c>
-      <c r="G35" s="265"/>
+      <c r="G35" s="154"/>
       <c r="H35" s="18"/>
       <c r="I35" s="18"/>
       <c r="J35" s="19"/>
@@ -5682,12 +5529,12 @@
       <c r="C36" s="77" t="s">
         <v>134</v>
       </c>
-      <c r="D36" s="261"/>
+      <c r="D36" s="151"/>
       <c r="E36" s="125"/>
       <c r="F36" s="78" t="s">
         <v>135</v>
       </c>
-      <c r="G36" s="261"/>
+      <c r="G36" s="151"/>
       <c r="H36" s="18"/>
       <c r="I36" s="18"/>
       <c r="J36" s="19"/>
@@ -5802,12 +5649,12 @@
       <c r="Y39" s="18"/>
     </row>
     <row r="40" spans="2:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B40" s="266"/>
-      <c r="C40" s="267"/>
-      <c r="D40" s="268"/>
-      <c r="E40" s="268"/>
-      <c r="F40" s="268"/>
-      <c r="G40" s="269"/>
+      <c r="B40" s="187"/>
+      <c r="C40" s="188"/>
+      <c r="D40" s="191"/>
+      <c r="E40" s="191"/>
+      <c r="F40" s="191"/>
+      <c r="G40" s="193"/>
       <c r="H40" s="20"/>
       <c r="I40" s="18"/>
       <c r="J40" s="18"/>
@@ -5828,12 +5675,12 @@
       <c r="Y40" s="18"/>
     </row>
     <row r="41" spans="2:26" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B41" s="270"/>
-      <c r="C41" s="271"/>
-      <c r="D41" s="272"/>
-      <c r="E41" s="272"/>
-      <c r="F41" s="272"/>
-      <c r="G41" s="273"/>
+      <c r="B41" s="189"/>
+      <c r="C41" s="190"/>
+      <c r="D41" s="192"/>
+      <c r="E41" s="192"/>
+      <c r="F41" s="192"/>
+      <c r="G41" s="194"/>
       <c r="H41" s="20"/>
       <c r="I41" s="18"/>
       <c r="J41" s="18"/>
@@ -5854,12 +5701,12 @@
       <c r="Y41" s="18"/>
     </row>
     <row r="42" spans="2:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B42" s="266"/>
-      <c r="C42" s="267"/>
-      <c r="D42" s="268"/>
-      <c r="E42" s="268"/>
-      <c r="F42" s="268"/>
-      <c r="G42" s="269"/>
+      <c r="B42" s="187"/>
+      <c r="C42" s="188"/>
+      <c r="D42" s="191"/>
+      <c r="E42" s="191"/>
+      <c r="F42" s="191"/>
+      <c r="G42" s="193"/>
       <c r="H42" s="20"/>
       <c r="I42" s="18"/>
       <c r="J42" s="18"/>
@@ -5880,12 +5727,12 @@
       <c r="Y42" s="18"/>
     </row>
     <row r="43" spans="2:26" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B43" s="270"/>
-      <c r="C43" s="271"/>
-      <c r="D43" s="272"/>
-      <c r="E43" s="272"/>
-      <c r="F43" s="272"/>
-      <c r="G43" s="273"/>
+      <c r="B43" s="189"/>
+      <c r="C43" s="190"/>
+      <c r="D43" s="192"/>
+      <c r="E43" s="192"/>
+      <c r="F43" s="192"/>
+      <c r="G43" s="194"/>
       <c r="H43" s="20"/>
       <c r="I43" s="18"/>
       <c r="J43" s="18"/>
@@ -5906,12 +5753,12 @@
       <c r="Y43" s="18"/>
     </row>
     <row r="44" spans="2:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B44" s="266"/>
-      <c r="C44" s="267"/>
-      <c r="D44" s="268"/>
-      <c r="E44" s="268"/>
-      <c r="F44" s="268"/>
-      <c r="G44" s="269"/>
+      <c r="B44" s="187"/>
+      <c r="C44" s="188"/>
+      <c r="D44" s="191"/>
+      <c r="E44" s="191"/>
+      <c r="F44" s="191"/>
+      <c r="G44" s="193"/>
       <c r="H44" s="20"/>
       <c r="I44" s="18"/>
       <c r="J44" s="18"/>
@@ -5932,12 +5779,12 @@
       <c r="Y44" s="18"/>
     </row>
     <row r="45" spans="2:26" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B45" s="270"/>
-      <c r="C45" s="271"/>
-      <c r="D45" s="272"/>
-      <c r="E45" s="272"/>
-      <c r="F45" s="272"/>
-      <c r="G45" s="273"/>
+      <c r="B45" s="189"/>
+      <c r="C45" s="190"/>
+      <c r="D45" s="192"/>
+      <c r="E45" s="192"/>
+      <c r="F45" s="192"/>
+      <c r="G45" s="194"/>
       <c r="H45" s="20"/>
       <c r="I45" s="18"/>
       <c r="J45" s="18"/>
@@ -5958,12 +5805,12 @@
       <c r="Y45" s="18"/>
     </row>
     <row r="46" spans="2:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B46" s="266"/>
-      <c r="C46" s="267"/>
-      <c r="D46" s="268"/>
-      <c r="E46" s="268"/>
-      <c r="F46" s="268"/>
-      <c r="G46" s="269"/>
+      <c r="B46" s="187"/>
+      <c r="C46" s="188"/>
+      <c r="D46" s="191"/>
+      <c r="E46" s="191"/>
+      <c r="F46" s="191"/>
+      <c r="G46" s="193"/>
       <c r="H46" s="20"/>
       <c r="I46" s="18"/>
       <c r="J46" s="18"/>
@@ -5984,12 +5831,12 @@
       <c r="Y46" s="18"/>
     </row>
     <row r="47" spans="2:26" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B47" s="270"/>
-      <c r="C47" s="271"/>
-      <c r="D47" s="272"/>
-      <c r="E47" s="272"/>
-      <c r="F47" s="272"/>
-      <c r="G47" s="273"/>
+      <c r="B47" s="189"/>
+      <c r="C47" s="190"/>
+      <c r="D47" s="192"/>
+      <c r="E47" s="192"/>
+      <c r="F47" s="192"/>
+      <c r="G47" s="194"/>
       <c r="H47" s="20"/>
       <c r="I47" s="18"/>
       <c r="J47" s="18"/>
@@ -6010,12 +5857,12 @@
       <c r="Y47" s="18"/>
     </row>
     <row r="48" spans="2:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B48" s="266"/>
-      <c r="C48" s="267"/>
-      <c r="D48" s="268"/>
-      <c r="E48" s="268"/>
-      <c r="F48" s="268"/>
-      <c r="G48" s="269"/>
+      <c r="B48" s="187"/>
+      <c r="C48" s="188"/>
+      <c r="D48" s="191"/>
+      <c r="E48" s="191"/>
+      <c r="F48" s="191"/>
+      <c r="G48" s="193"/>
       <c r="H48" s="20"/>
       <c r="I48" s="18"/>
       <c r="J48" s="18"/>
@@ -6036,12 +5883,12 @@
       <c r="Y48" s="18"/>
     </row>
     <row r="49" spans="2:26" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B49" s="270"/>
-      <c r="C49" s="271"/>
-      <c r="D49" s="272"/>
-      <c r="E49" s="272"/>
-      <c r="F49" s="272"/>
-      <c r="G49" s="273"/>
+      <c r="B49" s="189"/>
+      <c r="C49" s="190"/>
+      <c r="D49" s="192"/>
+      <c r="E49" s="192"/>
+      <c r="F49" s="192"/>
+      <c r="G49" s="194"/>
       <c r="H49" s="20"/>
       <c r="I49" s="18"/>
       <c r="J49" s="18"/>
@@ -6062,12 +5909,12 @@
       <c r="Y49" s="18"/>
     </row>
     <row r="50" spans="2:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B50" s="266"/>
-      <c r="C50" s="267"/>
-      <c r="D50" s="268"/>
-      <c r="E50" s="268"/>
-      <c r="F50" s="268"/>
-      <c r="G50" s="269"/>
+      <c r="B50" s="187"/>
+      <c r="C50" s="188"/>
+      <c r="D50" s="191"/>
+      <c r="E50" s="191"/>
+      <c r="F50" s="191"/>
+      <c r="G50" s="193"/>
       <c r="H50" s="20"/>
       <c r="I50" s="18"/>
       <c r="J50" s="18"/>
@@ -6088,12 +5935,12 @@
       <c r="Y50" s="18"/>
     </row>
     <row r="51" spans="2:26" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B51" s="270"/>
-      <c r="C51" s="271"/>
-      <c r="D51" s="272"/>
-      <c r="E51" s="272"/>
-      <c r="F51" s="272"/>
-      <c r="G51" s="273"/>
+      <c r="B51" s="189"/>
+      <c r="C51" s="190"/>
+      <c r="D51" s="192"/>
+      <c r="E51" s="192"/>
+      <c r="F51" s="192"/>
+      <c r="G51" s="194"/>
       <c r="H51" s="20"/>
       <c r="I51" s="18"/>
       <c r="J51" s="18"/>
@@ -6114,12 +5961,12 @@
       <c r="Y51" s="18"/>
     </row>
     <row r="52" spans="2:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B52" s="266"/>
-      <c r="C52" s="267"/>
-      <c r="D52" s="268"/>
-      <c r="E52" s="268"/>
-      <c r="F52" s="268"/>
-      <c r="G52" s="269"/>
+      <c r="B52" s="187"/>
+      <c r="C52" s="188"/>
+      <c r="D52" s="191"/>
+      <c r="E52" s="191"/>
+      <c r="F52" s="191"/>
+      <c r="G52" s="193"/>
       <c r="H52" s="20"/>
       <c r="I52" s="18"/>
       <c r="J52" s="18"/>
@@ -6140,12 +5987,12 @@
       <c r="Y52" s="18"/>
     </row>
     <row r="53" spans="2:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B53" s="270"/>
-      <c r="C53" s="271"/>
-      <c r="D53" s="272"/>
-      <c r="E53" s="272"/>
-      <c r="F53" s="272"/>
-      <c r="G53" s="273"/>
+      <c r="B53" s="189"/>
+      <c r="C53" s="190"/>
+      <c r="D53" s="192"/>
+      <c r="E53" s="192"/>
+      <c r="F53" s="192"/>
+      <c r="G53" s="194"/>
       <c r="H53" s="20"/>
       <c r="I53" s="18"/>
       <c r="J53" s="18"/>
@@ -6220,14 +6067,14 @@
       <c r="Y55" s="22"/>
     </row>
     <row r="56" spans="2:26" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B56" s="194" t="s">
+      <c r="B56" s="167" t="s">
         <v>147</v>
       </c>
-      <c r="C56" s="195"/>
-      <c r="D56" s="195"/>
-      <c r="E56" s="195"/>
-      <c r="F56" s="195"/>
-      <c r="G56" s="196"/>
+      <c r="C56" s="168"/>
+      <c r="D56" s="168"/>
+      <c r="E56" s="168"/>
+      <c r="F56" s="168"/>
+      <c r="G56" s="169"/>
       <c r="H56" s="22"/>
       <c r="I56" s="22"/>
       <c r="J56" s="22"/>
@@ -6369,11 +6216,11 @@
       <c r="D61" s="104" t="s">
         <v>84</v>
       </c>
-      <c r="E61" s="276"/>
+      <c r="E61" s="195"/>
       <c r="F61" s="104" t="s">
         <v>152</v>
       </c>
-      <c r="G61" s="276"/>
+      <c r="G61" s="195"/>
       <c r="H61" s="18"/>
       <c r="I61" s="18"/>
       <c r="J61" s="18"/>
@@ -6395,12 +6242,12 @@
       <c r="Z61" s="18"/>
     </row>
     <row r="62" spans="2:26" ht="32.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B62" s="274"/>
-      <c r="C62" s="275"/>
+      <c r="B62" s="155"/>
+      <c r="C62" s="156"/>
       <c r="D62" s="101"/>
-      <c r="E62" s="277"/>
+      <c r="E62" s="196"/>
       <c r="F62" s="101"/>
-      <c r="G62" s="277"/>
+      <c r="G62" s="196"/>
       <c r="H62" s="18"/>
       <c r="I62" s="18"/>
       <c r="J62" s="18"/>
@@ -6477,9 +6324,9 @@
       <c r="Z64" s="18"/>
     </row>
     <row r="65" spans="2:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B65" s="283"/>
-      <c r="C65" s="283"/>
-      <c r="D65" s="283"/>
+      <c r="B65" s="197"/>
+      <c r="C65" s="197"/>
+      <c r="D65" s="197"/>
       <c r="E65" s="17"/>
       <c r="F65" s="17"/>
       <c r="G65" s="17"/>
@@ -6504,9 +6351,9 @@
       <c r="Z65" s="18"/>
     </row>
     <row r="66" spans="2:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B66" s="283"/>
-      <c r="C66" s="283"/>
-      <c r="D66" s="283"/>
+      <c r="B66" s="197"/>
+      <c r="C66" s="197"/>
+      <c r="D66" s="197"/>
       <c r="E66" s="17"/>
       <c r="F66" s="17"/>
       <c r="G66" s="17"/>
@@ -6531,10 +6378,10 @@
       <c r="Z66" s="18"/>
     </row>
     <row r="67" spans="2:26" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B67" s="284"/>
-      <c r="C67" s="284"/>
-      <c r="D67" s="284"/>
-      <c r="F67" s="278"/>
+      <c r="B67" s="198"/>
+      <c r="C67" s="198"/>
+      <c r="D67" s="198"/>
+      <c r="F67" s="157"/>
       <c r="G67" s="18"/>
       <c r="H67" s="18"/>
       <c r="I67" s="18"/>
@@ -6557,11 +6404,11 @@
       <c r="Z67" s="18"/>
     </row>
     <row r="68" spans="2:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B68" s="193" t="s">
+      <c r="B68" s="166" t="s">
         <v>89</v>
       </c>
-      <c r="C68" s="193"/>
-      <c r="D68" s="193"/>
+      <c r="C68" s="166"/>
+      <c r="D68" s="166"/>
       <c r="F68" s="19" t="s">
         <v>91</v>
       </c>
@@ -6587,11 +6434,11 @@
       <c r="Z68" s="18"/>
     </row>
     <row r="69" spans="2:26" x14ac:dyDescent="0.25">
-      <c r="B69" s="281"/>
-      <c r="C69" s="281"/>
-      <c r="D69" s="281"/>
-      <c r="F69" s="279"/>
-      <c r="G69" s="279"/>
+      <c r="B69" s="199"/>
+      <c r="C69" s="199"/>
+      <c r="D69" s="199"/>
+      <c r="F69" s="202"/>
+      <c r="G69" s="202"/>
       <c r="H69" s="18"/>
       <c r="I69" s="18"/>
       <c r="J69" s="18"/>
@@ -6613,11 +6460,11 @@
       <c r="Z69" s="18"/>
     </row>
     <row r="70" spans="2:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B70" s="281"/>
-      <c r="C70" s="281"/>
-      <c r="D70" s="281"/>
-      <c r="F70" s="279"/>
-      <c r="G70" s="279"/>
+      <c r="B70" s="199"/>
+      <c r="C70" s="199"/>
+      <c r="D70" s="199"/>
+      <c r="F70" s="202"/>
+      <c r="G70" s="202"/>
       <c r="H70" s="18"/>
       <c r="I70" s="18"/>
       <c r="J70" s="18"/>
@@ -6639,11 +6486,11 @@
       <c r="Z70" s="18"/>
     </row>
     <row r="71" spans="2:26" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B71" s="282"/>
-      <c r="C71" s="282"/>
-      <c r="D71" s="282"/>
-      <c r="F71" s="280"/>
-      <c r="G71" s="280"/>
+      <c r="B71" s="200"/>
+      <c r="C71" s="200"/>
+      <c r="D71" s="200"/>
+      <c r="F71" s="203"/>
+      <c r="G71" s="203"/>
       <c r="H71" s="18"/>
       <c r="I71" s="18"/>
       <c r="J71" s="18"/>
@@ -6665,15 +6512,15 @@
       <c r="Z71" s="18"/>
     </row>
     <row r="72" spans="2:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B72" s="179" t="s">
+      <c r="B72" s="201" t="s">
         <v>93</v>
       </c>
-      <c r="C72" s="179"/>
-      <c r="D72" s="179"/>
-      <c r="F72" s="193" t="s">
+      <c r="C72" s="201"/>
+      <c r="D72" s="201"/>
+      <c r="F72" s="166" t="s">
         <v>154</v>
       </c>
-      <c r="G72" s="193"/>
+      <c r="G72" s="166"/>
       <c r="H72" s="18"/>
       <c r="I72" s="18"/>
       <c r="J72" s="18"/>
@@ -6751,14 +6598,14 @@
       <c r="Z74" s="18"/>
     </row>
     <row r="75" spans="2:26" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B75" s="183" t="s">
+      <c r="B75" s="204" t="s">
         <v>156</v>
       </c>
-      <c r="C75" s="184"/>
-      <c r="D75" s="184"/>
-      <c r="E75" s="184"/>
-      <c r="F75" s="184"/>
-      <c r="G75" s="185"/>
+      <c r="C75" s="205"/>
+      <c r="D75" s="205"/>
+      <c r="E75" s="205"/>
+      <c r="F75" s="205"/>
+      <c r="G75" s="206"/>
       <c r="H75" s="10"/>
       <c r="I75" s="9"/>
       <c r="J75" s="9"/>
@@ -6780,14 +6627,14 @@
       <c r="Z75" s="9"/>
     </row>
     <row r="76" spans="2:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B76" s="186" t="s">
+      <c r="B76" s="207" t="s">
         <v>157</v>
       </c>
-      <c r="C76" s="187"/>
-      <c r="D76" s="187"/>
-      <c r="E76" s="187"/>
-      <c r="F76" s="187"/>
-      <c r="G76" s="188"/>
+      <c r="C76" s="208"/>
+      <c r="D76" s="208"/>
+      <c r="E76" s="208"/>
+      <c r="F76" s="208"/>
+      <c r="G76" s="209"/>
       <c r="H76" s="10"/>
       <c r="I76" s="35"/>
       <c r="J76" s="9"/>
@@ -6809,14 +6656,14 @@
       <c r="Z76" s="9"/>
     </row>
     <row r="77" spans="2:26" s="10" customFormat="1" ht="63" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B77" s="241" t="s">
-        <v>190</v>
-      </c>
-      <c r="C77" s="242"/>
-      <c r="D77" s="242"/>
-      <c r="E77" s="242"/>
-      <c r="F77" s="242"/>
-      <c r="G77" s="254"/>
+      <c r="B77" s="161" t="s">
+        <v>188</v>
+      </c>
+      <c r="C77" s="163"/>
+      <c r="D77" s="163"/>
+      <c r="E77" s="163"/>
+      <c r="F77" s="163"/>
+      <c r="G77" s="179"/>
     </row>
     <row r="78" spans="2:26" x14ac:dyDescent="0.25">
       <c r="H78" s="10"/>
@@ -6841,13 +6688,49 @@
     </row>
     <row r="79" spans="2:26" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="h74j79N81pE9k28tS1hEwUnpWaq69PEBI419soBWgitnMz2Gg7k5LLyOyhb9pf6OY+cnVsCY9sIu412olw5/uQ==" saltValue="lqfSFUpefv9aiStoeeQPzg==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="63">
-    <mergeCell ref="E14:G14"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="B14:D14"/>
-    <mergeCell ref="F28:F29"/>
-    <mergeCell ref="G28:G29"/>
+    <mergeCell ref="B77:G77"/>
+    <mergeCell ref="E61:E62"/>
+    <mergeCell ref="G61:G62"/>
+    <mergeCell ref="B65:D67"/>
+    <mergeCell ref="B69:D71"/>
+    <mergeCell ref="B72:D72"/>
+    <mergeCell ref="F69:G71"/>
+    <mergeCell ref="B75:G75"/>
+    <mergeCell ref="B76:G76"/>
+    <mergeCell ref="B52:C53"/>
+    <mergeCell ref="D52:D53"/>
+    <mergeCell ref="E52:E53"/>
+    <mergeCell ref="F52:F53"/>
+    <mergeCell ref="G52:G53"/>
+    <mergeCell ref="B50:C51"/>
+    <mergeCell ref="D50:D51"/>
+    <mergeCell ref="E50:E51"/>
+    <mergeCell ref="F50:F51"/>
+    <mergeCell ref="G50:G51"/>
+    <mergeCell ref="B48:C49"/>
+    <mergeCell ref="D48:D49"/>
+    <mergeCell ref="E48:E49"/>
+    <mergeCell ref="F48:F49"/>
+    <mergeCell ref="G48:G49"/>
+    <mergeCell ref="B46:C47"/>
+    <mergeCell ref="D46:D47"/>
+    <mergeCell ref="E46:E47"/>
+    <mergeCell ref="F46:F47"/>
+    <mergeCell ref="G46:G47"/>
+    <mergeCell ref="B44:C45"/>
+    <mergeCell ref="D44:D45"/>
+    <mergeCell ref="E44:E45"/>
+    <mergeCell ref="F44:F45"/>
+    <mergeCell ref="G44:G45"/>
+    <mergeCell ref="E40:E41"/>
+    <mergeCell ref="F40:F41"/>
+    <mergeCell ref="G40:G41"/>
+    <mergeCell ref="B42:C43"/>
+    <mergeCell ref="D42:D43"/>
+    <mergeCell ref="E42:E43"/>
+    <mergeCell ref="F42:F43"/>
+    <mergeCell ref="G42:G43"/>
     <mergeCell ref="F72:G72"/>
     <mergeCell ref="B68:D68"/>
     <mergeCell ref="B56:G56"/>
@@ -6864,51 +6747,14 @@
     <mergeCell ref="B22:G22"/>
     <mergeCell ref="B40:C41"/>
     <mergeCell ref="D40:D41"/>
-    <mergeCell ref="E40:E41"/>
-    <mergeCell ref="F40:F41"/>
-    <mergeCell ref="G40:G41"/>
-    <mergeCell ref="B42:C43"/>
-    <mergeCell ref="D42:D43"/>
-    <mergeCell ref="E42:E43"/>
-    <mergeCell ref="F42:F43"/>
-    <mergeCell ref="G42:G43"/>
-    <mergeCell ref="B44:C45"/>
-    <mergeCell ref="D44:D45"/>
-    <mergeCell ref="E44:E45"/>
-    <mergeCell ref="F44:F45"/>
-    <mergeCell ref="G44:G45"/>
-    <mergeCell ref="B46:C47"/>
-    <mergeCell ref="D46:D47"/>
-    <mergeCell ref="E46:E47"/>
-    <mergeCell ref="F46:F47"/>
-    <mergeCell ref="G46:G47"/>
-    <mergeCell ref="B48:C49"/>
-    <mergeCell ref="D48:D49"/>
-    <mergeCell ref="E48:E49"/>
-    <mergeCell ref="F48:F49"/>
-    <mergeCell ref="G48:G49"/>
-    <mergeCell ref="B50:C51"/>
-    <mergeCell ref="D50:D51"/>
-    <mergeCell ref="E50:E51"/>
-    <mergeCell ref="F50:F51"/>
-    <mergeCell ref="G50:G51"/>
-    <mergeCell ref="B52:C53"/>
-    <mergeCell ref="D52:D53"/>
-    <mergeCell ref="E52:E53"/>
-    <mergeCell ref="F52:F53"/>
-    <mergeCell ref="G52:G53"/>
-    <mergeCell ref="B77:G77"/>
-    <mergeCell ref="E61:E62"/>
-    <mergeCell ref="G61:G62"/>
-    <mergeCell ref="B65:D67"/>
-    <mergeCell ref="B69:D71"/>
-    <mergeCell ref="B72:D72"/>
-    <mergeCell ref="F69:G71"/>
-    <mergeCell ref="B75:G75"/>
-    <mergeCell ref="B76:G76"/>
+    <mergeCell ref="E14:G14"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="B14:D14"/>
+    <mergeCell ref="F28:F29"/>
+    <mergeCell ref="G28:G29"/>
   </mergeCells>
-  <conditionalFormatting sqref="B11:G11 B14:G14 B17:G17 B20:G20 C23:D23 F23:G23 B40:G53 E61 G61 B62:C62 B65:D71 F67 F69:G72 B77:G77">
-    <cfRule type="containsBlanks" dxfId="0" priority="1">
+  <conditionalFormatting sqref="B11:G11 B14:G14 B17:G17 B20:G20 B40:G53 E61 G61 B62:C62 B65:D71 F67 F69:G72 B77:G77">
+    <cfRule type="containsBlanks" dxfId="1" priority="1">
       <formula>LEN(TRIM(B11))=0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -7040,124 +6886,124 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:24" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A1" s="197" t="s">
+      <c r="A1" s="275" t="s">
         <v>158</v>
       </c>
-      <c r="B1" s="197"/>
-      <c r="C1" s="197"/>
-      <c r="D1" s="197"/>
-      <c r="E1" s="197"/>
-      <c r="F1" s="197"/>
-      <c r="G1" s="197"/>
-      <c r="H1" s="197"/>
-      <c r="I1" s="197"/>
-      <c r="J1" s="197"/>
-      <c r="K1" s="197"/>
-      <c r="L1" s="197"/>
-      <c r="M1" s="197"/>
-      <c r="N1" s="197"/>
-      <c r="O1" s="197"/>
-      <c r="P1" s="197"/>
-      <c r="Q1" s="197"/>
-      <c r="R1" s="197"/>
-      <c r="S1" s="197"/>
-      <c r="T1" s="197"/>
-      <c r="U1" s="197" t="s">
+      <c r="B1" s="275"/>
+      <c r="C1" s="275"/>
+      <c r="D1" s="275"/>
+      <c r="E1" s="275"/>
+      <c r="F1" s="275"/>
+      <c r="G1" s="275"/>
+      <c r="H1" s="275"/>
+      <c r="I1" s="275"/>
+      <c r="J1" s="275"/>
+      <c r="K1" s="275"/>
+      <c r="L1" s="275"/>
+      <c r="M1" s="275"/>
+      <c r="N1" s="275"/>
+      <c r="O1" s="275"/>
+      <c r="P1" s="275"/>
+      <c r="Q1" s="275"/>
+      <c r="R1" s="275"/>
+      <c r="S1" s="275"/>
+      <c r="T1" s="275"/>
+      <c r="U1" s="275" t="s">
         <v>159</v>
       </c>
-      <c r="V1" s="197"/>
-      <c r="W1" s="197"/>
-      <c r="X1" s="197"/>
+      <c r="V1" s="275"/>
+      <c r="W1" s="275"/>
+      <c r="X1" s="275"/>
     </row>
     <row r="2" spans="1:24" ht="33" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="197"/>
-      <c r="B2" s="197"/>
-      <c r="C2" s="197"/>
-      <c r="D2" s="197"/>
-      <c r="E2" s="197"/>
-      <c r="F2" s="197"/>
-      <c r="G2" s="197"/>
-      <c r="H2" s="197"/>
-      <c r="I2" s="197"/>
-      <c r="J2" s="197"/>
-      <c r="K2" s="197"/>
-      <c r="L2" s="197"/>
-      <c r="M2" s="197"/>
-      <c r="N2" s="197"/>
-      <c r="O2" s="197"/>
-      <c r="P2" s="197"/>
-      <c r="Q2" s="197"/>
-      <c r="R2" s="197"/>
-      <c r="S2" s="197"/>
-      <c r="T2" s="197"/>
-      <c r="U2" s="205" t="s">
+      <c r="A2" s="275"/>
+      <c r="B2" s="275"/>
+      <c r="C2" s="275"/>
+      <c r="D2" s="275"/>
+      <c r="E2" s="275"/>
+      <c r="F2" s="275"/>
+      <c r="G2" s="275"/>
+      <c r="H2" s="275"/>
+      <c r="I2" s="275"/>
+      <c r="J2" s="275"/>
+      <c r="K2" s="275"/>
+      <c r="L2" s="275"/>
+      <c r="M2" s="275"/>
+      <c r="N2" s="275"/>
+      <c r="O2" s="275"/>
+      <c r="P2" s="275"/>
+      <c r="Q2" s="275"/>
+      <c r="R2" s="275"/>
+      <c r="S2" s="275"/>
+      <c r="T2" s="275"/>
+      <c r="U2" s="255" t="s">
         <v>160</v>
       </c>
-      <c r="V2" s="205"/>
-      <c r="W2" s="205"/>
-      <c r="X2" s="205"/>
+      <c r="V2" s="255"/>
+      <c r="W2" s="255"/>
+      <c r="X2" s="255"/>
     </row>
     <row r="3" spans="1:24" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="U3" s="206"/>
-      <c r="V3" s="206"/>
-      <c r="W3" s="206"/>
-      <c r="X3" s="206"/>
+      <c r="U3" s="282"/>
+      <c r="V3" s="282"/>
+      <c r="W3" s="282"/>
+      <c r="X3" s="282"/>
     </row>
     <row r="4" spans="1:24" s="2" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="202" t="s">
+      <c r="A4" s="279" t="s">
         <v>161</v>
       </c>
-      <c r="B4" s="203"/>
-      <c r="C4" s="203"/>
-      <c r="D4" s="203"/>
-      <c r="E4" s="203"/>
-      <c r="F4" s="203"/>
-      <c r="G4" s="203"/>
-      <c r="H4" s="203"/>
-      <c r="I4" s="203"/>
-      <c r="J4" s="203"/>
-      <c r="K4" s="203"/>
-      <c r="L4" s="203"/>
-      <c r="M4" s="204"/>
-      <c r="N4" s="202" t="s">
+      <c r="B4" s="280"/>
+      <c r="C4" s="280"/>
+      <c r="D4" s="280"/>
+      <c r="E4" s="280"/>
+      <c r="F4" s="280"/>
+      <c r="G4" s="280"/>
+      <c r="H4" s="280"/>
+      <c r="I4" s="280"/>
+      <c r="J4" s="280"/>
+      <c r="K4" s="280"/>
+      <c r="L4" s="280"/>
+      <c r="M4" s="281"/>
+      <c r="N4" s="279" t="s">
         <v>162</v>
       </c>
-      <c r="O4" s="203"/>
-      <c r="P4" s="203"/>
-      <c r="Q4" s="203"/>
-      <c r="R4" s="203"/>
-      <c r="S4" s="203"/>
-      <c r="T4" s="203"/>
-      <c r="U4" s="203"/>
-      <c r="V4" s="203"/>
-      <c r="W4" s="203"/>
-      <c r="X4" s="204"/>
+      <c r="O4" s="280"/>
+      <c r="P4" s="280"/>
+      <c r="Q4" s="280"/>
+      <c r="R4" s="280"/>
+      <c r="S4" s="280"/>
+      <c r="T4" s="280"/>
+      <c r="U4" s="280"/>
+      <c r="V4" s="280"/>
+      <c r="W4" s="280"/>
+      <c r="X4" s="281"/>
     </row>
     <row r="5" spans="1:24" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="199"/>
-      <c r="B5" s="200"/>
-      <c r="C5" s="200"/>
-      <c r="D5" s="200"/>
-      <c r="E5" s="200"/>
-      <c r="F5" s="200"/>
-      <c r="G5" s="200"/>
-      <c r="H5" s="200"/>
-      <c r="I5" s="200"/>
-      <c r="J5" s="200"/>
-      <c r="K5" s="200"/>
-      <c r="L5" s="200"/>
-      <c r="M5" s="201"/>
-      <c r="N5" s="199"/>
-      <c r="O5" s="200"/>
-      <c r="P5" s="200"/>
-      <c r="Q5" s="200"/>
-      <c r="R5" s="200"/>
-      <c r="S5" s="200"/>
-      <c r="T5" s="200"/>
-      <c r="U5" s="200"/>
-      <c r="V5" s="200"/>
-      <c r="W5" s="200"/>
-      <c r="X5" s="201"/>
+      <c r="A5" s="276"/>
+      <c r="B5" s="277"/>
+      <c r="C5" s="277"/>
+      <c r="D5" s="277"/>
+      <c r="E5" s="277"/>
+      <c r="F5" s="277"/>
+      <c r="G5" s="277"/>
+      <c r="H5" s="277"/>
+      <c r="I5" s="277"/>
+      <c r="J5" s="277"/>
+      <c r="K5" s="277"/>
+      <c r="L5" s="277"/>
+      <c r="M5" s="278"/>
+      <c r="N5" s="276"/>
+      <c r="O5" s="277"/>
+      <c r="P5" s="277"/>
+      <c r="Q5" s="277"/>
+      <c r="R5" s="277"/>
+      <c r="S5" s="277"/>
+      <c r="T5" s="277"/>
+      <c r="U5" s="277"/>
+      <c r="V5" s="277"/>
+      <c r="W5" s="277"/>
+      <c r="X5" s="278"/>
     </row>
     <row r="6" spans="1:24" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3"/>
@@ -7186,66 +7032,66 @@
       <c r="X6" s="3"/>
     </row>
     <row r="7" spans="1:24" s="2" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="198" t="s">
+      <c r="A7" s="253" t="s">
         <v>163</v>
       </c>
-      <c r="B7" s="198"/>
-      <c r="C7" s="198"/>
-      <c r="D7" s="198"/>
-      <c r="E7" s="198"/>
-      <c r="F7" s="198"/>
-      <c r="G7" s="198"/>
-      <c r="H7" s="198"/>
-      <c r="I7" s="198"/>
-      <c r="J7" s="198" t="s">
+      <c r="B7" s="253"/>
+      <c r="C7" s="253"/>
+      <c r="D7" s="253"/>
+      <c r="E7" s="253"/>
+      <c r="F7" s="253"/>
+      <c r="G7" s="253"/>
+      <c r="H7" s="253"/>
+      <c r="I7" s="253"/>
+      <c r="J7" s="253" t="s">
         <v>32</v>
       </c>
-      <c r="K7" s="198"/>
-      <c r="L7" s="198"/>
-      <c r="M7" s="198"/>
-      <c r="N7" s="198"/>
-      <c r="O7" s="198"/>
-      <c r="P7" s="198" t="s">
+      <c r="K7" s="253"/>
+      <c r="L7" s="253"/>
+      <c r="M7" s="253"/>
+      <c r="N7" s="253"/>
+      <c r="O7" s="253"/>
+      <c r="P7" s="253" t="s">
         <v>58</v>
       </c>
-      <c r="Q7" s="198"/>
-      <c r="R7" s="198"/>
-      <c r="S7" s="198"/>
-      <c r="T7" s="198"/>
-      <c r="U7" s="198"/>
-      <c r="V7" s="198"/>
-      <c r="W7" s="198"/>
-      <c r="X7" s="198"/>
+      <c r="Q7" s="253"/>
+      <c r="R7" s="253"/>
+      <c r="S7" s="253"/>
+      <c r="T7" s="253"/>
+      <c r="U7" s="253"/>
+      <c r="V7" s="253"/>
+      <c r="W7" s="253"/>
+      <c r="X7" s="253"/>
     </row>
     <row r="8" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="207"/>
-      <c r="B8" s="207"/>
-      <c r="C8" s="207"/>
-      <c r="D8" s="207"/>
-      <c r="E8" s="207"/>
-      <c r="F8" s="207"/>
-      <c r="G8" s="207"/>
-      <c r="H8" s="207"/>
-      <c r="I8" s="207"/>
-      <c r="J8" s="208" t="s">
+      <c r="A8" s="260"/>
+      <c r="B8" s="260"/>
+      <c r="C8" s="260"/>
+      <c r="D8" s="260"/>
+      <c r="E8" s="260"/>
+      <c r="F8" s="260"/>
+      <c r="G8" s="260"/>
+      <c r="H8" s="260"/>
+      <c r="I8" s="260"/>
+      <c r="J8" s="261" t="s">
         <v>164</v>
       </c>
-      <c r="K8" s="209"/>
-      <c r="L8" s="209"/>
-      <c r="M8" s="209"/>
-      <c r="N8" s="209"/>
-      <c r="O8" s="210"/>
-      <c r="P8" s="208" t="s">
+      <c r="K8" s="262"/>
+      <c r="L8" s="262"/>
+      <c r="M8" s="262"/>
+      <c r="N8" s="262"/>
+      <c r="O8" s="263"/>
+      <c r="P8" s="261" t="s">
         <v>165</v>
       </c>
-      <c r="Q8" s="209"/>
-      <c r="R8" s="209"/>
-      <c r="S8" s="209"/>
-      <c r="T8" s="209"/>
-      <c r="U8" s="209"/>
-      <c r="V8" s="209"/>
-      <c r="W8" s="209"/>
-      <c r="X8" s="210"/>
+      <c r="Q8" s="262"/>
+      <c r="R8" s="262"/>
+      <c r="S8" s="262"/>
+      <c r="T8" s="262"/>
+      <c r="U8" s="262"/>
+      <c r="V8" s="262"/>
+      <c r="W8" s="262"/>
+      <c r="X8" s="263"/>
     </row>
     <row r="9" spans="1:24" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3"/>
@@ -7274,66 +7120,66 @@
       <c r="X9" s="3"/>
     </row>
     <row r="10" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="211" t="s">
+      <c r="A10" s="273" t="s">
         <v>166</v>
       </c>
-      <c r="B10" s="211"/>
-      <c r="C10" s="211"/>
-      <c r="D10" s="211"/>
-      <c r="E10" s="211"/>
-      <c r="F10" s="211"/>
-      <c r="G10" s="211"/>
-      <c r="H10" s="211"/>
-      <c r="I10" s="211"/>
-      <c r="J10" s="211"/>
-      <c r="K10" s="211"/>
-      <c r="L10" s="211"/>
-      <c r="M10" s="211"/>
-      <c r="N10" s="211"/>
-      <c r="O10" s="211"/>
-      <c r="P10" s="211"/>
-      <c r="Q10" s="211"/>
-      <c r="R10" s="211"/>
-      <c r="S10" s="211"/>
-      <c r="T10" s="211"/>
-      <c r="U10" s="211"/>
-      <c r="V10" s="211"/>
-      <c r="W10" s="211"/>
-      <c r="X10" s="211"/>
+      <c r="B10" s="273"/>
+      <c r="C10" s="273"/>
+      <c r="D10" s="273"/>
+      <c r="E10" s="273"/>
+      <c r="F10" s="273"/>
+      <c r="G10" s="273"/>
+      <c r="H10" s="273"/>
+      <c r="I10" s="273"/>
+      <c r="J10" s="273"/>
+      <c r="K10" s="273"/>
+      <c r="L10" s="273"/>
+      <c r="M10" s="273"/>
+      <c r="N10" s="273"/>
+      <c r="O10" s="273"/>
+      <c r="P10" s="273"/>
+      <c r="Q10" s="273"/>
+      <c r="R10" s="273"/>
+      <c r="S10" s="273"/>
+      <c r="T10" s="273"/>
+      <c r="U10" s="273"/>
+      <c r="V10" s="273"/>
+      <c r="W10" s="273"/>
+      <c r="X10" s="273"/>
     </row>
     <row r="11" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="212" t="s">
+      <c r="A11" s="274" t="s">
         <v>126</v>
       </c>
-      <c r="B11" s="212"/>
-      <c r="C11" s="212"/>
-      <c r="D11" s="212"/>
-      <c r="E11" s="212"/>
-      <c r="F11" s="212"/>
-      <c r="G11" s="212" t="s">
+      <c r="B11" s="274"/>
+      <c r="C11" s="274"/>
+      <c r="D11" s="274"/>
+      <c r="E11" s="274"/>
+      <c r="F11" s="274"/>
+      <c r="G11" s="274" t="s">
         <v>167</v>
       </c>
-      <c r="H11" s="212"/>
-      <c r="I11" s="212"/>
-      <c r="J11" s="212"/>
-      <c r="K11" s="212"/>
-      <c r="L11" s="212"/>
-      <c r="M11" s="212" t="s">
+      <c r="H11" s="274"/>
+      <c r="I11" s="274"/>
+      <c r="J11" s="274"/>
+      <c r="K11" s="274"/>
+      <c r="L11" s="274"/>
+      <c r="M11" s="274" t="s">
         <v>168</v>
       </c>
-      <c r="N11" s="212"/>
-      <c r="O11" s="212"/>
-      <c r="P11" s="212"/>
-      <c r="Q11" s="212"/>
-      <c r="R11" s="212"/>
-      <c r="S11" s="212" t="s">
+      <c r="N11" s="274"/>
+      <c r="O11" s="274"/>
+      <c r="P11" s="274"/>
+      <c r="Q11" s="274"/>
+      <c r="R11" s="274"/>
+      <c r="S11" s="274" t="s">
         <v>169</v>
       </c>
-      <c r="T11" s="212"/>
-      <c r="U11" s="212"/>
-      <c r="V11" s="212"/>
-      <c r="W11" s="212"/>
-      <c r="X11" s="212"/>
+      <c r="T11" s="274"/>
+      <c r="U11" s="274"/>
+      <c r="V11" s="274"/>
+      <c r="W11" s="274"/>
+      <c r="X11" s="274"/>
     </row>
     <row r="12" spans="1:24" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3"/>
@@ -7362,66 +7208,66 @@
       <c r="X12" s="3"/>
     </row>
     <row r="13" spans="1:24" s="2" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="198" t="s">
+      <c r="A13" s="253" t="s">
         <v>170</v>
       </c>
-      <c r="B13" s="198"/>
-      <c r="C13" s="198"/>
-      <c r="D13" s="198"/>
-      <c r="E13" s="198"/>
-      <c r="F13" s="198"/>
-      <c r="G13" s="198"/>
-      <c r="H13" s="198"/>
-      <c r="I13" s="198"/>
-      <c r="J13" s="198" t="s">
+      <c r="B13" s="253"/>
+      <c r="C13" s="253"/>
+      <c r="D13" s="253"/>
+      <c r="E13" s="253"/>
+      <c r="F13" s="253"/>
+      <c r="G13" s="253"/>
+      <c r="H13" s="253"/>
+      <c r="I13" s="253"/>
+      <c r="J13" s="253" t="s">
         <v>32</v>
       </c>
-      <c r="K13" s="198"/>
-      <c r="L13" s="198"/>
-      <c r="M13" s="198"/>
-      <c r="N13" s="198"/>
-      <c r="O13" s="198"/>
-      <c r="P13" s="198" t="s">
+      <c r="K13" s="253"/>
+      <c r="L13" s="253"/>
+      <c r="M13" s="253"/>
+      <c r="N13" s="253"/>
+      <c r="O13" s="253"/>
+      <c r="P13" s="253" t="s">
         <v>58</v>
       </c>
-      <c r="Q13" s="198"/>
-      <c r="R13" s="198"/>
-      <c r="S13" s="198"/>
-      <c r="T13" s="198"/>
-      <c r="U13" s="198"/>
-      <c r="V13" s="198"/>
-      <c r="W13" s="198"/>
-      <c r="X13" s="198"/>
+      <c r="Q13" s="253"/>
+      <c r="R13" s="253"/>
+      <c r="S13" s="253"/>
+      <c r="T13" s="253"/>
+      <c r="U13" s="253"/>
+      <c r="V13" s="253"/>
+      <c r="W13" s="253"/>
+      <c r="X13" s="253"/>
     </row>
     <row r="14" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="207"/>
-      <c r="B14" s="207"/>
-      <c r="C14" s="207"/>
-      <c r="D14" s="207"/>
-      <c r="E14" s="207"/>
-      <c r="F14" s="207"/>
-      <c r="G14" s="207"/>
-      <c r="H14" s="207"/>
-      <c r="I14" s="207"/>
-      <c r="J14" s="208" t="s">
+      <c r="A14" s="260"/>
+      <c r="B14" s="260"/>
+      <c r="C14" s="260"/>
+      <c r="D14" s="260"/>
+      <c r="E14" s="260"/>
+      <c r="F14" s="260"/>
+      <c r="G14" s="260"/>
+      <c r="H14" s="260"/>
+      <c r="I14" s="260"/>
+      <c r="J14" s="261" t="s">
         <v>171</v>
       </c>
-      <c r="K14" s="209"/>
-      <c r="L14" s="209"/>
-      <c r="M14" s="209"/>
-      <c r="N14" s="209"/>
-      <c r="O14" s="210"/>
-      <c r="P14" s="208" t="s">
+      <c r="K14" s="262"/>
+      <c r="L14" s="262"/>
+      <c r="M14" s="262"/>
+      <c r="N14" s="262"/>
+      <c r="O14" s="263"/>
+      <c r="P14" s="261" t="s">
         <v>172</v>
       </c>
-      <c r="Q14" s="209"/>
-      <c r="R14" s="209"/>
-      <c r="S14" s="209"/>
-      <c r="T14" s="209"/>
-      <c r="U14" s="209"/>
-      <c r="V14" s="209"/>
-      <c r="W14" s="209"/>
-      <c r="X14" s="210"/>
+      <c r="Q14" s="262"/>
+      <c r="R14" s="262"/>
+      <c r="S14" s="262"/>
+      <c r="T14" s="262"/>
+      <c r="U14" s="262"/>
+      <c r="V14" s="262"/>
+      <c r="W14" s="262"/>
+      <c r="X14" s="263"/>
     </row>
     <row r="15" spans="1:24" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3"/>
@@ -7450,172 +7296,184 @@
       <c r="X15" s="3"/>
     </row>
     <row r="16" spans="1:24" s="4" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="218" t="s">
+      <c r="A16" s="264" t="s">
         <v>173</v>
       </c>
-      <c r="B16" s="218"/>
-      <c r="C16" s="218"/>
-      <c r="D16" s="218"/>
-      <c r="E16" s="218"/>
-      <c r="F16" s="218"/>
-      <c r="G16" s="218"/>
-      <c r="H16" s="218"/>
-      <c r="I16" s="218"/>
-      <c r="J16" s="219" t="s">
+      <c r="B16" s="264"/>
+      <c r="C16" s="264"/>
+      <c r="D16" s="264"/>
+      <c r="E16" s="264"/>
+      <c r="F16" s="264"/>
+      <c r="G16" s="264"/>
+      <c r="H16" s="264"/>
+      <c r="I16" s="264"/>
+      <c r="J16" s="265" t="s">
         <v>174</v>
       </c>
-      <c r="K16" s="219"/>
-      <c r="L16" s="219"/>
-      <c r="M16" s="219"/>
-      <c r="N16" s="218" t="s">
+      <c r="K16" s="265"/>
+      <c r="L16" s="265"/>
+      <c r="M16" s="265"/>
+      <c r="N16" s="264" t="s">
         <v>175</v>
       </c>
-      <c r="O16" s="218"/>
-      <c r="P16" s="218"/>
-      <c r="Q16" s="218"/>
-      <c r="R16" s="218"/>
-      <c r="S16" s="218"/>
-      <c r="T16" s="220" t="s">
+      <c r="O16" s="264"/>
+      <c r="P16" s="264"/>
+      <c r="Q16" s="264"/>
+      <c r="R16" s="264"/>
+      <c r="S16" s="264"/>
+      <c r="T16" s="266" t="s">
         <v>176</v>
       </c>
-      <c r="U16" s="220"/>
-      <c r="V16" s="220"/>
-      <c r="W16" s="220"/>
-      <c r="X16" s="220"/>
+      <c r="U16" s="266"/>
+      <c r="V16" s="266"/>
+      <c r="W16" s="266"/>
+      <c r="X16" s="266"/>
     </row>
     <row r="17" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="213" t="s">
+      <c r="A17" s="254" t="s">
         <v>177</v>
       </c>
-      <c r="B17" s="205"/>
-      <c r="C17" s="205"/>
-      <c r="D17" s="205"/>
-      <c r="E17" s="205"/>
-      <c r="F17" s="205"/>
-      <c r="G17" s="205"/>
-      <c r="H17" s="205"/>
-      <c r="I17" s="214"/>
-      <c r="J17" s="221" t="s">
+      <c r="B17" s="255"/>
+      <c r="C17" s="255"/>
+      <c r="D17" s="255"/>
+      <c r="E17" s="255"/>
+      <c r="F17" s="255"/>
+      <c r="G17" s="255"/>
+      <c r="H17" s="255"/>
+      <c r="I17" s="256"/>
+      <c r="J17" s="267" t="s">
         <v>178</v>
       </c>
-      <c r="K17" s="222"/>
-      <c r="L17" s="222"/>
-      <c r="M17" s="223"/>
-      <c r="N17" s="213" t="s">
+      <c r="K17" s="268"/>
+      <c r="L17" s="268"/>
+      <c r="M17" s="269"/>
+      <c r="N17" s="254" t="s">
         <v>179</v>
       </c>
-      <c r="O17" s="205"/>
-      <c r="P17" s="205"/>
-      <c r="Q17" s="205"/>
-      <c r="R17" s="205"/>
-      <c r="S17" s="214"/>
-      <c r="T17" s="213" t="s">
+      <c r="O17" s="255"/>
+      <c r="P17" s="255"/>
+      <c r="Q17" s="255"/>
+      <c r="R17" s="255"/>
+      <c r="S17" s="256"/>
+      <c r="T17" s="254" t="s">
         <v>180</v>
       </c>
-      <c r="U17" s="205"/>
-      <c r="V17" s="205"/>
-      <c r="W17" s="205"/>
-      <c r="X17" s="214"/>
+      <c r="U17" s="255"/>
+      <c r="V17" s="255"/>
+      <c r="W17" s="255"/>
+      <c r="X17" s="256"/>
     </row>
     <row r="18" spans="1:24" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="215"/>
-      <c r="B18" s="216"/>
-      <c r="C18" s="216"/>
-      <c r="D18" s="216"/>
-      <c r="E18" s="216"/>
-      <c r="F18" s="216"/>
-      <c r="G18" s="216"/>
-      <c r="H18" s="216"/>
-      <c r="I18" s="217"/>
-      <c r="J18" s="224"/>
-      <c r="K18" s="225"/>
-      <c r="L18" s="225"/>
-      <c r="M18" s="226"/>
-      <c r="N18" s="215"/>
-      <c r="O18" s="216"/>
-      <c r="P18" s="216"/>
-      <c r="Q18" s="216"/>
-      <c r="R18" s="216"/>
-      <c r="S18" s="217"/>
-      <c r="T18" s="215"/>
-      <c r="U18" s="216"/>
-      <c r="V18" s="216"/>
-      <c r="W18" s="216"/>
-      <c r="X18" s="217"/>
+      <c r="A18" s="257"/>
+      <c r="B18" s="258"/>
+      <c r="C18" s="258"/>
+      <c r="D18" s="258"/>
+      <c r="E18" s="258"/>
+      <c r="F18" s="258"/>
+      <c r="G18" s="258"/>
+      <c r="H18" s="258"/>
+      <c r="I18" s="259"/>
+      <c r="J18" s="270"/>
+      <c r="K18" s="271"/>
+      <c r="L18" s="271"/>
+      <c r="M18" s="272"/>
+      <c r="N18" s="257"/>
+      <c r="O18" s="258"/>
+      <c r="P18" s="258"/>
+      <c r="Q18" s="258"/>
+      <c r="R18" s="258"/>
+      <c r="S18" s="259"/>
+      <c r="T18" s="257"/>
+      <c r="U18" s="258"/>
+      <c r="V18" s="258"/>
+      <c r="W18" s="258"/>
+      <c r="X18" s="259"/>
     </row>
     <row r="19" spans="1:24" ht="39" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="20" spans="1:24" ht="39" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="21" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A21" s="230" t="s">
+      <c r="A21" s="252" t="s">
         <v>181</v>
       </c>
-      <c r="B21" s="230"/>
-      <c r="C21" s="230"/>
-      <c r="D21" s="230"/>
-      <c r="E21" s="230"/>
-      <c r="F21" s="230"/>
-      <c r="G21" s="230"/>
-      <c r="H21" s="230"/>
+      <c r="B21" s="252"/>
+      <c r="C21" s="252"/>
+      <c r="D21" s="252"/>
+      <c r="E21" s="252"/>
+      <c r="F21" s="252"/>
+      <c r="G21" s="252"/>
+      <c r="H21" s="252"/>
       <c r="I21" s="5"/>
-      <c r="J21" s="230" t="s">
+      <c r="J21" s="252" t="s">
         <v>182</v>
       </c>
-      <c r="K21" s="230"/>
-      <c r="L21" s="230"/>
-      <c r="M21" s="230"/>
-      <c r="N21" s="230"/>
-      <c r="O21" s="230"/>
-      <c r="P21" s="230"/>
+      <c r="K21" s="252"/>
+      <c r="L21" s="252"/>
+      <c r="M21" s="252"/>
+      <c r="N21" s="252"/>
+      <c r="O21" s="252"/>
+      <c r="P21" s="252"/>
       <c r="Q21" s="6"/>
-      <c r="R21" s="230" t="s">
+      <c r="R21" s="252" t="s">
         <v>183</v>
       </c>
-      <c r="S21" s="230"/>
-      <c r="T21" s="230"/>
-      <c r="U21" s="230"/>
-      <c r="V21" s="230"/>
-      <c r="W21" s="230"/>
-      <c r="X21" s="230"/>
+      <c r="S21" s="252"/>
+      <c r="T21" s="252"/>
+      <c r="U21" s="252"/>
+      <c r="V21" s="252"/>
+      <c r="W21" s="252"/>
+      <c r="X21" s="252"/>
     </row>
     <row r="23" spans="1:24" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="P23" s="227" t="s">
+      <c r="P23" s="249" t="s">
         <v>184</v>
       </c>
-      <c r="Q23" s="227"/>
-      <c r="R23" s="227"/>
-      <c r="S23" s="227"/>
-      <c r="T23" s="227"/>
-      <c r="U23" s="228" t="s">
+      <c r="Q23" s="249"/>
+      <c r="R23" s="249"/>
+      <c r="S23" s="249"/>
+      <c r="T23" s="249"/>
+      <c r="U23" s="250" t="s">
         <v>185</v>
       </c>
-      <c r="V23" s="228"/>
-      <c r="W23" s="228"/>
-      <c r="X23" s="228"/>
+      <c r="V23" s="250"/>
+      <c r="W23" s="250"/>
+      <c r="X23" s="250"/>
     </row>
     <row r="24" spans="1:24" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="P24" s="227" t="s">
+      <c r="P24" s="249" t="s">
         <v>186</v>
       </c>
-      <c r="Q24" s="227"/>
-      <c r="R24" s="227"/>
-      <c r="S24" s="227"/>
-      <c r="T24" s="227"/>
-      <c r="U24" s="229" t="s">
+      <c r="Q24" s="249"/>
+      <c r="R24" s="249"/>
+      <c r="S24" s="249"/>
+      <c r="T24" s="249"/>
+      <c r="U24" s="251" t="s">
         <v>187</v>
       </c>
-      <c r="V24" s="229"/>
-      <c r="W24" s="229"/>
-      <c r="X24" s="229"/>
+      <c r="V24" s="251"/>
+      <c r="W24" s="251"/>
+      <c r="X24" s="251"/>
     </row>
   </sheetData>
   <mergeCells count="40">
-    <mergeCell ref="P23:T23"/>
-    <mergeCell ref="U23:X23"/>
-    <mergeCell ref="P24:T24"/>
-    <mergeCell ref="U24:X24"/>
-    <mergeCell ref="A21:H21"/>
-    <mergeCell ref="J21:P21"/>
-    <mergeCell ref="R21:X21"/>
+    <mergeCell ref="A1:T1"/>
+    <mergeCell ref="U1:X1"/>
+    <mergeCell ref="A2:T2"/>
+    <mergeCell ref="A7:I7"/>
+    <mergeCell ref="J7:O7"/>
+    <mergeCell ref="P7:X7"/>
+    <mergeCell ref="A5:M5"/>
+    <mergeCell ref="A4:M4"/>
+    <mergeCell ref="N4:X4"/>
+    <mergeCell ref="N5:X5"/>
+    <mergeCell ref="U2:X3"/>
+    <mergeCell ref="A8:I8"/>
+    <mergeCell ref="J8:O8"/>
+    <mergeCell ref="P8:X8"/>
+    <mergeCell ref="A10:X10"/>
+    <mergeCell ref="A11:F11"/>
+    <mergeCell ref="G11:L11"/>
+    <mergeCell ref="M11:R11"/>
+    <mergeCell ref="S11:X11"/>
     <mergeCell ref="A13:I13"/>
     <mergeCell ref="J13:O13"/>
     <mergeCell ref="P13:X13"/>
@@ -7630,25 +7488,13 @@
     <mergeCell ref="T16:X16"/>
     <mergeCell ref="A17:I18"/>
     <mergeCell ref="J17:M18"/>
-    <mergeCell ref="A8:I8"/>
-    <mergeCell ref="J8:O8"/>
-    <mergeCell ref="P8:X8"/>
-    <mergeCell ref="A10:X10"/>
-    <mergeCell ref="A11:F11"/>
-    <mergeCell ref="G11:L11"/>
-    <mergeCell ref="M11:R11"/>
-    <mergeCell ref="S11:X11"/>
-    <mergeCell ref="A1:T1"/>
-    <mergeCell ref="U1:X1"/>
-    <mergeCell ref="A2:T2"/>
-    <mergeCell ref="A7:I7"/>
-    <mergeCell ref="J7:O7"/>
-    <mergeCell ref="P7:X7"/>
-    <mergeCell ref="A5:M5"/>
-    <mergeCell ref="A4:M4"/>
-    <mergeCell ref="N4:X4"/>
-    <mergeCell ref="N5:X5"/>
-    <mergeCell ref="U2:X3"/>
+    <mergeCell ref="P23:T23"/>
+    <mergeCell ref="U23:X23"/>
+    <mergeCell ref="P24:T24"/>
+    <mergeCell ref="U24:X24"/>
+    <mergeCell ref="A21:H21"/>
+    <mergeCell ref="J21:P21"/>
+    <mergeCell ref="R21:X21"/>
   </mergeCells>
   <pageMargins left="0.51181102362204722" right="0.51181102362204722" top="0.35433070866141736" bottom="0.35433070866141736" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup scale="95" orientation="landscape" horizontalDpi="4294967294" verticalDpi="200" r:id="rId1"/>
@@ -7657,18 +7503,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <TaxCatchAll xmlns="41dd0a9e-964d-48c8-9389-7445c2a187f7" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="edbb1c21-1b45-407e-8894-c97732534993">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <_Flow_SignoffStatus xmlns="edbb1c21-1b45-407e-8894-c97732534993" xsi:nil="true"/>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <FechayHora xmlns="edbb1c21-1b45-407e-8894-c97732534993" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -7962,22 +7802,24 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <TaxCatchAll xmlns="41dd0a9e-964d-48c8-9389-7445c2a187f7" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="edbb1c21-1b45-407e-8894-c97732534993">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <_Flow_SignoffStatus xmlns="edbb1c21-1b45-407e-8894-c97732534993" xsi:nil="true"/>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <FechayHora xmlns="edbb1c21-1b45-407e-8894-c97732534993" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBE5A30C-34BC-4387-870E-CFF8B53C216A}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7CCE7917-804F-4951-9FEA-F53AEA82B8BE}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="41dd0a9e-964d-48c8-9389-7445c2a187f7"/>
-    <ds:schemaRef ds:uri="edbb1c21-1b45-407e-8894-c97732534993"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -8003,9 +7845,13 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7CCE7917-804F-4951-9FEA-F53AEA82B8BE}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBE5A30C-34BC-4387-870E-CFF8B53C216A}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="41dd0a9e-964d-48c8-9389-7445c2a187f7"/>
+    <ds:schemaRef ds:uri="edbb1c21-1b45-407e-8894-c97732534993"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Actualizar formatos GFPI-F023 y bitácoras GFPI-F-147V4.
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Formatos/BITACORAS GFPI-F-147V4.xlsx
+++ b/Formatos/BITACORAS GFPI-F-147V4.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SEANT\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SEANT\OneDrive\Documents\Seto 2026\sena\Manual SENA Etapa Productiva\manual-aprendiz-sena\Formatos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FA325372-B3D4-4C73-B306-A8EC3281E55B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C00FB21-90C9-41D6-AC50-EF2816FA0BA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2287,189 +2287,331 @@
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="93" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="96" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="93" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="93" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="15" fontId="32" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="82" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement i="0"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="107" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement i="0"/>
+        </ext>
+      </extLst>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="94" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="108" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="109" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="110" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="61" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="72" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="91" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="57" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="58" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="59" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="66" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="67" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="63" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="98" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="100" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="101" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="92" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="93" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="89" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="90" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="64" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="64" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="66" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="67" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="84" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="85" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="86" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="66" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="67" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="85" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="86" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="5" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="5" borderId="57" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="95" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="96" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="99" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="100" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="77" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="78" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="68" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="85" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="86" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="71" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="75" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="59" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="2" borderId="70" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="2" borderId="74" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="2" borderId="58" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="70" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="74" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="69" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="73" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="63" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="97" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="65" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="71" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="75" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="59" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="62" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="53" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="102" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="70" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="74" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="61" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="60" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="54" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="70" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="74" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="71" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="75" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="59" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="19" fillId="6" borderId="79" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2497,12 +2639,6 @@
     <xf numFmtId="0" fontId="20" fillId="0" borderId="105" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2513,423 +2649,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="59" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="106" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="93" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="68" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="85" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="86" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="2" borderId="70" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="2" borderId="74" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="2" borderId="58" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="69" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="73" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="63" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="77" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="78" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="97" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="100" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="98" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="100" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="101" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="63" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="89" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="90" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="64" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="64" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="7" borderId="76" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="7" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="7" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="7" borderId="87" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="7" borderId="88" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="66" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="67" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="84" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="85" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="86" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="66" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="67" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="85" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="86" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="5" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="5" borderId="57" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="95" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="96" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="99" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="83" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="52" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="58" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="59" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="61" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="72" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="91" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="57" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="58" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="59" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="66" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="67" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="108" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="109" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="110" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="15" fontId="32" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="106" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2948,62 +2667,308 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="82" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
-          <xfpb:xfComplement i="0"/>
-        </ext>
-      </extLst>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="107" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
-          <xfpb:xfComplement i="0"/>
-        </ext>
-      </extLst>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="83" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="106" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="52" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="58" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="59" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="70" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="74" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="61" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="60" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="54" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="94" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="65" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="71" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="75" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="59" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="62" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="53" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="102" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="76" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="87" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="88" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="96" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="93" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="93" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="93" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="11">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFE6DE74"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFDEE16D"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFE9E96D"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFE6E95D"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFE2ED51"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="4">
     <dxf>
       <fill>
         <patternFill>
@@ -3021,21 +2986,7 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFDEE16D"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFE9E96D"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFE6E95D"/>
+          <bgColor rgb="FFE1EF57"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3519,19 +3470,19 @@
     <col min="7" max="7" width="22.5703125" style="9" customWidth="1"/>
     <col min="8" max="8" width="32.7109375" style="9" customWidth="1"/>
     <col min="9" max="9" width="34.42578125" style="9" customWidth="1"/>
-    <col min="10" max="10" width="8.42578125" style="9" hidden="1"/>
-    <col min="11" max="11" width="6.42578125" style="9" hidden="1"/>
-    <col min="12" max="17" width="5.7109375" style="9" hidden="1"/>
-    <col min="18" max="18" width="4.7109375" style="9" hidden="1"/>
-    <col min="19" max="19" width="5.85546875" style="9" hidden="1"/>
-    <col min="20" max="20" width="7.42578125" style="9" hidden="1"/>
-    <col min="21" max="21" width="7.140625" style="9" hidden="1"/>
-    <col min="22" max="23" width="5.7109375" style="9" hidden="1"/>
-    <col min="24" max="24" width="5" style="9" hidden="1"/>
-    <col min="25" max="25" width="6.42578125" style="9" hidden="1"/>
-    <col min="26" max="26" width="8.140625" style="9" hidden="1"/>
-    <col min="27" max="27" width="5.140625" style="9" hidden="1"/>
-    <col min="28" max="28" width="24.42578125" style="8" hidden="1"/>
+    <col min="10" max="10" width="8.42578125" style="9" hidden="1" customWidth="1"/>
+    <col min="11" max="11" width="6.42578125" style="9" hidden="1" customWidth="1"/>
+    <col min="12" max="17" width="5.7109375" style="9" hidden="1" customWidth="1"/>
+    <col min="18" max="18" width="4.7109375" style="9" hidden="1" customWidth="1"/>
+    <col min="19" max="19" width="5.85546875" style="9" hidden="1" customWidth="1"/>
+    <col min="20" max="20" width="7.42578125" style="9" hidden="1" customWidth="1"/>
+    <col min="21" max="21" width="7.140625" style="9" hidden="1" customWidth="1"/>
+    <col min="22" max="23" width="5.7109375" style="9" hidden="1" customWidth="1"/>
+    <col min="24" max="24" width="5" style="9" hidden="1" customWidth="1"/>
+    <col min="25" max="25" width="6.42578125" style="9" hidden="1" customWidth="1"/>
+    <col min="26" max="26" width="8.140625" style="9" hidden="1" customWidth="1"/>
+    <col min="27" max="27" width="5.140625" style="9" hidden="1" customWidth="1"/>
+    <col min="28" max="28" width="24.42578125" style="8" hidden="1" customWidth="1"/>
     <col min="29" max="16384" width="11.42578125" style="7" hidden="1"/>
   </cols>
   <sheetData>
@@ -3598,16 +3549,16 @@
       <c r="AB2" s="7"/>
     </row>
     <row r="3" spans="2:28" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="118" t="s">
+      <c r="B3" s="162" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="119"/>
-      <c r="D3" s="119"/>
-      <c r="E3" s="119"/>
-      <c r="F3" s="119"/>
-      <c r="G3" s="119"/>
-      <c r="H3" s="119"/>
-      <c r="I3" s="120"/>
+      <c r="C3" s="163"/>
+      <c r="D3" s="163"/>
+      <c r="E3" s="163"/>
+      <c r="F3" s="163"/>
+      <c r="G3" s="163"/>
+      <c r="H3" s="163"/>
+      <c r="I3" s="164"/>
       <c r="J3" s="8"/>
       <c r="K3" s="7"/>
       <c r="L3" s="7"/>
@@ -3629,16 +3580,16 @@
       <c r="AB3" s="7"/>
     </row>
     <row r="4" spans="2:28" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="124" t="s">
+      <c r="B4" s="168" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="125"/>
-      <c r="D4" s="125"/>
-      <c r="E4" s="125"/>
-      <c r="F4" s="125"/>
-      <c r="G4" s="125"/>
-      <c r="H4" s="125"/>
-      <c r="I4" s="126"/>
+      <c r="C4" s="169"/>
+      <c r="D4" s="169"/>
+      <c r="E4" s="169"/>
+      <c r="F4" s="169"/>
+      <c r="G4" s="169"/>
+      <c r="H4" s="169"/>
+      <c r="I4" s="170"/>
       <c r="J4" s="8"/>
       <c r="K4" s="7"/>
       <c r="L4" s="7"/>
@@ -3660,16 +3611,16 @@
       <c r="AB4" s="7"/>
     </row>
     <row r="5" spans="2:28" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="121" t="s">
+      <c r="B5" s="165" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="122"/>
-      <c r="D5" s="122"/>
-      <c r="E5" s="122"/>
-      <c r="F5" s="122"/>
-      <c r="G5" s="122"/>
-      <c r="H5" s="122"/>
-      <c r="I5" s="123"/>
+      <c r="C5" s="166"/>
+      <c r="D5" s="166"/>
+      <c r="E5" s="166"/>
+      <c r="F5" s="166"/>
+      <c r="G5" s="166"/>
+      <c r="H5" s="166"/>
+      <c r="I5" s="167"/>
       <c r="J5" s="8"/>
       <c r="K5" s="8"/>
       <c r="L5" s="7"/>
@@ -3691,16 +3642,16 @@
       <c r="AB5" s="7"/>
     </row>
     <row r="6" spans="2:28" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="124" t="s">
+      <c r="B6" s="168" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="125"/>
-      <c r="D6" s="125"/>
-      <c r="E6" s="125"/>
-      <c r="F6" s="125"/>
-      <c r="G6" s="125"/>
-      <c r="H6" s="125"/>
-      <c r="I6" s="126"/>
+      <c r="C6" s="169"/>
+      <c r="D6" s="169"/>
+      <c r="E6" s="169"/>
+      <c r="F6" s="169"/>
+      <c r="G6" s="169"/>
+      <c r="H6" s="169"/>
+      <c r="I6" s="170"/>
       <c r="J6" s="8"/>
       <c r="K6" s="8"/>
       <c r="L6" s="7"/>
@@ -3722,16 +3673,16 @@
       <c r="AB6" s="7"/>
     </row>
     <row r="7" spans="2:28" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="121" t="s">
+      <c r="B7" s="165" t="s">
         <v>6</v>
       </c>
-      <c r="C7" s="122"/>
-      <c r="D7" s="122"/>
-      <c r="E7" s="122"/>
-      <c r="F7" s="122"/>
-      <c r="G7" s="122"/>
-      <c r="H7" s="122"/>
-      <c r="I7" s="123"/>
+      <c r="C7" s="166"/>
+      <c r="D7" s="166"/>
+      <c r="E7" s="166"/>
+      <c r="F7" s="166"/>
+      <c r="G7" s="166"/>
+      <c r="H7" s="166"/>
+      <c r="I7" s="167"/>
       <c r="J7" s="7"/>
       <c r="K7" s="7"/>
       <c r="L7" s="7"/>
@@ -3756,21 +3707,21 @@
       <c r="B8" s="53" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="272" t="b">
+      <c r="C8" s="175" t="b">
         <v>0</v>
       </c>
-      <c r="D8" s="273"/>
-      <c r="E8" s="203" t="s">
+      <c r="D8" s="176"/>
+      <c r="E8" s="177" t="s">
         <v>8</v>
       </c>
-      <c r="F8" s="133"/>
-      <c r="G8" s="274" t="b">
+      <c r="F8" s="178"/>
+      <c r="G8" s="58" t="b">
         <v>0</v>
       </c>
       <c r="H8" s="54" t="s">
         <v>9</v>
       </c>
-      <c r="I8" s="275" t="b">
+      <c r="I8" s="59" t="b">
         <v>0</v>
       </c>
       <c r="J8" s="7"/>
@@ -3799,8 +3750,8 @@
       <c r="D9" s="18"/>
       <c r="E9" s="23"/>
       <c r="F9" s="23"/>
-      <c r="G9" s="86"/>
-      <c r="H9" s="86"/>
+      <c r="G9" s="190"/>
+      <c r="H9" s="190"/>
       <c r="I9" s="18"/>
       <c r="J9" s="7"/>
       <c r="K9" s="7"/>
@@ -3823,18 +3774,18 @@
       <c r="AB9" s="7"/>
     </row>
     <row r="10" spans="2:28" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="112" t="s">
+      <c r="B10" s="151" t="s">
         <v>10</v>
       </c>
-      <c r="C10" s="113"/>
-      <c r="D10" s="114"/>
-      <c r="E10" s="111" t="s">
+      <c r="C10" s="152"/>
+      <c r="D10" s="153"/>
+      <c r="E10" s="149" t="s">
         <v>11</v>
       </c>
-      <c r="F10" s="111"/>
-      <c r="G10" s="111"/>
-      <c r="H10" s="111"/>
-      <c r="I10" s="111"/>
+      <c r="F10" s="149"/>
+      <c r="G10" s="149"/>
+      <c r="H10" s="149"/>
+      <c r="I10" s="149"/>
       <c r="J10" s="7"/>
       <c r="K10" s="7"/>
       <c r="L10" s="7"/>
@@ -3856,14 +3807,14 @@
       <c r="AB10" s="7"/>
     </row>
     <row r="11" spans="2:28" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="115"/>
-      <c r="C11" s="116"/>
-      <c r="D11" s="117"/>
-      <c r="E11" s="270"/>
-      <c r="F11" s="270"/>
-      <c r="G11" s="270"/>
-      <c r="H11" s="270"/>
-      <c r="I11" s="270"/>
+      <c r="B11" s="141"/>
+      <c r="C11" s="142"/>
+      <c r="D11" s="143"/>
+      <c r="E11" s="189"/>
+      <c r="F11" s="189"/>
+      <c r="G11" s="189"/>
+      <c r="H11" s="189"/>
+      <c r="I11" s="189"/>
       <c r="J11" s="7"/>
       <c r="K11" s="7"/>
       <c r="L11" s="7"/>
@@ -3890,8 +3841,8 @@
       <c r="D12" s="18"/>
       <c r="E12" s="23"/>
       <c r="F12" s="23"/>
-      <c r="G12" s="86"/>
-      <c r="H12" s="86"/>
+      <c r="G12" s="190"/>
+      <c r="H12" s="190"/>
       <c r="I12" s="18"/>
       <c r="J12" s="7"/>
       <c r="K12" s="7"/>
@@ -3914,16 +3865,16 @@
       <c r="AB12" s="7"/>
     </row>
     <row r="13" spans="2:28" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="109" t="s">
+      <c r="B13" s="187" t="s">
         <v>12</v>
       </c>
-      <c r="C13" s="109"/>
-      <c r="D13" s="109"/>
-      <c r="E13" s="109"/>
-      <c r="F13" s="109"/>
-      <c r="G13" s="109"/>
-      <c r="H13" s="109"/>
-      <c r="I13" s="110"/>
+      <c r="C13" s="187"/>
+      <c r="D13" s="187"/>
+      <c r="E13" s="187"/>
+      <c r="F13" s="187"/>
+      <c r="G13" s="187"/>
+      <c r="H13" s="187"/>
+      <c r="I13" s="188"/>
       <c r="J13" s="7"/>
       <c r="K13" s="7"/>
       <c r="L13" s="7"/>
@@ -3945,32 +3896,32 @@
       <c r="AB13" s="7"/>
     </row>
     <row r="14" spans="2:28" s="9" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="112" t="s">
+      <c r="B14" s="151" t="s">
         <v>13</v>
       </c>
-      <c r="C14" s="113"/>
-      <c r="D14" s="114"/>
+      <c r="C14" s="152"/>
+      <c r="D14" s="153"/>
       <c r="E14" s="55" t="s">
         <v>14</v>
       </c>
-      <c r="F14" s="204" t="s">
+      <c r="F14" s="179" t="s">
         <v>15</v>
       </c>
-      <c r="G14" s="205"/>
-      <c r="H14" s="111" t="s">
+      <c r="G14" s="180"/>
+      <c r="H14" s="149" t="s">
         <v>16</v>
       </c>
-      <c r="I14" s="127"/>
+      <c r="I14" s="150"/>
     </row>
     <row r="15" spans="2:28" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="130"/>
-      <c r="C15" s="131"/>
-      <c r="D15" s="132"/>
+      <c r="B15" s="172"/>
+      <c r="C15" s="173"/>
+      <c r="D15" s="174"/>
       <c r="E15" s="37"/>
-      <c r="F15" s="206"/>
-      <c r="G15" s="207"/>
-      <c r="H15" s="128"/>
-      <c r="I15" s="129"/>
+      <c r="F15" s="181"/>
+      <c r="G15" s="182"/>
+      <c r="H15" s="160"/>
+      <c r="I15" s="171"/>
       <c r="J15" s="7"/>
       <c r="K15" s="7"/>
       <c r="L15" s="7"/>
@@ -3992,20 +3943,20 @@
       <c r="AB15" s="7"/>
     </row>
     <row r="16" spans="2:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="105" t="s">
+      <c r="B16" s="183" t="s">
         <v>17</v>
       </c>
-      <c r="C16" s="106"/>
-      <c r="D16" s="107"/>
-      <c r="E16" s="108" t="s">
+      <c r="C16" s="184"/>
+      <c r="D16" s="185"/>
+      <c r="E16" s="186" t="s">
         <v>18</v>
       </c>
-      <c r="F16" s="108"/>
-      <c r="G16" s="108"/>
-      <c r="H16" s="211" t="s">
+      <c r="F16" s="186"/>
+      <c r="G16" s="186"/>
+      <c r="H16" s="78" t="s">
         <v>19</v>
       </c>
-      <c r="I16" s="212"/>
+      <c r="I16" s="79"/>
       <c r="J16" s="7"/>
       <c r="K16" s="7"/>
       <c r="L16" s="7"/>
@@ -4027,14 +3978,14 @@
       <c r="AB16" s="7"/>
     </row>
     <row r="17" spans="2:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="115"/>
-      <c r="C17" s="116"/>
-      <c r="D17" s="117"/>
-      <c r="E17" s="210"/>
-      <c r="F17" s="210"/>
-      <c r="G17" s="210"/>
-      <c r="H17" s="145"/>
-      <c r="I17" s="146"/>
+      <c r="B17" s="141"/>
+      <c r="C17" s="142"/>
+      <c r="D17" s="143"/>
+      <c r="E17" s="77"/>
+      <c r="F17" s="77"/>
+      <c r="G17" s="77"/>
+      <c r="H17" s="80"/>
+      <c r="I17" s="81"/>
       <c r="J17" s="7"/>
       <c r="K17" s="7"/>
       <c r="L17" s="7"/>
@@ -4056,20 +4007,20 @@
       <c r="AB17" s="7"/>
     </row>
     <row r="18" spans="2:28" s="47" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="112" t="s">
+      <c r="B18" s="151" t="s">
         <v>20</v>
       </c>
-      <c r="C18" s="113"/>
-      <c r="D18" s="114"/>
-      <c r="E18" s="111" t="s">
+      <c r="C18" s="152"/>
+      <c r="D18" s="153"/>
+      <c r="E18" s="149" t="s">
         <v>21</v>
       </c>
-      <c r="F18" s="111"/>
-      <c r="G18" s="111"/>
-      <c r="H18" s="111" t="s">
+      <c r="F18" s="149"/>
+      <c r="G18" s="149"/>
+      <c r="H18" s="149" t="s">
         <v>22</v>
       </c>
-      <c r="I18" s="127"/>
+      <c r="I18" s="150"/>
       <c r="J18" s="7"/>
       <c r="K18" s="7"/>
       <c r="L18" s="7"/>
@@ -4091,14 +4042,14 @@
       <c r="AB18" s="7"/>
     </row>
     <row r="19" spans="2:28" s="47" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="147"/>
-      <c r="C19" s="148"/>
-      <c r="D19" s="149"/>
-      <c r="E19" s="145"/>
-      <c r="F19" s="145"/>
-      <c r="G19" s="145"/>
-      <c r="H19" s="145"/>
-      <c r="I19" s="146"/>
+      <c r="B19" s="154"/>
+      <c r="C19" s="155"/>
+      <c r="D19" s="156"/>
+      <c r="E19" s="80"/>
+      <c r="F19" s="80"/>
+      <c r="G19" s="80"/>
+      <c r="H19" s="80"/>
+      <c r="I19" s="81"/>
       <c r="J19" s="7"/>
       <c r="K19" s="7"/>
       <c r="L19" s="7"/>
@@ -4120,20 +4071,20 @@
       <c r="AB19" s="7"/>
     </row>
     <row r="20" spans="2:28" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="142" t="s">
+      <c r="B20" s="146" t="s">
         <v>23</v>
       </c>
-      <c r="C20" s="143"/>
-      <c r="D20" s="144"/>
-      <c r="E20" s="140" t="s">
+      <c r="C20" s="147"/>
+      <c r="D20" s="148"/>
+      <c r="E20" s="144" t="s">
         <v>24</v>
       </c>
-      <c r="F20" s="140"/>
-      <c r="G20" s="140"/>
-      <c r="H20" s="140" t="s">
+      <c r="F20" s="144"/>
+      <c r="G20" s="144"/>
+      <c r="H20" s="144" t="s">
         <v>25</v>
       </c>
-      <c r="I20" s="141"/>
+      <c r="I20" s="145"/>
       <c r="J20" s="16"/>
       <c r="K20" s="16"/>
       <c r="L20" s="16"/>
@@ -4153,14 +4104,14 @@
       <c r="AA20" s="16"/>
     </row>
     <row r="21" spans="2:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="115"/>
-      <c r="C21" s="116"/>
-      <c r="D21" s="117"/>
-      <c r="E21" s="128"/>
-      <c r="F21" s="128"/>
-      <c r="G21" s="128"/>
-      <c r="H21" s="155"/>
-      <c r="I21" s="156"/>
+      <c r="B21" s="141"/>
+      <c r="C21" s="142"/>
+      <c r="D21" s="143"/>
+      <c r="E21" s="160"/>
+      <c r="F21" s="160"/>
+      <c r="G21" s="160"/>
+      <c r="H21" s="158"/>
+      <c r="I21" s="159"/>
       <c r="J21" s="18"/>
       <c r="K21" s="18"/>
       <c r="L21" s="18"/>
@@ -4185,8 +4136,8 @@
       <c r="D22" s="13"/>
       <c r="E22" s="33"/>
       <c r="F22" s="33"/>
-      <c r="G22" s="85"/>
-      <c r="H22" s="85"/>
+      <c r="G22" s="69"/>
+      <c r="H22" s="69"/>
       <c r="I22" s="13"/>
       <c r="J22" s="13"/>
       <c r="K22" s="13"/>
@@ -4208,16 +4159,16 @@
       <c r="AA22" s="13"/>
     </row>
     <row r="23" spans="2:28" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="150" t="s">
+      <c r="B23" s="133" t="s">
         <v>26</v>
       </c>
-      <c r="C23" s="151"/>
-      <c r="D23" s="151"/>
-      <c r="E23" s="151"/>
-      <c r="F23" s="151"/>
-      <c r="G23" s="151"/>
-      <c r="H23" s="151"/>
-      <c r="I23" s="152"/>
+      <c r="C23" s="134"/>
+      <c r="D23" s="134"/>
+      <c r="E23" s="134"/>
+      <c r="F23" s="134"/>
+      <c r="G23" s="134"/>
+      <c r="H23" s="134"/>
+      <c r="I23" s="135"/>
       <c r="J23" s="13"/>
       <c r="K23" s="13"/>
       <c r="L23" s="13"/>
@@ -4238,20 +4189,20 @@
       <c r="AA23" s="13"/>
     </row>
     <row r="24" spans="2:28" s="9" customFormat="1" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="153" t="s">
+      <c r="B24" s="157" t="s">
         <v>27</v>
       </c>
-      <c r="C24" s="154"/>
-      <c r="D24" s="154"/>
-      <c r="E24" s="154"/>
-      <c r="F24" s="94" t="s">
+      <c r="C24" s="97"/>
+      <c r="D24" s="97"/>
+      <c r="E24" s="97"/>
+      <c r="F24" s="161" t="s">
         <v>28</v>
       </c>
-      <c r="G24" s="94"/>
-      <c r="H24" s="154" t="s">
+      <c r="G24" s="161"/>
+      <c r="H24" s="97" t="s">
         <v>29</v>
       </c>
-      <c r="I24" s="158"/>
+      <c r="I24" s="98"/>
       <c r="J24" s="18"/>
       <c r="K24" s="18"/>
       <c r="M24" s="16"/>
@@ -4264,14 +4215,14 @@
       <c r="AB24" s="10"/>
     </row>
     <row r="25" spans="2:28" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="202"/>
-      <c r="C25" s="157"/>
-      <c r="D25" s="157"/>
-      <c r="E25" s="157"/>
-      <c r="F25" s="157"/>
-      <c r="G25" s="157"/>
-      <c r="H25" s="159"/>
-      <c r="I25" s="160"/>
+      <c r="B25" s="131"/>
+      <c r="C25" s="132"/>
+      <c r="D25" s="132"/>
+      <c r="E25" s="132"/>
+      <c r="F25" s="132"/>
+      <c r="G25" s="132"/>
+      <c r="H25" s="99"/>
+      <c r="I25" s="100"/>
       <c r="J25" s="18"/>
       <c r="K25" s="18"/>
       <c r="M25" s="18"/>
@@ -4288,8 +4239,8 @@
       <c r="D26" s="13"/>
       <c r="E26" s="33"/>
       <c r="F26" s="33"/>
-      <c r="G26" s="85"/>
-      <c r="H26" s="85"/>
+      <c r="G26" s="69"/>
+      <c r="H26" s="69"/>
       <c r="I26" s="13"/>
       <c r="J26" s="13"/>
       <c r="K26" s="13"/>
@@ -4311,16 +4262,16 @@
       <c r="AA26" s="13"/>
     </row>
     <row r="27" spans="2:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B27" s="199" t="s">
+      <c r="B27" s="128" t="s">
         <v>30</v>
       </c>
-      <c r="C27" s="200"/>
-      <c r="D27" s="200"/>
-      <c r="E27" s="200"/>
-      <c r="F27" s="200"/>
-      <c r="G27" s="200"/>
-      <c r="H27" s="200"/>
-      <c r="I27" s="201"/>
+      <c r="C27" s="129"/>
+      <c r="D27" s="129"/>
+      <c r="E27" s="129"/>
+      <c r="F27" s="129"/>
+      <c r="G27" s="129"/>
+      <c r="H27" s="129"/>
+      <c r="I27" s="130"/>
       <c r="J27" s="13"/>
       <c r="K27" s="13"/>
       <c r="L27" s="13"/>
@@ -4341,22 +4292,22 @@
       <c r="AA27" s="13"/>
     </row>
     <row r="28" spans="2:28" s="9" customFormat="1" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B28" s="161" t="s">
+      <c r="B28" s="101" t="s">
         <v>31</v>
       </c>
-      <c r="C28" s="154"/>
-      <c r="D28" s="154"/>
-      <c r="E28" s="94" t="s">
+      <c r="C28" s="97"/>
+      <c r="D28" s="97"/>
+      <c r="E28" s="161" t="s">
         <v>32</v>
       </c>
-      <c r="F28" s="94"/>
+      <c r="F28" s="161"/>
       <c r="G28" s="49" t="s">
         <v>33</v>
       </c>
-      <c r="H28" s="154" t="s">
+      <c r="H28" s="97" t="s">
         <v>34</v>
       </c>
-      <c r="I28" s="162"/>
+      <c r="I28" s="104"/>
       <c r="J28" s="16"/>
       <c r="N28" s="16"/>
       <c r="O28" s="16"/>
@@ -4373,14 +4324,14 @@
       <c r="AB28" s="10"/>
     </row>
     <row r="29" spans="2:28" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B29" s="93"/>
-      <c r="C29" s="58"/>
-      <c r="D29" s="58"/>
-      <c r="E29" s="58"/>
-      <c r="F29" s="58"/>
+      <c r="B29" s="102"/>
+      <c r="C29" s="103"/>
+      <c r="D29" s="103"/>
+      <c r="E29" s="103"/>
+      <c r="F29" s="103"/>
       <c r="G29" s="52"/>
-      <c r="H29" s="58"/>
-      <c r="I29" s="92"/>
+      <c r="H29" s="103"/>
+      <c r="I29" s="194"/>
       <c r="J29" s="18"/>
       <c r="N29" s="18"/>
       <c r="O29" s="18"/>
@@ -4401,8 +4352,8 @@
       <c r="D30" s="13"/>
       <c r="E30" s="33"/>
       <c r="F30" s="33"/>
-      <c r="G30" s="85"/>
-      <c r="H30" s="85"/>
+      <c r="G30" s="69"/>
+      <c r="H30" s="69"/>
       <c r="I30" s="13"/>
       <c r="J30" s="13"/>
       <c r="K30" s="13"/>
@@ -4424,16 +4375,16 @@
       <c r="AA30" s="13"/>
     </row>
     <row r="31" spans="2:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B31" s="150" t="s">
+      <c r="B31" s="133" t="s">
         <v>35</v>
       </c>
-      <c r="C31" s="151"/>
-      <c r="D31" s="151"/>
-      <c r="E31" s="151"/>
-      <c r="F31" s="151"/>
-      <c r="G31" s="151"/>
-      <c r="H31" s="151"/>
-      <c r="I31" s="152"/>
+      <c r="C31" s="134"/>
+      <c r="D31" s="134"/>
+      <c r="E31" s="134"/>
+      <c r="F31" s="134"/>
+      <c r="G31" s="134"/>
+      <c r="H31" s="134"/>
+      <c r="I31" s="135"/>
       <c r="J31" s="7"/>
       <c r="K31" s="7"/>
       <c r="L31" s="7"/>
@@ -4455,18 +4406,18 @@
       <c r="AB31" s="7"/>
     </row>
     <row r="32" spans="2:28" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B32" s="95" t="s">
+      <c r="B32" s="195" t="s">
         <v>36</v>
       </c>
-      <c r="C32" s="96"/>
-      <c r="D32" s="96"/>
-      <c r="E32" s="96"/>
-      <c r="F32" s="97"/>
-      <c r="G32" s="101" t="s">
+      <c r="C32" s="196"/>
+      <c r="D32" s="196"/>
+      <c r="E32" s="196"/>
+      <c r="F32" s="197"/>
+      <c r="G32" s="201" t="s">
         <v>37</v>
       </c>
-      <c r="H32" s="96"/>
-      <c r="I32" s="102"/>
+      <c r="H32" s="196"/>
+      <c r="I32" s="202"/>
       <c r="J32" s="7"/>
       <c r="K32" s="7"/>
       <c r="L32" s="7"/>
@@ -4488,18 +4439,18 @@
       <c r="AB32" s="7"/>
     </row>
     <row r="33" spans="2:28" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B33" s="98" t="s">
+      <c r="B33" s="198" t="s">
         <v>104</v>
       </c>
-      <c r="C33" s="99"/>
-      <c r="D33" s="99"/>
-      <c r="E33" s="99"/>
-      <c r="F33" s="100"/>
-      <c r="G33" s="103" t="s">
+      <c r="C33" s="199"/>
+      <c r="D33" s="199"/>
+      <c r="E33" s="199"/>
+      <c r="F33" s="200"/>
+      <c r="G33" s="203" t="s">
         <v>105</v>
       </c>
-      <c r="H33" s="99"/>
-      <c r="I33" s="104"/>
+      <c r="H33" s="199"/>
+      <c r="I33" s="204"/>
       <c r="J33" s="7"/>
       <c r="K33" s="7"/>
       <c r="L33" s="7"/>
@@ -4526,8 +4477,8 @@
       <c r="D34" s="13"/>
       <c r="E34" s="33"/>
       <c r="F34" s="33"/>
-      <c r="G34" s="85"/>
-      <c r="H34" s="85"/>
+      <c r="G34" s="69"/>
+      <c r="H34" s="69"/>
       <c r="I34" s="13"/>
       <c r="J34" s="13"/>
       <c r="K34" s="13"/>
@@ -4549,16 +4500,16 @@
       <c r="AA34" s="13"/>
     </row>
     <row r="35" spans="2:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B35" s="219" t="s">
+      <c r="B35" s="89" t="s">
         <v>38</v>
       </c>
-      <c r="C35" s="220"/>
-      <c r="D35" s="220"/>
-      <c r="E35" s="220"/>
-      <c r="F35" s="220"/>
-      <c r="G35" s="220"/>
-      <c r="H35" s="220"/>
-      <c r="I35" s="221"/>
+      <c r="C35" s="90"/>
+      <c r="D35" s="90"/>
+      <c r="E35" s="90"/>
+      <c r="F35" s="90"/>
+      <c r="G35" s="90"/>
+      <c r="H35" s="90"/>
+      <c r="I35" s="91"/>
       <c r="J35" s="39"/>
       <c r="K35" s="19"/>
       <c r="L35" s="19"/>
@@ -4582,19 +4533,19 @@
       <c r="B36" s="41" t="s">
         <v>39</v>
       </c>
-      <c r="C36" s="137" t="s">
+      <c r="C36" s="138" t="s">
         <v>40</v>
       </c>
-      <c r="D36" s="138"/>
-      <c r="E36" s="138"/>
-      <c r="F36" s="139"/>
+      <c r="D36" s="139"/>
+      <c r="E36" s="139"/>
+      <c r="F36" s="140"/>
       <c r="G36" s="41" t="s">
         <v>39</v>
       </c>
-      <c r="H36" s="135" t="s">
+      <c r="H36" s="136" t="s">
         <v>41</v>
       </c>
-      <c r="I36" s="136"/>
+      <c r="I36" s="137"/>
       <c r="J36" s="40"/>
       <c r="K36" s="19"/>
       <c r="L36" s="19"/>
@@ -4615,18 +4566,18 @@
       <c r="AA36" s="20"/>
     </row>
     <row r="37" spans="2:28" s="11" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B37" s="169" t="s">
+      <c r="B37" s="83" t="s">
         <v>42</v>
       </c>
-      <c r="C37" s="183"/>
-      <c r="D37" s="184"/>
-      <c r="E37" s="184"/>
-      <c r="F37" s="185"/>
-      <c r="G37" s="169" t="s">
+      <c r="C37" s="112"/>
+      <c r="D37" s="113"/>
+      <c r="E37" s="113"/>
+      <c r="F37" s="114"/>
+      <c r="G37" s="83" t="s">
         <v>43</v>
       </c>
-      <c r="H37" s="163"/>
-      <c r="I37" s="164"/>
+      <c r="H37" s="92"/>
+      <c r="I37" s="93"/>
       <c r="J37" s="39"/>
       <c r="K37" s="16"/>
       <c r="L37" s="18"/>
@@ -4645,14 +4596,14 @@
       <c r="AB37" s="12"/>
     </row>
     <row r="38" spans="2:28" s="11" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B38" s="170"/>
-      <c r="C38" s="186"/>
-      <c r="D38" s="85"/>
-      <c r="E38" s="85"/>
-      <c r="F38" s="187"/>
-      <c r="G38" s="172"/>
-      <c r="H38" s="165"/>
-      <c r="I38" s="166"/>
+      <c r="B38" s="107"/>
+      <c r="C38" s="115"/>
+      <c r="D38" s="69"/>
+      <c r="E38" s="69"/>
+      <c r="F38" s="116"/>
+      <c r="G38" s="109"/>
+      <c r="H38" s="94"/>
+      <c r="I38" s="95"/>
       <c r="J38" s="39"/>
       <c r="K38" s="16"/>
       <c r="L38" s="18"/>
@@ -4670,16 +4621,16 @@
       <c r="AB38" s="12"/>
     </row>
     <row r="39" spans="2:28" s="11" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B39" s="170"/>
-      <c r="C39" s="186"/>
-      <c r="D39" s="85"/>
-      <c r="E39" s="85"/>
-      <c r="F39" s="187"/>
-      <c r="G39" s="169" t="s">
+      <c r="B39" s="107"/>
+      <c r="C39" s="115"/>
+      <c r="D39" s="69"/>
+      <c r="E39" s="69"/>
+      <c r="F39" s="116"/>
+      <c r="G39" s="83" t="s">
         <v>44</v>
       </c>
-      <c r="H39" s="163"/>
-      <c r="I39" s="164"/>
+      <c r="H39" s="92"/>
+      <c r="I39" s="93"/>
       <c r="J39" s="39"/>
       <c r="K39" s="16"/>
       <c r="L39" s="18"/>
@@ -4698,14 +4649,14 @@
       <c r="AB39" s="12"/>
     </row>
     <row r="40" spans="2:28" s="11" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B40" s="171"/>
-      <c r="C40" s="188"/>
-      <c r="D40" s="189"/>
-      <c r="E40" s="189"/>
-      <c r="F40" s="190"/>
-      <c r="G40" s="172"/>
-      <c r="H40" s="165"/>
-      <c r="I40" s="166"/>
+      <c r="B40" s="108"/>
+      <c r="C40" s="117"/>
+      <c r="D40" s="118"/>
+      <c r="E40" s="118"/>
+      <c r="F40" s="119"/>
+      <c r="G40" s="109"/>
+      <c r="H40" s="94"/>
+      <c r="I40" s="95"/>
       <c r="J40" s="39"/>
       <c r="K40" s="16"/>
       <c r="L40" s="18"/>
@@ -4724,18 +4675,18 @@
       <c r="AB40" s="12"/>
     </row>
     <row r="41" spans="2:28" s="11" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B41" s="197" t="s">
+      <c r="B41" s="126" t="s">
         <v>45</v>
       </c>
-      <c r="C41" s="191"/>
-      <c r="D41" s="192"/>
-      <c r="E41" s="192"/>
-      <c r="F41" s="193"/>
-      <c r="G41" s="169" t="s">
+      <c r="C41" s="120"/>
+      <c r="D41" s="121"/>
+      <c r="E41" s="121"/>
+      <c r="F41" s="122"/>
+      <c r="G41" s="83" t="s">
         <v>46</v>
       </c>
-      <c r="H41" s="215"/>
-      <c r="I41" s="216"/>
+      <c r="H41" s="85"/>
+      <c r="I41" s="86"/>
       <c r="J41" s="56"/>
       <c r="K41" s="16"/>
       <c r="L41" s="17"/>
@@ -4757,14 +4708,14 @@
       <c r="AB41" s="12"/>
     </row>
     <row r="42" spans="2:28" s="38" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B42" s="198"/>
-      <c r="C42" s="194"/>
-      <c r="D42" s="195"/>
-      <c r="E42" s="195"/>
-      <c r="F42" s="196"/>
-      <c r="G42" s="214"/>
-      <c r="H42" s="217"/>
-      <c r="I42" s="218"/>
+      <c r="B42" s="127"/>
+      <c r="C42" s="123"/>
+      <c r="D42" s="124"/>
+      <c r="E42" s="124"/>
+      <c r="F42" s="125"/>
+      <c r="G42" s="84"/>
+      <c r="H42" s="87"/>
+      <c r="I42" s="88"/>
       <c r="J42" s="56"/>
       <c r="K42" s="16"/>
       <c r="L42" s="17"/>
@@ -4791,8 +4742,8 @@
       <c r="D43" s="43"/>
       <c r="E43" s="43"/>
       <c r="F43" s="43"/>
-      <c r="G43" s="178"/>
-      <c r="H43" s="179"/>
+      <c r="G43" s="110"/>
+      <c r="H43" s="111"/>
       <c r="I43" s="43"/>
       <c r="J43" s="56"/>
       <c r="K43" s="16"/>
@@ -4815,16 +4766,16 @@
       <c r="AB43" s="12"/>
     </row>
     <row r="44" spans="2:28" s="11" customFormat="1" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B44" s="167" t="s">
+      <c r="B44" s="105" t="s">
         <v>47</v>
       </c>
-      <c r="C44" s="167"/>
-      <c r="D44" s="167"/>
-      <c r="E44" s="167"/>
-      <c r="F44" s="167"/>
-      <c r="G44" s="167"/>
-      <c r="H44" s="167"/>
-      <c r="I44" s="168"/>
+      <c r="C44" s="105"/>
+      <c r="D44" s="105"/>
+      <c r="E44" s="105"/>
+      <c r="F44" s="105"/>
+      <c r="G44" s="105"/>
+      <c r="H44" s="105"/>
+      <c r="I44" s="106"/>
       <c r="J44" s="16"/>
       <c r="K44" s="16"/>
       <c r="L44" s="17"/>
@@ -4846,24 +4797,24 @@
       <c r="AB44" s="12"/>
     </row>
     <row r="45" spans="2:28" ht="68.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B45" s="176" t="s">
+      <c r="B45" s="209" t="s">
         <v>48</v>
       </c>
-      <c r="C45" s="177"/>
-      <c r="D45" s="180" t="s">
+      <c r="C45" s="210"/>
+      <c r="D45" s="211" t="s">
         <v>49</v>
       </c>
-      <c r="E45" s="181"/>
-      <c r="F45" s="175" t="s">
+      <c r="E45" s="212"/>
+      <c r="F45" s="208" t="s">
         <v>50</v>
       </c>
-      <c r="G45" s="175" t="s">
+      <c r="G45" s="208" t="s">
         <v>51</v>
       </c>
-      <c r="H45" s="173" t="s">
+      <c r="H45" s="206" t="s">
         <v>52</v>
       </c>
-      <c r="I45" s="213" t="s">
+      <c r="I45" s="82" t="s">
         <v>53</v>
       </c>
       <c r="J45" s="16"/>
@@ -4886,14 +4837,14 @@
       <c r="AA45" s="16"/>
     </row>
     <row r="46" spans="2:28" ht="66.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B46" s="176"/>
-      <c r="C46" s="177"/>
-      <c r="D46" s="182"/>
-      <c r="E46" s="177"/>
-      <c r="F46" s="209"/>
-      <c r="G46" s="175"/>
-      <c r="H46" s="174"/>
-      <c r="I46" s="213"/>
+      <c r="B46" s="209"/>
+      <c r="C46" s="210"/>
+      <c r="D46" s="213"/>
+      <c r="E46" s="210"/>
+      <c r="F46" s="214"/>
+      <c r="G46" s="208"/>
+      <c r="H46" s="207"/>
+      <c r="I46" s="82"/>
       <c r="J46" s="16"/>
       <c r="K46" s="16"/>
       <c r="L46" s="16"/>
@@ -4914,14 +4865,14 @@
       <c r="AA46" s="16"/>
     </row>
     <row r="47" spans="2:28" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B47" s="89"/>
-      <c r="C47" s="57"/>
-      <c r="D47" s="57"/>
-      <c r="E47" s="57"/>
-      <c r="F47" s="90"/>
-      <c r="G47" s="57"/>
-      <c r="H47" s="57"/>
-      <c r="I47" s="91"/>
+      <c r="B47" s="192"/>
+      <c r="C47" s="193"/>
+      <c r="D47" s="193"/>
+      <c r="E47" s="193"/>
+      <c r="F47" s="205"/>
+      <c r="G47" s="193"/>
+      <c r="H47" s="193"/>
+      <c r="I47" s="191"/>
       <c r="J47" s="18"/>
       <c r="K47" s="16"/>
       <c r="L47" s="16"/>
@@ -4942,14 +4893,14 @@
       <c r="AA47" s="16"/>
     </row>
     <row r="48" spans="2:28" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B48" s="89"/>
-      <c r="C48" s="57"/>
-      <c r="D48" s="57"/>
-      <c r="E48" s="57"/>
-      <c r="F48" s="90"/>
-      <c r="G48" s="57"/>
-      <c r="H48" s="57"/>
-      <c r="I48" s="91"/>
+      <c r="B48" s="192"/>
+      <c r="C48" s="193"/>
+      <c r="D48" s="193"/>
+      <c r="E48" s="193"/>
+      <c r="F48" s="205"/>
+      <c r="G48" s="193"/>
+      <c r="H48" s="193"/>
+      <c r="I48" s="191"/>
       <c r="J48" s="18"/>
       <c r="K48" s="16"/>
       <c r="L48" s="16"/>
@@ -4970,14 +4921,14 @@
       <c r="AA48" s="16"/>
     </row>
     <row r="49" spans="2:28" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B49" s="89"/>
-      <c r="C49" s="57"/>
-      <c r="D49" s="57"/>
-      <c r="E49" s="57"/>
-      <c r="F49" s="90"/>
-      <c r="G49" s="57"/>
-      <c r="H49" s="57"/>
-      <c r="I49" s="91"/>
+      <c r="B49" s="192"/>
+      <c r="C49" s="193"/>
+      <c r="D49" s="193"/>
+      <c r="E49" s="193"/>
+      <c r="F49" s="205"/>
+      <c r="G49" s="193"/>
+      <c r="H49" s="193"/>
+      <c r="I49" s="191"/>
       <c r="J49" s="18"/>
       <c r="K49" s="16"/>
       <c r="L49" s="16"/>
@@ -4998,14 +4949,14 @@
       <c r="AA49" s="16"/>
     </row>
     <row r="50" spans="2:28" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B50" s="89"/>
-      <c r="C50" s="57"/>
-      <c r="D50" s="57"/>
-      <c r="E50" s="57"/>
-      <c r="F50" s="90"/>
-      <c r="G50" s="57"/>
-      <c r="H50" s="57"/>
-      <c r="I50" s="91"/>
+      <c r="B50" s="192"/>
+      <c r="C50" s="193"/>
+      <c r="D50" s="193"/>
+      <c r="E50" s="193"/>
+      <c r="F50" s="205"/>
+      <c r="G50" s="193"/>
+      <c r="H50" s="193"/>
+      <c r="I50" s="191"/>
       <c r="J50" s="18"/>
       <c r="K50" s="16"/>
       <c r="L50" s="16"/>
@@ -5026,14 +4977,14 @@
       <c r="AA50" s="16"/>
     </row>
     <row r="51" spans="2:28" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B51" s="89"/>
-      <c r="C51" s="57"/>
-      <c r="D51" s="57"/>
-      <c r="E51" s="57"/>
-      <c r="F51" s="90"/>
-      <c r="G51" s="57"/>
-      <c r="H51" s="57"/>
-      <c r="I51" s="91"/>
+      <c r="B51" s="192"/>
+      <c r="C51" s="193"/>
+      <c r="D51" s="193"/>
+      <c r="E51" s="193"/>
+      <c r="F51" s="205"/>
+      <c r="G51" s="193"/>
+      <c r="H51" s="193"/>
+      <c r="I51" s="191"/>
       <c r="J51" s="18"/>
       <c r="K51" s="16"/>
       <c r="L51" s="16"/>
@@ -5054,14 +5005,14 @@
       <c r="AA51" s="16"/>
     </row>
     <row r="52" spans="2:28" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B52" s="89"/>
-      <c r="C52" s="57"/>
-      <c r="D52" s="57"/>
-      <c r="E52" s="57"/>
-      <c r="F52" s="90"/>
-      <c r="G52" s="57"/>
-      <c r="H52" s="57"/>
-      <c r="I52" s="91"/>
+      <c r="B52" s="192"/>
+      <c r="C52" s="193"/>
+      <c r="D52" s="193"/>
+      <c r="E52" s="193"/>
+      <c r="F52" s="205"/>
+      <c r="G52" s="193"/>
+      <c r="H52" s="193"/>
+      <c r="I52" s="191"/>
       <c r="J52" s="18"/>
       <c r="K52" s="16"/>
       <c r="L52" s="16"/>
@@ -5082,14 +5033,14 @@
       <c r="AA52" s="16"/>
     </row>
     <row r="53" spans="2:28" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B53" s="89"/>
-      <c r="C53" s="57"/>
-      <c r="D53" s="57"/>
-      <c r="E53" s="57"/>
-      <c r="F53" s="90"/>
-      <c r="G53" s="57"/>
-      <c r="H53" s="57"/>
-      <c r="I53" s="91"/>
+      <c r="B53" s="192"/>
+      <c r="C53" s="193"/>
+      <c r="D53" s="193"/>
+      <c r="E53" s="193"/>
+      <c r="F53" s="205"/>
+      <c r="G53" s="193"/>
+      <c r="H53" s="193"/>
+      <c r="I53" s="191"/>
       <c r="J53" s="18"/>
       <c r="K53" s="16"/>
       <c r="L53" s="16"/>
@@ -5110,14 +5061,14 @@
       <c r="AA53" s="16"/>
     </row>
     <row r="54" spans="2:28" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B54" s="89"/>
-      <c r="C54" s="57"/>
-      <c r="D54" s="57"/>
-      <c r="E54" s="57"/>
-      <c r="F54" s="90"/>
-      <c r="G54" s="57"/>
-      <c r="H54" s="57"/>
-      <c r="I54" s="91"/>
+      <c r="B54" s="192"/>
+      <c r="C54" s="193"/>
+      <c r="D54" s="193"/>
+      <c r="E54" s="193"/>
+      <c r="F54" s="205"/>
+      <c r="G54" s="193"/>
+      <c r="H54" s="193"/>
+      <c r="I54" s="191"/>
       <c r="J54" s="18"/>
       <c r="K54" s="16"/>
       <c r="L54" s="16"/>
@@ -5138,14 +5089,14 @@
       <c r="AA54" s="16"/>
     </row>
     <row r="55" spans="2:28" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B55" s="89"/>
-      <c r="C55" s="57"/>
-      <c r="D55" s="57"/>
-      <c r="E55" s="57"/>
-      <c r="F55" s="90"/>
-      <c r="G55" s="57"/>
-      <c r="H55" s="57"/>
-      <c r="I55" s="91"/>
+      <c r="B55" s="192"/>
+      <c r="C55" s="193"/>
+      <c r="D55" s="193"/>
+      <c r="E55" s="193"/>
+      <c r="F55" s="205"/>
+      <c r="G55" s="193"/>
+      <c r="H55" s="193"/>
+      <c r="I55" s="191"/>
       <c r="J55" s="18"/>
       <c r="K55" s="16"/>
       <c r="L55" s="16"/>
@@ -5166,14 +5117,14 @@
       <c r="AA55" s="16"/>
     </row>
     <row r="56" spans="2:28" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B56" s="93"/>
-      <c r="C56" s="58"/>
-      <c r="D56" s="58"/>
-      <c r="E56" s="58"/>
-      <c r="F56" s="134"/>
-      <c r="G56" s="58"/>
-      <c r="H56" s="58"/>
-      <c r="I56" s="92"/>
+      <c r="B56" s="102"/>
+      <c r="C56" s="103"/>
+      <c r="D56" s="103"/>
+      <c r="E56" s="103"/>
+      <c r="F56" s="241"/>
+      <c r="G56" s="103"/>
+      <c r="H56" s="103"/>
+      <c r="I56" s="194"/>
       <c r="J56" s="18"/>
       <c r="K56" s="16"/>
       <c r="L56" s="16"/>
@@ -5199,8 +5150,8 @@
       <c r="D57" s="18"/>
       <c r="E57" s="23"/>
       <c r="F57" s="23"/>
-      <c r="G57" s="86"/>
-      <c r="H57" s="86"/>
+      <c r="G57" s="190"/>
+      <c r="H57" s="190"/>
       <c r="I57" s="18"/>
       <c r="J57" s="18"/>
       <c r="K57" s="16"/>
@@ -5222,16 +5173,16 @@
       <c r="AA57" s="16"/>
     </row>
     <row r="58" spans="2:28" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B58" s="66" t="s">
+      <c r="B58" s="215" t="s">
         <v>54</v>
       </c>
-      <c r="C58" s="67"/>
-      <c r="D58" s="67"/>
-      <c r="E58" s="67"/>
-      <c r="F58" s="67"/>
-      <c r="G58" s="67"/>
-      <c r="H58" s="67"/>
-      <c r="I58" s="68"/>
+      <c r="C58" s="216"/>
+      <c r="D58" s="216"/>
+      <c r="E58" s="216"/>
+      <c r="F58" s="216"/>
+      <c r="G58" s="216"/>
+      <c r="H58" s="216"/>
+      <c r="I58" s="217"/>
       <c r="J58" s="18"/>
       <c r="K58" s="16"/>
       <c r="L58" s="16"/>
@@ -5252,16 +5203,16 @@
       <c r="AA58" s="16"/>
     </row>
     <row r="59" spans="2:28" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B59" s="222" t="s">
+      <c r="B59" s="61" t="s">
         <v>55</v>
       </c>
-      <c r="C59" s="223"/>
-      <c r="D59" s="223"/>
-      <c r="E59" s="223"/>
-      <c r="F59" s="223"/>
-      <c r="G59" s="223"/>
-      <c r="H59" s="223"/>
-      <c r="I59" s="224"/>
+      <c r="C59" s="62"/>
+      <c r="D59" s="62"/>
+      <c r="E59" s="62"/>
+      <c r="F59" s="62"/>
+      <c r="G59" s="62"/>
+      <c r="H59" s="62"/>
+      <c r="I59" s="63"/>
       <c r="J59" s="19"/>
       <c r="K59" s="19"/>
       <c r="L59" s="19"/>
@@ -5282,16 +5233,16 @@
       <c r="AA59" s="19"/>
     </row>
     <row r="60" spans="2:28" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B60" s="66" t="s">
+      <c r="B60" s="215" t="s">
         <v>56</v>
       </c>
-      <c r="C60" s="67"/>
-      <c r="D60" s="67"/>
-      <c r="E60" s="67"/>
-      <c r="F60" s="67"/>
-      <c r="G60" s="67"/>
-      <c r="H60" s="67"/>
-      <c r="I60" s="68"/>
+      <c r="C60" s="216"/>
+      <c r="D60" s="216"/>
+      <c r="E60" s="216"/>
+      <c r="F60" s="216"/>
+      <c r="G60" s="216"/>
+      <c r="H60" s="216"/>
+      <c r="I60" s="217"/>
       <c r="J60" s="19"/>
       <c r="K60" s="19"/>
       <c r="L60" s="19"/>
@@ -5312,16 +5263,16 @@
       <c r="AA60" s="19"/>
     </row>
     <row r="61" spans="2:28" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B61" s="70" t="s">
+      <c r="B61" s="230" t="s">
         <v>57</v>
       </c>
-      <c r="C61" s="71"/>
-      <c r="D61" s="71"/>
-      <c r="E61" s="71"/>
-      <c r="F61" s="71"/>
-      <c r="G61" s="71"/>
-      <c r="H61" s="71"/>
-      <c r="I61" s="72"/>
+      <c r="C61" s="231"/>
+      <c r="D61" s="231"/>
+      <c r="E61" s="231"/>
+      <c r="F61" s="231"/>
+      <c r="G61" s="231"/>
+      <c r="H61" s="231"/>
+      <c r="I61" s="232"/>
       <c r="J61" s="22"/>
       <c r="K61" s="22"/>
       <c r="L61" s="22"/>
@@ -5342,14 +5293,14 @@
       <c r="AA61" s="22"/>
     </row>
     <row r="62" spans="2:28" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B62" s="73"/>
-      <c r="C62" s="74"/>
-      <c r="D62" s="74"/>
-      <c r="E62" s="74"/>
-      <c r="F62" s="74"/>
-      <c r="G62" s="74"/>
-      <c r="H62" s="74"/>
-      <c r="I62" s="75"/>
+      <c r="B62" s="233"/>
+      <c r="C62" s="234"/>
+      <c r="D62" s="234"/>
+      <c r="E62" s="234"/>
+      <c r="F62" s="234"/>
+      <c r="G62" s="234"/>
+      <c r="H62" s="234"/>
+      <c r="I62" s="235"/>
       <c r="J62" s="22"/>
       <c r="K62" s="22"/>
       <c r="L62" s="22"/>
@@ -5370,16 +5321,16 @@
       <c r="AA62" s="22"/>
     </row>
     <row r="63" spans="2:28" s="46" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B63" s="73" t="s">
+      <c r="B63" s="233" t="s">
         <v>58</v>
       </c>
-      <c r="C63" s="74"/>
-      <c r="D63" s="74"/>
-      <c r="E63" s="74"/>
-      <c r="F63" s="74"/>
-      <c r="G63" s="74"/>
-      <c r="H63" s="74"/>
-      <c r="I63" s="75"/>
+      <c r="C63" s="234"/>
+      <c r="D63" s="234"/>
+      <c r="E63" s="234"/>
+      <c r="F63" s="234"/>
+      <c r="G63" s="234"/>
+      <c r="H63" s="234"/>
+      <c r="I63" s="235"/>
       <c r="J63" s="44"/>
       <c r="K63" s="44"/>
       <c r="L63" s="44"/>
@@ -5401,16 +5352,16 @@
       <c r="AB63" s="45"/>
     </row>
     <row r="64" spans="2:28" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B64" s="78" t="s">
+      <c r="B64" s="236" t="s">
         <v>59</v>
       </c>
-      <c r="C64" s="79"/>
-      <c r="D64" s="79"/>
-      <c r="E64" s="79"/>
-      <c r="F64" s="79"/>
-      <c r="G64" s="79"/>
-      <c r="H64" s="79"/>
-      <c r="I64" s="80"/>
+      <c r="C64" s="237"/>
+      <c r="D64" s="237"/>
+      <c r="E64" s="237"/>
+      <c r="F64" s="237"/>
+      <c r="G64" s="237"/>
+      <c r="H64" s="237"/>
+      <c r="I64" s="238"/>
       <c r="J64" s="22"/>
       <c r="K64" s="22"/>
       <c r="L64" s="22"/>
@@ -5434,19 +5385,19 @@
       <c r="B65" s="50" t="s">
         <v>60</v>
       </c>
-      <c r="C65" s="76" t="s">
+      <c r="C65" s="221" t="s">
         <v>61</v>
       </c>
-      <c r="D65" s="76"/>
-      <c r="E65" s="76" t="s">
+      <c r="D65" s="221"/>
+      <c r="E65" s="221" t="s">
         <v>62</v>
       </c>
-      <c r="F65" s="76"/>
-      <c r="G65" s="266"/>
-      <c r="H65" s="76" t="s">
+      <c r="F65" s="221"/>
+      <c r="G65" s="73"/>
+      <c r="H65" s="221" t="s">
         <v>63</v>
       </c>
-      <c r="I65" s="268"/>
+      <c r="I65" s="75"/>
       <c r="J65" s="16"/>
       <c r="K65" s="16"/>
       <c r="L65" s="16"/>
@@ -5469,13 +5420,13 @@
     </row>
     <row r="66" spans="2:28" ht="32.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B66" s="51"/>
-      <c r="C66" s="83"/>
-      <c r="D66" s="83"/>
-      <c r="E66" s="77"/>
-      <c r="F66" s="77"/>
-      <c r="G66" s="267"/>
-      <c r="H66" s="77"/>
-      <c r="I66" s="269"/>
+      <c r="C66" s="239"/>
+      <c r="D66" s="239"/>
+      <c r="E66" s="222"/>
+      <c r="F66" s="222"/>
+      <c r="G66" s="74"/>
+      <c r="H66" s="222"/>
+      <c r="I66" s="76"/>
       <c r="J66" s="16"/>
       <c r="K66" s="16"/>
       <c r="L66" s="16"/>
@@ -5502,8 +5453,8 @@
       <c r="D67" s="17"/>
       <c r="E67" s="34"/>
       <c r="F67" s="34"/>
-      <c r="G67" s="81"/>
-      <c r="H67" s="81"/>
+      <c r="G67" s="218"/>
+      <c r="H67" s="218"/>
       <c r="I67" s="17"/>
       <c r="J67" s="16"/>
       <c r="K67" s="16"/>
@@ -5526,16 +5477,16 @@
       <c r="AB67" s="16"/>
     </row>
     <row r="68" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B68" s="69" t="s">
+      <c r="B68" s="229" t="s">
         <v>64</v>
       </c>
-      <c r="C68" s="69"/>
-      <c r="D68" s="69"/>
-      <c r="E68" s="69"/>
-      <c r="F68" s="69"/>
-      <c r="G68" s="69"/>
-      <c r="H68" s="69"/>
-      <c r="I68" s="69"/>
+      <c r="C68" s="229"/>
+      <c r="D68" s="229"/>
+      <c r="E68" s="229"/>
+      <c r="F68" s="229"/>
+      <c r="G68" s="229"/>
+      <c r="H68" s="229"/>
+      <c r="I68" s="229"/>
       <c r="J68" s="16"/>
       <c r="K68" s="16"/>
       <c r="L68" s="16"/>
@@ -5562,8 +5513,8 @@
       <c r="D69" s="15"/>
       <c r="E69" s="35"/>
       <c r="F69" s="35"/>
-      <c r="G69" s="82"/>
-      <c r="H69" s="82"/>
+      <c r="G69" s="67"/>
+      <c r="H69" s="67"/>
       <c r="I69" s="15"/>
       <c r="J69" s="16"/>
       <c r="K69" s="16"/>
@@ -5586,13 +5537,13 @@
       <c r="AB69" s="16"/>
     </row>
     <row r="70" spans="2:28" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B70" s="82"/>
-      <c r="C70" s="82"/>
-      <c r="D70" s="82"/>
-      <c r="E70" s="82"/>
+      <c r="B70" s="67"/>
+      <c r="C70" s="67"/>
+      <c r="D70" s="67"/>
+      <c r="E70" s="67"/>
       <c r="F70" s="35"/>
-      <c r="G70" s="82"/>
-      <c r="H70" s="82"/>
+      <c r="G70" s="67"/>
+      <c r="H70" s="67"/>
       <c r="I70" s="15"/>
       <c r="J70" s="16"/>
       <c r="K70" s="16"/>
@@ -5615,12 +5566,12 @@
       <c r="AB70" s="16"/>
     </row>
     <row r="71" spans="2:28" ht="36" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B71" s="262"/>
-      <c r="C71" s="262"/>
-      <c r="D71" s="262"/>
-      <c r="E71" s="262"/>
+      <c r="B71" s="68"/>
+      <c r="C71" s="68"/>
+      <c r="D71" s="68"/>
+      <c r="E71" s="68"/>
       <c r="F71" s="26"/>
-      <c r="H71" s="271"/>
+      <c r="H71" s="57"/>
       <c r="I71" s="16"/>
       <c r="J71" s="16"/>
       <c r="K71" s="16"/>
@@ -5643,12 +5594,12 @@
       <c r="AB71" s="16"/>
     </row>
     <row r="72" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B72" s="65" t="s">
+      <c r="B72" s="220" t="s">
         <v>65</v>
       </c>
-      <c r="C72" s="65"/>
-      <c r="D72" s="65"/>
-      <c r="E72" s="65"/>
+      <c r="C72" s="220"/>
+      <c r="D72" s="220"/>
+      <c r="E72" s="220"/>
       <c r="F72" s="17"/>
       <c r="H72" s="17" t="s">
         <v>66</v>
@@ -5680,8 +5631,8 @@
       <c r="D73" s="16"/>
       <c r="E73" s="26"/>
       <c r="F73" s="26"/>
-      <c r="G73" s="87"/>
-      <c r="H73" s="208"/>
+      <c r="G73" s="60"/>
+      <c r="H73" s="96"/>
       <c r="I73" s="16"/>
       <c r="J73" s="16"/>
       <c r="K73" s="16"/>
@@ -5704,13 +5655,13 @@
       <c r="AB73" s="16"/>
     </row>
     <row r="74" spans="2:28" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B74" s="264"/>
-      <c r="C74" s="264"/>
-      <c r="D74" s="264"/>
-      <c r="E74" s="264"/>
+      <c r="B74" s="71"/>
+      <c r="C74" s="71"/>
+      <c r="D74" s="71"/>
+      <c r="E74" s="71"/>
       <c r="F74" s="26"/>
-      <c r="H74" s="85"/>
-      <c r="I74" s="85"/>
+      <c r="H74" s="69"/>
+      <c r="I74" s="69"/>
       <c r="J74" s="16"/>
       <c r="K74" s="16"/>
       <c r="L74" s="16"/>
@@ -5732,13 +5683,13 @@
       <c r="AB74" s="16"/>
     </row>
     <row r="75" spans="2:28" ht="38.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B75" s="265"/>
-      <c r="C75" s="265"/>
-      <c r="D75" s="265"/>
-      <c r="E75" s="265"/>
+      <c r="B75" s="72"/>
+      <c r="C75" s="72"/>
+      <c r="D75" s="72"/>
+      <c r="E75" s="72"/>
       <c r="F75" s="26"/>
-      <c r="H75" s="263"/>
-      <c r="I75" s="263"/>
+      <c r="H75" s="70"/>
+      <c r="I75" s="70"/>
       <c r="J75" s="16"/>
       <c r="K75" s="16"/>
       <c r="L75" s="16"/>
@@ -5767,10 +5718,10 @@
       <c r="D76" s="24"/>
       <c r="E76" s="26"/>
       <c r="F76" s="26"/>
-      <c r="H76" s="65" t="s">
+      <c r="H76" s="220" t="s">
         <v>68</v>
       </c>
-      <c r="I76" s="65"/>
+      <c r="I76" s="220"/>
       <c r="J76" s="16"/>
       <c r="K76" s="16"/>
       <c r="L76" s="16"/>
@@ -5797,8 +5748,8 @@
       <c r="D77" s="24"/>
       <c r="E77" s="26"/>
       <c r="F77" s="26"/>
-      <c r="G77" s="87"/>
-      <c r="H77" s="81"/>
+      <c r="G77" s="60"/>
+      <c r="H77" s="218"/>
       <c r="I77" s="17"/>
       <c r="J77" s="16"/>
       <c r="K77" s="16"/>
@@ -5821,16 +5772,16 @@
       <c r="AB77" s="16"/>
     </row>
     <row r="78" spans="2:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B78" s="84" t="s">
+      <c r="B78" s="240" t="s">
         <v>69</v>
       </c>
-      <c r="C78" s="84"/>
-      <c r="D78" s="84"/>
-      <c r="E78" s="84"/>
-      <c r="F78" s="84"/>
-      <c r="G78" s="84"/>
-      <c r="H78" s="84"/>
-      <c r="I78" s="84"/>
+      <c r="C78" s="240"/>
+      <c r="D78" s="240"/>
+      <c r="E78" s="240"/>
+      <c r="F78" s="240"/>
+      <c r="G78" s="240"/>
+      <c r="H78" s="240"/>
+      <c r="I78" s="240"/>
       <c r="J78" s="16"/>
       <c r="K78" s="16"/>
       <c r="L78" s="16"/>
@@ -5852,14 +5803,14 @@
       <c r="AB78" s="16"/>
     </row>
     <row r="79" spans="2:28" x14ac:dyDescent="0.25">
-      <c r="B79" s="84"/>
-      <c r="C79" s="84"/>
-      <c r="D79" s="84"/>
-      <c r="E79" s="84"/>
-      <c r="F79" s="84"/>
-      <c r="G79" s="84"/>
-      <c r="H79" s="84"/>
-      <c r="I79" s="84"/>
+      <c r="B79" s="240"/>
+      <c r="C79" s="240"/>
+      <c r="D79" s="240"/>
+      <c r="E79" s="240"/>
+      <c r="F79" s="240"/>
+      <c r="G79" s="240"/>
+      <c r="H79" s="240"/>
+      <c r="I79" s="240"/>
       <c r="J79" s="16"/>
       <c r="K79" s="16"/>
       <c r="L79" s="16"/>
@@ -5886,8 +5837,8 @@
       <c r="D80" s="48"/>
       <c r="E80" s="48"/>
       <c r="F80" s="48"/>
-      <c r="G80" s="88"/>
-      <c r="H80" s="88"/>
+      <c r="G80" s="219"/>
+      <c r="H80" s="219"/>
       <c r="I80" s="48"/>
       <c r="J80" s="16"/>
       <c r="K80" s="16"/>
@@ -5910,16 +5861,16 @@
       <c r="AB80" s="16"/>
     </row>
     <row r="81" spans="2:28" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B81" s="59" t="s">
+      <c r="B81" s="223" t="s">
         <v>70</v>
       </c>
-      <c r="C81" s="60"/>
-      <c r="D81" s="60"/>
-      <c r="E81" s="60"/>
-      <c r="F81" s="60"/>
-      <c r="G81" s="60"/>
-      <c r="H81" s="60"/>
-      <c r="I81" s="61"/>
+      <c r="C81" s="224"/>
+      <c r="D81" s="224"/>
+      <c r="E81" s="224"/>
+      <c r="F81" s="224"/>
+      <c r="G81" s="224"/>
+      <c r="H81" s="224"/>
+      <c r="I81" s="225"/>
       <c r="J81" s="8"/>
       <c r="K81" s="7"/>
       <c r="L81" s="7"/>
@@ -5941,16 +5892,16 @@
       <c r="AB81" s="7"/>
     </row>
     <row r="82" spans="2:28" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B82" s="62" t="s">
+      <c r="B82" s="226" t="s">
         <v>71</v>
       </c>
-      <c r="C82" s="63"/>
-      <c r="D82" s="63"/>
-      <c r="E82" s="63"/>
-      <c r="F82" s="63"/>
-      <c r="G82" s="63"/>
-      <c r="H82" s="63"/>
-      <c r="I82" s="64"/>
+      <c r="C82" s="227"/>
+      <c r="D82" s="227"/>
+      <c r="E82" s="227"/>
+      <c r="F82" s="227"/>
+      <c r="G82" s="227"/>
+      <c r="H82" s="227"/>
+      <c r="I82" s="228"/>
       <c r="J82" s="8"/>
       <c r="K82" s="25"/>
       <c r="L82" s="7"/>
@@ -5972,18 +5923,18 @@
       <c r="AB82" s="7"/>
     </row>
     <row r="83" spans="2:28" s="8" customFormat="1" ht="48" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B83" s="259"/>
-      <c r="C83" s="260"/>
-      <c r="D83" s="260"/>
-      <c r="E83" s="260"/>
-      <c r="F83" s="260"/>
-      <c r="G83" s="260"/>
-      <c r="H83" s="260"/>
-      <c r="I83" s="261"/>
+      <c r="B83" s="64"/>
+      <c r="C83" s="65"/>
+      <c r="D83" s="65"/>
+      <c r="E83" s="65"/>
+      <c r="F83" s="65"/>
+      <c r="G83" s="65"/>
+      <c r="H83" s="65"/>
+      <c r="I83" s="66"/>
     </row>
     <row r="84" spans="2:28" hidden="1" x14ac:dyDescent="0.25">
-      <c r="G84" s="87"/>
-      <c r="H84" s="87"/>
+      <c r="G84" s="60"/>
+      <c r="H84" s="60"/>
       <c r="J84" s="8"/>
       <c r="K84" s="7"/>
       <c r="L84" s="7"/>
@@ -6005,141 +5956,247 @@
       <c r="AB84" s="7"/>
     </row>
     <row r="85" spans="2:28" hidden="1" x14ac:dyDescent="0.25">
-      <c r="G85" s="87"/>
-      <c r="H85" s="87"/>
+      <c r="G85" s="60"/>
+      <c r="H85" s="60"/>
     </row>
     <row r="86" spans="2:28" hidden="1" x14ac:dyDescent="0.25">
-      <c r="G86" s="87"/>
-      <c r="H86" s="87"/>
+      <c r="G86" s="60"/>
+      <c r="H86" s="60"/>
     </row>
     <row r="87" spans="2:28" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G87" s="87"/>
-      <c r="H87" s="87"/>
+      <c r="G87" s="60"/>
+      <c r="H87" s="60"/>
     </row>
     <row r="88" spans="2:28" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G88" s="87"/>
-      <c r="H88" s="87"/>
+      <c r="G88" s="60"/>
+      <c r="H88" s="60"/>
     </row>
     <row r="89" spans="2:28" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G89" s="87"/>
-      <c r="H89" s="87"/>
+      <c r="G89" s="60"/>
+      <c r="H89" s="60"/>
     </row>
     <row r="90" spans="2:28" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G90" s="87"/>
-      <c r="H90" s="87"/>
+      <c r="G90" s="60"/>
+      <c r="H90" s="60"/>
     </row>
     <row r="91" spans="2:28" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G91" s="87"/>
-      <c r="H91" s="87"/>
+      <c r="G91" s="60"/>
+      <c r="H91" s="60"/>
     </row>
     <row r="92" spans="2:28" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G92" s="87"/>
-      <c r="H92" s="87"/>
+      <c r="G92" s="60"/>
+      <c r="H92" s="60"/>
     </row>
     <row r="93" spans="2:28" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G93" s="87"/>
-      <c r="H93" s="87"/>
+      <c r="G93" s="60"/>
+      <c r="H93" s="60"/>
     </row>
     <row r="94" spans="2:28" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G94" s="87"/>
-      <c r="H94" s="87"/>
+      <c r="G94" s="60"/>
+      <c r="H94" s="60"/>
     </row>
     <row r="95" spans="2:28" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G95" s="87"/>
-      <c r="H95" s="87"/>
+      <c r="G95" s="60"/>
+      <c r="H95" s="60"/>
     </row>
     <row r="96" spans="2:28" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G96" s="87"/>
-      <c r="H96" s="87"/>
+      <c r="G96" s="60"/>
+      <c r="H96" s="60"/>
     </row>
     <row r="97" spans="7:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G97" s="87"/>
-      <c r="H97" s="87"/>
+      <c r="G97" s="60"/>
+      <c r="H97" s="60"/>
     </row>
     <row r="98" spans="7:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G98" s="87"/>
-      <c r="H98" s="87"/>
+      <c r="G98" s="60"/>
+      <c r="H98" s="60"/>
     </row>
     <row r="99" spans="7:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G99" s="87"/>
-      <c r="H99" s="87"/>
+      <c r="G99" s="60"/>
+      <c r="H99" s="60"/>
     </row>
     <row r="100" spans="7:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G100" s="87"/>
-      <c r="H100" s="87"/>
+      <c r="G100" s="60"/>
+      <c r="H100" s="60"/>
     </row>
     <row r="101" spans="7:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G101" s="87"/>
-      <c r="H101" s="87"/>
+      <c r="G101" s="60"/>
+      <c r="H101" s="60"/>
     </row>
     <row r="102" spans="7:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G102" s="87"/>
-      <c r="H102" s="87"/>
+      <c r="G102" s="60"/>
+      <c r="H102" s="60"/>
     </row>
     <row r="103" spans="7:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G103" s="87"/>
-      <c r="H103" s="87"/>
+      <c r="G103" s="60"/>
+      <c r="H103" s="60"/>
     </row>
     <row r="104" spans="7:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G104" s="87"/>
-      <c r="H104" s="87"/>
+      <c r="G104" s="60"/>
+      <c r="H104" s="60"/>
     </row>
     <row r="105" spans="7:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G105" s="87"/>
-      <c r="H105" s="87"/>
+      <c r="G105" s="60"/>
+      <c r="H105" s="60"/>
     </row>
     <row r="106" spans="7:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G106" s="87"/>
-      <c r="H106" s="87"/>
+      <c r="G106" s="60"/>
+      <c r="H106" s="60"/>
     </row>
     <row r="107" spans="7:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G107" s="87"/>
-      <c r="H107" s="87"/>
+      <c r="G107" s="60"/>
+      <c r="H107" s="60"/>
     </row>
     <row r="108" spans="7:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G108" s="87"/>
-      <c r="H108" s="87"/>
+      <c r="G108" s="60"/>
+      <c r="H108" s="60"/>
     </row>
     <row r="109" spans="7:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G109" s="87"/>
-      <c r="H109" s="87"/>
+      <c r="G109" s="60"/>
+      <c r="H109" s="60"/>
     </row>
     <row r="110" spans="7:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G110" s="87"/>
-      <c r="H110" s="87"/>
+      <c r="G110" s="60"/>
+      <c r="H110" s="60"/>
     </row>
     <row r="111" spans="7:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G111" s="87"/>
-      <c r="H111" s="87"/>
+      <c r="G111" s="60"/>
+      <c r="H111" s="60"/>
     </row>
     <row r="112" spans="7:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G112" s="87"/>
-      <c r="H112" s="87"/>
+      <c r="G112" s="60"/>
+      <c r="H112" s="60"/>
     </row>
     <row r="113" spans="7:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G113" s="87"/>
-      <c r="H113" s="87"/>
+      <c r="G113" s="60"/>
+      <c r="H113" s="60"/>
     </row>
   </sheetData>
   <mergeCells count="171">
-    <mergeCell ref="G112:H112"/>
-    <mergeCell ref="G113:H113"/>
-    <mergeCell ref="B59:I59"/>
-    <mergeCell ref="G106:H106"/>
-    <mergeCell ref="G107:H107"/>
-    <mergeCell ref="G108:H108"/>
-    <mergeCell ref="G109:H109"/>
-    <mergeCell ref="G110:H110"/>
-    <mergeCell ref="G101:H101"/>
-    <mergeCell ref="G102:H102"/>
-    <mergeCell ref="G103:H103"/>
-    <mergeCell ref="G104:H104"/>
-    <mergeCell ref="B83:I83"/>
-    <mergeCell ref="B70:E71"/>
-    <mergeCell ref="H74:I75"/>
-    <mergeCell ref="B74:E75"/>
-    <mergeCell ref="G65:G66"/>
-    <mergeCell ref="I65:I66"/>
+    <mergeCell ref="B55:C56"/>
+    <mergeCell ref="D55:E56"/>
+    <mergeCell ref="B81:I81"/>
+    <mergeCell ref="B82:I82"/>
+    <mergeCell ref="B72:E72"/>
+    <mergeCell ref="B60:I60"/>
+    <mergeCell ref="B68:I68"/>
+    <mergeCell ref="B61:I62"/>
+    <mergeCell ref="B63:I63"/>
+    <mergeCell ref="H65:H66"/>
+    <mergeCell ref="B64:I64"/>
+    <mergeCell ref="G67:H67"/>
+    <mergeCell ref="G69:H69"/>
+    <mergeCell ref="G70:H70"/>
+    <mergeCell ref="C65:D65"/>
+    <mergeCell ref="C66:D66"/>
+    <mergeCell ref="B78:I79"/>
+    <mergeCell ref="F55:F56"/>
+    <mergeCell ref="G55:G56"/>
+    <mergeCell ref="H55:H56"/>
+    <mergeCell ref="D45:E46"/>
+    <mergeCell ref="F45:F46"/>
+    <mergeCell ref="G26:H26"/>
+    <mergeCell ref="B58:I58"/>
+    <mergeCell ref="G57:H57"/>
+    <mergeCell ref="G77:H77"/>
+    <mergeCell ref="G80:H80"/>
+    <mergeCell ref="D47:E48"/>
+    <mergeCell ref="B47:C48"/>
+    <mergeCell ref="F47:F48"/>
+    <mergeCell ref="G47:G48"/>
+    <mergeCell ref="H47:H48"/>
+    <mergeCell ref="I47:I48"/>
+    <mergeCell ref="B49:C50"/>
+    <mergeCell ref="D49:E50"/>
+    <mergeCell ref="F49:F50"/>
+    <mergeCell ref="G49:G50"/>
+    <mergeCell ref="H49:H50"/>
+    <mergeCell ref="I49:I50"/>
+    <mergeCell ref="B51:C52"/>
+    <mergeCell ref="D51:E52"/>
+    <mergeCell ref="F51:F52"/>
+    <mergeCell ref="I55:I56"/>
+    <mergeCell ref="H76:I76"/>
+    <mergeCell ref="B16:D16"/>
+    <mergeCell ref="E16:G16"/>
+    <mergeCell ref="B13:I13"/>
+    <mergeCell ref="E10:I10"/>
+    <mergeCell ref="E11:I11"/>
+    <mergeCell ref="B10:D10"/>
+    <mergeCell ref="B11:D11"/>
+    <mergeCell ref="G9:H9"/>
+    <mergeCell ref="G12:H12"/>
+    <mergeCell ref="B3:I3"/>
+    <mergeCell ref="B5:I5"/>
+    <mergeCell ref="B4:I4"/>
+    <mergeCell ref="B6:I6"/>
+    <mergeCell ref="B7:I7"/>
+    <mergeCell ref="H14:I14"/>
+    <mergeCell ref="H15:I15"/>
+    <mergeCell ref="B14:D14"/>
+    <mergeCell ref="B15:D15"/>
+    <mergeCell ref="C8:D8"/>
+    <mergeCell ref="E8:F8"/>
+    <mergeCell ref="F14:G14"/>
+    <mergeCell ref="F15:G15"/>
+    <mergeCell ref="B23:I23"/>
+    <mergeCell ref="B24:E24"/>
+    <mergeCell ref="H21:I21"/>
+    <mergeCell ref="E21:G21"/>
+    <mergeCell ref="E20:G20"/>
+    <mergeCell ref="F24:G24"/>
+    <mergeCell ref="F25:G25"/>
+    <mergeCell ref="G105:H105"/>
+    <mergeCell ref="G96:H96"/>
+    <mergeCell ref="G97:H97"/>
+    <mergeCell ref="G98:H98"/>
+    <mergeCell ref="G99:H99"/>
+    <mergeCell ref="G100:H100"/>
+    <mergeCell ref="G91:H91"/>
+    <mergeCell ref="G92:H92"/>
+    <mergeCell ref="G93:H93"/>
+    <mergeCell ref="G94:H94"/>
+    <mergeCell ref="G95:H95"/>
+    <mergeCell ref="I51:I52"/>
+    <mergeCell ref="B53:C54"/>
+    <mergeCell ref="H29:I29"/>
+    <mergeCell ref="E28:F28"/>
+    <mergeCell ref="E29:F29"/>
+    <mergeCell ref="B32:F32"/>
+    <mergeCell ref="B17:D17"/>
+    <mergeCell ref="H20:I20"/>
+    <mergeCell ref="B20:D20"/>
+    <mergeCell ref="B21:D21"/>
+    <mergeCell ref="E18:G18"/>
+    <mergeCell ref="H18:I18"/>
+    <mergeCell ref="E19:G19"/>
+    <mergeCell ref="H19:I19"/>
+    <mergeCell ref="B18:D18"/>
+    <mergeCell ref="B19:D19"/>
+    <mergeCell ref="G39:G40"/>
+    <mergeCell ref="G43:H43"/>
+    <mergeCell ref="C37:F40"/>
+    <mergeCell ref="C41:F42"/>
+    <mergeCell ref="B41:B42"/>
+    <mergeCell ref="B27:I27"/>
+    <mergeCell ref="B25:E25"/>
+    <mergeCell ref="B31:I31"/>
+    <mergeCell ref="G86:H86"/>
+    <mergeCell ref="H36:I36"/>
+    <mergeCell ref="C36:F36"/>
+    <mergeCell ref="B33:F33"/>
+    <mergeCell ref="G32:I32"/>
+    <mergeCell ref="G33:I33"/>
+    <mergeCell ref="D53:E54"/>
+    <mergeCell ref="F53:F54"/>
+    <mergeCell ref="G53:G54"/>
+    <mergeCell ref="H53:H54"/>
+    <mergeCell ref="I53:I54"/>
+    <mergeCell ref="G51:G52"/>
+    <mergeCell ref="H51:H52"/>
+    <mergeCell ref="H45:H46"/>
+    <mergeCell ref="G45:G46"/>
+    <mergeCell ref="B45:C46"/>
     <mergeCell ref="E17:G17"/>
     <mergeCell ref="H16:I16"/>
     <mergeCell ref="H17:I17"/>
@@ -6164,147 +6221,41 @@
     <mergeCell ref="B44:I44"/>
     <mergeCell ref="B37:B40"/>
     <mergeCell ref="G37:G38"/>
-    <mergeCell ref="G39:G40"/>
-    <mergeCell ref="G43:H43"/>
-    <mergeCell ref="C37:F40"/>
-    <mergeCell ref="C41:F42"/>
-    <mergeCell ref="B41:B42"/>
-    <mergeCell ref="B27:I27"/>
-    <mergeCell ref="B25:E25"/>
-    <mergeCell ref="B31:I31"/>
-    <mergeCell ref="G86:H86"/>
+    <mergeCell ref="G112:H112"/>
+    <mergeCell ref="G113:H113"/>
+    <mergeCell ref="B59:I59"/>
+    <mergeCell ref="G106:H106"/>
+    <mergeCell ref="G107:H107"/>
+    <mergeCell ref="G108:H108"/>
+    <mergeCell ref="G109:H109"/>
+    <mergeCell ref="G110:H110"/>
+    <mergeCell ref="G101:H101"/>
+    <mergeCell ref="G102:H102"/>
+    <mergeCell ref="G103:H103"/>
+    <mergeCell ref="G104:H104"/>
+    <mergeCell ref="B83:I83"/>
+    <mergeCell ref="B70:E71"/>
+    <mergeCell ref="H74:I75"/>
+    <mergeCell ref="B74:E75"/>
+    <mergeCell ref="G65:G66"/>
+    <mergeCell ref="I65:I66"/>
     <mergeCell ref="G87:H87"/>
     <mergeCell ref="G88:H88"/>
     <mergeCell ref="G89:H89"/>
     <mergeCell ref="G90:H90"/>
-    <mergeCell ref="H36:I36"/>
-    <mergeCell ref="C36:F36"/>
-    <mergeCell ref="B17:D17"/>
-    <mergeCell ref="H20:I20"/>
-    <mergeCell ref="B20:D20"/>
-    <mergeCell ref="B21:D21"/>
-    <mergeCell ref="E18:G18"/>
-    <mergeCell ref="H18:I18"/>
-    <mergeCell ref="E19:G19"/>
-    <mergeCell ref="H19:I19"/>
-    <mergeCell ref="B18:D18"/>
-    <mergeCell ref="B19:D19"/>
-    <mergeCell ref="B23:I23"/>
-    <mergeCell ref="B24:E24"/>
-    <mergeCell ref="H21:I21"/>
-    <mergeCell ref="E21:G21"/>
-    <mergeCell ref="E20:G20"/>
-    <mergeCell ref="F24:G24"/>
-    <mergeCell ref="F25:G25"/>
-    <mergeCell ref="G105:H105"/>
-    <mergeCell ref="G96:H96"/>
-    <mergeCell ref="G97:H97"/>
-    <mergeCell ref="G98:H98"/>
-    <mergeCell ref="G99:H99"/>
-    <mergeCell ref="G100:H100"/>
-    <mergeCell ref="G91:H91"/>
-    <mergeCell ref="G92:H92"/>
-    <mergeCell ref="G93:H93"/>
-    <mergeCell ref="G94:H94"/>
-    <mergeCell ref="G95:H95"/>
-    <mergeCell ref="B3:I3"/>
-    <mergeCell ref="B5:I5"/>
-    <mergeCell ref="B4:I4"/>
-    <mergeCell ref="B6:I6"/>
-    <mergeCell ref="B7:I7"/>
-    <mergeCell ref="H14:I14"/>
-    <mergeCell ref="H15:I15"/>
-    <mergeCell ref="B14:D14"/>
-    <mergeCell ref="B15:D15"/>
-    <mergeCell ref="C8:D8"/>
-    <mergeCell ref="E8:F8"/>
-    <mergeCell ref="F14:G14"/>
-    <mergeCell ref="F15:G15"/>
-    <mergeCell ref="B16:D16"/>
-    <mergeCell ref="E16:G16"/>
-    <mergeCell ref="B13:I13"/>
-    <mergeCell ref="E10:I10"/>
-    <mergeCell ref="E11:I11"/>
-    <mergeCell ref="B10:D10"/>
-    <mergeCell ref="B11:D11"/>
-    <mergeCell ref="G9:H9"/>
-    <mergeCell ref="G12:H12"/>
-    <mergeCell ref="I51:I52"/>
-    <mergeCell ref="B53:C54"/>
-    <mergeCell ref="H29:I29"/>
-    <mergeCell ref="E28:F28"/>
-    <mergeCell ref="E29:F29"/>
-    <mergeCell ref="B32:F32"/>
-    <mergeCell ref="B33:F33"/>
-    <mergeCell ref="G32:I32"/>
-    <mergeCell ref="G33:I33"/>
-    <mergeCell ref="D53:E54"/>
-    <mergeCell ref="F53:F54"/>
-    <mergeCell ref="G53:G54"/>
-    <mergeCell ref="H53:H54"/>
-    <mergeCell ref="I53:I54"/>
-    <mergeCell ref="G51:G52"/>
-    <mergeCell ref="H51:H52"/>
-    <mergeCell ref="H45:H46"/>
-    <mergeCell ref="G45:G46"/>
-    <mergeCell ref="B45:C46"/>
-    <mergeCell ref="D45:E46"/>
-    <mergeCell ref="F45:F46"/>
-    <mergeCell ref="G26:H26"/>
-    <mergeCell ref="B58:I58"/>
-    <mergeCell ref="G57:H57"/>
-    <mergeCell ref="G77:H77"/>
-    <mergeCell ref="G80:H80"/>
-    <mergeCell ref="D47:E48"/>
-    <mergeCell ref="B47:C48"/>
-    <mergeCell ref="F47:F48"/>
-    <mergeCell ref="G47:G48"/>
-    <mergeCell ref="H47:H48"/>
-    <mergeCell ref="I47:I48"/>
-    <mergeCell ref="B49:C50"/>
-    <mergeCell ref="D49:E50"/>
-    <mergeCell ref="F49:F50"/>
-    <mergeCell ref="G49:G50"/>
-    <mergeCell ref="H49:H50"/>
-    <mergeCell ref="I49:I50"/>
-    <mergeCell ref="B51:C52"/>
-    <mergeCell ref="D51:E52"/>
-    <mergeCell ref="F51:F52"/>
-    <mergeCell ref="I55:I56"/>
-    <mergeCell ref="H76:I76"/>
     <mergeCell ref="E65:F66"/>
-    <mergeCell ref="B55:C56"/>
-    <mergeCell ref="D55:E56"/>
-    <mergeCell ref="B81:I81"/>
-    <mergeCell ref="B82:I82"/>
-    <mergeCell ref="B72:E72"/>
-    <mergeCell ref="B60:I60"/>
-    <mergeCell ref="B68:I68"/>
-    <mergeCell ref="B61:I62"/>
-    <mergeCell ref="B63:I63"/>
-    <mergeCell ref="H65:H66"/>
-    <mergeCell ref="B64:I64"/>
-    <mergeCell ref="G67:H67"/>
-    <mergeCell ref="G69:H69"/>
-    <mergeCell ref="G70:H70"/>
-    <mergeCell ref="C65:D65"/>
-    <mergeCell ref="C66:D66"/>
-    <mergeCell ref="B78:I79"/>
-    <mergeCell ref="F55:F56"/>
-    <mergeCell ref="G55:G56"/>
-    <mergeCell ref="H55:H56"/>
   </mergeCells>
-  <conditionalFormatting sqref="B11:I11 B15:I15 B17:I17 B19:I19 B21:I21 B25:I25 B29:I29 C37:F42 H37:I42 B47:I56 B70:E71 B74:E75 H74:I75 B83:I83">
-    <cfRule type="containsBlanks" dxfId="6" priority="3">
+  <conditionalFormatting sqref="B11:I11 B15:I15 B17:I17 B19:I19 B21:I21 B25:I25 B29:I29 C37:F42 H37:I42 B47:I56 B70:E71 H74:I75 B83:I83">
+    <cfRule type="containsBlanks" dxfId="3" priority="3">
       <formula>LEN(TRIM(B11))=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B66:D66 G65:G66 I65:I66 H71">
-    <cfRule type="containsBlanks" dxfId="5" priority="4">
+  <conditionalFormatting sqref="G65:G66 I65:I66 B66:D66 H71">
+    <cfRule type="containsBlanks" dxfId="2" priority="4">
       <formula>LEN(TRIM(B65))=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations xWindow="1156" yWindow="532" count="37">
+  <dataValidations xWindow="1156" yWindow="532" count="36">
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Desde dd/mm/aa hasta dd/mm/aa" prompt="Ingresar la fehca de inicio y fin de la bitácora" sqref="E11:I11" xr:uid="{CD2FA053-183B-41CA-B267-B4277B8CA158}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Desplegar y seleccionar" prompt="Desplegar y seleccionar el numero de bitacora actual" sqref="B11:D11" xr:uid="{3D01CEB2-123B-4C72-96E2-63C296030E46}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Ingresar Nombres y apellidos de aprendiz, tal como regista en su docuemnto de identificacion" sqref="B15:D15" xr:uid="{A585EB3A-7529-4958-B886-65F5282307D7}"/>
@@ -6330,10 +6281,9 @@
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Ingresar la competencia del programa que abarca la actividad realizada, debe ser de las competencias concertadas inicialmente en el formato F023 visita 1" sqref="D47:E56" xr:uid="{0D8BD481-B72E-43AC-9736-661B2F1B5B5C}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Ingresar fecha de inicio de la actividad" sqref="F47:F56" xr:uid="{32DD5E98-EAF7-430B-97F3-79C3622F702E}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Ingresar fecha de finalizacion de la actividad" sqref="G47:G56" xr:uid="{145C53F1-D232-49E6-A4AB-B178BD1CDE8E}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="NO VAN CAPTURAS DE PANTALLA" prompt="Ejemplo 1: Documento: Documento (material del curso de diseño web revisado y aplicado. _x000a_Ejemplo 2:  Proceso (validación de ejecución de parchados_x000a_en servidores)._x000a_Ejemplo 3: Producto: Aplicacion WEB (Se aclara son ejemplos)" sqref="H55:H56" xr:uid="{1B955B8F-68CD-419F-B5E8-35AC173B4957}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="NO VAN CAPTURAS DE PANTALLA" prompt="Ejemplo 1: Documento: Documento (material del curso de diseño web revisado y aplicado. _x000a_Ejemplo 2:  Proceso (validación de ejecución de parchados_x000a_en servidores)._x000a_Ejemplo 3: Producto: Aplicacion WEB (Se aclara son ejemplos)" sqref="H49:H56" xr:uid="{1B955B8F-68CD-419F-B5E8-35AC173B4957}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="NO VAN CAPTURAS DE PANTALLA" prompt="Si se presentan situaciones relevantes en el desarrollo de la actividad, favor relacionarla. (Ejemplo, retrasos, incumplimientos. etc). SI POR TEMAS DE CONFIDENCIALIDAD D ELA INFORMACION NO SE PUEDEN ANEXAR CAPTURAS, FAVOR DEJARLO POR ESCRITO ACA." sqref="I47:I56" xr:uid="{67EE6F84-95FA-40E8-86A9-4393D2B1D5BB}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="NO VAN CAPTURAS DE PANTALLA" prompt="Ejemplo 1: Documento: Documento (material del curso de diseño web revisado y aplicado. _x000a_Ejemplo 2:  Proceso (validación de ejecución de parchados_x000a_en servidores)._x000a_Ejemplo 3: Producto: Aplicacion WEB (Se aclara son ejemplos). NO VAN CAPTURAS DE PANTALLA" sqref="H47:H48" xr:uid="{CBCC16C2-11EE-4F06-BE98-4BF1A24BDE5E}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="NO VAN CAPTURAS DE PANTALLA" prompt="Ejemplo 1: Documento: Documento (material del curso de diseño web revisado y aplicado. _x000a_Ejemplo 2:  Proceso (validación de ejecución de parchados_x000a_en servidores)._x000a_Ejemplo 3: Producto: Aplicacion WEB (Se aclara son ejemplos)" sqref="H49:H50 H51:H52 H53:H54" xr:uid="{A6E5627A-DA4C-474D-9B26-651BDA97F470}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Si / NO" prompt="Si / NO" sqref="B66" xr:uid="{399AC36A-2FBC-4A36-BEF2-DB6479D0AE91}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Indiquie el nivel asignado de riego del 1 al 5" sqref="C66:D66" xr:uid="{0B51F00F-01A3-4D67-B07C-4E070A35CC22}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Si / No" prompt="Si / No" sqref="G65:G66" xr:uid="{635C8396-AD4E-4569-B1B1-E0EA70CFBAA0}"/>
@@ -6430,124 +6380,124 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:24" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A1" s="251" t="s">
+      <c r="A1" s="242" t="s">
         <v>72</v>
       </c>
-      <c r="B1" s="251"/>
-      <c r="C1" s="251"/>
-      <c r="D1" s="251"/>
-      <c r="E1" s="251"/>
-      <c r="F1" s="251"/>
-      <c r="G1" s="251"/>
-      <c r="H1" s="251"/>
-      <c r="I1" s="251"/>
-      <c r="J1" s="251"/>
-      <c r="K1" s="251"/>
-      <c r="L1" s="251"/>
-      <c r="M1" s="251"/>
-      <c r="N1" s="251"/>
-      <c r="O1" s="251"/>
-      <c r="P1" s="251"/>
-      <c r="Q1" s="251"/>
-      <c r="R1" s="251"/>
-      <c r="S1" s="251"/>
-      <c r="T1" s="251"/>
-      <c r="U1" s="251" t="s">
+      <c r="B1" s="242"/>
+      <c r="C1" s="242"/>
+      <c r="D1" s="242"/>
+      <c r="E1" s="242"/>
+      <c r="F1" s="242"/>
+      <c r="G1" s="242"/>
+      <c r="H1" s="242"/>
+      <c r="I1" s="242"/>
+      <c r="J1" s="242"/>
+      <c r="K1" s="242"/>
+      <c r="L1" s="242"/>
+      <c r="M1" s="242"/>
+      <c r="N1" s="242"/>
+      <c r="O1" s="242"/>
+      <c r="P1" s="242"/>
+      <c r="Q1" s="242"/>
+      <c r="R1" s="242"/>
+      <c r="S1" s="242"/>
+      <c r="T1" s="242"/>
+      <c r="U1" s="242" t="s">
         <v>73</v>
       </c>
-      <c r="V1" s="251"/>
-      <c r="W1" s="251"/>
-      <c r="X1" s="251"/>
+      <c r="V1" s="242"/>
+      <c r="W1" s="242"/>
+      <c r="X1" s="242"/>
     </row>
     <row r="2" spans="1:24" ht="33" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="251"/>
-      <c r="B2" s="251"/>
-      <c r="C2" s="251"/>
-      <c r="D2" s="251"/>
-      <c r="E2" s="251"/>
-      <c r="F2" s="251"/>
-      <c r="G2" s="251"/>
-      <c r="H2" s="251"/>
-      <c r="I2" s="251"/>
-      <c r="J2" s="251"/>
-      <c r="K2" s="251"/>
-      <c r="L2" s="251"/>
-      <c r="M2" s="251"/>
-      <c r="N2" s="251"/>
-      <c r="O2" s="251"/>
-      <c r="P2" s="251"/>
-      <c r="Q2" s="251"/>
-      <c r="R2" s="251"/>
-      <c r="S2" s="251"/>
-      <c r="T2" s="251"/>
-      <c r="U2" s="231" t="s">
+      <c r="A2" s="242"/>
+      <c r="B2" s="242"/>
+      <c r="C2" s="242"/>
+      <c r="D2" s="242"/>
+      <c r="E2" s="242"/>
+      <c r="F2" s="242"/>
+      <c r="G2" s="242"/>
+      <c r="H2" s="242"/>
+      <c r="I2" s="242"/>
+      <c r="J2" s="242"/>
+      <c r="K2" s="242"/>
+      <c r="L2" s="242"/>
+      <c r="M2" s="242"/>
+      <c r="N2" s="242"/>
+      <c r="O2" s="242"/>
+      <c r="P2" s="242"/>
+      <c r="Q2" s="242"/>
+      <c r="R2" s="242"/>
+      <c r="S2" s="242"/>
+      <c r="T2" s="242"/>
+      <c r="U2" s="250" t="s">
         <v>74</v>
       </c>
-      <c r="V2" s="231"/>
-      <c r="W2" s="231"/>
-      <c r="X2" s="231"/>
+      <c r="V2" s="250"/>
+      <c r="W2" s="250"/>
+      <c r="X2" s="250"/>
     </row>
     <row r="3" spans="1:24" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="U3" s="258"/>
-      <c r="V3" s="258"/>
-      <c r="W3" s="258"/>
-      <c r="X3" s="258"/>
+      <c r="U3" s="251"/>
+      <c r="V3" s="251"/>
+      <c r="W3" s="251"/>
+      <c r="X3" s="251"/>
     </row>
     <row r="4" spans="1:24" s="2" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="255" t="s">
+      <c r="A4" s="247" t="s">
         <v>75</v>
       </c>
-      <c r="B4" s="256"/>
-      <c r="C4" s="256"/>
-      <c r="D4" s="256"/>
-      <c r="E4" s="256"/>
-      <c r="F4" s="256"/>
-      <c r="G4" s="256"/>
-      <c r="H4" s="256"/>
-      <c r="I4" s="256"/>
-      <c r="J4" s="256"/>
-      <c r="K4" s="256"/>
-      <c r="L4" s="256"/>
-      <c r="M4" s="257"/>
-      <c r="N4" s="255" t="s">
+      <c r="B4" s="248"/>
+      <c r="C4" s="248"/>
+      <c r="D4" s="248"/>
+      <c r="E4" s="248"/>
+      <c r="F4" s="248"/>
+      <c r="G4" s="248"/>
+      <c r="H4" s="248"/>
+      <c r="I4" s="248"/>
+      <c r="J4" s="248"/>
+      <c r="K4" s="248"/>
+      <c r="L4" s="248"/>
+      <c r="M4" s="249"/>
+      <c r="N4" s="247" t="s">
         <v>76</v>
       </c>
-      <c r="O4" s="256"/>
-      <c r="P4" s="256"/>
-      <c r="Q4" s="256"/>
-      <c r="R4" s="256"/>
-      <c r="S4" s="256"/>
-      <c r="T4" s="256"/>
-      <c r="U4" s="256"/>
-      <c r="V4" s="256"/>
-      <c r="W4" s="256"/>
-      <c r="X4" s="257"/>
+      <c r="O4" s="248"/>
+      <c r="P4" s="248"/>
+      <c r="Q4" s="248"/>
+      <c r="R4" s="248"/>
+      <c r="S4" s="248"/>
+      <c r="T4" s="248"/>
+      <c r="U4" s="248"/>
+      <c r="V4" s="248"/>
+      <c r="W4" s="248"/>
+      <c r="X4" s="249"/>
     </row>
     <row r="5" spans="1:24" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="252"/>
-      <c r="B5" s="253"/>
-      <c r="C5" s="253"/>
-      <c r="D5" s="253"/>
-      <c r="E5" s="253"/>
-      <c r="F5" s="253"/>
-      <c r="G5" s="253"/>
-      <c r="H5" s="253"/>
-      <c r="I5" s="253"/>
-      <c r="J5" s="253"/>
-      <c r="K5" s="253"/>
-      <c r="L5" s="253"/>
-      <c r="M5" s="254"/>
-      <c r="N5" s="252"/>
-      <c r="O5" s="253"/>
-      <c r="P5" s="253"/>
-      <c r="Q5" s="253"/>
-      <c r="R5" s="253"/>
-      <c r="S5" s="253"/>
-      <c r="T5" s="253"/>
-      <c r="U5" s="253"/>
-      <c r="V5" s="253"/>
-      <c r="W5" s="253"/>
-      <c r="X5" s="254"/>
+      <c r="A5" s="244"/>
+      <c r="B5" s="245"/>
+      <c r="C5" s="245"/>
+      <c r="D5" s="245"/>
+      <c r="E5" s="245"/>
+      <c r="F5" s="245"/>
+      <c r="G5" s="245"/>
+      <c r="H5" s="245"/>
+      <c r="I5" s="245"/>
+      <c r="J5" s="245"/>
+      <c r="K5" s="245"/>
+      <c r="L5" s="245"/>
+      <c r="M5" s="246"/>
+      <c r="N5" s="244"/>
+      <c r="O5" s="245"/>
+      <c r="P5" s="245"/>
+      <c r="Q5" s="245"/>
+      <c r="R5" s="245"/>
+      <c r="S5" s="245"/>
+      <c r="T5" s="245"/>
+      <c r="U5" s="245"/>
+      <c r="V5" s="245"/>
+      <c r="W5" s="245"/>
+      <c r="X5" s="246"/>
     </row>
     <row r="6" spans="1:24" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3"/>
@@ -6576,66 +6526,66 @@
       <c r="X6" s="3"/>
     </row>
     <row r="7" spans="1:24" s="2" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="229" t="s">
+      <c r="A7" s="243" t="s">
         <v>77</v>
       </c>
-      <c r="B7" s="229"/>
-      <c r="C7" s="229"/>
-      <c r="D7" s="229"/>
-      <c r="E7" s="229"/>
-      <c r="F7" s="229"/>
-      <c r="G7" s="229"/>
-      <c r="H7" s="229"/>
-      <c r="I7" s="229"/>
-      <c r="J7" s="229" t="s">
+      <c r="B7" s="243"/>
+      <c r="C7" s="243"/>
+      <c r="D7" s="243"/>
+      <c r="E7" s="243"/>
+      <c r="F7" s="243"/>
+      <c r="G7" s="243"/>
+      <c r="H7" s="243"/>
+      <c r="I7" s="243"/>
+      <c r="J7" s="243" t="s">
         <v>78</v>
       </c>
-      <c r="K7" s="229"/>
-      <c r="L7" s="229"/>
-      <c r="M7" s="229"/>
-      <c r="N7" s="229"/>
-      <c r="O7" s="229"/>
-      <c r="P7" s="229" t="s">
+      <c r="K7" s="243"/>
+      <c r="L7" s="243"/>
+      <c r="M7" s="243"/>
+      <c r="N7" s="243"/>
+      <c r="O7" s="243"/>
+      <c r="P7" s="243" t="s">
         <v>79</v>
       </c>
-      <c r="Q7" s="229"/>
-      <c r="R7" s="229"/>
-      <c r="S7" s="229"/>
-      <c r="T7" s="229"/>
-      <c r="U7" s="229"/>
-      <c r="V7" s="229"/>
-      <c r="W7" s="229"/>
-      <c r="X7" s="229"/>
+      <c r="Q7" s="243"/>
+      <c r="R7" s="243"/>
+      <c r="S7" s="243"/>
+      <c r="T7" s="243"/>
+      <c r="U7" s="243"/>
+      <c r="V7" s="243"/>
+      <c r="W7" s="243"/>
+      <c r="X7" s="243"/>
     </row>
     <row r="8" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="236"/>
-      <c r="B8" s="236"/>
-      <c r="C8" s="236"/>
-      <c r="D8" s="236"/>
-      <c r="E8" s="236"/>
-      <c r="F8" s="236"/>
-      <c r="G8" s="236"/>
-      <c r="H8" s="236"/>
-      <c r="I8" s="236"/>
-      <c r="J8" s="237" t="s">
+      <c r="A8" s="252"/>
+      <c r="B8" s="252"/>
+      <c r="C8" s="252"/>
+      <c r="D8" s="252"/>
+      <c r="E8" s="252"/>
+      <c r="F8" s="252"/>
+      <c r="G8" s="252"/>
+      <c r="H8" s="252"/>
+      <c r="I8" s="252"/>
+      <c r="J8" s="253" t="s">
         <v>80</v>
       </c>
-      <c r="K8" s="238"/>
-      <c r="L8" s="238"/>
-      <c r="M8" s="238"/>
-      <c r="N8" s="238"/>
-      <c r="O8" s="239"/>
-      <c r="P8" s="237" t="s">
+      <c r="K8" s="254"/>
+      <c r="L8" s="254"/>
+      <c r="M8" s="254"/>
+      <c r="N8" s="254"/>
+      <c r="O8" s="255"/>
+      <c r="P8" s="253" t="s">
         <v>81</v>
       </c>
-      <c r="Q8" s="238"/>
-      <c r="R8" s="238"/>
-      <c r="S8" s="238"/>
-      <c r="T8" s="238"/>
-      <c r="U8" s="238"/>
-      <c r="V8" s="238"/>
-      <c r="W8" s="238"/>
-      <c r="X8" s="239"/>
+      <c r="Q8" s="254"/>
+      <c r="R8" s="254"/>
+      <c r="S8" s="254"/>
+      <c r="T8" s="254"/>
+      <c r="U8" s="254"/>
+      <c r="V8" s="254"/>
+      <c r="W8" s="254"/>
+      <c r="X8" s="255"/>
     </row>
     <row r="9" spans="1:24" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3"/>
@@ -6664,66 +6614,66 @@
       <c r="X9" s="3"/>
     </row>
     <row r="10" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="249" t="s">
+      <c r="A10" s="256" t="s">
         <v>82</v>
       </c>
-      <c r="B10" s="249"/>
-      <c r="C10" s="249"/>
-      <c r="D10" s="249"/>
-      <c r="E10" s="249"/>
-      <c r="F10" s="249"/>
-      <c r="G10" s="249"/>
-      <c r="H10" s="249"/>
-      <c r="I10" s="249"/>
-      <c r="J10" s="249"/>
-      <c r="K10" s="249"/>
-      <c r="L10" s="249"/>
-      <c r="M10" s="249"/>
-      <c r="N10" s="249"/>
-      <c r="O10" s="249"/>
-      <c r="P10" s="249"/>
-      <c r="Q10" s="249"/>
-      <c r="R10" s="249"/>
-      <c r="S10" s="249"/>
-      <c r="T10" s="249"/>
-      <c r="U10" s="249"/>
-      <c r="V10" s="249"/>
-      <c r="W10" s="249"/>
-      <c r="X10" s="249"/>
+      <c r="B10" s="256"/>
+      <c r="C10" s="256"/>
+      <c r="D10" s="256"/>
+      <c r="E10" s="256"/>
+      <c r="F10" s="256"/>
+      <c r="G10" s="256"/>
+      <c r="H10" s="256"/>
+      <c r="I10" s="256"/>
+      <c r="J10" s="256"/>
+      <c r="K10" s="256"/>
+      <c r="L10" s="256"/>
+      <c r="M10" s="256"/>
+      <c r="N10" s="256"/>
+      <c r="O10" s="256"/>
+      <c r="P10" s="256"/>
+      <c r="Q10" s="256"/>
+      <c r="R10" s="256"/>
+      <c r="S10" s="256"/>
+      <c r="T10" s="256"/>
+      <c r="U10" s="256"/>
+      <c r="V10" s="256"/>
+      <c r="W10" s="256"/>
+      <c r="X10" s="256"/>
     </row>
     <row r="11" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="250" t="s">
+      <c r="A11" s="257" t="s">
         <v>83</v>
       </c>
-      <c r="B11" s="250"/>
-      <c r="C11" s="250"/>
-      <c r="D11" s="250"/>
-      <c r="E11" s="250"/>
-      <c r="F11" s="250"/>
-      <c r="G11" s="250" t="s">
+      <c r="B11" s="257"/>
+      <c r="C11" s="257"/>
+      <c r="D11" s="257"/>
+      <c r="E11" s="257"/>
+      <c r="F11" s="257"/>
+      <c r="G11" s="257" t="s">
         <v>84</v>
       </c>
-      <c r="H11" s="250"/>
-      <c r="I11" s="250"/>
-      <c r="J11" s="250"/>
-      <c r="K11" s="250"/>
-      <c r="L11" s="250"/>
-      <c r="M11" s="250" t="s">
+      <c r="H11" s="257"/>
+      <c r="I11" s="257"/>
+      <c r="J11" s="257"/>
+      <c r="K11" s="257"/>
+      <c r="L11" s="257"/>
+      <c r="M11" s="257" t="s">
         <v>85</v>
       </c>
-      <c r="N11" s="250"/>
-      <c r="O11" s="250"/>
-      <c r="P11" s="250"/>
-      <c r="Q11" s="250"/>
-      <c r="R11" s="250"/>
-      <c r="S11" s="250" t="s">
+      <c r="N11" s="257"/>
+      <c r="O11" s="257"/>
+      <c r="P11" s="257"/>
+      <c r="Q11" s="257"/>
+      <c r="R11" s="257"/>
+      <c r="S11" s="257" t="s">
         <v>86</v>
       </c>
-      <c r="T11" s="250"/>
-      <c r="U11" s="250"/>
-      <c r="V11" s="250"/>
-      <c r="W11" s="250"/>
-      <c r="X11" s="250"/>
+      <c r="T11" s="257"/>
+      <c r="U11" s="257"/>
+      <c r="V11" s="257"/>
+      <c r="W11" s="257"/>
+      <c r="X11" s="257"/>
     </row>
     <row r="12" spans="1:24" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3"/>
@@ -6752,66 +6702,66 @@
       <c r="X12" s="3"/>
     </row>
     <row r="13" spans="1:24" s="2" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="229" t="s">
+      <c r="A13" s="243" t="s">
         <v>87</v>
       </c>
-      <c r="B13" s="229"/>
-      <c r="C13" s="229"/>
-      <c r="D13" s="229"/>
-      <c r="E13" s="229"/>
-      <c r="F13" s="229"/>
-      <c r="G13" s="229"/>
-      <c r="H13" s="229"/>
-      <c r="I13" s="229"/>
-      <c r="J13" s="229" t="s">
+      <c r="B13" s="243"/>
+      <c r="C13" s="243"/>
+      <c r="D13" s="243"/>
+      <c r="E13" s="243"/>
+      <c r="F13" s="243"/>
+      <c r="G13" s="243"/>
+      <c r="H13" s="243"/>
+      <c r="I13" s="243"/>
+      <c r="J13" s="243" t="s">
         <v>78</v>
       </c>
-      <c r="K13" s="229"/>
-      <c r="L13" s="229"/>
-      <c r="M13" s="229"/>
-      <c r="N13" s="229"/>
-      <c r="O13" s="229"/>
-      <c r="P13" s="229" t="s">
+      <c r="K13" s="243"/>
+      <c r="L13" s="243"/>
+      <c r="M13" s="243"/>
+      <c r="N13" s="243"/>
+      <c r="O13" s="243"/>
+      <c r="P13" s="243" t="s">
         <v>79</v>
       </c>
-      <c r="Q13" s="229"/>
-      <c r="R13" s="229"/>
-      <c r="S13" s="229"/>
-      <c r="T13" s="229"/>
-      <c r="U13" s="229"/>
-      <c r="V13" s="229"/>
-      <c r="W13" s="229"/>
-      <c r="X13" s="229"/>
+      <c r="Q13" s="243"/>
+      <c r="R13" s="243"/>
+      <c r="S13" s="243"/>
+      <c r="T13" s="243"/>
+      <c r="U13" s="243"/>
+      <c r="V13" s="243"/>
+      <c r="W13" s="243"/>
+      <c r="X13" s="243"/>
     </row>
     <row r="14" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="236"/>
-      <c r="B14" s="236"/>
-      <c r="C14" s="236"/>
-      <c r="D14" s="236"/>
-      <c r="E14" s="236"/>
-      <c r="F14" s="236"/>
-      <c r="G14" s="236"/>
-      <c r="H14" s="236"/>
-      <c r="I14" s="236"/>
-      <c r="J14" s="237" t="s">
+      <c r="A14" s="252"/>
+      <c r="B14" s="252"/>
+      <c r="C14" s="252"/>
+      <c r="D14" s="252"/>
+      <c r="E14" s="252"/>
+      <c r="F14" s="252"/>
+      <c r="G14" s="252"/>
+      <c r="H14" s="252"/>
+      <c r="I14" s="252"/>
+      <c r="J14" s="253" t="s">
         <v>88</v>
       </c>
-      <c r="K14" s="238"/>
-      <c r="L14" s="238"/>
-      <c r="M14" s="238"/>
-      <c r="N14" s="238"/>
-      <c r="O14" s="239"/>
-      <c r="P14" s="237" t="s">
+      <c r="K14" s="254"/>
+      <c r="L14" s="254"/>
+      <c r="M14" s="254"/>
+      <c r="N14" s="254"/>
+      <c r="O14" s="255"/>
+      <c r="P14" s="253" t="s">
         <v>89</v>
       </c>
-      <c r="Q14" s="238"/>
-      <c r="R14" s="238"/>
-      <c r="S14" s="238"/>
-      <c r="T14" s="238"/>
-      <c r="U14" s="238"/>
-      <c r="V14" s="238"/>
-      <c r="W14" s="238"/>
-      <c r="X14" s="239"/>
+      <c r="Q14" s="254"/>
+      <c r="R14" s="254"/>
+      <c r="S14" s="254"/>
+      <c r="T14" s="254"/>
+      <c r="U14" s="254"/>
+      <c r="V14" s="254"/>
+      <c r="W14" s="254"/>
+      <c r="X14" s="255"/>
     </row>
     <row r="15" spans="1:24" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3"/>
@@ -6840,184 +6790,172 @@
       <c r="X15" s="3"/>
     </row>
     <row r="16" spans="1:24" s="4" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="240" t="s">
+      <c r="A16" s="263" t="s">
         <v>90</v>
       </c>
-      <c r="B16" s="240"/>
-      <c r="C16" s="240"/>
-      <c r="D16" s="240"/>
-      <c r="E16" s="240"/>
-      <c r="F16" s="240"/>
-      <c r="G16" s="240"/>
-      <c r="H16" s="240"/>
-      <c r="I16" s="240"/>
-      <c r="J16" s="241" t="s">
+      <c r="B16" s="263"/>
+      <c r="C16" s="263"/>
+      <c r="D16" s="263"/>
+      <c r="E16" s="263"/>
+      <c r="F16" s="263"/>
+      <c r="G16" s="263"/>
+      <c r="H16" s="263"/>
+      <c r="I16" s="263"/>
+      <c r="J16" s="264" t="s">
         <v>91</v>
       </c>
-      <c r="K16" s="241"/>
-      <c r="L16" s="241"/>
-      <c r="M16" s="241"/>
-      <c r="N16" s="240" t="s">
+      <c r="K16" s="264"/>
+      <c r="L16" s="264"/>
+      <c r="M16" s="264"/>
+      <c r="N16" s="263" t="s">
         <v>92</v>
       </c>
-      <c r="O16" s="240"/>
-      <c r="P16" s="240"/>
-      <c r="Q16" s="240"/>
-      <c r="R16" s="240"/>
-      <c r="S16" s="240"/>
-      <c r="T16" s="242" t="s">
+      <c r="O16" s="263"/>
+      <c r="P16" s="263"/>
+      <c r="Q16" s="263"/>
+      <c r="R16" s="263"/>
+      <c r="S16" s="263"/>
+      <c r="T16" s="265" t="s">
         <v>93</v>
       </c>
-      <c r="U16" s="242"/>
-      <c r="V16" s="242"/>
-      <c r="W16" s="242"/>
-      <c r="X16" s="242"/>
+      <c r="U16" s="265"/>
+      <c r="V16" s="265"/>
+      <c r="W16" s="265"/>
+      <c r="X16" s="265"/>
     </row>
     <row r="17" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="230" t="s">
+      <c r="A17" s="258" t="s">
         <v>94</v>
       </c>
-      <c r="B17" s="231"/>
-      <c r="C17" s="231"/>
-      <c r="D17" s="231"/>
-      <c r="E17" s="231"/>
-      <c r="F17" s="231"/>
-      <c r="G17" s="231"/>
-      <c r="H17" s="231"/>
-      <c r="I17" s="232"/>
-      <c r="J17" s="243" t="s">
+      <c r="B17" s="250"/>
+      <c r="C17" s="250"/>
+      <c r="D17" s="250"/>
+      <c r="E17" s="250"/>
+      <c r="F17" s="250"/>
+      <c r="G17" s="250"/>
+      <c r="H17" s="250"/>
+      <c r="I17" s="259"/>
+      <c r="J17" s="266" t="s">
         <v>95</v>
       </c>
-      <c r="K17" s="244"/>
-      <c r="L17" s="244"/>
-      <c r="M17" s="245"/>
-      <c r="N17" s="230" t="s">
+      <c r="K17" s="267"/>
+      <c r="L17" s="267"/>
+      <c r="M17" s="268"/>
+      <c r="N17" s="258" t="s">
         <v>96</v>
       </c>
-      <c r="O17" s="231"/>
-      <c r="P17" s="231"/>
-      <c r="Q17" s="231"/>
-      <c r="R17" s="231"/>
-      <c r="S17" s="232"/>
-      <c r="T17" s="230" t="s">
+      <c r="O17" s="250"/>
+      <c r="P17" s="250"/>
+      <c r="Q17" s="250"/>
+      <c r="R17" s="250"/>
+      <c r="S17" s="259"/>
+      <c r="T17" s="258" t="s">
         <v>97</v>
       </c>
-      <c r="U17" s="231"/>
-      <c r="V17" s="231"/>
-      <c r="W17" s="231"/>
-      <c r="X17" s="232"/>
+      <c r="U17" s="250"/>
+      <c r="V17" s="250"/>
+      <c r="W17" s="250"/>
+      <c r="X17" s="259"/>
     </row>
     <row r="18" spans="1:24" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="233"/>
-      <c r="B18" s="234"/>
-      <c r="C18" s="234"/>
-      <c r="D18" s="234"/>
-      <c r="E18" s="234"/>
-      <c r="F18" s="234"/>
-      <c r="G18" s="234"/>
-      <c r="H18" s="234"/>
-      <c r="I18" s="235"/>
-      <c r="J18" s="246"/>
-      <c r="K18" s="247"/>
-      <c r="L18" s="247"/>
-      <c r="M18" s="248"/>
-      <c r="N18" s="233"/>
-      <c r="O18" s="234"/>
-      <c r="P18" s="234"/>
-      <c r="Q18" s="234"/>
-      <c r="R18" s="234"/>
-      <c r="S18" s="235"/>
-      <c r="T18" s="233"/>
-      <c r="U18" s="234"/>
-      <c r="V18" s="234"/>
-      <c r="W18" s="234"/>
-      <c r="X18" s="235"/>
+      <c r="A18" s="260"/>
+      <c r="B18" s="261"/>
+      <c r="C18" s="261"/>
+      <c r="D18" s="261"/>
+      <c r="E18" s="261"/>
+      <c r="F18" s="261"/>
+      <c r="G18" s="261"/>
+      <c r="H18" s="261"/>
+      <c r="I18" s="262"/>
+      <c r="J18" s="269"/>
+      <c r="K18" s="270"/>
+      <c r="L18" s="270"/>
+      <c r="M18" s="271"/>
+      <c r="N18" s="260"/>
+      <c r="O18" s="261"/>
+      <c r="P18" s="261"/>
+      <c r="Q18" s="261"/>
+      <c r="R18" s="261"/>
+      <c r="S18" s="262"/>
+      <c r="T18" s="260"/>
+      <c r="U18" s="261"/>
+      <c r="V18" s="261"/>
+      <c r="W18" s="261"/>
+      <c r="X18" s="262"/>
     </row>
     <row r="19" spans="1:24" ht="39" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="20" spans="1:24" ht="39" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="21" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A21" s="228" t="s">
+      <c r="A21" s="275" t="s">
         <v>98</v>
       </c>
-      <c r="B21" s="228"/>
-      <c r="C21" s="228"/>
-      <c r="D21" s="228"/>
-      <c r="E21" s="228"/>
-      <c r="F21" s="228"/>
-      <c r="G21" s="228"/>
-      <c r="H21" s="228"/>
+      <c r="B21" s="275"/>
+      <c r="C21" s="275"/>
+      <c r="D21" s="275"/>
+      <c r="E21" s="275"/>
+      <c r="F21" s="275"/>
+      <c r="G21" s="275"/>
+      <c r="H21" s="275"/>
       <c r="I21" s="5"/>
-      <c r="J21" s="228" t="s">
+      <c r="J21" s="275" t="s">
         <v>65</v>
       </c>
-      <c r="K21" s="228"/>
-      <c r="L21" s="228"/>
-      <c r="M21" s="228"/>
-      <c r="N21" s="228"/>
-      <c r="O21" s="228"/>
-      <c r="P21" s="228"/>
+      <c r="K21" s="275"/>
+      <c r="L21" s="275"/>
+      <c r="M21" s="275"/>
+      <c r="N21" s="275"/>
+      <c r="O21" s="275"/>
+      <c r="P21" s="275"/>
       <c r="Q21" s="6"/>
-      <c r="R21" s="228" t="s">
+      <c r="R21" s="275" t="s">
         <v>99</v>
       </c>
-      <c r="S21" s="228"/>
-      <c r="T21" s="228"/>
-      <c r="U21" s="228"/>
-      <c r="V21" s="228"/>
-      <c r="W21" s="228"/>
-      <c r="X21" s="228"/>
+      <c r="S21" s="275"/>
+      <c r="T21" s="275"/>
+      <c r="U21" s="275"/>
+      <c r="V21" s="275"/>
+      <c r="W21" s="275"/>
+      <c r="X21" s="275"/>
     </row>
     <row r="23" spans="1:24" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="P23" s="225" t="s">
+      <c r="P23" s="272" t="s">
         <v>100</v>
       </c>
-      <c r="Q23" s="225"/>
-      <c r="R23" s="225"/>
-      <c r="S23" s="225"/>
-      <c r="T23" s="225"/>
-      <c r="U23" s="226" t="s">
+      <c r="Q23" s="272"/>
+      <c r="R23" s="272"/>
+      <c r="S23" s="272"/>
+      <c r="T23" s="272"/>
+      <c r="U23" s="273" t="s">
         <v>101</v>
       </c>
-      <c r="V23" s="226"/>
-      <c r="W23" s="226"/>
-      <c r="X23" s="226"/>
+      <c r="V23" s="273"/>
+      <c r="W23" s="273"/>
+      <c r="X23" s="273"/>
     </row>
     <row r="24" spans="1:24" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="P24" s="225" t="s">
+      <c r="P24" s="272" t="s">
         <v>102</v>
       </c>
-      <c r="Q24" s="225"/>
-      <c r="R24" s="225"/>
-      <c r="S24" s="225"/>
-      <c r="T24" s="225"/>
-      <c r="U24" s="227" t="s">
+      <c r="Q24" s="272"/>
+      <c r="R24" s="272"/>
+      <c r="S24" s="272"/>
+      <c r="T24" s="272"/>
+      <c r="U24" s="274" t="s">
         <v>103</v>
       </c>
-      <c r="V24" s="227"/>
-      <c r="W24" s="227"/>
-      <c r="X24" s="227"/>
+      <c r="V24" s="274"/>
+      <c r="W24" s="274"/>
+      <c r="X24" s="274"/>
     </row>
   </sheetData>
   <mergeCells count="40">
-    <mergeCell ref="A1:T1"/>
-    <mergeCell ref="U1:X1"/>
-    <mergeCell ref="A2:T2"/>
-    <mergeCell ref="A7:I7"/>
-    <mergeCell ref="J7:O7"/>
-    <mergeCell ref="P7:X7"/>
-    <mergeCell ref="A5:M5"/>
-    <mergeCell ref="A4:M4"/>
-    <mergeCell ref="N4:X4"/>
-    <mergeCell ref="N5:X5"/>
-    <mergeCell ref="U2:X3"/>
-    <mergeCell ref="A8:I8"/>
-    <mergeCell ref="J8:O8"/>
-    <mergeCell ref="P8:X8"/>
-    <mergeCell ref="A10:X10"/>
-    <mergeCell ref="A11:F11"/>
-    <mergeCell ref="G11:L11"/>
-    <mergeCell ref="M11:R11"/>
-    <mergeCell ref="S11:X11"/>
+    <mergeCell ref="P23:T23"/>
+    <mergeCell ref="U23:X23"/>
+    <mergeCell ref="P24:T24"/>
+    <mergeCell ref="U24:X24"/>
+    <mergeCell ref="A21:H21"/>
+    <mergeCell ref="J21:P21"/>
+    <mergeCell ref="R21:X21"/>
     <mergeCell ref="A13:I13"/>
     <mergeCell ref="J13:O13"/>
     <mergeCell ref="P13:X13"/>
@@ -7032,13 +6970,25 @@
     <mergeCell ref="T16:X16"/>
     <mergeCell ref="A17:I18"/>
     <mergeCell ref="J17:M18"/>
-    <mergeCell ref="P23:T23"/>
-    <mergeCell ref="U23:X23"/>
-    <mergeCell ref="P24:T24"/>
-    <mergeCell ref="U24:X24"/>
-    <mergeCell ref="A21:H21"/>
-    <mergeCell ref="J21:P21"/>
-    <mergeCell ref="R21:X21"/>
+    <mergeCell ref="A8:I8"/>
+    <mergeCell ref="J8:O8"/>
+    <mergeCell ref="P8:X8"/>
+    <mergeCell ref="A10:X10"/>
+    <mergeCell ref="A11:F11"/>
+    <mergeCell ref="G11:L11"/>
+    <mergeCell ref="M11:R11"/>
+    <mergeCell ref="S11:X11"/>
+    <mergeCell ref="A1:T1"/>
+    <mergeCell ref="U1:X1"/>
+    <mergeCell ref="A2:T2"/>
+    <mergeCell ref="A7:I7"/>
+    <mergeCell ref="J7:O7"/>
+    <mergeCell ref="P7:X7"/>
+    <mergeCell ref="A5:M5"/>
+    <mergeCell ref="A4:M4"/>
+    <mergeCell ref="N4:X4"/>
+    <mergeCell ref="N5:X5"/>
+    <mergeCell ref="U2:X3"/>
   </mergeCells>
   <pageMargins left="0.51181102362204722" right="0.51181102362204722" top="0.35433070866141736" bottom="0.35433070866141736" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup scale="95" orientation="landscape" horizontalDpi="4294967294" verticalDpi="200" r:id="rId1"/>
@@ -7047,6 +6997,37 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <TaxCatchAll xmlns="41dd0a9e-964d-48c8-9389-7445c2a187f7" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="edbb1c21-1b45-407e-8894-c97732534993">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <_Flow_SignoffStatus xmlns="edbb1c21-1b45-407e-8894-c97732534993" xsi:nil="true"/>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <_x0031_010005470 xmlns="edbb1c21-1b45-407e-8894-c97732534993">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </_x0031_010005470>
+    <FechayHora xmlns="edbb1c21-1b45-407e-8894-c97732534993" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x01010080239B14884FBB46AB47CE62E6B5D997" ma:contentTypeVersion="24" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="95cfff668db4ca1e5f6e9375137a4a8e">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="edbb1c21-1b45-407e-8894-c97732534993" xmlns:ns3="41dd0a9e-964d-48c8-9389-7445c2a187f7" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="6912f17aaadcd6a9684df23b147afc35" ns1:_="" ns2:_="" ns3:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -7356,38 +7337,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <TaxCatchAll xmlns="41dd0a9e-964d-48c8-9389-7445c2a187f7" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="edbb1c21-1b45-407e-8894-c97732534993">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <_Flow_SignoffStatus xmlns="edbb1c21-1b45-407e-8894-c97732534993" xsi:nil="true"/>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <_x0031_010005470 xmlns="edbb1c21-1b45-407e-8894-c97732534993">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </_x0031_010005470>
-    <FechayHora xmlns="edbb1c21-1b45-407e-8894-c97732534993" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2FFAC935-8881-451D-93ED-25958414B4DF}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AAD99F47-C05E-4B8B-A445-C498A7984441}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="41dd0a9e-964d-48c8-9389-7445c2a187f7"/>
+    <ds:schemaRef ds:uri="edbb1c21-1b45-407e-8894-c97732534993"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2E0DC6A2-D4C3-4E6B-B67E-9AED22EC483E}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -7405,24 +7375,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AAD99F47-C05E-4B8B-A445-C498A7984441}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="41dd0a9e-964d-48c8-9389-7445c2a187f7"/>
-    <ds:schemaRef ds:uri="edbb1c21-1b45-407e-8894-c97732534993"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2FFAC935-8881-451D-93ED-25958414B4DF}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Actualiza formatos: Bitacoras y Visitas GFPI
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Formatos/BITACORAS GFPI-F-147V4.xlsx
+++ b/Formatos/BITACORAS GFPI-F-147V4.xlsx
@@ -5,18 +5,22 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SEANT\OneDrive\Documents\Seto 2026\sena\Manual SENA Etapa Productiva\manual-aprendiz-sena\Formatos\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/834af06e427efe68/Documents/Seto 2026/sena/Manual SENA Etapa Productiva/manual-aprendiz-sena/Formatos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C00FB21-90C9-41D6-AC50-EF2816FA0BA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="27" documentId="8_{FA325372-B3D4-4C73-B306-A8EC3281E55B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{46246EDD-3969-4EDF-B7E7-BA3848425155}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Formato Bitácora Individual" sheetId="6" r:id="rId1"/>
-    <sheet name="Hoja1" sheetId="7" state="hidden" r:id="rId2"/>
-    <sheet name="Instructivo" sheetId="4" state="hidden" r:id="rId3"/>
+    <sheet name="BD_SENA" sheetId="8" state="hidden" r:id="rId2"/>
+    <sheet name="Hoja1" sheetId="7" state="hidden" r:id="rId3"/>
+    <sheet name="Instructivo" sheetId="4" state="hidden" r:id="rId4"/>
   </sheets>
+  <externalReferences>
+    <externalReference r:id="rId5"/>
+  </externalReferences>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Formato Bitácora Individual'!$A$1:$I$83</definedName>
   </definedNames>
@@ -40,8 +44,30 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="123">
   <si>
     <t>Código: 
 GFPI-F-147</t>
@@ -455,12 +481,63 @@
   <si>
     <t>satorres@sena.edu.co   /    storres@timespanish.com</t>
   </si>
+  <si>
+    <t>PROGRAMA</t>
+  </si>
+  <si>
+    <t>COMPETENCIA</t>
+  </si>
+  <si>
+    <t>RESULTADO DE APRENDIZAJE (RAP)</t>
+  </si>
+  <si>
+    <t>Análisis y Desarrollo de Software</t>
+  </si>
+  <si>
+    <t>38392 - Establecer requisitos de la solución de software de acuerdo con estándares y procedimiento técnico</t>
+  </si>
+  <si>
+    <t>38376 - Evaluar requisitos de la solución de software de acuerdo con metodologías de análisis y estándares</t>
+  </si>
+  <si>
+    <t>38362 - Diseñar la solución de software de acuerdo con procedimientos y requisitos técnicos</t>
+  </si>
+  <si>
+    <t>38368 - Desarrollar la solución de software de acuerdo con el diseño y metodologías de desarrollo</t>
+  </si>
+  <si>
+    <t>38369 - Controlar la calidad del servicio de software de acuerdo con los estándares técnicos</t>
+  </si>
+  <si>
+    <t>38367 - Estructurar propuesta técnica de servicio de tecnología de la información según requisitos técnicos y normativa</t>
+  </si>
+  <si>
+    <t>38356 - Implementar la solución de software de acuerdo con los requisitos de operación y modelos de referencia</t>
+  </si>
+  <si>
+    <t>Programación de Software</t>
+  </si>
+  <si>
+    <t>220501095 - Construir el sistema de información de acuerdo con el diseño y estándares técnicos</t>
+  </si>
+  <si>
+    <t>220501096 - Verificar la calidad del software de acuerdo con el plan de pruebas y estándares</t>
+  </si>
+  <si>
+    <t>220501097 - Desplegar la solución de software de acuerdo con los requisitos de operación y modelos de referencia</t>
+  </si>
+  <si>
+    <t>220501101 - Probar el software desarrollado de acuerdo con el plan de pruebas y especificaciones del cliente</t>
+  </si>
+  <si>
+    <t>37371 - Utilizar herramientas informáticas de acuerdo con las necesidades de manejo de información</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="35" x14ac:knownFonts="1">
+  <fonts count="36" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -698,6 +775,12 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="8">
     <fill>
@@ -743,7 +826,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="111">
+  <borders count="118">
     <border>
       <left/>
       <right/>
@@ -2117,11 +2200,98 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="276">
+  <cellXfs count="283">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -2964,11 +3134,39 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="111" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="112" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="113" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="114" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="115" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="116" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="117" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="4">
+  <dxfs count="11">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -2997,10 +3195,138 @@
         </patternFill>
       </fill>
     </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color rgb="FFCCCCCC"/>
+        </left>
+        <right style="medium">
+          <color rgb="FFCCCCCC"/>
+        </right>
+        <top style="medium">
+          <color rgb="FFCCCCCC"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FFCCCCCC"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="medium">
+          <color rgb="FFCCCCCC"/>
+        </right>
+        <top style="medium">
+          <color rgb="FFCCCCCC"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FFCCCCCC"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="medium">
+          <color rgb="FFCCCCCC"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="medium">
+          <color rgb="FFCCCCCC"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="medium">
+          <color rgb="FFCCCCCC"/>
+        </left>
+        <right style="medium">
+          <color rgb="FFCCCCCC"/>
+        </right>
+        <top style="medium">
+          <color rgb="FFCCCCCC"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FFCCCCCC"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="medium">
+          <color rgb="FFCCCCCC"/>
+        </left>
+        <right style="medium">
+          <color rgb="FFCCCCCC"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FFCD03A7"/>
       <color rgb="FFE1EF57"/>
       <color rgb="FFE6DE74"/>
       <color rgb="FFDEE16D"/>
@@ -3151,6 +3477,24 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:absoluteUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
+    <sheetNames>
+      <sheetName val="Formato Visita 1"/>
+      <sheetName val="BD_SENA"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0"/>
+      <sheetData sheetId="1"/>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
+</file>
+
 <file path=xl/featurePropertyBag/featurePropertyBag.xml><?xml version="1.0" encoding="utf-8"?>
 <FeaturePropertyBags xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag">
   <bag type="Checkbox"/>
@@ -3166,6 +3510,18 @@
     </a>
   </bag>
 </FeaturePropertyBags>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{02E4A812-C304-4BF6-9E0E-42EEF04E5155}" name="TablaSena" displayName="TablaSena" ref="A1:C39" totalsRowShown="0" headerRowDxfId="10" headerRowBorderDxfId="8" tableBorderDxfId="9" totalsRowBorderDxfId="7">
+  <autoFilter ref="A1:C39" xr:uid="{02E4A812-C304-4BF6-9E0E-42EEF04E5155}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{58F25D10-8D0D-47B3-B80D-DEB8D02185E0}" name="PROGRAMA" dataDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{9B09017C-CA14-4900-8C8E-9C5637EB0DAC}" name="COMPETENCIA" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{C711739C-0421-472E-BA8E-7EC306B5B970}" name="RESULTADO DE APRENDIZAJE (RAP)"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium6" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -6245,17 +6601,22 @@
     <mergeCell ref="G90:H90"/>
     <mergeCell ref="E65:F66"/>
   </mergeCells>
-  <conditionalFormatting sqref="B11:I11 B15:I15 B17:I17 B19:I19 B21:I21 B25:I25 B29:I29 C37:F42 H37:I42 B47:I56 B70:E71 H74:I75 B83:I83">
-    <cfRule type="containsBlanks" dxfId="3" priority="3">
+  <conditionalFormatting sqref="B11:I11 B15:I15 B17:I17 B19:I19 B21:I21 B25:I25 B29:I29 C37:F42 H37:I42 B70:E71 B74:E75 H74:I75 B83:I83">
+    <cfRule type="containsBlanks" dxfId="4" priority="4">
       <formula>LEN(TRIM(B11))=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G65:G66 I65:I66 B66:D66 H71">
-    <cfRule type="containsBlanks" dxfId="2" priority="4">
+    <cfRule type="containsBlanks" dxfId="3" priority="5">
       <formula>LEN(TRIM(B65))=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations xWindow="1156" yWindow="532" count="36">
+  <conditionalFormatting sqref="B47:I56">
+    <cfRule type="containsBlanks" dxfId="0" priority="1">
+      <formula>LEN(TRIM(B47))=0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations xWindow="1156" yWindow="532" count="34">
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Desde dd/mm/aa hasta dd/mm/aa" prompt="Ingresar la fehca de inicio y fin de la bitácora" sqref="E11:I11" xr:uid="{CD2FA053-183B-41CA-B267-B4277B8CA158}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Desplegar y seleccionar" prompt="Desplegar y seleccionar el numero de bitacora actual" sqref="B11:D11" xr:uid="{3D01CEB2-123B-4C72-96E2-63C296030E46}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Ingresar Nombres y apellidos de aprendiz, tal como regista en su docuemnto de identificacion" sqref="B15:D15" xr:uid="{A585EB3A-7529-4958-B886-65F5282307D7}"/>
@@ -6266,7 +6627,6 @@
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Ingrese su correo personal" sqref="E17:G17" xr:uid="{32F1EB00-C1DD-4D21-B121-582E1CBC1029}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Ingrese los datos de direccion de recidencia actual, incluyendo ciudad" sqref="H17:I17" xr:uid="{3DB420C9-8C3F-4FD2-BB93-3002ADC0D6C3}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Ingrese el numero de ficha al que pertenece" sqref="B19:D19" xr:uid="{DFFFBA8D-FBA5-4BD3-AC44-D2490892B2EA}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Ingresar el programa de formacion al que pertenece" sqref="H19:I19" xr:uid="{B93300CA-489F-49BB-A3E5-3614F8952259}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Técnico o Tecnólogo?" sqref="E19:G19" xr:uid="{4135DBDF-CCD6-4F5E-ABDB-9335530EEA9D}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Ingresar si aplica" prompt="Presencial o Virtual?  . si no aplica favor colocar un PUNTO (.)" sqref="B21:D21" xr:uid="{8ADE279D-8C86-42BB-9BD1-0C0783D232C0}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle=" Ingresar si aplica" prompt="SI o No. . si no aplica favor colocar un PUNTO (.)" sqref="E21:G21" xr:uid="{119BC392-23A1-4BFC-A774-9304C7DDB712}"/>
@@ -6278,11 +6638,10 @@
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Ingresar numero de contacto." sqref="G29" xr:uid="{8643D366-4A6B-4DA2-A344-53B316943693}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Correo electrónico del jefe inmediato" sqref="H29:I29" xr:uid="{85054B10-E824-4537-9671-AA0ADB26EDBD}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Ingresar las actividades desarrolladas. ejemplo :Sesión informativa sobre seguridad de infraestructura y validación de protocolos . Solución del fallo en el sistema de correos automáticos (debugging y validación).etc..." sqref="B47:C56" xr:uid="{1EF4E3E9-6D3D-4AE1-8170-FF1AAEA1E1B9}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Ingresar la competencia del programa que abarca la actividad realizada, debe ser de las competencias concertadas inicialmente en el formato F023 visita 1" sqref="D47:E56" xr:uid="{0D8BD481-B72E-43AC-9736-661B2F1B5B5C}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Ingresar fecha de inicio de la actividad" sqref="F47:F56" xr:uid="{32DD5E98-EAF7-430B-97F3-79C3622F702E}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Ingresar fecha de finalizacion de la actividad" sqref="G47:G56" xr:uid="{145C53F1-D232-49E6-A4AB-B178BD1CDE8E}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="NO VAN CAPTURAS DE PANTALLA" prompt="Ejemplo 1: Documento: Documento (material del curso de diseño web revisado y aplicado. _x000a_Ejemplo 2:  Proceso (validación de ejecución de parchados_x000a_en servidores)._x000a_Ejemplo 3: Producto: Aplicacion WEB (Se aclara son ejemplos)" sqref="H49:H56" xr:uid="{1B955B8F-68CD-419F-B5E8-35AC173B4957}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="NO VAN CAPTURAS DE PANTALLA" prompt="Si se presentan situaciones relevantes en el desarrollo de la actividad, favor relacionarla. (Ejemplo, retrasos, incumplimientos. etc). SI POR TEMAS DE CONFIDENCIALIDAD D ELA INFORMACION NO SE PUEDEN ANEXAR CAPTURAS, FAVOR DEJARLO POR ESCRITO ACA." sqref="I47:I56" xr:uid="{67EE6F84-95FA-40E8-86A9-4393D2B1D5BB}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="NO VAN CAPTURAS DE PANTALLA" prompt="Ingresar informacion del desarrollo de la actividad. si hay otro tipo de informa favor relacionarla. (Ejemplo, retrasos, incumplimientos. etc). SI POR TEMAS DE CONFIDENCIALIDAD D ELA INFORMACION NO SE PUEDEN ANEXAR CAPTURAS, FAVOR DEJARLO POR ESCRITO ACA." sqref="I47:I56" xr:uid="{67EE6F84-95FA-40E8-86A9-4393D2B1D5BB}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="NO VAN CAPTURAS DE PANTALLA" prompt="Ejemplo 1: Documento: Documento (material del curso de diseño web revisado y aplicado. _x000a_Ejemplo 2:  Proceso (validación de ejecución de parchados_x000a_en servidores)._x000a_Ejemplo 3: Producto: Aplicacion WEB (Se aclara son ejemplos). NO VAN CAPTURAS DE PANTALLA" sqref="H47:H48" xr:uid="{CBCC16C2-11EE-4F06-BE98-4BF1A24BDE5E}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Si / NO" prompt="Si / NO" sqref="B66" xr:uid="{399AC36A-2FBC-4A36-BEF2-DB6479D0AE91}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Indiquie el nivel asignado de riego del 1 al 5" sqref="C66:D66" xr:uid="{0B51F00F-01A3-4D67-B07C-4E070A35CC22}"/>
@@ -6296,10 +6655,395 @@
   <pageMargins left="0.51181102362204722" right="0.51181102362204722" top="0.35433070866141736" bottom="0.35433070866141736" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="5" scale="47" fitToHeight="0" orientation="portrait" horizontalDpi="4294967294" r:id="rId1"/>
   <drawing r:id="rId2"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xWindow="1156" yWindow="532" count="2">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Ingresar el programa de formacion al que pertenece" xr:uid="{B93300CA-489F-49BB-A3E5-3614F8952259}">
+          <x14:formula1>
+            <xm:f>_xlfn.ANCHORARRAY(BD_SENA!$E$2)</xm:f>
+          </x14:formula1>
+          <xm:sqref>H19:I19</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Ingresar la competencia del programa que abarca la actividad realizada, debe ser de las competencias concertadas inicialmente en el formato F023 visita 1" xr:uid="{0D8BD481-B72E-43AC-9736-661B2F1B5B5C}">
+          <x14:formula1>
+            <xm:f>_xlfn.ANCHORARRAY(BD_SENA!$F$2)</xm:f>
+          </x14:formula1>
+          <xm:sqref>D47:E56</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+  </extLst>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D67D322E-43FB-4E8B-8CF8-610E011BE901}">
+  <dimension ref="A1:K39"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="17.42578125" customWidth="1"/>
+    <col min="2" max="2" width="58.7109375" customWidth="1"/>
+    <col min="3" max="3" width="133" customWidth="1"/>
+    <col min="5" max="5" width="29.28515625" customWidth="1"/>
+    <col min="6" max="6" width="23" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="276" t="s">
+        <v>106</v>
+      </c>
+      <c r="B1" s="277" t="s">
+        <v>107</v>
+      </c>
+      <c r="C1" s="278" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" ht="39" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="279" t="s">
+        <v>109</v>
+      </c>
+      <c r="B2" s="280" t="s">
+        <v>110</v>
+      </c>
+      <c r="E2" t="str" cm="1">
+        <f t="array" ref="E2:E3">_xlfn.UNIQUE(TablaSena[PROGRAMA])</f>
+        <v>Análisis y Desarrollo de Software</v>
+      </c>
+      <c r="F2" t="str" cm="1">
+        <f t="array" ref="F2">_xlfn.UNIQUE(_xlfn._xlws.FILTER(TablaSena[COMPETENCIA], TablaSena[PROGRAMA]='[1]Formato Visita 1'!$C$11, "Seleccione Programa"))</f>
+        <v>Seleccione Programa</v>
+      </c>
+      <c r="G2" t="str" cm="1">
+        <f t="array" ref="G2">_xlfn._xlws.FILTER(TablaSena[RESULTADO DE APRENDIZAJE (RAP)], TablaSena[COMPETENCIA]='[1]Formato Visita 1'!$C$50, "...")</f>
+        <v>...</v>
+      </c>
+      <c r="H2" t="str" cm="1">
+        <f t="array" ref="H2">_xlfn._xlws.FILTER(TablaSena[RESULTADO DE APRENDIZAJE (RAP)], TablaSena[COMPETENCIA]='[1]Formato Visita 1'!$C$51, "...")</f>
+        <v>...</v>
+      </c>
+      <c r="I2" t="str" cm="1">
+        <f t="array" ref="I2">_xlfn._xlws.FILTER(TablaSena[RESULTADO DE APRENDIZAJE (RAP)], TablaSena[COMPETENCIA]='[1]Formato Visita 1'!$C$52, "...")</f>
+        <v>...</v>
+      </c>
+      <c r="J2" t="str" cm="1">
+        <f t="array" ref="J2">_xlfn._xlws.FILTER(TablaSena[RESULTADO DE APRENDIZAJE (RAP)], TablaSena[COMPETENCIA]='[1]Formato Visita 1'!$C$53, "...")</f>
+        <v>...</v>
+      </c>
+      <c r="K2" t="str" cm="1">
+        <f t="array" ref="K2">_xlfn._xlws.FILTER(TablaSena[RESULTADO DE APRENDIZAJE (RAP)], TablaSena[COMPETENCIA]='[1]Formato Visita 1'!$C$54, "...")</f>
+        <v>...</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="39" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="279" t="s">
+        <v>109</v>
+      </c>
+      <c r="B3" s="280" t="s">
+        <v>110</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Programación de Software</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="39" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="279" t="s">
+        <v>109</v>
+      </c>
+      <c r="B4" s="280" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="39" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="279" t="s">
+        <v>109</v>
+      </c>
+      <c r="B5" s="280" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="39" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="279" t="s">
+        <v>109</v>
+      </c>
+      <c r="B6" s="280" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="39" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="279" t="s">
+        <v>109</v>
+      </c>
+      <c r="B7" s="280" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="39" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="279" t="s">
+        <v>109</v>
+      </c>
+      <c r="B8" s="280" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" ht="39" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="279" t="s">
+        <v>109</v>
+      </c>
+      <c r="B9" s="280" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="39" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="279" t="s">
+        <v>109</v>
+      </c>
+      <c r="B10" s="280" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" ht="39" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="279" t="s">
+        <v>109</v>
+      </c>
+      <c r="B11" s="280" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" ht="39" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="279" t="s">
+        <v>109</v>
+      </c>
+      <c r="B12" s="280" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" ht="39" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="279" t="s">
+        <v>109</v>
+      </c>
+      <c r="B13" s="280" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="39" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="279" t="s">
+        <v>109</v>
+      </c>
+      <c r="B14" s="280" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" ht="39" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="279" t="s">
+        <v>109</v>
+      </c>
+      <c r="B15" s="280" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" ht="39" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="279" t="s">
+        <v>109</v>
+      </c>
+      <c r="B16" s="280" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" ht="39" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="279" t="s">
+        <v>109</v>
+      </c>
+      <c r="B17" s="280" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="39" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="279" t="s">
+        <v>109</v>
+      </c>
+      <c r="B18" s="280" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="39" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="279" t="s">
+        <v>109</v>
+      </c>
+      <c r="B19" s="280" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="39" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="279" t="s">
+        <v>109</v>
+      </c>
+      <c r="B20" s="280" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="39" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="279" t="s">
+        <v>109</v>
+      </c>
+      <c r="B21" s="280" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="39" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="279" t="s">
+        <v>109</v>
+      </c>
+      <c r="B22" s="280" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="39" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="279" t="s">
+        <v>109</v>
+      </c>
+      <c r="B23" s="280" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="39" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="279" t="s">
+        <v>109</v>
+      </c>
+      <c r="B24" s="280" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="39" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="279" t="s">
+        <v>109</v>
+      </c>
+      <c r="B25" s="280" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" ht="39" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="279" t="s">
+        <v>109</v>
+      </c>
+      <c r="B26" s="280" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" ht="39" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="279" t="s">
+        <v>109</v>
+      </c>
+      <c r="B27" s="280" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="279" t="s">
+        <v>117</v>
+      </c>
+      <c r="B28" s="280" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="279" t="s">
+        <v>117</v>
+      </c>
+      <c r="B29" s="280" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="279" t="s">
+        <v>117</v>
+      </c>
+      <c r="B30" s="280" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="279" t="s">
+        <v>117</v>
+      </c>
+      <c r="B31" s="280" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="279" t="s">
+        <v>117</v>
+      </c>
+      <c r="B32" s="280" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="279" t="s">
+        <v>117</v>
+      </c>
+      <c r="B33" s="280" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="279" t="s">
+        <v>117</v>
+      </c>
+      <c r="B34" s="280" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="279" t="s">
+        <v>117</v>
+      </c>
+      <c r="B35" s="280" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="279" t="s">
+        <v>117</v>
+      </c>
+      <c r="B36" s="280" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="279" t="s">
+        <v>117</v>
+      </c>
+      <c r="B37" s="280" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="279" t="s">
+        <v>117</v>
+      </c>
+      <c r="B38" s="280" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A39" s="281" t="s">
+        <v>117</v>
+      </c>
+      <c r="B39" s="282" t="s">
+        <v>122</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D237D29B-37DE-45D6-8EA7-98C4A952DFFE}">
   <dimension ref="D1:D12"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -6369,7 +7113,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:X24"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
Actualiza formato de bitácoras GFPI-F-147V4.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Formatos/BITACORAS GFPI-F-147V4.xlsx
+++ b/Formatos/BITACORAS GFPI-F-147V4.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uniminuto0-my.sharepoint.com/personal/sergio_torres_mar_uniminuto_edu_co/Documents/Documentos/Seto 2026/sena/Manual SENA Etapa Productiva/manual-aprendiz-sena/Formatos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEF1DC7A-FFF1-4291-A724-1398C9A655DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="8" documentId="13_ncr:1_{BEF1DC7A-FFF1-4291-A724-1398C9A655DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{83410BEE-54F5-4C5C-AC98-DB36869CF98A}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -2635,178 +2635,376 @@
     <xf numFmtId="0" fontId="35" fillId="0" borderId="117" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="119" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="118" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="108" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="109" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="110" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="96" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="93" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="98" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="100" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="101" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="92" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="93" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="63" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="64" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="64" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="91" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="57" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="58" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="59" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="66" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="67" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="89" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="90" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="66" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="67" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="84" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="85" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="86" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="66" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="67" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="85" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="86" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="5" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="5" borderId="57" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="95" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="96" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="99" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="100" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="77" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="78" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="68" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="85" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="86" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="71" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="75" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="59" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="62" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="53" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="102" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="92" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="93" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="96" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="93" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="93" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="93" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="76" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="71" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="75" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="59" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="2" borderId="70" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="2" borderId="74" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="2" borderId="58" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="70" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="74" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="69" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="73" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="63" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="97" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="7" borderId="87" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="7" borderId="88" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="94" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="70" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="74" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="61" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="60" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="54" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="70" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="74" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="71" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="75" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="59" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="65" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="6" borderId="79" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2835,12 +3033,6 @@
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="105" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2888,308 +3080,212 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="59" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="70" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="77" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="74" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="78" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="97" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="61" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="100" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="65" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="2" borderId="70" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="2" borderId="74" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="2" borderId="58" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="69" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="73" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="63" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="64" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="66" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="67" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="84" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="85" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="86" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="66" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="67" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="85" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="86" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="5" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="5" borderId="57" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="95" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="60" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="96" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="54" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="61" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="72" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="87" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="88" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="99" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="68" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="85" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="86" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="71" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="75" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="59" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="62" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="53" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="102" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="7" borderId="76" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="7" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="7" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="61" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="72" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="91" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="57" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="58" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="59" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="66" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="67" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="63" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="98" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="100" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="101" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="89" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="90" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="64" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="93" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="93" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="108" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="109" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="110" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
@@ -3202,108 +3298,33 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="119" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="118" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="10">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFE1EF57"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFE2ED51"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -3414,13 +3435,6 @@
     </dxf>
     <dxf>
       <border outline="0">
-        <bottom style="medium">
-          <color rgb="FFCCCCCC"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
         <left style="medium">
           <color rgb="FFCCCCCC"/>
         </left>
@@ -3430,6 +3444,13 @@
         <top style="medium">
           <color rgb="FFCCCCCC"/>
         </top>
+        <bottom style="medium">
+          <color rgb="FFCCCCCC"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
         <bottom style="medium">
           <color rgb="FFCCCCCC"/>
         </bottom>
@@ -3463,27 +3484,6 @@
         <top/>
         <bottom/>
       </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFE1EF57"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFE2ED51"/>
-        </patternFill>
-      </fill>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -3651,7 +3651,23 @@
       <sheetName val="BD_SENA"/>
     </sheetNames>
     <sheetDataSet>
-      <sheetData sheetId="0"/>
+      <sheetData sheetId="0">
+        <row r="50">
+          <cell r="C50"/>
+        </row>
+        <row r="51">
+          <cell r="C51"/>
+        </row>
+        <row r="52">
+          <cell r="C52"/>
+        </row>
+        <row r="53">
+          <cell r="C53"/>
+        </row>
+        <row r="54">
+          <cell r="C54"/>
+        </row>
+      </sheetData>
       <sheetData sheetId="1"/>
     </sheetDataSet>
   </externalBook>
@@ -3676,12 +3692,12 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{99010CAF-386D-41BE-AE72-8D38EFA83A09}" name="TablaSena" displayName="TablaSena" ref="A1:C39" totalsRowShown="0" headerRowDxfId="6" headerRowBorderDxfId="4" tableBorderDxfId="5" totalsRowBorderDxfId="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{99010CAF-386D-41BE-AE72-8D38EFA83A09}" name="TablaSena" displayName="TablaSena" ref="A1:C39" totalsRowShown="0" headerRowDxfId="9" headerRowBorderDxfId="8" tableBorderDxfId="7" totalsRowBorderDxfId="6">
   <autoFilter ref="A1:C39" xr:uid="{99010CAF-386D-41BE-AE72-8D38EFA83A09}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{61F34070-348E-42B3-BF87-5A1CD2BB6FD7}" name="PROGRAMA" dataDxfId="2"/>
-    <tableColumn id="2" xr3:uid="{7B4CB996-89B6-45DE-A53A-D02152366731}" name="COMPETENCIA" dataDxfId="1"/>
-    <tableColumn id="3" xr3:uid="{529DD12A-961C-42BF-9AA1-50D419FC6C5E}" name="RESULTADO DE APRENDIZAJE (RAP)" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{61F34070-348E-42B3-BF87-5A1CD2BB6FD7}" name="PROGRAMA" dataDxfId="5"/>
+    <tableColumn id="2" xr3:uid="{7B4CB996-89B6-45DE-A53A-D02152366731}" name="COMPETENCIA" dataDxfId="4"/>
+    <tableColumn id="3" xr3:uid="{529DD12A-961C-42BF-9AA1-50D419FC6C5E}" name="RESULTADO DE APRENDIZAJE (RAP)" dataDxfId="3"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium6" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -4068,16 +4084,16 @@
       <c r="AB2" s="7"/>
     </row>
     <row r="3" spans="2:28" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="125" t="s">
+      <c r="B3" s="191" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="126"/>
-      <c r="D3" s="126"/>
-      <c r="E3" s="126"/>
-      <c r="F3" s="126"/>
-      <c r="G3" s="126"/>
-      <c r="H3" s="126"/>
-      <c r="I3" s="127"/>
+      <c r="C3" s="192"/>
+      <c r="D3" s="192"/>
+      <c r="E3" s="192"/>
+      <c r="F3" s="192"/>
+      <c r="G3" s="192"/>
+      <c r="H3" s="192"/>
+      <c r="I3" s="193"/>
       <c r="J3" s="8"/>
       <c r="K3" s="7"/>
       <c r="L3" s="7"/>
@@ -4099,16 +4115,16 @@
       <c r="AB3" s="7"/>
     </row>
     <row r="4" spans="2:28" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="131" t="s">
+      <c r="B4" s="197" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="132"/>
-      <c r="D4" s="132"/>
-      <c r="E4" s="132"/>
-      <c r="F4" s="132"/>
-      <c r="G4" s="132"/>
-      <c r="H4" s="132"/>
-      <c r="I4" s="133"/>
+      <c r="C4" s="198"/>
+      <c r="D4" s="198"/>
+      <c r="E4" s="198"/>
+      <c r="F4" s="198"/>
+      <c r="G4" s="198"/>
+      <c r="H4" s="198"/>
+      <c r="I4" s="199"/>
       <c r="J4" s="8"/>
       <c r="K4" s="7"/>
       <c r="L4" s="7"/>
@@ -4130,16 +4146,16 @@
       <c r="AB4" s="7"/>
     </row>
     <row r="5" spans="2:28" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="128" t="s">
+      <c r="B5" s="194" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="129"/>
-      <c r="D5" s="129"/>
-      <c r="E5" s="129"/>
-      <c r="F5" s="129"/>
-      <c r="G5" s="129"/>
-      <c r="H5" s="129"/>
-      <c r="I5" s="130"/>
+      <c r="C5" s="195"/>
+      <c r="D5" s="195"/>
+      <c r="E5" s="195"/>
+      <c r="F5" s="195"/>
+      <c r="G5" s="195"/>
+      <c r="H5" s="195"/>
+      <c r="I5" s="196"/>
       <c r="J5" s="8"/>
       <c r="K5" s="8"/>
       <c r="L5" s="7"/>
@@ -4161,16 +4177,16 @@
       <c r="AB5" s="7"/>
     </row>
     <row r="6" spans="2:28" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="131" t="s">
+      <c r="B6" s="197" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="132"/>
-      <c r="D6" s="132"/>
-      <c r="E6" s="132"/>
-      <c r="F6" s="132"/>
-      <c r="G6" s="132"/>
-      <c r="H6" s="132"/>
-      <c r="I6" s="133"/>
+      <c r="C6" s="198"/>
+      <c r="D6" s="198"/>
+      <c r="E6" s="198"/>
+      <c r="F6" s="198"/>
+      <c r="G6" s="198"/>
+      <c r="H6" s="198"/>
+      <c r="I6" s="199"/>
       <c r="J6" s="8"/>
       <c r="K6" s="8"/>
       <c r="L6" s="7"/>
@@ -4192,16 +4208,16 @@
       <c r="AB6" s="7"/>
     </row>
     <row r="7" spans="2:28" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="128" t="s">
+      <c r="B7" s="194" t="s">
         <v>6</v>
       </c>
-      <c r="C7" s="129"/>
-      <c r="D7" s="129"/>
-      <c r="E7" s="129"/>
-      <c r="F7" s="129"/>
-      <c r="G7" s="129"/>
-      <c r="H7" s="129"/>
-      <c r="I7" s="130"/>
+      <c r="C7" s="195"/>
+      <c r="D7" s="195"/>
+      <c r="E7" s="195"/>
+      <c r="F7" s="195"/>
+      <c r="G7" s="195"/>
+      <c r="H7" s="195"/>
+      <c r="I7" s="196"/>
       <c r="J7" s="7"/>
       <c r="K7" s="7"/>
       <c r="L7" s="7"/>
@@ -4226,14 +4242,14 @@
       <c r="B8" s="53" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="140" t="b">
+      <c r="C8" s="204" t="b">
         <v>0</v>
       </c>
-      <c r="D8" s="141"/>
-      <c r="E8" s="142" t="s">
+      <c r="D8" s="205"/>
+      <c r="E8" s="206" t="s">
         <v>8</v>
       </c>
-      <c r="F8" s="143"/>
+      <c r="F8" s="207"/>
       <c r="G8" s="58" t="b">
         <v>0</v>
       </c>
@@ -4269,8 +4285,8 @@
       <c r="D9" s="18"/>
       <c r="E9" s="23"/>
       <c r="F9" s="23"/>
-      <c r="G9" s="106"/>
-      <c r="H9" s="106"/>
+      <c r="G9" s="219"/>
+      <c r="H9" s="219"/>
       <c r="I9" s="18"/>
       <c r="J9" s="7"/>
       <c r="K9" s="7"/>
@@ -4293,18 +4309,18 @@
       <c r="AB9" s="7"/>
     </row>
     <row r="10" spans="2:28" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="119" t="s">
+      <c r="B10" s="175" t="s">
         <v>10</v>
       </c>
-      <c r="C10" s="120"/>
-      <c r="D10" s="121"/>
-      <c r="E10" s="117" t="s">
+      <c r="C10" s="176"/>
+      <c r="D10" s="177"/>
+      <c r="E10" s="171" t="s">
         <v>11</v>
       </c>
-      <c r="F10" s="117"/>
-      <c r="G10" s="117"/>
-      <c r="H10" s="117"/>
-      <c r="I10" s="117"/>
+      <c r="F10" s="171"/>
+      <c r="G10" s="171"/>
+      <c r="H10" s="171"/>
+      <c r="I10" s="171"/>
       <c r="J10" s="7"/>
       <c r="K10" s="7"/>
       <c r="L10" s="7"/>
@@ -4326,14 +4342,14 @@
       <c r="AB10" s="7"/>
     </row>
     <row r="11" spans="2:28" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="122"/>
-      <c r="C11" s="123"/>
-      <c r="D11" s="124"/>
-      <c r="E11" s="118"/>
-      <c r="F11" s="118"/>
-      <c r="G11" s="118"/>
-      <c r="H11" s="118"/>
-      <c r="I11" s="118"/>
+      <c r="B11" s="163"/>
+      <c r="C11" s="164"/>
+      <c r="D11" s="165"/>
+      <c r="E11" s="218"/>
+      <c r="F11" s="218"/>
+      <c r="G11" s="218"/>
+      <c r="H11" s="218"/>
+      <c r="I11" s="218"/>
       <c r="J11" s="7"/>
       <c r="K11" s="7"/>
       <c r="L11" s="7"/>
@@ -4360,8 +4376,8 @@
       <c r="D12" s="18"/>
       <c r="E12" s="23"/>
       <c r="F12" s="23"/>
-      <c r="G12" s="106"/>
-      <c r="H12" s="106"/>
+      <c r="G12" s="219"/>
+      <c r="H12" s="219"/>
       <c r="I12" s="18"/>
       <c r="J12" s="7"/>
       <c r="K12" s="7"/>
@@ -4384,16 +4400,16 @@
       <c r="AB12" s="7"/>
     </row>
     <row r="13" spans="2:28" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="115" t="s">
+      <c r="B13" s="216" t="s">
         <v>12</v>
       </c>
-      <c r="C13" s="115"/>
-      <c r="D13" s="115"/>
-      <c r="E13" s="115"/>
-      <c r="F13" s="115"/>
-      <c r="G13" s="115"/>
-      <c r="H13" s="115"/>
-      <c r="I13" s="116"/>
+      <c r="C13" s="216"/>
+      <c r="D13" s="216"/>
+      <c r="E13" s="216"/>
+      <c r="F13" s="216"/>
+      <c r="G13" s="216"/>
+      <c r="H13" s="216"/>
+      <c r="I13" s="217"/>
       <c r="J13" s="7"/>
       <c r="K13" s="7"/>
       <c r="L13" s="7"/>
@@ -4415,32 +4431,32 @@
       <c r="AB13" s="7"/>
     </row>
     <row r="14" spans="2:28" s="9" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="119" t="s">
+      <c r="B14" s="175" t="s">
         <v>13</v>
       </c>
-      <c r="C14" s="120"/>
-      <c r="D14" s="121"/>
+      <c r="C14" s="176"/>
+      <c r="D14" s="177"/>
       <c r="E14" s="55" t="s">
         <v>14</v>
       </c>
-      <c r="F14" s="144" t="s">
+      <c r="F14" s="208" t="s">
         <v>15</v>
       </c>
-      <c r="G14" s="145"/>
-      <c r="H14" s="117" t="s">
+      <c r="G14" s="209"/>
+      <c r="H14" s="171" t="s">
         <v>16</v>
       </c>
-      <c r="I14" s="134"/>
+      <c r="I14" s="172"/>
     </row>
     <row r="15" spans="2:28" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="137"/>
-      <c r="C15" s="138"/>
-      <c r="D15" s="139"/>
+      <c r="B15" s="201"/>
+      <c r="C15" s="202"/>
+      <c r="D15" s="203"/>
       <c r="E15" s="37"/>
-      <c r="F15" s="146"/>
-      <c r="G15" s="147"/>
-      <c r="H15" s="135"/>
-      <c r="I15" s="136"/>
+      <c r="F15" s="210"/>
+      <c r="G15" s="211"/>
+      <c r="H15" s="185"/>
+      <c r="I15" s="200"/>
       <c r="J15" s="7"/>
       <c r="K15" s="7"/>
       <c r="L15" s="7"/>
@@ -4462,20 +4478,20 @@
       <c r="AB15" s="7"/>
     </row>
     <row r="16" spans="2:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="111" t="s">
+      <c r="B16" s="212" t="s">
         <v>17</v>
       </c>
-      <c r="C16" s="112"/>
-      <c r="D16" s="113"/>
-      <c r="E16" s="114" t="s">
+      <c r="C16" s="213"/>
+      <c r="D16" s="214"/>
+      <c r="E16" s="215" t="s">
         <v>18</v>
       </c>
-      <c r="F16" s="114"/>
-      <c r="G16" s="114"/>
-      <c r="H16" s="210" t="s">
+      <c r="F16" s="215"/>
+      <c r="G16" s="215"/>
+      <c r="H16" s="220" t="s">
         <v>19</v>
       </c>
-      <c r="I16" s="211"/>
+      <c r="I16" s="221"/>
       <c r="J16" s="7"/>
       <c r="K16" s="7"/>
       <c r="L16" s="7"/>
@@ -4497,14 +4513,14 @@
       <c r="AB16" s="7"/>
     </row>
     <row r="17" spans="2:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="122"/>
-      <c r="C17" s="123"/>
-      <c r="D17" s="124"/>
-      <c r="E17" s="209"/>
-      <c r="F17" s="209"/>
-      <c r="G17" s="209"/>
-      <c r="H17" s="165"/>
-      <c r="I17" s="166"/>
+      <c r="B17" s="163"/>
+      <c r="C17" s="164"/>
+      <c r="D17" s="165"/>
+      <c r="E17" s="181"/>
+      <c r="F17" s="181"/>
+      <c r="G17" s="181"/>
+      <c r="H17" s="173"/>
+      <c r="I17" s="174"/>
       <c r="J17" s="7"/>
       <c r="K17" s="7"/>
       <c r="L17" s="7"/>
@@ -4526,20 +4542,20 @@
       <c r="AB17" s="7"/>
     </row>
     <row r="18" spans="2:28" s="47" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="119" t="s">
+      <c r="B18" s="175" t="s">
         <v>20</v>
       </c>
-      <c r="C18" s="120"/>
-      <c r="D18" s="121"/>
-      <c r="E18" s="117" t="s">
+      <c r="C18" s="176"/>
+      <c r="D18" s="177"/>
+      <c r="E18" s="171" t="s">
         <v>21</v>
       </c>
-      <c r="F18" s="117"/>
-      <c r="G18" s="117"/>
-      <c r="H18" s="117" t="s">
+      <c r="F18" s="171"/>
+      <c r="G18" s="171"/>
+      <c r="H18" s="171" t="s">
         <v>22</v>
       </c>
-      <c r="I18" s="134"/>
+      <c r="I18" s="172"/>
       <c r="J18" s="7"/>
       <c r="K18" s="7"/>
       <c r="L18" s="7"/>
@@ -4561,14 +4577,14 @@
       <c r="AB18" s="7"/>
     </row>
     <row r="19" spans="2:28" s="47" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="167"/>
-      <c r="C19" s="168"/>
-      <c r="D19" s="169"/>
-      <c r="E19" s="165"/>
-      <c r="F19" s="165"/>
-      <c r="G19" s="165"/>
-      <c r="H19" s="165"/>
-      <c r="I19" s="166"/>
+      <c r="B19" s="178"/>
+      <c r="C19" s="179"/>
+      <c r="D19" s="180"/>
+      <c r="E19" s="173"/>
+      <c r="F19" s="173"/>
+      <c r="G19" s="173"/>
+      <c r="H19" s="173"/>
+      <c r="I19" s="174"/>
       <c r="J19" s="7"/>
       <c r="K19" s="7"/>
       <c r="L19" s="7"/>
@@ -4590,20 +4606,20 @@
       <c r="AB19" s="7"/>
     </row>
     <row r="20" spans="2:28" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="162" t="s">
+      <c r="B20" s="168" t="s">
         <v>23</v>
       </c>
-      <c r="C20" s="163"/>
-      <c r="D20" s="164"/>
-      <c r="E20" s="155" t="s">
+      <c r="C20" s="169"/>
+      <c r="D20" s="170"/>
+      <c r="E20" s="166" t="s">
         <v>24</v>
       </c>
-      <c r="F20" s="155"/>
-      <c r="G20" s="155"/>
-      <c r="H20" s="155" t="s">
+      <c r="F20" s="166"/>
+      <c r="G20" s="166"/>
+      <c r="H20" s="166" t="s">
         <v>25</v>
       </c>
-      <c r="I20" s="161"/>
+      <c r="I20" s="167"/>
       <c r="J20" s="16"/>
       <c r="K20" s="16"/>
       <c r="L20" s="16"/>
@@ -4623,14 +4639,14 @@
       <c r="AA20" s="16"/>
     </row>
     <row r="21" spans="2:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="122"/>
-      <c r="C21" s="123"/>
-      <c r="D21" s="124"/>
-      <c r="E21" s="135"/>
-      <c r="F21" s="135"/>
-      <c r="G21" s="135"/>
-      <c r="H21" s="153"/>
-      <c r="I21" s="154"/>
+      <c r="B21" s="163"/>
+      <c r="C21" s="164"/>
+      <c r="D21" s="165"/>
+      <c r="E21" s="185"/>
+      <c r="F21" s="185"/>
+      <c r="G21" s="185"/>
+      <c r="H21" s="183"/>
+      <c r="I21" s="184"/>
       <c r="J21" s="18"/>
       <c r="K21" s="18"/>
       <c r="L21" s="18"/>
@@ -4655,8 +4671,8 @@
       <c r="D22" s="13"/>
       <c r="E22" s="33"/>
       <c r="F22" s="33"/>
-      <c r="G22" s="105"/>
-      <c r="H22" s="105"/>
+      <c r="G22" s="78"/>
+      <c r="H22" s="78"/>
       <c r="I22" s="13"/>
       <c r="J22" s="13"/>
       <c r="K22" s="13"/>
@@ -4678,16 +4694,16 @@
       <c r="AA22" s="13"/>
     </row>
     <row r="23" spans="2:28" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="148" t="s">
+      <c r="B23" s="139" t="s">
         <v>26</v>
       </c>
-      <c r="C23" s="149"/>
-      <c r="D23" s="149"/>
-      <c r="E23" s="149"/>
-      <c r="F23" s="149"/>
-      <c r="G23" s="149"/>
-      <c r="H23" s="149"/>
-      <c r="I23" s="150"/>
+      <c r="C23" s="140"/>
+      <c r="D23" s="140"/>
+      <c r="E23" s="140"/>
+      <c r="F23" s="140"/>
+      <c r="G23" s="140"/>
+      <c r="H23" s="140"/>
+      <c r="I23" s="141"/>
       <c r="J23" s="13"/>
       <c r="K23" s="13"/>
       <c r="L23" s="13"/>
@@ -4708,20 +4724,20 @@
       <c r="AA23" s="13"/>
     </row>
     <row r="24" spans="2:28" s="9" customFormat="1" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="151" t="s">
+      <c r="B24" s="182" t="s">
         <v>27</v>
       </c>
-      <c r="C24" s="152"/>
-      <c r="D24" s="152"/>
-      <c r="E24" s="152"/>
-      <c r="F24" s="156" t="s">
+      <c r="C24" s="88"/>
+      <c r="D24" s="88"/>
+      <c r="E24" s="88"/>
+      <c r="F24" s="186" t="s">
         <v>28</v>
       </c>
-      <c r="G24" s="156"/>
-      <c r="H24" s="152" t="s">
+      <c r="G24" s="186"/>
+      <c r="H24" s="88" t="s">
         <v>29</v>
       </c>
-      <c r="I24" s="226"/>
+      <c r="I24" s="89"/>
       <c r="J24" s="18"/>
       <c r="K24" s="18"/>
       <c r="M24" s="16"/>
@@ -4734,14 +4750,14 @@
       <c r="AB24" s="10"/>
     </row>
     <row r="25" spans="2:28" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="193"/>
-      <c r="C25" s="157"/>
-      <c r="D25" s="157"/>
-      <c r="E25" s="157"/>
-      <c r="F25" s="157"/>
-      <c r="G25" s="157"/>
-      <c r="H25" s="227"/>
-      <c r="I25" s="228"/>
+      <c r="B25" s="137"/>
+      <c r="C25" s="138"/>
+      <c r="D25" s="138"/>
+      <c r="E25" s="138"/>
+      <c r="F25" s="138"/>
+      <c r="G25" s="138"/>
+      <c r="H25" s="90"/>
+      <c r="I25" s="91"/>
       <c r="J25" s="18"/>
       <c r="K25" s="18"/>
       <c r="M25" s="18"/>
@@ -4758,8 +4774,8 @@
       <c r="D26" s="13"/>
       <c r="E26" s="33"/>
       <c r="F26" s="33"/>
-      <c r="G26" s="105"/>
-      <c r="H26" s="105"/>
+      <c r="G26" s="78"/>
+      <c r="H26" s="78"/>
       <c r="I26" s="13"/>
       <c r="J26" s="13"/>
       <c r="K26" s="13"/>
@@ -4781,16 +4797,16 @@
       <c r="AA26" s="13"/>
     </row>
     <row r="27" spans="2:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B27" s="190" t="s">
+      <c r="B27" s="134" t="s">
         <v>30</v>
       </c>
-      <c r="C27" s="191"/>
-      <c r="D27" s="191"/>
-      <c r="E27" s="191"/>
-      <c r="F27" s="191"/>
-      <c r="G27" s="191"/>
-      <c r="H27" s="191"/>
-      <c r="I27" s="192"/>
+      <c r="C27" s="135"/>
+      <c r="D27" s="135"/>
+      <c r="E27" s="135"/>
+      <c r="F27" s="135"/>
+      <c r="G27" s="135"/>
+      <c r="H27" s="135"/>
+      <c r="I27" s="136"/>
       <c r="J27" s="13"/>
       <c r="K27" s="13"/>
       <c r="L27" s="13"/>
@@ -4811,22 +4827,22 @@
       <c r="AA27" s="13"/>
     </row>
     <row r="28" spans="2:28" s="9" customFormat="1" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B28" s="229" t="s">
+      <c r="B28" s="92" t="s">
         <v>31</v>
       </c>
-      <c r="C28" s="152"/>
-      <c r="D28" s="152"/>
-      <c r="E28" s="156" t="s">
+      <c r="C28" s="88"/>
+      <c r="D28" s="88"/>
+      <c r="E28" s="186" t="s">
         <v>32</v>
       </c>
-      <c r="F28" s="156"/>
+      <c r="F28" s="186"/>
       <c r="G28" s="49" t="s">
         <v>33</v>
       </c>
-      <c r="H28" s="152" t="s">
+      <c r="H28" s="88" t="s">
         <v>34</v>
       </c>
-      <c r="I28" s="230"/>
+      <c r="I28" s="95"/>
       <c r="J28" s="16"/>
       <c r="N28" s="16"/>
       <c r="O28" s="16"/>
@@ -4843,14 +4859,14 @@
       <c r="AB28" s="10"/>
     </row>
     <row r="29" spans="2:28" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B29" s="69"/>
-      <c r="C29" s="70"/>
-      <c r="D29" s="70"/>
-      <c r="E29" s="70"/>
-      <c r="F29" s="70"/>
+      <c r="B29" s="93"/>
+      <c r="C29" s="94"/>
+      <c r="D29" s="94"/>
+      <c r="E29" s="94"/>
+      <c r="F29" s="94"/>
       <c r="G29" s="52"/>
-      <c r="H29" s="70"/>
-      <c r="I29" s="110"/>
+      <c r="H29" s="94"/>
+      <c r="I29" s="188"/>
       <c r="J29" s="18"/>
       <c r="N29" s="18"/>
       <c r="O29" s="18"/>
@@ -4871,8 +4887,8 @@
       <c r="D30" s="13"/>
       <c r="E30" s="33"/>
       <c r="F30" s="33"/>
-      <c r="G30" s="105"/>
-      <c r="H30" s="105"/>
+      <c r="G30" s="78"/>
+      <c r="H30" s="78"/>
       <c r="I30" s="13"/>
       <c r="J30" s="13"/>
       <c r="K30" s="13"/>
@@ -4894,16 +4910,16 @@
       <c r="AA30" s="13"/>
     </row>
     <row r="31" spans="2:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B31" s="148" t="s">
+      <c r="B31" s="139" t="s">
         <v>35</v>
       </c>
-      <c r="C31" s="149"/>
-      <c r="D31" s="149"/>
-      <c r="E31" s="149"/>
-      <c r="F31" s="149"/>
-      <c r="G31" s="149"/>
-      <c r="H31" s="149"/>
-      <c r="I31" s="150"/>
+      <c r="C31" s="140"/>
+      <c r="D31" s="140"/>
+      <c r="E31" s="140"/>
+      <c r="F31" s="140"/>
+      <c r="G31" s="140"/>
+      <c r="H31" s="140"/>
+      <c r="I31" s="141"/>
       <c r="J31" s="7"/>
       <c r="K31" s="7"/>
       <c r="L31" s="7"/>
@@ -4925,18 +4941,18 @@
       <c r="AB31" s="7"/>
     </row>
     <row r="32" spans="2:28" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B32" s="158" t="s">
+      <c r="B32" s="189" t="s">
         <v>36</v>
       </c>
-      <c r="C32" s="159"/>
-      <c r="D32" s="159"/>
-      <c r="E32" s="159"/>
-      <c r="F32" s="160"/>
-      <c r="G32" s="202" t="s">
+      <c r="C32" s="151"/>
+      <c r="D32" s="151"/>
+      <c r="E32" s="151"/>
+      <c r="F32" s="190"/>
+      <c r="G32" s="150" t="s">
         <v>37</v>
       </c>
-      <c r="H32" s="159"/>
-      <c r="I32" s="203"/>
+      <c r="H32" s="151"/>
+      <c r="I32" s="152"/>
       <c r="J32" s="7"/>
       <c r="K32" s="7"/>
       <c r="L32" s="7"/>
@@ -4958,18 +4974,18 @@
       <c r="AB32" s="7"/>
     </row>
     <row r="33" spans="2:28" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B33" s="199" t="s">
+      <c r="B33" s="147" t="s">
         <v>104</v>
       </c>
-      <c r="C33" s="200"/>
-      <c r="D33" s="200"/>
-      <c r="E33" s="200"/>
-      <c r="F33" s="201"/>
-      <c r="G33" s="204" t="s">
+      <c r="C33" s="148"/>
+      <c r="D33" s="148"/>
+      <c r="E33" s="148"/>
+      <c r="F33" s="149"/>
+      <c r="G33" s="153" t="s">
         <v>105</v>
       </c>
-      <c r="H33" s="200"/>
-      <c r="I33" s="205"/>
+      <c r="H33" s="148"/>
+      <c r="I33" s="154"/>
       <c r="J33" s="7"/>
       <c r="K33" s="7"/>
       <c r="L33" s="7"/>
@@ -4996,8 +5012,8 @@
       <c r="D34" s="13"/>
       <c r="E34" s="33"/>
       <c r="F34" s="33"/>
-      <c r="G34" s="105"/>
-      <c r="H34" s="105"/>
+      <c r="G34" s="78"/>
+      <c r="H34" s="78"/>
       <c r="I34" s="13"/>
       <c r="J34" s="13"/>
       <c r="K34" s="13"/>
@@ -5019,16 +5035,16 @@
       <c r="AA34" s="13"/>
     </row>
     <row r="35" spans="2:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B35" s="218" t="s">
+      <c r="B35" s="110" t="s">
         <v>38</v>
       </c>
-      <c r="C35" s="219"/>
-      <c r="D35" s="219"/>
-      <c r="E35" s="219"/>
-      <c r="F35" s="219"/>
-      <c r="G35" s="219"/>
-      <c r="H35" s="219"/>
-      <c r="I35" s="220"/>
+      <c r="C35" s="111"/>
+      <c r="D35" s="111"/>
+      <c r="E35" s="111"/>
+      <c r="F35" s="111"/>
+      <c r="G35" s="111"/>
+      <c r="H35" s="111"/>
+      <c r="I35" s="112"/>
       <c r="J35" s="39"/>
       <c r="K35" s="19"/>
       <c r="L35" s="19"/>
@@ -5052,19 +5068,19 @@
       <c r="B36" s="41" t="s">
         <v>39</v>
       </c>
-      <c r="C36" s="196" t="s">
+      <c r="C36" s="144" t="s">
         <v>40</v>
       </c>
-      <c r="D36" s="197"/>
-      <c r="E36" s="197"/>
-      <c r="F36" s="198"/>
+      <c r="D36" s="145"/>
+      <c r="E36" s="145"/>
+      <c r="F36" s="146"/>
       <c r="G36" s="41" t="s">
         <v>39</v>
       </c>
-      <c r="H36" s="194" t="s">
+      <c r="H36" s="142" t="s">
         <v>41</v>
       </c>
-      <c r="I36" s="195"/>
+      <c r="I36" s="143"/>
       <c r="J36" s="40"/>
       <c r="K36" s="19"/>
       <c r="L36" s="19"/>
@@ -5085,18 +5101,18 @@
       <c r="AA36" s="20"/>
     </row>
     <row r="37" spans="2:28" s="11" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B37" s="170" t="s">
+      <c r="B37" s="100" t="s">
         <v>42</v>
       </c>
-      <c r="C37" s="174"/>
-      <c r="D37" s="175"/>
-      <c r="E37" s="175"/>
-      <c r="F37" s="176"/>
-      <c r="G37" s="170" t="s">
+      <c r="C37" s="118"/>
+      <c r="D37" s="119"/>
+      <c r="E37" s="119"/>
+      <c r="F37" s="120"/>
+      <c r="G37" s="100" t="s">
         <v>43</v>
       </c>
-      <c r="H37" s="221"/>
-      <c r="I37" s="222"/>
+      <c r="H37" s="96"/>
+      <c r="I37" s="97"/>
       <c r="J37" s="39"/>
       <c r="K37" s="16"/>
       <c r="L37" s="18"/>
@@ -5115,14 +5131,14 @@
       <c r="AB37" s="12"/>
     </row>
     <row r="38" spans="2:28" s="11" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B38" s="233"/>
-      <c r="C38" s="177"/>
-      <c r="D38" s="105"/>
-      <c r="E38" s="105"/>
-      <c r="F38" s="178"/>
-      <c r="G38" s="171"/>
-      <c r="H38" s="223"/>
-      <c r="I38" s="224"/>
+      <c r="B38" s="101"/>
+      <c r="C38" s="121"/>
+      <c r="D38" s="78"/>
+      <c r="E38" s="78"/>
+      <c r="F38" s="122"/>
+      <c r="G38" s="103"/>
+      <c r="H38" s="98"/>
+      <c r="I38" s="99"/>
       <c r="J38" s="39"/>
       <c r="K38" s="16"/>
       <c r="L38" s="18"/>
@@ -5140,16 +5156,16 @@
       <c r="AB38" s="12"/>
     </row>
     <row r="39" spans="2:28" s="11" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B39" s="233"/>
-      <c r="C39" s="177"/>
-      <c r="D39" s="105"/>
-      <c r="E39" s="105"/>
-      <c r="F39" s="178"/>
-      <c r="G39" s="170" t="s">
+      <c r="B39" s="101"/>
+      <c r="C39" s="121"/>
+      <c r="D39" s="78"/>
+      <c r="E39" s="78"/>
+      <c r="F39" s="122"/>
+      <c r="G39" s="100" t="s">
         <v>44</v>
       </c>
-      <c r="H39" s="221"/>
-      <c r="I39" s="222"/>
+      <c r="H39" s="96"/>
+      <c r="I39" s="97"/>
       <c r="J39" s="39"/>
       <c r="K39" s="16"/>
       <c r="L39" s="18"/>
@@ -5168,14 +5184,14 @@
       <c r="AB39" s="12"/>
     </row>
     <row r="40" spans="2:28" s="11" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B40" s="234"/>
-      <c r="C40" s="179"/>
-      <c r="D40" s="180"/>
-      <c r="E40" s="180"/>
-      <c r="F40" s="181"/>
-      <c r="G40" s="171"/>
-      <c r="H40" s="223"/>
-      <c r="I40" s="224"/>
+      <c r="B40" s="102"/>
+      <c r="C40" s="123"/>
+      <c r="D40" s="124"/>
+      <c r="E40" s="124"/>
+      <c r="F40" s="125"/>
+      <c r="G40" s="103"/>
+      <c r="H40" s="98"/>
+      <c r="I40" s="99"/>
       <c r="J40" s="39"/>
       <c r="K40" s="16"/>
       <c r="L40" s="18"/>
@@ -5194,18 +5210,18 @@
       <c r="AB40" s="12"/>
     </row>
     <row r="41" spans="2:28" s="11" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B41" s="188" t="s">
+      <c r="B41" s="132" t="s">
         <v>45</v>
       </c>
-      <c r="C41" s="182"/>
-      <c r="D41" s="183"/>
-      <c r="E41" s="183"/>
-      <c r="F41" s="184"/>
-      <c r="G41" s="170" t="s">
+      <c r="C41" s="126"/>
+      <c r="D41" s="127"/>
+      <c r="E41" s="127"/>
+      <c r="F41" s="128"/>
+      <c r="G41" s="100" t="s">
         <v>46</v>
       </c>
-      <c r="H41" s="214"/>
-      <c r="I41" s="215"/>
+      <c r="H41" s="106"/>
+      <c r="I41" s="107"/>
       <c r="J41" s="56"/>
       <c r="K41" s="16"/>
       <c r="L41" s="17"/>
@@ -5227,14 +5243,14 @@
       <c r="AB41" s="12"/>
     </row>
     <row r="42" spans="2:28" s="38" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B42" s="189"/>
-      <c r="C42" s="185"/>
-      <c r="D42" s="186"/>
-      <c r="E42" s="186"/>
-      <c r="F42" s="187"/>
-      <c r="G42" s="213"/>
-      <c r="H42" s="216"/>
-      <c r="I42" s="217"/>
+      <c r="B42" s="133"/>
+      <c r="C42" s="129"/>
+      <c r="D42" s="130"/>
+      <c r="E42" s="130"/>
+      <c r="F42" s="131"/>
+      <c r="G42" s="105"/>
+      <c r="H42" s="108"/>
+      <c r="I42" s="109"/>
       <c r="J42" s="56"/>
       <c r="K42" s="16"/>
       <c r="L42" s="17"/>
@@ -5261,8 +5277,8 @@
       <c r="D43" s="43"/>
       <c r="E43" s="43"/>
       <c r="F43" s="43"/>
-      <c r="G43" s="172"/>
-      <c r="H43" s="173"/>
+      <c r="G43" s="116"/>
+      <c r="H43" s="117"/>
       <c r="I43" s="43"/>
       <c r="J43" s="56"/>
       <c r="K43" s="16"/>
@@ -5285,16 +5301,16 @@
       <c r="AB43" s="12"/>
     </row>
     <row r="44" spans="2:28" s="11" customFormat="1" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B44" s="231" t="s">
+      <c r="B44" s="114" t="s">
         <v>47</v>
       </c>
-      <c r="C44" s="231"/>
-      <c r="D44" s="231"/>
-      <c r="E44" s="231"/>
-      <c r="F44" s="231"/>
-      <c r="G44" s="231"/>
-      <c r="H44" s="231"/>
-      <c r="I44" s="232"/>
+      <c r="C44" s="114"/>
+      <c r="D44" s="114"/>
+      <c r="E44" s="114"/>
+      <c r="F44" s="114"/>
+      <c r="G44" s="114"/>
+      <c r="H44" s="114"/>
+      <c r="I44" s="115"/>
       <c r="J44" s="16"/>
       <c r="K44" s="16"/>
       <c r="L44" s="17"/>
@@ -5316,24 +5332,24 @@
       <c r="AB44" s="12"/>
     </row>
     <row r="45" spans="2:28" ht="68.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B45" s="208" t="s">
+      <c r="B45" s="161" t="s">
         <v>48</v>
       </c>
-      <c r="C45" s="102"/>
-      <c r="D45" s="99" t="s">
+      <c r="C45" s="162"/>
+      <c r="D45" s="222" t="s">
         <v>49</v>
       </c>
-      <c r="E45" s="100"/>
-      <c r="F45" s="103" t="s">
+      <c r="E45" s="223"/>
+      <c r="F45" s="160" t="s">
         <v>50</v>
       </c>
-      <c r="G45" s="103" t="s">
+      <c r="G45" s="160" t="s">
         <v>51</v>
       </c>
-      <c r="H45" s="206" t="s">
+      <c r="H45" s="158" t="s">
         <v>52</v>
       </c>
-      <c r="I45" s="212" t="s">
+      <c r="I45" s="104" t="s">
         <v>53</v>
       </c>
       <c r="J45" s="16"/>
@@ -5356,14 +5372,14 @@
       <c r="AA45" s="16"/>
     </row>
     <row r="46" spans="2:28" ht="66.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B46" s="208"/>
-      <c r="C46" s="102"/>
-      <c r="D46" s="101"/>
-      <c r="E46" s="102"/>
-      <c r="F46" s="104"/>
-      <c r="G46" s="103"/>
-      <c r="H46" s="207"/>
-      <c r="I46" s="212"/>
+      <c r="B46" s="161"/>
+      <c r="C46" s="162"/>
+      <c r="D46" s="224"/>
+      <c r="E46" s="162"/>
+      <c r="F46" s="225"/>
+      <c r="G46" s="160"/>
+      <c r="H46" s="159"/>
+      <c r="I46" s="104"/>
       <c r="J46" s="16"/>
       <c r="K46" s="16"/>
       <c r="L46" s="16"/>
@@ -5384,14 +5400,14 @@
       <c r="AA46" s="16"/>
     </row>
     <row r="47" spans="2:28" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B47" s="67"/>
-      <c r="C47" s="68"/>
-      <c r="D47" s="68"/>
-      <c r="E47" s="68"/>
-      <c r="F47" s="97"/>
-      <c r="G47" s="68"/>
-      <c r="H47" s="68"/>
-      <c r="I47" s="109"/>
+      <c r="B47" s="187"/>
+      <c r="C47" s="155"/>
+      <c r="D47" s="155"/>
+      <c r="E47" s="155"/>
+      <c r="F47" s="156"/>
+      <c r="G47" s="155"/>
+      <c r="H47" s="155"/>
+      <c r="I47" s="157"/>
       <c r="J47" s="18"/>
       <c r="K47" s="16"/>
       <c r="L47" s="16"/>
@@ -5412,14 +5428,14 @@
       <c r="AA47" s="16"/>
     </row>
     <row r="48" spans="2:28" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B48" s="67"/>
-      <c r="C48" s="68"/>
-      <c r="D48" s="68"/>
-      <c r="E48" s="68"/>
-      <c r="F48" s="97"/>
-      <c r="G48" s="68"/>
-      <c r="H48" s="68"/>
-      <c r="I48" s="109"/>
+      <c r="B48" s="187"/>
+      <c r="C48" s="155"/>
+      <c r="D48" s="155"/>
+      <c r="E48" s="155"/>
+      <c r="F48" s="156"/>
+      <c r="G48" s="155"/>
+      <c r="H48" s="155"/>
+      <c r="I48" s="157"/>
       <c r="J48" s="18"/>
       <c r="K48" s="16"/>
       <c r="L48" s="16"/>
@@ -5440,14 +5456,14 @@
       <c r="AA48" s="16"/>
     </row>
     <row r="49" spans="2:28" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B49" s="67"/>
-      <c r="C49" s="68"/>
-      <c r="D49" s="68"/>
-      <c r="E49" s="68"/>
-      <c r="F49" s="97"/>
-      <c r="G49" s="68"/>
-      <c r="H49" s="68"/>
-      <c r="I49" s="109"/>
+      <c r="B49" s="187"/>
+      <c r="C49" s="155"/>
+      <c r="D49" s="155"/>
+      <c r="E49" s="155"/>
+      <c r="F49" s="156"/>
+      <c r="G49" s="155"/>
+      <c r="H49" s="155"/>
+      <c r="I49" s="157"/>
       <c r="J49" s="18"/>
       <c r="K49" s="16"/>
       <c r="L49" s="16"/>
@@ -5468,14 +5484,14 @@
       <c r="AA49" s="16"/>
     </row>
     <row r="50" spans="2:28" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B50" s="67"/>
-      <c r="C50" s="68"/>
-      <c r="D50" s="68"/>
-      <c r="E50" s="68"/>
-      <c r="F50" s="97"/>
-      <c r="G50" s="68"/>
-      <c r="H50" s="68"/>
-      <c r="I50" s="109"/>
+      <c r="B50" s="187"/>
+      <c r="C50" s="155"/>
+      <c r="D50" s="155"/>
+      <c r="E50" s="155"/>
+      <c r="F50" s="156"/>
+      <c r="G50" s="155"/>
+      <c r="H50" s="155"/>
+      <c r="I50" s="157"/>
       <c r="J50" s="18"/>
       <c r="K50" s="16"/>
       <c r="L50" s="16"/>
@@ -5496,14 +5512,14 @@
       <c r="AA50" s="16"/>
     </row>
     <row r="51" spans="2:28" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B51" s="67"/>
-      <c r="C51" s="68"/>
-      <c r="D51" s="68"/>
-      <c r="E51" s="68"/>
-      <c r="F51" s="97"/>
-      <c r="G51" s="68"/>
-      <c r="H51" s="68"/>
-      <c r="I51" s="109"/>
+      <c r="B51" s="187"/>
+      <c r="C51" s="155"/>
+      <c r="D51" s="155"/>
+      <c r="E51" s="155"/>
+      <c r="F51" s="156"/>
+      <c r="G51" s="155"/>
+      <c r="H51" s="155"/>
+      <c r="I51" s="157"/>
       <c r="J51" s="18"/>
       <c r="K51" s="16"/>
       <c r="L51" s="16"/>
@@ -5524,14 +5540,14 @@
       <c r="AA51" s="16"/>
     </row>
     <row r="52" spans="2:28" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B52" s="67"/>
-      <c r="C52" s="68"/>
-      <c r="D52" s="68"/>
-      <c r="E52" s="68"/>
-      <c r="F52" s="97"/>
-      <c r="G52" s="68"/>
-      <c r="H52" s="68"/>
-      <c r="I52" s="109"/>
+      <c r="B52" s="187"/>
+      <c r="C52" s="155"/>
+      <c r="D52" s="155"/>
+      <c r="E52" s="155"/>
+      <c r="F52" s="156"/>
+      <c r="G52" s="155"/>
+      <c r="H52" s="155"/>
+      <c r="I52" s="157"/>
       <c r="J52" s="18"/>
       <c r="K52" s="16"/>
       <c r="L52" s="16"/>
@@ -5552,14 +5568,14 @@
       <c r="AA52" s="16"/>
     </row>
     <row r="53" spans="2:28" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B53" s="67"/>
-      <c r="C53" s="68"/>
-      <c r="D53" s="68"/>
-      <c r="E53" s="68"/>
-      <c r="F53" s="97"/>
-      <c r="G53" s="68"/>
-      <c r="H53" s="68"/>
-      <c r="I53" s="109"/>
+      <c r="B53" s="187"/>
+      <c r="C53" s="155"/>
+      <c r="D53" s="155"/>
+      <c r="E53" s="155"/>
+      <c r="F53" s="156"/>
+      <c r="G53" s="155"/>
+      <c r="H53" s="155"/>
+      <c r="I53" s="157"/>
       <c r="J53" s="18"/>
       <c r="K53" s="16"/>
       <c r="L53" s="16"/>
@@ -5580,14 +5596,14 @@
       <c r="AA53" s="16"/>
     </row>
     <row r="54" spans="2:28" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B54" s="67"/>
-      <c r="C54" s="68"/>
-      <c r="D54" s="68"/>
-      <c r="E54" s="68"/>
-      <c r="F54" s="97"/>
-      <c r="G54" s="68"/>
-      <c r="H54" s="68"/>
-      <c r="I54" s="109"/>
+      <c r="B54" s="187"/>
+      <c r="C54" s="155"/>
+      <c r="D54" s="155"/>
+      <c r="E54" s="155"/>
+      <c r="F54" s="156"/>
+      <c r="G54" s="155"/>
+      <c r="H54" s="155"/>
+      <c r="I54" s="157"/>
       <c r="J54" s="18"/>
       <c r="K54" s="16"/>
       <c r="L54" s="16"/>
@@ -5608,14 +5624,14 @@
       <c r="AA54" s="16"/>
     </row>
     <row r="55" spans="2:28" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B55" s="67"/>
-      <c r="C55" s="68"/>
-      <c r="D55" s="68"/>
-      <c r="E55" s="68"/>
-      <c r="F55" s="97"/>
-      <c r="G55" s="68"/>
-      <c r="H55" s="68"/>
-      <c r="I55" s="109"/>
+      <c r="B55" s="187"/>
+      <c r="C55" s="155"/>
+      <c r="D55" s="155"/>
+      <c r="E55" s="155"/>
+      <c r="F55" s="156"/>
+      <c r="G55" s="155"/>
+      <c r="H55" s="155"/>
+      <c r="I55" s="157"/>
       <c r="J55" s="18"/>
       <c r="K55" s="16"/>
       <c r="L55" s="16"/>
@@ -5636,14 +5652,14 @@
       <c r="AA55" s="16"/>
     </row>
     <row r="56" spans="2:28" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B56" s="69"/>
-      <c r="C56" s="70"/>
-      <c r="D56" s="70"/>
-      <c r="E56" s="70"/>
-      <c r="F56" s="98"/>
-      <c r="G56" s="70"/>
-      <c r="H56" s="70"/>
-      <c r="I56" s="110"/>
+      <c r="B56" s="93"/>
+      <c r="C56" s="94"/>
+      <c r="D56" s="94"/>
+      <c r="E56" s="94"/>
+      <c r="F56" s="250"/>
+      <c r="G56" s="94"/>
+      <c r="H56" s="94"/>
+      <c r="I56" s="188"/>
       <c r="J56" s="18"/>
       <c r="K56" s="16"/>
       <c r="L56" s="16"/>
@@ -5669,8 +5685,8 @@
       <c r="D57" s="18"/>
       <c r="E57" s="23"/>
       <c r="F57" s="23"/>
-      <c r="G57" s="106"/>
-      <c r="H57" s="106"/>
+      <c r="G57" s="219"/>
+      <c r="H57" s="219"/>
       <c r="I57" s="18"/>
       <c r="J57" s="18"/>
       <c r="K57" s="16"/>
@@ -5692,16 +5708,16 @@
       <c r="AA57" s="16"/>
     </row>
     <row r="58" spans="2:28" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B58" s="78" t="s">
+      <c r="B58" s="226" t="s">
         <v>54</v>
       </c>
-      <c r="C58" s="79"/>
-      <c r="D58" s="79"/>
-      <c r="E58" s="79"/>
-      <c r="F58" s="79"/>
-      <c r="G58" s="79"/>
-      <c r="H58" s="79"/>
-      <c r="I58" s="80"/>
+      <c r="C58" s="227"/>
+      <c r="D58" s="227"/>
+      <c r="E58" s="227"/>
+      <c r="F58" s="227"/>
+      <c r="G58" s="227"/>
+      <c r="H58" s="227"/>
+      <c r="I58" s="228"/>
       <c r="J58" s="18"/>
       <c r="K58" s="16"/>
       <c r="L58" s="16"/>
@@ -5722,16 +5738,16 @@
       <c r="AA58" s="16"/>
     </row>
     <row r="59" spans="2:28" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B59" s="235" t="s">
+      <c r="B59" s="70" t="s">
         <v>55</v>
       </c>
-      <c r="C59" s="236"/>
-      <c r="D59" s="236"/>
-      <c r="E59" s="236"/>
-      <c r="F59" s="236"/>
-      <c r="G59" s="236"/>
-      <c r="H59" s="236"/>
-      <c r="I59" s="237"/>
+      <c r="C59" s="71"/>
+      <c r="D59" s="71"/>
+      <c r="E59" s="71"/>
+      <c r="F59" s="71"/>
+      <c r="G59" s="71"/>
+      <c r="H59" s="71"/>
+      <c r="I59" s="72"/>
       <c r="J59" s="19"/>
       <c r="K59" s="19"/>
       <c r="L59" s="19"/>
@@ -5752,16 +5768,16 @@
       <c r="AA59" s="19"/>
     </row>
     <row r="60" spans="2:28" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B60" s="78" t="s">
+      <c r="B60" s="226" t="s">
         <v>56</v>
       </c>
-      <c r="C60" s="79"/>
-      <c r="D60" s="79"/>
-      <c r="E60" s="79"/>
-      <c r="F60" s="79"/>
-      <c r="G60" s="79"/>
-      <c r="H60" s="79"/>
-      <c r="I60" s="80"/>
+      <c r="C60" s="227"/>
+      <c r="D60" s="227"/>
+      <c r="E60" s="227"/>
+      <c r="F60" s="227"/>
+      <c r="G60" s="227"/>
+      <c r="H60" s="227"/>
+      <c r="I60" s="228"/>
       <c r="J60" s="19"/>
       <c r="K60" s="19"/>
       <c r="L60" s="19"/>
@@ -5782,16 +5798,16 @@
       <c r="AA60" s="19"/>
     </row>
     <row r="61" spans="2:28" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B61" s="82" t="s">
+      <c r="B61" s="239" t="s">
         <v>57</v>
       </c>
-      <c r="C61" s="83"/>
-      <c r="D61" s="83"/>
-      <c r="E61" s="83"/>
-      <c r="F61" s="83"/>
-      <c r="G61" s="83"/>
-      <c r="H61" s="83"/>
-      <c r="I61" s="84"/>
+      <c r="C61" s="240"/>
+      <c r="D61" s="240"/>
+      <c r="E61" s="240"/>
+      <c r="F61" s="240"/>
+      <c r="G61" s="240"/>
+      <c r="H61" s="240"/>
+      <c r="I61" s="241"/>
       <c r="J61" s="22"/>
       <c r="K61" s="22"/>
       <c r="L61" s="22"/>
@@ -5812,14 +5828,14 @@
       <c r="AA61" s="22"/>
     </row>
     <row r="62" spans="2:28" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B62" s="85"/>
-      <c r="C62" s="86"/>
-      <c r="D62" s="86"/>
-      <c r="E62" s="86"/>
-      <c r="F62" s="86"/>
-      <c r="G62" s="86"/>
-      <c r="H62" s="86"/>
-      <c r="I62" s="87"/>
+      <c r="B62" s="242"/>
+      <c r="C62" s="243"/>
+      <c r="D62" s="243"/>
+      <c r="E62" s="243"/>
+      <c r="F62" s="243"/>
+      <c r="G62" s="243"/>
+      <c r="H62" s="243"/>
+      <c r="I62" s="244"/>
       <c r="J62" s="22"/>
       <c r="K62" s="22"/>
       <c r="L62" s="22"/>
@@ -5840,16 +5856,16 @@
       <c r="AA62" s="22"/>
     </row>
     <row r="63" spans="2:28" s="46" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B63" s="85" t="s">
+      <c r="B63" s="242" t="s">
         <v>58</v>
       </c>
-      <c r="C63" s="86"/>
-      <c r="D63" s="86"/>
-      <c r="E63" s="86"/>
-      <c r="F63" s="86"/>
-      <c r="G63" s="86"/>
-      <c r="H63" s="86"/>
-      <c r="I63" s="87"/>
+      <c r="C63" s="243"/>
+      <c r="D63" s="243"/>
+      <c r="E63" s="243"/>
+      <c r="F63" s="243"/>
+      <c r="G63" s="243"/>
+      <c r="H63" s="243"/>
+      <c r="I63" s="244"/>
       <c r="J63" s="44"/>
       <c r="K63" s="44"/>
       <c r="L63" s="44"/>
@@ -5871,16 +5887,16 @@
       <c r="AB63" s="45"/>
     </row>
     <row r="64" spans="2:28" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B64" s="90" t="s">
+      <c r="B64" s="245" t="s">
         <v>59</v>
       </c>
-      <c r="C64" s="91"/>
-      <c r="D64" s="91"/>
-      <c r="E64" s="91"/>
-      <c r="F64" s="91"/>
-      <c r="G64" s="91"/>
-      <c r="H64" s="91"/>
-      <c r="I64" s="92"/>
+      <c r="C64" s="246"/>
+      <c r="D64" s="246"/>
+      <c r="E64" s="246"/>
+      <c r="F64" s="246"/>
+      <c r="G64" s="246"/>
+      <c r="H64" s="246"/>
+      <c r="I64" s="247"/>
       <c r="J64" s="22"/>
       <c r="K64" s="22"/>
       <c r="L64" s="22"/>
@@ -5904,19 +5920,19 @@
       <c r="B65" s="50" t="s">
         <v>60</v>
       </c>
-      <c r="C65" s="88" t="s">
+      <c r="C65" s="86" t="s">
         <v>61</v>
       </c>
-      <c r="D65" s="88"/>
-      <c r="E65" s="88" t="s">
+      <c r="D65" s="86"/>
+      <c r="E65" s="86" t="s">
         <v>62</v>
       </c>
-      <c r="F65" s="88"/>
-      <c r="G65" s="245"/>
-      <c r="H65" s="88" t="s">
+      <c r="F65" s="86"/>
+      <c r="G65" s="82"/>
+      <c r="H65" s="86" t="s">
         <v>63</v>
       </c>
-      <c r="I65" s="247"/>
+      <c r="I65" s="84"/>
       <c r="J65" s="16"/>
       <c r="K65" s="16"/>
       <c r="L65" s="16"/>
@@ -5939,13 +5955,13 @@
     </row>
     <row r="66" spans="2:28" ht="32.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B66" s="51"/>
-      <c r="C66" s="95"/>
-      <c r="D66" s="95"/>
-      <c r="E66" s="89"/>
-      <c r="F66" s="89"/>
-      <c r="G66" s="246"/>
-      <c r="H66" s="89"/>
-      <c r="I66" s="248"/>
+      <c r="C66" s="248"/>
+      <c r="D66" s="248"/>
+      <c r="E66" s="87"/>
+      <c r="F66" s="87"/>
+      <c r="G66" s="83"/>
+      <c r="H66" s="87"/>
+      <c r="I66" s="85"/>
       <c r="J66" s="16"/>
       <c r="K66" s="16"/>
       <c r="L66" s="16"/>
@@ -5972,8 +5988,8 @@
       <c r="D67" s="17"/>
       <c r="E67" s="34"/>
       <c r="F67" s="34"/>
-      <c r="G67" s="93"/>
-      <c r="H67" s="93"/>
+      <c r="G67" s="229"/>
+      <c r="H67" s="229"/>
       <c r="I67" s="17"/>
       <c r="J67" s="16"/>
       <c r="K67" s="16"/>
@@ -5996,16 +6012,16 @@
       <c r="AB67" s="16"/>
     </row>
     <row r="68" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B68" s="81" t="s">
+      <c r="B68" s="238" t="s">
         <v>64</v>
       </c>
-      <c r="C68" s="81"/>
-      <c r="D68" s="81"/>
-      <c r="E68" s="81"/>
-      <c r="F68" s="81"/>
-      <c r="G68" s="81"/>
-      <c r="H68" s="81"/>
-      <c r="I68" s="81"/>
+      <c r="C68" s="238"/>
+      <c r="D68" s="238"/>
+      <c r="E68" s="238"/>
+      <c r="F68" s="238"/>
+      <c r="G68" s="238"/>
+      <c r="H68" s="238"/>
+      <c r="I68" s="238"/>
       <c r="J68" s="16"/>
       <c r="K68" s="16"/>
       <c r="L68" s="16"/>
@@ -6032,8 +6048,8 @@
       <c r="D69" s="15"/>
       <c r="E69" s="35"/>
       <c r="F69" s="35"/>
-      <c r="G69" s="94"/>
-      <c r="H69" s="94"/>
+      <c r="G69" s="76"/>
+      <c r="H69" s="76"/>
       <c r="I69" s="15"/>
       <c r="J69" s="16"/>
       <c r="K69" s="16"/>
@@ -6056,13 +6072,13 @@
       <c r="AB69" s="16"/>
     </row>
     <row r="70" spans="2:28" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B70" s="94"/>
-      <c r="C70" s="94"/>
-      <c r="D70" s="94"/>
-      <c r="E70" s="94"/>
+      <c r="B70" s="76"/>
+      <c r="C70" s="76"/>
+      <c r="D70" s="76"/>
+      <c r="E70" s="76"/>
       <c r="F70" s="35"/>
-      <c r="G70" s="94"/>
-      <c r="H70" s="94"/>
+      <c r="G70" s="76"/>
+      <c r="H70" s="76"/>
       <c r="I70" s="15"/>
       <c r="J70" s="16"/>
       <c r="K70" s="16"/>
@@ -6085,10 +6101,10 @@
       <c r="AB70" s="16"/>
     </row>
     <row r="71" spans="2:28" ht="36" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B71" s="241"/>
-      <c r="C71" s="241"/>
-      <c r="D71" s="241"/>
-      <c r="E71" s="241"/>
+      <c r="B71" s="77"/>
+      <c r="C71" s="77"/>
+      <c r="D71" s="77"/>
+      <c r="E71" s="77"/>
       <c r="F71" s="26"/>
       <c r="H71" s="57"/>
       <c r="I71" s="16"/>
@@ -6113,12 +6129,12 @@
       <c r="AB71" s="16"/>
     </row>
     <row r="72" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B72" s="77" t="s">
+      <c r="B72" s="231" t="s">
         <v>65</v>
       </c>
-      <c r="C72" s="77"/>
-      <c r="D72" s="77"/>
-      <c r="E72" s="77"/>
+      <c r="C72" s="231"/>
+      <c r="D72" s="231"/>
+      <c r="E72" s="231"/>
       <c r="F72" s="17"/>
       <c r="H72" s="17" t="s">
         <v>66</v>
@@ -6150,8 +6166,8 @@
       <c r="D73" s="16"/>
       <c r="E73" s="26"/>
       <c r="F73" s="26"/>
-      <c r="G73" s="107"/>
-      <c r="H73" s="225"/>
+      <c r="G73" s="69"/>
+      <c r="H73" s="113"/>
       <c r="I73" s="16"/>
       <c r="J73" s="16"/>
       <c r="K73" s="16"/>
@@ -6174,13 +6190,13 @@
       <c r="AB73" s="16"/>
     </row>
     <row r="74" spans="2:28" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B74" s="243"/>
-      <c r="C74" s="243"/>
-      <c r="D74" s="243"/>
-      <c r="E74" s="243"/>
+      <c r="B74" s="80"/>
+      <c r="C74" s="80"/>
+      <c r="D74" s="80"/>
+      <c r="E74" s="80"/>
       <c r="F74" s="26"/>
-      <c r="H74" s="105"/>
-      <c r="I74" s="105"/>
+      <c r="H74" s="78"/>
+      <c r="I74" s="78"/>
       <c r="J74" s="16"/>
       <c r="K74" s="16"/>
       <c r="L74" s="16"/>
@@ -6202,13 +6218,13 @@
       <c r="AB74" s="16"/>
     </row>
     <row r="75" spans="2:28" ht="38.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B75" s="244"/>
-      <c r="C75" s="244"/>
-      <c r="D75" s="244"/>
-      <c r="E75" s="244"/>
+      <c r="B75" s="81"/>
+      <c r="C75" s="81"/>
+      <c r="D75" s="81"/>
+      <c r="E75" s="81"/>
       <c r="F75" s="26"/>
-      <c r="H75" s="242"/>
-      <c r="I75" s="242"/>
+      <c r="H75" s="79"/>
+      <c r="I75" s="79"/>
       <c r="J75" s="16"/>
       <c r="K75" s="16"/>
       <c r="L75" s="16"/>
@@ -6237,10 +6253,10 @@
       <c r="D76" s="24"/>
       <c r="E76" s="26"/>
       <c r="F76" s="26"/>
-      <c r="H76" s="77" t="s">
+      <c r="H76" s="231" t="s">
         <v>68</v>
       </c>
-      <c r="I76" s="77"/>
+      <c r="I76" s="231"/>
       <c r="J76" s="16"/>
       <c r="K76" s="16"/>
       <c r="L76" s="16"/>
@@ -6267,8 +6283,8 @@
       <c r="D77" s="24"/>
       <c r="E77" s="26"/>
       <c r="F77" s="26"/>
-      <c r="G77" s="107"/>
-      <c r="H77" s="93"/>
+      <c r="G77" s="69"/>
+      <c r="H77" s="229"/>
       <c r="I77" s="17"/>
       <c r="J77" s="16"/>
       <c r="K77" s="16"/>
@@ -6291,16 +6307,16 @@
       <c r="AB77" s="16"/>
     </row>
     <row r="78" spans="2:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B78" s="96" t="s">
+      <c r="B78" s="249" t="s">
         <v>69</v>
       </c>
-      <c r="C78" s="96"/>
-      <c r="D78" s="96"/>
-      <c r="E78" s="96"/>
-      <c r="F78" s="96"/>
-      <c r="G78" s="96"/>
-      <c r="H78" s="96"/>
-      <c r="I78" s="96"/>
+      <c r="C78" s="249"/>
+      <c r="D78" s="249"/>
+      <c r="E78" s="249"/>
+      <c r="F78" s="249"/>
+      <c r="G78" s="249"/>
+      <c r="H78" s="249"/>
+      <c r="I78" s="249"/>
       <c r="J78" s="16"/>
       <c r="K78" s="16"/>
       <c r="L78" s="16"/>
@@ -6322,14 +6338,14 @@
       <c r="AB78" s="16"/>
     </row>
     <row r="79" spans="2:28" x14ac:dyDescent="0.25">
-      <c r="B79" s="96"/>
-      <c r="C79" s="96"/>
-      <c r="D79" s="96"/>
-      <c r="E79" s="96"/>
-      <c r="F79" s="96"/>
-      <c r="G79" s="96"/>
-      <c r="H79" s="96"/>
-      <c r="I79" s="96"/>
+      <c r="B79" s="249"/>
+      <c r="C79" s="249"/>
+      <c r="D79" s="249"/>
+      <c r="E79" s="249"/>
+      <c r="F79" s="249"/>
+      <c r="G79" s="249"/>
+      <c r="H79" s="249"/>
+      <c r="I79" s="249"/>
       <c r="J79" s="16"/>
       <c r="K79" s="16"/>
       <c r="L79" s="16"/>
@@ -6356,8 +6372,8 @@
       <c r="D80" s="48"/>
       <c r="E80" s="48"/>
       <c r="F80" s="48"/>
-      <c r="G80" s="108"/>
-      <c r="H80" s="108"/>
+      <c r="G80" s="230"/>
+      <c r="H80" s="230"/>
       <c r="I80" s="48"/>
       <c r="J80" s="16"/>
       <c r="K80" s="16"/>
@@ -6380,16 +6396,16 @@
       <c r="AB80" s="16"/>
     </row>
     <row r="81" spans="2:28" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B81" s="71" t="s">
+      <c r="B81" s="232" t="s">
         <v>70</v>
       </c>
-      <c r="C81" s="72"/>
-      <c r="D81" s="72"/>
-      <c r="E81" s="72"/>
-      <c r="F81" s="72"/>
-      <c r="G81" s="72"/>
-      <c r="H81" s="72"/>
-      <c r="I81" s="73"/>
+      <c r="C81" s="233"/>
+      <c r="D81" s="233"/>
+      <c r="E81" s="233"/>
+      <c r="F81" s="233"/>
+      <c r="G81" s="233"/>
+      <c r="H81" s="233"/>
+      <c r="I81" s="234"/>
       <c r="J81" s="8"/>
       <c r="K81" s="7"/>
       <c r="L81" s="7"/>
@@ -6411,16 +6427,16 @@
       <c r="AB81" s="7"/>
     </row>
     <row r="82" spans="2:28" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B82" s="74" t="s">
+      <c r="B82" s="235" t="s">
         <v>71</v>
       </c>
-      <c r="C82" s="75"/>
-      <c r="D82" s="75"/>
-      <c r="E82" s="75"/>
-      <c r="F82" s="75"/>
-      <c r="G82" s="75"/>
-      <c r="H82" s="75"/>
-      <c r="I82" s="76"/>
+      <c r="C82" s="236"/>
+      <c r="D82" s="236"/>
+      <c r="E82" s="236"/>
+      <c r="F82" s="236"/>
+      <c r="G82" s="236"/>
+      <c r="H82" s="236"/>
+      <c r="I82" s="237"/>
       <c r="J82" s="8"/>
       <c r="K82" s="25"/>
       <c r="L82" s="7"/>
@@ -6441,19 +6457,19 @@
       <c r="AA82" s="7"/>
       <c r="AB82" s="7"/>
     </row>
-    <row r="83" spans="2:28" s="8" customFormat="1" ht="48" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B83" s="238"/>
-      <c r="C83" s="239"/>
-      <c r="D83" s="239"/>
-      <c r="E83" s="239"/>
-      <c r="F83" s="239"/>
-      <c r="G83" s="239"/>
-      <c r="H83" s="239"/>
-      <c r="I83" s="240"/>
+    <row r="83" spans="2:28" s="8" customFormat="1" ht="207.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B83" s="73"/>
+      <c r="C83" s="74"/>
+      <c r="D83" s="74"/>
+      <c r="E83" s="74"/>
+      <c r="F83" s="74"/>
+      <c r="G83" s="74"/>
+      <c r="H83" s="74"/>
+      <c r="I83" s="75"/>
     </row>
     <row r="84" spans="2:28" hidden="1" x14ac:dyDescent="0.25">
-      <c r="G84" s="107"/>
-      <c r="H84" s="107"/>
+      <c r="G84" s="69"/>
+      <c r="H84" s="69"/>
       <c r="J84" s="8"/>
       <c r="K84" s="7"/>
       <c r="L84" s="7"/>
@@ -6475,222 +6491,171 @@
       <c r="AB84" s="7"/>
     </row>
     <row r="85" spans="2:28" hidden="1" x14ac:dyDescent="0.25">
-      <c r="G85" s="107"/>
-      <c r="H85" s="107"/>
+      <c r="G85" s="69"/>
+      <c r="H85" s="69"/>
     </row>
     <row r="86" spans="2:28" hidden="1" x14ac:dyDescent="0.25">
-      <c r="G86" s="107"/>
-      <c r="H86" s="107"/>
+      <c r="G86" s="69"/>
+      <c r="H86" s="69"/>
     </row>
     <row r="87" spans="2:28" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G87" s="107"/>
-      <c r="H87" s="107"/>
+      <c r="G87" s="69"/>
+      <c r="H87" s="69"/>
     </row>
     <row r="88" spans="2:28" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G88" s="107"/>
-      <c r="H88" s="107"/>
+      <c r="G88" s="69"/>
+      <c r="H88" s="69"/>
     </row>
     <row r="89" spans="2:28" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G89" s="107"/>
-      <c r="H89" s="107"/>
+      <c r="G89" s="69"/>
+      <c r="H89" s="69"/>
     </row>
     <row r="90" spans="2:28" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G90" s="107"/>
-      <c r="H90" s="107"/>
+      <c r="G90" s="69"/>
+      <c r="H90" s="69"/>
     </row>
     <row r="91" spans="2:28" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G91" s="107"/>
-      <c r="H91" s="107"/>
+      <c r="G91" s="69"/>
+      <c r="H91" s="69"/>
     </row>
     <row r="92" spans="2:28" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G92" s="107"/>
-      <c r="H92" s="107"/>
+      <c r="G92" s="69"/>
+      <c r="H92" s="69"/>
     </row>
     <row r="93" spans="2:28" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G93" s="107"/>
-      <c r="H93" s="107"/>
+      <c r="G93" s="69"/>
+      <c r="H93" s="69"/>
     </row>
     <row r="94" spans="2:28" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G94" s="107"/>
-      <c r="H94" s="107"/>
+      <c r="G94" s="69"/>
+      <c r="H94" s="69"/>
     </row>
     <row r="95" spans="2:28" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G95" s="107"/>
-      <c r="H95" s="107"/>
+      <c r="G95" s="69"/>
+      <c r="H95" s="69"/>
     </row>
     <row r="96" spans="2:28" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G96" s="107"/>
-      <c r="H96" s="107"/>
+      <c r="G96" s="69"/>
+      <c r="H96" s="69"/>
     </row>
     <row r="97" spans="7:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G97" s="107"/>
-      <c r="H97" s="107"/>
+      <c r="G97" s="69"/>
+      <c r="H97" s="69"/>
     </row>
     <row r="98" spans="7:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G98" s="107"/>
-      <c r="H98" s="107"/>
+      <c r="G98" s="69"/>
+      <c r="H98" s="69"/>
     </row>
     <row r="99" spans="7:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G99" s="107"/>
-      <c r="H99" s="107"/>
+      <c r="G99" s="69"/>
+      <c r="H99" s="69"/>
     </row>
     <row r="100" spans="7:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G100" s="107"/>
-      <c r="H100" s="107"/>
+      <c r="G100" s="69"/>
+      <c r="H100" s="69"/>
     </row>
     <row r="101" spans="7:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G101" s="107"/>
-      <c r="H101" s="107"/>
+      <c r="G101" s="69"/>
+      <c r="H101" s="69"/>
     </row>
     <row r="102" spans="7:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G102" s="107"/>
-      <c r="H102" s="107"/>
+      <c r="G102" s="69"/>
+      <c r="H102" s="69"/>
     </row>
     <row r="103" spans="7:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G103" s="107"/>
-      <c r="H103" s="107"/>
+      <c r="G103" s="69"/>
+      <c r="H103" s="69"/>
     </row>
     <row r="104" spans="7:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G104" s="107"/>
-      <c r="H104" s="107"/>
+      <c r="G104" s="69"/>
+      <c r="H104" s="69"/>
     </row>
     <row r="105" spans="7:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G105" s="107"/>
-      <c r="H105" s="107"/>
+      <c r="G105" s="69"/>
+      <c r="H105" s="69"/>
     </row>
     <row r="106" spans="7:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G106" s="107"/>
-      <c r="H106" s="107"/>
+      <c r="G106" s="69"/>
+      <c r="H106" s="69"/>
     </row>
     <row r="107" spans="7:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G107" s="107"/>
-      <c r="H107" s="107"/>
+      <c r="G107" s="69"/>
+      <c r="H107" s="69"/>
     </row>
     <row r="108" spans="7:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G108" s="107"/>
-      <c r="H108" s="107"/>
+      <c r="G108" s="69"/>
+      <c r="H108" s="69"/>
     </row>
     <row r="109" spans="7:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G109" s="107"/>
-      <c r="H109" s="107"/>
+      <c r="G109" s="69"/>
+      <c r="H109" s="69"/>
     </row>
     <row r="110" spans="7:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G110" s="107"/>
-      <c r="H110" s="107"/>
+      <c r="G110" s="69"/>
+      <c r="H110" s="69"/>
     </row>
     <row r="111" spans="7:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G111" s="107"/>
-      <c r="H111" s="107"/>
+      <c r="G111" s="69"/>
+      <c r="H111" s="69"/>
     </row>
     <row r="112" spans="7:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G112" s="107"/>
-      <c r="H112" s="107"/>
+      <c r="G112" s="69"/>
+      <c r="H112" s="69"/>
     </row>
     <row r="113" spans="7:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G113" s="107"/>
-      <c r="H113" s="107"/>
+      <c r="G113" s="69"/>
+      <c r="H113" s="69"/>
     </row>
   </sheetData>
   <mergeCells count="171">
-    <mergeCell ref="G112:H112"/>
-    <mergeCell ref="G113:H113"/>
-    <mergeCell ref="B59:I59"/>
-    <mergeCell ref="G106:H106"/>
-    <mergeCell ref="G107:H107"/>
-    <mergeCell ref="G108:H108"/>
-    <mergeCell ref="G109:H109"/>
-    <mergeCell ref="G110:H110"/>
-    <mergeCell ref="G101:H101"/>
-    <mergeCell ref="G102:H102"/>
-    <mergeCell ref="G103:H103"/>
-    <mergeCell ref="G104:H104"/>
-    <mergeCell ref="B83:I83"/>
-    <mergeCell ref="B70:E71"/>
-    <mergeCell ref="H74:I75"/>
-    <mergeCell ref="B74:E75"/>
-    <mergeCell ref="G65:G66"/>
-    <mergeCell ref="I65:I66"/>
-    <mergeCell ref="G87:H87"/>
-    <mergeCell ref="G88:H88"/>
-    <mergeCell ref="G89:H89"/>
-    <mergeCell ref="G90:H90"/>
-    <mergeCell ref="E65:F66"/>
-    <mergeCell ref="G30:H30"/>
-    <mergeCell ref="G34:H34"/>
-    <mergeCell ref="G22:H22"/>
-    <mergeCell ref="H24:I24"/>
-    <mergeCell ref="H25:I25"/>
-    <mergeCell ref="B28:D28"/>
-    <mergeCell ref="B29:D29"/>
-    <mergeCell ref="H28:I28"/>
-    <mergeCell ref="H37:I38"/>
-    <mergeCell ref="B37:B40"/>
-    <mergeCell ref="G37:G38"/>
-    <mergeCell ref="I45:I46"/>
-    <mergeCell ref="G41:G42"/>
-    <mergeCell ref="H41:I42"/>
-    <mergeCell ref="B35:I35"/>
-    <mergeCell ref="H39:I40"/>
-    <mergeCell ref="G111:H111"/>
-    <mergeCell ref="G84:H84"/>
-    <mergeCell ref="G85:H85"/>
-    <mergeCell ref="G73:H73"/>
-    <mergeCell ref="B44:I44"/>
-    <mergeCell ref="G39:G40"/>
-    <mergeCell ref="G43:H43"/>
-    <mergeCell ref="C37:F40"/>
-    <mergeCell ref="C41:F42"/>
-    <mergeCell ref="B41:B42"/>
-    <mergeCell ref="B27:I27"/>
-    <mergeCell ref="B25:E25"/>
-    <mergeCell ref="B31:I31"/>
-    <mergeCell ref="G86:H86"/>
-    <mergeCell ref="H36:I36"/>
-    <mergeCell ref="C36:F36"/>
-    <mergeCell ref="B33:F33"/>
-    <mergeCell ref="G32:I32"/>
-    <mergeCell ref="G33:I33"/>
-    <mergeCell ref="D53:E54"/>
-    <mergeCell ref="F53:F54"/>
-    <mergeCell ref="G53:G54"/>
-    <mergeCell ref="H53:H54"/>
-    <mergeCell ref="I53:I54"/>
-    <mergeCell ref="G51:G52"/>
-    <mergeCell ref="H51:H52"/>
-    <mergeCell ref="H45:H46"/>
-    <mergeCell ref="G45:G46"/>
-    <mergeCell ref="B45:C46"/>
-    <mergeCell ref="B17:D17"/>
-    <mergeCell ref="H20:I20"/>
-    <mergeCell ref="B20:D20"/>
-    <mergeCell ref="B21:D21"/>
-    <mergeCell ref="E18:G18"/>
-    <mergeCell ref="H18:I18"/>
-    <mergeCell ref="E19:G19"/>
-    <mergeCell ref="H19:I19"/>
-    <mergeCell ref="B18:D18"/>
-    <mergeCell ref="B19:D19"/>
-    <mergeCell ref="E17:G17"/>
-    <mergeCell ref="H17:I17"/>
-    <mergeCell ref="B23:I23"/>
-    <mergeCell ref="B24:E24"/>
-    <mergeCell ref="H21:I21"/>
-    <mergeCell ref="E21:G21"/>
-    <mergeCell ref="E20:G20"/>
-    <mergeCell ref="F24:G24"/>
-    <mergeCell ref="F25:G25"/>
-    <mergeCell ref="G105:H105"/>
-    <mergeCell ref="G96:H96"/>
-    <mergeCell ref="G97:H97"/>
-    <mergeCell ref="G98:H98"/>
-    <mergeCell ref="G99:H99"/>
-    <mergeCell ref="G100:H100"/>
-    <mergeCell ref="G91:H91"/>
-    <mergeCell ref="G92:H92"/>
-    <mergeCell ref="G93:H93"/>
-    <mergeCell ref="G94:H94"/>
-    <mergeCell ref="G95:H95"/>
-    <mergeCell ref="I51:I52"/>
+    <mergeCell ref="B81:I81"/>
+    <mergeCell ref="B82:I82"/>
+    <mergeCell ref="B72:E72"/>
+    <mergeCell ref="B60:I60"/>
+    <mergeCell ref="B68:I68"/>
+    <mergeCell ref="B61:I62"/>
+    <mergeCell ref="B63:I63"/>
+    <mergeCell ref="H65:H66"/>
+    <mergeCell ref="B64:I64"/>
+    <mergeCell ref="G67:H67"/>
+    <mergeCell ref="G69:H69"/>
+    <mergeCell ref="G70:H70"/>
+    <mergeCell ref="C65:D65"/>
+    <mergeCell ref="C66:D66"/>
+    <mergeCell ref="B78:I79"/>
+    <mergeCell ref="G77:H77"/>
+    <mergeCell ref="G80:H80"/>
+    <mergeCell ref="D47:E48"/>
+    <mergeCell ref="B47:C48"/>
+    <mergeCell ref="F47:F48"/>
+    <mergeCell ref="G47:G48"/>
+    <mergeCell ref="H47:H48"/>
+    <mergeCell ref="I47:I48"/>
+    <mergeCell ref="B49:C50"/>
+    <mergeCell ref="D49:E50"/>
+    <mergeCell ref="F49:F50"/>
+    <mergeCell ref="G49:G50"/>
+    <mergeCell ref="H49:H50"/>
+    <mergeCell ref="I49:I50"/>
+    <mergeCell ref="B51:C52"/>
+    <mergeCell ref="D51:E52"/>
+    <mergeCell ref="F51:F52"/>
+    <mergeCell ref="I55:I56"/>
+    <mergeCell ref="H76:I76"/>
+    <mergeCell ref="B55:C56"/>
+    <mergeCell ref="D55:E56"/>
+    <mergeCell ref="F55:F56"/>
+    <mergeCell ref="G55:G56"/>
+    <mergeCell ref="H55:H56"/>
+    <mergeCell ref="B11:D11"/>
+    <mergeCell ref="G9:H9"/>
+    <mergeCell ref="G12:H12"/>
+    <mergeCell ref="H16:I16"/>
+    <mergeCell ref="D45:E46"/>
+    <mergeCell ref="F45:F46"/>
+    <mergeCell ref="G26:H26"/>
+    <mergeCell ref="B58:I58"/>
+    <mergeCell ref="G57:H57"/>
     <mergeCell ref="B53:C54"/>
     <mergeCell ref="H29:I29"/>
     <mergeCell ref="E28:F28"/>
@@ -6715,67 +6680,118 @@
     <mergeCell ref="E10:I10"/>
     <mergeCell ref="E11:I11"/>
     <mergeCell ref="B10:D10"/>
-    <mergeCell ref="B11:D11"/>
-    <mergeCell ref="G9:H9"/>
-    <mergeCell ref="G12:H12"/>
-    <mergeCell ref="H16:I16"/>
-    <mergeCell ref="D45:E46"/>
-    <mergeCell ref="F45:F46"/>
-    <mergeCell ref="G26:H26"/>
-    <mergeCell ref="B58:I58"/>
-    <mergeCell ref="G57:H57"/>
-    <mergeCell ref="G77:H77"/>
-    <mergeCell ref="G80:H80"/>
-    <mergeCell ref="D47:E48"/>
-    <mergeCell ref="B47:C48"/>
-    <mergeCell ref="F47:F48"/>
-    <mergeCell ref="G47:G48"/>
-    <mergeCell ref="H47:H48"/>
-    <mergeCell ref="I47:I48"/>
-    <mergeCell ref="B49:C50"/>
-    <mergeCell ref="D49:E50"/>
-    <mergeCell ref="F49:F50"/>
-    <mergeCell ref="G49:G50"/>
-    <mergeCell ref="H49:H50"/>
-    <mergeCell ref="I49:I50"/>
-    <mergeCell ref="B51:C52"/>
-    <mergeCell ref="D51:E52"/>
-    <mergeCell ref="F51:F52"/>
-    <mergeCell ref="I55:I56"/>
-    <mergeCell ref="H76:I76"/>
-    <mergeCell ref="B55:C56"/>
-    <mergeCell ref="D55:E56"/>
-    <mergeCell ref="B81:I81"/>
-    <mergeCell ref="B82:I82"/>
-    <mergeCell ref="B72:E72"/>
-    <mergeCell ref="B60:I60"/>
-    <mergeCell ref="B68:I68"/>
-    <mergeCell ref="B61:I62"/>
-    <mergeCell ref="B63:I63"/>
-    <mergeCell ref="H65:H66"/>
-    <mergeCell ref="B64:I64"/>
-    <mergeCell ref="G67:H67"/>
-    <mergeCell ref="G69:H69"/>
-    <mergeCell ref="G70:H70"/>
-    <mergeCell ref="C65:D65"/>
-    <mergeCell ref="C66:D66"/>
-    <mergeCell ref="B78:I79"/>
-    <mergeCell ref="F55:F56"/>
-    <mergeCell ref="G55:G56"/>
-    <mergeCell ref="H55:H56"/>
+    <mergeCell ref="G96:H96"/>
+    <mergeCell ref="G97:H97"/>
+    <mergeCell ref="G98:H98"/>
+    <mergeCell ref="G99:H99"/>
+    <mergeCell ref="G100:H100"/>
+    <mergeCell ref="G91:H91"/>
+    <mergeCell ref="G92:H92"/>
+    <mergeCell ref="G93:H93"/>
+    <mergeCell ref="G94:H94"/>
+    <mergeCell ref="G95:H95"/>
+    <mergeCell ref="H51:H52"/>
+    <mergeCell ref="H45:H46"/>
+    <mergeCell ref="G45:G46"/>
+    <mergeCell ref="B45:C46"/>
+    <mergeCell ref="B17:D17"/>
+    <mergeCell ref="H20:I20"/>
+    <mergeCell ref="B20:D20"/>
+    <mergeCell ref="B21:D21"/>
+    <mergeCell ref="E18:G18"/>
+    <mergeCell ref="H18:I18"/>
+    <mergeCell ref="E19:G19"/>
+    <mergeCell ref="H19:I19"/>
+    <mergeCell ref="B18:D18"/>
+    <mergeCell ref="B19:D19"/>
+    <mergeCell ref="E17:G17"/>
+    <mergeCell ref="H17:I17"/>
+    <mergeCell ref="B23:I23"/>
+    <mergeCell ref="B24:E24"/>
+    <mergeCell ref="H21:I21"/>
+    <mergeCell ref="E21:G21"/>
+    <mergeCell ref="E20:G20"/>
+    <mergeCell ref="F24:G24"/>
+    <mergeCell ref="F25:G25"/>
+    <mergeCell ref="I51:I52"/>
+    <mergeCell ref="I45:I46"/>
+    <mergeCell ref="G41:G42"/>
+    <mergeCell ref="H41:I42"/>
+    <mergeCell ref="B35:I35"/>
+    <mergeCell ref="H39:I40"/>
+    <mergeCell ref="G111:H111"/>
+    <mergeCell ref="G84:H84"/>
+    <mergeCell ref="G85:H85"/>
+    <mergeCell ref="G73:H73"/>
+    <mergeCell ref="B44:I44"/>
+    <mergeCell ref="G39:G40"/>
+    <mergeCell ref="G43:H43"/>
+    <mergeCell ref="C37:F40"/>
+    <mergeCell ref="C41:F42"/>
+    <mergeCell ref="B41:B42"/>
+    <mergeCell ref="G86:H86"/>
+    <mergeCell ref="H36:I36"/>
+    <mergeCell ref="C36:F36"/>
+    <mergeCell ref="D53:E54"/>
+    <mergeCell ref="F53:F54"/>
+    <mergeCell ref="G53:G54"/>
+    <mergeCell ref="H53:H54"/>
+    <mergeCell ref="I53:I54"/>
+    <mergeCell ref="G51:G52"/>
+    <mergeCell ref="G30:H30"/>
+    <mergeCell ref="G34:H34"/>
+    <mergeCell ref="G22:H22"/>
+    <mergeCell ref="H24:I24"/>
+    <mergeCell ref="H25:I25"/>
+    <mergeCell ref="B28:D28"/>
+    <mergeCell ref="B29:D29"/>
+    <mergeCell ref="H28:I28"/>
+    <mergeCell ref="H37:I38"/>
+    <mergeCell ref="B37:B40"/>
+    <mergeCell ref="G37:G38"/>
+    <mergeCell ref="B27:I27"/>
+    <mergeCell ref="B25:E25"/>
+    <mergeCell ref="B31:I31"/>
+    <mergeCell ref="B33:F33"/>
+    <mergeCell ref="G32:I32"/>
+    <mergeCell ref="G33:I33"/>
+    <mergeCell ref="G112:H112"/>
+    <mergeCell ref="G113:H113"/>
+    <mergeCell ref="B59:I59"/>
+    <mergeCell ref="G106:H106"/>
+    <mergeCell ref="G107:H107"/>
+    <mergeCell ref="G108:H108"/>
+    <mergeCell ref="G109:H109"/>
+    <mergeCell ref="G110:H110"/>
+    <mergeCell ref="G101:H101"/>
+    <mergeCell ref="G102:H102"/>
+    <mergeCell ref="G103:H103"/>
+    <mergeCell ref="G104:H104"/>
+    <mergeCell ref="B83:I83"/>
+    <mergeCell ref="B70:E71"/>
+    <mergeCell ref="H74:I75"/>
+    <mergeCell ref="B74:E75"/>
+    <mergeCell ref="G65:G66"/>
+    <mergeCell ref="I65:I66"/>
+    <mergeCell ref="G87:H87"/>
+    <mergeCell ref="G88:H88"/>
+    <mergeCell ref="G89:H89"/>
+    <mergeCell ref="G90:H90"/>
+    <mergeCell ref="E65:F66"/>
+    <mergeCell ref="G105:H105"/>
   </mergeCells>
   <conditionalFormatting sqref="B11:I11 B15:I15 B17:I17 B19:I19 B21:I21 B25:I25 B29:I29 C37:F42 H37:I42 B70:E71 B74:E75 H74:I75 B83:I83">
-    <cfRule type="containsBlanks" dxfId="9" priority="4">
+    <cfRule type="containsBlanks" dxfId="2" priority="4">
       <formula>LEN(TRIM(B11))=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B47:I56">
-    <cfRule type="containsBlanks" dxfId="8" priority="1">
+    <cfRule type="containsBlanks" dxfId="1" priority="1">
       <formula>LEN(TRIM(B47))=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G65:G66 I65:I66 B66:D66 H71">
-    <cfRule type="containsBlanks" dxfId="7" priority="5">
+    <cfRule type="containsBlanks" dxfId="0" priority="5">
       <formula>LEN(TRIM(B65))=0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6870,7 +6886,7 @@
       <c r="B2" s="64" t="s">
         <v>110</v>
       </c>
-      <c r="C2" s="283" t="s">
+      <c r="C2" s="67" t="s">
         <v>123</v>
       </c>
       <c r="E2" t="str" cm="1">
@@ -6909,7 +6925,7 @@
       <c r="B3" s="64" t="s">
         <v>110</v>
       </c>
-      <c r="C3" s="283" t="s">
+      <c r="C3" s="67" t="s">
         <v>124</v>
       </c>
       <c r="E3" t="str">
@@ -6923,7 +6939,7 @@
       <c r="B4" s="64" t="s">
         <v>110</v>
       </c>
-      <c r="C4" s="283" t="s">
+      <c r="C4" s="67" t="s">
         <v>125</v>
       </c>
     </row>
@@ -6934,7 +6950,7 @@
       <c r="B5" s="64" t="s">
         <v>110</v>
       </c>
-      <c r="C5" s="283" t="s">
+      <c r="C5" s="67" t="s">
         <v>126</v>
       </c>
     </row>
@@ -6945,7 +6961,7 @@
       <c r="B6" s="64" t="s">
         <v>111</v>
       </c>
-      <c r="C6" s="283" t="s">
+      <c r="C6" s="67" t="s">
         <v>127</v>
       </c>
     </row>
@@ -6956,7 +6972,7 @@
       <c r="B7" s="64" t="s">
         <v>111</v>
       </c>
-      <c r="C7" s="283" t="s">
+      <c r="C7" s="67" t="s">
         <v>128</v>
       </c>
     </row>
@@ -6967,7 +6983,7 @@
       <c r="B8" s="64" t="s">
         <v>111</v>
       </c>
-      <c r="C8" s="283" t="s">
+      <c r="C8" s="67" t="s">
         <v>129</v>
       </c>
     </row>
@@ -6978,7 +6994,7 @@
       <c r="B9" s="64" t="s">
         <v>111</v>
       </c>
-      <c r="C9" s="283" t="s">
+      <c r="C9" s="67" t="s">
         <v>130</v>
       </c>
     </row>
@@ -6989,7 +7005,7 @@
       <c r="B10" s="64" t="s">
         <v>112</v>
       </c>
-      <c r="C10" s="283" t="s">
+      <c r="C10" s="67" t="s">
         <v>131</v>
       </c>
     </row>
@@ -7000,7 +7016,7 @@
       <c r="B11" s="64" t="s">
         <v>112</v>
       </c>
-      <c r="C11" s="283" t="s">
+      <c r="C11" s="67" t="s">
         <v>132</v>
       </c>
     </row>
@@ -7011,7 +7027,7 @@
       <c r="B12" s="64" t="s">
         <v>112</v>
       </c>
-      <c r="C12" s="283" t="s">
+      <c r="C12" s="67" t="s">
         <v>133</v>
       </c>
     </row>
@@ -7022,7 +7038,7 @@
       <c r="B13" s="64" t="s">
         <v>112</v>
       </c>
-      <c r="C13" s="283" t="s">
+      <c r="C13" s="67" t="s">
         <v>134</v>
       </c>
     </row>
@@ -7033,7 +7049,7 @@
       <c r="B14" s="64" t="s">
         <v>113</v>
       </c>
-      <c r="C14" s="283" t="s">
+      <c r="C14" s="67" t="s">
         <v>135</v>
       </c>
     </row>
@@ -7044,7 +7060,7 @@
       <c r="B15" s="64" t="s">
         <v>113</v>
       </c>
-      <c r="C15" s="283" t="s">
+      <c r="C15" s="67" t="s">
         <v>136</v>
       </c>
     </row>
@@ -7055,7 +7071,7 @@
       <c r="B16" s="64" t="s">
         <v>113</v>
       </c>
-      <c r="C16" s="283" t="s">
+      <c r="C16" s="67" t="s">
         <v>137</v>
       </c>
     </row>
@@ -7066,7 +7082,7 @@
       <c r="B17" s="64" t="s">
         <v>113</v>
       </c>
-      <c r="C17" s="283" t="s">
+      <c r="C17" s="67" t="s">
         <v>138</v>
       </c>
     </row>
@@ -7077,7 +7093,7 @@
       <c r="B18" s="64" t="s">
         <v>113</v>
       </c>
-      <c r="C18" s="283" t="s">
+      <c r="C18" s="67" t="s">
         <v>139</v>
       </c>
     </row>
@@ -7088,7 +7104,7 @@
       <c r="B19" s="64" t="s">
         <v>114</v>
       </c>
-      <c r="C19" s="283" t="s">
+      <c r="C19" s="67" t="s">
         <v>140</v>
       </c>
     </row>
@@ -7099,7 +7115,7 @@
       <c r="B20" s="64" t="s">
         <v>114</v>
       </c>
-      <c r="C20" s="283" t="s">
+      <c r="C20" s="67" t="s">
         <v>141</v>
       </c>
     </row>
@@ -7110,7 +7126,7 @@
       <c r="B21" s="64" t="s">
         <v>114</v>
       </c>
-      <c r="C21" s="283" t="s">
+      <c r="C21" s="67" t="s">
         <v>142</v>
       </c>
     </row>
@@ -7121,7 +7137,7 @@
       <c r="B22" s="64" t="s">
         <v>115</v>
       </c>
-      <c r="C22" s="283" t="s">
+      <c r="C22" s="67" t="s">
         <v>143</v>
       </c>
     </row>
@@ -7132,7 +7148,7 @@
       <c r="B23" s="64" t="s">
         <v>115</v>
       </c>
-      <c r="C23" s="283" t="s">
+      <c r="C23" s="67" t="s">
         <v>144</v>
       </c>
     </row>
@@ -7143,7 +7159,7 @@
       <c r="B24" s="64" t="s">
         <v>116</v>
       </c>
-      <c r="C24" s="283" t="s">
+      <c r="C24" s="67" t="s">
         <v>145</v>
       </c>
     </row>
@@ -7154,7 +7170,7 @@
       <c r="B25" s="64" t="s">
         <v>116</v>
       </c>
-      <c r="C25" s="283" t="s">
+      <c r="C25" s="67" t="s">
         <v>146</v>
       </c>
     </row>
@@ -7165,7 +7181,7 @@
       <c r="B26" s="64" t="s">
         <v>116</v>
       </c>
-      <c r="C26" s="283" t="s">
+      <c r="C26" s="67" t="s">
         <v>147</v>
       </c>
     </row>
@@ -7176,7 +7192,7 @@
       <c r="B27" s="64" t="s">
         <v>116</v>
       </c>
-      <c r="C27" s="283" t="s">
+      <c r="C27" s="67" t="s">
         <v>148</v>
       </c>
     </row>
@@ -7187,7 +7203,7 @@
       <c r="B28" s="64" t="s">
         <v>118</v>
       </c>
-      <c r="C28" s="283" t="s">
+      <c r="C28" s="67" t="s">
         <v>149</v>
       </c>
     </row>
@@ -7198,7 +7214,7 @@
       <c r="B29" s="64" t="s">
         <v>118</v>
       </c>
-      <c r="C29" s="283" t="s">
+      <c r="C29" s="67" t="s">
         <v>150</v>
       </c>
     </row>
@@ -7209,7 +7225,7 @@
       <c r="B30" s="64" t="s">
         <v>118</v>
       </c>
-      <c r="C30" s="283" t="s">
+      <c r="C30" s="67" t="s">
         <v>151</v>
       </c>
     </row>
@@ -7220,7 +7236,7 @@
       <c r="B31" s="64" t="s">
         <v>118</v>
       </c>
-      <c r="C31" s="283" t="s">
+      <c r="C31" s="67" t="s">
         <v>152</v>
       </c>
     </row>
@@ -7231,7 +7247,7 @@
       <c r="B32" s="64" t="s">
         <v>119</v>
       </c>
-      <c r="C32" s="283" t="s">
+      <c r="C32" s="67" t="s">
         <v>153</v>
       </c>
     </row>
@@ -7242,7 +7258,7 @@
       <c r="B33" s="64" t="s">
         <v>119</v>
       </c>
-      <c r="C33" s="283" t="s">
+      <c r="C33" s="67" t="s">
         <v>154</v>
       </c>
     </row>
@@ -7253,7 +7269,7 @@
       <c r="B34" s="64" t="s">
         <v>119</v>
       </c>
-      <c r="C34" s="283" t="s">
+      <c r="C34" s="67" t="s">
         <v>155</v>
       </c>
     </row>
@@ -7264,7 +7280,7 @@
       <c r="B35" s="64" t="s">
         <v>120</v>
       </c>
-      <c r="C35" s="283" t="s">
+      <c r="C35" s="67" t="s">
         <v>156</v>
       </c>
     </row>
@@ -7275,7 +7291,7 @@
       <c r="B36" s="64" t="s">
         <v>120</v>
       </c>
-      <c r="C36" s="283" t="s">
+      <c r="C36" s="67" t="s">
         <v>157</v>
       </c>
     </row>
@@ -7286,7 +7302,7 @@
       <c r="B37" s="64" t="s">
         <v>121</v>
       </c>
-      <c r="C37" s="283" t="s">
+      <c r="C37" s="67" t="s">
         <v>158</v>
       </c>
     </row>
@@ -7297,7 +7313,7 @@
       <c r="B38" s="64" t="s">
         <v>121</v>
       </c>
-      <c r="C38" s="283" t="s">
+      <c r="C38" s="67" t="s">
         <v>159</v>
       </c>
     </row>
@@ -7308,7 +7324,7 @@
       <c r="B39" s="66" t="s">
         <v>122</v>
       </c>
-      <c r="C39" s="284" t="s">
+      <c r="C39" s="68" t="s">
         <v>160</v>
       </c>
     </row>
@@ -7401,124 +7417,124 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:24" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A1" s="275" t="s">
+      <c r="A1" s="251" t="s">
         <v>72</v>
       </c>
-      <c r="B1" s="275"/>
-      <c r="C1" s="275"/>
-      <c r="D1" s="275"/>
-      <c r="E1" s="275"/>
-      <c r="F1" s="275"/>
-      <c r="G1" s="275"/>
-      <c r="H1" s="275"/>
-      <c r="I1" s="275"/>
-      <c r="J1" s="275"/>
-      <c r="K1" s="275"/>
-      <c r="L1" s="275"/>
-      <c r="M1" s="275"/>
-      <c r="N1" s="275"/>
-      <c r="O1" s="275"/>
-      <c r="P1" s="275"/>
-      <c r="Q1" s="275"/>
-      <c r="R1" s="275"/>
-      <c r="S1" s="275"/>
-      <c r="T1" s="275"/>
-      <c r="U1" s="275" t="s">
+      <c r="B1" s="251"/>
+      <c r="C1" s="251"/>
+      <c r="D1" s="251"/>
+      <c r="E1" s="251"/>
+      <c r="F1" s="251"/>
+      <c r="G1" s="251"/>
+      <c r="H1" s="251"/>
+      <c r="I1" s="251"/>
+      <c r="J1" s="251"/>
+      <c r="K1" s="251"/>
+      <c r="L1" s="251"/>
+      <c r="M1" s="251"/>
+      <c r="N1" s="251"/>
+      <c r="O1" s="251"/>
+      <c r="P1" s="251"/>
+      <c r="Q1" s="251"/>
+      <c r="R1" s="251"/>
+      <c r="S1" s="251"/>
+      <c r="T1" s="251"/>
+      <c r="U1" s="251" t="s">
         <v>73</v>
       </c>
-      <c r="V1" s="275"/>
-      <c r="W1" s="275"/>
-      <c r="X1" s="275"/>
+      <c r="V1" s="251"/>
+      <c r="W1" s="251"/>
+      <c r="X1" s="251"/>
     </row>
     <row r="2" spans="1:24" ht="33" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="275"/>
-      <c r="B2" s="275"/>
-      <c r="C2" s="275"/>
-      <c r="D2" s="275"/>
-      <c r="E2" s="275"/>
-      <c r="F2" s="275"/>
-      <c r="G2" s="275"/>
-      <c r="H2" s="275"/>
-      <c r="I2" s="275"/>
-      <c r="J2" s="275"/>
-      <c r="K2" s="275"/>
-      <c r="L2" s="275"/>
-      <c r="M2" s="275"/>
-      <c r="N2" s="275"/>
-      <c r="O2" s="275"/>
-      <c r="P2" s="275"/>
-      <c r="Q2" s="275"/>
-      <c r="R2" s="275"/>
-      <c r="S2" s="275"/>
-      <c r="T2" s="275"/>
-      <c r="U2" s="255" t="s">
+      <c r="A2" s="251"/>
+      <c r="B2" s="251"/>
+      <c r="C2" s="251"/>
+      <c r="D2" s="251"/>
+      <c r="E2" s="251"/>
+      <c r="F2" s="251"/>
+      <c r="G2" s="251"/>
+      <c r="H2" s="251"/>
+      <c r="I2" s="251"/>
+      <c r="J2" s="251"/>
+      <c r="K2" s="251"/>
+      <c r="L2" s="251"/>
+      <c r="M2" s="251"/>
+      <c r="N2" s="251"/>
+      <c r="O2" s="251"/>
+      <c r="P2" s="251"/>
+      <c r="Q2" s="251"/>
+      <c r="R2" s="251"/>
+      <c r="S2" s="251"/>
+      <c r="T2" s="251"/>
+      <c r="U2" s="259" t="s">
         <v>74</v>
       </c>
-      <c r="V2" s="255"/>
-      <c r="W2" s="255"/>
-      <c r="X2" s="255"/>
+      <c r="V2" s="259"/>
+      <c r="W2" s="259"/>
+      <c r="X2" s="259"/>
     </row>
     <row r="3" spans="1:24" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="U3" s="282"/>
-      <c r="V3" s="282"/>
-      <c r="W3" s="282"/>
-      <c r="X3" s="282"/>
+      <c r="U3" s="260"/>
+      <c r="V3" s="260"/>
+      <c r="W3" s="260"/>
+      <c r="X3" s="260"/>
     </row>
     <row r="4" spans="1:24" s="2" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="279" t="s">
+      <c r="A4" s="256" t="s">
         <v>75</v>
       </c>
-      <c r="B4" s="280"/>
-      <c r="C4" s="280"/>
-      <c r="D4" s="280"/>
-      <c r="E4" s="280"/>
-      <c r="F4" s="280"/>
-      <c r="G4" s="280"/>
-      <c r="H4" s="280"/>
-      <c r="I4" s="280"/>
-      <c r="J4" s="280"/>
-      <c r="K4" s="280"/>
-      <c r="L4" s="280"/>
-      <c r="M4" s="281"/>
-      <c r="N4" s="279" t="s">
+      <c r="B4" s="257"/>
+      <c r="C4" s="257"/>
+      <c r="D4" s="257"/>
+      <c r="E4" s="257"/>
+      <c r="F4" s="257"/>
+      <c r="G4" s="257"/>
+      <c r="H4" s="257"/>
+      <c r="I4" s="257"/>
+      <c r="J4" s="257"/>
+      <c r="K4" s="257"/>
+      <c r="L4" s="257"/>
+      <c r="M4" s="258"/>
+      <c r="N4" s="256" t="s">
         <v>76</v>
       </c>
-      <c r="O4" s="280"/>
-      <c r="P4" s="280"/>
-      <c r="Q4" s="280"/>
-      <c r="R4" s="280"/>
-      <c r="S4" s="280"/>
-      <c r="T4" s="280"/>
-      <c r="U4" s="280"/>
-      <c r="V4" s="280"/>
-      <c r="W4" s="280"/>
-      <c r="X4" s="281"/>
+      <c r="O4" s="257"/>
+      <c r="P4" s="257"/>
+      <c r="Q4" s="257"/>
+      <c r="R4" s="257"/>
+      <c r="S4" s="257"/>
+      <c r="T4" s="257"/>
+      <c r="U4" s="257"/>
+      <c r="V4" s="257"/>
+      <c r="W4" s="257"/>
+      <c r="X4" s="258"/>
     </row>
     <row r="5" spans="1:24" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="276"/>
-      <c r="B5" s="277"/>
-      <c r="C5" s="277"/>
-      <c r="D5" s="277"/>
-      <c r="E5" s="277"/>
-      <c r="F5" s="277"/>
-      <c r="G5" s="277"/>
-      <c r="H5" s="277"/>
-      <c r="I5" s="277"/>
-      <c r="J5" s="277"/>
-      <c r="K5" s="277"/>
-      <c r="L5" s="277"/>
-      <c r="M5" s="278"/>
-      <c r="N5" s="276"/>
-      <c r="O5" s="277"/>
-      <c r="P5" s="277"/>
-      <c r="Q5" s="277"/>
-      <c r="R5" s="277"/>
-      <c r="S5" s="277"/>
-      <c r="T5" s="277"/>
-      <c r="U5" s="277"/>
-      <c r="V5" s="277"/>
-      <c r="W5" s="277"/>
-      <c r="X5" s="278"/>
+      <c r="A5" s="253"/>
+      <c r="B5" s="254"/>
+      <c r="C5" s="254"/>
+      <c r="D5" s="254"/>
+      <c r="E5" s="254"/>
+      <c r="F5" s="254"/>
+      <c r="G5" s="254"/>
+      <c r="H5" s="254"/>
+      <c r="I5" s="254"/>
+      <c r="J5" s="254"/>
+      <c r="K5" s="254"/>
+      <c r="L5" s="254"/>
+      <c r="M5" s="255"/>
+      <c r="N5" s="253"/>
+      <c r="O5" s="254"/>
+      <c r="P5" s="254"/>
+      <c r="Q5" s="254"/>
+      <c r="R5" s="254"/>
+      <c r="S5" s="254"/>
+      <c r="T5" s="254"/>
+      <c r="U5" s="254"/>
+      <c r="V5" s="254"/>
+      <c r="W5" s="254"/>
+      <c r="X5" s="255"/>
     </row>
     <row r="6" spans="1:24" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3"/>
@@ -7547,66 +7563,66 @@
       <c r="X6" s="3"/>
     </row>
     <row r="7" spans="1:24" s="2" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="253" t="s">
+      <c r="A7" s="252" t="s">
         <v>77</v>
       </c>
-      <c r="B7" s="253"/>
-      <c r="C7" s="253"/>
-      <c r="D7" s="253"/>
-      <c r="E7" s="253"/>
-      <c r="F7" s="253"/>
-      <c r="G7" s="253"/>
-      <c r="H7" s="253"/>
-      <c r="I7" s="253"/>
-      <c r="J7" s="253" t="s">
+      <c r="B7" s="252"/>
+      <c r="C7" s="252"/>
+      <c r="D7" s="252"/>
+      <c r="E7" s="252"/>
+      <c r="F7" s="252"/>
+      <c r="G7" s="252"/>
+      <c r="H7" s="252"/>
+      <c r="I7" s="252"/>
+      <c r="J7" s="252" t="s">
         <v>78</v>
       </c>
-      <c r="K7" s="253"/>
-      <c r="L7" s="253"/>
-      <c r="M7" s="253"/>
-      <c r="N7" s="253"/>
-      <c r="O7" s="253"/>
-      <c r="P7" s="253" t="s">
+      <c r="K7" s="252"/>
+      <c r="L7" s="252"/>
+      <c r="M7" s="252"/>
+      <c r="N7" s="252"/>
+      <c r="O7" s="252"/>
+      <c r="P7" s="252" t="s">
         <v>79</v>
       </c>
-      <c r="Q7" s="253"/>
-      <c r="R7" s="253"/>
-      <c r="S7" s="253"/>
-      <c r="T7" s="253"/>
-      <c r="U7" s="253"/>
-      <c r="V7" s="253"/>
-      <c r="W7" s="253"/>
-      <c r="X7" s="253"/>
+      <c r="Q7" s="252"/>
+      <c r="R7" s="252"/>
+      <c r="S7" s="252"/>
+      <c r="T7" s="252"/>
+      <c r="U7" s="252"/>
+      <c r="V7" s="252"/>
+      <c r="W7" s="252"/>
+      <c r="X7" s="252"/>
     </row>
     <row r="8" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="260"/>
-      <c r="B8" s="260"/>
-      <c r="C8" s="260"/>
-      <c r="D8" s="260"/>
-      <c r="E8" s="260"/>
-      <c r="F8" s="260"/>
-      <c r="G8" s="260"/>
-      <c r="H8" s="260"/>
-      <c r="I8" s="260"/>
-      <c r="J8" s="261" t="s">
+      <c r="A8" s="261"/>
+      <c r="B8" s="261"/>
+      <c r="C8" s="261"/>
+      <c r="D8" s="261"/>
+      <c r="E8" s="261"/>
+      <c r="F8" s="261"/>
+      <c r="G8" s="261"/>
+      <c r="H8" s="261"/>
+      <c r="I8" s="261"/>
+      <c r="J8" s="262" t="s">
         <v>80</v>
       </c>
-      <c r="K8" s="262"/>
-      <c r="L8" s="262"/>
-      <c r="M8" s="262"/>
-      <c r="N8" s="262"/>
-      <c r="O8" s="263"/>
-      <c r="P8" s="261" t="s">
+      <c r="K8" s="263"/>
+      <c r="L8" s="263"/>
+      <c r="M8" s="263"/>
+      <c r="N8" s="263"/>
+      <c r="O8" s="264"/>
+      <c r="P8" s="262" t="s">
         <v>81</v>
       </c>
-      <c r="Q8" s="262"/>
-      <c r="R8" s="262"/>
-      <c r="S8" s="262"/>
-      <c r="T8" s="262"/>
-      <c r="U8" s="262"/>
-      <c r="V8" s="262"/>
-      <c r="W8" s="262"/>
-      <c r="X8" s="263"/>
+      <c r="Q8" s="263"/>
+      <c r="R8" s="263"/>
+      <c r="S8" s="263"/>
+      <c r="T8" s="263"/>
+      <c r="U8" s="263"/>
+      <c r="V8" s="263"/>
+      <c r="W8" s="263"/>
+      <c r="X8" s="264"/>
     </row>
     <row r="9" spans="1:24" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3"/>
@@ -7635,66 +7651,66 @@
       <c r="X9" s="3"/>
     </row>
     <row r="10" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="273" t="s">
+      <c r="A10" s="265" t="s">
         <v>82</v>
       </c>
-      <c r="B10" s="273"/>
-      <c r="C10" s="273"/>
-      <c r="D10" s="273"/>
-      <c r="E10" s="273"/>
-      <c r="F10" s="273"/>
-      <c r="G10" s="273"/>
-      <c r="H10" s="273"/>
-      <c r="I10" s="273"/>
-      <c r="J10" s="273"/>
-      <c r="K10" s="273"/>
-      <c r="L10" s="273"/>
-      <c r="M10" s="273"/>
-      <c r="N10" s="273"/>
-      <c r="O10" s="273"/>
-      <c r="P10" s="273"/>
-      <c r="Q10" s="273"/>
-      <c r="R10" s="273"/>
-      <c r="S10" s="273"/>
-      <c r="T10" s="273"/>
-      <c r="U10" s="273"/>
-      <c r="V10" s="273"/>
-      <c r="W10" s="273"/>
-      <c r="X10" s="273"/>
+      <c r="B10" s="265"/>
+      <c r="C10" s="265"/>
+      <c r="D10" s="265"/>
+      <c r="E10" s="265"/>
+      <c r="F10" s="265"/>
+      <c r="G10" s="265"/>
+      <c r="H10" s="265"/>
+      <c r="I10" s="265"/>
+      <c r="J10" s="265"/>
+      <c r="K10" s="265"/>
+      <c r="L10" s="265"/>
+      <c r="M10" s="265"/>
+      <c r="N10" s="265"/>
+      <c r="O10" s="265"/>
+      <c r="P10" s="265"/>
+      <c r="Q10" s="265"/>
+      <c r="R10" s="265"/>
+      <c r="S10" s="265"/>
+      <c r="T10" s="265"/>
+      <c r="U10" s="265"/>
+      <c r="V10" s="265"/>
+      <c r="W10" s="265"/>
+      <c r="X10" s="265"/>
     </row>
     <row r="11" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="274" t="s">
+      <c r="A11" s="266" t="s">
         <v>83</v>
       </c>
-      <c r="B11" s="274"/>
-      <c r="C11" s="274"/>
-      <c r="D11" s="274"/>
-      <c r="E11" s="274"/>
-      <c r="F11" s="274"/>
-      <c r="G11" s="274" t="s">
+      <c r="B11" s="266"/>
+      <c r="C11" s="266"/>
+      <c r="D11" s="266"/>
+      <c r="E11" s="266"/>
+      <c r="F11" s="266"/>
+      <c r="G11" s="266" t="s">
         <v>84</v>
       </c>
-      <c r="H11" s="274"/>
-      <c r="I11" s="274"/>
-      <c r="J11" s="274"/>
-      <c r="K11" s="274"/>
-      <c r="L11" s="274"/>
-      <c r="M11" s="274" t="s">
+      <c r="H11" s="266"/>
+      <c r="I11" s="266"/>
+      <c r="J11" s="266"/>
+      <c r="K11" s="266"/>
+      <c r="L11" s="266"/>
+      <c r="M11" s="266" t="s">
         <v>85</v>
       </c>
-      <c r="N11" s="274"/>
-      <c r="O11" s="274"/>
-      <c r="P11" s="274"/>
-      <c r="Q11" s="274"/>
-      <c r="R11" s="274"/>
-      <c r="S11" s="274" t="s">
+      <c r="N11" s="266"/>
+      <c r="O11" s="266"/>
+      <c r="P11" s="266"/>
+      <c r="Q11" s="266"/>
+      <c r="R11" s="266"/>
+      <c r="S11" s="266" t="s">
         <v>86</v>
       </c>
-      <c r="T11" s="274"/>
-      <c r="U11" s="274"/>
-      <c r="V11" s="274"/>
-      <c r="W11" s="274"/>
-      <c r="X11" s="274"/>
+      <c r="T11" s="266"/>
+      <c r="U11" s="266"/>
+      <c r="V11" s="266"/>
+      <c r="W11" s="266"/>
+      <c r="X11" s="266"/>
     </row>
     <row r="12" spans="1:24" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3"/>
@@ -7723,66 +7739,66 @@
       <c r="X12" s="3"/>
     </row>
     <row r="13" spans="1:24" s="2" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="253" t="s">
+      <c r="A13" s="252" t="s">
         <v>87</v>
       </c>
-      <c r="B13" s="253"/>
-      <c r="C13" s="253"/>
-      <c r="D13" s="253"/>
-      <c r="E13" s="253"/>
-      <c r="F13" s="253"/>
-      <c r="G13" s="253"/>
-      <c r="H13" s="253"/>
-      <c r="I13" s="253"/>
-      <c r="J13" s="253" t="s">
+      <c r="B13" s="252"/>
+      <c r="C13" s="252"/>
+      <c r="D13" s="252"/>
+      <c r="E13" s="252"/>
+      <c r="F13" s="252"/>
+      <c r="G13" s="252"/>
+      <c r="H13" s="252"/>
+      <c r="I13" s="252"/>
+      <c r="J13" s="252" t="s">
         <v>78</v>
       </c>
-      <c r="K13" s="253"/>
-      <c r="L13" s="253"/>
-      <c r="M13" s="253"/>
-      <c r="N13" s="253"/>
-      <c r="O13" s="253"/>
-      <c r="P13" s="253" t="s">
+      <c r="K13" s="252"/>
+      <c r="L13" s="252"/>
+      <c r="M13" s="252"/>
+      <c r="N13" s="252"/>
+      <c r="O13" s="252"/>
+      <c r="P13" s="252" t="s">
         <v>79</v>
       </c>
-      <c r="Q13" s="253"/>
-      <c r="R13" s="253"/>
-      <c r="S13" s="253"/>
-      <c r="T13" s="253"/>
-      <c r="U13" s="253"/>
-      <c r="V13" s="253"/>
-      <c r="W13" s="253"/>
-      <c r="X13" s="253"/>
+      <c r="Q13" s="252"/>
+      <c r="R13" s="252"/>
+      <c r="S13" s="252"/>
+      <c r="T13" s="252"/>
+      <c r="U13" s="252"/>
+      <c r="V13" s="252"/>
+      <c r="W13" s="252"/>
+      <c r="X13" s="252"/>
     </row>
     <row r="14" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="260"/>
-      <c r="B14" s="260"/>
-      <c r="C14" s="260"/>
-      <c r="D14" s="260"/>
-      <c r="E14" s="260"/>
-      <c r="F14" s="260"/>
-      <c r="G14" s="260"/>
-      <c r="H14" s="260"/>
-      <c r="I14" s="260"/>
-      <c r="J14" s="261" t="s">
+      <c r="A14" s="261"/>
+      <c r="B14" s="261"/>
+      <c r="C14" s="261"/>
+      <c r="D14" s="261"/>
+      <c r="E14" s="261"/>
+      <c r="F14" s="261"/>
+      <c r="G14" s="261"/>
+      <c r="H14" s="261"/>
+      <c r="I14" s="261"/>
+      <c r="J14" s="262" t="s">
         <v>88</v>
       </c>
-      <c r="K14" s="262"/>
-      <c r="L14" s="262"/>
-      <c r="M14" s="262"/>
-      <c r="N14" s="262"/>
-      <c r="O14" s="263"/>
-      <c r="P14" s="261" t="s">
+      <c r="K14" s="263"/>
+      <c r="L14" s="263"/>
+      <c r="M14" s="263"/>
+      <c r="N14" s="263"/>
+      <c r="O14" s="264"/>
+      <c r="P14" s="262" t="s">
         <v>89</v>
       </c>
-      <c r="Q14" s="262"/>
-      <c r="R14" s="262"/>
-      <c r="S14" s="262"/>
-      <c r="T14" s="262"/>
-      <c r="U14" s="262"/>
-      <c r="V14" s="262"/>
-      <c r="W14" s="262"/>
-      <c r="X14" s="263"/>
+      <c r="Q14" s="263"/>
+      <c r="R14" s="263"/>
+      <c r="S14" s="263"/>
+      <c r="T14" s="263"/>
+      <c r="U14" s="263"/>
+      <c r="V14" s="263"/>
+      <c r="W14" s="263"/>
+      <c r="X14" s="264"/>
     </row>
     <row r="15" spans="1:24" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3"/>
@@ -7811,184 +7827,172 @@
       <c r="X15" s="3"/>
     </row>
     <row r="16" spans="1:24" s="4" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="264" t="s">
+      <c r="A16" s="272" t="s">
         <v>90</v>
       </c>
-      <c r="B16" s="264"/>
-      <c r="C16" s="264"/>
-      <c r="D16" s="264"/>
-      <c r="E16" s="264"/>
-      <c r="F16" s="264"/>
-      <c r="G16" s="264"/>
-      <c r="H16" s="264"/>
-      <c r="I16" s="264"/>
-      <c r="J16" s="265" t="s">
+      <c r="B16" s="272"/>
+      <c r="C16" s="272"/>
+      <c r="D16" s="272"/>
+      <c r="E16" s="272"/>
+      <c r="F16" s="272"/>
+      <c r="G16" s="272"/>
+      <c r="H16" s="272"/>
+      <c r="I16" s="272"/>
+      <c r="J16" s="273" t="s">
         <v>91</v>
       </c>
-      <c r="K16" s="265"/>
-      <c r="L16" s="265"/>
-      <c r="M16" s="265"/>
-      <c r="N16" s="264" t="s">
+      <c r="K16" s="273"/>
+      <c r="L16" s="273"/>
+      <c r="M16" s="273"/>
+      <c r="N16" s="272" t="s">
         <v>92</v>
       </c>
-      <c r="O16" s="264"/>
-      <c r="P16" s="264"/>
-      <c r="Q16" s="264"/>
-      <c r="R16" s="264"/>
-      <c r="S16" s="264"/>
-      <c r="T16" s="266" t="s">
+      <c r="O16" s="272"/>
+      <c r="P16" s="272"/>
+      <c r="Q16" s="272"/>
+      <c r="R16" s="272"/>
+      <c r="S16" s="272"/>
+      <c r="T16" s="274" t="s">
         <v>93</v>
       </c>
-      <c r="U16" s="266"/>
-      <c r="V16" s="266"/>
-      <c r="W16" s="266"/>
-      <c r="X16" s="266"/>
+      <c r="U16" s="274"/>
+      <c r="V16" s="274"/>
+      <c r="W16" s="274"/>
+      <c r="X16" s="274"/>
     </row>
     <row r="17" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="254" t="s">
+      <c r="A17" s="267" t="s">
         <v>94</v>
       </c>
-      <c r="B17" s="255"/>
-      <c r="C17" s="255"/>
-      <c r="D17" s="255"/>
-      <c r="E17" s="255"/>
-      <c r="F17" s="255"/>
-      <c r="G17" s="255"/>
-      <c r="H17" s="255"/>
-      <c r="I17" s="256"/>
-      <c r="J17" s="267" t="s">
+      <c r="B17" s="259"/>
+      <c r="C17" s="259"/>
+      <c r="D17" s="259"/>
+      <c r="E17" s="259"/>
+      <c r="F17" s="259"/>
+      <c r="G17" s="259"/>
+      <c r="H17" s="259"/>
+      <c r="I17" s="268"/>
+      <c r="J17" s="275" t="s">
         <v>95</v>
       </c>
-      <c r="K17" s="268"/>
-      <c r="L17" s="268"/>
-      <c r="M17" s="269"/>
-      <c r="N17" s="254" t="s">
+      <c r="K17" s="276"/>
+      <c r="L17" s="276"/>
+      <c r="M17" s="277"/>
+      <c r="N17" s="267" t="s">
         <v>96</v>
       </c>
-      <c r="O17" s="255"/>
-      <c r="P17" s="255"/>
-      <c r="Q17" s="255"/>
-      <c r="R17" s="255"/>
-      <c r="S17" s="256"/>
-      <c r="T17" s="254" t="s">
+      <c r="O17" s="259"/>
+      <c r="P17" s="259"/>
+      <c r="Q17" s="259"/>
+      <c r="R17" s="259"/>
+      <c r="S17" s="268"/>
+      <c r="T17" s="267" t="s">
         <v>97</v>
       </c>
-      <c r="U17" s="255"/>
-      <c r="V17" s="255"/>
-      <c r="W17" s="255"/>
-      <c r="X17" s="256"/>
+      <c r="U17" s="259"/>
+      <c r="V17" s="259"/>
+      <c r="W17" s="259"/>
+      <c r="X17" s="268"/>
     </row>
     <row r="18" spans="1:24" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="257"/>
-      <c r="B18" s="258"/>
-      <c r="C18" s="258"/>
-      <c r="D18" s="258"/>
-      <c r="E18" s="258"/>
-      <c r="F18" s="258"/>
-      <c r="G18" s="258"/>
-      <c r="H18" s="258"/>
-      <c r="I18" s="259"/>
-      <c r="J18" s="270"/>
-      <c r="K18" s="271"/>
-      <c r="L18" s="271"/>
-      <c r="M18" s="272"/>
-      <c r="N18" s="257"/>
-      <c r="O18" s="258"/>
-      <c r="P18" s="258"/>
-      <c r="Q18" s="258"/>
-      <c r="R18" s="258"/>
-      <c r="S18" s="259"/>
-      <c r="T18" s="257"/>
-      <c r="U18" s="258"/>
-      <c r="V18" s="258"/>
-      <c r="W18" s="258"/>
-      <c r="X18" s="259"/>
+      <c r="A18" s="269"/>
+      <c r="B18" s="270"/>
+      <c r="C18" s="270"/>
+      <c r="D18" s="270"/>
+      <c r="E18" s="270"/>
+      <c r="F18" s="270"/>
+      <c r="G18" s="270"/>
+      <c r="H18" s="270"/>
+      <c r="I18" s="271"/>
+      <c r="J18" s="278"/>
+      <c r="K18" s="279"/>
+      <c r="L18" s="279"/>
+      <c r="M18" s="280"/>
+      <c r="N18" s="269"/>
+      <c r="O18" s="270"/>
+      <c r="P18" s="270"/>
+      <c r="Q18" s="270"/>
+      <c r="R18" s="270"/>
+      <c r="S18" s="271"/>
+      <c r="T18" s="269"/>
+      <c r="U18" s="270"/>
+      <c r="V18" s="270"/>
+      <c r="W18" s="270"/>
+      <c r="X18" s="271"/>
     </row>
     <row r="19" spans="1:24" ht="39" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="20" spans="1:24" ht="39" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="21" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A21" s="252" t="s">
+      <c r="A21" s="284" t="s">
         <v>98</v>
       </c>
-      <c r="B21" s="252"/>
-      <c r="C21" s="252"/>
-      <c r="D21" s="252"/>
-      <c r="E21" s="252"/>
-      <c r="F21" s="252"/>
-      <c r="G21" s="252"/>
-      <c r="H21" s="252"/>
+      <c r="B21" s="284"/>
+      <c r="C21" s="284"/>
+      <c r="D21" s="284"/>
+      <c r="E21" s="284"/>
+      <c r="F21" s="284"/>
+      <c r="G21" s="284"/>
+      <c r="H21" s="284"/>
       <c r="I21" s="5"/>
-      <c r="J21" s="252" t="s">
+      <c r="J21" s="284" t="s">
         <v>65</v>
       </c>
-      <c r="K21" s="252"/>
-      <c r="L21" s="252"/>
-      <c r="M21" s="252"/>
-      <c r="N21" s="252"/>
-      <c r="O21" s="252"/>
-      <c r="P21" s="252"/>
+      <c r="K21" s="284"/>
+      <c r="L21" s="284"/>
+      <c r="M21" s="284"/>
+      <c r="N21" s="284"/>
+      <c r="O21" s="284"/>
+      <c r="P21" s="284"/>
       <c r="Q21" s="6"/>
-      <c r="R21" s="252" t="s">
+      <c r="R21" s="284" t="s">
         <v>99</v>
       </c>
-      <c r="S21" s="252"/>
-      <c r="T21" s="252"/>
-      <c r="U21" s="252"/>
-      <c r="V21" s="252"/>
-      <c r="W21" s="252"/>
-      <c r="X21" s="252"/>
+      <c r="S21" s="284"/>
+      <c r="T21" s="284"/>
+      <c r="U21" s="284"/>
+      <c r="V21" s="284"/>
+      <c r="W21" s="284"/>
+      <c r="X21" s="284"/>
     </row>
     <row r="23" spans="1:24" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="P23" s="249" t="s">
+      <c r="P23" s="281" t="s">
         <v>100</v>
       </c>
-      <c r="Q23" s="249"/>
-      <c r="R23" s="249"/>
-      <c r="S23" s="249"/>
-      <c r="T23" s="249"/>
-      <c r="U23" s="250" t="s">
+      <c r="Q23" s="281"/>
+      <c r="R23" s="281"/>
+      <c r="S23" s="281"/>
+      <c r="T23" s="281"/>
+      <c r="U23" s="282" t="s">
         <v>101</v>
       </c>
-      <c r="V23" s="250"/>
-      <c r="W23" s="250"/>
-      <c r="X23" s="250"/>
+      <c r="V23" s="282"/>
+      <c r="W23" s="282"/>
+      <c r="X23" s="282"/>
     </row>
     <row r="24" spans="1:24" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="P24" s="249" t="s">
+      <c r="P24" s="281" t="s">
         <v>102</v>
       </c>
-      <c r="Q24" s="249"/>
-      <c r="R24" s="249"/>
-      <c r="S24" s="249"/>
-      <c r="T24" s="249"/>
-      <c r="U24" s="251" t="s">
+      <c r="Q24" s="281"/>
+      <c r="R24" s="281"/>
+      <c r="S24" s="281"/>
+      <c r="T24" s="281"/>
+      <c r="U24" s="283" t="s">
         <v>103</v>
       </c>
-      <c r="V24" s="251"/>
-      <c r="W24" s="251"/>
-      <c r="X24" s="251"/>
+      <c r="V24" s="283"/>
+      <c r="W24" s="283"/>
+      <c r="X24" s="283"/>
     </row>
   </sheetData>
   <mergeCells count="40">
-    <mergeCell ref="A1:T1"/>
-    <mergeCell ref="U1:X1"/>
-    <mergeCell ref="A2:T2"/>
-    <mergeCell ref="A7:I7"/>
-    <mergeCell ref="J7:O7"/>
-    <mergeCell ref="P7:X7"/>
-    <mergeCell ref="A5:M5"/>
-    <mergeCell ref="A4:M4"/>
-    <mergeCell ref="N4:X4"/>
-    <mergeCell ref="N5:X5"/>
-    <mergeCell ref="U2:X3"/>
-    <mergeCell ref="A8:I8"/>
-    <mergeCell ref="J8:O8"/>
-    <mergeCell ref="P8:X8"/>
-    <mergeCell ref="A10:X10"/>
-    <mergeCell ref="A11:F11"/>
-    <mergeCell ref="G11:L11"/>
-    <mergeCell ref="M11:R11"/>
-    <mergeCell ref="S11:X11"/>
+    <mergeCell ref="P23:T23"/>
+    <mergeCell ref="U23:X23"/>
+    <mergeCell ref="P24:T24"/>
+    <mergeCell ref="U24:X24"/>
+    <mergeCell ref="A21:H21"/>
+    <mergeCell ref="J21:P21"/>
+    <mergeCell ref="R21:X21"/>
     <mergeCell ref="A13:I13"/>
     <mergeCell ref="J13:O13"/>
     <mergeCell ref="P13:X13"/>
@@ -8003,13 +8007,25 @@
     <mergeCell ref="T16:X16"/>
     <mergeCell ref="A17:I18"/>
     <mergeCell ref="J17:M18"/>
-    <mergeCell ref="P23:T23"/>
-    <mergeCell ref="U23:X23"/>
-    <mergeCell ref="P24:T24"/>
-    <mergeCell ref="U24:X24"/>
-    <mergeCell ref="A21:H21"/>
-    <mergeCell ref="J21:P21"/>
-    <mergeCell ref="R21:X21"/>
+    <mergeCell ref="A8:I8"/>
+    <mergeCell ref="J8:O8"/>
+    <mergeCell ref="P8:X8"/>
+    <mergeCell ref="A10:X10"/>
+    <mergeCell ref="A11:F11"/>
+    <mergeCell ref="G11:L11"/>
+    <mergeCell ref="M11:R11"/>
+    <mergeCell ref="S11:X11"/>
+    <mergeCell ref="A1:T1"/>
+    <mergeCell ref="U1:X1"/>
+    <mergeCell ref="A2:T2"/>
+    <mergeCell ref="A7:I7"/>
+    <mergeCell ref="J7:O7"/>
+    <mergeCell ref="P7:X7"/>
+    <mergeCell ref="A5:M5"/>
+    <mergeCell ref="A4:M4"/>
+    <mergeCell ref="N4:X4"/>
+    <mergeCell ref="N5:X5"/>
+    <mergeCell ref="U2:X3"/>
   </mergeCells>
   <pageMargins left="0.51181102362204722" right="0.51181102362204722" top="0.35433070866141736" bottom="0.35433070866141736" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup scale="95" orientation="landscape" horizontalDpi="4294967294" verticalDpi="200" r:id="rId1"/>
@@ -8018,6 +8034,37 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <TaxCatchAll xmlns="41dd0a9e-964d-48c8-9389-7445c2a187f7" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="edbb1c21-1b45-407e-8894-c97732534993">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <_Flow_SignoffStatus xmlns="edbb1c21-1b45-407e-8894-c97732534993" xsi:nil="true"/>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <_x0031_010005470 xmlns="edbb1c21-1b45-407e-8894-c97732534993">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </_x0031_010005470>
+    <FechayHora xmlns="edbb1c21-1b45-407e-8894-c97732534993" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x01010080239B14884FBB46AB47CE62E6B5D997" ma:contentTypeVersion="24" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="95cfff668db4ca1e5f6e9375137a4a8e">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="edbb1c21-1b45-407e-8894-c97732534993" xmlns:ns3="41dd0a9e-964d-48c8-9389-7445c2a187f7" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="6912f17aaadcd6a9684df23b147afc35" ns1:_="" ns2:_="" ns3:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -8327,38 +8374,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <TaxCatchAll xmlns="41dd0a9e-964d-48c8-9389-7445c2a187f7" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="edbb1c21-1b45-407e-8894-c97732534993">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <_Flow_SignoffStatus xmlns="edbb1c21-1b45-407e-8894-c97732534993" xsi:nil="true"/>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <_x0031_010005470 xmlns="edbb1c21-1b45-407e-8894-c97732534993">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </_x0031_010005470>
-    <FechayHora xmlns="edbb1c21-1b45-407e-8894-c97732534993" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2FFAC935-8881-451D-93ED-25958414B4DF}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AAD99F47-C05E-4B8B-A445-C498A7984441}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="41dd0a9e-964d-48c8-9389-7445c2a187f7"/>
+    <ds:schemaRef ds:uri="edbb1c21-1b45-407e-8894-c97732534993"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2E0DC6A2-D4C3-4E6B-B67E-9AED22EC483E}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -8376,24 +8412,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AAD99F47-C05E-4B8B-A445-C498A7984441}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="41dd0a9e-964d-48c8-9389-7445c2a187f7"/>
-    <ds:schemaRef ds:uri="edbb1c21-1b45-407e-8894-c97732534993"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2FFAC935-8881-451D-93ED-25958414B4DF}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Actualiza Formatos a F-165 V4 y sincroniza descargas del portal.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Formatos/BITACORAS GFPI-F-147V4.xlsx
+++ b/Formatos/BITACORAS GFPI-F-147V4.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uniminuto0-my.sharepoint.com/personal/sergio_torres_mar_uniminuto_edu_co/Documents/Documentos/Seto 2026/sena/Manual SENA Etapa Productiva/manual-aprendiz-sena/Formatos/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uniminuto0-my.sharepoint.com/personal/sergio_torres_mar_uniminuto_edu_co/Documents/Documentos/Seto 2026/SETO/sena/Manual SENA Etapa Productiva/manual-aprendiz-sena/Formatos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="8" documentId="13_ncr:1_{BEF1DC7A-FFF1-4291-A724-1398C9A655DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{83410BEE-54F5-4C5C-AC98-DB36869CF98A}"/>
+  <xr:revisionPtr revIDLastSave="15" documentId="13_ncr:1_{BEF1DC7A-FFF1-4291-A724-1398C9A655DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{34869B08-79A4-49EA-A549-21A9B73FC24F}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Bitacora" sheetId="6" r:id="rId1"/>
@@ -2429,7 +2429,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="285">
+  <cellXfs count="284">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -2598,48 +2598,71 @@
     <xf numFmtId="15" fontId="32" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="111" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="112" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="113" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="114" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="115" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="116" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="117" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="119" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="118" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="82" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
-          <xfpb:xfComplement i="0"/>
-        </ext>
-      </extLst>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="107" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
-          <xfpb:xfComplement i="0"/>
-        </ext>
-      </extLst>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="111" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="112" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="113" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="114" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="115" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="116" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="117" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="119" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="118" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="77" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="78" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="71" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="75" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="59" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="62" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="53" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="102" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -2692,34 +2715,82 @@
     <xf numFmtId="0" fontId="17" fillId="0" borderId="110" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="96" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="93" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="98" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="100" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="101" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="92" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="93" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="89" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="90" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="64" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="66" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="67" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="84" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="85" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="86" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="66" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="67" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="85" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="86" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="5" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="5" borderId="57" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2732,9 +2803,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="5" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2743,7 +2811,34 @@
     <xf numFmtId="0" fontId="12" fillId="5" borderId="64" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="64" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="96" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="93" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="97" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="100" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="7" borderId="91" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2773,67 +2868,40 @@
     <xf numFmtId="0" fontId="11" fillId="3" borderId="67" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="89" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="90" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="66" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="67" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="84" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="85" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="86" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="66" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="67" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="85" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="86" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="5" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="5" borderId="57" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="68" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="85" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="86" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="98" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="100" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="101" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="92" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="93" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="7" borderId="95" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2848,105 +2916,6 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="99" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="100" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="77" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="78" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="68" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="85" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="86" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="71" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="75" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="59" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="62" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="53" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="102" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="7" borderId="76" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="7" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="7" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="71" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="75" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="59" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="2" borderId="70" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="2" borderId="74" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="2" borderId="58" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2978,33 +2947,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="97" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="94" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="65" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="6" borderId="79" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3048,26 +2990,13 @@
     </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="106" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
-          <xfpb:xfComplement i="0"/>
-        </ext>
-      </extLst>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="82" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
-          <xfpb:xfComplement i="0"/>
-        </ext>
-      </extLst>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="83" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="106" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="18" fillId="4" borderId="52" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3080,6 +3009,72 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="59" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="60" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="54" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="71" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="75" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="59" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="61" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="72" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="87" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="88" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="94" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="65" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="70" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3092,53 +3087,32 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="61" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="60" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="76" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="2" borderId="70" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="2" borderId="74" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="2" borderId="58" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="93" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="54" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="61" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="72" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="7" borderId="87" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="7" borderId="88" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3188,14 +3162,17 @@
     <xf numFmtId="0" fontId="28" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="93" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="93" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -3314,7 +3291,7 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FF92D050"/>
+          <bgColor rgb="FFFFFF00"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3489,6 +3466,7 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FFFFFF00"/>
       <color rgb="FFCD03A7"/>
       <color rgb="FFE1EF57"/>
       <color rgb="FFE6DE74"/>
@@ -3674,21 +3652,8 @@
 </externalLink>
 </file>
 
-<file path=xl/featurePropertyBag/featurePropertyBag.xml><?xml version="1.0" encoding="utf-8"?>
-<FeaturePropertyBags xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag">
-  <bag type="Checkbox"/>
-  <bag type="XFControls">
-    <bagId k="CellControl">0</bagId>
-  </bag>
-  <bag type="XFComplement">
-    <bagId k="XFControls">1</bagId>
-  </bag>
-  <bag type="XFComplements" extRef="XFComplementsMapperExtRef">
-    <a k="MappedFeaturePropertyBags">
-      <bagId>2</bagId>
-    </a>
-  </bag>
-</FeaturePropertyBags>
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4084,16 +4049,16 @@
       <c r="AB2" s="7"/>
     </row>
     <row r="3" spans="2:28" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="191" t="s">
+      <c r="B3" s="175" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="192"/>
-      <c r="D3" s="192"/>
-      <c r="E3" s="192"/>
-      <c r="F3" s="192"/>
-      <c r="G3" s="192"/>
-      <c r="H3" s="192"/>
-      <c r="I3" s="193"/>
+      <c r="C3" s="176"/>
+      <c r="D3" s="176"/>
+      <c r="E3" s="176"/>
+      <c r="F3" s="176"/>
+      <c r="G3" s="176"/>
+      <c r="H3" s="176"/>
+      <c r="I3" s="177"/>
       <c r="J3" s="8"/>
       <c r="K3" s="7"/>
       <c r="L3" s="7"/>
@@ -4115,16 +4080,16 @@
       <c r="AB3" s="7"/>
     </row>
     <row r="4" spans="2:28" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="197" t="s">
+      <c r="B4" s="181" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="198"/>
-      <c r="D4" s="198"/>
-      <c r="E4" s="198"/>
-      <c r="F4" s="198"/>
-      <c r="G4" s="198"/>
-      <c r="H4" s="198"/>
-      <c r="I4" s="199"/>
+      <c r="C4" s="182"/>
+      <c r="D4" s="182"/>
+      <c r="E4" s="182"/>
+      <c r="F4" s="182"/>
+      <c r="G4" s="182"/>
+      <c r="H4" s="182"/>
+      <c r="I4" s="183"/>
       <c r="J4" s="8"/>
       <c r="K4" s="7"/>
       <c r="L4" s="7"/>
@@ -4146,16 +4111,16 @@
       <c r="AB4" s="7"/>
     </row>
     <row r="5" spans="2:28" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="194" t="s">
+      <c r="B5" s="178" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="195"/>
-      <c r="D5" s="195"/>
-      <c r="E5" s="195"/>
-      <c r="F5" s="195"/>
-      <c r="G5" s="195"/>
-      <c r="H5" s="195"/>
-      <c r="I5" s="196"/>
+      <c r="C5" s="179"/>
+      <c r="D5" s="179"/>
+      <c r="E5" s="179"/>
+      <c r="F5" s="179"/>
+      <c r="G5" s="179"/>
+      <c r="H5" s="179"/>
+      <c r="I5" s="180"/>
       <c r="J5" s="8"/>
       <c r="K5" s="8"/>
       <c r="L5" s="7"/>
@@ -4177,16 +4142,16 @@
       <c r="AB5" s="7"/>
     </row>
     <row r="6" spans="2:28" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="197" t="s">
+      <c r="B6" s="181" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="198"/>
-      <c r="D6" s="198"/>
-      <c r="E6" s="198"/>
-      <c r="F6" s="198"/>
-      <c r="G6" s="198"/>
-      <c r="H6" s="198"/>
-      <c r="I6" s="199"/>
+      <c r="C6" s="182"/>
+      <c r="D6" s="182"/>
+      <c r="E6" s="182"/>
+      <c r="F6" s="182"/>
+      <c r="G6" s="182"/>
+      <c r="H6" s="182"/>
+      <c r="I6" s="183"/>
       <c r="J6" s="8"/>
       <c r="K6" s="8"/>
       <c r="L6" s="7"/>
@@ -4208,16 +4173,16 @@
       <c r="AB6" s="7"/>
     </row>
     <row r="7" spans="2:28" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="194" t="s">
+      <c r="B7" s="178" t="s">
         <v>6</v>
       </c>
-      <c r="C7" s="195"/>
-      <c r="D7" s="195"/>
-      <c r="E7" s="195"/>
-      <c r="F7" s="195"/>
-      <c r="G7" s="195"/>
-      <c r="H7" s="195"/>
-      <c r="I7" s="196"/>
+      <c r="C7" s="179"/>
+      <c r="D7" s="179"/>
+      <c r="E7" s="179"/>
+      <c r="F7" s="179"/>
+      <c r="G7" s="179"/>
+      <c r="H7" s="179"/>
+      <c r="I7" s="180"/>
       <c r="J7" s="7"/>
       <c r="K7" s="7"/>
       <c r="L7" s="7"/>
@@ -4242,23 +4207,17 @@
       <c r="B8" s="53" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="204" t="b">
-        <v>0</v>
-      </c>
-      <c r="D8" s="205"/>
-      <c r="E8" s="206" t="s">
+      <c r="C8" s="188"/>
+      <c r="D8" s="189"/>
+      <c r="E8" s="190" t="s">
         <v>8</v>
       </c>
-      <c r="F8" s="207"/>
-      <c r="G8" s="58" t="b">
-        <v>0</v>
-      </c>
+      <c r="F8" s="188"/>
+      <c r="G8" s="67"/>
       <c r="H8" s="54" t="s">
         <v>9</v>
       </c>
-      <c r="I8" s="59" t="b">
-        <v>0</v>
-      </c>
+      <c r="I8" s="68"/>
       <c r="J8" s="7"/>
       <c r="K8" s="7"/>
       <c r="L8" s="7"/>
@@ -4285,8 +4244,8 @@
       <c r="D9" s="18"/>
       <c r="E9" s="23"/>
       <c r="F9" s="23"/>
-      <c r="G9" s="219"/>
-      <c r="H9" s="219"/>
+      <c r="G9" s="201"/>
+      <c r="H9" s="201"/>
       <c r="I9" s="18"/>
       <c r="J9" s="7"/>
       <c r="K9" s="7"/>
@@ -4309,18 +4268,18 @@
       <c r="AB9" s="7"/>
     </row>
     <row r="10" spans="2:28" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="175" t="s">
+      <c r="B10" s="168" t="s">
         <v>10</v>
       </c>
-      <c r="C10" s="176"/>
-      <c r="D10" s="177"/>
-      <c r="E10" s="171" t="s">
+      <c r="C10" s="169"/>
+      <c r="D10" s="170"/>
+      <c r="E10" s="164" t="s">
         <v>11</v>
       </c>
-      <c r="F10" s="171"/>
-      <c r="G10" s="171"/>
-      <c r="H10" s="171"/>
-      <c r="I10" s="171"/>
+      <c r="F10" s="164"/>
+      <c r="G10" s="164"/>
+      <c r="H10" s="164"/>
+      <c r="I10" s="164"/>
       <c r="J10" s="7"/>
       <c r="K10" s="7"/>
       <c r="L10" s="7"/>
@@ -4342,14 +4301,14 @@
       <c r="AB10" s="7"/>
     </row>
     <row r="11" spans="2:28" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="163"/>
-      <c r="C11" s="164"/>
-      <c r="D11" s="165"/>
-      <c r="E11" s="218"/>
-      <c r="F11" s="218"/>
-      <c r="G11" s="218"/>
-      <c r="H11" s="218"/>
-      <c r="I11" s="218"/>
+      <c r="B11" s="198"/>
+      <c r="C11" s="199"/>
+      <c r="D11" s="200"/>
+      <c r="E11" s="197"/>
+      <c r="F11" s="197"/>
+      <c r="G11" s="197"/>
+      <c r="H11" s="197"/>
+      <c r="I11" s="197"/>
       <c r="J11" s="7"/>
       <c r="K11" s="7"/>
       <c r="L11" s="7"/>
@@ -4376,8 +4335,8 @@
       <c r="D12" s="18"/>
       <c r="E12" s="23"/>
       <c r="F12" s="23"/>
-      <c r="G12" s="219"/>
-      <c r="H12" s="219"/>
+      <c r="G12" s="201"/>
+      <c r="H12" s="201"/>
       <c r="I12" s="18"/>
       <c r="J12" s="7"/>
       <c r="K12" s="7"/>
@@ -4400,16 +4359,16 @@
       <c r="AB12" s="7"/>
     </row>
     <row r="13" spans="2:28" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="216" t="s">
+      <c r="B13" s="195" t="s">
         <v>12</v>
       </c>
-      <c r="C13" s="216"/>
-      <c r="D13" s="216"/>
-      <c r="E13" s="216"/>
-      <c r="F13" s="216"/>
-      <c r="G13" s="216"/>
-      <c r="H13" s="216"/>
-      <c r="I13" s="217"/>
+      <c r="C13" s="195"/>
+      <c r="D13" s="195"/>
+      <c r="E13" s="195"/>
+      <c r="F13" s="195"/>
+      <c r="G13" s="195"/>
+      <c r="H13" s="195"/>
+      <c r="I13" s="196"/>
       <c r="J13" s="7"/>
       <c r="K13" s="7"/>
       <c r="L13" s="7"/>
@@ -4431,32 +4390,32 @@
       <c r="AB13" s="7"/>
     </row>
     <row r="14" spans="2:28" s="9" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="175" t="s">
+      <c r="B14" s="168" t="s">
         <v>13</v>
       </c>
-      <c r="C14" s="176"/>
-      <c r="D14" s="177"/>
+      <c r="C14" s="169"/>
+      <c r="D14" s="170"/>
       <c r="E14" s="55" t="s">
         <v>14</v>
       </c>
-      <c r="F14" s="208" t="s">
+      <c r="F14" s="191" t="s">
         <v>15</v>
       </c>
-      <c r="G14" s="209"/>
-      <c r="H14" s="171" t="s">
+      <c r="G14" s="192"/>
+      <c r="H14" s="164" t="s">
         <v>16</v>
       </c>
-      <c r="I14" s="172"/>
+      <c r="I14" s="165"/>
     </row>
     <row r="15" spans="2:28" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="201"/>
-      <c r="C15" s="202"/>
-      <c r="D15" s="203"/>
+      <c r="B15" s="185"/>
+      <c r="C15" s="186"/>
+      <c r="D15" s="187"/>
       <c r="E15" s="37"/>
-      <c r="F15" s="210"/>
-      <c r="G15" s="211"/>
-      <c r="H15" s="185"/>
-      <c r="I15" s="200"/>
+      <c r="F15" s="193"/>
+      <c r="G15" s="194"/>
+      <c r="H15" s="135"/>
+      <c r="I15" s="184"/>
       <c r="J15" s="7"/>
       <c r="K15" s="7"/>
       <c r="L15" s="7"/>
@@ -4478,20 +4437,20 @@
       <c r="AB15" s="7"/>
     </row>
     <row r="16" spans="2:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="212" t="s">
+      <c r="B16" s="217" t="s">
         <v>17</v>
       </c>
-      <c r="C16" s="213"/>
-      <c r="D16" s="214"/>
-      <c r="E16" s="215" t="s">
+      <c r="C16" s="218"/>
+      <c r="D16" s="219"/>
+      <c r="E16" s="220" t="s">
         <v>18</v>
       </c>
-      <c r="F16" s="215"/>
-      <c r="G16" s="215"/>
-      <c r="H16" s="220" t="s">
+      <c r="F16" s="220"/>
+      <c r="G16" s="220"/>
+      <c r="H16" s="202" t="s">
         <v>19</v>
       </c>
-      <c r="I16" s="221"/>
+      <c r="I16" s="203"/>
       <c r="J16" s="7"/>
       <c r="K16" s="7"/>
       <c r="L16" s="7"/>
@@ -4513,14 +4472,14 @@
       <c r="AB16" s="7"/>
     </row>
     <row r="17" spans="2:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="163"/>
-      <c r="C17" s="164"/>
-      <c r="D17" s="165"/>
-      <c r="E17" s="181"/>
-      <c r="F17" s="181"/>
-      <c r="G17" s="181"/>
-      <c r="H17" s="173"/>
-      <c r="I17" s="174"/>
+      <c r="B17" s="198"/>
+      <c r="C17" s="199"/>
+      <c r="D17" s="200"/>
+      <c r="E17" s="174"/>
+      <c r="F17" s="174"/>
+      <c r="G17" s="174"/>
+      <c r="H17" s="166"/>
+      <c r="I17" s="167"/>
       <c r="J17" s="7"/>
       <c r="K17" s="7"/>
       <c r="L17" s="7"/>
@@ -4542,20 +4501,20 @@
       <c r="AB17" s="7"/>
     </row>
     <row r="18" spans="2:28" s="47" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="175" t="s">
+      <c r="B18" s="168" t="s">
         <v>20</v>
       </c>
-      <c r="C18" s="176"/>
-      <c r="D18" s="177"/>
-      <c r="E18" s="171" t="s">
+      <c r="C18" s="169"/>
+      <c r="D18" s="170"/>
+      <c r="E18" s="164" t="s">
         <v>21</v>
       </c>
-      <c r="F18" s="171"/>
-      <c r="G18" s="171"/>
-      <c r="H18" s="171" t="s">
+      <c r="F18" s="164"/>
+      <c r="G18" s="164"/>
+      <c r="H18" s="164" t="s">
         <v>22</v>
       </c>
-      <c r="I18" s="172"/>
+      <c r="I18" s="165"/>
       <c r="J18" s="7"/>
       <c r="K18" s="7"/>
       <c r="L18" s="7"/>
@@ -4577,14 +4536,14 @@
       <c r="AB18" s="7"/>
     </row>
     <row r="19" spans="2:28" s="47" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="178"/>
-      <c r="C19" s="179"/>
-      <c r="D19" s="180"/>
-      <c r="E19" s="173"/>
-      <c r="F19" s="173"/>
-      <c r="G19" s="173"/>
-      <c r="H19" s="173"/>
-      <c r="I19" s="174"/>
+      <c r="B19" s="171"/>
+      <c r="C19" s="172"/>
+      <c r="D19" s="173"/>
+      <c r="E19" s="166"/>
+      <c r="F19" s="166"/>
+      <c r="G19" s="166"/>
+      <c r="H19" s="166"/>
+      <c r="I19" s="167"/>
       <c r="J19" s="7"/>
       <c r="K19" s="7"/>
       <c r="L19" s="7"/>
@@ -4606,20 +4565,20 @@
       <c r="AB19" s="7"/>
     </row>
     <row r="20" spans="2:28" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="168" t="s">
+      <c r="B20" s="225" t="s">
         <v>23</v>
       </c>
-      <c r="C20" s="169"/>
-      <c r="D20" s="170"/>
-      <c r="E20" s="166" t="s">
+      <c r="C20" s="226"/>
+      <c r="D20" s="227"/>
+      <c r="E20" s="136" t="s">
         <v>24</v>
       </c>
-      <c r="F20" s="166"/>
-      <c r="G20" s="166"/>
-      <c r="H20" s="166" t="s">
+      <c r="F20" s="136"/>
+      <c r="G20" s="136"/>
+      <c r="H20" s="136" t="s">
         <v>25</v>
       </c>
-      <c r="I20" s="167"/>
+      <c r="I20" s="224"/>
       <c r="J20" s="16"/>
       <c r="K20" s="16"/>
       <c r="L20" s="16"/>
@@ -4639,14 +4598,14 @@
       <c r="AA20" s="16"/>
     </row>
     <row r="21" spans="2:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="163"/>
-      <c r="C21" s="164"/>
-      <c r="D21" s="165"/>
-      <c r="E21" s="185"/>
-      <c r="F21" s="185"/>
-      <c r="G21" s="185"/>
-      <c r="H21" s="183"/>
-      <c r="I21" s="184"/>
+      <c r="B21" s="198"/>
+      <c r="C21" s="199"/>
+      <c r="D21" s="200"/>
+      <c r="E21" s="135"/>
+      <c r="F21" s="135"/>
+      <c r="G21" s="135"/>
+      <c r="H21" s="133"/>
+      <c r="I21" s="134"/>
       <c r="J21" s="18"/>
       <c r="K21" s="18"/>
       <c r="L21" s="18"/>
@@ -4671,8 +4630,8 @@
       <c r="D22" s="13"/>
       <c r="E22" s="33"/>
       <c r="F22" s="33"/>
-      <c r="G22" s="78"/>
-      <c r="H22" s="78"/>
+      <c r="G22" s="89"/>
+      <c r="H22" s="89"/>
       <c r="I22" s="13"/>
       <c r="J22" s="13"/>
       <c r="K22" s="13"/>
@@ -4694,16 +4653,16 @@
       <c r="AA22" s="13"/>
     </row>
     <row r="23" spans="2:28" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="139" t="s">
+      <c r="B23" s="69" t="s">
         <v>26</v>
       </c>
-      <c r="C23" s="140"/>
-      <c r="D23" s="140"/>
-      <c r="E23" s="140"/>
-      <c r="F23" s="140"/>
-      <c r="G23" s="140"/>
-      <c r="H23" s="140"/>
-      <c r="I23" s="141"/>
+      <c r="C23" s="70"/>
+      <c r="D23" s="70"/>
+      <c r="E23" s="70"/>
+      <c r="F23" s="70"/>
+      <c r="G23" s="70"/>
+      <c r="H23" s="70"/>
+      <c r="I23" s="71"/>
       <c r="J23" s="13"/>
       <c r="K23" s="13"/>
       <c r="L23" s="13"/>
@@ -4724,20 +4683,20 @@
       <c r="AA23" s="13"/>
     </row>
     <row r="24" spans="2:28" s="9" customFormat="1" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="182" t="s">
+      <c r="B24" s="131" t="s">
         <v>27</v>
       </c>
-      <c r="C24" s="88"/>
-      <c r="D24" s="88"/>
-      <c r="E24" s="88"/>
-      <c r="F24" s="186" t="s">
+      <c r="C24" s="132"/>
+      <c r="D24" s="132"/>
+      <c r="E24" s="132"/>
+      <c r="F24" s="137" t="s">
         <v>28</v>
       </c>
-      <c r="G24" s="186"/>
-      <c r="H24" s="88" t="s">
+      <c r="G24" s="137"/>
+      <c r="H24" s="132" t="s">
         <v>29</v>
       </c>
-      <c r="I24" s="89"/>
+      <c r="I24" s="153"/>
       <c r="J24" s="18"/>
       <c r="K24" s="18"/>
       <c r="M24" s="16"/>
@@ -4750,14 +4709,14 @@
       <c r="AB24" s="10"/>
     </row>
     <row r="25" spans="2:28" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="137"/>
+      <c r="B25" s="163"/>
       <c r="C25" s="138"/>
       <c r="D25" s="138"/>
       <c r="E25" s="138"/>
       <c r="F25" s="138"/>
       <c r="G25" s="138"/>
-      <c r="H25" s="90"/>
-      <c r="I25" s="91"/>
+      <c r="H25" s="154"/>
+      <c r="I25" s="155"/>
       <c r="J25" s="18"/>
       <c r="K25" s="18"/>
       <c r="M25" s="18"/>
@@ -4774,8 +4733,8 @@
       <c r="D26" s="13"/>
       <c r="E26" s="33"/>
       <c r="F26" s="33"/>
-      <c r="G26" s="78"/>
-      <c r="H26" s="78"/>
+      <c r="G26" s="89"/>
+      <c r="H26" s="89"/>
       <c r="I26" s="13"/>
       <c r="J26" s="13"/>
       <c r="K26" s="13"/>
@@ -4797,16 +4756,16 @@
       <c r="AA26" s="13"/>
     </row>
     <row r="27" spans="2:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B27" s="134" t="s">
+      <c r="B27" s="160" t="s">
         <v>30</v>
       </c>
-      <c r="C27" s="135"/>
-      <c r="D27" s="135"/>
-      <c r="E27" s="135"/>
-      <c r="F27" s="135"/>
-      <c r="G27" s="135"/>
-      <c r="H27" s="135"/>
-      <c r="I27" s="136"/>
+      <c r="C27" s="161"/>
+      <c r="D27" s="161"/>
+      <c r="E27" s="161"/>
+      <c r="F27" s="161"/>
+      <c r="G27" s="161"/>
+      <c r="H27" s="161"/>
+      <c r="I27" s="162"/>
       <c r="J27" s="13"/>
       <c r="K27" s="13"/>
       <c r="L27" s="13"/>
@@ -4827,22 +4786,22 @@
       <c r="AA27" s="13"/>
     </row>
     <row r="28" spans="2:28" s="9" customFormat="1" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B28" s="92" t="s">
+      <c r="B28" s="156" t="s">
         <v>31</v>
       </c>
-      <c r="C28" s="88"/>
-      <c r="D28" s="88"/>
-      <c r="E28" s="186" t="s">
+      <c r="C28" s="132"/>
+      <c r="D28" s="132"/>
+      <c r="E28" s="137" t="s">
         <v>32</v>
       </c>
-      <c r="F28" s="186"/>
+      <c r="F28" s="137"/>
       <c r="G28" s="49" t="s">
         <v>33</v>
       </c>
-      <c r="H28" s="88" t="s">
+      <c r="H28" s="132" t="s">
         <v>34</v>
       </c>
-      <c r="I28" s="95"/>
+      <c r="I28" s="159"/>
       <c r="J28" s="16"/>
       <c r="N28" s="16"/>
       <c r="O28" s="16"/>
@@ -4859,14 +4818,14 @@
       <c r="AB28" s="10"/>
     </row>
     <row r="29" spans="2:28" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B29" s="93"/>
-      <c r="C29" s="94"/>
-      <c r="D29" s="94"/>
-      <c r="E29" s="94"/>
-      <c r="F29" s="94"/>
+      <c r="B29" s="157"/>
+      <c r="C29" s="158"/>
+      <c r="D29" s="158"/>
+      <c r="E29" s="158"/>
+      <c r="F29" s="158"/>
       <c r="G29" s="52"/>
-      <c r="H29" s="94"/>
-      <c r="I29" s="188"/>
+      <c r="H29" s="158"/>
+      <c r="I29" s="214"/>
       <c r="J29" s="18"/>
       <c r="N29" s="18"/>
       <c r="O29" s="18"/>
@@ -4887,8 +4846,8 @@
       <c r="D30" s="13"/>
       <c r="E30" s="33"/>
       <c r="F30" s="33"/>
-      <c r="G30" s="78"/>
-      <c r="H30" s="78"/>
+      <c r="G30" s="89"/>
+      <c r="H30" s="89"/>
       <c r="I30" s="13"/>
       <c r="J30" s="13"/>
       <c r="K30" s="13"/>
@@ -4910,16 +4869,16 @@
       <c r="AA30" s="13"/>
     </row>
     <row r="31" spans="2:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B31" s="139" t="s">
+      <c r="B31" s="69" t="s">
         <v>35</v>
       </c>
-      <c r="C31" s="140"/>
-      <c r="D31" s="140"/>
-      <c r="E31" s="140"/>
-      <c r="F31" s="140"/>
-      <c r="G31" s="140"/>
-      <c r="H31" s="140"/>
-      <c r="I31" s="141"/>
+      <c r="C31" s="70"/>
+      <c r="D31" s="70"/>
+      <c r="E31" s="70"/>
+      <c r="F31" s="70"/>
+      <c r="G31" s="70"/>
+      <c r="H31" s="70"/>
+      <c r="I31" s="71"/>
       <c r="J31" s="7"/>
       <c r="K31" s="7"/>
       <c r="L31" s="7"/>
@@ -4941,18 +4900,18 @@
       <c r="AB31" s="7"/>
     </row>
     <row r="32" spans="2:28" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B32" s="189" t="s">
+      <c r="B32" s="215" t="s">
         <v>36</v>
       </c>
-      <c r="C32" s="151"/>
-      <c r="D32" s="151"/>
-      <c r="E32" s="151"/>
-      <c r="F32" s="190"/>
-      <c r="G32" s="150" t="s">
+      <c r="C32" s="76"/>
+      <c r="D32" s="76"/>
+      <c r="E32" s="76"/>
+      <c r="F32" s="216"/>
+      <c r="G32" s="75" t="s">
         <v>37</v>
       </c>
-      <c r="H32" s="151"/>
-      <c r="I32" s="152"/>
+      <c r="H32" s="76"/>
+      <c r="I32" s="77"/>
       <c r="J32" s="7"/>
       <c r="K32" s="7"/>
       <c r="L32" s="7"/>
@@ -4974,18 +4933,18 @@
       <c r="AB32" s="7"/>
     </row>
     <row r="33" spans="2:28" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B33" s="147" t="s">
+      <c r="B33" s="72" t="s">
         <v>104</v>
       </c>
-      <c r="C33" s="148"/>
-      <c r="D33" s="148"/>
-      <c r="E33" s="148"/>
-      <c r="F33" s="149"/>
-      <c r="G33" s="153" t="s">
+      <c r="C33" s="73"/>
+      <c r="D33" s="73"/>
+      <c r="E33" s="73"/>
+      <c r="F33" s="74"/>
+      <c r="G33" s="78" t="s">
         <v>105</v>
       </c>
-      <c r="H33" s="148"/>
-      <c r="I33" s="154"/>
+      <c r="H33" s="73"/>
+      <c r="I33" s="79"/>
       <c r="J33" s="7"/>
       <c r="K33" s="7"/>
       <c r="L33" s="7"/>
@@ -5012,8 +4971,8 @@
       <c r="D34" s="13"/>
       <c r="E34" s="33"/>
       <c r="F34" s="33"/>
-      <c r="G34" s="78"/>
-      <c r="H34" s="78"/>
+      <c r="G34" s="89"/>
+      <c r="H34" s="89"/>
       <c r="I34" s="13"/>
       <c r="J34" s="13"/>
       <c r="K34" s="13"/>
@@ -5035,16 +4994,16 @@
       <c r="AA34" s="13"/>
     </row>
     <row r="35" spans="2:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B35" s="110" t="s">
+      <c r="B35" s="145" t="s">
         <v>38</v>
       </c>
-      <c r="C35" s="111"/>
-      <c r="D35" s="111"/>
-      <c r="E35" s="111"/>
-      <c r="F35" s="111"/>
-      <c r="G35" s="111"/>
-      <c r="H35" s="111"/>
-      <c r="I35" s="112"/>
+      <c r="C35" s="146"/>
+      <c r="D35" s="146"/>
+      <c r="E35" s="146"/>
+      <c r="F35" s="146"/>
+      <c r="G35" s="146"/>
+      <c r="H35" s="146"/>
+      <c r="I35" s="147"/>
       <c r="J35" s="39"/>
       <c r="K35" s="19"/>
       <c r="L35" s="19"/>
@@ -5068,19 +5027,19 @@
       <c r="B36" s="41" t="s">
         <v>39</v>
       </c>
-      <c r="C36" s="144" t="s">
+      <c r="C36" s="150" t="s">
         <v>40</v>
       </c>
-      <c r="D36" s="145"/>
-      <c r="E36" s="145"/>
-      <c r="F36" s="146"/>
+      <c r="D36" s="151"/>
+      <c r="E36" s="151"/>
+      <c r="F36" s="152"/>
       <c r="G36" s="41" t="s">
         <v>39</v>
       </c>
-      <c r="H36" s="142" t="s">
+      <c r="H36" s="148" t="s">
         <v>41</v>
       </c>
-      <c r="I36" s="143"/>
+      <c r="I36" s="149"/>
       <c r="J36" s="40"/>
       <c r="K36" s="19"/>
       <c r="L36" s="19"/>
@@ -5104,15 +5063,15 @@
       <c r="B37" s="100" t="s">
         <v>42</v>
       </c>
-      <c r="C37" s="118"/>
-      <c r="D37" s="119"/>
-      <c r="E37" s="119"/>
-      <c r="F37" s="120"/>
+      <c r="C37" s="104"/>
+      <c r="D37" s="105"/>
+      <c r="E37" s="105"/>
+      <c r="F37" s="106"/>
       <c r="G37" s="100" t="s">
         <v>43</v>
       </c>
-      <c r="H37" s="96"/>
-      <c r="I37" s="97"/>
+      <c r="H37" s="123"/>
+      <c r="I37" s="124"/>
       <c r="J37" s="39"/>
       <c r="K37" s="16"/>
       <c r="L37" s="18"/>
@@ -5131,14 +5090,14 @@
       <c r="AB37" s="12"/>
     </row>
     <row r="38" spans="2:28" s="11" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B38" s="101"/>
-      <c r="C38" s="121"/>
-      <c r="D38" s="78"/>
-      <c r="E38" s="78"/>
-      <c r="F38" s="122"/>
-      <c r="G38" s="103"/>
-      <c r="H38" s="98"/>
-      <c r="I38" s="99"/>
+      <c r="B38" s="127"/>
+      <c r="C38" s="107"/>
+      <c r="D38" s="89"/>
+      <c r="E38" s="89"/>
+      <c r="F38" s="108"/>
+      <c r="G38" s="101"/>
+      <c r="H38" s="125"/>
+      <c r="I38" s="126"/>
       <c r="J38" s="39"/>
       <c r="K38" s="16"/>
       <c r="L38" s="18"/>
@@ -5156,16 +5115,16 @@
       <c r="AB38" s="12"/>
     </row>
     <row r="39" spans="2:28" s="11" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B39" s="101"/>
-      <c r="C39" s="121"/>
-      <c r="D39" s="78"/>
-      <c r="E39" s="78"/>
-      <c r="F39" s="122"/>
+      <c r="B39" s="127"/>
+      <c r="C39" s="107"/>
+      <c r="D39" s="89"/>
+      <c r="E39" s="89"/>
+      <c r="F39" s="108"/>
       <c r="G39" s="100" t="s">
         <v>44</v>
       </c>
-      <c r="H39" s="96"/>
-      <c r="I39" s="97"/>
+      <c r="H39" s="123"/>
+      <c r="I39" s="124"/>
       <c r="J39" s="39"/>
       <c r="K39" s="16"/>
       <c r="L39" s="18"/>
@@ -5184,14 +5143,14 @@
       <c r="AB39" s="12"/>
     </row>
     <row r="40" spans="2:28" s="11" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B40" s="102"/>
-      <c r="C40" s="123"/>
-      <c r="D40" s="124"/>
-      <c r="E40" s="124"/>
-      <c r="F40" s="125"/>
-      <c r="G40" s="103"/>
-      <c r="H40" s="98"/>
-      <c r="I40" s="99"/>
+      <c r="B40" s="128"/>
+      <c r="C40" s="109"/>
+      <c r="D40" s="110"/>
+      <c r="E40" s="110"/>
+      <c r="F40" s="111"/>
+      <c r="G40" s="101"/>
+      <c r="H40" s="125"/>
+      <c r="I40" s="126"/>
       <c r="J40" s="39"/>
       <c r="K40" s="16"/>
       <c r="L40" s="18"/>
@@ -5210,18 +5169,18 @@
       <c r="AB40" s="12"/>
     </row>
     <row r="41" spans="2:28" s="11" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B41" s="132" t="s">
+      <c r="B41" s="118" t="s">
         <v>45</v>
       </c>
-      <c r="C41" s="126"/>
-      <c r="D41" s="127"/>
-      <c r="E41" s="127"/>
-      <c r="F41" s="128"/>
+      <c r="C41" s="112"/>
+      <c r="D41" s="113"/>
+      <c r="E41" s="113"/>
+      <c r="F41" s="114"/>
       <c r="G41" s="100" t="s">
         <v>46</v>
       </c>
-      <c r="H41" s="106"/>
-      <c r="I41" s="107"/>
+      <c r="H41" s="141"/>
+      <c r="I41" s="142"/>
       <c r="J41" s="56"/>
       <c r="K41" s="16"/>
       <c r="L41" s="17"/>
@@ -5243,14 +5202,14 @@
       <c r="AB41" s="12"/>
     </row>
     <row r="42" spans="2:28" s="38" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B42" s="133"/>
-      <c r="C42" s="129"/>
-      <c r="D42" s="130"/>
-      <c r="E42" s="130"/>
-      <c r="F42" s="131"/>
-      <c r="G42" s="105"/>
-      <c r="H42" s="108"/>
-      <c r="I42" s="109"/>
+      <c r="B42" s="119"/>
+      <c r="C42" s="115"/>
+      <c r="D42" s="116"/>
+      <c r="E42" s="116"/>
+      <c r="F42" s="117"/>
+      <c r="G42" s="140"/>
+      <c r="H42" s="143"/>
+      <c r="I42" s="144"/>
       <c r="J42" s="56"/>
       <c r="K42" s="16"/>
       <c r="L42" s="17"/>
@@ -5277,8 +5236,8 @@
       <c r="D43" s="43"/>
       <c r="E43" s="43"/>
       <c r="F43" s="43"/>
-      <c r="G43" s="116"/>
-      <c r="H43" s="117"/>
+      <c r="G43" s="102"/>
+      <c r="H43" s="103"/>
       <c r="I43" s="43"/>
       <c r="J43" s="56"/>
       <c r="K43" s="16"/>
@@ -5301,16 +5260,16 @@
       <c r="AB43" s="12"/>
     </row>
     <row r="44" spans="2:28" s="11" customFormat="1" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B44" s="114" t="s">
+      <c r="B44" s="98" t="s">
         <v>47</v>
       </c>
-      <c r="C44" s="114"/>
-      <c r="D44" s="114"/>
-      <c r="E44" s="114"/>
-      <c r="F44" s="114"/>
-      <c r="G44" s="114"/>
-      <c r="H44" s="114"/>
-      <c r="I44" s="115"/>
+      <c r="C44" s="98"/>
+      <c r="D44" s="98"/>
+      <c r="E44" s="98"/>
+      <c r="F44" s="98"/>
+      <c r="G44" s="98"/>
+      <c r="H44" s="98"/>
+      <c r="I44" s="99"/>
       <c r="J44" s="16"/>
       <c r="K44" s="16"/>
       <c r="L44" s="17"/>
@@ -5332,24 +5291,24 @@
       <c r="AB44" s="12"/>
     </row>
     <row r="45" spans="2:28" ht="68.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B45" s="161" t="s">
+      <c r="B45" s="223" t="s">
         <v>48</v>
       </c>
-      <c r="C45" s="162"/>
-      <c r="D45" s="222" t="s">
+      <c r="C45" s="207"/>
+      <c r="D45" s="204" t="s">
         <v>49</v>
       </c>
-      <c r="E45" s="223"/>
-      <c r="F45" s="160" t="s">
+      <c r="E45" s="205"/>
+      <c r="F45" s="208" t="s">
         <v>50</v>
       </c>
-      <c r="G45" s="160" t="s">
+      <c r="G45" s="208" t="s">
         <v>51</v>
       </c>
-      <c r="H45" s="158" t="s">
+      <c r="H45" s="221" t="s">
         <v>52</v>
       </c>
-      <c r="I45" s="104" t="s">
+      <c r="I45" s="139" t="s">
         <v>53</v>
       </c>
       <c r="J45" s="16"/>
@@ -5372,14 +5331,14 @@
       <c r="AA45" s="16"/>
     </row>
     <row r="46" spans="2:28" ht="66.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B46" s="161"/>
-      <c r="C46" s="162"/>
-      <c r="D46" s="224"/>
-      <c r="E46" s="162"/>
-      <c r="F46" s="225"/>
-      <c r="G46" s="160"/>
-      <c r="H46" s="159"/>
-      <c r="I46" s="104"/>
+      <c r="B46" s="223"/>
+      <c r="C46" s="207"/>
+      <c r="D46" s="206"/>
+      <c r="E46" s="207"/>
+      <c r="F46" s="209"/>
+      <c r="G46" s="208"/>
+      <c r="H46" s="222"/>
+      <c r="I46" s="139"/>
       <c r="J46" s="16"/>
       <c r="K46" s="16"/>
       <c r="L46" s="16"/>
@@ -5400,14 +5359,14 @@
       <c r="AA46" s="16"/>
     </row>
     <row r="47" spans="2:28" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B47" s="187"/>
-      <c r="C47" s="155"/>
-      <c r="D47" s="155"/>
-      <c r="E47" s="155"/>
-      <c r="F47" s="156"/>
-      <c r="G47" s="155"/>
-      <c r="H47" s="155"/>
-      <c r="I47" s="157"/>
+      <c r="B47" s="213"/>
+      <c r="C47" s="120"/>
+      <c r="D47" s="120"/>
+      <c r="E47" s="120"/>
+      <c r="F47" s="121"/>
+      <c r="G47" s="120"/>
+      <c r="H47" s="120"/>
+      <c r="I47" s="122"/>
       <c r="J47" s="18"/>
       <c r="K47" s="16"/>
       <c r="L47" s="16"/>
@@ -5428,14 +5387,14 @@
       <c r="AA47" s="16"/>
     </row>
     <row r="48" spans="2:28" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B48" s="187"/>
-      <c r="C48" s="155"/>
-      <c r="D48" s="155"/>
-      <c r="E48" s="155"/>
-      <c r="F48" s="156"/>
-      <c r="G48" s="155"/>
-      <c r="H48" s="155"/>
-      <c r="I48" s="157"/>
+      <c r="B48" s="213"/>
+      <c r="C48" s="120"/>
+      <c r="D48" s="120"/>
+      <c r="E48" s="120"/>
+      <c r="F48" s="121"/>
+      <c r="G48" s="120"/>
+      <c r="H48" s="120"/>
+      <c r="I48" s="122"/>
       <c r="J48" s="18"/>
       <c r="K48" s="16"/>
       <c r="L48" s="16"/>
@@ -5456,14 +5415,14 @@
       <c r="AA48" s="16"/>
     </row>
     <row r="49" spans="2:28" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B49" s="187"/>
-      <c r="C49" s="155"/>
-      <c r="D49" s="155"/>
-      <c r="E49" s="155"/>
-      <c r="F49" s="156"/>
-      <c r="G49" s="155"/>
-      <c r="H49" s="155"/>
-      <c r="I49" s="157"/>
+      <c r="B49" s="213"/>
+      <c r="C49" s="120"/>
+      <c r="D49" s="120"/>
+      <c r="E49" s="120"/>
+      <c r="F49" s="121"/>
+      <c r="G49" s="120"/>
+      <c r="H49" s="120"/>
+      <c r="I49" s="122"/>
       <c r="J49" s="18"/>
       <c r="K49" s="16"/>
       <c r="L49" s="16"/>
@@ -5484,14 +5443,14 @@
       <c r="AA49" s="16"/>
     </row>
     <row r="50" spans="2:28" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B50" s="187"/>
-      <c r="C50" s="155"/>
-      <c r="D50" s="155"/>
-      <c r="E50" s="155"/>
-      <c r="F50" s="156"/>
-      <c r="G50" s="155"/>
-      <c r="H50" s="155"/>
-      <c r="I50" s="157"/>
+      <c r="B50" s="213"/>
+      <c r="C50" s="120"/>
+      <c r="D50" s="120"/>
+      <c r="E50" s="120"/>
+      <c r="F50" s="121"/>
+      <c r="G50" s="120"/>
+      <c r="H50" s="120"/>
+      <c r="I50" s="122"/>
       <c r="J50" s="18"/>
       <c r="K50" s="16"/>
       <c r="L50" s="16"/>
@@ -5512,14 +5471,14 @@
       <c r="AA50" s="16"/>
     </row>
     <row r="51" spans="2:28" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B51" s="187"/>
-      <c r="C51" s="155"/>
-      <c r="D51" s="155"/>
-      <c r="E51" s="155"/>
-      <c r="F51" s="156"/>
-      <c r="G51" s="155"/>
-      <c r="H51" s="155"/>
-      <c r="I51" s="157"/>
+      <c r="B51" s="213"/>
+      <c r="C51" s="120"/>
+      <c r="D51" s="120"/>
+      <c r="E51" s="120"/>
+      <c r="F51" s="121"/>
+      <c r="G51" s="120"/>
+      <c r="H51" s="120"/>
+      <c r="I51" s="122"/>
       <c r="J51" s="18"/>
       <c r="K51" s="16"/>
       <c r="L51" s="16"/>
@@ -5540,14 +5499,14 @@
       <c r="AA51" s="16"/>
     </row>
     <row r="52" spans="2:28" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B52" s="187"/>
-      <c r="C52" s="155"/>
-      <c r="D52" s="155"/>
-      <c r="E52" s="155"/>
-      <c r="F52" s="156"/>
-      <c r="G52" s="155"/>
-      <c r="H52" s="155"/>
-      <c r="I52" s="157"/>
+      <c r="B52" s="213"/>
+      <c r="C52" s="120"/>
+      <c r="D52" s="120"/>
+      <c r="E52" s="120"/>
+      <c r="F52" s="121"/>
+      <c r="G52" s="120"/>
+      <c r="H52" s="120"/>
+      <c r="I52" s="122"/>
       <c r="J52" s="18"/>
       <c r="K52" s="16"/>
       <c r="L52" s="16"/>
@@ -5568,14 +5527,14 @@
       <c r="AA52" s="16"/>
     </row>
     <row r="53" spans="2:28" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B53" s="187"/>
-      <c r="C53" s="155"/>
-      <c r="D53" s="155"/>
-      <c r="E53" s="155"/>
-      <c r="F53" s="156"/>
-      <c r="G53" s="155"/>
-      <c r="H53" s="155"/>
-      <c r="I53" s="157"/>
+      <c r="B53" s="213"/>
+      <c r="C53" s="120"/>
+      <c r="D53" s="120"/>
+      <c r="E53" s="120"/>
+      <c r="F53" s="121"/>
+      <c r="G53" s="120"/>
+      <c r="H53" s="120"/>
+      <c r="I53" s="122"/>
       <c r="J53" s="18"/>
       <c r="K53" s="16"/>
       <c r="L53" s="16"/>
@@ -5596,14 +5555,14 @@
       <c r="AA53" s="16"/>
     </row>
     <row r="54" spans="2:28" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B54" s="187"/>
-      <c r="C54" s="155"/>
-      <c r="D54" s="155"/>
-      <c r="E54" s="155"/>
-      <c r="F54" s="156"/>
-      <c r="G54" s="155"/>
-      <c r="H54" s="155"/>
-      <c r="I54" s="157"/>
+      <c r="B54" s="213"/>
+      <c r="C54" s="120"/>
+      <c r="D54" s="120"/>
+      <c r="E54" s="120"/>
+      <c r="F54" s="121"/>
+      <c r="G54" s="120"/>
+      <c r="H54" s="120"/>
+      <c r="I54" s="122"/>
       <c r="J54" s="18"/>
       <c r="K54" s="16"/>
       <c r="L54" s="16"/>
@@ -5624,14 +5583,14 @@
       <c r="AA54" s="16"/>
     </row>
     <row r="55" spans="2:28" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B55" s="187"/>
-      <c r="C55" s="155"/>
-      <c r="D55" s="155"/>
-      <c r="E55" s="155"/>
-      <c r="F55" s="156"/>
-      <c r="G55" s="155"/>
-      <c r="H55" s="155"/>
-      <c r="I55" s="157"/>
+      <c r="B55" s="213"/>
+      <c r="C55" s="120"/>
+      <c r="D55" s="120"/>
+      <c r="E55" s="120"/>
+      <c r="F55" s="121"/>
+      <c r="G55" s="120"/>
+      <c r="H55" s="120"/>
+      <c r="I55" s="122"/>
       <c r="J55" s="18"/>
       <c r="K55" s="16"/>
       <c r="L55" s="16"/>
@@ -5652,14 +5611,14 @@
       <c r="AA55" s="16"/>
     </row>
     <row r="56" spans="2:28" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B56" s="93"/>
-      <c r="C56" s="94"/>
-      <c r="D56" s="94"/>
-      <c r="E56" s="94"/>
-      <c r="F56" s="250"/>
-      <c r="G56" s="94"/>
-      <c r="H56" s="94"/>
-      <c r="I56" s="188"/>
+      <c r="B56" s="157"/>
+      <c r="C56" s="158"/>
+      <c r="D56" s="158"/>
+      <c r="E56" s="158"/>
+      <c r="F56" s="229"/>
+      <c r="G56" s="158"/>
+      <c r="H56" s="158"/>
+      <c r="I56" s="214"/>
       <c r="J56" s="18"/>
       <c r="K56" s="16"/>
       <c r="L56" s="16"/>
@@ -5685,8 +5644,8 @@
       <c r="D57" s="18"/>
       <c r="E57" s="23"/>
       <c r="F57" s="23"/>
-      <c r="G57" s="219"/>
-      <c r="H57" s="219"/>
+      <c r="G57" s="201"/>
+      <c r="H57" s="201"/>
       <c r="I57" s="18"/>
       <c r="J57" s="18"/>
       <c r="K57" s="16"/>
@@ -5708,16 +5667,16 @@
       <c r="AA57" s="16"/>
     </row>
     <row r="58" spans="2:28" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B58" s="226" t="s">
+      <c r="B58" s="210" t="s">
         <v>54</v>
       </c>
-      <c r="C58" s="227"/>
-      <c r="D58" s="227"/>
-      <c r="E58" s="227"/>
-      <c r="F58" s="227"/>
-      <c r="G58" s="227"/>
-      <c r="H58" s="227"/>
-      <c r="I58" s="228"/>
+      <c r="C58" s="211"/>
+      <c r="D58" s="211"/>
+      <c r="E58" s="211"/>
+      <c r="F58" s="211"/>
+      <c r="G58" s="211"/>
+      <c r="H58" s="211"/>
+      <c r="I58" s="212"/>
       <c r="J58" s="18"/>
       <c r="K58" s="16"/>
       <c r="L58" s="16"/>
@@ -5738,16 +5697,16 @@
       <c r="AA58" s="16"/>
     </row>
     <row r="59" spans="2:28" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B59" s="70" t="s">
+      <c r="B59" s="81" t="s">
         <v>55</v>
       </c>
-      <c r="C59" s="71"/>
-      <c r="D59" s="71"/>
-      <c r="E59" s="71"/>
-      <c r="F59" s="71"/>
-      <c r="G59" s="71"/>
-      <c r="H59" s="71"/>
-      <c r="I59" s="72"/>
+      <c r="C59" s="82"/>
+      <c r="D59" s="82"/>
+      <c r="E59" s="82"/>
+      <c r="F59" s="82"/>
+      <c r="G59" s="82"/>
+      <c r="H59" s="82"/>
+      <c r="I59" s="83"/>
       <c r="J59" s="19"/>
       <c r="K59" s="19"/>
       <c r="L59" s="19"/>
@@ -5768,16 +5727,16 @@
       <c r="AA59" s="19"/>
     </row>
     <row r="60" spans="2:28" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B60" s="226" t="s">
+      <c r="B60" s="210" t="s">
         <v>56</v>
       </c>
-      <c r="C60" s="227"/>
-      <c r="D60" s="227"/>
-      <c r="E60" s="227"/>
-      <c r="F60" s="227"/>
-      <c r="G60" s="227"/>
-      <c r="H60" s="227"/>
-      <c r="I60" s="228"/>
+      <c r="C60" s="211"/>
+      <c r="D60" s="211"/>
+      <c r="E60" s="211"/>
+      <c r="F60" s="211"/>
+      <c r="G60" s="211"/>
+      <c r="H60" s="211"/>
+      <c r="I60" s="212"/>
       <c r="J60" s="19"/>
       <c r="K60" s="19"/>
       <c r="L60" s="19"/>
@@ -5798,16 +5757,16 @@
       <c r="AA60" s="19"/>
     </row>
     <row r="61" spans="2:28" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B61" s="239" t="s">
+      <c r="B61" s="237" t="s">
         <v>57</v>
       </c>
-      <c r="C61" s="240"/>
-      <c r="D61" s="240"/>
-      <c r="E61" s="240"/>
-      <c r="F61" s="240"/>
-      <c r="G61" s="240"/>
-      <c r="H61" s="240"/>
-      <c r="I61" s="241"/>
+      <c r="C61" s="238"/>
+      <c r="D61" s="238"/>
+      <c r="E61" s="238"/>
+      <c r="F61" s="238"/>
+      <c r="G61" s="238"/>
+      <c r="H61" s="238"/>
+      <c r="I61" s="239"/>
       <c r="J61" s="22"/>
       <c r="K61" s="22"/>
       <c r="L61" s="22"/>
@@ -5828,14 +5787,14 @@
       <c r="AA61" s="22"/>
     </row>
     <row r="62" spans="2:28" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B62" s="242"/>
-      <c r="C62" s="243"/>
-      <c r="D62" s="243"/>
-      <c r="E62" s="243"/>
-      <c r="F62" s="243"/>
-      <c r="G62" s="243"/>
-      <c r="H62" s="243"/>
-      <c r="I62" s="244"/>
+      <c r="B62" s="240"/>
+      <c r="C62" s="241"/>
+      <c r="D62" s="241"/>
+      <c r="E62" s="241"/>
+      <c r="F62" s="241"/>
+      <c r="G62" s="241"/>
+      <c r="H62" s="241"/>
+      <c r="I62" s="242"/>
       <c r="J62" s="22"/>
       <c r="K62" s="22"/>
       <c r="L62" s="22"/>
@@ -5856,16 +5815,16 @@
       <c r="AA62" s="22"/>
     </row>
     <row r="63" spans="2:28" s="46" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B63" s="242" t="s">
+      <c r="B63" s="240" t="s">
         <v>58</v>
       </c>
-      <c r="C63" s="243"/>
-      <c r="D63" s="243"/>
-      <c r="E63" s="243"/>
-      <c r="F63" s="243"/>
-      <c r="G63" s="243"/>
-      <c r="H63" s="243"/>
-      <c r="I63" s="244"/>
+      <c r="C63" s="241"/>
+      <c r="D63" s="241"/>
+      <c r="E63" s="241"/>
+      <c r="F63" s="241"/>
+      <c r="G63" s="241"/>
+      <c r="H63" s="241"/>
+      <c r="I63" s="242"/>
       <c r="J63" s="44"/>
       <c r="K63" s="44"/>
       <c r="L63" s="44"/>
@@ -5887,16 +5846,16 @@
       <c r="AB63" s="45"/>
     </row>
     <row r="64" spans="2:28" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B64" s="245" t="s">
+      <c r="B64" s="243" t="s">
         <v>59</v>
       </c>
-      <c r="C64" s="246"/>
-      <c r="D64" s="246"/>
-      <c r="E64" s="246"/>
-      <c r="F64" s="246"/>
-      <c r="G64" s="246"/>
-      <c r="H64" s="246"/>
-      <c r="I64" s="247"/>
+      <c r="C64" s="244"/>
+      <c r="D64" s="244"/>
+      <c r="E64" s="244"/>
+      <c r="F64" s="244"/>
+      <c r="G64" s="244"/>
+      <c r="H64" s="244"/>
+      <c r="I64" s="245"/>
       <c r="J64" s="22"/>
       <c r="K64" s="22"/>
       <c r="L64" s="22"/>
@@ -5920,19 +5879,19 @@
       <c r="B65" s="50" t="s">
         <v>60</v>
       </c>
-      <c r="C65" s="86" t="s">
+      <c r="C65" s="129" t="s">
         <v>61</v>
       </c>
-      <c r="D65" s="86"/>
-      <c r="E65" s="86" t="s">
+      <c r="D65" s="129"/>
+      <c r="E65" s="129" t="s">
         <v>62</v>
       </c>
-      <c r="F65" s="86"/>
-      <c r="G65" s="82"/>
-      <c r="H65" s="86" t="s">
+      <c r="F65" s="129"/>
+      <c r="G65" s="93"/>
+      <c r="H65" s="129" t="s">
         <v>63</v>
       </c>
-      <c r="I65" s="84"/>
+      <c r="I65" s="95"/>
       <c r="J65" s="16"/>
       <c r="K65" s="16"/>
       <c r="L65" s="16"/>
@@ -5955,13 +5914,13 @@
     </row>
     <row r="66" spans="2:28" ht="32.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B66" s="51"/>
-      <c r="C66" s="248"/>
-      <c r="D66" s="248"/>
-      <c r="E66" s="87"/>
-      <c r="F66" s="87"/>
-      <c r="G66" s="83"/>
-      <c r="H66" s="87"/>
-      <c r="I66" s="85"/>
+      <c r="C66" s="247"/>
+      <c r="D66" s="247"/>
+      <c r="E66" s="130"/>
+      <c r="F66" s="130"/>
+      <c r="G66" s="94"/>
+      <c r="H66" s="130"/>
+      <c r="I66" s="96"/>
       <c r="J66" s="16"/>
       <c r="K66" s="16"/>
       <c r="L66" s="16"/>
@@ -5988,8 +5947,8 @@
       <c r="D67" s="17"/>
       <c r="E67" s="34"/>
       <c r="F67" s="34"/>
-      <c r="G67" s="229"/>
-      <c r="H67" s="229"/>
+      <c r="G67" s="246"/>
+      <c r="H67" s="246"/>
       <c r="I67" s="17"/>
       <c r="J67" s="16"/>
       <c r="K67" s="16"/>
@@ -6012,16 +5971,16 @@
       <c r="AB67" s="16"/>
     </row>
     <row r="68" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B68" s="238" t="s">
+      <c r="B68" s="236" t="s">
         <v>64</v>
       </c>
-      <c r="C68" s="238"/>
-      <c r="D68" s="238"/>
-      <c r="E68" s="238"/>
-      <c r="F68" s="238"/>
-      <c r="G68" s="238"/>
-      <c r="H68" s="238"/>
-      <c r="I68" s="238"/>
+      <c r="C68" s="236"/>
+      <c r="D68" s="236"/>
+      <c r="E68" s="236"/>
+      <c r="F68" s="236"/>
+      <c r="G68" s="236"/>
+      <c r="H68" s="236"/>
+      <c r="I68" s="236"/>
       <c r="J68" s="16"/>
       <c r="K68" s="16"/>
       <c r="L68" s="16"/>
@@ -6048,8 +6007,8 @@
       <c r="D69" s="15"/>
       <c r="E69" s="35"/>
       <c r="F69" s="35"/>
-      <c r="G69" s="76"/>
-      <c r="H69" s="76"/>
+      <c r="G69" s="87"/>
+      <c r="H69" s="87"/>
       <c r="I69" s="15"/>
       <c r="J69" s="16"/>
       <c r="K69" s="16"/>
@@ -6072,13 +6031,13 @@
       <c r="AB69" s="16"/>
     </row>
     <row r="70" spans="2:28" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B70" s="76"/>
-      <c r="C70" s="76"/>
-      <c r="D70" s="76"/>
-      <c r="E70" s="76"/>
+      <c r="B70" s="87"/>
+      <c r="C70" s="87"/>
+      <c r="D70" s="87"/>
+      <c r="E70" s="87"/>
       <c r="F70" s="35"/>
-      <c r="G70" s="76"/>
-      <c r="H70" s="76"/>
+      <c r="G70" s="87"/>
+      <c r="H70" s="87"/>
       <c r="I70" s="15"/>
       <c r="J70" s="16"/>
       <c r="K70" s="16"/>
@@ -6101,10 +6060,10 @@
       <c r="AB70" s="16"/>
     </row>
     <row r="71" spans="2:28" ht="36" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B71" s="77"/>
-      <c r="C71" s="77"/>
-      <c r="D71" s="77"/>
-      <c r="E71" s="77"/>
+      <c r="B71" s="88"/>
+      <c r="C71" s="88"/>
+      <c r="D71" s="88"/>
+      <c r="E71" s="88"/>
       <c r="F71" s="26"/>
       <c r="H71" s="57"/>
       <c r="I71" s="16"/>
@@ -6129,12 +6088,12 @@
       <c r="AB71" s="16"/>
     </row>
     <row r="72" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B72" s="231" t="s">
+      <c r="B72" s="228" t="s">
         <v>65</v>
       </c>
-      <c r="C72" s="231"/>
-      <c r="D72" s="231"/>
-      <c r="E72" s="231"/>
+      <c r="C72" s="228"/>
+      <c r="D72" s="228"/>
+      <c r="E72" s="228"/>
       <c r="F72" s="17"/>
       <c r="H72" s="17" t="s">
         <v>66</v>
@@ -6166,8 +6125,8 @@
       <c r="D73" s="16"/>
       <c r="E73" s="26"/>
       <c r="F73" s="26"/>
-      <c r="G73" s="69"/>
-      <c r="H73" s="113"/>
+      <c r="G73" s="80"/>
+      <c r="H73" s="97"/>
       <c r="I73" s="16"/>
       <c r="J73" s="16"/>
       <c r="K73" s="16"/>
@@ -6190,13 +6149,13 @@
       <c r="AB73" s="16"/>
     </row>
     <row r="74" spans="2:28" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B74" s="80"/>
-      <c r="C74" s="80"/>
-      <c r="D74" s="80"/>
-      <c r="E74" s="80"/>
+      <c r="B74" s="91"/>
+      <c r="C74" s="91"/>
+      <c r="D74" s="91"/>
+      <c r="E74" s="91"/>
       <c r="F74" s="26"/>
-      <c r="H74" s="78"/>
-      <c r="I74" s="78"/>
+      <c r="H74" s="89"/>
+      <c r="I74" s="89"/>
       <c r="J74" s="16"/>
       <c r="K74" s="16"/>
       <c r="L74" s="16"/>
@@ -6218,13 +6177,13 @@
       <c r="AB74" s="16"/>
     </row>
     <row r="75" spans="2:28" ht="38.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B75" s="81"/>
-      <c r="C75" s="81"/>
-      <c r="D75" s="81"/>
-      <c r="E75" s="81"/>
+      <c r="B75" s="92"/>
+      <c r="C75" s="92"/>
+      <c r="D75" s="92"/>
+      <c r="E75" s="92"/>
       <c r="F75" s="26"/>
-      <c r="H75" s="79"/>
-      <c r="I75" s="79"/>
+      <c r="H75" s="90"/>
+      <c r="I75" s="90"/>
       <c r="J75" s="16"/>
       <c r="K75" s="16"/>
       <c r="L75" s="16"/>
@@ -6253,10 +6212,10 @@
       <c r="D76" s="24"/>
       <c r="E76" s="26"/>
       <c r="F76" s="26"/>
-      <c r="H76" s="231" t="s">
+      <c r="H76" s="228" t="s">
         <v>68</v>
       </c>
-      <c r="I76" s="231"/>
+      <c r="I76" s="228"/>
       <c r="J76" s="16"/>
       <c r="K76" s="16"/>
       <c r="L76" s="16"/>
@@ -6283,8 +6242,8 @@
       <c r="D77" s="24"/>
       <c r="E77" s="26"/>
       <c r="F77" s="26"/>
-      <c r="G77" s="69"/>
-      <c r="H77" s="229"/>
+      <c r="G77" s="80"/>
+      <c r="H77" s="246"/>
       <c r="I77" s="17"/>
       <c r="J77" s="16"/>
       <c r="K77" s="16"/>
@@ -6307,16 +6266,16 @@
       <c r="AB77" s="16"/>
     </row>
     <row r="78" spans="2:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B78" s="249" t="s">
+      <c r="B78" s="248" t="s">
         <v>69</v>
       </c>
-      <c r="C78" s="249"/>
-      <c r="D78" s="249"/>
-      <c r="E78" s="249"/>
-      <c r="F78" s="249"/>
-      <c r="G78" s="249"/>
-      <c r="H78" s="249"/>
-      <c r="I78" s="249"/>
+      <c r="C78" s="248"/>
+      <c r="D78" s="248"/>
+      <c r="E78" s="248"/>
+      <c r="F78" s="248"/>
+      <c r="G78" s="248"/>
+      <c r="H78" s="248"/>
+      <c r="I78" s="248"/>
       <c r="J78" s="16"/>
       <c r="K78" s="16"/>
       <c r="L78" s="16"/>
@@ -6338,14 +6297,14 @@
       <c r="AB78" s="16"/>
     </row>
     <row r="79" spans="2:28" x14ac:dyDescent="0.25">
-      <c r="B79" s="249"/>
-      <c r="C79" s="249"/>
-      <c r="D79" s="249"/>
-      <c r="E79" s="249"/>
-      <c r="F79" s="249"/>
-      <c r="G79" s="249"/>
-      <c r="H79" s="249"/>
-      <c r="I79" s="249"/>
+      <c r="B79" s="248"/>
+      <c r="C79" s="248"/>
+      <c r="D79" s="248"/>
+      <c r="E79" s="248"/>
+      <c r="F79" s="248"/>
+      <c r="G79" s="248"/>
+      <c r="H79" s="248"/>
+      <c r="I79" s="248"/>
       <c r="J79" s="16"/>
       <c r="K79" s="16"/>
       <c r="L79" s="16"/>
@@ -6372,8 +6331,8 @@
       <c r="D80" s="48"/>
       <c r="E80" s="48"/>
       <c r="F80" s="48"/>
-      <c r="G80" s="230"/>
-      <c r="H80" s="230"/>
+      <c r="G80" s="249"/>
+      <c r="H80" s="249"/>
       <c r="I80" s="48"/>
       <c r="J80" s="16"/>
       <c r="K80" s="16"/>
@@ -6396,16 +6355,16 @@
       <c r="AB80" s="16"/>
     </row>
     <row r="81" spans="2:28" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B81" s="232" t="s">
+      <c r="B81" s="230" t="s">
         <v>70</v>
       </c>
-      <c r="C81" s="233"/>
-      <c r="D81" s="233"/>
-      <c r="E81" s="233"/>
-      <c r="F81" s="233"/>
-      <c r="G81" s="233"/>
-      <c r="H81" s="233"/>
-      <c r="I81" s="234"/>
+      <c r="C81" s="231"/>
+      <c r="D81" s="231"/>
+      <c r="E81" s="231"/>
+      <c r="F81" s="231"/>
+      <c r="G81" s="231"/>
+      <c r="H81" s="231"/>
+      <c r="I81" s="232"/>
       <c r="J81" s="8"/>
       <c r="K81" s="7"/>
       <c r="L81" s="7"/>
@@ -6427,16 +6386,16 @@
       <c r="AB81" s="7"/>
     </row>
     <row r="82" spans="2:28" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B82" s="235" t="s">
+      <c r="B82" s="233" t="s">
         <v>71</v>
       </c>
-      <c r="C82" s="236"/>
-      <c r="D82" s="236"/>
-      <c r="E82" s="236"/>
-      <c r="F82" s="236"/>
-      <c r="G82" s="236"/>
-      <c r="H82" s="236"/>
-      <c r="I82" s="237"/>
+      <c r="C82" s="234"/>
+      <c r="D82" s="234"/>
+      <c r="E82" s="234"/>
+      <c r="F82" s="234"/>
+      <c r="G82" s="234"/>
+      <c r="H82" s="234"/>
+      <c r="I82" s="235"/>
       <c r="J82" s="8"/>
       <c r="K82" s="25"/>
       <c r="L82" s="7"/>
@@ -6457,19 +6416,19 @@
       <c r="AA82" s="7"/>
       <c r="AB82" s="7"/>
     </row>
-    <row r="83" spans="2:28" s="8" customFormat="1" ht="207.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B83" s="73"/>
-      <c r="C83" s="74"/>
-      <c r="D83" s="74"/>
-      <c r="E83" s="74"/>
-      <c r="F83" s="74"/>
-      <c r="G83" s="74"/>
-      <c r="H83" s="74"/>
-      <c r="I83" s="75"/>
+    <row r="83" spans="2:28" s="8" customFormat="1" ht="249" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B83" s="84"/>
+      <c r="C83" s="85"/>
+      <c r="D83" s="85"/>
+      <c r="E83" s="85"/>
+      <c r="F83" s="85"/>
+      <c r="G83" s="85"/>
+      <c r="H83" s="85"/>
+      <c r="I83" s="86"/>
     </row>
     <row r="84" spans="2:28" hidden="1" x14ac:dyDescent="0.25">
-      <c r="G84" s="69"/>
-      <c r="H84" s="69"/>
+      <c r="G84" s="80"/>
+      <c r="H84" s="80"/>
       <c r="J84" s="8"/>
       <c r="K84" s="7"/>
       <c r="L84" s="7"/>
@@ -6491,120 +6450,120 @@
       <c r="AB84" s="7"/>
     </row>
     <row r="85" spans="2:28" hidden="1" x14ac:dyDescent="0.25">
-      <c r="G85" s="69"/>
-      <c r="H85" s="69"/>
+      <c r="G85" s="80"/>
+      <c r="H85" s="80"/>
     </row>
     <row r="86" spans="2:28" hidden="1" x14ac:dyDescent="0.25">
-      <c r="G86" s="69"/>
-      <c r="H86" s="69"/>
+      <c r="G86" s="80"/>
+      <c r="H86" s="80"/>
     </row>
     <row r="87" spans="2:28" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G87" s="69"/>
-      <c r="H87" s="69"/>
+      <c r="G87" s="80"/>
+      <c r="H87" s="80"/>
     </row>
     <row r="88" spans="2:28" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G88" s="69"/>
-      <c r="H88" s="69"/>
+      <c r="G88" s="80"/>
+      <c r="H88" s="80"/>
     </row>
     <row r="89" spans="2:28" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G89" s="69"/>
-      <c r="H89" s="69"/>
+      <c r="G89" s="80"/>
+      <c r="H89" s="80"/>
     </row>
     <row r="90" spans="2:28" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G90" s="69"/>
-      <c r="H90" s="69"/>
+      <c r="G90" s="80"/>
+      <c r="H90" s="80"/>
     </row>
     <row r="91" spans="2:28" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G91" s="69"/>
-      <c r="H91" s="69"/>
+      <c r="G91" s="80"/>
+      <c r="H91" s="80"/>
     </row>
     <row r="92" spans="2:28" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G92" s="69"/>
-      <c r="H92" s="69"/>
+      <c r="G92" s="80"/>
+      <c r="H92" s="80"/>
     </row>
     <row r="93" spans="2:28" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G93" s="69"/>
-      <c r="H93" s="69"/>
+      <c r="G93" s="80"/>
+      <c r="H93" s="80"/>
     </row>
     <row r="94" spans="2:28" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G94" s="69"/>
-      <c r="H94" s="69"/>
+      <c r="G94" s="80"/>
+      <c r="H94" s="80"/>
     </row>
     <row r="95" spans="2:28" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G95" s="69"/>
-      <c r="H95" s="69"/>
+      <c r="G95" s="80"/>
+      <c r="H95" s="80"/>
     </row>
     <row r="96" spans="2:28" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G96" s="69"/>
-      <c r="H96" s="69"/>
+      <c r="G96" s="80"/>
+      <c r="H96" s="80"/>
     </row>
     <row r="97" spans="7:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G97" s="69"/>
-      <c r="H97" s="69"/>
+      <c r="G97" s="80"/>
+      <c r="H97" s="80"/>
     </row>
     <row r="98" spans="7:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G98" s="69"/>
-      <c r="H98" s="69"/>
+      <c r="G98" s="80"/>
+      <c r="H98" s="80"/>
     </row>
     <row r="99" spans="7:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G99" s="69"/>
-      <c r="H99" s="69"/>
+      <c r="G99" s="80"/>
+      <c r="H99" s="80"/>
     </row>
     <row r="100" spans="7:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G100" s="69"/>
-      <c r="H100" s="69"/>
+      <c r="G100" s="80"/>
+      <c r="H100" s="80"/>
     </row>
     <row r="101" spans="7:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G101" s="69"/>
-      <c r="H101" s="69"/>
+      <c r="G101" s="80"/>
+      <c r="H101" s="80"/>
     </row>
     <row r="102" spans="7:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G102" s="69"/>
-      <c r="H102" s="69"/>
+      <c r="G102" s="80"/>
+      <c r="H102" s="80"/>
     </row>
     <row r="103" spans="7:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G103" s="69"/>
-      <c r="H103" s="69"/>
+      <c r="G103" s="80"/>
+      <c r="H103" s="80"/>
     </row>
     <row r="104" spans="7:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G104" s="69"/>
-      <c r="H104" s="69"/>
+      <c r="G104" s="80"/>
+      <c r="H104" s="80"/>
     </row>
     <row r="105" spans="7:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G105" s="69"/>
-      <c r="H105" s="69"/>
+      <c r="G105" s="80"/>
+      <c r="H105" s="80"/>
     </row>
     <row r="106" spans="7:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G106" s="69"/>
-      <c r="H106" s="69"/>
+      <c r="G106" s="80"/>
+      <c r="H106" s="80"/>
     </row>
     <row r="107" spans="7:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G107" s="69"/>
-      <c r="H107" s="69"/>
+      <c r="G107" s="80"/>
+      <c r="H107" s="80"/>
     </row>
     <row r="108" spans="7:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G108" s="69"/>
-      <c r="H108" s="69"/>
+      <c r="G108" s="80"/>
+      <c r="H108" s="80"/>
     </row>
     <row r="109" spans="7:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G109" s="69"/>
-      <c r="H109" s="69"/>
+      <c r="G109" s="80"/>
+      <c r="H109" s="80"/>
     </row>
     <row r="110" spans="7:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G110" s="69"/>
-      <c r="H110" s="69"/>
+      <c r="G110" s="80"/>
+      <c r="H110" s="80"/>
     </row>
     <row r="111" spans="7:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G111" s="69"/>
-      <c r="H111" s="69"/>
+      <c r="G111" s="80"/>
+      <c r="H111" s="80"/>
     </row>
     <row r="112" spans="7:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G112" s="69"/>
-      <c r="H112" s="69"/>
+      <c r="G112" s="80"/>
+      <c r="H112" s="80"/>
     </row>
     <row r="113" spans="7:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G113" s="69"/>
-      <c r="H113" s="69"/>
+      <c r="G113" s="80"/>
+      <c r="H113" s="80"/>
     </row>
   </sheetData>
   <mergeCells count="171">
@@ -6625,6 +6584,13 @@
     <mergeCell ref="B78:I79"/>
     <mergeCell ref="G77:H77"/>
     <mergeCell ref="G80:H80"/>
+    <mergeCell ref="I55:I56"/>
+    <mergeCell ref="H76:I76"/>
+    <mergeCell ref="B55:C56"/>
+    <mergeCell ref="D55:E56"/>
+    <mergeCell ref="F55:F56"/>
+    <mergeCell ref="G55:G56"/>
+    <mergeCell ref="H55:H56"/>
     <mergeCell ref="D47:E48"/>
     <mergeCell ref="B47:C48"/>
     <mergeCell ref="F47:F48"/>
@@ -6637,19 +6603,6 @@
     <mergeCell ref="G49:G50"/>
     <mergeCell ref="H49:H50"/>
     <mergeCell ref="I49:I50"/>
-    <mergeCell ref="B51:C52"/>
-    <mergeCell ref="D51:E52"/>
-    <mergeCell ref="F51:F52"/>
-    <mergeCell ref="I55:I56"/>
-    <mergeCell ref="H76:I76"/>
-    <mergeCell ref="B55:C56"/>
-    <mergeCell ref="D55:E56"/>
-    <mergeCell ref="F55:F56"/>
-    <mergeCell ref="G55:G56"/>
-    <mergeCell ref="H55:H56"/>
-    <mergeCell ref="B11:D11"/>
-    <mergeCell ref="G9:H9"/>
-    <mergeCell ref="G12:H12"/>
     <mergeCell ref="H16:I16"/>
     <mergeCell ref="D45:E46"/>
     <mergeCell ref="F45:F46"/>
@@ -6661,6 +6614,19 @@
     <mergeCell ref="E28:F28"/>
     <mergeCell ref="E29:F29"/>
     <mergeCell ref="B32:F32"/>
+    <mergeCell ref="B16:D16"/>
+    <mergeCell ref="E16:G16"/>
+    <mergeCell ref="H51:H52"/>
+    <mergeCell ref="H45:H46"/>
+    <mergeCell ref="G45:G46"/>
+    <mergeCell ref="B45:C46"/>
+    <mergeCell ref="B17:D17"/>
+    <mergeCell ref="H20:I20"/>
+    <mergeCell ref="B20:D20"/>
+    <mergeCell ref="B21:D21"/>
+    <mergeCell ref="B51:C52"/>
+    <mergeCell ref="D51:E52"/>
+    <mergeCell ref="F51:F52"/>
     <mergeCell ref="B3:I3"/>
     <mergeCell ref="B5:I5"/>
     <mergeCell ref="B4:I4"/>
@@ -6674,12 +6640,13 @@
     <mergeCell ref="E8:F8"/>
     <mergeCell ref="F14:G14"/>
     <mergeCell ref="F15:G15"/>
-    <mergeCell ref="B16:D16"/>
-    <mergeCell ref="E16:G16"/>
     <mergeCell ref="B13:I13"/>
     <mergeCell ref="E10:I10"/>
     <mergeCell ref="E11:I11"/>
     <mergeCell ref="B10:D10"/>
+    <mergeCell ref="B11:D11"/>
+    <mergeCell ref="G9:H9"/>
+    <mergeCell ref="G12:H12"/>
     <mergeCell ref="G96:H96"/>
     <mergeCell ref="G97:H97"/>
     <mergeCell ref="G98:H98"/>
@@ -6690,14 +6657,6 @@
     <mergeCell ref="G93:H93"/>
     <mergeCell ref="G94:H94"/>
     <mergeCell ref="G95:H95"/>
-    <mergeCell ref="H51:H52"/>
-    <mergeCell ref="H45:H46"/>
-    <mergeCell ref="G45:G46"/>
-    <mergeCell ref="B45:C46"/>
-    <mergeCell ref="B17:D17"/>
-    <mergeCell ref="H20:I20"/>
-    <mergeCell ref="B20:D20"/>
-    <mergeCell ref="B21:D21"/>
     <mergeCell ref="E18:G18"/>
     <mergeCell ref="H18:I18"/>
     <mergeCell ref="E19:G19"/>
@@ -6719,6 +6678,18 @@
     <mergeCell ref="H41:I42"/>
     <mergeCell ref="B35:I35"/>
     <mergeCell ref="H39:I40"/>
+    <mergeCell ref="H36:I36"/>
+    <mergeCell ref="C36:F36"/>
+    <mergeCell ref="G30:H30"/>
+    <mergeCell ref="G34:H34"/>
+    <mergeCell ref="G22:H22"/>
+    <mergeCell ref="H24:I24"/>
+    <mergeCell ref="H25:I25"/>
+    <mergeCell ref="B28:D28"/>
+    <mergeCell ref="B29:D29"/>
+    <mergeCell ref="H28:I28"/>
+    <mergeCell ref="B27:I27"/>
+    <mergeCell ref="B25:E25"/>
     <mergeCell ref="G111:H111"/>
     <mergeCell ref="G84:H84"/>
     <mergeCell ref="G85:H85"/>
@@ -6730,27 +6701,19 @@
     <mergeCell ref="C41:F42"/>
     <mergeCell ref="B41:B42"/>
     <mergeCell ref="G86:H86"/>
-    <mergeCell ref="H36:I36"/>
-    <mergeCell ref="C36:F36"/>
     <mergeCell ref="D53:E54"/>
     <mergeCell ref="F53:F54"/>
     <mergeCell ref="G53:G54"/>
     <mergeCell ref="H53:H54"/>
     <mergeCell ref="I53:I54"/>
     <mergeCell ref="G51:G52"/>
-    <mergeCell ref="G30:H30"/>
-    <mergeCell ref="G34:H34"/>
-    <mergeCell ref="G22:H22"/>
-    <mergeCell ref="H24:I24"/>
-    <mergeCell ref="H25:I25"/>
-    <mergeCell ref="B28:D28"/>
-    <mergeCell ref="B29:D29"/>
-    <mergeCell ref="H28:I28"/>
     <mergeCell ref="H37:I38"/>
     <mergeCell ref="B37:B40"/>
     <mergeCell ref="G37:G38"/>
-    <mergeCell ref="B27:I27"/>
-    <mergeCell ref="B25:E25"/>
+    <mergeCell ref="G89:H89"/>
+    <mergeCell ref="G90:H90"/>
+    <mergeCell ref="E65:F66"/>
+    <mergeCell ref="G105:H105"/>
     <mergeCell ref="B31:I31"/>
     <mergeCell ref="B33:F33"/>
     <mergeCell ref="G32:I32"/>
@@ -6775,18 +6738,14 @@
     <mergeCell ref="I65:I66"/>
     <mergeCell ref="G87:H87"/>
     <mergeCell ref="G88:H88"/>
-    <mergeCell ref="G89:H89"/>
-    <mergeCell ref="G90:H90"/>
-    <mergeCell ref="E65:F66"/>
-    <mergeCell ref="G105:H105"/>
   </mergeCells>
-  <conditionalFormatting sqref="B11:I11 B15:I15 B17:I17 B19:I19 B21:I21 B25:I25 B29:I29 C37:F42 H37:I42 B70:E71 B74:E75 H74:I75 B83:I83">
+  <conditionalFormatting sqref="B11:I11 B15:I15 B17:I17 B19:I19 B21:I21 B25:I25 B29:I29 C37:F42 H37:I42 B70:E71 H74:I75 B83:I83">
     <cfRule type="containsBlanks" dxfId="2" priority="4">
       <formula>LEN(TRIM(B11))=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B47:I56">
-    <cfRule type="containsBlanks" dxfId="1" priority="1">
+    <cfRule type="containsBlanks" dxfId="1" priority="6">
       <formula>LEN(TRIM(B47))=0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6869,24 +6828,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="60" t="s">
+      <c r="A1" s="58" t="s">
         <v>106</v>
       </c>
-      <c r="B1" s="61" t="s">
+      <c r="B1" s="59" t="s">
         <v>107</v>
       </c>
-      <c r="C1" s="62" t="s">
+      <c r="C1" s="60" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="39" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="63" t="s">
+      <c r="A2" s="61" t="s">
         <v>109</v>
       </c>
-      <c r="B2" s="64" t="s">
+      <c r="B2" s="62" t="s">
         <v>110</v>
       </c>
-      <c r="C2" s="67" t="s">
+      <c r="C2" s="65" t="s">
         <v>123</v>
       </c>
       <c r="E2" t="str" cm="1">
@@ -6919,13 +6878,13 @@
       </c>
     </row>
     <row r="3" spans="1:11" ht="39" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="63" t="s">
+      <c r="A3" s="61" t="s">
         <v>109</v>
       </c>
-      <c r="B3" s="64" t="s">
+      <c r="B3" s="62" t="s">
         <v>110</v>
       </c>
-      <c r="C3" s="67" t="s">
+      <c r="C3" s="65" t="s">
         <v>124</v>
       </c>
       <c r="E3" t="str">
@@ -6933,398 +6892,398 @@
       </c>
     </row>
     <row r="4" spans="1:11" ht="39" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="63" t="s">
+      <c r="A4" s="61" t="s">
         <v>109</v>
       </c>
-      <c r="B4" s="64" t="s">
+      <c r="B4" s="62" t="s">
         <v>110</v>
       </c>
-      <c r="C4" s="67" t="s">
+      <c r="C4" s="65" t="s">
         <v>125</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="39" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="63" t="s">
+      <c r="A5" s="61" t="s">
         <v>109</v>
       </c>
-      <c r="B5" s="64" t="s">
+      <c r="B5" s="62" t="s">
         <v>110</v>
       </c>
-      <c r="C5" s="67" t="s">
+      <c r="C5" s="65" t="s">
         <v>126</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="39" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="63" t="s">
+      <c r="A6" s="61" t="s">
         <v>109</v>
       </c>
-      <c r="B6" s="64" t="s">
+      <c r="B6" s="62" t="s">
         <v>111</v>
       </c>
-      <c r="C6" s="67" t="s">
+      <c r="C6" s="65" t="s">
         <v>127</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="39" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="63" t="s">
+      <c r="A7" s="61" t="s">
         <v>109</v>
       </c>
-      <c r="B7" s="64" t="s">
+      <c r="B7" s="62" t="s">
         <v>111</v>
       </c>
-      <c r="C7" s="67" t="s">
+      <c r="C7" s="65" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="8" spans="1:11" ht="39" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="63" t="s">
+      <c r="A8" s="61" t="s">
         <v>109</v>
       </c>
-      <c r="B8" s="64" t="s">
+      <c r="B8" s="62" t="s">
         <v>111</v>
       </c>
-      <c r="C8" s="67" t="s">
+      <c r="C8" s="65" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="9" spans="1:11" ht="39" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="63" t="s">
+      <c r="A9" s="61" t="s">
         <v>109</v>
       </c>
-      <c r="B9" s="64" t="s">
+      <c r="B9" s="62" t="s">
         <v>111</v>
       </c>
-      <c r="C9" s="67" t="s">
+      <c r="C9" s="65" t="s">
         <v>130</v>
       </c>
     </row>
     <row r="10" spans="1:11" ht="39" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="63" t="s">
+      <c r="A10" s="61" t="s">
         <v>109</v>
       </c>
-      <c r="B10" s="64" t="s">
+      <c r="B10" s="62" t="s">
         <v>112</v>
       </c>
-      <c r="C10" s="67" t="s">
+      <c r="C10" s="65" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="11" spans="1:11" ht="39" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="63" t="s">
+      <c r="A11" s="61" t="s">
         <v>109</v>
       </c>
-      <c r="B11" s="64" t="s">
+      <c r="B11" s="62" t="s">
         <v>112</v>
       </c>
-      <c r="C11" s="67" t="s">
+      <c r="C11" s="65" t="s">
         <v>132</v>
       </c>
     </row>
     <row r="12" spans="1:11" ht="39" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="63" t="s">
+      <c r="A12" s="61" t="s">
         <v>109</v>
       </c>
-      <c r="B12" s="64" t="s">
+      <c r="B12" s="62" t="s">
         <v>112</v>
       </c>
-      <c r="C12" s="67" t="s">
+      <c r="C12" s="65" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="13" spans="1:11" ht="39" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="63" t="s">
+      <c r="A13" s="61" t="s">
         <v>109</v>
       </c>
-      <c r="B13" s="64" t="s">
+      <c r="B13" s="62" t="s">
         <v>112</v>
       </c>
-      <c r="C13" s="67" t="s">
+      <c r="C13" s="65" t="s">
         <v>134</v>
       </c>
     </row>
     <row r="14" spans="1:11" ht="39" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="63" t="s">
+      <c r="A14" s="61" t="s">
         <v>109</v>
       </c>
-      <c r="B14" s="64" t="s">
+      <c r="B14" s="62" t="s">
         <v>113</v>
       </c>
-      <c r="C14" s="67" t="s">
+      <c r="C14" s="65" t="s">
         <v>135</v>
       </c>
     </row>
     <row r="15" spans="1:11" ht="39" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="63" t="s">
+      <c r="A15" s="61" t="s">
         <v>109</v>
       </c>
-      <c r="B15" s="64" t="s">
+      <c r="B15" s="62" t="s">
         <v>113</v>
       </c>
-      <c r="C15" s="67" t="s">
+      <c r="C15" s="65" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="16" spans="1:11" ht="39" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="63" t="s">
+      <c r="A16" s="61" t="s">
         <v>109</v>
       </c>
-      <c r="B16" s="64" t="s">
+      <c r="B16" s="62" t="s">
         <v>113</v>
       </c>
-      <c r="C16" s="67" t="s">
+      <c r="C16" s="65" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="39" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="63" t="s">
+      <c r="A17" s="61" t="s">
         <v>109</v>
       </c>
-      <c r="B17" s="64" t="s">
+      <c r="B17" s="62" t="s">
         <v>113</v>
       </c>
-      <c r="C17" s="67" t="s">
+      <c r="C17" s="65" t="s">
         <v>138</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="39" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="63" t="s">
+      <c r="A18" s="61" t="s">
         <v>109</v>
       </c>
-      <c r="B18" s="64" t="s">
+      <c r="B18" s="62" t="s">
         <v>113</v>
       </c>
-      <c r="C18" s="67" t="s">
+      <c r="C18" s="65" t="s">
         <v>139</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="39" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="63" t="s">
+      <c r="A19" s="61" t="s">
         <v>109</v>
       </c>
-      <c r="B19" s="64" t="s">
+      <c r="B19" s="62" t="s">
         <v>114</v>
       </c>
-      <c r="C19" s="67" t="s">
+      <c r="C19" s="65" t="s">
         <v>140</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="39" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="63" t="s">
+      <c r="A20" s="61" t="s">
         <v>109</v>
       </c>
-      <c r="B20" s="64" t="s">
+      <c r="B20" s="62" t="s">
         <v>114</v>
       </c>
-      <c r="C20" s="67" t="s">
+      <c r="C20" s="65" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="39" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="63" t="s">
+      <c r="A21" s="61" t="s">
         <v>109</v>
       </c>
-      <c r="B21" s="64" t="s">
+      <c r="B21" s="62" t="s">
         <v>114</v>
       </c>
-      <c r="C21" s="67" t="s">
+      <c r="C21" s="65" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="22" spans="1:3" ht="39" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="63" t="s">
+      <c r="A22" s="61" t="s">
         <v>109</v>
       </c>
-      <c r="B22" s="64" t="s">
+      <c r="B22" s="62" t="s">
         <v>115</v>
       </c>
-      <c r="C22" s="67" t="s">
+      <c r="C22" s="65" t="s">
         <v>143</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="39" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="63" t="s">
+      <c r="A23" s="61" t="s">
         <v>109</v>
       </c>
-      <c r="B23" s="64" t="s">
+      <c r="B23" s="62" t="s">
         <v>115</v>
       </c>
-      <c r="C23" s="67" t="s">
+      <c r="C23" s="65" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="39" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="63" t="s">
+      <c r="A24" s="61" t="s">
         <v>109</v>
       </c>
-      <c r="B24" s="64" t="s">
+      <c r="B24" s="62" t="s">
         <v>116</v>
       </c>
-      <c r="C24" s="67" t="s">
+      <c r="C24" s="65" t="s">
         <v>145</v>
       </c>
     </row>
     <row r="25" spans="1:3" ht="39" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="63" t="s">
+      <c r="A25" s="61" t="s">
         <v>109</v>
       </c>
-      <c r="B25" s="64" t="s">
+      <c r="B25" s="62" t="s">
         <v>116</v>
       </c>
-      <c r="C25" s="67" t="s">
+      <c r="C25" s="65" t="s">
         <v>146</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="39" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="63" t="s">
+      <c r="A26" s="61" t="s">
         <v>109</v>
       </c>
-      <c r="B26" s="64" t="s">
+      <c r="B26" s="62" t="s">
         <v>116</v>
       </c>
-      <c r="C26" s="67" t="s">
+      <c r="C26" s="65" t="s">
         <v>147</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="39" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="63" t="s">
+      <c r="A27" s="61" t="s">
         <v>109</v>
       </c>
-      <c r="B27" s="64" t="s">
+      <c r="B27" s="62" t="s">
         <v>116</v>
       </c>
-      <c r="C27" s="67" t="s">
+      <c r="C27" s="65" t="s">
         <v>148</v>
       </c>
     </row>
     <row r="28" spans="1:3" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="63" t="s">
+      <c r="A28" s="61" t="s">
         <v>117</v>
       </c>
-      <c r="B28" s="64" t="s">
+      <c r="B28" s="62" t="s">
         <v>118</v>
       </c>
-      <c r="C28" s="67" t="s">
+      <c r="C28" s="65" t="s">
         <v>149</v>
       </c>
     </row>
     <row r="29" spans="1:3" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="63" t="s">
+      <c r="A29" s="61" t="s">
         <v>117</v>
       </c>
-      <c r="B29" s="64" t="s">
+      <c r="B29" s="62" t="s">
         <v>118</v>
       </c>
-      <c r="C29" s="67" t="s">
+      <c r="C29" s="65" t="s">
         <v>150</v>
       </c>
     </row>
     <row r="30" spans="1:3" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="63" t="s">
+      <c r="A30" s="61" t="s">
         <v>117</v>
       </c>
-      <c r="B30" s="64" t="s">
+      <c r="B30" s="62" t="s">
         <v>118</v>
       </c>
-      <c r="C30" s="67" t="s">
+      <c r="C30" s="65" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="31" spans="1:3" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="63" t="s">
+      <c r="A31" s="61" t="s">
         <v>117</v>
       </c>
-      <c r="B31" s="64" t="s">
+      <c r="B31" s="62" t="s">
         <v>118</v>
       </c>
-      <c r="C31" s="67" t="s">
+      <c r="C31" s="65" t="s">
         <v>152</v>
       </c>
     </row>
     <row r="32" spans="1:3" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="63" t="s">
+      <c r="A32" s="61" t="s">
         <v>117</v>
       </c>
-      <c r="B32" s="64" t="s">
+      <c r="B32" s="62" t="s">
         <v>119</v>
       </c>
-      <c r="C32" s="67" t="s">
+      <c r="C32" s="65" t="s">
         <v>153</v>
       </c>
     </row>
     <row r="33" spans="1:3" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="63" t="s">
+      <c r="A33" s="61" t="s">
         <v>117</v>
       </c>
-      <c r="B33" s="64" t="s">
+      <c r="B33" s="62" t="s">
         <v>119</v>
       </c>
-      <c r="C33" s="67" t="s">
+      <c r="C33" s="65" t="s">
         <v>154</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="63" t="s">
+      <c r="A34" s="61" t="s">
         <v>117</v>
       </c>
-      <c r="B34" s="64" t="s">
+      <c r="B34" s="62" t="s">
         <v>119</v>
       </c>
-      <c r="C34" s="67" t="s">
+      <c r="C34" s="65" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="35" spans="1:3" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="63" t="s">
+      <c r="A35" s="61" t="s">
         <v>117</v>
       </c>
-      <c r="B35" s="64" t="s">
+      <c r="B35" s="62" t="s">
         <v>120</v>
       </c>
-      <c r="C35" s="67" t="s">
+      <c r="C35" s="65" t="s">
         <v>156</v>
       </c>
     </row>
     <row r="36" spans="1:3" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="63" t="s">
+      <c r="A36" s="61" t="s">
         <v>117</v>
       </c>
-      <c r="B36" s="64" t="s">
+      <c r="B36" s="62" t="s">
         <v>120</v>
       </c>
-      <c r="C36" s="67" t="s">
+      <c r="C36" s="65" t="s">
         <v>157</v>
       </c>
     </row>
     <row r="37" spans="1:3" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="63" t="s">
+      <c r="A37" s="61" t="s">
         <v>117</v>
       </c>
-      <c r="B37" s="64" t="s">
+      <c r="B37" s="62" t="s">
         <v>121</v>
       </c>
-      <c r="C37" s="67" t="s">
+      <c r="C37" s="65" t="s">
         <v>158</v>
       </c>
     </row>
     <row r="38" spans="1:3" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="63" t="s">
+      <c r="A38" s="61" t="s">
         <v>117</v>
       </c>
-      <c r="B38" s="64" t="s">
+      <c r="B38" s="62" t="s">
         <v>121</v>
       </c>
-      <c r="C38" s="67" t="s">
+      <c r="C38" s="65" t="s">
         <v>159</v>
       </c>
     </row>
     <row r="39" spans="1:3" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A39" s="65" t="s">
+      <c r="A39" s="63" t="s">
         <v>117</v>
       </c>
-      <c r="B39" s="66" t="s">
+      <c r="B39" s="64" t="s">
         <v>122</v>
       </c>
-      <c r="C39" s="68" t="s">
+      <c r="C39" s="66" t="s">
         <v>160</v>
       </c>
     </row>
@@ -7417,124 +7376,124 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:24" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A1" s="251" t="s">
+      <c r="A1" s="250" t="s">
         <v>72</v>
       </c>
-      <c r="B1" s="251"/>
-      <c r="C1" s="251"/>
-      <c r="D1" s="251"/>
-      <c r="E1" s="251"/>
-      <c r="F1" s="251"/>
-      <c r="G1" s="251"/>
-      <c r="H1" s="251"/>
-      <c r="I1" s="251"/>
-      <c r="J1" s="251"/>
-      <c r="K1" s="251"/>
-      <c r="L1" s="251"/>
-      <c r="M1" s="251"/>
-      <c r="N1" s="251"/>
-      <c r="O1" s="251"/>
-      <c r="P1" s="251"/>
-      <c r="Q1" s="251"/>
-      <c r="R1" s="251"/>
-      <c r="S1" s="251"/>
-      <c r="T1" s="251"/>
-      <c r="U1" s="251" t="s">
+      <c r="B1" s="250"/>
+      <c r="C1" s="250"/>
+      <c r="D1" s="250"/>
+      <c r="E1" s="250"/>
+      <c r="F1" s="250"/>
+      <c r="G1" s="250"/>
+      <c r="H1" s="250"/>
+      <c r="I1" s="250"/>
+      <c r="J1" s="250"/>
+      <c r="K1" s="250"/>
+      <c r="L1" s="250"/>
+      <c r="M1" s="250"/>
+      <c r="N1" s="250"/>
+      <c r="O1" s="250"/>
+      <c r="P1" s="250"/>
+      <c r="Q1" s="250"/>
+      <c r="R1" s="250"/>
+      <c r="S1" s="250"/>
+      <c r="T1" s="250"/>
+      <c r="U1" s="250" t="s">
         <v>73</v>
       </c>
-      <c r="V1" s="251"/>
-      <c r="W1" s="251"/>
-      <c r="X1" s="251"/>
+      <c r="V1" s="250"/>
+      <c r="W1" s="250"/>
+      <c r="X1" s="250"/>
     </row>
     <row r="2" spans="1:24" ht="33" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="251"/>
-      <c r="B2" s="251"/>
-      <c r="C2" s="251"/>
-      <c r="D2" s="251"/>
-      <c r="E2" s="251"/>
-      <c r="F2" s="251"/>
-      <c r="G2" s="251"/>
-      <c r="H2" s="251"/>
-      <c r="I2" s="251"/>
-      <c r="J2" s="251"/>
-      <c r="K2" s="251"/>
-      <c r="L2" s="251"/>
-      <c r="M2" s="251"/>
-      <c r="N2" s="251"/>
-      <c r="O2" s="251"/>
-      <c r="P2" s="251"/>
-      <c r="Q2" s="251"/>
-      <c r="R2" s="251"/>
-      <c r="S2" s="251"/>
-      <c r="T2" s="251"/>
-      <c r="U2" s="259" t="s">
+      <c r="A2" s="250"/>
+      <c r="B2" s="250"/>
+      <c r="C2" s="250"/>
+      <c r="D2" s="250"/>
+      <c r="E2" s="250"/>
+      <c r="F2" s="250"/>
+      <c r="G2" s="250"/>
+      <c r="H2" s="250"/>
+      <c r="I2" s="250"/>
+      <c r="J2" s="250"/>
+      <c r="K2" s="250"/>
+      <c r="L2" s="250"/>
+      <c r="M2" s="250"/>
+      <c r="N2" s="250"/>
+      <c r="O2" s="250"/>
+      <c r="P2" s="250"/>
+      <c r="Q2" s="250"/>
+      <c r="R2" s="250"/>
+      <c r="S2" s="250"/>
+      <c r="T2" s="250"/>
+      <c r="U2" s="258" t="s">
         <v>74</v>
       </c>
-      <c r="V2" s="259"/>
-      <c r="W2" s="259"/>
-      <c r="X2" s="259"/>
+      <c r="V2" s="258"/>
+      <c r="W2" s="258"/>
+      <c r="X2" s="258"/>
     </row>
     <row r="3" spans="1:24" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="U3" s="260"/>
-      <c r="V3" s="260"/>
-      <c r="W3" s="260"/>
-      <c r="X3" s="260"/>
+      <c r="U3" s="259"/>
+      <c r="V3" s="259"/>
+      <c r="W3" s="259"/>
+      <c r="X3" s="259"/>
     </row>
     <row r="4" spans="1:24" s="2" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="256" t="s">
+      <c r="A4" s="255" t="s">
         <v>75</v>
       </c>
-      <c r="B4" s="257"/>
-      <c r="C4" s="257"/>
-      <c r="D4" s="257"/>
-      <c r="E4" s="257"/>
-      <c r="F4" s="257"/>
-      <c r="G4" s="257"/>
-      <c r="H4" s="257"/>
-      <c r="I4" s="257"/>
-      <c r="J4" s="257"/>
-      <c r="K4" s="257"/>
-      <c r="L4" s="257"/>
-      <c r="M4" s="258"/>
-      <c r="N4" s="256" t="s">
+      <c r="B4" s="256"/>
+      <c r="C4" s="256"/>
+      <c r="D4" s="256"/>
+      <c r="E4" s="256"/>
+      <c r="F4" s="256"/>
+      <c r="G4" s="256"/>
+      <c r="H4" s="256"/>
+      <c r="I4" s="256"/>
+      <c r="J4" s="256"/>
+      <c r="K4" s="256"/>
+      <c r="L4" s="256"/>
+      <c r="M4" s="257"/>
+      <c r="N4" s="255" t="s">
         <v>76</v>
       </c>
-      <c r="O4" s="257"/>
-      <c r="P4" s="257"/>
-      <c r="Q4" s="257"/>
-      <c r="R4" s="257"/>
-      <c r="S4" s="257"/>
-      <c r="T4" s="257"/>
-      <c r="U4" s="257"/>
-      <c r="V4" s="257"/>
-      <c r="W4" s="257"/>
-      <c r="X4" s="258"/>
+      <c r="O4" s="256"/>
+      <c r="P4" s="256"/>
+      <c r="Q4" s="256"/>
+      <c r="R4" s="256"/>
+      <c r="S4" s="256"/>
+      <c r="T4" s="256"/>
+      <c r="U4" s="256"/>
+      <c r="V4" s="256"/>
+      <c r="W4" s="256"/>
+      <c r="X4" s="257"/>
     </row>
     <row r="5" spans="1:24" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="253"/>
-      <c r="B5" s="254"/>
-      <c r="C5" s="254"/>
-      <c r="D5" s="254"/>
-      <c r="E5" s="254"/>
-      <c r="F5" s="254"/>
-      <c r="G5" s="254"/>
-      <c r="H5" s="254"/>
-      <c r="I5" s="254"/>
-      <c r="J5" s="254"/>
-      <c r="K5" s="254"/>
-      <c r="L5" s="254"/>
-      <c r="M5" s="255"/>
-      <c r="N5" s="253"/>
-      <c r="O5" s="254"/>
-      <c r="P5" s="254"/>
-      <c r="Q5" s="254"/>
-      <c r="R5" s="254"/>
-      <c r="S5" s="254"/>
-      <c r="T5" s="254"/>
-      <c r="U5" s="254"/>
-      <c r="V5" s="254"/>
-      <c r="W5" s="254"/>
-      <c r="X5" s="255"/>
+      <c r="A5" s="252"/>
+      <c r="B5" s="253"/>
+      <c r="C5" s="253"/>
+      <c r="D5" s="253"/>
+      <c r="E5" s="253"/>
+      <c r="F5" s="253"/>
+      <c r="G5" s="253"/>
+      <c r="H5" s="253"/>
+      <c r="I5" s="253"/>
+      <c r="J5" s="253"/>
+      <c r="K5" s="253"/>
+      <c r="L5" s="253"/>
+      <c r="M5" s="254"/>
+      <c r="N5" s="252"/>
+      <c r="O5" s="253"/>
+      <c r="P5" s="253"/>
+      <c r="Q5" s="253"/>
+      <c r="R5" s="253"/>
+      <c r="S5" s="253"/>
+      <c r="T5" s="253"/>
+      <c r="U5" s="253"/>
+      <c r="V5" s="253"/>
+      <c r="W5" s="253"/>
+      <c r="X5" s="254"/>
     </row>
     <row r="6" spans="1:24" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3"/>
@@ -7563,66 +7522,66 @@
       <c r="X6" s="3"/>
     </row>
     <row r="7" spans="1:24" s="2" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="252" t="s">
+      <c r="A7" s="251" t="s">
         <v>77</v>
       </c>
-      <c r="B7" s="252"/>
-      <c r="C7" s="252"/>
-      <c r="D7" s="252"/>
-      <c r="E7" s="252"/>
-      <c r="F7" s="252"/>
-      <c r="G7" s="252"/>
-      <c r="H7" s="252"/>
-      <c r="I7" s="252"/>
-      <c r="J7" s="252" t="s">
+      <c r="B7" s="251"/>
+      <c r="C7" s="251"/>
+      <c r="D7" s="251"/>
+      <c r="E7" s="251"/>
+      <c r="F7" s="251"/>
+      <c r="G7" s="251"/>
+      <c r="H7" s="251"/>
+      <c r="I7" s="251"/>
+      <c r="J7" s="251" t="s">
         <v>78</v>
       </c>
-      <c r="K7" s="252"/>
-      <c r="L7" s="252"/>
-      <c r="M7" s="252"/>
-      <c r="N7" s="252"/>
-      <c r="O7" s="252"/>
-      <c r="P7" s="252" t="s">
+      <c r="K7" s="251"/>
+      <c r="L7" s="251"/>
+      <c r="M7" s="251"/>
+      <c r="N7" s="251"/>
+      <c r="O7" s="251"/>
+      <c r="P7" s="251" t="s">
         <v>79</v>
       </c>
-      <c r="Q7" s="252"/>
-      <c r="R7" s="252"/>
-      <c r="S7" s="252"/>
-      <c r="T7" s="252"/>
-      <c r="U7" s="252"/>
-      <c r="V7" s="252"/>
-      <c r="W7" s="252"/>
-      <c r="X7" s="252"/>
+      <c r="Q7" s="251"/>
+      <c r="R7" s="251"/>
+      <c r="S7" s="251"/>
+      <c r="T7" s="251"/>
+      <c r="U7" s="251"/>
+      <c r="V7" s="251"/>
+      <c r="W7" s="251"/>
+      <c r="X7" s="251"/>
     </row>
     <row r="8" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="261"/>
-      <c r="B8" s="261"/>
-      <c r="C8" s="261"/>
-      <c r="D8" s="261"/>
-      <c r="E8" s="261"/>
-      <c r="F8" s="261"/>
-      <c r="G8" s="261"/>
-      <c r="H8" s="261"/>
-      <c r="I8" s="261"/>
-      <c r="J8" s="262" t="s">
+      <c r="A8" s="260"/>
+      <c r="B8" s="260"/>
+      <c r="C8" s="260"/>
+      <c r="D8" s="260"/>
+      <c r="E8" s="260"/>
+      <c r="F8" s="260"/>
+      <c r="G8" s="260"/>
+      <c r="H8" s="260"/>
+      <c r="I8" s="260"/>
+      <c r="J8" s="261" t="s">
         <v>80</v>
       </c>
-      <c r="K8" s="263"/>
-      <c r="L8" s="263"/>
-      <c r="M8" s="263"/>
-      <c r="N8" s="263"/>
-      <c r="O8" s="264"/>
-      <c r="P8" s="262" t="s">
+      <c r="K8" s="262"/>
+      <c r="L8" s="262"/>
+      <c r="M8" s="262"/>
+      <c r="N8" s="262"/>
+      <c r="O8" s="263"/>
+      <c r="P8" s="261" t="s">
         <v>81</v>
       </c>
-      <c r="Q8" s="263"/>
-      <c r="R8" s="263"/>
-      <c r="S8" s="263"/>
-      <c r="T8" s="263"/>
-      <c r="U8" s="263"/>
-      <c r="V8" s="263"/>
-      <c r="W8" s="263"/>
-      <c r="X8" s="264"/>
+      <c r="Q8" s="262"/>
+      <c r="R8" s="262"/>
+      <c r="S8" s="262"/>
+      <c r="T8" s="262"/>
+      <c r="U8" s="262"/>
+      <c r="V8" s="262"/>
+      <c r="W8" s="262"/>
+      <c r="X8" s="263"/>
     </row>
     <row r="9" spans="1:24" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3"/>
@@ -7651,66 +7610,66 @@
       <c r="X9" s="3"/>
     </row>
     <row r="10" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="265" t="s">
+      <c r="A10" s="264" t="s">
         <v>82</v>
       </c>
-      <c r="B10" s="265"/>
-      <c r="C10" s="265"/>
-      <c r="D10" s="265"/>
-      <c r="E10" s="265"/>
-      <c r="F10" s="265"/>
-      <c r="G10" s="265"/>
-      <c r="H10" s="265"/>
-      <c r="I10" s="265"/>
-      <c r="J10" s="265"/>
-      <c r="K10" s="265"/>
-      <c r="L10" s="265"/>
-      <c r="M10" s="265"/>
-      <c r="N10" s="265"/>
-      <c r="O10" s="265"/>
-      <c r="P10" s="265"/>
-      <c r="Q10" s="265"/>
-      <c r="R10" s="265"/>
-      <c r="S10" s="265"/>
-      <c r="T10" s="265"/>
-      <c r="U10" s="265"/>
-      <c r="V10" s="265"/>
-      <c r="W10" s="265"/>
-      <c r="X10" s="265"/>
+      <c r="B10" s="264"/>
+      <c r="C10" s="264"/>
+      <c r="D10" s="264"/>
+      <c r="E10" s="264"/>
+      <c r="F10" s="264"/>
+      <c r="G10" s="264"/>
+      <c r="H10" s="264"/>
+      <c r="I10" s="264"/>
+      <c r="J10" s="264"/>
+      <c r="K10" s="264"/>
+      <c r="L10" s="264"/>
+      <c r="M10" s="264"/>
+      <c r="N10" s="264"/>
+      <c r="O10" s="264"/>
+      <c r="P10" s="264"/>
+      <c r="Q10" s="264"/>
+      <c r="R10" s="264"/>
+      <c r="S10" s="264"/>
+      <c r="T10" s="264"/>
+      <c r="U10" s="264"/>
+      <c r="V10" s="264"/>
+      <c r="W10" s="264"/>
+      <c r="X10" s="264"/>
     </row>
     <row r="11" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="266" t="s">
+      <c r="A11" s="265" t="s">
         <v>83</v>
       </c>
-      <c r="B11" s="266"/>
-      <c r="C11" s="266"/>
-      <c r="D11" s="266"/>
-      <c r="E11" s="266"/>
-      <c r="F11" s="266"/>
-      <c r="G11" s="266" t="s">
+      <c r="B11" s="265"/>
+      <c r="C11" s="265"/>
+      <c r="D11" s="265"/>
+      <c r="E11" s="265"/>
+      <c r="F11" s="265"/>
+      <c r="G11" s="265" t="s">
         <v>84</v>
       </c>
-      <c r="H11" s="266"/>
-      <c r="I11" s="266"/>
-      <c r="J11" s="266"/>
-      <c r="K11" s="266"/>
-      <c r="L11" s="266"/>
-      <c r="M11" s="266" t="s">
+      <c r="H11" s="265"/>
+      <c r="I11" s="265"/>
+      <c r="J11" s="265"/>
+      <c r="K11" s="265"/>
+      <c r="L11" s="265"/>
+      <c r="M11" s="265" t="s">
         <v>85</v>
       </c>
-      <c r="N11" s="266"/>
-      <c r="O11" s="266"/>
-      <c r="P11" s="266"/>
-      <c r="Q11" s="266"/>
-      <c r="R11" s="266"/>
-      <c r="S11" s="266" t="s">
+      <c r="N11" s="265"/>
+      <c r="O11" s="265"/>
+      <c r="P11" s="265"/>
+      <c r="Q11" s="265"/>
+      <c r="R11" s="265"/>
+      <c r="S11" s="265" t="s">
         <v>86</v>
       </c>
-      <c r="T11" s="266"/>
-      <c r="U11" s="266"/>
-      <c r="V11" s="266"/>
-      <c r="W11" s="266"/>
-      <c r="X11" s="266"/>
+      <c r="T11" s="265"/>
+      <c r="U11" s="265"/>
+      <c r="V11" s="265"/>
+      <c r="W11" s="265"/>
+      <c r="X11" s="265"/>
     </row>
     <row r="12" spans="1:24" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3"/>
@@ -7739,66 +7698,66 @@
       <c r="X12" s="3"/>
     </row>
     <row r="13" spans="1:24" s="2" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="252" t="s">
+      <c r="A13" s="251" t="s">
         <v>87</v>
       </c>
-      <c r="B13" s="252"/>
-      <c r="C13" s="252"/>
-      <c r="D13" s="252"/>
-      <c r="E13" s="252"/>
-      <c r="F13" s="252"/>
-      <c r="G13" s="252"/>
-      <c r="H13" s="252"/>
-      <c r="I13" s="252"/>
-      <c r="J13" s="252" t="s">
+      <c r="B13" s="251"/>
+      <c r="C13" s="251"/>
+      <c r="D13" s="251"/>
+      <c r="E13" s="251"/>
+      <c r="F13" s="251"/>
+      <c r="G13" s="251"/>
+      <c r="H13" s="251"/>
+      <c r="I13" s="251"/>
+      <c r="J13" s="251" t="s">
         <v>78</v>
       </c>
-      <c r="K13" s="252"/>
-      <c r="L13" s="252"/>
-      <c r="M13" s="252"/>
-      <c r="N13" s="252"/>
-      <c r="O13" s="252"/>
-      <c r="P13" s="252" t="s">
+      <c r="K13" s="251"/>
+      <c r="L13" s="251"/>
+      <c r="M13" s="251"/>
+      <c r="N13" s="251"/>
+      <c r="O13" s="251"/>
+      <c r="P13" s="251" t="s">
         <v>79</v>
       </c>
-      <c r="Q13" s="252"/>
-      <c r="R13" s="252"/>
-      <c r="S13" s="252"/>
-      <c r="T13" s="252"/>
-      <c r="U13" s="252"/>
-      <c r="V13" s="252"/>
-      <c r="W13" s="252"/>
-      <c r="X13" s="252"/>
+      <c r="Q13" s="251"/>
+      <c r="R13" s="251"/>
+      <c r="S13" s="251"/>
+      <c r="T13" s="251"/>
+      <c r="U13" s="251"/>
+      <c r="V13" s="251"/>
+      <c r="W13" s="251"/>
+      <c r="X13" s="251"/>
     </row>
     <row r="14" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="261"/>
-      <c r="B14" s="261"/>
-      <c r="C14" s="261"/>
-      <c r="D14" s="261"/>
-      <c r="E14" s="261"/>
-      <c r="F14" s="261"/>
-      <c r="G14" s="261"/>
-      <c r="H14" s="261"/>
-      <c r="I14" s="261"/>
-      <c r="J14" s="262" t="s">
+      <c r="A14" s="260"/>
+      <c r="B14" s="260"/>
+      <c r="C14" s="260"/>
+      <c r="D14" s="260"/>
+      <c r="E14" s="260"/>
+      <c r="F14" s="260"/>
+      <c r="G14" s="260"/>
+      <c r="H14" s="260"/>
+      <c r="I14" s="260"/>
+      <c r="J14" s="261" t="s">
         <v>88</v>
       </c>
-      <c r="K14" s="263"/>
-      <c r="L14" s="263"/>
-      <c r="M14" s="263"/>
-      <c r="N14" s="263"/>
-      <c r="O14" s="264"/>
-      <c r="P14" s="262" t="s">
+      <c r="K14" s="262"/>
+      <c r="L14" s="262"/>
+      <c r="M14" s="262"/>
+      <c r="N14" s="262"/>
+      <c r="O14" s="263"/>
+      <c r="P14" s="261" t="s">
         <v>89</v>
       </c>
-      <c r="Q14" s="263"/>
-      <c r="R14" s="263"/>
-      <c r="S14" s="263"/>
-      <c r="T14" s="263"/>
-      <c r="U14" s="263"/>
-      <c r="V14" s="263"/>
-      <c r="W14" s="263"/>
-      <c r="X14" s="264"/>
+      <c r="Q14" s="262"/>
+      <c r="R14" s="262"/>
+      <c r="S14" s="262"/>
+      <c r="T14" s="262"/>
+      <c r="U14" s="262"/>
+      <c r="V14" s="262"/>
+      <c r="W14" s="262"/>
+      <c r="X14" s="263"/>
     </row>
     <row r="15" spans="1:24" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3"/>
@@ -7827,162 +7786,162 @@
       <c r="X15" s="3"/>
     </row>
     <row r="16" spans="1:24" s="4" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="272" t="s">
+      <c r="A16" s="271" t="s">
         <v>90</v>
       </c>
-      <c r="B16" s="272"/>
-      <c r="C16" s="272"/>
-      <c r="D16" s="272"/>
-      <c r="E16" s="272"/>
-      <c r="F16" s="272"/>
-      <c r="G16" s="272"/>
-      <c r="H16" s="272"/>
-      <c r="I16" s="272"/>
-      <c r="J16" s="273" t="s">
+      <c r="B16" s="271"/>
+      <c r="C16" s="271"/>
+      <c r="D16" s="271"/>
+      <c r="E16" s="271"/>
+      <c r="F16" s="271"/>
+      <c r="G16" s="271"/>
+      <c r="H16" s="271"/>
+      <c r="I16" s="271"/>
+      <c r="J16" s="272" t="s">
         <v>91</v>
       </c>
-      <c r="K16" s="273"/>
-      <c r="L16" s="273"/>
-      <c r="M16" s="273"/>
-      <c r="N16" s="272" t="s">
+      <c r="K16" s="272"/>
+      <c r="L16" s="272"/>
+      <c r="M16" s="272"/>
+      <c r="N16" s="271" t="s">
         <v>92</v>
       </c>
-      <c r="O16" s="272"/>
-      <c r="P16" s="272"/>
-      <c r="Q16" s="272"/>
-      <c r="R16" s="272"/>
-      <c r="S16" s="272"/>
-      <c r="T16" s="274" t="s">
+      <c r="O16" s="271"/>
+      <c r="P16" s="271"/>
+      <c r="Q16" s="271"/>
+      <c r="R16" s="271"/>
+      <c r="S16" s="271"/>
+      <c r="T16" s="273" t="s">
         <v>93</v>
       </c>
-      <c r="U16" s="274"/>
-      <c r="V16" s="274"/>
-      <c r="W16" s="274"/>
-      <c r="X16" s="274"/>
+      <c r="U16" s="273"/>
+      <c r="V16" s="273"/>
+      <c r="W16" s="273"/>
+      <c r="X16" s="273"/>
     </row>
     <row r="17" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="267" t="s">
+      <c r="A17" s="266" t="s">
         <v>94</v>
       </c>
-      <c r="B17" s="259"/>
-      <c r="C17" s="259"/>
-      <c r="D17" s="259"/>
-      <c r="E17" s="259"/>
-      <c r="F17" s="259"/>
-      <c r="G17" s="259"/>
-      <c r="H17" s="259"/>
-      <c r="I17" s="268"/>
-      <c r="J17" s="275" t="s">
+      <c r="B17" s="258"/>
+      <c r="C17" s="258"/>
+      <c r="D17" s="258"/>
+      <c r="E17" s="258"/>
+      <c r="F17" s="258"/>
+      <c r="G17" s="258"/>
+      <c r="H17" s="258"/>
+      <c r="I17" s="267"/>
+      <c r="J17" s="274" t="s">
         <v>95</v>
       </c>
-      <c r="K17" s="276"/>
-      <c r="L17" s="276"/>
-      <c r="M17" s="277"/>
-      <c r="N17" s="267" t="s">
+      <c r="K17" s="275"/>
+      <c r="L17" s="275"/>
+      <c r="M17" s="276"/>
+      <c r="N17" s="266" t="s">
         <v>96</v>
       </c>
-      <c r="O17" s="259"/>
-      <c r="P17" s="259"/>
-      <c r="Q17" s="259"/>
-      <c r="R17" s="259"/>
-      <c r="S17" s="268"/>
-      <c r="T17" s="267" t="s">
+      <c r="O17" s="258"/>
+      <c r="P17" s="258"/>
+      <c r="Q17" s="258"/>
+      <c r="R17" s="258"/>
+      <c r="S17" s="267"/>
+      <c r="T17" s="266" t="s">
         <v>97</v>
       </c>
-      <c r="U17" s="259"/>
-      <c r="V17" s="259"/>
-      <c r="W17" s="259"/>
-      <c r="X17" s="268"/>
+      <c r="U17" s="258"/>
+      <c r="V17" s="258"/>
+      <c r="W17" s="258"/>
+      <c r="X17" s="267"/>
     </row>
     <row r="18" spans="1:24" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="269"/>
-      <c r="B18" s="270"/>
-      <c r="C18" s="270"/>
-      <c r="D18" s="270"/>
-      <c r="E18" s="270"/>
-      <c r="F18" s="270"/>
-      <c r="G18" s="270"/>
-      <c r="H18" s="270"/>
-      <c r="I18" s="271"/>
-      <c r="J18" s="278"/>
-      <c r="K18" s="279"/>
-      <c r="L18" s="279"/>
-      <c r="M18" s="280"/>
-      <c r="N18" s="269"/>
-      <c r="O18" s="270"/>
-      <c r="P18" s="270"/>
-      <c r="Q18" s="270"/>
-      <c r="R18" s="270"/>
-      <c r="S18" s="271"/>
-      <c r="T18" s="269"/>
-      <c r="U18" s="270"/>
-      <c r="V18" s="270"/>
-      <c r="W18" s="270"/>
-      <c r="X18" s="271"/>
+      <c r="A18" s="268"/>
+      <c r="B18" s="269"/>
+      <c r="C18" s="269"/>
+      <c r="D18" s="269"/>
+      <c r="E18" s="269"/>
+      <c r="F18" s="269"/>
+      <c r="G18" s="269"/>
+      <c r="H18" s="269"/>
+      <c r="I18" s="270"/>
+      <c r="J18" s="277"/>
+      <c r="K18" s="278"/>
+      <c r="L18" s="278"/>
+      <c r="M18" s="279"/>
+      <c r="N18" s="268"/>
+      <c r="O18" s="269"/>
+      <c r="P18" s="269"/>
+      <c r="Q18" s="269"/>
+      <c r="R18" s="269"/>
+      <c r="S18" s="270"/>
+      <c r="T18" s="268"/>
+      <c r="U18" s="269"/>
+      <c r="V18" s="269"/>
+      <c r="W18" s="269"/>
+      <c r="X18" s="270"/>
     </row>
     <row r="19" spans="1:24" ht="39" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="20" spans="1:24" ht="39" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="21" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A21" s="284" t="s">
+      <c r="A21" s="283" t="s">
         <v>98</v>
       </c>
-      <c r="B21" s="284"/>
-      <c r="C21" s="284"/>
-      <c r="D21" s="284"/>
-      <c r="E21" s="284"/>
-      <c r="F21" s="284"/>
-      <c r="G21" s="284"/>
-      <c r="H21" s="284"/>
+      <c r="B21" s="283"/>
+      <c r="C21" s="283"/>
+      <c r="D21" s="283"/>
+      <c r="E21" s="283"/>
+      <c r="F21" s="283"/>
+      <c r="G21" s="283"/>
+      <c r="H21" s="283"/>
       <c r="I21" s="5"/>
-      <c r="J21" s="284" t="s">
+      <c r="J21" s="283" t="s">
         <v>65</v>
       </c>
-      <c r="K21" s="284"/>
-      <c r="L21" s="284"/>
-      <c r="M21" s="284"/>
-      <c r="N21" s="284"/>
-      <c r="O21" s="284"/>
-      <c r="P21" s="284"/>
+      <c r="K21" s="283"/>
+      <c r="L21" s="283"/>
+      <c r="M21" s="283"/>
+      <c r="N21" s="283"/>
+      <c r="O21" s="283"/>
+      <c r="P21" s="283"/>
       <c r="Q21" s="6"/>
-      <c r="R21" s="284" t="s">
+      <c r="R21" s="283" t="s">
         <v>99</v>
       </c>
-      <c r="S21" s="284"/>
-      <c r="T21" s="284"/>
-      <c r="U21" s="284"/>
-      <c r="V21" s="284"/>
-      <c r="W21" s="284"/>
-      <c r="X21" s="284"/>
+      <c r="S21" s="283"/>
+      <c r="T21" s="283"/>
+      <c r="U21" s="283"/>
+      <c r="V21" s="283"/>
+      <c r="W21" s="283"/>
+      <c r="X21" s="283"/>
     </row>
     <row r="23" spans="1:24" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="P23" s="281" t="s">
+      <c r="P23" s="280" t="s">
         <v>100</v>
       </c>
-      <c r="Q23" s="281"/>
-      <c r="R23" s="281"/>
-      <c r="S23" s="281"/>
-      <c r="T23" s="281"/>
-      <c r="U23" s="282" t="s">
+      <c r="Q23" s="280"/>
+      <c r="R23" s="280"/>
+      <c r="S23" s="280"/>
+      <c r="T23" s="280"/>
+      <c r="U23" s="281" t="s">
         <v>101</v>
       </c>
-      <c r="V23" s="282"/>
-      <c r="W23" s="282"/>
-      <c r="X23" s="282"/>
+      <c r="V23" s="281"/>
+      <c r="W23" s="281"/>
+      <c r="X23" s="281"/>
     </row>
     <row r="24" spans="1:24" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="P24" s="281" t="s">
+      <c r="P24" s="280" t="s">
         <v>102</v>
       </c>
-      <c r="Q24" s="281"/>
-      <c r="R24" s="281"/>
-      <c r="S24" s="281"/>
-      <c r="T24" s="281"/>
-      <c r="U24" s="283" t="s">
+      <c r="Q24" s="280"/>
+      <c r="R24" s="280"/>
+      <c r="S24" s="280"/>
+      <c r="T24" s="280"/>
+      <c r="U24" s="282" t="s">
         <v>103</v>
       </c>
-      <c r="V24" s="283"/>
-      <c r="W24" s="283"/>
-      <c r="X24" s="283"/>
+      <c r="V24" s="282"/>
+      <c r="W24" s="282"/>
+      <c r="X24" s="282"/>
     </row>
   </sheetData>
   <mergeCells count="40">

</xml_diff>

<commit_message>
Actualiza formatos de Bitácora F-147 y Visita 3 en el centro de descargas.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Formatos/BITACORAS GFPI-F-147V4.xlsx
+++ b/Formatos/BITACORAS GFPI-F-147V4.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uniminuto0-my.sharepoint.com/personal/sergio_torres_mar_uniminuto_edu_co/Documents/Documentos/Seto 2026/SETO/sena/Manual SENA Etapa Productiva/manual-aprendiz-sena/Formatos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="15" documentId="13_ncr:1_{BEF1DC7A-FFF1-4291-A724-1398C9A655DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{34869B08-79A4-49EA-A549-21A9B73FC24F}"/>
+  <xr:revisionPtr revIDLastSave="25" documentId="13_ncr:1_{BEF1DC7A-FFF1-4291-A724-1398C9A655DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C48CE772-E924-4622-97BD-AE0184CF7A9F}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-105" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Bitacora" sheetId="6" r:id="rId1"/>
@@ -651,7 +651,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="36" x14ac:knownFonts="1">
+  <fonts count="37" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -895,6 +895,11 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="8">
     <fill>
@@ -2429,7 +2434,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="284">
+  <cellXfs count="289">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -2631,6 +2636,303 @@
     <xf numFmtId="0" fontId="21" fillId="0" borderId="107" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="96" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="93" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="93" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="94" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="92" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="93" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="93" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="61" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="72" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="87" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="88" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="65" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="70" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="74" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="61" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="76" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="71" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="75" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="59" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="2" borderId="70" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="2" borderId="74" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="2" borderId="58" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="79" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="80" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="103" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="104" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="105" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="104" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="105" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="70" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="74" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="71" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="75" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="59" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="106" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="82" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="83" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="52" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="58" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="59" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="60" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="54" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="69" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="73" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="63" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="7" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2640,6 +2942,177 @@
     <xf numFmtId="0" fontId="11" fillId="7" borderId="78" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="97" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="100" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="91" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="57" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="58" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="59" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="66" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="67" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="63" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="68" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="85" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="86" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="98" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="100" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="101" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="95" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="96" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="99" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="89" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="90" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="64" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="66" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="67" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="84" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="85" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="86" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="66" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="67" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="85" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="86" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="5" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="5" borderId="57" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="64" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="2" borderId="71" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2652,9 +3125,6 @@
     <xf numFmtId="0" fontId="12" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="2" borderId="62" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2663,9 +3133,6 @@
     </xf>
     <xf numFmtId="0" fontId="12" fillId="2" borderId="102" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="3" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2685,13 +3152,7 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2715,471 +3176,87 @@
     <xf numFmtId="0" fontId="17" fillId="0" borderId="110" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="89" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="90" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="64" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="66" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="67" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="84" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="85" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="86" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="66" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="67" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="85" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="86" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="5" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="5" borderId="57" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="63" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="64" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="96" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="93" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="97" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="100" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="91" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="57" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="58" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="59" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="66" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="67" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="68" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="85" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="86" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="98" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="100" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="101" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="92" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="93" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="95" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="96" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="99" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="70" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="74" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="69" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="73" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="63" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="79" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="80" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="103" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="104" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="105" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="104" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="105" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="71" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="75" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="59" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="106" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="82" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="83" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="52" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="58" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="59" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="60" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="54" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="71" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="75" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="59" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="61" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="72" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="7" borderId="87" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="7" borderId="88" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="94" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="65" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="70" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="74" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="61" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="7" borderId="76" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="7" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="7" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="2" borderId="70" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="2" borderId="74" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="2" borderId="58" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="93" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="93" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -3198,89 +3275,74 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="93" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="94" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="93" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="10">
+  <dxfs count="16">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFE1EF57"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -3657,12 +3719,12 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{99010CAF-386D-41BE-AE72-8D38EFA83A09}" name="TablaSena" displayName="TablaSena" ref="A1:C39" totalsRowShown="0" headerRowDxfId="9" headerRowBorderDxfId="8" tableBorderDxfId="7" totalsRowBorderDxfId="6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{99010CAF-386D-41BE-AE72-8D38EFA83A09}" name="TablaSena" displayName="TablaSena" ref="A1:C39" totalsRowShown="0" headerRowDxfId="15" headerRowBorderDxfId="14" tableBorderDxfId="13" totalsRowBorderDxfId="12">
   <autoFilter ref="A1:C39" xr:uid="{99010CAF-386D-41BE-AE72-8D38EFA83A09}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{61F34070-348E-42B3-BF87-5A1CD2BB6FD7}" name="PROGRAMA" dataDxfId="5"/>
-    <tableColumn id="2" xr3:uid="{7B4CB996-89B6-45DE-A53A-D02152366731}" name="COMPETENCIA" dataDxfId="4"/>
-    <tableColumn id="3" xr3:uid="{529DD12A-961C-42BF-9AA1-50D419FC6C5E}" name="RESULTADO DE APRENDIZAJE (RAP)" dataDxfId="3"/>
+    <tableColumn id="1" xr3:uid="{61F34070-348E-42B3-BF87-5A1CD2BB6FD7}" name="PROGRAMA" dataDxfId="11"/>
+    <tableColumn id="2" xr3:uid="{7B4CB996-89B6-45DE-A53A-D02152366731}" name="COMPETENCIA" dataDxfId="10"/>
+    <tableColumn id="3" xr3:uid="{529DD12A-961C-42BF-9AA1-50D419FC6C5E}" name="RESULTADO DE APRENDIZAJE (RAP)" dataDxfId="9"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium6" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3958,7 +4020,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AB113"/>
+  <dimension ref="A1:XFD113"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="0" defaultRowHeight="15" customHeight="1" zeroHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2.28515625" style="36" customWidth="1"/>
@@ -3969,7 +4031,7 @@
     <col min="6" max="6" width="22.5703125" style="36" customWidth="1"/>
     <col min="7" max="7" width="22.5703125" style="9" customWidth="1"/>
     <col min="8" max="8" width="32.7109375" style="9" customWidth="1"/>
-    <col min="9" max="9" width="34.42578125" style="9" customWidth="1"/>
+    <col min="9" max="9" width="27.42578125" style="9" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="8.42578125" style="9" hidden="1" customWidth="1"/>
     <col min="11" max="11" width="6.42578125" style="9" hidden="1" customWidth="1"/>
     <col min="12" max="17" width="5.7109375" style="9" hidden="1" customWidth="1"/>
@@ -3983,7 +4045,8 @@
     <col min="26" max="26" width="8.140625" style="9" hidden="1" customWidth="1"/>
     <col min="27" max="27" width="5.140625" style="9" hidden="1" customWidth="1"/>
     <col min="28" max="28" width="24.42578125" style="8" hidden="1" customWidth="1"/>
-    <col min="29" max="16384" width="11.42578125" style="7" hidden="1"/>
+    <col min="29" max="16383" width="11.42578125" style="7" hidden="1"/>
+    <col min="16384" max="16384" width="1.28515625" style="7" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:28" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -4049,16 +4112,16 @@
       <c r="AB2" s="7"/>
     </row>
     <row r="3" spans="2:28" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="175" t="s">
+      <c r="B3" s="133" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="176"/>
-      <c r="D3" s="176"/>
-      <c r="E3" s="176"/>
-      <c r="F3" s="176"/>
-      <c r="G3" s="176"/>
-      <c r="H3" s="176"/>
-      <c r="I3" s="177"/>
+      <c r="C3" s="134"/>
+      <c r="D3" s="134"/>
+      <c r="E3" s="134"/>
+      <c r="F3" s="134"/>
+      <c r="G3" s="134"/>
+      <c r="H3" s="134"/>
+      <c r="I3" s="135"/>
       <c r="J3" s="8"/>
       <c r="K3" s="7"/>
       <c r="L3" s="7"/>
@@ -4080,16 +4143,16 @@
       <c r="AB3" s="7"/>
     </row>
     <row r="4" spans="2:28" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="181" t="s">
+      <c r="B4" s="139" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="182"/>
-      <c r="D4" s="182"/>
-      <c r="E4" s="182"/>
-      <c r="F4" s="182"/>
-      <c r="G4" s="182"/>
-      <c r="H4" s="182"/>
-      <c r="I4" s="183"/>
+      <c r="C4" s="140"/>
+      <c r="D4" s="140"/>
+      <c r="E4" s="140"/>
+      <c r="F4" s="140"/>
+      <c r="G4" s="140"/>
+      <c r="H4" s="140"/>
+      <c r="I4" s="141"/>
       <c r="J4" s="8"/>
       <c r="K4" s="7"/>
       <c r="L4" s="7"/>
@@ -4111,16 +4174,16 @@
       <c r="AB4" s="7"/>
     </row>
     <row r="5" spans="2:28" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="178" t="s">
+      <c r="B5" s="136" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="179"/>
-      <c r="D5" s="179"/>
-      <c r="E5" s="179"/>
-      <c r="F5" s="179"/>
-      <c r="G5" s="179"/>
-      <c r="H5" s="179"/>
-      <c r="I5" s="180"/>
+      <c r="C5" s="137"/>
+      <c r="D5" s="137"/>
+      <c r="E5" s="137"/>
+      <c r="F5" s="137"/>
+      <c r="G5" s="137"/>
+      <c r="H5" s="137"/>
+      <c r="I5" s="138"/>
       <c r="J5" s="8"/>
       <c r="K5" s="8"/>
       <c r="L5" s="7"/>
@@ -4142,16 +4205,16 @@
       <c r="AB5" s="7"/>
     </row>
     <row r="6" spans="2:28" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="181" t="s">
+      <c r="B6" s="139" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="182"/>
-      <c r="D6" s="182"/>
-      <c r="E6" s="182"/>
-      <c r="F6" s="182"/>
-      <c r="G6" s="182"/>
-      <c r="H6" s="182"/>
-      <c r="I6" s="183"/>
+      <c r="C6" s="140"/>
+      <c r="D6" s="140"/>
+      <c r="E6" s="140"/>
+      <c r="F6" s="140"/>
+      <c r="G6" s="140"/>
+      <c r="H6" s="140"/>
+      <c r="I6" s="141"/>
       <c r="J6" s="8"/>
       <c r="K6" s="8"/>
       <c r="L6" s="7"/>
@@ -4173,16 +4236,16 @@
       <c r="AB6" s="7"/>
     </row>
     <row r="7" spans="2:28" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="178" t="s">
+      <c r="B7" s="136" t="s">
         <v>6</v>
       </c>
-      <c r="C7" s="179"/>
-      <c r="D7" s="179"/>
-      <c r="E7" s="179"/>
-      <c r="F7" s="179"/>
-      <c r="G7" s="179"/>
-      <c r="H7" s="179"/>
-      <c r="I7" s="180"/>
+      <c r="C7" s="137"/>
+      <c r="D7" s="137"/>
+      <c r="E7" s="137"/>
+      <c r="F7" s="137"/>
+      <c r="G7" s="137"/>
+      <c r="H7" s="137"/>
+      <c r="I7" s="138"/>
       <c r="J7" s="7"/>
       <c r="K7" s="7"/>
       <c r="L7" s="7"/>
@@ -4207,12 +4270,12 @@
       <c r="B8" s="53" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="188"/>
-      <c r="D8" s="189"/>
-      <c r="E8" s="190" t="s">
+      <c r="C8" s="152"/>
+      <c r="D8" s="153"/>
+      <c r="E8" s="154" t="s">
         <v>8</v>
       </c>
-      <c r="F8" s="188"/>
+      <c r="F8" s="152"/>
       <c r="G8" s="67"/>
       <c r="H8" s="54" t="s">
         <v>9</v>
@@ -4244,8 +4307,8 @@
       <c r="D9" s="18"/>
       <c r="E9" s="23"/>
       <c r="F9" s="23"/>
-      <c r="G9" s="201"/>
-      <c r="H9" s="201"/>
+      <c r="G9" s="113"/>
+      <c r="H9" s="113"/>
       <c r="I9" s="18"/>
       <c r="J9" s="7"/>
       <c r="K9" s="7"/>
@@ -4268,18 +4331,18 @@
       <c r="AB9" s="7"/>
     </row>
     <row r="10" spans="2:28" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="168" t="s">
+      <c r="B10" s="146" t="s">
         <v>10</v>
       </c>
-      <c r="C10" s="169"/>
-      <c r="D10" s="170"/>
-      <c r="E10" s="164" t="s">
+      <c r="C10" s="147"/>
+      <c r="D10" s="148"/>
+      <c r="E10" s="142" t="s">
         <v>11</v>
       </c>
-      <c r="F10" s="164"/>
-      <c r="G10" s="164"/>
-      <c r="H10" s="164"/>
-      <c r="I10" s="164"/>
+      <c r="F10" s="142"/>
+      <c r="G10" s="142"/>
+      <c r="H10" s="142"/>
+      <c r="I10" s="142"/>
       <c r="J10" s="7"/>
       <c r="K10" s="7"/>
       <c r="L10" s="7"/>
@@ -4301,14 +4364,14 @@
       <c r="AB10" s="7"/>
     </row>
     <row r="11" spans="2:28" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="198"/>
-      <c r="C11" s="199"/>
-      <c r="D11" s="200"/>
-      <c r="E11" s="197"/>
-      <c r="F11" s="197"/>
-      <c r="G11" s="197"/>
-      <c r="H11" s="197"/>
-      <c r="I11" s="197"/>
+      <c r="B11" s="125"/>
+      <c r="C11" s="126"/>
+      <c r="D11" s="127"/>
+      <c r="E11" s="161"/>
+      <c r="F11" s="161"/>
+      <c r="G11" s="161"/>
+      <c r="H11" s="161"/>
+      <c r="I11" s="161"/>
       <c r="J11" s="7"/>
       <c r="K11" s="7"/>
       <c r="L11" s="7"/>
@@ -4335,8 +4398,8 @@
       <c r="D12" s="18"/>
       <c r="E12" s="23"/>
       <c r="F12" s="23"/>
-      <c r="G12" s="201"/>
-      <c r="H12" s="201"/>
+      <c r="G12" s="113"/>
+      <c r="H12" s="113"/>
       <c r="I12" s="18"/>
       <c r="J12" s="7"/>
       <c r="K12" s="7"/>
@@ -4359,16 +4422,16 @@
       <c r="AB12" s="7"/>
     </row>
     <row r="13" spans="2:28" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="195" t="s">
+      <c r="B13" s="159" t="s">
         <v>12</v>
       </c>
-      <c r="C13" s="195"/>
-      <c r="D13" s="195"/>
-      <c r="E13" s="195"/>
-      <c r="F13" s="195"/>
-      <c r="G13" s="195"/>
-      <c r="H13" s="195"/>
-      <c r="I13" s="196"/>
+      <c r="C13" s="159"/>
+      <c r="D13" s="159"/>
+      <c r="E13" s="159"/>
+      <c r="F13" s="159"/>
+      <c r="G13" s="159"/>
+      <c r="H13" s="159"/>
+      <c r="I13" s="160"/>
       <c r="J13" s="7"/>
       <c r="K13" s="7"/>
       <c r="L13" s="7"/>
@@ -4390,32 +4453,32 @@
       <c r="AB13" s="7"/>
     </row>
     <row r="14" spans="2:28" s="9" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="168" t="s">
+      <c r="B14" s="146" t="s">
         <v>13</v>
       </c>
-      <c r="C14" s="169"/>
-      <c r="D14" s="170"/>
+      <c r="C14" s="147"/>
+      <c r="D14" s="148"/>
       <c r="E14" s="55" t="s">
         <v>14</v>
       </c>
-      <c r="F14" s="191" t="s">
+      <c r="F14" s="155" t="s">
         <v>15</v>
       </c>
-      <c r="G14" s="192"/>
-      <c r="H14" s="164" t="s">
+      <c r="G14" s="156"/>
+      <c r="H14" s="142" t="s">
         <v>16</v>
       </c>
-      <c r="I14" s="165"/>
+      <c r="I14" s="143"/>
     </row>
     <row r="15" spans="2:28" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="185"/>
-      <c r="C15" s="186"/>
-      <c r="D15" s="187"/>
+      <c r="B15" s="149"/>
+      <c r="C15" s="150"/>
+      <c r="D15" s="151"/>
       <c r="E15" s="37"/>
-      <c r="F15" s="193"/>
-      <c r="G15" s="194"/>
-      <c r="H15" s="135"/>
-      <c r="I15" s="184"/>
+      <c r="F15" s="157"/>
+      <c r="G15" s="158"/>
+      <c r="H15" s="144"/>
+      <c r="I15" s="145"/>
       <c r="J15" s="7"/>
       <c r="K15" s="7"/>
       <c r="L15" s="7"/>
@@ -4437,20 +4500,20 @@
       <c r="AB15" s="7"/>
     </row>
     <row r="16" spans="2:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="217" t="s">
+      <c r="B16" s="118" t="s">
         <v>17</v>
       </c>
-      <c r="C16" s="218"/>
-      <c r="D16" s="219"/>
-      <c r="E16" s="220" t="s">
+      <c r="C16" s="119"/>
+      <c r="D16" s="120"/>
+      <c r="E16" s="121" t="s">
         <v>18</v>
       </c>
-      <c r="F16" s="220"/>
-      <c r="G16" s="220"/>
-      <c r="H16" s="202" t="s">
+      <c r="F16" s="121"/>
+      <c r="G16" s="121"/>
+      <c r="H16" s="104" t="s">
         <v>19</v>
       </c>
-      <c r="I16" s="203"/>
+      <c r="I16" s="105"/>
       <c r="J16" s="7"/>
       <c r="K16" s="7"/>
       <c r="L16" s="7"/>
@@ -4472,14 +4535,14 @@
       <c r="AB16" s="7"/>
     </row>
     <row r="17" spans="2:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="198"/>
-      <c r="C17" s="199"/>
-      <c r="D17" s="200"/>
-      <c r="E17" s="174"/>
-      <c r="F17" s="174"/>
-      <c r="G17" s="174"/>
-      <c r="H17" s="166"/>
-      <c r="I17" s="167"/>
+      <c r="B17" s="125"/>
+      <c r="C17" s="126"/>
+      <c r="D17" s="127"/>
+      <c r="E17" s="167"/>
+      <c r="F17" s="167"/>
+      <c r="G17" s="167"/>
+      <c r="H17" s="162"/>
+      <c r="I17" s="163"/>
       <c r="J17" s="7"/>
       <c r="K17" s="7"/>
       <c r="L17" s="7"/>
@@ -4501,20 +4564,20 @@
       <c r="AB17" s="7"/>
     </row>
     <row r="18" spans="2:28" s="47" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="168" t="s">
+      <c r="B18" s="146" t="s">
         <v>20</v>
       </c>
-      <c r="C18" s="169"/>
-      <c r="D18" s="170"/>
-      <c r="E18" s="164" t="s">
+      <c r="C18" s="147"/>
+      <c r="D18" s="148"/>
+      <c r="E18" s="142" t="s">
         <v>21</v>
       </c>
-      <c r="F18" s="164"/>
-      <c r="G18" s="164"/>
-      <c r="H18" s="164" t="s">
+      <c r="F18" s="142"/>
+      <c r="G18" s="142"/>
+      <c r="H18" s="142" t="s">
         <v>22</v>
       </c>
-      <c r="I18" s="165"/>
+      <c r="I18" s="143"/>
       <c r="J18" s="7"/>
       <c r="K18" s="7"/>
       <c r="L18" s="7"/>
@@ -4536,14 +4599,14 @@
       <c r="AB18" s="7"/>
     </row>
     <row r="19" spans="2:28" s="47" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="171"/>
-      <c r="C19" s="172"/>
-      <c r="D19" s="173"/>
-      <c r="E19" s="166"/>
-      <c r="F19" s="166"/>
-      <c r="G19" s="166"/>
-      <c r="H19" s="166"/>
-      <c r="I19" s="167"/>
+      <c r="B19" s="164"/>
+      <c r="C19" s="165"/>
+      <c r="D19" s="166"/>
+      <c r="E19" s="162"/>
+      <c r="F19" s="162"/>
+      <c r="G19" s="162"/>
+      <c r="H19" s="162"/>
+      <c r="I19" s="163"/>
       <c r="J19" s="7"/>
       <c r="K19" s="7"/>
       <c r="L19" s="7"/>
@@ -4565,20 +4628,20 @@
       <c r="AB19" s="7"/>
     </row>
     <row r="20" spans="2:28" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="225" t="s">
+      <c r="B20" s="130" t="s">
         <v>23</v>
       </c>
-      <c r="C20" s="226"/>
-      <c r="D20" s="227"/>
-      <c r="E20" s="136" t="s">
+      <c r="C20" s="131"/>
+      <c r="D20" s="132"/>
+      <c r="E20" s="128" t="s">
         <v>24</v>
       </c>
-      <c r="F20" s="136"/>
-      <c r="G20" s="136"/>
-      <c r="H20" s="136" t="s">
+      <c r="F20" s="128"/>
+      <c r="G20" s="128"/>
+      <c r="H20" s="128" t="s">
         <v>25</v>
       </c>
-      <c r="I20" s="224"/>
+      <c r="I20" s="129"/>
       <c r="J20" s="16"/>
       <c r="K20" s="16"/>
       <c r="L20" s="16"/>
@@ -4598,14 +4661,14 @@
       <c r="AA20" s="16"/>
     </row>
     <row r="21" spans="2:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="198"/>
-      <c r="C21" s="199"/>
-      <c r="D21" s="200"/>
-      <c r="E21" s="135"/>
-      <c r="F21" s="135"/>
-      <c r="G21" s="135"/>
-      <c r="H21" s="133"/>
-      <c r="I21" s="134"/>
+      <c r="B21" s="125"/>
+      <c r="C21" s="126"/>
+      <c r="D21" s="127"/>
+      <c r="E21" s="144"/>
+      <c r="F21" s="144"/>
+      <c r="G21" s="144"/>
+      <c r="H21" s="173"/>
+      <c r="I21" s="174"/>
       <c r="J21" s="18"/>
       <c r="K21" s="18"/>
       <c r="L21" s="18"/>
@@ -4630,8 +4693,8 @@
       <c r="D22" s="13"/>
       <c r="E22" s="33"/>
       <c r="F22" s="33"/>
-      <c r="G22" s="89"/>
-      <c r="H22" s="89"/>
+      <c r="G22" s="112"/>
+      <c r="H22" s="112"/>
       <c r="I22" s="13"/>
       <c r="J22" s="13"/>
       <c r="K22" s="13"/>
@@ -4653,16 +4716,16 @@
       <c r="AA22" s="13"/>
     </row>
     <row r="23" spans="2:28" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="69" t="s">
+      <c r="B23" s="168" t="s">
         <v>26</v>
       </c>
-      <c r="C23" s="70"/>
-      <c r="D23" s="70"/>
-      <c r="E23" s="70"/>
-      <c r="F23" s="70"/>
-      <c r="G23" s="70"/>
-      <c r="H23" s="70"/>
-      <c r="I23" s="71"/>
+      <c r="C23" s="169"/>
+      <c r="D23" s="169"/>
+      <c r="E23" s="169"/>
+      <c r="F23" s="169"/>
+      <c r="G23" s="169"/>
+      <c r="H23" s="169"/>
+      <c r="I23" s="170"/>
       <c r="J23" s="13"/>
       <c r="K23" s="13"/>
       <c r="L23" s="13"/>
@@ -4683,20 +4746,20 @@
       <c r="AA23" s="13"/>
     </row>
     <row r="24" spans="2:28" s="9" customFormat="1" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="131" t="s">
+      <c r="B24" s="171" t="s">
         <v>27</v>
       </c>
-      <c r="C24" s="132"/>
-      <c r="D24" s="132"/>
-      <c r="E24" s="132"/>
-      <c r="F24" s="137" t="s">
+      <c r="C24" s="172"/>
+      <c r="D24" s="172"/>
+      <c r="E24" s="172"/>
+      <c r="F24" s="114" t="s">
         <v>28</v>
       </c>
-      <c r="G24" s="137"/>
-      <c r="H24" s="132" t="s">
+      <c r="G24" s="114"/>
+      <c r="H24" s="172" t="s">
         <v>29</v>
       </c>
-      <c r="I24" s="153"/>
+      <c r="I24" s="195"/>
       <c r="J24" s="18"/>
       <c r="K24" s="18"/>
       <c r="M24" s="16"/>
@@ -4709,14 +4772,14 @@
       <c r="AB24" s="10"/>
     </row>
     <row r="25" spans="2:28" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="163"/>
-      <c r="C25" s="138"/>
-      <c r="D25" s="138"/>
-      <c r="E25" s="138"/>
-      <c r="F25" s="138"/>
-      <c r="G25" s="138"/>
-      <c r="H25" s="154"/>
-      <c r="I25" s="155"/>
+      <c r="B25" s="203"/>
+      <c r="C25" s="175"/>
+      <c r="D25" s="175"/>
+      <c r="E25" s="175"/>
+      <c r="F25" s="175"/>
+      <c r="G25" s="175"/>
+      <c r="H25" s="196"/>
+      <c r="I25" s="197"/>
       <c r="J25" s="18"/>
       <c r="K25" s="18"/>
       <c r="M25" s="18"/>
@@ -4733,8 +4796,8 @@
       <c r="D26" s="13"/>
       <c r="E26" s="33"/>
       <c r="F26" s="33"/>
-      <c r="G26" s="89"/>
-      <c r="H26" s="89"/>
+      <c r="G26" s="112"/>
+      <c r="H26" s="112"/>
       <c r="I26" s="13"/>
       <c r="J26" s="13"/>
       <c r="K26" s="13"/>
@@ -4756,16 +4819,16 @@
       <c r="AA26" s="13"/>
     </row>
     <row r="27" spans="2:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B27" s="160" t="s">
+      <c r="B27" s="200" t="s">
         <v>30</v>
       </c>
-      <c r="C27" s="161"/>
-      <c r="D27" s="161"/>
-      <c r="E27" s="161"/>
-      <c r="F27" s="161"/>
-      <c r="G27" s="161"/>
-      <c r="H27" s="161"/>
-      <c r="I27" s="162"/>
+      <c r="C27" s="201"/>
+      <c r="D27" s="201"/>
+      <c r="E27" s="201"/>
+      <c r="F27" s="201"/>
+      <c r="G27" s="201"/>
+      <c r="H27" s="201"/>
+      <c r="I27" s="202"/>
       <c r="J27" s="13"/>
       <c r="K27" s="13"/>
       <c r="L27" s="13"/>
@@ -4786,22 +4849,22 @@
       <c r="AA27" s="13"/>
     </row>
     <row r="28" spans="2:28" s="9" customFormat="1" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B28" s="156" t="s">
+      <c r="B28" s="198" t="s">
         <v>31</v>
       </c>
-      <c r="C28" s="132"/>
-      <c r="D28" s="132"/>
-      <c r="E28" s="137" t="s">
+      <c r="C28" s="172"/>
+      <c r="D28" s="172"/>
+      <c r="E28" s="114" t="s">
         <v>32</v>
       </c>
-      <c r="F28" s="137"/>
+      <c r="F28" s="114"/>
       <c r="G28" s="49" t="s">
         <v>33</v>
       </c>
-      <c r="H28" s="132" t="s">
+      <c r="H28" s="172" t="s">
         <v>34</v>
       </c>
-      <c r="I28" s="159"/>
+      <c r="I28" s="199"/>
       <c r="J28" s="16"/>
       <c r="N28" s="16"/>
       <c r="O28" s="16"/>
@@ -4818,14 +4881,14 @@
       <c r="AB28" s="10"/>
     </row>
     <row r="29" spans="2:28" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B29" s="157"/>
-      <c r="C29" s="158"/>
-      <c r="D29" s="158"/>
-      <c r="E29" s="158"/>
-      <c r="F29" s="158"/>
+      <c r="B29" s="100"/>
+      <c r="C29" s="101"/>
+      <c r="D29" s="101"/>
+      <c r="E29" s="101"/>
+      <c r="F29" s="101"/>
       <c r="G29" s="52"/>
-      <c r="H29" s="158"/>
-      <c r="I29" s="214"/>
+      <c r="H29" s="101"/>
+      <c r="I29" s="97"/>
       <c r="J29" s="18"/>
       <c r="N29" s="18"/>
       <c r="O29" s="18"/>
@@ -4846,8 +4909,8 @@
       <c r="D30" s="13"/>
       <c r="E30" s="33"/>
       <c r="F30" s="33"/>
-      <c r="G30" s="89"/>
-      <c r="H30" s="89"/>
+      <c r="G30" s="112"/>
+      <c r="H30" s="112"/>
       <c r="I30" s="13"/>
       <c r="J30" s="13"/>
       <c r="K30" s="13"/>
@@ -4869,16 +4932,16 @@
       <c r="AA30" s="13"/>
     </row>
     <row r="31" spans="2:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B31" s="69" t="s">
+      <c r="B31" s="168" t="s">
         <v>35</v>
       </c>
-      <c r="C31" s="70"/>
-      <c r="D31" s="70"/>
-      <c r="E31" s="70"/>
-      <c r="F31" s="70"/>
-      <c r="G31" s="70"/>
-      <c r="H31" s="70"/>
-      <c r="I31" s="71"/>
+      <c r="C31" s="169"/>
+      <c r="D31" s="169"/>
+      <c r="E31" s="169"/>
+      <c r="F31" s="169"/>
+      <c r="G31" s="169"/>
+      <c r="H31" s="169"/>
+      <c r="I31" s="170"/>
       <c r="J31" s="7"/>
       <c r="K31" s="7"/>
       <c r="L31" s="7"/>
@@ -4900,18 +4963,18 @@
       <c r="AB31" s="7"/>
     </row>
     <row r="32" spans="2:28" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B32" s="215" t="s">
+      <c r="B32" s="115" t="s">
         <v>36</v>
       </c>
-      <c r="C32" s="76"/>
-      <c r="D32" s="76"/>
-      <c r="E32" s="76"/>
-      <c r="F32" s="216"/>
-      <c r="G32" s="75" t="s">
+      <c r="C32" s="116"/>
+      <c r="D32" s="116"/>
+      <c r="E32" s="116"/>
+      <c r="F32" s="117"/>
+      <c r="G32" s="231" t="s">
         <v>37</v>
       </c>
-      <c r="H32" s="76"/>
-      <c r="I32" s="77"/>
+      <c r="H32" s="116"/>
+      <c r="I32" s="232"/>
       <c r="J32" s="7"/>
       <c r="K32" s="7"/>
       <c r="L32" s="7"/>
@@ -4933,18 +4996,18 @@
       <c r="AB32" s="7"/>
     </row>
     <row r="33" spans="2:28" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B33" s="72" t="s">
+      <c r="B33" s="228" t="s">
         <v>104</v>
       </c>
-      <c r="C33" s="73"/>
-      <c r="D33" s="73"/>
-      <c r="E33" s="73"/>
-      <c r="F33" s="74"/>
-      <c r="G33" s="78" t="s">
+      <c r="C33" s="229"/>
+      <c r="D33" s="229"/>
+      <c r="E33" s="229"/>
+      <c r="F33" s="230"/>
+      <c r="G33" s="233" t="s">
         <v>105</v>
       </c>
-      <c r="H33" s="73"/>
-      <c r="I33" s="79"/>
+      <c r="H33" s="229"/>
+      <c r="I33" s="234"/>
       <c r="J33" s="7"/>
       <c r="K33" s="7"/>
       <c r="L33" s="7"/>
@@ -4971,8 +5034,8 @@
       <c r="D34" s="13"/>
       <c r="E34" s="33"/>
       <c r="F34" s="33"/>
-      <c r="G34" s="89"/>
-      <c r="H34" s="89"/>
+      <c r="G34" s="112"/>
+      <c r="H34" s="112"/>
       <c r="I34" s="13"/>
       <c r="J34" s="13"/>
       <c r="K34" s="13"/>
@@ -4994,16 +5057,16 @@
       <c r="AA34" s="13"/>
     </row>
     <row r="35" spans="2:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B35" s="145" t="s">
+      <c r="B35" s="183" t="s">
         <v>38</v>
       </c>
-      <c r="C35" s="146"/>
-      <c r="D35" s="146"/>
-      <c r="E35" s="146"/>
-      <c r="F35" s="146"/>
-      <c r="G35" s="146"/>
-      <c r="H35" s="146"/>
-      <c r="I35" s="147"/>
+      <c r="C35" s="184"/>
+      <c r="D35" s="184"/>
+      <c r="E35" s="184"/>
+      <c r="F35" s="184"/>
+      <c r="G35" s="184"/>
+      <c r="H35" s="184"/>
+      <c r="I35" s="185"/>
       <c r="J35" s="39"/>
       <c r="K35" s="19"/>
       <c r="L35" s="19"/>
@@ -5027,19 +5090,19 @@
       <c r="B36" s="41" t="s">
         <v>39</v>
       </c>
-      <c r="C36" s="150" t="s">
+      <c r="C36" s="192" t="s">
         <v>40</v>
       </c>
-      <c r="D36" s="151"/>
-      <c r="E36" s="151"/>
-      <c r="F36" s="152"/>
+      <c r="D36" s="193"/>
+      <c r="E36" s="193"/>
+      <c r="F36" s="194"/>
       <c r="G36" s="41" t="s">
         <v>39</v>
       </c>
-      <c r="H36" s="148" t="s">
+      <c r="H36" s="190" t="s">
         <v>41</v>
       </c>
-      <c r="I36" s="149"/>
+      <c r="I36" s="191"/>
       <c r="J36" s="40"/>
       <c r="K36" s="19"/>
       <c r="L36" s="19"/>
@@ -5060,18 +5123,18 @@
       <c r="AA36" s="20"/>
     </row>
     <row r="37" spans="2:28" s="11" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B37" s="100" t="s">
+      <c r="B37" s="177" t="s">
         <v>42</v>
       </c>
-      <c r="C37" s="104"/>
-      <c r="D37" s="105"/>
-      <c r="E37" s="105"/>
-      <c r="F37" s="106"/>
-      <c r="G37" s="100" t="s">
+      <c r="C37" s="210"/>
+      <c r="D37" s="211"/>
+      <c r="E37" s="211"/>
+      <c r="F37" s="212"/>
+      <c r="G37" s="177" t="s">
         <v>43</v>
       </c>
-      <c r="H37" s="123"/>
-      <c r="I37" s="124"/>
+      <c r="H37" s="186"/>
+      <c r="I37" s="187"/>
       <c r="J37" s="39"/>
       <c r="K37" s="16"/>
       <c r="L37" s="18"/>
@@ -5090,14 +5153,14 @@
       <c r="AB37" s="12"/>
     </row>
     <row r="38" spans="2:28" s="11" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B38" s="127"/>
-      <c r="C38" s="107"/>
-      <c r="D38" s="89"/>
-      <c r="E38" s="89"/>
-      <c r="F38" s="108"/>
-      <c r="G38" s="101"/>
-      <c r="H38" s="125"/>
-      <c r="I38" s="126"/>
+      <c r="B38" s="226"/>
+      <c r="C38" s="213"/>
+      <c r="D38" s="112"/>
+      <c r="E38" s="112"/>
+      <c r="F38" s="214"/>
+      <c r="G38" s="207"/>
+      <c r="H38" s="188"/>
+      <c r="I38" s="189"/>
       <c r="J38" s="39"/>
       <c r="K38" s="16"/>
       <c r="L38" s="18"/>
@@ -5115,16 +5178,16 @@
       <c r="AB38" s="12"/>
     </row>
     <row r="39" spans="2:28" s="11" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B39" s="127"/>
-      <c r="C39" s="107"/>
-      <c r="D39" s="89"/>
-      <c r="E39" s="89"/>
-      <c r="F39" s="108"/>
-      <c r="G39" s="100" t="s">
+      <c r="B39" s="226"/>
+      <c r="C39" s="213"/>
+      <c r="D39" s="112"/>
+      <c r="E39" s="112"/>
+      <c r="F39" s="214"/>
+      <c r="G39" s="177" t="s">
         <v>44</v>
       </c>
-      <c r="H39" s="123"/>
-      <c r="I39" s="124"/>
+      <c r="H39" s="186"/>
+      <c r="I39" s="187"/>
       <c r="J39" s="39"/>
       <c r="K39" s="16"/>
       <c r="L39" s="18"/>
@@ -5143,14 +5206,14 @@
       <c r="AB39" s="12"/>
     </row>
     <row r="40" spans="2:28" s="11" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B40" s="128"/>
-      <c r="C40" s="109"/>
-      <c r="D40" s="110"/>
-      <c r="E40" s="110"/>
-      <c r="F40" s="111"/>
-      <c r="G40" s="101"/>
-      <c r="H40" s="125"/>
-      <c r="I40" s="126"/>
+      <c r="B40" s="227"/>
+      <c r="C40" s="215"/>
+      <c r="D40" s="216"/>
+      <c r="E40" s="216"/>
+      <c r="F40" s="217"/>
+      <c r="G40" s="207"/>
+      <c r="H40" s="188"/>
+      <c r="I40" s="189"/>
       <c r="J40" s="39"/>
       <c r="K40" s="16"/>
       <c r="L40" s="18"/>
@@ -5169,18 +5232,18 @@
       <c r="AB40" s="12"/>
     </row>
     <row r="41" spans="2:28" s="11" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B41" s="118" t="s">
+      <c r="B41" s="224" t="s">
         <v>45</v>
       </c>
-      <c r="C41" s="112"/>
-      <c r="D41" s="113"/>
-      <c r="E41" s="113"/>
-      <c r="F41" s="114"/>
-      <c r="G41" s="100" t="s">
+      <c r="C41" s="218"/>
+      <c r="D41" s="219"/>
+      <c r="E41" s="219"/>
+      <c r="F41" s="220"/>
+      <c r="G41" s="177" t="s">
         <v>46</v>
       </c>
-      <c r="H41" s="141"/>
-      <c r="I41" s="142"/>
+      <c r="H41" s="179"/>
+      <c r="I41" s="180"/>
       <c r="J41" s="56"/>
       <c r="K41" s="16"/>
       <c r="L41" s="17"/>
@@ -5202,14 +5265,14 @@
       <c r="AB41" s="12"/>
     </row>
     <row r="42" spans="2:28" s="38" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B42" s="119"/>
-      <c r="C42" s="115"/>
-      <c r="D42" s="116"/>
-      <c r="E42" s="116"/>
-      <c r="F42" s="117"/>
-      <c r="G42" s="140"/>
-      <c r="H42" s="143"/>
-      <c r="I42" s="144"/>
+      <c r="B42" s="225"/>
+      <c r="C42" s="221"/>
+      <c r="D42" s="222"/>
+      <c r="E42" s="222"/>
+      <c r="F42" s="223"/>
+      <c r="G42" s="178"/>
+      <c r="H42" s="181"/>
+      <c r="I42" s="182"/>
       <c r="J42" s="56"/>
       <c r="K42" s="16"/>
       <c r="L42" s="17"/>
@@ -5236,8 +5299,8 @@
       <c r="D43" s="43"/>
       <c r="E43" s="43"/>
       <c r="F43" s="43"/>
-      <c r="G43" s="102"/>
-      <c r="H43" s="103"/>
+      <c r="G43" s="208"/>
+      <c r="H43" s="209"/>
       <c r="I43" s="43"/>
       <c r="J43" s="56"/>
       <c r="K43" s="16"/>
@@ -5260,16 +5323,16 @@
       <c r="AB43" s="12"/>
     </row>
     <row r="44" spans="2:28" s="11" customFormat="1" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B44" s="98" t="s">
+      <c r="B44" s="205" t="s">
         <v>47</v>
       </c>
-      <c r="C44" s="98"/>
-      <c r="D44" s="98"/>
-      <c r="E44" s="98"/>
-      <c r="F44" s="98"/>
-      <c r="G44" s="98"/>
-      <c r="H44" s="98"/>
-      <c r="I44" s="99"/>
+      <c r="C44" s="205"/>
+      <c r="D44" s="205"/>
+      <c r="E44" s="205"/>
+      <c r="F44" s="205"/>
+      <c r="G44" s="205"/>
+      <c r="H44" s="205"/>
+      <c r="I44" s="206"/>
       <c r="J44" s="16"/>
       <c r="K44" s="16"/>
       <c r="L44" s="17"/>
@@ -5291,24 +5354,24 @@
       <c r="AB44" s="12"/>
     </row>
     <row r="45" spans="2:28" ht="68.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B45" s="223" t="s">
+      <c r="B45" s="124" t="s">
         <v>48</v>
       </c>
-      <c r="C45" s="207"/>
-      <c r="D45" s="204" t="s">
+      <c r="C45" s="109"/>
+      <c r="D45" s="106" t="s">
         <v>49</v>
       </c>
-      <c r="E45" s="205"/>
-      <c r="F45" s="208" t="s">
+      <c r="E45" s="107"/>
+      <c r="F45" s="110" t="s">
         <v>50</v>
       </c>
-      <c r="G45" s="208" t="s">
+      <c r="G45" s="110" t="s">
         <v>51</v>
       </c>
-      <c r="H45" s="221" t="s">
+      <c r="H45" s="122" t="s">
         <v>52</v>
       </c>
-      <c r="I45" s="139" t="s">
+      <c r="I45" s="176" t="s">
         <v>53</v>
       </c>
       <c r="J45" s="16"/>
@@ -5331,14 +5394,14 @@
       <c r="AA45" s="16"/>
     </row>
     <row r="46" spans="2:28" ht="66.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B46" s="223"/>
-      <c r="C46" s="207"/>
-      <c r="D46" s="206"/>
-      <c r="E46" s="207"/>
-      <c r="F46" s="209"/>
-      <c r="G46" s="208"/>
-      <c r="H46" s="222"/>
-      <c r="I46" s="139"/>
+      <c r="B46" s="124"/>
+      <c r="C46" s="109"/>
+      <c r="D46" s="108"/>
+      <c r="E46" s="109"/>
+      <c r="F46" s="111"/>
+      <c r="G46" s="110"/>
+      <c r="H46" s="123"/>
+      <c r="I46" s="176"/>
       <c r="J46" s="16"/>
       <c r="K46" s="16"/>
       <c r="L46" s="16"/>
@@ -5359,14 +5422,14 @@
       <c r="AA46" s="16"/>
     </row>
     <row r="47" spans="2:28" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B47" s="213"/>
-      <c r="C47" s="120"/>
-      <c r="D47" s="120"/>
-      <c r="E47" s="120"/>
-      <c r="F47" s="121"/>
-      <c r="G47" s="120"/>
-      <c r="H47" s="120"/>
-      <c r="I47" s="122"/>
+      <c r="B47" s="98"/>
+      <c r="C47" s="99"/>
+      <c r="D47" s="283"/>
+      <c r="E47" s="283"/>
+      <c r="F47" s="102"/>
+      <c r="G47" s="99"/>
+      <c r="H47" s="287"/>
+      <c r="I47" s="285"/>
       <c r="J47" s="18"/>
       <c r="K47" s="16"/>
       <c r="L47" s="16"/>
@@ -5387,14 +5450,14 @@
       <c r="AA47" s="16"/>
     </row>
     <row r="48" spans="2:28" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B48" s="213"/>
-      <c r="C48" s="120"/>
-      <c r="D48" s="120"/>
-      <c r="E48" s="120"/>
-      <c r="F48" s="121"/>
-      <c r="G48" s="120"/>
-      <c r="H48" s="120"/>
-      <c r="I48" s="122"/>
+      <c r="B48" s="98"/>
+      <c r="C48" s="99"/>
+      <c r="D48" s="283"/>
+      <c r="E48" s="283"/>
+      <c r="F48" s="102"/>
+      <c r="G48" s="99"/>
+      <c r="H48" s="287"/>
+      <c r="I48" s="285"/>
       <c r="J48" s="18"/>
       <c r="K48" s="16"/>
       <c r="L48" s="16"/>
@@ -5415,14 +5478,14 @@
       <c r="AA48" s="16"/>
     </row>
     <row r="49" spans="2:28" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B49" s="213"/>
-      <c r="C49" s="120"/>
-      <c r="D49" s="120"/>
-      <c r="E49" s="120"/>
-      <c r="F49" s="121"/>
-      <c r="G49" s="120"/>
-      <c r="H49" s="120"/>
-      <c r="I49" s="122"/>
+      <c r="B49" s="98"/>
+      <c r="C49" s="99"/>
+      <c r="D49" s="283"/>
+      <c r="E49" s="283"/>
+      <c r="F49" s="102"/>
+      <c r="G49" s="99"/>
+      <c r="H49" s="287"/>
+      <c r="I49" s="285"/>
       <c r="J49" s="18"/>
       <c r="K49" s="16"/>
       <c r="L49" s="16"/>
@@ -5443,14 +5506,14 @@
       <c r="AA49" s="16"/>
     </row>
     <row r="50" spans="2:28" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B50" s="213"/>
-      <c r="C50" s="120"/>
-      <c r="D50" s="120"/>
-      <c r="E50" s="120"/>
-      <c r="F50" s="121"/>
-      <c r="G50" s="120"/>
-      <c r="H50" s="120"/>
-      <c r="I50" s="122"/>
+      <c r="B50" s="98"/>
+      <c r="C50" s="99"/>
+      <c r="D50" s="283"/>
+      <c r="E50" s="283"/>
+      <c r="F50" s="102"/>
+      <c r="G50" s="99"/>
+      <c r="H50" s="287"/>
+      <c r="I50" s="285"/>
       <c r="J50" s="18"/>
       <c r="K50" s="16"/>
       <c r="L50" s="16"/>
@@ -5471,14 +5534,14 @@
       <c r="AA50" s="16"/>
     </row>
     <row r="51" spans="2:28" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B51" s="213"/>
-      <c r="C51" s="120"/>
-      <c r="D51" s="120"/>
-      <c r="E51" s="120"/>
-      <c r="F51" s="121"/>
-      <c r="G51" s="120"/>
-      <c r="H51" s="120"/>
-      <c r="I51" s="122"/>
+      <c r="B51" s="98"/>
+      <c r="C51" s="99"/>
+      <c r="D51" s="283"/>
+      <c r="E51" s="283"/>
+      <c r="F51" s="102"/>
+      <c r="G51" s="99"/>
+      <c r="H51" s="287"/>
+      <c r="I51" s="285"/>
       <c r="J51" s="18"/>
       <c r="K51" s="16"/>
       <c r="L51" s="16"/>
@@ -5499,14 +5562,14 @@
       <c r="AA51" s="16"/>
     </row>
     <row r="52" spans="2:28" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B52" s="213"/>
-      <c r="C52" s="120"/>
-      <c r="D52" s="120"/>
-      <c r="E52" s="120"/>
-      <c r="F52" s="121"/>
-      <c r="G52" s="120"/>
-      <c r="H52" s="120"/>
-      <c r="I52" s="122"/>
+      <c r="B52" s="98"/>
+      <c r="C52" s="99"/>
+      <c r="D52" s="283"/>
+      <c r="E52" s="283"/>
+      <c r="F52" s="102"/>
+      <c r="G52" s="99"/>
+      <c r="H52" s="287"/>
+      <c r="I52" s="285"/>
       <c r="J52" s="18"/>
       <c r="K52" s="16"/>
       <c r="L52" s="16"/>
@@ -5527,14 +5590,14 @@
       <c r="AA52" s="16"/>
     </row>
     <row r="53" spans="2:28" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B53" s="213"/>
-      <c r="C53" s="120"/>
-      <c r="D53" s="120"/>
-      <c r="E53" s="120"/>
-      <c r="F53" s="121"/>
-      <c r="G53" s="120"/>
-      <c r="H53" s="120"/>
-      <c r="I53" s="122"/>
+      <c r="B53" s="98"/>
+      <c r="C53" s="99"/>
+      <c r="D53" s="283"/>
+      <c r="E53" s="283"/>
+      <c r="F53" s="102"/>
+      <c r="G53" s="99"/>
+      <c r="H53" s="287"/>
+      <c r="I53" s="285"/>
       <c r="J53" s="18"/>
       <c r="K53" s="16"/>
       <c r="L53" s="16"/>
@@ -5555,14 +5618,14 @@
       <c r="AA53" s="16"/>
     </row>
     <row r="54" spans="2:28" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B54" s="213"/>
-      <c r="C54" s="120"/>
-      <c r="D54" s="120"/>
-      <c r="E54" s="120"/>
-      <c r="F54" s="121"/>
-      <c r="G54" s="120"/>
-      <c r="H54" s="120"/>
-      <c r="I54" s="122"/>
+      <c r="B54" s="98"/>
+      <c r="C54" s="99"/>
+      <c r="D54" s="283"/>
+      <c r="E54" s="283"/>
+      <c r="F54" s="102"/>
+      <c r="G54" s="99"/>
+      <c r="H54" s="287"/>
+      <c r="I54" s="285"/>
       <c r="J54" s="18"/>
       <c r="K54" s="16"/>
       <c r="L54" s="16"/>
@@ -5583,14 +5646,14 @@
       <c r="AA54" s="16"/>
     </row>
     <row r="55" spans="2:28" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B55" s="213"/>
-      <c r="C55" s="120"/>
-      <c r="D55" s="120"/>
-      <c r="E55" s="120"/>
-      <c r="F55" s="121"/>
-      <c r="G55" s="120"/>
-      <c r="H55" s="120"/>
-      <c r="I55" s="122"/>
+      <c r="B55" s="98"/>
+      <c r="C55" s="99"/>
+      <c r="D55" s="283"/>
+      <c r="E55" s="283"/>
+      <c r="F55" s="102"/>
+      <c r="G55" s="99"/>
+      <c r="H55" s="287"/>
+      <c r="I55" s="285"/>
       <c r="J55" s="18"/>
       <c r="K55" s="16"/>
       <c r="L55" s="16"/>
@@ -5611,14 +5674,14 @@
       <c r="AA55" s="16"/>
     </row>
     <row r="56" spans="2:28" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B56" s="157"/>
-      <c r="C56" s="158"/>
-      <c r="D56" s="158"/>
-      <c r="E56" s="158"/>
-      <c r="F56" s="229"/>
-      <c r="G56" s="158"/>
-      <c r="H56" s="158"/>
-      <c r="I56" s="214"/>
+      <c r="B56" s="100"/>
+      <c r="C56" s="101"/>
+      <c r="D56" s="284"/>
+      <c r="E56" s="284"/>
+      <c r="F56" s="103"/>
+      <c r="G56" s="101"/>
+      <c r="H56" s="288"/>
+      <c r="I56" s="286"/>
       <c r="J56" s="18"/>
       <c r="K56" s="16"/>
       <c r="L56" s="16"/>
@@ -5644,8 +5707,8 @@
       <c r="D57" s="18"/>
       <c r="E57" s="23"/>
       <c r="F57" s="23"/>
-      <c r="G57" s="201"/>
-      <c r="H57" s="201"/>
+      <c r="G57" s="113"/>
+      <c r="H57" s="113"/>
       <c r="I57" s="18"/>
       <c r="J57" s="18"/>
       <c r="K57" s="16"/>
@@ -5667,16 +5730,16 @@
       <c r="AA57" s="16"/>
     </row>
     <row r="58" spans="2:28" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B58" s="210" t="s">
+      <c r="B58" s="76" t="s">
         <v>54</v>
       </c>
-      <c r="C58" s="211"/>
-      <c r="D58" s="211"/>
-      <c r="E58" s="211"/>
-      <c r="F58" s="211"/>
-      <c r="G58" s="211"/>
-      <c r="H58" s="211"/>
-      <c r="I58" s="212"/>
+      <c r="C58" s="77"/>
+      <c r="D58" s="77"/>
+      <c r="E58" s="77"/>
+      <c r="F58" s="77"/>
+      <c r="G58" s="77"/>
+      <c r="H58" s="77"/>
+      <c r="I58" s="78"/>
       <c r="J58" s="18"/>
       <c r="K58" s="16"/>
       <c r="L58" s="16"/>
@@ -5697,16 +5760,16 @@
       <c r="AA58" s="16"/>
     </row>
     <row r="59" spans="2:28" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B59" s="81" t="s">
+      <c r="B59" s="235" t="s">
         <v>55</v>
       </c>
-      <c r="C59" s="82"/>
-      <c r="D59" s="82"/>
-      <c r="E59" s="82"/>
-      <c r="F59" s="82"/>
-      <c r="G59" s="82"/>
-      <c r="H59" s="82"/>
-      <c r="I59" s="83"/>
+      <c r="C59" s="236"/>
+      <c r="D59" s="236"/>
+      <c r="E59" s="236"/>
+      <c r="F59" s="236"/>
+      <c r="G59" s="236"/>
+      <c r="H59" s="236"/>
+      <c r="I59" s="237"/>
       <c r="J59" s="19"/>
       <c r="K59" s="19"/>
       <c r="L59" s="19"/>
@@ -5727,16 +5790,16 @@
       <c r="AA59" s="19"/>
     </row>
     <row r="60" spans="2:28" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B60" s="210" t="s">
+      <c r="B60" s="76" t="s">
         <v>56</v>
       </c>
-      <c r="C60" s="211"/>
-      <c r="D60" s="211"/>
-      <c r="E60" s="211"/>
-      <c r="F60" s="211"/>
-      <c r="G60" s="211"/>
-      <c r="H60" s="211"/>
-      <c r="I60" s="212"/>
+      <c r="C60" s="77"/>
+      <c r="D60" s="77"/>
+      <c r="E60" s="77"/>
+      <c r="F60" s="77"/>
+      <c r="G60" s="77"/>
+      <c r="H60" s="77"/>
+      <c r="I60" s="78"/>
       <c r="J60" s="19"/>
       <c r="K60" s="19"/>
       <c r="L60" s="19"/>
@@ -5757,16 +5820,16 @@
       <c r="AA60" s="19"/>
     </row>
     <row r="61" spans="2:28" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B61" s="237" t="s">
+      <c r="B61" s="80" t="s">
         <v>57</v>
       </c>
-      <c r="C61" s="238"/>
-      <c r="D61" s="238"/>
-      <c r="E61" s="238"/>
-      <c r="F61" s="238"/>
-      <c r="G61" s="238"/>
-      <c r="H61" s="238"/>
-      <c r="I61" s="239"/>
+      <c r="C61" s="81"/>
+      <c r="D61" s="81"/>
+      <c r="E61" s="81"/>
+      <c r="F61" s="81"/>
+      <c r="G61" s="81"/>
+      <c r="H61" s="81"/>
+      <c r="I61" s="82"/>
       <c r="J61" s="22"/>
       <c r="K61" s="22"/>
       <c r="L61" s="22"/>
@@ -5787,14 +5850,14 @@
       <c r="AA61" s="22"/>
     </row>
     <row r="62" spans="2:28" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B62" s="240"/>
-      <c r="C62" s="241"/>
-      <c r="D62" s="241"/>
-      <c r="E62" s="241"/>
-      <c r="F62" s="241"/>
-      <c r="G62" s="241"/>
-      <c r="H62" s="241"/>
-      <c r="I62" s="242"/>
+      <c r="B62" s="83"/>
+      <c r="C62" s="84"/>
+      <c r="D62" s="84"/>
+      <c r="E62" s="84"/>
+      <c r="F62" s="84"/>
+      <c r="G62" s="84"/>
+      <c r="H62" s="84"/>
+      <c r="I62" s="85"/>
       <c r="J62" s="22"/>
       <c r="K62" s="22"/>
       <c r="L62" s="22"/>
@@ -5815,16 +5878,16 @@
       <c r="AA62" s="22"/>
     </row>
     <row r="63" spans="2:28" s="46" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B63" s="240" t="s">
+      <c r="B63" s="83" t="s">
         <v>58</v>
       </c>
-      <c r="C63" s="241"/>
-      <c r="D63" s="241"/>
-      <c r="E63" s="241"/>
-      <c r="F63" s="241"/>
-      <c r="G63" s="241"/>
-      <c r="H63" s="241"/>
-      <c r="I63" s="242"/>
+      <c r="C63" s="84"/>
+      <c r="D63" s="84"/>
+      <c r="E63" s="84"/>
+      <c r="F63" s="84"/>
+      <c r="G63" s="84"/>
+      <c r="H63" s="84"/>
+      <c r="I63" s="85"/>
       <c r="J63" s="44"/>
       <c r="K63" s="44"/>
       <c r="L63" s="44"/>
@@ -5846,16 +5909,16 @@
       <c r="AB63" s="45"/>
     </row>
     <row r="64" spans="2:28" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B64" s="243" t="s">
+      <c r="B64" s="88" t="s">
         <v>59</v>
       </c>
-      <c r="C64" s="244"/>
-      <c r="D64" s="244"/>
-      <c r="E64" s="244"/>
-      <c r="F64" s="244"/>
-      <c r="G64" s="244"/>
-      <c r="H64" s="244"/>
-      <c r="I64" s="245"/>
+      <c r="C64" s="89"/>
+      <c r="D64" s="89"/>
+      <c r="E64" s="89"/>
+      <c r="F64" s="89"/>
+      <c r="G64" s="89"/>
+      <c r="H64" s="89"/>
+      <c r="I64" s="90"/>
       <c r="J64" s="22"/>
       <c r="K64" s="22"/>
       <c r="L64" s="22"/>
@@ -5879,19 +5942,19 @@
       <c r="B65" s="50" t="s">
         <v>60</v>
       </c>
-      <c r="C65" s="129" t="s">
+      <c r="C65" s="86" t="s">
         <v>61</v>
       </c>
-      <c r="D65" s="129"/>
-      <c r="E65" s="129" t="s">
+      <c r="D65" s="86"/>
+      <c r="E65" s="86" t="s">
         <v>62</v>
       </c>
-      <c r="F65" s="129"/>
-      <c r="G65" s="93"/>
-      <c r="H65" s="129" t="s">
+      <c r="F65" s="86"/>
+      <c r="G65" s="245"/>
+      <c r="H65" s="86" t="s">
         <v>63</v>
       </c>
-      <c r="I65" s="95"/>
+      <c r="I65" s="247"/>
       <c r="J65" s="16"/>
       <c r="K65" s="16"/>
       <c r="L65" s="16"/>
@@ -5914,13 +5977,13 @@
     </row>
     <row r="66" spans="2:28" ht="32.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B66" s="51"/>
-      <c r="C66" s="247"/>
-      <c r="D66" s="247"/>
-      <c r="E66" s="130"/>
-      <c r="F66" s="130"/>
-      <c r="G66" s="94"/>
-      <c r="H66" s="130"/>
-      <c r="I66" s="96"/>
+      <c r="C66" s="93"/>
+      <c r="D66" s="93"/>
+      <c r="E66" s="87"/>
+      <c r="F66" s="87"/>
+      <c r="G66" s="246"/>
+      <c r="H66" s="87"/>
+      <c r="I66" s="248"/>
       <c r="J66" s="16"/>
       <c r="K66" s="16"/>
       <c r="L66" s="16"/>
@@ -5947,8 +6010,8 @@
       <c r="D67" s="17"/>
       <c r="E67" s="34"/>
       <c r="F67" s="34"/>
-      <c r="G67" s="246"/>
-      <c r="H67" s="246"/>
+      <c r="G67" s="91"/>
+      <c r="H67" s="91"/>
       <c r="I67" s="17"/>
       <c r="J67" s="16"/>
       <c r="K67" s="16"/>
@@ -5971,16 +6034,16 @@
       <c r="AB67" s="16"/>
     </row>
     <row r="68" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B68" s="236" t="s">
+      <c r="B68" s="79" t="s">
         <v>64</v>
       </c>
-      <c r="C68" s="236"/>
-      <c r="D68" s="236"/>
-      <c r="E68" s="236"/>
-      <c r="F68" s="236"/>
-      <c r="G68" s="236"/>
-      <c r="H68" s="236"/>
-      <c r="I68" s="236"/>
+      <c r="C68" s="79"/>
+      <c r="D68" s="79"/>
+      <c r="E68" s="79"/>
+      <c r="F68" s="79"/>
+      <c r="G68" s="79"/>
+      <c r="H68" s="79"/>
+      <c r="I68" s="79"/>
       <c r="J68" s="16"/>
       <c r="K68" s="16"/>
       <c r="L68" s="16"/>
@@ -6007,8 +6070,8 @@
       <c r="D69" s="15"/>
       <c r="E69" s="35"/>
       <c r="F69" s="35"/>
-      <c r="G69" s="87"/>
-      <c r="H69" s="87"/>
+      <c r="G69" s="92"/>
+      <c r="H69" s="92"/>
       <c r="I69" s="15"/>
       <c r="J69" s="16"/>
       <c r="K69" s="16"/>
@@ -6031,13 +6094,13 @@
       <c r="AB69" s="16"/>
     </row>
     <row r="70" spans="2:28" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B70" s="87"/>
-      <c r="C70" s="87"/>
-      <c r="D70" s="87"/>
-      <c r="E70" s="87"/>
+      <c r="B70" s="92"/>
+      <c r="C70" s="92"/>
+      <c r="D70" s="92"/>
+      <c r="E70" s="92"/>
       <c r="F70" s="35"/>
-      <c r="G70" s="87"/>
-      <c r="H70" s="87"/>
+      <c r="G70" s="92"/>
+      <c r="H70" s="92"/>
       <c r="I70" s="15"/>
       <c r="J70" s="16"/>
       <c r="K70" s="16"/>
@@ -6060,10 +6123,10 @@
       <c r="AB70" s="16"/>
     </row>
     <row r="71" spans="2:28" ht="36" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B71" s="88"/>
-      <c r="C71" s="88"/>
-      <c r="D71" s="88"/>
-      <c r="E71" s="88"/>
+      <c r="B71" s="241"/>
+      <c r="C71" s="241"/>
+      <c r="D71" s="241"/>
+      <c r="E71" s="241"/>
       <c r="F71" s="26"/>
       <c r="H71" s="57"/>
       <c r="I71" s="16"/>
@@ -6088,12 +6151,12 @@
       <c r="AB71" s="16"/>
     </row>
     <row r="72" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B72" s="228" t="s">
+      <c r="B72" s="75" t="s">
         <v>65</v>
       </c>
-      <c r="C72" s="228"/>
-      <c r="D72" s="228"/>
-      <c r="E72" s="228"/>
+      <c r="C72" s="75"/>
+      <c r="D72" s="75"/>
+      <c r="E72" s="75"/>
       <c r="F72" s="17"/>
       <c r="H72" s="17" t="s">
         <v>66</v>
@@ -6125,8 +6188,8 @@
       <c r="D73" s="16"/>
       <c r="E73" s="26"/>
       <c r="F73" s="26"/>
-      <c r="G73" s="80"/>
-      <c r="H73" s="97"/>
+      <c r="G73" s="95"/>
+      <c r="H73" s="204"/>
       <c r="I73" s="16"/>
       <c r="J73" s="16"/>
       <c r="K73" s="16"/>
@@ -6149,13 +6212,13 @@
       <c r="AB73" s="16"/>
     </row>
     <row r="74" spans="2:28" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B74" s="91"/>
-      <c r="C74" s="91"/>
-      <c r="D74" s="91"/>
-      <c r="E74" s="91"/>
+      <c r="B74" s="243"/>
+      <c r="C74" s="243"/>
+      <c r="D74" s="243"/>
+      <c r="E74" s="243"/>
       <c r="F74" s="26"/>
-      <c r="H74" s="89"/>
-      <c r="I74" s="89"/>
+      <c r="H74" s="112"/>
+      <c r="I74" s="112"/>
       <c r="J74" s="16"/>
       <c r="K74" s="16"/>
       <c r="L74" s="16"/>
@@ -6177,13 +6240,13 @@
       <c r="AB74" s="16"/>
     </row>
     <row r="75" spans="2:28" ht="38.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B75" s="92"/>
-      <c r="C75" s="92"/>
-      <c r="D75" s="92"/>
-      <c r="E75" s="92"/>
+      <c r="B75" s="244"/>
+      <c r="C75" s="244"/>
+      <c r="D75" s="244"/>
+      <c r="E75" s="244"/>
       <c r="F75" s="26"/>
-      <c r="H75" s="90"/>
-      <c r="I75" s="90"/>
+      <c r="H75" s="242"/>
+      <c r="I75" s="242"/>
       <c r="J75" s="16"/>
       <c r="K75" s="16"/>
       <c r="L75" s="16"/>
@@ -6212,10 +6275,10 @@
       <c r="D76" s="24"/>
       <c r="E76" s="26"/>
       <c r="F76" s="26"/>
-      <c r="H76" s="228" t="s">
+      <c r="H76" s="75" t="s">
         <v>68</v>
       </c>
-      <c r="I76" s="228"/>
+      <c r="I76" s="75"/>
       <c r="J76" s="16"/>
       <c r="K76" s="16"/>
       <c r="L76" s="16"/>
@@ -6242,8 +6305,8 @@
       <c r="D77" s="24"/>
       <c r="E77" s="26"/>
       <c r="F77" s="26"/>
-      <c r="G77" s="80"/>
-      <c r="H77" s="246"/>
+      <c r="G77" s="95"/>
+      <c r="H77" s="91"/>
       <c r="I77" s="17"/>
       <c r="J77" s="16"/>
       <c r="K77" s="16"/>
@@ -6266,16 +6329,16 @@
       <c r="AB77" s="16"/>
     </row>
     <row r="78" spans="2:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B78" s="248" t="s">
+      <c r="B78" s="94" t="s">
         <v>69</v>
       </c>
-      <c r="C78" s="248"/>
-      <c r="D78" s="248"/>
-      <c r="E78" s="248"/>
-      <c r="F78" s="248"/>
-      <c r="G78" s="248"/>
-      <c r="H78" s="248"/>
-      <c r="I78" s="248"/>
+      <c r="C78" s="94"/>
+      <c r="D78" s="94"/>
+      <c r="E78" s="94"/>
+      <c r="F78" s="94"/>
+      <c r="G78" s="94"/>
+      <c r="H78" s="94"/>
+      <c r="I78" s="94"/>
       <c r="J78" s="16"/>
       <c r="K78" s="16"/>
       <c r="L78" s="16"/>
@@ -6297,14 +6360,14 @@
       <c r="AB78" s="16"/>
     </row>
     <row r="79" spans="2:28" x14ac:dyDescent="0.25">
-      <c r="B79" s="248"/>
-      <c r="C79" s="248"/>
-      <c r="D79" s="248"/>
-      <c r="E79" s="248"/>
-      <c r="F79" s="248"/>
-      <c r="G79" s="248"/>
-      <c r="H79" s="248"/>
-      <c r="I79" s="248"/>
+      <c r="B79" s="94"/>
+      <c r="C79" s="94"/>
+      <c r="D79" s="94"/>
+      <c r="E79" s="94"/>
+      <c r="F79" s="94"/>
+      <c r="G79" s="94"/>
+      <c r="H79" s="94"/>
+      <c r="I79" s="94"/>
       <c r="J79" s="16"/>
       <c r="K79" s="16"/>
       <c r="L79" s="16"/>
@@ -6331,8 +6394,8 @@
       <c r="D80" s="48"/>
       <c r="E80" s="48"/>
       <c r="F80" s="48"/>
-      <c r="G80" s="249"/>
-      <c r="H80" s="249"/>
+      <c r="G80" s="96"/>
+      <c r="H80" s="96"/>
       <c r="I80" s="48"/>
       <c r="J80" s="16"/>
       <c r="K80" s="16"/>
@@ -6355,16 +6418,16 @@
       <c r="AB80" s="16"/>
     </row>
     <row r="81" spans="2:28" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B81" s="230" t="s">
+      <c r="B81" s="69" t="s">
         <v>70</v>
       </c>
-      <c r="C81" s="231"/>
-      <c r="D81" s="231"/>
-      <c r="E81" s="231"/>
-      <c r="F81" s="231"/>
-      <c r="G81" s="231"/>
-      <c r="H81" s="231"/>
-      <c r="I81" s="232"/>
+      <c r="C81" s="70"/>
+      <c r="D81" s="70"/>
+      <c r="E81" s="70"/>
+      <c r="F81" s="70"/>
+      <c r="G81" s="70"/>
+      <c r="H81" s="70"/>
+      <c r="I81" s="71"/>
       <c r="J81" s="8"/>
       <c r="K81" s="7"/>
       <c r="L81" s="7"/>
@@ -6386,16 +6449,16 @@
       <c r="AB81" s="7"/>
     </row>
     <row r="82" spans="2:28" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B82" s="233" t="s">
+      <c r="B82" s="72" t="s">
         <v>71</v>
       </c>
-      <c r="C82" s="234"/>
-      <c r="D82" s="234"/>
-      <c r="E82" s="234"/>
-      <c r="F82" s="234"/>
-      <c r="G82" s="234"/>
-      <c r="H82" s="234"/>
-      <c r="I82" s="235"/>
+      <c r="C82" s="73"/>
+      <c r="D82" s="73"/>
+      <c r="E82" s="73"/>
+      <c r="F82" s="73"/>
+      <c r="G82" s="73"/>
+      <c r="H82" s="73"/>
+      <c r="I82" s="74"/>
       <c r="J82" s="8"/>
       <c r="K82" s="25"/>
       <c r="L82" s="7"/>
@@ -6417,18 +6480,18 @@
       <c r="AB82" s="7"/>
     </row>
     <row r="83" spans="2:28" s="8" customFormat="1" ht="249" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B83" s="84"/>
-      <c r="C83" s="85"/>
-      <c r="D83" s="85"/>
-      <c r="E83" s="85"/>
-      <c r="F83" s="85"/>
-      <c r="G83" s="85"/>
-      <c r="H83" s="85"/>
-      <c r="I83" s="86"/>
+      <c r="B83" s="238"/>
+      <c r="C83" s="239"/>
+      <c r="D83" s="239"/>
+      <c r="E83" s="239"/>
+      <c r="F83" s="239"/>
+      <c r="G83" s="239"/>
+      <c r="H83" s="239"/>
+      <c r="I83" s="240"/>
     </row>
     <row r="84" spans="2:28" hidden="1" x14ac:dyDescent="0.25">
-      <c r="G84" s="80"/>
-      <c r="H84" s="80"/>
+      <c r="G84" s="95"/>
+      <c r="H84" s="95"/>
       <c r="J84" s="8"/>
       <c r="K84" s="7"/>
       <c r="L84" s="7"/>
@@ -6450,159 +6513,234 @@
       <c r="AB84" s="7"/>
     </row>
     <row r="85" spans="2:28" hidden="1" x14ac:dyDescent="0.25">
-      <c r="G85" s="80"/>
-      <c r="H85" s="80"/>
+      <c r="G85" s="95"/>
+      <c r="H85" s="95"/>
     </row>
     <row r="86" spans="2:28" hidden="1" x14ac:dyDescent="0.25">
-      <c r="G86" s="80"/>
-      <c r="H86" s="80"/>
+      <c r="G86" s="95"/>
+      <c r="H86" s="95"/>
     </row>
     <row r="87" spans="2:28" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G87" s="80"/>
-      <c r="H87" s="80"/>
+      <c r="G87" s="95"/>
+      <c r="H87" s="95"/>
     </row>
     <row r="88" spans="2:28" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G88" s="80"/>
-      <c r="H88" s="80"/>
+      <c r="G88" s="95"/>
+      <c r="H88" s="95"/>
     </row>
     <row r="89" spans="2:28" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G89" s="80"/>
-      <c r="H89" s="80"/>
+      <c r="G89" s="95"/>
+      <c r="H89" s="95"/>
     </row>
     <row r="90" spans="2:28" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G90" s="80"/>
-      <c r="H90" s="80"/>
+      <c r="G90" s="95"/>
+      <c r="H90" s="95"/>
     </row>
     <row r="91" spans="2:28" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G91" s="80"/>
-      <c r="H91" s="80"/>
+      <c r="G91" s="95"/>
+      <c r="H91" s="95"/>
     </row>
     <row r="92" spans="2:28" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G92" s="80"/>
-      <c r="H92" s="80"/>
+      <c r="G92" s="95"/>
+      <c r="H92" s="95"/>
     </row>
     <row r="93" spans="2:28" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G93" s="80"/>
-      <c r="H93" s="80"/>
+      <c r="G93" s="95"/>
+      <c r="H93" s="95"/>
     </row>
     <row r="94" spans="2:28" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G94" s="80"/>
-      <c r="H94" s="80"/>
+      <c r="G94" s="95"/>
+      <c r="H94" s="95"/>
     </row>
     <row r="95" spans="2:28" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G95" s="80"/>
-      <c r="H95" s="80"/>
+      <c r="G95" s="95"/>
+      <c r="H95" s="95"/>
     </row>
     <row r="96" spans="2:28" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G96" s="80"/>
-      <c r="H96" s="80"/>
+      <c r="G96" s="95"/>
+      <c r="H96" s="95"/>
     </row>
     <row r="97" spans="7:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G97" s="80"/>
-      <c r="H97" s="80"/>
+      <c r="G97" s="95"/>
+      <c r="H97" s="95"/>
     </row>
     <row r="98" spans="7:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G98" s="80"/>
-      <c r="H98" s="80"/>
+      <c r="G98" s="95"/>
+      <c r="H98" s="95"/>
     </row>
     <row r="99" spans="7:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G99" s="80"/>
-      <c r="H99" s="80"/>
+      <c r="G99" s="95"/>
+      <c r="H99" s="95"/>
     </row>
     <row r="100" spans="7:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G100" s="80"/>
-      <c r="H100" s="80"/>
+      <c r="G100" s="95"/>
+      <c r="H100" s="95"/>
     </row>
     <row r="101" spans="7:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G101" s="80"/>
-      <c r="H101" s="80"/>
+      <c r="G101" s="95"/>
+      <c r="H101" s="95"/>
     </row>
     <row r="102" spans="7:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G102" s="80"/>
-      <c r="H102" s="80"/>
+      <c r="G102" s="95"/>
+      <c r="H102" s="95"/>
     </row>
     <row r="103" spans="7:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G103" s="80"/>
-      <c r="H103" s="80"/>
+      <c r="G103" s="95"/>
+      <c r="H103" s="95"/>
     </row>
     <row r="104" spans="7:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G104" s="80"/>
-      <c r="H104" s="80"/>
+      <c r="G104" s="95"/>
+      <c r="H104" s="95"/>
     </row>
     <row r="105" spans="7:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G105" s="80"/>
-      <c r="H105" s="80"/>
+      <c r="G105" s="95"/>
+      <c r="H105" s="95"/>
     </row>
     <row r="106" spans="7:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G106" s="80"/>
-      <c r="H106" s="80"/>
+      <c r="G106" s="95"/>
+      <c r="H106" s="95"/>
     </row>
     <row r="107" spans="7:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G107" s="80"/>
-      <c r="H107" s="80"/>
+      <c r="G107" s="95"/>
+      <c r="H107" s="95"/>
     </row>
     <row r="108" spans="7:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G108" s="80"/>
-      <c r="H108" s="80"/>
+      <c r="G108" s="95"/>
+      <c r="H108" s="95"/>
     </row>
     <row r="109" spans="7:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G109" s="80"/>
-      <c r="H109" s="80"/>
+      <c r="G109" s="95"/>
+      <c r="H109" s="95"/>
     </row>
     <row r="110" spans="7:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G110" s="80"/>
-      <c r="H110" s="80"/>
+      <c r="G110" s="95"/>
+      <c r="H110" s="95"/>
     </row>
     <row r="111" spans="7:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G111" s="80"/>
-      <c r="H111" s="80"/>
+      <c r="G111" s="95"/>
+      <c r="H111" s="95"/>
     </row>
     <row r="112" spans="7:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G112" s="80"/>
-      <c r="H112" s="80"/>
+      <c r="G112" s="95"/>
+      <c r="H112" s="95"/>
     </row>
     <row r="113" spans="7:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G113" s="80"/>
-      <c r="H113" s="80"/>
+      <c r="G113" s="95"/>
+      <c r="H113" s="95"/>
     </row>
   </sheetData>
   <mergeCells count="171">
-    <mergeCell ref="B81:I81"/>
-    <mergeCell ref="B82:I82"/>
-    <mergeCell ref="B72:E72"/>
-    <mergeCell ref="B60:I60"/>
-    <mergeCell ref="B68:I68"/>
-    <mergeCell ref="B61:I62"/>
-    <mergeCell ref="B63:I63"/>
-    <mergeCell ref="H65:H66"/>
-    <mergeCell ref="B64:I64"/>
-    <mergeCell ref="G67:H67"/>
-    <mergeCell ref="G69:H69"/>
-    <mergeCell ref="G70:H70"/>
-    <mergeCell ref="C65:D65"/>
-    <mergeCell ref="C66:D66"/>
-    <mergeCell ref="B78:I79"/>
-    <mergeCell ref="G77:H77"/>
-    <mergeCell ref="G80:H80"/>
-    <mergeCell ref="I55:I56"/>
-    <mergeCell ref="H76:I76"/>
-    <mergeCell ref="B55:C56"/>
-    <mergeCell ref="D55:E56"/>
-    <mergeCell ref="F55:F56"/>
-    <mergeCell ref="G55:G56"/>
-    <mergeCell ref="H55:H56"/>
-    <mergeCell ref="D47:E48"/>
-    <mergeCell ref="B47:C48"/>
-    <mergeCell ref="F47:F48"/>
-    <mergeCell ref="G47:G48"/>
-    <mergeCell ref="H47:H48"/>
-    <mergeCell ref="I47:I48"/>
-    <mergeCell ref="B49:C50"/>
-    <mergeCell ref="D49:E50"/>
-    <mergeCell ref="F49:F50"/>
-    <mergeCell ref="G49:G50"/>
-    <mergeCell ref="H49:H50"/>
-    <mergeCell ref="I49:I50"/>
+    <mergeCell ref="B31:I31"/>
+    <mergeCell ref="B33:F33"/>
+    <mergeCell ref="G32:I32"/>
+    <mergeCell ref="G33:I33"/>
+    <mergeCell ref="G112:H112"/>
+    <mergeCell ref="G113:H113"/>
+    <mergeCell ref="B59:I59"/>
+    <mergeCell ref="G106:H106"/>
+    <mergeCell ref="G107:H107"/>
+    <mergeCell ref="G108:H108"/>
+    <mergeCell ref="G109:H109"/>
+    <mergeCell ref="G110:H110"/>
+    <mergeCell ref="G101:H101"/>
+    <mergeCell ref="G102:H102"/>
+    <mergeCell ref="G103:H103"/>
+    <mergeCell ref="G104:H104"/>
+    <mergeCell ref="B83:I83"/>
+    <mergeCell ref="B70:E71"/>
+    <mergeCell ref="H74:I75"/>
+    <mergeCell ref="B74:E75"/>
+    <mergeCell ref="G65:G66"/>
+    <mergeCell ref="I65:I66"/>
+    <mergeCell ref="G87:H87"/>
+    <mergeCell ref="G88:H88"/>
+    <mergeCell ref="G111:H111"/>
+    <mergeCell ref="G84:H84"/>
+    <mergeCell ref="G85:H85"/>
+    <mergeCell ref="G73:H73"/>
+    <mergeCell ref="B44:I44"/>
+    <mergeCell ref="G39:G40"/>
+    <mergeCell ref="G43:H43"/>
+    <mergeCell ref="C37:F40"/>
+    <mergeCell ref="C41:F42"/>
+    <mergeCell ref="B41:B42"/>
+    <mergeCell ref="G86:H86"/>
+    <mergeCell ref="D53:E54"/>
+    <mergeCell ref="F53:F54"/>
+    <mergeCell ref="G53:G54"/>
+    <mergeCell ref="H53:H54"/>
+    <mergeCell ref="I53:I54"/>
+    <mergeCell ref="G51:G52"/>
+    <mergeCell ref="H37:I38"/>
+    <mergeCell ref="B37:B40"/>
+    <mergeCell ref="G37:G38"/>
+    <mergeCell ref="G89:H89"/>
+    <mergeCell ref="G90:H90"/>
+    <mergeCell ref="E65:F66"/>
+    <mergeCell ref="G105:H105"/>
+    <mergeCell ref="B24:E24"/>
+    <mergeCell ref="H21:I21"/>
+    <mergeCell ref="E21:G21"/>
+    <mergeCell ref="E20:G20"/>
+    <mergeCell ref="F24:G24"/>
+    <mergeCell ref="F25:G25"/>
+    <mergeCell ref="I51:I52"/>
+    <mergeCell ref="I45:I46"/>
+    <mergeCell ref="G41:G42"/>
+    <mergeCell ref="H41:I42"/>
+    <mergeCell ref="B35:I35"/>
+    <mergeCell ref="H39:I40"/>
+    <mergeCell ref="H36:I36"/>
+    <mergeCell ref="C36:F36"/>
+    <mergeCell ref="G30:H30"/>
+    <mergeCell ref="G34:H34"/>
+    <mergeCell ref="G22:H22"/>
+    <mergeCell ref="H24:I24"/>
+    <mergeCell ref="H25:I25"/>
+    <mergeCell ref="B28:D28"/>
+    <mergeCell ref="B29:D29"/>
+    <mergeCell ref="H28:I28"/>
+    <mergeCell ref="B27:I27"/>
+    <mergeCell ref="B25:E25"/>
+    <mergeCell ref="E18:G18"/>
+    <mergeCell ref="H18:I18"/>
+    <mergeCell ref="E19:G19"/>
+    <mergeCell ref="H19:I19"/>
+    <mergeCell ref="B18:D18"/>
+    <mergeCell ref="B19:D19"/>
+    <mergeCell ref="E17:G17"/>
+    <mergeCell ref="H17:I17"/>
+    <mergeCell ref="B23:I23"/>
+    <mergeCell ref="G96:H96"/>
+    <mergeCell ref="G97:H97"/>
+    <mergeCell ref="G98:H98"/>
+    <mergeCell ref="G99:H99"/>
+    <mergeCell ref="G100:H100"/>
+    <mergeCell ref="G91:H91"/>
+    <mergeCell ref="G92:H92"/>
+    <mergeCell ref="G93:H93"/>
+    <mergeCell ref="G94:H94"/>
+    <mergeCell ref="G95:H95"/>
+    <mergeCell ref="B3:I3"/>
+    <mergeCell ref="B5:I5"/>
+    <mergeCell ref="B4:I4"/>
+    <mergeCell ref="B6:I6"/>
+    <mergeCell ref="B7:I7"/>
+    <mergeCell ref="H14:I14"/>
+    <mergeCell ref="H15:I15"/>
+    <mergeCell ref="B14:D14"/>
+    <mergeCell ref="B15:D15"/>
+    <mergeCell ref="C8:D8"/>
+    <mergeCell ref="E8:F8"/>
+    <mergeCell ref="F14:G14"/>
+    <mergeCell ref="F15:G15"/>
+    <mergeCell ref="B13:I13"/>
+    <mergeCell ref="E10:I10"/>
+    <mergeCell ref="E11:I11"/>
+    <mergeCell ref="B10:D10"/>
+    <mergeCell ref="B11:D11"/>
+    <mergeCell ref="G9:H9"/>
+    <mergeCell ref="G12:H12"/>
     <mergeCell ref="H16:I16"/>
     <mergeCell ref="D45:E46"/>
     <mergeCell ref="F45:F46"/>
@@ -6627,130 +6765,55 @@
     <mergeCell ref="B51:C52"/>
     <mergeCell ref="D51:E52"/>
     <mergeCell ref="F51:F52"/>
-    <mergeCell ref="B3:I3"/>
-    <mergeCell ref="B5:I5"/>
-    <mergeCell ref="B4:I4"/>
-    <mergeCell ref="B6:I6"/>
-    <mergeCell ref="B7:I7"/>
-    <mergeCell ref="H14:I14"/>
-    <mergeCell ref="H15:I15"/>
-    <mergeCell ref="B14:D14"/>
-    <mergeCell ref="B15:D15"/>
-    <mergeCell ref="C8:D8"/>
-    <mergeCell ref="E8:F8"/>
-    <mergeCell ref="F14:G14"/>
-    <mergeCell ref="F15:G15"/>
-    <mergeCell ref="B13:I13"/>
-    <mergeCell ref="E10:I10"/>
-    <mergeCell ref="E11:I11"/>
-    <mergeCell ref="B10:D10"/>
-    <mergeCell ref="B11:D11"/>
-    <mergeCell ref="G9:H9"/>
-    <mergeCell ref="G12:H12"/>
-    <mergeCell ref="G96:H96"/>
-    <mergeCell ref="G97:H97"/>
-    <mergeCell ref="G98:H98"/>
-    <mergeCell ref="G99:H99"/>
-    <mergeCell ref="G100:H100"/>
-    <mergeCell ref="G91:H91"/>
-    <mergeCell ref="G92:H92"/>
-    <mergeCell ref="G93:H93"/>
-    <mergeCell ref="G94:H94"/>
-    <mergeCell ref="G95:H95"/>
-    <mergeCell ref="E18:G18"/>
-    <mergeCell ref="H18:I18"/>
-    <mergeCell ref="E19:G19"/>
-    <mergeCell ref="H19:I19"/>
-    <mergeCell ref="B18:D18"/>
-    <mergeCell ref="B19:D19"/>
-    <mergeCell ref="E17:G17"/>
-    <mergeCell ref="H17:I17"/>
-    <mergeCell ref="B23:I23"/>
-    <mergeCell ref="B24:E24"/>
-    <mergeCell ref="H21:I21"/>
-    <mergeCell ref="E21:G21"/>
-    <mergeCell ref="E20:G20"/>
-    <mergeCell ref="F24:G24"/>
-    <mergeCell ref="F25:G25"/>
-    <mergeCell ref="I51:I52"/>
-    <mergeCell ref="I45:I46"/>
-    <mergeCell ref="G41:G42"/>
-    <mergeCell ref="H41:I42"/>
-    <mergeCell ref="B35:I35"/>
-    <mergeCell ref="H39:I40"/>
-    <mergeCell ref="H36:I36"/>
-    <mergeCell ref="C36:F36"/>
-    <mergeCell ref="G30:H30"/>
-    <mergeCell ref="G34:H34"/>
-    <mergeCell ref="G22:H22"/>
-    <mergeCell ref="H24:I24"/>
-    <mergeCell ref="H25:I25"/>
-    <mergeCell ref="B28:D28"/>
-    <mergeCell ref="B29:D29"/>
-    <mergeCell ref="H28:I28"/>
-    <mergeCell ref="B27:I27"/>
-    <mergeCell ref="B25:E25"/>
-    <mergeCell ref="G111:H111"/>
-    <mergeCell ref="G84:H84"/>
-    <mergeCell ref="G85:H85"/>
-    <mergeCell ref="G73:H73"/>
-    <mergeCell ref="B44:I44"/>
-    <mergeCell ref="G39:G40"/>
-    <mergeCell ref="G43:H43"/>
-    <mergeCell ref="C37:F40"/>
-    <mergeCell ref="C41:F42"/>
-    <mergeCell ref="B41:B42"/>
-    <mergeCell ref="G86:H86"/>
-    <mergeCell ref="D53:E54"/>
-    <mergeCell ref="F53:F54"/>
-    <mergeCell ref="G53:G54"/>
-    <mergeCell ref="H53:H54"/>
-    <mergeCell ref="I53:I54"/>
-    <mergeCell ref="G51:G52"/>
-    <mergeCell ref="H37:I38"/>
-    <mergeCell ref="B37:B40"/>
-    <mergeCell ref="G37:G38"/>
-    <mergeCell ref="G89:H89"/>
-    <mergeCell ref="G90:H90"/>
-    <mergeCell ref="E65:F66"/>
-    <mergeCell ref="G105:H105"/>
-    <mergeCell ref="B31:I31"/>
-    <mergeCell ref="B33:F33"/>
-    <mergeCell ref="G32:I32"/>
-    <mergeCell ref="G33:I33"/>
-    <mergeCell ref="G112:H112"/>
-    <mergeCell ref="G113:H113"/>
-    <mergeCell ref="B59:I59"/>
-    <mergeCell ref="G106:H106"/>
-    <mergeCell ref="G107:H107"/>
-    <mergeCell ref="G108:H108"/>
-    <mergeCell ref="G109:H109"/>
-    <mergeCell ref="G110:H110"/>
-    <mergeCell ref="G101:H101"/>
-    <mergeCell ref="G102:H102"/>
-    <mergeCell ref="G103:H103"/>
-    <mergeCell ref="G104:H104"/>
-    <mergeCell ref="B83:I83"/>
-    <mergeCell ref="B70:E71"/>
-    <mergeCell ref="H74:I75"/>
-    <mergeCell ref="B74:E75"/>
-    <mergeCell ref="G65:G66"/>
-    <mergeCell ref="I65:I66"/>
-    <mergeCell ref="G87:H87"/>
-    <mergeCell ref="G88:H88"/>
+    <mergeCell ref="I55:I56"/>
+    <mergeCell ref="H76:I76"/>
+    <mergeCell ref="B55:C56"/>
+    <mergeCell ref="D55:E56"/>
+    <mergeCell ref="F55:F56"/>
+    <mergeCell ref="G55:G56"/>
+    <mergeCell ref="H55:H56"/>
+    <mergeCell ref="D47:E48"/>
+    <mergeCell ref="B47:C48"/>
+    <mergeCell ref="F47:F48"/>
+    <mergeCell ref="G47:G48"/>
+    <mergeCell ref="H47:H48"/>
+    <mergeCell ref="I47:I48"/>
+    <mergeCell ref="B49:C50"/>
+    <mergeCell ref="D49:E50"/>
+    <mergeCell ref="F49:F50"/>
+    <mergeCell ref="G49:G50"/>
+    <mergeCell ref="H49:H50"/>
+    <mergeCell ref="I49:I50"/>
+    <mergeCell ref="B81:I81"/>
+    <mergeCell ref="B82:I82"/>
+    <mergeCell ref="B72:E72"/>
+    <mergeCell ref="B60:I60"/>
+    <mergeCell ref="B68:I68"/>
+    <mergeCell ref="B61:I62"/>
+    <mergeCell ref="B63:I63"/>
+    <mergeCell ref="H65:H66"/>
+    <mergeCell ref="B64:I64"/>
+    <mergeCell ref="G67:H67"/>
+    <mergeCell ref="G69:H69"/>
+    <mergeCell ref="G70:H70"/>
+    <mergeCell ref="C65:D65"/>
+    <mergeCell ref="C66:D66"/>
+    <mergeCell ref="B78:I79"/>
+    <mergeCell ref="G77:H77"/>
+    <mergeCell ref="G80:H80"/>
   </mergeCells>
   <conditionalFormatting sqref="B11:I11 B15:I15 B17:I17 B19:I19 B21:I21 B25:I25 B29:I29 C37:F42 H37:I42 B70:E71 H74:I75 B83:I83">
-    <cfRule type="containsBlanks" dxfId="2" priority="4">
+    <cfRule type="containsBlanks" dxfId="5" priority="7">
       <formula>LEN(TRIM(B11))=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B47:I56">
-    <cfRule type="containsBlanks" dxfId="1" priority="6">
+    <cfRule type="containsBlanks" dxfId="4" priority="6">
       <formula>LEN(TRIM(B47))=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G65:G66 I65:I66 B66:D66 H71">
-    <cfRule type="containsBlanks" dxfId="0" priority="5">
+    <cfRule type="containsBlanks" dxfId="3" priority="8">
       <formula>LEN(TRIM(B65))=0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6791,7 +6854,7 @@
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Ingresar Capturas de pantalla ev" prompt="Ingresa las evidencias de cumplimiento, como capturas de pantalla o fotografias segun sea el caso" sqref="B83:I83" xr:uid="{40D2D8F2-1FE7-4A55-AF5E-54C9B05900F3}"/>
   </dataValidations>
   <pageMargins left="0.51181102362204722" right="0.51181102362204722" top="0.35433070866141736" bottom="0.35433070866141736" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="5" scale="47" fitToHeight="0" orientation="portrait" horizontalDpi="4294967294" r:id="rId1"/>
+  <pageSetup paperSize="5" scale="49" fitToHeight="0" orientation="portrait" horizontalDpi="4294967294" r:id="rId1"/>
   <drawing r:id="rId2"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
@@ -7376,124 +7439,124 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:24" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A1" s="250" t="s">
+      <c r="A1" s="275" t="s">
         <v>72</v>
       </c>
-      <c r="B1" s="250"/>
-      <c r="C1" s="250"/>
-      <c r="D1" s="250"/>
-      <c r="E1" s="250"/>
-      <c r="F1" s="250"/>
-      <c r="G1" s="250"/>
-      <c r="H1" s="250"/>
-      <c r="I1" s="250"/>
-      <c r="J1" s="250"/>
-      <c r="K1" s="250"/>
-      <c r="L1" s="250"/>
-      <c r="M1" s="250"/>
-      <c r="N1" s="250"/>
-      <c r="O1" s="250"/>
-      <c r="P1" s="250"/>
-      <c r="Q1" s="250"/>
-      <c r="R1" s="250"/>
-      <c r="S1" s="250"/>
-      <c r="T1" s="250"/>
-      <c r="U1" s="250" t="s">
+      <c r="B1" s="275"/>
+      <c r="C1" s="275"/>
+      <c r="D1" s="275"/>
+      <c r="E1" s="275"/>
+      <c r="F1" s="275"/>
+      <c r="G1" s="275"/>
+      <c r="H1" s="275"/>
+      <c r="I1" s="275"/>
+      <c r="J1" s="275"/>
+      <c r="K1" s="275"/>
+      <c r="L1" s="275"/>
+      <c r="M1" s="275"/>
+      <c r="N1" s="275"/>
+      <c r="O1" s="275"/>
+      <c r="P1" s="275"/>
+      <c r="Q1" s="275"/>
+      <c r="R1" s="275"/>
+      <c r="S1" s="275"/>
+      <c r="T1" s="275"/>
+      <c r="U1" s="275" t="s">
         <v>73</v>
       </c>
-      <c r="V1" s="250"/>
-      <c r="W1" s="250"/>
-      <c r="X1" s="250"/>
+      <c r="V1" s="275"/>
+      <c r="W1" s="275"/>
+      <c r="X1" s="275"/>
     </row>
     <row r="2" spans="1:24" ht="33" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="250"/>
-      <c r="B2" s="250"/>
-      <c r="C2" s="250"/>
-      <c r="D2" s="250"/>
-      <c r="E2" s="250"/>
-      <c r="F2" s="250"/>
-      <c r="G2" s="250"/>
-      <c r="H2" s="250"/>
-      <c r="I2" s="250"/>
-      <c r="J2" s="250"/>
-      <c r="K2" s="250"/>
-      <c r="L2" s="250"/>
-      <c r="M2" s="250"/>
-      <c r="N2" s="250"/>
-      <c r="O2" s="250"/>
-      <c r="P2" s="250"/>
-      <c r="Q2" s="250"/>
-      <c r="R2" s="250"/>
-      <c r="S2" s="250"/>
-      <c r="T2" s="250"/>
-      <c r="U2" s="258" t="s">
+      <c r="A2" s="275"/>
+      <c r="B2" s="275"/>
+      <c r="C2" s="275"/>
+      <c r="D2" s="275"/>
+      <c r="E2" s="275"/>
+      <c r="F2" s="275"/>
+      <c r="G2" s="275"/>
+      <c r="H2" s="275"/>
+      <c r="I2" s="275"/>
+      <c r="J2" s="275"/>
+      <c r="K2" s="275"/>
+      <c r="L2" s="275"/>
+      <c r="M2" s="275"/>
+      <c r="N2" s="275"/>
+      <c r="O2" s="275"/>
+      <c r="P2" s="275"/>
+      <c r="Q2" s="275"/>
+      <c r="R2" s="275"/>
+      <c r="S2" s="275"/>
+      <c r="T2" s="275"/>
+      <c r="U2" s="255" t="s">
         <v>74</v>
       </c>
-      <c r="V2" s="258"/>
-      <c r="W2" s="258"/>
-      <c r="X2" s="258"/>
+      <c r="V2" s="255"/>
+      <c r="W2" s="255"/>
+      <c r="X2" s="255"/>
     </row>
     <row r="3" spans="1:24" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="U3" s="259"/>
-      <c r="V3" s="259"/>
-      <c r="W3" s="259"/>
-      <c r="X3" s="259"/>
+      <c r="U3" s="282"/>
+      <c r="V3" s="282"/>
+      <c r="W3" s="282"/>
+      <c r="X3" s="282"/>
     </row>
     <row r="4" spans="1:24" s="2" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="255" t="s">
+      <c r="A4" s="279" t="s">
         <v>75</v>
       </c>
-      <c r="B4" s="256"/>
-      <c r="C4" s="256"/>
-      <c r="D4" s="256"/>
-      <c r="E4" s="256"/>
-      <c r="F4" s="256"/>
-      <c r="G4" s="256"/>
-      <c r="H4" s="256"/>
-      <c r="I4" s="256"/>
-      <c r="J4" s="256"/>
-      <c r="K4" s="256"/>
-      <c r="L4" s="256"/>
-      <c r="M4" s="257"/>
-      <c r="N4" s="255" t="s">
+      <c r="B4" s="280"/>
+      <c r="C4" s="280"/>
+      <c r="D4" s="280"/>
+      <c r="E4" s="280"/>
+      <c r="F4" s="280"/>
+      <c r="G4" s="280"/>
+      <c r="H4" s="280"/>
+      <c r="I4" s="280"/>
+      <c r="J4" s="280"/>
+      <c r="K4" s="280"/>
+      <c r="L4" s="280"/>
+      <c r="M4" s="281"/>
+      <c r="N4" s="279" t="s">
         <v>76</v>
       </c>
-      <c r="O4" s="256"/>
-      <c r="P4" s="256"/>
-      <c r="Q4" s="256"/>
-      <c r="R4" s="256"/>
-      <c r="S4" s="256"/>
-      <c r="T4" s="256"/>
-      <c r="U4" s="256"/>
-      <c r="V4" s="256"/>
-      <c r="W4" s="256"/>
-      <c r="X4" s="257"/>
+      <c r="O4" s="280"/>
+      <c r="P4" s="280"/>
+      <c r="Q4" s="280"/>
+      <c r="R4" s="280"/>
+      <c r="S4" s="280"/>
+      <c r="T4" s="280"/>
+      <c r="U4" s="280"/>
+      <c r="V4" s="280"/>
+      <c r="W4" s="280"/>
+      <c r="X4" s="281"/>
     </row>
     <row r="5" spans="1:24" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="252"/>
-      <c r="B5" s="253"/>
-      <c r="C5" s="253"/>
-      <c r="D5" s="253"/>
-      <c r="E5" s="253"/>
-      <c r="F5" s="253"/>
-      <c r="G5" s="253"/>
-      <c r="H5" s="253"/>
-      <c r="I5" s="253"/>
-      <c r="J5" s="253"/>
-      <c r="K5" s="253"/>
-      <c r="L5" s="253"/>
-      <c r="M5" s="254"/>
-      <c r="N5" s="252"/>
-      <c r="O5" s="253"/>
-      <c r="P5" s="253"/>
-      <c r="Q5" s="253"/>
-      <c r="R5" s="253"/>
-      <c r="S5" s="253"/>
-      <c r="T5" s="253"/>
-      <c r="U5" s="253"/>
-      <c r="V5" s="253"/>
-      <c r="W5" s="253"/>
-      <c r="X5" s="254"/>
+      <c r="A5" s="276"/>
+      <c r="B5" s="277"/>
+      <c r="C5" s="277"/>
+      <c r="D5" s="277"/>
+      <c r="E5" s="277"/>
+      <c r="F5" s="277"/>
+      <c r="G5" s="277"/>
+      <c r="H5" s="277"/>
+      <c r="I5" s="277"/>
+      <c r="J5" s="277"/>
+      <c r="K5" s="277"/>
+      <c r="L5" s="277"/>
+      <c r="M5" s="278"/>
+      <c r="N5" s="276"/>
+      <c r="O5" s="277"/>
+      <c r="P5" s="277"/>
+      <c r="Q5" s="277"/>
+      <c r="R5" s="277"/>
+      <c r="S5" s="277"/>
+      <c r="T5" s="277"/>
+      <c r="U5" s="277"/>
+      <c r="V5" s="277"/>
+      <c r="W5" s="277"/>
+      <c r="X5" s="278"/>
     </row>
     <row r="6" spans="1:24" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3"/>
@@ -7522,36 +7585,36 @@
       <c r="X6" s="3"/>
     </row>
     <row r="7" spans="1:24" s="2" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="251" t="s">
+      <c r="A7" s="253" t="s">
         <v>77</v>
       </c>
-      <c r="B7" s="251"/>
-      <c r="C7" s="251"/>
-      <c r="D7" s="251"/>
-      <c r="E7" s="251"/>
-      <c r="F7" s="251"/>
-      <c r="G7" s="251"/>
-      <c r="H7" s="251"/>
-      <c r="I7" s="251"/>
-      <c r="J7" s="251" t="s">
+      <c r="B7" s="253"/>
+      <c r="C7" s="253"/>
+      <c r="D7" s="253"/>
+      <c r="E7" s="253"/>
+      <c r="F7" s="253"/>
+      <c r="G7" s="253"/>
+      <c r="H7" s="253"/>
+      <c r="I7" s="253"/>
+      <c r="J7" s="253" t="s">
         <v>78</v>
       </c>
-      <c r="K7" s="251"/>
-      <c r="L7" s="251"/>
-      <c r="M7" s="251"/>
-      <c r="N7" s="251"/>
-      <c r="O7" s="251"/>
-      <c r="P7" s="251" t="s">
+      <c r="K7" s="253"/>
+      <c r="L7" s="253"/>
+      <c r="M7" s="253"/>
+      <c r="N7" s="253"/>
+      <c r="O7" s="253"/>
+      <c r="P7" s="253" t="s">
         <v>79</v>
       </c>
-      <c r="Q7" s="251"/>
-      <c r="R7" s="251"/>
-      <c r="S7" s="251"/>
-      <c r="T7" s="251"/>
-      <c r="U7" s="251"/>
-      <c r="V7" s="251"/>
-      <c r="W7" s="251"/>
-      <c r="X7" s="251"/>
+      <c r="Q7" s="253"/>
+      <c r="R7" s="253"/>
+      <c r="S7" s="253"/>
+      <c r="T7" s="253"/>
+      <c r="U7" s="253"/>
+      <c r="V7" s="253"/>
+      <c r="W7" s="253"/>
+      <c r="X7" s="253"/>
     </row>
     <row r="8" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="260"/>
@@ -7610,66 +7673,66 @@
       <c r="X9" s="3"/>
     </row>
     <row r="10" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="264" t="s">
+      <c r="A10" s="273" t="s">
         <v>82</v>
       </c>
-      <c r="B10" s="264"/>
-      <c r="C10" s="264"/>
-      <c r="D10" s="264"/>
-      <c r="E10" s="264"/>
-      <c r="F10" s="264"/>
-      <c r="G10" s="264"/>
-      <c r="H10" s="264"/>
-      <c r="I10" s="264"/>
-      <c r="J10" s="264"/>
-      <c r="K10" s="264"/>
-      <c r="L10" s="264"/>
-      <c r="M10" s="264"/>
-      <c r="N10" s="264"/>
-      <c r="O10" s="264"/>
-      <c r="P10" s="264"/>
-      <c r="Q10" s="264"/>
-      <c r="R10" s="264"/>
-      <c r="S10" s="264"/>
-      <c r="T10" s="264"/>
-      <c r="U10" s="264"/>
-      <c r="V10" s="264"/>
-      <c r="W10" s="264"/>
-      <c r="X10" s="264"/>
+      <c r="B10" s="273"/>
+      <c r="C10" s="273"/>
+      <c r="D10" s="273"/>
+      <c r="E10" s="273"/>
+      <c r="F10" s="273"/>
+      <c r="G10" s="273"/>
+      <c r="H10" s="273"/>
+      <c r="I10" s="273"/>
+      <c r="J10" s="273"/>
+      <c r="K10" s="273"/>
+      <c r="L10" s="273"/>
+      <c r="M10" s="273"/>
+      <c r="N10" s="273"/>
+      <c r="O10" s="273"/>
+      <c r="P10" s="273"/>
+      <c r="Q10" s="273"/>
+      <c r="R10" s="273"/>
+      <c r="S10" s="273"/>
+      <c r="T10" s="273"/>
+      <c r="U10" s="273"/>
+      <c r="V10" s="273"/>
+      <c r="W10" s="273"/>
+      <c r="X10" s="273"/>
     </row>
     <row r="11" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="265" t="s">
+      <c r="A11" s="274" t="s">
         <v>83</v>
       </c>
-      <c r="B11" s="265"/>
-      <c r="C11" s="265"/>
-      <c r="D11" s="265"/>
-      <c r="E11" s="265"/>
-      <c r="F11" s="265"/>
-      <c r="G11" s="265" t="s">
+      <c r="B11" s="274"/>
+      <c r="C11" s="274"/>
+      <c r="D11" s="274"/>
+      <c r="E11" s="274"/>
+      <c r="F11" s="274"/>
+      <c r="G11" s="274" t="s">
         <v>84</v>
       </c>
-      <c r="H11" s="265"/>
-      <c r="I11" s="265"/>
-      <c r="J11" s="265"/>
-      <c r="K11" s="265"/>
-      <c r="L11" s="265"/>
-      <c r="M11" s="265" t="s">
+      <c r="H11" s="274"/>
+      <c r="I11" s="274"/>
+      <c r="J11" s="274"/>
+      <c r="K11" s="274"/>
+      <c r="L11" s="274"/>
+      <c r="M11" s="274" t="s">
         <v>85</v>
       </c>
-      <c r="N11" s="265"/>
-      <c r="O11" s="265"/>
-      <c r="P11" s="265"/>
-      <c r="Q11" s="265"/>
-      <c r="R11" s="265"/>
-      <c r="S11" s="265" t="s">
+      <c r="N11" s="274"/>
+      <c r="O11" s="274"/>
+      <c r="P11" s="274"/>
+      <c r="Q11" s="274"/>
+      <c r="R11" s="274"/>
+      <c r="S11" s="274" t="s">
         <v>86</v>
       </c>
-      <c r="T11" s="265"/>
-      <c r="U11" s="265"/>
-      <c r="V11" s="265"/>
-      <c r="W11" s="265"/>
-      <c r="X11" s="265"/>
+      <c r="T11" s="274"/>
+      <c r="U11" s="274"/>
+      <c r="V11" s="274"/>
+      <c r="W11" s="274"/>
+      <c r="X11" s="274"/>
     </row>
     <row r="12" spans="1:24" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3"/>
@@ -7698,36 +7761,36 @@
       <c r="X12" s="3"/>
     </row>
     <row r="13" spans="1:24" s="2" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="251" t="s">
+      <c r="A13" s="253" t="s">
         <v>87</v>
       </c>
-      <c r="B13" s="251"/>
-      <c r="C13" s="251"/>
-      <c r="D13" s="251"/>
-      <c r="E13" s="251"/>
-      <c r="F13" s="251"/>
-      <c r="G13" s="251"/>
-      <c r="H13" s="251"/>
-      <c r="I13" s="251"/>
-      <c r="J13" s="251" t="s">
+      <c r="B13" s="253"/>
+      <c r="C13" s="253"/>
+      <c r="D13" s="253"/>
+      <c r="E13" s="253"/>
+      <c r="F13" s="253"/>
+      <c r="G13" s="253"/>
+      <c r="H13" s="253"/>
+      <c r="I13" s="253"/>
+      <c r="J13" s="253" t="s">
         <v>78</v>
       </c>
-      <c r="K13" s="251"/>
-      <c r="L13" s="251"/>
-      <c r="M13" s="251"/>
-      <c r="N13" s="251"/>
-      <c r="O13" s="251"/>
-      <c r="P13" s="251" t="s">
+      <c r="K13" s="253"/>
+      <c r="L13" s="253"/>
+      <c r="M13" s="253"/>
+      <c r="N13" s="253"/>
+      <c r="O13" s="253"/>
+      <c r="P13" s="253" t="s">
         <v>79</v>
       </c>
-      <c r="Q13" s="251"/>
-      <c r="R13" s="251"/>
-      <c r="S13" s="251"/>
-      <c r="T13" s="251"/>
-      <c r="U13" s="251"/>
-      <c r="V13" s="251"/>
-      <c r="W13" s="251"/>
-      <c r="X13" s="251"/>
+      <c r="Q13" s="253"/>
+      <c r="R13" s="253"/>
+      <c r="S13" s="253"/>
+      <c r="T13" s="253"/>
+      <c r="U13" s="253"/>
+      <c r="V13" s="253"/>
+      <c r="W13" s="253"/>
+      <c r="X13" s="253"/>
     </row>
     <row r="14" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="260"/>
@@ -7786,172 +7849,184 @@
       <c r="X15" s="3"/>
     </row>
     <row r="16" spans="1:24" s="4" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="271" t="s">
+      <c r="A16" s="264" t="s">
         <v>90</v>
       </c>
-      <c r="B16" s="271"/>
-      <c r="C16" s="271"/>
-      <c r="D16" s="271"/>
-      <c r="E16" s="271"/>
-      <c r="F16" s="271"/>
-      <c r="G16" s="271"/>
-      <c r="H16" s="271"/>
-      <c r="I16" s="271"/>
-      <c r="J16" s="272" t="s">
+      <c r="B16" s="264"/>
+      <c r="C16" s="264"/>
+      <c r="D16" s="264"/>
+      <c r="E16" s="264"/>
+      <c r="F16" s="264"/>
+      <c r="G16" s="264"/>
+      <c r="H16" s="264"/>
+      <c r="I16" s="264"/>
+      <c r="J16" s="265" t="s">
         <v>91</v>
       </c>
-      <c r="K16" s="272"/>
-      <c r="L16" s="272"/>
-      <c r="M16" s="272"/>
-      <c r="N16" s="271" t="s">
+      <c r="K16" s="265"/>
+      <c r="L16" s="265"/>
+      <c r="M16" s="265"/>
+      <c r="N16" s="264" t="s">
         <v>92</v>
       </c>
-      <c r="O16" s="271"/>
-      <c r="P16" s="271"/>
-      <c r="Q16" s="271"/>
-      <c r="R16" s="271"/>
-      <c r="S16" s="271"/>
-      <c r="T16" s="273" t="s">
+      <c r="O16" s="264"/>
+      <c r="P16" s="264"/>
+      <c r="Q16" s="264"/>
+      <c r="R16" s="264"/>
+      <c r="S16" s="264"/>
+      <c r="T16" s="266" t="s">
         <v>93</v>
       </c>
-      <c r="U16" s="273"/>
-      <c r="V16" s="273"/>
-      <c r="W16" s="273"/>
-      <c r="X16" s="273"/>
+      <c r="U16" s="266"/>
+      <c r="V16" s="266"/>
+      <c r="W16" s="266"/>
+      <c r="X16" s="266"/>
     </row>
     <row r="17" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="266" t="s">
+      <c r="A17" s="254" t="s">
         <v>94</v>
       </c>
-      <c r="B17" s="258"/>
-      <c r="C17" s="258"/>
-      <c r="D17" s="258"/>
-      <c r="E17" s="258"/>
-      <c r="F17" s="258"/>
-      <c r="G17" s="258"/>
-      <c r="H17" s="258"/>
-      <c r="I17" s="267"/>
-      <c r="J17" s="274" t="s">
+      <c r="B17" s="255"/>
+      <c r="C17" s="255"/>
+      <c r="D17" s="255"/>
+      <c r="E17" s="255"/>
+      <c r="F17" s="255"/>
+      <c r="G17" s="255"/>
+      <c r="H17" s="255"/>
+      <c r="I17" s="256"/>
+      <c r="J17" s="267" t="s">
         <v>95</v>
       </c>
-      <c r="K17" s="275"/>
-      <c r="L17" s="275"/>
-      <c r="M17" s="276"/>
-      <c r="N17" s="266" t="s">
+      <c r="K17" s="268"/>
+      <c r="L17" s="268"/>
+      <c r="M17" s="269"/>
+      <c r="N17" s="254" t="s">
         <v>96</v>
       </c>
-      <c r="O17" s="258"/>
-      <c r="P17" s="258"/>
-      <c r="Q17" s="258"/>
-      <c r="R17" s="258"/>
-      <c r="S17" s="267"/>
-      <c r="T17" s="266" t="s">
+      <c r="O17" s="255"/>
+      <c r="P17" s="255"/>
+      <c r="Q17" s="255"/>
+      <c r="R17" s="255"/>
+      <c r="S17" s="256"/>
+      <c r="T17" s="254" t="s">
         <v>97</v>
       </c>
-      <c r="U17" s="258"/>
-      <c r="V17" s="258"/>
-      <c r="W17" s="258"/>
-      <c r="X17" s="267"/>
+      <c r="U17" s="255"/>
+      <c r="V17" s="255"/>
+      <c r="W17" s="255"/>
+      <c r="X17" s="256"/>
     </row>
     <row r="18" spans="1:24" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="268"/>
-      <c r="B18" s="269"/>
-      <c r="C18" s="269"/>
-      <c r="D18" s="269"/>
-      <c r="E18" s="269"/>
-      <c r="F18" s="269"/>
-      <c r="G18" s="269"/>
-      <c r="H18" s="269"/>
-      <c r="I18" s="270"/>
-      <c r="J18" s="277"/>
-      <c r="K18" s="278"/>
-      <c r="L18" s="278"/>
-      <c r="M18" s="279"/>
-      <c r="N18" s="268"/>
-      <c r="O18" s="269"/>
-      <c r="P18" s="269"/>
-      <c r="Q18" s="269"/>
-      <c r="R18" s="269"/>
-      <c r="S18" s="270"/>
-      <c r="T18" s="268"/>
-      <c r="U18" s="269"/>
-      <c r="V18" s="269"/>
-      <c r="W18" s="269"/>
-      <c r="X18" s="270"/>
+      <c r="A18" s="257"/>
+      <c r="B18" s="258"/>
+      <c r="C18" s="258"/>
+      <c r="D18" s="258"/>
+      <c r="E18" s="258"/>
+      <c r="F18" s="258"/>
+      <c r="G18" s="258"/>
+      <c r="H18" s="258"/>
+      <c r="I18" s="259"/>
+      <c r="J18" s="270"/>
+      <c r="K18" s="271"/>
+      <c r="L18" s="271"/>
+      <c r="M18" s="272"/>
+      <c r="N18" s="257"/>
+      <c r="O18" s="258"/>
+      <c r="P18" s="258"/>
+      <c r="Q18" s="258"/>
+      <c r="R18" s="258"/>
+      <c r="S18" s="259"/>
+      <c r="T18" s="257"/>
+      <c r="U18" s="258"/>
+      <c r="V18" s="258"/>
+      <c r="W18" s="258"/>
+      <c r="X18" s="259"/>
     </row>
     <row r="19" spans="1:24" ht="39" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="20" spans="1:24" ht="39" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="21" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A21" s="283" t="s">
+      <c r="A21" s="252" t="s">
         <v>98</v>
       </c>
-      <c r="B21" s="283"/>
-      <c r="C21" s="283"/>
-      <c r="D21" s="283"/>
-      <c r="E21" s="283"/>
-      <c r="F21" s="283"/>
-      <c r="G21" s="283"/>
-      <c r="H21" s="283"/>
+      <c r="B21" s="252"/>
+      <c r="C21" s="252"/>
+      <c r="D21" s="252"/>
+      <c r="E21" s="252"/>
+      <c r="F21" s="252"/>
+      <c r="G21" s="252"/>
+      <c r="H21" s="252"/>
       <c r="I21" s="5"/>
-      <c r="J21" s="283" t="s">
+      <c r="J21" s="252" t="s">
         <v>65</v>
       </c>
-      <c r="K21" s="283"/>
-      <c r="L21" s="283"/>
-      <c r="M21" s="283"/>
-      <c r="N21" s="283"/>
-      <c r="O21" s="283"/>
-      <c r="P21" s="283"/>
+      <c r="K21" s="252"/>
+      <c r="L21" s="252"/>
+      <c r="M21" s="252"/>
+      <c r="N21" s="252"/>
+      <c r="O21" s="252"/>
+      <c r="P21" s="252"/>
       <c r="Q21" s="6"/>
-      <c r="R21" s="283" t="s">
+      <c r="R21" s="252" t="s">
         <v>99</v>
       </c>
-      <c r="S21" s="283"/>
-      <c r="T21" s="283"/>
-      <c r="U21" s="283"/>
-      <c r="V21" s="283"/>
-      <c r="W21" s="283"/>
-      <c r="X21" s="283"/>
+      <c r="S21" s="252"/>
+      <c r="T21" s="252"/>
+      <c r="U21" s="252"/>
+      <c r="V21" s="252"/>
+      <c r="W21" s="252"/>
+      <c r="X21" s="252"/>
     </row>
     <row r="23" spans="1:24" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="P23" s="280" t="s">
+      <c r="P23" s="249" t="s">
         <v>100</v>
       </c>
-      <c r="Q23" s="280"/>
-      <c r="R23" s="280"/>
-      <c r="S23" s="280"/>
-      <c r="T23" s="280"/>
-      <c r="U23" s="281" t="s">
+      <c r="Q23" s="249"/>
+      <c r="R23" s="249"/>
+      <c r="S23" s="249"/>
+      <c r="T23" s="249"/>
+      <c r="U23" s="250" t="s">
         <v>101</v>
       </c>
-      <c r="V23" s="281"/>
-      <c r="W23" s="281"/>
-      <c r="X23" s="281"/>
+      <c r="V23" s="250"/>
+      <c r="W23" s="250"/>
+      <c r="X23" s="250"/>
     </row>
     <row r="24" spans="1:24" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="P24" s="280" t="s">
+      <c r="P24" s="249" t="s">
         <v>102</v>
       </c>
-      <c r="Q24" s="280"/>
-      <c r="R24" s="280"/>
-      <c r="S24" s="280"/>
-      <c r="T24" s="280"/>
-      <c r="U24" s="282" t="s">
+      <c r="Q24" s="249"/>
+      <c r="R24" s="249"/>
+      <c r="S24" s="249"/>
+      <c r="T24" s="249"/>
+      <c r="U24" s="251" t="s">
         <v>103</v>
       </c>
-      <c r="V24" s="282"/>
-      <c r="W24" s="282"/>
-      <c r="X24" s="282"/>
+      <c r="V24" s="251"/>
+      <c r="W24" s="251"/>
+      <c r="X24" s="251"/>
     </row>
   </sheetData>
   <mergeCells count="40">
-    <mergeCell ref="P23:T23"/>
-    <mergeCell ref="U23:X23"/>
-    <mergeCell ref="P24:T24"/>
-    <mergeCell ref="U24:X24"/>
-    <mergeCell ref="A21:H21"/>
-    <mergeCell ref="J21:P21"/>
-    <mergeCell ref="R21:X21"/>
+    <mergeCell ref="A1:T1"/>
+    <mergeCell ref="U1:X1"/>
+    <mergeCell ref="A2:T2"/>
+    <mergeCell ref="A7:I7"/>
+    <mergeCell ref="J7:O7"/>
+    <mergeCell ref="P7:X7"/>
+    <mergeCell ref="A5:M5"/>
+    <mergeCell ref="A4:M4"/>
+    <mergeCell ref="N4:X4"/>
+    <mergeCell ref="N5:X5"/>
+    <mergeCell ref="U2:X3"/>
+    <mergeCell ref="A8:I8"/>
+    <mergeCell ref="J8:O8"/>
+    <mergeCell ref="P8:X8"/>
+    <mergeCell ref="A10:X10"/>
+    <mergeCell ref="A11:F11"/>
+    <mergeCell ref="G11:L11"/>
+    <mergeCell ref="M11:R11"/>
+    <mergeCell ref="S11:X11"/>
     <mergeCell ref="A13:I13"/>
     <mergeCell ref="J13:O13"/>
     <mergeCell ref="P13:X13"/>
@@ -7966,25 +8041,13 @@
     <mergeCell ref="T16:X16"/>
     <mergeCell ref="A17:I18"/>
     <mergeCell ref="J17:M18"/>
-    <mergeCell ref="A8:I8"/>
-    <mergeCell ref="J8:O8"/>
-    <mergeCell ref="P8:X8"/>
-    <mergeCell ref="A10:X10"/>
-    <mergeCell ref="A11:F11"/>
-    <mergeCell ref="G11:L11"/>
-    <mergeCell ref="M11:R11"/>
-    <mergeCell ref="S11:X11"/>
-    <mergeCell ref="A1:T1"/>
-    <mergeCell ref="U1:X1"/>
-    <mergeCell ref="A2:T2"/>
-    <mergeCell ref="A7:I7"/>
-    <mergeCell ref="J7:O7"/>
-    <mergeCell ref="P7:X7"/>
-    <mergeCell ref="A5:M5"/>
-    <mergeCell ref="A4:M4"/>
-    <mergeCell ref="N4:X4"/>
-    <mergeCell ref="N5:X5"/>
-    <mergeCell ref="U2:X3"/>
+    <mergeCell ref="P23:T23"/>
+    <mergeCell ref="U23:X23"/>
+    <mergeCell ref="P24:T24"/>
+    <mergeCell ref="U24:X24"/>
+    <mergeCell ref="A21:H21"/>
+    <mergeCell ref="J21:P21"/>
+    <mergeCell ref="R21:X21"/>
   </mergeCells>
   <pageMargins left="0.51181102362204722" right="0.51181102362204722" top="0.35433070866141736" bottom="0.35433070866141736" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup scale="95" orientation="landscape" horizontalDpi="4294967294" verticalDpi="200" r:id="rId1"/>
@@ -7993,37 +8056,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <TaxCatchAll xmlns="41dd0a9e-964d-48c8-9389-7445c2a187f7" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="edbb1c21-1b45-407e-8894-c97732534993">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <_Flow_SignoffStatus xmlns="edbb1c21-1b45-407e-8894-c97732534993" xsi:nil="true"/>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <_x0031_010005470 xmlns="edbb1c21-1b45-407e-8894-c97732534993">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </_x0031_010005470>
-    <FechayHora xmlns="edbb1c21-1b45-407e-8894-c97732534993" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x01010080239B14884FBB46AB47CE62E6B5D997" ma:contentTypeVersion="24" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="95cfff668db4ca1e5f6e9375137a4a8e">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="edbb1c21-1b45-407e-8894-c97732534993" xmlns:ns3="41dd0a9e-964d-48c8-9389-7445c2a187f7" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="6912f17aaadcd6a9684df23b147afc35" ns1:_="" ns2:_="" ns3:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -8333,10 +8365,53 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <TaxCatchAll xmlns="41dd0a9e-964d-48c8-9389-7445c2a187f7" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="edbb1c21-1b45-407e-8894-c97732534993">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <_Flow_SignoffStatus xmlns="edbb1c21-1b45-407e-8894-c97732534993" xsi:nil="true"/>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <_x0031_010005470 xmlns="edbb1c21-1b45-407e-8894-c97732534993">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </_x0031_010005470>
+    <FechayHora xmlns="edbb1c21-1b45-407e-8894-c97732534993" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2FFAC935-8881-451D-93ED-25958414B4DF}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2E0DC6A2-D4C3-4E6B-B67E-9AED22EC483E}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="edbb1c21-1b45-407e-8894-c97732534993"/>
+    <ds:schemaRef ds:uri="41dd0a9e-964d-48c8-9389-7445c2a187f7"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -8354,21 +8429,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2E0DC6A2-D4C3-4E6B-B67E-9AED22EC483E}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2FFAC935-8881-451D-93ED-25958414B4DF}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="edbb1c21-1b45-407e-8894-c97732534993"/>
-    <ds:schemaRef ds:uri="41dd0a9e-964d-48c8-9389-7445c2a187f7"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Actualiza formatos de Visitas 1-3 y Bitácora F-147 en el centro de descargas.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Formatos/BITACORAS GFPI-F-147V4.xlsx
+++ b/Formatos/BITACORAS GFPI-F-147V4.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uniminuto0-my.sharepoint.com/personal/sergio_torres_mar_uniminuto_edu_co/Documents/Documentos/Seto 2026/SETO/sena/Manual SENA Etapa Productiva/manual-aprendiz-sena/Formatos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="25" documentId="13_ncr:1_{BEF1DC7A-FFF1-4291-A724-1398C9A655DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C48CE772-E924-4622-97BD-AE0184CF7A9F}"/>
+  <xr:revisionPtr revIDLastSave="28" documentId="13_ncr:1_{BEF1DC7A-FFF1-4291-A724-1398C9A655DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BE7C01BD-B2B8-415E-96E3-3A793F80C382}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-105" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Bitacora" sheetId="6" r:id="rId1"/>
@@ -373,278 +373,278 @@
     </r>
   </si>
   <si>
+    <t xml:space="preserve"> (No aplica documentos de la empresa u otros aspectos sensibles)</t>
+  </si>
+  <si>
+    <t>BITACORA DE SEGUIMIENTO</t>
+  </si>
+  <si>
+    <t>Consecutivo</t>
+  </si>
+  <si>
+    <t>A medida que vaya realizando las bitacoras le coloca el número respectivo, es decir, si es la primera bitacora será el # 1</t>
+  </si>
+  <si>
+    <t>Nombre de la empresa donde esta realizando las prácticas académicas</t>
+  </si>
+  <si>
+    <t>NIT DE LA EMPRESA</t>
+  </si>
+  <si>
+    <t>Nombre del jefe inmediato</t>
+  </si>
+  <si>
+    <t>Teléfono de contacto</t>
+  </si>
+  <si>
+    <t>Correo electrónico</t>
+  </si>
+  <si>
+    <t>Telefono de la empresa</t>
+  </si>
+  <si>
+    <t>Correo electrónico del jefe inmediato</t>
+  </si>
+  <si>
+    <t>Seleccione con una "X" el tipo de contrato</t>
+  </si>
+  <si>
+    <t>CONTRATO DE APRENDIZAJE</t>
+  </si>
+  <si>
+    <t>ASESORIA MYPIMES</t>
+  </si>
+  <si>
+    <t>CONTRATO LABORAL</t>
+  </si>
+  <si>
+    <t>PROYECTO</t>
+  </si>
+  <si>
+    <t>Nombre del aprendiz</t>
+  </si>
+  <si>
+    <t>Telefono del aprendiz</t>
+  </si>
+  <si>
+    <t>Correo electrónico del aprendiz</t>
+  </si>
+  <si>
+    <t>DESCRIPCION DE LA ACTIVIDAD</t>
+  </si>
+  <si>
+    <t>PERIODO / MES</t>
+  </si>
+  <si>
+    <t>EVIDENCIA DE CUMPLIMIENTO</t>
+  </si>
+  <si>
+    <t>OBSERVACIONES DEL APRENDIZ Y/O JEFE INMEDIATO</t>
+  </si>
+  <si>
+    <t>Se detalla la actividad realzada</t>
+  </si>
+  <si>
+    <t>Se ubica el mes que realiza la actividad escrita en la celda anterior</t>
+  </si>
+  <si>
+    <t>Se coloca el nombre del registro, por ejemplo, si la actividad fue una inspección, entonces la evidencia es la inspección</t>
+  </si>
+  <si>
+    <t>Se diligencia sólo si tienen alguna observación, si no la tienen se deja en blanco</t>
+  </si>
+  <si>
+    <t>Firma del jefe inmediato y sello de la empresa</t>
+  </si>
+  <si>
+    <t>Firma del instructor</t>
+  </si>
+  <si>
+    <t>Fecha de entrega de la bitácora:</t>
+  </si>
+  <si>
+    <t>Lo diligencia el instructor que recibe la bitácora</t>
+  </si>
+  <si>
+    <t>Firma de recibido:</t>
+  </si>
+  <si>
+    <t>firma el instructor que recibe la bitácora</t>
+  </si>
+  <si>
+    <t>SERGIO ANDRES TORRES MARTINEZ</t>
+  </si>
+  <si>
+    <t>satorres@sena.edu.co   /    storres@timespanish.com</t>
+  </si>
+  <si>
+    <t>PROGRAMA</t>
+  </si>
+  <si>
+    <t>COMPETENCIA</t>
+  </si>
+  <si>
+    <t>RESULTADO DE APRENDIZAJE (RAP)</t>
+  </si>
+  <si>
+    <t>Análisis y Desarrollo de Software</t>
+  </si>
+  <si>
+    <t>38392 - Establecer requisitos de la solución de software de acuerdo con estándares y procedimiento técnico</t>
+  </si>
+  <si>
+    <t>38376 - Evaluar requisitos de la solución de software de acuerdo con metodologías de análisis y estándares</t>
+  </si>
+  <si>
+    <t>38362 - Diseñar la solución de software de acuerdo con procedimientos y requisitos técnicos</t>
+  </si>
+  <si>
+    <t>38368 - Desarrollar la solución de software de acuerdo con el diseño y metodologías de desarrollo</t>
+  </si>
+  <si>
+    <t>38369 - Controlar la calidad del servicio de software de acuerdo con los estándares técnicos</t>
+  </si>
+  <si>
+    <t>38367 - Estructurar propuesta técnica de servicio de tecnología de la información según requisitos técnicos y normativa</t>
+  </si>
+  <si>
+    <t>38356 - Implementar la solución de software de acuerdo con los requisitos de operación y modelos de referencia</t>
+  </si>
+  <si>
+    <t>Programación de Software</t>
+  </si>
+  <si>
+    <t>220501095 - Construir el sistema de información de acuerdo con el diseño y estándares técnicos</t>
+  </si>
+  <si>
+    <t>220501096 - Verificar la calidad del software de acuerdo con el plan de pruebas y estándares</t>
+  </si>
+  <si>
+    <t>220501097 - Desplegar la solución de software de acuerdo con los requisitos de operación y modelos de referencia</t>
+  </si>
+  <si>
+    <t>220501101 - Probar el software desarrollado de acuerdo con el plan de pruebas y especificaciones del cliente</t>
+  </si>
+  <si>
+    <t>37371 - Utilizar herramientas informáticas de acuerdo con las necesidades de manejo de información</t>
+  </si>
+  <si>
+    <t>593346 - 01 CARACTERIZAR LOS PROCESOS DE LA ORGANIZACIÓN DE ACUERDO CON EL SOFTWARE A CONSTRUIR</t>
+  </si>
+  <si>
+    <t>593345 - 04 VALIDAR EL INFORME DE REQUISITOS DE ACUERDO CON LAS NECESIDADES DEL CLIENTE</t>
+  </si>
+  <si>
+    <t>593344 - 02 RECOLECTAR INFORMACIÓN DEL SOFTWARE A CONSTRUIR DE ACUERDO CON LAS NECESIDADES DEL CLIENTE</t>
+  </si>
+  <si>
+    <t>38392 - 03 ESTABLECER LOS REQUISITOS DEL SOFTWARE DE ACUERDO CON LA INFORMACIÓN RECOLECTADA</t>
+  </si>
+  <si>
+    <t>592375 - 01 PLANEAR ACTIVIDADES DE ANÁLISIS DE ACUERDO CON LA METODOLOGÍA SELECCIONADA</t>
+  </si>
+  <si>
+    <t>592374 - 04 VERIFICAR LOS MODELOS REALIZADOS EN LA FASE DE ANÁLISIS DE ACUERDO CON LO ESTABLECIDO EN EL INFORME DE REQUISITOS</t>
+  </si>
+  <si>
+    <t>592376 - 03 DESARROLLAR PROCESOS LÓGICOS A TRAVÉS DE LA IMPLEMENTACIÓN DE ALGORITMOS</t>
+  </si>
+  <si>
+    <t>592373 - 02 MODELAR LAS FUNCIONES DEL SOFTWARE DE ACUERDO CON EL INFORME DE REQUISITOS</t>
+  </si>
+  <si>
+    <t>593101 - 02 ESTRUCTURAR EL MODELO DE DATOS DEL SOFTWARE DE ACUERDO CON LAS ESPECIFICACIONES DEL ANÁLISIS</t>
+  </si>
+  <si>
+    <t>593103 - 01 ELABORAR LOS ARTEFACTOS DE DISEÑO DEL SOFTWARE SIGUIENDO LAS PRÁCTICAS DE LA METODOLOGÍA SELECCIONADA</t>
+  </si>
+  <si>
+    <t>593102 - 04 VERIFICAR LOS ENTREGABLES DE LA FASE DE DISEÑO DEL SOFTWARE DE ACUERDO CON LO ESTABLECIDO EN EL INFORME DE ANÁLISIS</t>
+  </si>
+  <si>
+    <t>593100 - 03 DETERMINAR LAS CARACTERÍSTICAS TÉCNICAS DE LA INTERFAZ GRÁFICA DEL SOFTWARE ADOPTANDO ESTÁNDARES</t>
+  </si>
+  <si>
+    <t>593107 - 02 CONSTRUIR LA BASE DE DATOS PARA EL SOFTWARE A PARTIR DEL MODELO DE DATOS</t>
+  </si>
+  <si>
+    <t>593106 - 01 PLANEAR ACTIVIDADES DE CONSTRUCCIÓN DEL SOFTWARE DE ACUERDO CON EL DISEÑO ESTABLECIDO</t>
+  </si>
+  <si>
+    <t>593104 - 03 CREAR COMPONENTES FRONT-END DEL SOFTWARE DE ACUERDO CON EL DISEÑO</t>
+  </si>
+  <si>
+    <t>593108 - 04 CODIFICAR EL SOFTWARE DE ACUERDO CON EL DISEÑO ESTABLECIDO</t>
+  </si>
+  <si>
+    <t>593105 - 05 REALIZAR PRUEBAS AL SOFTWARE PARA VERIFICAR SU FUNCIONALIDAD</t>
+  </si>
+  <si>
+    <t>593146 - 01 INCORPORAR ACTIVIDADES DE ASEGURAMIENTO DE LA CALIDAD DEL SOFTWARE DE ACUERDO CON ESTÁNDARES DE LA INDUSTRIA</t>
+  </si>
+  <si>
+    <t>593144 - 02 VERIFICAR LA CALIDAD DEL SOFTWARE DE ACUERDO CON LAS PRÁCTICAS ASOCIADAS EN LOS PROCESOS DE DESARROLLO</t>
+  </si>
+  <si>
+    <t>593145 - 03 REALIZAR ACTIVIDADES DE MEJORA DE LA CALIDAD DEL SOFTWARE A PARTIR DE LOS RESULTADOS DE LA VERIFICACIÓN</t>
+  </si>
+  <si>
+    <t>593060 - 01 DEFINIR ESPECIFICACIONES TÉCNICAS DEL SOFTWARE DE ACUERDO CON LAS CARACTERÍSTICAS DEL SOFTWARE A CONSTRUIR</t>
+  </si>
+  <si>
+    <t>593062 - 02 ELABORAR PROPUESTA TÉCNICA DEL SOFTWARE DE ACUERDO CON LAS ESPECIFICACIONES TÉCNICAS DEFINIDAS</t>
+  </si>
+  <si>
+    <t>593111 - 01 PLANEAR ACTIVIDADES DE IMPLANTACIÓN DEL SOFTWARE DE ACUERDO CON LAS CONDICIONES DEL SISTEMA</t>
+  </si>
+  <si>
+    <t>593109 - 03 DOCUMENTAR EL PROCESO DE IMPLANTACIÓN DE SOFTWARE SIGUIENDO ESTÁNDARES DE CALIDAD</t>
+  </si>
+  <si>
+    <t>593112 - 04 IMPLANTAR EL SOFTWARE DE ACUERDO CON LOS NIVELES DE SERVICIO ESTABLECIDOS CON EL CLIENTE</t>
+  </si>
+  <si>
+    <t>593110 - 02 DESPLEGAR EL SOFTWARE DE ACUERDO CON LA ARQUITECTURA Y LAS POLÍTICAS ESTABLECIDAS</t>
+  </si>
+  <si>
+    <t>220501095-01 Codificar los módulos del software de acuerdo con el diseño y estándares técnicos</t>
+  </si>
+  <si>
+    <t>220501095-02 Construir la base de datos de acuerdo con el modelo lógico y el motor seleccionado</t>
+  </si>
+  <si>
+    <t>220501095-03 Integrar los componentes del software según la arquitectura definida</t>
+  </si>
+  <si>
+    <t>220501095-04 Realizar las pruebas unitarias a los módulos codificados</t>
+  </si>
+  <si>
+    <t>220501096-01 Ejecutar las pruebas de software de acuerdo con el plan establecido</t>
+  </si>
+  <si>
+    <t>220501096-02 Reportar los defectos encontrados durante la ejecución de las pruebas</t>
+  </si>
+  <si>
+    <t>220501096-03 Ajustar los entregables de software según los resultados de las pruebas</t>
+  </si>
+  <si>
+    <t>220501097-01 Elaborar el plan de despliegue de la solución de software</t>
+  </si>
+  <si>
+    <t>220501097-02 Realizar la instalación y configuración del software en el entorno productivo</t>
+  </si>
+  <si>
+    <t>220501101-01 Validar el cumplimiento de los requisitos del software</t>
+  </si>
+  <si>
+    <t>220501101-02 Documentar los errores y sugerencias de mejora según protocolos</t>
+  </si>
+  <si>
+    <t>593154 - 01 ALISTAR HERRAMIENTAS DE TECNOLOGÍAS DE LA INFORMACIÓN Y LA COMUNICACIÓN (TIC), DE ACUERDO CON LAS NECESIDADES DE PROCESAMIENTO DE INFORMACIÓN Y COMUNICACIÓN</t>
+  </si>
+  <si>
     <t xml:space="preserve">Anexo: 
-Es opcional relacionar evidencia fotográfica de las actividades desarrolladas </t>
-  </si>
-  <si>
-    <t xml:space="preserve"> (No aplica documentos de la empresa u otros aspectos sensibles)</t>
-  </si>
-  <si>
-    <t>BITACORA DE SEGUIMIENTO</t>
-  </si>
-  <si>
-    <t>Consecutivo</t>
-  </si>
-  <si>
-    <t>A medida que vaya realizando las bitacoras le coloca el número respectivo, es decir, si es la primera bitacora será el # 1</t>
-  </si>
-  <si>
-    <t>Nombre de la empresa donde esta realizando las prácticas académicas</t>
-  </si>
-  <si>
-    <t>NIT DE LA EMPRESA</t>
-  </si>
-  <si>
-    <t>Nombre del jefe inmediato</t>
-  </si>
-  <si>
-    <t>Teléfono de contacto</t>
-  </si>
-  <si>
-    <t>Correo electrónico</t>
-  </si>
-  <si>
-    <t>Telefono de la empresa</t>
-  </si>
-  <si>
-    <t>Correo electrónico del jefe inmediato</t>
-  </si>
-  <si>
-    <t>Seleccione con una "X" el tipo de contrato</t>
-  </si>
-  <si>
-    <t>CONTRATO DE APRENDIZAJE</t>
-  </si>
-  <si>
-    <t>ASESORIA MYPIMES</t>
-  </si>
-  <si>
-    <t>CONTRATO LABORAL</t>
-  </si>
-  <si>
-    <t>PROYECTO</t>
-  </si>
-  <si>
-    <t>Nombre del aprendiz</t>
-  </si>
-  <si>
-    <t>Telefono del aprendiz</t>
-  </si>
-  <si>
-    <t>Correo electrónico del aprendiz</t>
-  </si>
-  <si>
-    <t>DESCRIPCION DE LA ACTIVIDAD</t>
-  </si>
-  <si>
-    <t>PERIODO / MES</t>
-  </si>
-  <si>
-    <t>EVIDENCIA DE CUMPLIMIENTO</t>
-  </si>
-  <si>
-    <t>OBSERVACIONES DEL APRENDIZ Y/O JEFE INMEDIATO</t>
-  </si>
-  <si>
-    <t>Se detalla la actividad realzada</t>
-  </si>
-  <si>
-    <t>Se ubica el mes que realiza la actividad escrita en la celda anterior</t>
-  </si>
-  <si>
-    <t>Se coloca el nombre del registro, por ejemplo, si la actividad fue una inspección, entonces la evidencia es la inspección</t>
-  </si>
-  <si>
-    <t>Se diligencia sólo si tienen alguna observación, si no la tienen se deja en blanco</t>
-  </si>
-  <si>
-    <t>Firma del jefe inmediato y sello de la empresa</t>
-  </si>
-  <si>
-    <t>Firma del instructor</t>
-  </si>
-  <si>
-    <t>Fecha de entrega de la bitácora:</t>
-  </si>
-  <si>
-    <t>Lo diligencia el instructor que recibe la bitácora</t>
-  </si>
-  <si>
-    <t>Firma de recibido:</t>
-  </si>
-  <si>
-    <t>firma el instructor que recibe la bitácora</t>
-  </si>
-  <si>
-    <t>SERGIO ANDRES TORRES MARTINEZ</t>
-  </si>
-  <si>
-    <t>satorres@sena.edu.co   /    storres@timespanish.com</t>
-  </si>
-  <si>
-    <t>PROGRAMA</t>
-  </si>
-  <si>
-    <t>COMPETENCIA</t>
-  </si>
-  <si>
-    <t>RESULTADO DE APRENDIZAJE (RAP)</t>
-  </si>
-  <si>
-    <t>Análisis y Desarrollo de Software</t>
-  </si>
-  <si>
-    <t>38392 - Establecer requisitos de la solución de software de acuerdo con estándares y procedimiento técnico</t>
-  </si>
-  <si>
-    <t>38376 - Evaluar requisitos de la solución de software de acuerdo con metodologías de análisis y estándares</t>
-  </si>
-  <si>
-    <t>38362 - Diseñar la solución de software de acuerdo con procedimientos y requisitos técnicos</t>
-  </si>
-  <si>
-    <t>38368 - Desarrollar la solución de software de acuerdo con el diseño y metodologías de desarrollo</t>
-  </si>
-  <si>
-    <t>38369 - Controlar la calidad del servicio de software de acuerdo con los estándares técnicos</t>
-  </si>
-  <si>
-    <t>38367 - Estructurar propuesta técnica de servicio de tecnología de la información según requisitos técnicos y normativa</t>
-  </si>
-  <si>
-    <t>38356 - Implementar la solución de software de acuerdo con los requisitos de operación y modelos de referencia</t>
-  </si>
-  <si>
-    <t>Programación de Software</t>
-  </si>
-  <si>
-    <t>220501095 - Construir el sistema de información de acuerdo con el diseño y estándares técnicos</t>
-  </si>
-  <si>
-    <t>220501096 - Verificar la calidad del software de acuerdo con el plan de pruebas y estándares</t>
-  </si>
-  <si>
-    <t>220501097 - Desplegar la solución de software de acuerdo con los requisitos de operación y modelos de referencia</t>
-  </si>
-  <si>
-    <t>220501101 - Probar el software desarrollado de acuerdo con el plan de pruebas y especificaciones del cliente</t>
-  </si>
-  <si>
-    <t>37371 - Utilizar herramientas informáticas de acuerdo con las necesidades de manejo de información</t>
-  </si>
-  <si>
-    <t>593346 - 01 CARACTERIZAR LOS PROCESOS DE LA ORGANIZACIÓN DE ACUERDO CON EL SOFTWARE A CONSTRUIR</t>
-  </si>
-  <si>
-    <t>593345 - 04 VALIDAR EL INFORME DE REQUISITOS DE ACUERDO CON LAS NECESIDADES DEL CLIENTE</t>
-  </si>
-  <si>
-    <t>593344 - 02 RECOLECTAR INFORMACIÓN DEL SOFTWARE A CONSTRUIR DE ACUERDO CON LAS NECESIDADES DEL CLIENTE</t>
-  </si>
-  <si>
-    <t>38392 - 03 ESTABLECER LOS REQUISITOS DEL SOFTWARE DE ACUERDO CON LA INFORMACIÓN RECOLECTADA</t>
-  </si>
-  <si>
-    <t>592375 - 01 PLANEAR ACTIVIDADES DE ANÁLISIS DE ACUERDO CON LA METODOLOGÍA SELECCIONADA</t>
-  </si>
-  <si>
-    <t>592374 - 04 VERIFICAR LOS MODELOS REALIZADOS EN LA FASE DE ANÁLISIS DE ACUERDO CON LO ESTABLECIDO EN EL INFORME DE REQUISITOS</t>
-  </si>
-  <si>
-    <t>592376 - 03 DESARROLLAR PROCESOS LÓGICOS A TRAVÉS DE LA IMPLEMENTACIÓN DE ALGORITMOS</t>
-  </si>
-  <si>
-    <t>592373 - 02 MODELAR LAS FUNCIONES DEL SOFTWARE DE ACUERDO CON EL INFORME DE REQUISITOS</t>
-  </si>
-  <si>
-    <t>593101 - 02 ESTRUCTURAR EL MODELO DE DATOS DEL SOFTWARE DE ACUERDO CON LAS ESPECIFICACIONES DEL ANÁLISIS</t>
-  </si>
-  <si>
-    <t>593103 - 01 ELABORAR LOS ARTEFACTOS DE DISEÑO DEL SOFTWARE SIGUIENDO LAS PRÁCTICAS DE LA METODOLOGÍA SELECCIONADA</t>
-  </si>
-  <si>
-    <t>593102 - 04 VERIFICAR LOS ENTREGABLES DE LA FASE DE DISEÑO DEL SOFTWARE DE ACUERDO CON LO ESTABLECIDO EN EL INFORME DE ANÁLISIS</t>
-  </si>
-  <si>
-    <t>593100 - 03 DETERMINAR LAS CARACTERÍSTICAS TÉCNICAS DE LA INTERFAZ GRÁFICA DEL SOFTWARE ADOPTANDO ESTÁNDARES</t>
-  </si>
-  <si>
-    <t>593107 - 02 CONSTRUIR LA BASE DE DATOS PARA EL SOFTWARE A PARTIR DEL MODELO DE DATOS</t>
-  </si>
-  <si>
-    <t>593106 - 01 PLANEAR ACTIVIDADES DE CONSTRUCCIÓN DEL SOFTWARE DE ACUERDO CON EL DISEÑO ESTABLECIDO</t>
-  </si>
-  <si>
-    <t>593104 - 03 CREAR COMPONENTES FRONT-END DEL SOFTWARE DE ACUERDO CON EL DISEÑO</t>
-  </si>
-  <si>
-    <t>593108 - 04 CODIFICAR EL SOFTWARE DE ACUERDO CON EL DISEÑO ESTABLECIDO</t>
-  </si>
-  <si>
-    <t>593105 - 05 REALIZAR PRUEBAS AL SOFTWARE PARA VERIFICAR SU FUNCIONALIDAD</t>
-  </si>
-  <si>
-    <t>593146 - 01 INCORPORAR ACTIVIDADES DE ASEGURAMIENTO DE LA CALIDAD DEL SOFTWARE DE ACUERDO CON ESTÁNDARES DE LA INDUSTRIA</t>
-  </si>
-  <si>
-    <t>593144 - 02 VERIFICAR LA CALIDAD DEL SOFTWARE DE ACUERDO CON LAS PRÁCTICAS ASOCIADAS EN LOS PROCESOS DE DESARROLLO</t>
-  </si>
-  <si>
-    <t>593145 - 03 REALIZAR ACTIVIDADES DE MEJORA DE LA CALIDAD DEL SOFTWARE A PARTIR DE LOS RESULTADOS DE LA VERIFICACIÓN</t>
-  </si>
-  <si>
-    <t>593060 - 01 DEFINIR ESPECIFICACIONES TÉCNICAS DEL SOFTWARE DE ACUERDO CON LAS CARACTERÍSTICAS DEL SOFTWARE A CONSTRUIR</t>
-  </si>
-  <si>
-    <t>593062 - 02 ELABORAR PROPUESTA TÉCNICA DEL SOFTWARE DE ACUERDO CON LAS ESPECIFICACIONES TÉCNICAS DEFINIDAS</t>
-  </si>
-  <si>
-    <t>593111 - 01 PLANEAR ACTIVIDADES DE IMPLANTACIÓN DEL SOFTWARE DE ACUERDO CON LAS CONDICIONES DEL SISTEMA</t>
-  </si>
-  <si>
-    <t>593109 - 03 DOCUMENTAR EL PROCESO DE IMPLANTACIÓN DE SOFTWARE SIGUIENDO ESTÁNDARES DE CALIDAD</t>
-  </si>
-  <si>
-    <t>593112 - 04 IMPLANTAR EL SOFTWARE DE ACUERDO CON LOS NIVELES DE SERVICIO ESTABLECIDOS CON EL CLIENTE</t>
-  </si>
-  <si>
-    <t>593110 - 02 DESPLEGAR EL SOFTWARE DE ACUERDO CON LA ARQUITECTURA Y LAS POLÍTICAS ESTABLECIDAS</t>
-  </si>
-  <si>
-    <t>220501095-01 Codificar los módulos del software de acuerdo con el diseño y estándares técnicos</t>
-  </si>
-  <si>
-    <t>220501095-02 Construir la base de datos de acuerdo con el modelo lógico y el motor seleccionado</t>
-  </si>
-  <si>
-    <t>220501095-03 Integrar los componentes del software según la arquitectura definida</t>
-  </si>
-  <si>
-    <t>220501095-04 Realizar las pruebas unitarias a los módulos codificados</t>
-  </si>
-  <si>
-    <t>220501096-01 Ejecutar las pruebas de software de acuerdo con el plan establecido</t>
-  </si>
-  <si>
-    <t>220501096-02 Reportar los defectos encontrados durante la ejecución de las pruebas</t>
-  </si>
-  <si>
-    <t>220501096-03 Ajustar los entregables de software según los resultados de las pruebas</t>
-  </si>
-  <si>
-    <t>220501097-01 Elaborar el plan de despliegue de la solución de software</t>
-  </si>
-  <si>
-    <t>220501097-02 Realizar la instalación y configuración del software en el entorno productivo</t>
-  </si>
-  <si>
-    <t>220501101-01 Validar el cumplimiento de los requisitos del software</t>
-  </si>
-  <si>
-    <t>220501101-02 Documentar los errores y sugerencias de mejora según protocolos</t>
-  </si>
-  <si>
-    <t>593154 - 01 ALISTAR HERRAMIENTAS DE TECNOLOGÍAS DE LA INFORMACIÓN Y LA COMUNICACIÓN (TIC), DE ACUERDO CON LAS NECESIDADES DE PROCESAMIENTO DE INFORMACIÓN Y COMUNICACIÓN</t>
+Relacionar evidencia fotográfica de las actividades desarrolladas </t>
   </si>
 </sst>
 </file>
@@ -2720,7 +2720,10 @@
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="94" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="94" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2734,6 +2737,12 @@
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="93" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="93" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2741,6 +2750,12 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="93" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="93" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="61" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2771,6 +2786,9 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="94" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3276,38 +3294,13 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="93" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="94" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="93" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="16">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFE1EF57"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="10">
     <dxf>
       <fill>
         <patternFill>
@@ -3326,41 +3319,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFE1EF57"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFE2ED51"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3714,17 +3672,13 @@
 </externalLink>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{99010CAF-386D-41BE-AE72-8D38EFA83A09}" name="TablaSena" displayName="TablaSena" ref="A1:C39" totalsRowShown="0" headerRowDxfId="15" headerRowBorderDxfId="14" tableBorderDxfId="13" totalsRowBorderDxfId="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{99010CAF-386D-41BE-AE72-8D38EFA83A09}" name="TablaSena" displayName="TablaSena" ref="A1:C39" totalsRowShown="0" headerRowDxfId="9" headerRowBorderDxfId="8" tableBorderDxfId="7" totalsRowBorderDxfId="6">
   <autoFilter ref="A1:C39" xr:uid="{99010CAF-386D-41BE-AE72-8D38EFA83A09}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{61F34070-348E-42B3-BF87-5A1CD2BB6FD7}" name="PROGRAMA" dataDxfId="11"/>
-    <tableColumn id="2" xr3:uid="{7B4CB996-89B6-45DE-A53A-D02152366731}" name="COMPETENCIA" dataDxfId="10"/>
-    <tableColumn id="3" xr3:uid="{529DD12A-961C-42BF-9AA1-50D419FC6C5E}" name="RESULTADO DE APRENDIZAJE (RAP)" dataDxfId="9"/>
+    <tableColumn id="1" xr3:uid="{61F34070-348E-42B3-BF87-5A1CD2BB6FD7}" name="PROGRAMA" dataDxfId="5"/>
+    <tableColumn id="2" xr3:uid="{7B4CB996-89B6-45DE-A53A-D02152366731}" name="COMPETENCIA" dataDxfId="4"/>
+    <tableColumn id="3" xr3:uid="{529DD12A-961C-42BF-9AA1-50D419FC6C5E}" name="RESULTADO DE APRENDIZAJE (RAP)" dataDxfId="3"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium6" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -4020,7 +3974,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:XFD113"/>
+  <dimension ref="A1:XFC113"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="0" defaultRowHeight="15" customHeight="1" zeroHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2.28515625" style="36" customWidth="1"/>
@@ -4112,16 +4066,16 @@
       <c r="AB2" s="7"/>
     </row>
     <row r="3" spans="2:28" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="133" t="s">
+      <c r="B3" s="139" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="134"/>
-      <c r="D3" s="134"/>
-      <c r="E3" s="134"/>
-      <c r="F3" s="134"/>
-      <c r="G3" s="134"/>
-      <c r="H3" s="134"/>
-      <c r="I3" s="135"/>
+      <c r="C3" s="140"/>
+      <c r="D3" s="140"/>
+      <c r="E3" s="140"/>
+      <c r="F3" s="140"/>
+      <c r="G3" s="140"/>
+      <c r="H3" s="140"/>
+      <c r="I3" s="141"/>
       <c r="J3" s="8"/>
       <c r="K3" s="7"/>
       <c r="L3" s="7"/>
@@ -4143,16 +4097,16 @@
       <c r="AB3" s="7"/>
     </row>
     <row r="4" spans="2:28" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="139" t="s">
+      <c r="B4" s="145" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="140"/>
-      <c r="D4" s="140"/>
-      <c r="E4" s="140"/>
-      <c r="F4" s="140"/>
-      <c r="G4" s="140"/>
-      <c r="H4" s="140"/>
-      <c r="I4" s="141"/>
+      <c r="C4" s="146"/>
+      <c r="D4" s="146"/>
+      <c r="E4" s="146"/>
+      <c r="F4" s="146"/>
+      <c r="G4" s="146"/>
+      <c r="H4" s="146"/>
+      <c r="I4" s="147"/>
       <c r="J4" s="8"/>
       <c r="K4" s="7"/>
       <c r="L4" s="7"/>
@@ -4174,16 +4128,16 @@
       <c r="AB4" s="7"/>
     </row>
     <row r="5" spans="2:28" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="136" t="s">
+      <c r="B5" s="142" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="137"/>
-      <c r="D5" s="137"/>
-      <c r="E5" s="137"/>
-      <c r="F5" s="137"/>
-      <c r="G5" s="137"/>
-      <c r="H5" s="137"/>
-      <c r="I5" s="138"/>
+      <c r="C5" s="143"/>
+      <c r="D5" s="143"/>
+      <c r="E5" s="143"/>
+      <c r="F5" s="143"/>
+      <c r="G5" s="143"/>
+      <c r="H5" s="143"/>
+      <c r="I5" s="144"/>
       <c r="J5" s="8"/>
       <c r="K5" s="8"/>
       <c r="L5" s="7"/>
@@ -4205,16 +4159,16 @@
       <c r="AB5" s="7"/>
     </row>
     <row r="6" spans="2:28" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="139" t="s">
+      <c r="B6" s="145" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="140"/>
-      <c r="D6" s="140"/>
-      <c r="E6" s="140"/>
-      <c r="F6" s="140"/>
-      <c r="G6" s="140"/>
-      <c r="H6" s="140"/>
-      <c r="I6" s="141"/>
+      <c r="C6" s="146"/>
+      <c r="D6" s="146"/>
+      <c r="E6" s="146"/>
+      <c r="F6" s="146"/>
+      <c r="G6" s="146"/>
+      <c r="H6" s="146"/>
+      <c r="I6" s="147"/>
       <c r="J6" s="8"/>
       <c r="K6" s="8"/>
       <c r="L6" s="7"/>
@@ -4236,16 +4190,16 @@
       <c r="AB6" s="7"/>
     </row>
     <row r="7" spans="2:28" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="136" t="s">
+      <c r="B7" s="142" t="s">
         <v>6</v>
       </c>
-      <c r="C7" s="137"/>
-      <c r="D7" s="137"/>
-      <c r="E7" s="137"/>
-      <c r="F7" s="137"/>
-      <c r="G7" s="137"/>
-      <c r="H7" s="137"/>
-      <c r="I7" s="138"/>
+      <c r="C7" s="143"/>
+      <c r="D7" s="143"/>
+      <c r="E7" s="143"/>
+      <c r="F7" s="143"/>
+      <c r="G7" s="143"/>
+      <c r="H7" s="143"/>
+      <c r="I7" s="144"/>
       <c r="J7" s="7"/>
       <c r="K7" s="7"/>
       <c r="L7" s="7"/>
@@ -4270,12 +4224,12 @@
       <c r="B8" s="53" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="152"/>
-      <c r="D8" s="153"/>
-      <c r="E8" s="154" t="s">
+      <c r="C8" s="158"/>
+      <c r="D8" s="159"/>
+      <c r="E8" s="160" t="s">
         <v>8</v>
       </c>
-      <c r="F8" s="152"/>
+      <c r="F8" s="158"/>
       <c r="G8" s="67"/>
       <c r="H8" s="54" t="s">
         <v>9</v>
@@ -4307,8 +4261,8 @@
       <c r="D9" s="18"/>
       <c r="E9" s="23"/>
       <c r="F9" s="23"/>
-      <c r="G9" s="113"/>
-      <c r="H9" s="113"/>
+      <c r="G9" s="118"/>
+      <c r="H9" s="118"/>
       <c r="I9" s="18"/>
       <c r="J9" s="7"/>
       <c r="K9" s="7"/>
@@ -4331,18 +4285,18 @@
       <c r="AB9" s="7"/>
     </row>
     <row r="10" spans="2:28" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="146" t="s">
+      <c r="B10" s="152" t="s">
         <v>10</v>
       </c>
-      <c r="C10" s="147"/>
-      <c r="D10" s="148"/>
-      <c r="E10" s="142" t="s">
+      <c r="C10" s="153"/>
+      <c r="D10" s="154"/>
+      <c r="E10" s="148" t="s">
         <v>11</v>
       </c>
-      <c r="F10" s="142"/>
-      <c r="G10" s="142"/>
-      <c r="H10" s="142"/>
-      <c r="I10" s="142"/>
+      <c r="F10" s="148"/>
+      <c r="G10" s="148"/>
+      <c r="H10" s="148"/>
+      <c r="I10" s="148"/>
       <c r="J10" s="7"/>
       <c r="K10" s="7"/>
       <c r="L10" s="7"/>
@@ -4364,14 +4318,14 @@
       <c r="AB10" s="7"/>
     </row>
     <row r="11" spans="2:28" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="125"/>
-      <c r="C11" s="126"/>
-      <c r="D11" s="127"/>
-      <c r="E11" s="161"/>
-      <c r="F11" s="161"/>
-      <c r="G11" s="161"/>
-      <c r="H11" s="161"/>
-      <c r="I11" s="161"/>
+      <c r="B11" s="131"/>
+      <c r="C11" s="132"/>
+      <c r="D11" s="133"/>
+      <c r="E11" s="167"/>
+      <c r="F11" s="167"/>
+      <c r="G11" s="167"/>
+      <c r="H11" s="167"/>
+      <c r="I11" s="167"/>
       <c r="J11" s="7"/>
       <c r="K11" s="7"/>
       <c r="L11" s="7"/>
@@ -4398,8 +4352,8 @@
       <c r="D12" s="18"/>
       <c r="E12" s="23"/>
       <c r="F12" s="23"/>
-      <c r="G12" s="113"/>
-      <c r="H12" s="113"/>
+      <c r="G12" s="118"/>
+      <c r="H12" s="118"/>
       <c r="I12" s="18"/>
       <c r="J12" s="7"/>
       <c r="K12" s="7"/>
@@ -4422,16 +4376,16 @@
       <c r="AB12" s="7"/>
     </row>
     <row r="13" spans="2:28" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="159" t="s">
+      <c r="B13" s="165" t="s">
         <v>12</v>
       </c>
-      <c r="C13" s="159"/>
-      <c r="D13" s="159"/>
-      <c r="E13" s="159"/>
-      <c r="F13" s="159"/>
-      <c r="G13" s="159"/>
-      <c r="H13" s="159"/>
-      <c r="I13" s="160"/>
+      <c r="C13" s="165"/>
+      <c r="D13" s="165"/>
+      <c r="E13" s="165"/>
+      <c r="F13" s="165"/>
+      <c r="G13" s="165"/>
+      <c r="H13" s="165"/>
+      <c r="I13" s="166"/>
       <c r="J13" s="7"/>
       <c r="K13" s="7"/>
       <c r="L13" s="7"/>
@@ -4453,32 +4407,32 @@
       <c r="AB13" s="7"/>
     </row>
     <row r="14" spans="2:28" s="9" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="146" t="s">
+      <c r="B14" s="152" t="s">
         <v>13</v>
       </c>
-      <c r="C14" s="147"/>
-      <c r="D14" s="148"/>
+      <c r="C14" s="153"/>
+      <c r="D14" s="154"/>
       <c r="E14" s="55" t="s">
         <v>14</v>
       </c>
-      <c r="F14" s="155" t="s">
+      <c r="F14" s="161" t="s">
         <v>15</v>
       </c>
-      <c r="G14" s="156"/>
-      <c r="H14" s="142" t="s">
+      <c r="G14" s="162"/>
+      <c r="H14" s="148" t="s">
         <v>16</v>
       </c>
-      <c r="I14" s="143"/>
+      <c r="I14" s="149"/>
     </row>
     <row r="15" spans="2:28" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="149"/>
-      <c r="C15" s="150"/>
-      <c r="D15" s="151"/>
+      <c r="B15" s="155"/>
+      <c r="C15" s="156"/>
+      <c r="D15" s="157"/>
       <c r="E15" s="37"/>
-      <c r="F15" s="157"/>
-      <c r="G15" s="158"/>
-      <c r="H15" s="144"/>
-      <c r="I15" s="145"/>
+      <c r="F15" s="163"/>
+      <c r="G15" s="164"/>
+      <c r="H15" s="150"/>
+      <c r="I15" s="151"/>
       <c r="J15" s="7"/>
       <c r="K15" s="7"/>
       <c r="L15" s="7"/>
@@ -4500,20 +4454,20 @@
       <c r="AB15" s="7"/>
     </row>
     <row r="16" spans="2:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="118" t="s">
+      <c r="B16" s="124" t="s">
         <v>17</v>
       </c>
-      <c r="C16" s="119"/>
-      <c r="D16" s="120"/>
-      <c r="E16" s="121" t="s">
+      <c r="C16" s="125"/>
+      <c r="D16" s="126"/>
+      <c r="E16" s="127" t="s">
         <v>18</v>
       </c>
-      <c r="F16" s="121"/>
-      <c r="G16" s="121"/>
-      <c r="H16" s="104" t="s">
+      <c r="F16" s="127"/>
+      <c r="G16" s="127"/>
+      <c r="H16" s="109" t="s">
         <v>19</v>
       </c>
-      <c r="I16" s="105"/>
+      <c r="I16" s="110"/>
       <c r="J16" s="7"/>
       <c r="K16" s="7"/>
       <c r="L16" s="7"/>
@@ -4535,14 +4489,14 @@
       <c r="AB16" s="7"/>
     </row>
     <row r="17" spans="2:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="125"/>
-      <c r="C17" s="126"/>
-      <c r="D17" s="127"/>
-      <c r="E17" s="167"/>
-      <c r="F17" s="167"/>
-      <c r="G17" s="167"/>
-      <c r="H17" s="162"/>
-      <c r="I17" s="163"/>
+      <c r="B17" s="131"/>
+      <c r="C17" s="132"/>
+      <c r="D17" s="133"/>
+      <c r="E17" s="173"/>
+      <c r="F17" s="173"/>
+      <c r="G17" s="173"/>
+      <c r="H17" s="168"/>
+      <c r="I17" s="169"/>
       <c r="J17" s="7"/>
       <c r="K17" s="7"/>
       <c r="L17" s="7"/>
@@ -4564,20 +4518,20 @@
       <c r="AB17" s="7"/>
     </row>
     <row r="18" spans="2:28" s="47" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="146" t="s">
+      <c r="B18" s="152" t="s">
         <v>20</v>
       </c>
-      <c r="C18" s="147"/>
-      <c r="D18" s="148"/>
-      <c r="E18" s="142" t="s">
+      <c r="C18" s="153"/>
+      <c r="D18" s="154"/>
+      <c r="E18" s="148" t="s">
         <v>21</v>
       </c>
-      <c r="F18" s="142"/>
-      <c r="G18" s="142"/>
-      <c r="H18" s="142" t="s">
+      <c r="F18" s="148"/>
+      <c r="G18" s="148"/>
+      <c r="H18" s="148" t="s">
         <v>22</v>
       </c>
-      <c r="I18" s="143"/>
+      <c r="I18" s="149"/>
       <c r="J18" s="7"/>
       <c r="K18" s="7"/>
       <c r="L18" s="7"/>
@@ -4599,14 +4553,14 @@
       <c r="AB18" s="7"/>
     </row>
     <row r="19" spans="2:28" s="47" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="164"/>
-      <c r="C19" s="165"/>
-      <c r="D19" s="166"/>
-      <c r="E19" s="162"/>
-      <c r="F19" s="162"/>
-      <c r="G19" s="162"/>
-      <c r="H19" s="162"/>
-      <c r="I19" s="163"/>
+      <c r="B19" s="170"/>
+      <c r="C19" s="171"/>
+      <c r="D19" s="172"/>
+      <c r="E19" s="168"/>
+      <c r="F19" s="168"/>
+      <c r="G19" s="168"/>
+      <c r="H19" s="168"/>
+      <c r="I19" s="169"/>
       <c r="J19" s="7"/>
       <c r="K19" s="7"/>
       <c r="L19" s="7"/>
@@ -4628,20 +4582,20 @@
       <c r="AB19" s="7"/>
     </row>
     <row r="20" spans="2:28" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="130" t="s">
+      <c r="B20" s="136" t="s">
         <v>23</v>
       </c>
-      <c r="C20" s="131"/>
-      <c r="D20" s="132"/>
-      <c r="E20" s="128" t="s">
+      <c r="C20" s="137"/>
+      <c r="D20" s="138"/>
+      <c r="E20" s="134" t="s">
         <v>24</v>
       </c>
-      <c r="F20" s="128"/>
-      <c r="G20" s="128"/>
-      <c r="H20" s="128" t="s">
+      <c r="F20" s="134"/>
+      <c r="G20" s="134"/>
+      <c r="H20" s="134" t="s">
         <v>25</v>
       </c>
-      <c r="I20" s="129"/>
+      <c r="I20" s="135"/>
       <c r="J20" s="16"/>
       <c r="K20" s="16"/>
       <c r="L20" s="16"/>
@@ -4661,14 +4615,14 @@
       <c r="AA20" s="16"/>
     </row>
     <row r="21" spans="2:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="125"/>
-      <c r="C21" s="126"/>
-      <c r="D21" s="127"/>
-      <c r="E21" s="144"/>
-      <c r="F21" s="144"/>
-      <c r="G21" s="144"/>
-      <c r="H21" s="173"/>
-      <c r="I21" s="174"/>
+      <c r="B21" s="131"/>
+      <c r="C21" s="132"/>
+      <c r="D21" s="133"/>
+      <c r="E21" s="150"/>
+      <c r="F21" s="150"/>
+      <c r="G21" s="150"/>
+      <c r="H21" s="179"/>
+      <c r="I21" s="180"/>
       <c r="J21" s="18"/>
       <c r="K21" s="18"/>
       <c r="L21" s="18"/>
@@ -4693,8 +4647,8 @@
       <c r="D22" s="13"/>
       <c r="E22" s="33"/>
       <c r="F22" s="33"/>
-      <c r="G22" s="112"/>
-      <c r="H22" s="112"/>
+      <c r="G22" s="117"/>
+      <c r="H22" s="117"/>
       <c r="I22" s="13"/>
       <c r="J22" s="13"/>
       <c r="K22" s="13"/>
@@ -4716,16 +4670,16 @@
       <c r="AA22" s="13"/>
     </row>
     <row r="23" spans="2:28" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="168" t="s">
+      <c r="B23" s="174" t="s">
         <v>26</v>
       </c>
-      <c r="C23" s="169"/>
-      <c r="D23" s="169"/>
-      <c r="E23" s="169"/>
-      <c r="F23" s="169"/>
-      <c r="G23" s="169"/>
-      <c r="H23" s="169"/>
-      <c r="I23" s="170"/>
+      <c r="C23" s="175"/>
+      <c r="D23" s="175"/>
+      <c r="E23" s="175"/>
+      <c r="F23" s="175"/>
+      <c r="G23" s="175"/>
+      <c r="H23" s="175"/>
+      <c r="I23" s="176"/>
       <c r="J23" s="13"/>
       <c r="K23" s="13"/>
       <c r="L23" s="13"/>
@@ -4746,20 +4700,20 @@
       <c r="AA23" s="13"/>
     </row>
     <row r="24" spans="2:28" s="9" customFormat="1" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="171" t="s">
+      <c r="B24" s="177" t="s">
         <v>27</v>
       </c>
-      <c r="C24" s="172"/>
-      <c r="D24" s="172"/>
-      <c r="E24" s="172"/>
-      <c r="F24" s="114" t="s">
+      <c r="C24" s="178"/>
+      <c r="D24" s="178"/>
+      <c r="E24" s="178"/>
+      <c r="F24" s="120" t="s">
         <v>28</v>
       </c>
-      <c r="G24" s="114"/>
-      <c r="H24" s="172" t="s">
+      <c r="G24" s="120"/>
+      <c r="H24" s="178" t="s">
         <v>29</v>
       </c>
-      <c r="I24" s="195"/>
+      <c r="I24" s="201"/>
       <c r="J24" s="18"/>
       <c r="K24" s="18"/>
       <c r="M24" s="16"/>
@@ -4772,14 +4726,14 @@
       <c r="AB24" s="10"/>
     </row>
     <row r="25" spans="2:28" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="203"/>
-      <c r="C25" s="175"/>
-      <c r="D25" s="175"/>
-      <c r="E25" s="175"/>
-      <c r="F25" s="175"/>
-      <c r="G25" s="175"/>
-      <c r="H25" s="196"/>
-      <c r="I25" s="197"/>
+      <c r="B25" s="209"/>
+      <c r="C25" s="181"/>
+      <c r="D25" s="181"/>
+      <c r="E25" s="181"/>
+      <c r="F25" s="181"/>
+      <c r="G25" s="181"/>
+      <c r="H25" s="202"/>
+      <c r="I25" s="203"/>
       <c r="J25" s="18"/>
       <c r="K25" s="18"/>
       <c r="M25" s="18"/>
@@ -4796,8 +4750,8 @@
       <c r="D26" s="13"/>
       <c r="E26" s="33"/>
       <c r="F26" s="33"/>
-      <c r="G26" s="112"/>
-      <c r="H26" s="112"/>
+      <c r="G26" s="117"/>
+      <c r="H26" s="117"/>
       <c r="I26" s="13"/>
       <c r="J26" s="13"/>
       <c r="K26" s="13"/>
@@ -4819,16 +4773,16 @@
       <c r="AA26" s="13"/>
     </row>
     <row r="27" spans="2:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B27" s="200" t="s">
+      <c r="B27" s="206" t="s">
         <v>30</v>
       </c>
-      <c r="C27" s="201"/>
-      <c r="D27" s="201"/>
-      <c r="E27" s="201"/>
-      <c r="F27" s="201"/>
-      <c r="G27" s="201"/>
-      <c r="H27" s="201"/>
-      <c r="I27" s="202"/>
+      <c r="C27" s="207"/>
+      <c r="D27" s="207"/>
+      <c r="E27" s="207"/>
+      <c r="F27" s="207"/>
+      <c r="G27" s="207"/>
+      <c r="H27" s="207"/>
+      <c r="I27" s="208"/>
       <c r="J27" s="13"/>
       <c r="K27" s="13"/>
       <c r="L27" s="13"/>
@@ -4849,22 +4803,22 @@
       <c r="AA27" s="13"/>
     </row>
     <row r="28" spans="2:28" s="9" customFormat="1" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B28" s="198" t="s">
+      <c r="B28" s="204" t="s">
         <v>31</v>
       </c>
-      <c r="C28" s="172"/>
-      <c r="D28" s="172"/>
-      <c r="E28" s="114" t="s">
+      <c r="C28" s="178"/>
+      <c r="D28" s="178"/>
+      <c r="E28" s="120" t="s">
         <v>32</v>
       </c>
-      <c r="F28" s="114"/>
+      <c r="F28" s="120"/>
       <c r="G28" s="49" t="s">
         <v>33</v>
       </c>
-      <c r="H28" s="172" t="s">
+      <c r="H28" s="178" t="s">
         <v>34</v>
       </c>
-      <c r="I28" s="199"/>
+      <c r="I28" s="205"/>
       <c r="J28" s="16"/>
       <c r="N28" s="16"/>
       <c r="O28" s="16"/>
@@ -4881,14 +4835,14 @@
       <c r="AB28" s="10"/>
     </row>
     <row r="29" spans="2:28" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B29" s="100"/>
-      <c r="C29" s="101"/>
-      <c r="D29" s="101"/>
-      <c r="E29" s="101"/>
-      <c r="F29" s="101"/>
+      <c r="B29" s="101"/>
+      <c r="C29" s="102"/>
+      <c r="D29" s="102"/>
+      <c r="E29" s="102"/>
+      <c r="F29" s="102"/>
       <c r="G29" s="52"/>
-      <c r="H29" s="101"/>
-      <c r="I29" s="97"/>
+      <c r="H29" s="102"/>
+      <c r="I29" s="119"/>
       <c r="J29" s="18"/>
       <c r="N29" s="18"/>
       <c r="O29" s="18"/>
@@ -4909,8 +4863,8 @@
       <c r="D30" s="13"/>
       <c r="E30" s="33"/>
       <c r="F30" s="33"/>
-      <c r="G30" s="112"/>
-      <c r="H30" s="112"/>
+      <c r="G30" s="117"/>
+      <c r="H30" s="117"/>
       <c r="I30" s="13"/>
       <c r="J30" s="13"/>
       <c r="K30" s="13"/>
@@ -4932,16 +4886,16 @@
       <c r="AA30" s="13"/>
     </row>
     <row r="31" spans="2:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B31" s="168" t="s">
+      <c r="B31" s="174" t="s">
         <v>35</v>
       </c>
-      <c r="C31" s="169"/>
-      <c r="D31" s="169"/>
-      <c r="E31" s="169"/>
-      <c r="F31" s="169"/>
-      <c r="G31" s="169"/>
-      <c r="H31" s="169"/>
-      <c r="I31" s="170"/>
+      <c r="C31" s="175"/>
+      <c r="D31" s="175"/>
+      <c r="E31" s="175"/>
+      <c r="F31" s="175"/>
+      <c r="G31" s="175"/>
+      <c r="H31" s="175"/>
+      <c r="I31" s="176"/>
       <c r="J31" s="7"/>
       <c r="K31" s="7"/>
       <c r="L31" s="7"/>
@@ -4963,18 +4917,18 @@
       <c r="AB31" s="7"/>
     </row>
     <row r="32" spans="2:28" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B32" s="115" t="s">
+      <c r="B32" s="121" t="s">
         <v>36</v>
       </c>
-      <c r="C32" s="116"/>
-      <c r="D32" s="116"/>
-      <c r="E32" s="116"/>
-      <c r="F32" s="117"/>
-      <c r="G32" s="231" t="s">
+      <c r="C32" s="122"/>
+      <c r="D32" s="122"/>
+      <c r="E32" s="122"/>
+      <c r="F32" s="123"/>
+      <c r="G32" s="237" t="s">
         <v>37</v>
       </c>
-      <c r="H32" s="116"/>
-      <c r="I32" s="232"/>
+      <c r="H32" s="122"/>
+      <c r="I32" s="238"/>
       <c r="J32" s="7"/>
       <c r="K32" s="7"/>
       <c r="L32" s="7"/>
@@ -4996,18 +4950,18 @@
       <c r="AB32" s="7"/>
     </row>
     <row r="33" spans="2:28" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B33" s="228" t="s">
+      <c r="B33" s="234" t="s">
+        <v>103</v>
+      </c>
+      <c r="C33" s="235"/>
+      <c r="D33" s="235"/>
+      <c r="E33" s="235"/>
+      <c r="F33" s="236"/>
+      <c r="G33" s="239" t="s">
         <v>104</v>
       </c>
-      <c r="C33" s="229"/>
-      <c r="D33" s="229"/>
-      <c r="E33" s="229"/>
-      <c r="F33" s="230"/>
-      <c r="G33" s="233" t="s">
-        <v>105</v>
-      </c>
-      <c r="H33" s="229"/>
-      <c r="I33" s="234"/>
+      <c r="H33" s="235"/>
+      <c r="I33" s="240"/>
       <c r="J33" s="7"/>
       <c r="K33" s="7"/>
       <c r="L33" s="7"/>
@@ -5034,8 +4988,8 @@
       <c r="D34" s="13"/>
       <c r="E34" s="33"/>
       <c r="F34" s="33"/>
-      <c r="G34" s="112"/>
-      <c r="H34" s="112"/>
+      <c r="G34" s="117"/>
+      <c r="H34" s="117"/>
       <c r="I34" s="13"/>
       <c r="J34" s="13"/>
       <c r="K34" s="13"/>
@@ -5057,16 +5011,16 @@
       <c r="AA34" s="13"/>
     </row>
     <row r="35" spans="2:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B35" s="183" t="s">
+      <c r="B35" s="189" t="s">
         <v>38</v>
       </c>
-      <c r="C35" s="184"/>
-      <c r="D35" s="184"/>
-      <c r="E35" s="184"/>
-      <c r="F35" s="184"/>
-      <c r="G35" s="184"/>
-      <c r="H35" s="184"/>
-      <c r="I35" s="185"/>
+      <c r="C35" s="190"/>
+      <c r="D35" s="190"/>
+      <c r="E35" s="190"/>
+      <c r="F35" s="190"/>
+      <c r="G35" s="190"/>
+      <c r="H35" s="190"/>
+      <c r="I35" s="191"/>
       <c r="J35" s="39"/>
       <c r="K35" s="19"/>
       <c r="L35" s="19"/>
@@ -5090,19 +5044,19 @@
       <c r="B36" s="41" t="s">
         <v>39</v>
       </c>
-      <c r="C36" s="192" t="s">
+      <c r="C36" s="198" t="s">
         <v>40</v>
       </c>
-      <c r="D36" s="193"/>
-      <c r="E36" s="193"/>
-      <c r="F36" s="194"/>
+      <c r="D36" s="199"/>
+      <c r="E36" s="199"/>
+      <c r="F36" s="200"/>
       <c r="G36" s="41" t="s">
         <v>39</v>
       </c>
-      <c r="H36" s="190" t="s">
+      <c r="H36" s="196" t="s">
         <v>41</v>
       </c>
-      <c r="I36" s="191"/>
+      <c r="I36" s="197"/>
       <c r="J36" s="40"/>
       <c r="K36" s="19"/>
       <c r="L36" s="19"/>
@@ -5123,18 +5077,18 @@
       <c r="AA36" s="20"/>
     </row>
     <row r="37" spans="2:28" s="11" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B37" s="177" t="s">
+      <c r="B37" s="183" t="s">
         <v>42</v>
       </c>
-      <c r="C37" s="210"/>
-      <c r="D37" s="211"/>
-      <c r="E37" s="211"/>
-      <c r="F37" s="212"/>
-      <c r="G37" s="177" t="s">
+      <c r="C37" s="216"/>
+      <c r="D37" s="217"/>
+      <c r="E37" s="217"/>
+      <c r="F37" s="218"/>
+      <c r="G37" s="183" t="s">
         <v>43</v>
       </c>
-      <c r="H37" s="186"/>
-      <c r="I37" s="187"/>
+      <c r="H37" s="192"/>
+      <c r="I37" s="193"/>
       <c r="J37" s="39"/>
       <c r="K37" s="16"/>
       <c r="L37" s="18"/>
@@ -5153,14 +5107,14 @@
       <c r="AB37" s="12"/>
     </row>
     <row r="38" spans="2:28" s="11" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B38" s="226"/>
-      <c r="C38" s="213"/>
-      <c r="D38" s="112"/>
-      <c r="E38" s="112"/>
-      <c r="F38" s="214"/>
-      <c r="G38" s="207"/>
-      <c r="H38" s="188"/>
-      <c r="I38" s="189"/>
+      <c r="B38" s="232"/>
+      <c r="C38" s="219"/>
+      <c r="D38" s="117"/>
+      <c r="E38" s="117"/>
+      <c r="F38" s="220"/>
+      <c r="G38" s="213"/>
+      <c r="H38" s="194"/>
+      <c r="I38" s="195"/>
       <c r="J38" s="39"/>
       <c r="K38" s="16"/>
       <c r="L38" s="18"/>
@@ -5178,16 +5132,16 @@
       <c r="AB38" s="12"/>
     </row>
     <row r="39" spans="2:28" s="11" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B39" s="226"/>
-      <c r="C39" s="213"/>
-      <c r="D39" s="112"/>
-      <c r="E39" s="112"/>
-      <c r="F39" s="214"/>
-      <c r="G39" s="177" t="s">
+      <c r="B39" s="232"/>
+      <c r="C39" s="219"/>
+      <c r="D39" s="117"/>
+      <c r="E39" s="117"/>
+      <c r="F39" s="220"/>
+      <c r="G39" s="183" t="s">
         <v>44</v>
       </c>
-      <c r="H39" s="186"/>
-      <c r="I39" s="187"/>
+      <c r="H39" s="192"/>
+      <c r="I39" s="193"/>
       <c r="J39" s="39"/>
       <c r="K39" s="16"/>
       <c r="L39" s="18"/>
@@ -5206,14 +5160,14 @@
       <c r="AB39" s="12"/>
     </row>
     <row r="40" spans="2:28" s="11" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B40" s="227"/>
-      <c r="C40" s="215"/>
-      <c r="D40" s="216"/>
-      <c r="E40" s="216"/>
-      <c r="F40" s="217"/>
-      <c r="G40" s="207"/>
-      <c r="H40" s="188"/>
-      <c r="I40" s="189"/>
+      <c r="B40" s="233"/>
+      <c r="C40" s="221"/>
+      <c r="D40" s="222"/>
+      <c r="E40" s="222"/>
+      <c r="F40" s="223"/>
+      <c r="G40" s="213"/>
+      <c r="H40" s="194"/>
+      <c r="I40" s="195"/>
       <c r="J40" s="39"/>
       <c r="K40" s="16"/>
       <c r="L40" s="18"/>
@@ -5232,18 +5186,18 @@
       <c r="AB40" s="12"/>
     </row>
     <row r="41" spans="2:28" s="11" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B41" s="224" t="s">
+      <c r="B41" s="230" t="s">
         <v>45</v>
       </c>
-      <c r="C41" s="218"/>
-      <c r="D41" s="219"/>
-      <c r="E41" s="219"/>
-      <c r="F41" s="220"/>
-      <c r="G41" s="177" t="s">
+      <c r="C41" s="224"/>
+      <c r="D41" s="225"/>
+      <c r="E41" s="225"/>
+      <c r="F41" s="226"/>
+      <c r="G41" s="183" t="s">
         <v>46</v>
       </c>
-      <c r="H41" s="179"/>
-      <c r="I41" s="180"/>
+      <c r="H41" s="185"/>
+      <c r="I41" s="186"/>
       <c r="J41" s="56"/>
       <c r="K41" s="16"/>
       <c r="L41" s="17"/>
@@ -5265,14 +5219,14 @@
       <c r="AB41" s="12"/>
     </row>
     <row r="42" spans="2:28" s="38" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B42" s="225"/>
-      <c r="C42" s="221"/>
-      <c r="D42" s="222"/>
-      <c r="E42" s="222"/>
-      <c r="F42" s="223"/>
-      <c r="G42" s="178"/>
-      <c r="H42" s="181"/>
-      <c r="I42" s="182"/>
+      <c r="B42" s="231"/>
+      <c r="C42" s="227"/>
+      <c r="D42" s="228"/>
+      <c r="E42" s="228"/>
+      <c r="F42" s="229"/>
+      <c r="G42" s="184"/>
+      <c r="H42" s="187"/>
+      <c r="I42" s="188"/>
       <c r="J42" s="56"/>
       <c r="K42" s="16"/>
       <c r="L42" s="17"/>
@@ -5299,8 +5253,8 @@
       <c r="D43" s="43"/>
       <c r="E43" s="43"/>
       <c r="F43" s="43"/>
-      <c r="G43" s="208"/>
-      <c r="H43" s="209"/>
+      <c r="G43" s="214"/>
+      <c r="H43" s="215"/>
       <c r="I43" s="43"/>
       <c r="J43" s="56"/>
       <c r="K43" s="16"/>
@@ -5323,16 +5277,16 @@
       <c r="AB43" s="12"/>
     </row>
     <row r="44" spans="2:28" s="11" customFormat="1" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B44" s="205" t="s">
+      <c r="B44" s="211" t="s">
         <v>47</v>
       </c>
-      <c r="C44" s="205"/>
-      <c r="D44" s="205"/>
-      <c r="E44" s="205"/>
-      <c r="F44" s="205"/>
-      <c r="G44" s="205"/>
-      <c r="H44" s="205"/>
-      <c r="I44" s="206"/>
+      <c r="C44" s="211"/>
+      <c r="D44" s="211"/>
+      <c r="E44" s="211"/>
+      <c r="F44" s="211"/>
+      <c r="G44" s="211"/>
+      <c r="H44" s="211"/>
+      <c r="I44" s="212"/>
       <c r="J44" s="16"/>
       <c r="K44" s="16"/>
       <c r="L44" s="17"/>
@@ -5354,24 +5308,24 @@
       <c r="AB44" s="12"/>
     </row>
     <row r="45" spans="2:28" ht="68.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B45" s="124" t="s">
+      <c r="B45" s="130" t="s">
         <v>48</v>
       </c>
-      <c r="C45" s="109"/>
-      <c r="D45" s="106" t="s">
+      <c r="C45" s="114"/>
+      <c r="D45" s="111" t="s">
         <v>49</v>
       </c>
-      <c r="E45" s="107"/>
-      <c r="F45" s="110" t="s">
+      <c r="E45" s="112"/>
+      <c r="F45" s="115" t="s">
         <v>50</v>
       </c>
-      <c r="G45" s="110" t="s">
+      <c r="G45" s="115" t="s">
         <v>51</v>
       </c>
-      <c r="H45" s="122" t="s">
+      <c r="H45" s="128" t="s">
         <v>52</v>
       </c>
-      <c r="I45" s="176" t="s">
+      <c r="I45" s="182" t="s">
         <v>53</v>
       </c>
       <c r="J45" s="16"/>
@@ -5394,14 +5348,14 @@
       <c r="AA45" s="16"/>
     </row>
     <row r="46" spans="2:28" ht="66.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B46" s="124"/>
-      <c r="C46" s="109"/>
-      <c r="D46" s="108"/>
-      <c r="E46" s="109"/>
-      <c r="F46" s="111"/>
-      <c r="G46" s="110"/>
-      <c r="H46" s="123"/>
-      <c r="I46" s="176"/>
+      <c r="B46" s="130"/>
+      <c r="C46" s="114"/>
+      <c r="D46" s="113"/>
+      <c r="E46" s="114"/>
+      <c r="F46" s="116"/>
+      <c r="G46" s="115"/>
+      <c r="H46" s="129"/>
+      <c r="I46" s="182"/>
       <c r="J46" s="16"/>
       <c r="K46" s="16"/>
       <c r="L46" s="16"/>
@@ -5422,14 +5376,14 @@
       <c r="AA46" s="16"/>
     </row>
     <row r="47" spans="2:28" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B47" s="98"/>
-      <c r="C47" s="99"/>
-      <c r="D47" s="283"/>
-      <c r="E47" s="283"/>
-      <c r="F47" s="102"/>
-      <c r="G47" s="99"/>
-      <c r="H47" s="287"/>
-      <c r="I47" s="285"/>
+      <c r="B47" s="99"/>
+      <c r="C47" s="100"/>
+      <c r="D47" s="103"/>
+      <c r="E47" s="103"/>
+      <c r="F47" s="105"/>
+      <c r="G47" s="100"/>
+      <c r="H47" s="107"/>
+      <c r="I47" s="97"/>
       <c r="J47" s="18"/>
       <c r="K47" s="16"/>
       <c r="L47" s="16"/>
@@ -5450,14 +5404,14 @@
       <c r="AA47" s="16"/>
     </row>
     <row r="48" spans="2:28" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B48" s="98"/>
-      <c r="C48" s="99"/>
-      <c r="D48" s="283"/>
-      <c r="E48" s="283"/>
-      <c r="F48" s="102"/>
-      <c r="G48" s="99"/>
-      <c r="H48" s="287"/>
-      <c r="I48" s="285"/>
+      <c r="B48" s="99"/>
+      <c r="C48" s="100"/>
+      <c r="D48" s="103"/>
+      <c r="E48" s="103"/>
+      <c r="F48" s="105"/>
+      <c r="G48" s="100"/>
+      <c r="H48" s="107"/>
+      <c r="I48" s="97"/>
       <c r="J48" s="18"/>
       <c r="K48" s="16"/>
       <c r="L48" s="16"/>
@@ -5478,14 +5432,14 @@
       <c r="AA48" s="16"/>
     </row>
     <row r="49" spans="2:28" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B49" s="98"/>
-      <c r="C49" s="99"/>
-      <c r="D49" s="283"/>
-      <c r="E49" s="283"/>
-      <c r="F49" s="102"/>
-      <c r="G49" s="99"/>
-      <c r="H49" s="287"/>
-      <c r="I49" s="285"/>
+      <c r="B49" s="99"/>
+      <c r="C49" s="100"/>
+      <c r="D49" s="103"/>
+      <c r="E49" s="103"/>
+      <c r="F49" s="105"/>
+      <c r="G49" s="100"/>
+      <c r="H49" s="107"/>
+      <c r="I49" s="97"/>
       <c r="J49" s="18"/>
       <c r="K49" s="16"/>
       <c r="L49" s="16"/>
@@ -5506,14 +5460,14 @@
       <c r="AA49" s="16"/>
     </row>
     <row r="50" spans="2:28" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B50" s="98"/>
-      <c r="C50" s="99"/>
-      <c r="D50" s="283"/>
-      <c r="E50" s="283"/>
-      <c r="F50" s="102"/>
-      <c r="G50" s="99"/>
-      <c r="H50" s="287"/>
-      <c r="I50" s="285"/>
+      <c r="B50" s="99"/>
+      <c r="C50" s="100"/>
+      <c r="D50" s="103"/>
+      <c r="E50" s="103"/>
+      <c r="F50" s="105"/>
+      <c r="G50" s="100"/>
+      <c r="H50" s="107"/>
+      <c r="I50" s="97"/>
       <c r="J50" s="18"/>
       <c r="K50" s="16"/>
       <c r="L50" s="16"/>
@@ -5534,14 +5488,14 @@
       <c r="AA50" s="16"/>
     </row>
     <row r="51" spans="2:28" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B51" s="98"/>
-      <c r="C51" s="99"/>
-      <c r="D51" s="283"/>
-      <c r="E51" s="283"/>
-      <c r="F51" s="102"/>
-      <c r="G51" s="99"/>
-      <c r="H51" s="287"/>
-      <c r="I51" s="285"/>
+      <c r="B51" s="99"/>
+      <c r="C51" s="100"/>
+      <c r="D51" s="103"/>
+      <c r="E51" s="103"/>
+      <c r="F51" s="105"/>
+      <c r="G51" s="100"/>
+      <c r="H51" s="107"/>
+      <c r="I51" s="97"/>
       <c r="J51" s="18"/>
       <c r="K51" s="16"/>
       <c r="L51" s="16"/>
@@ -5562,14 +5516,14 @@
       <c r="AA51" s="16"/>
     </row>
     <row r="52" spans="2:28" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B52" s="98"/>
-      <c r="C52" s="99"/>
-      <c r="D52" s="283"/>
-      <c r="E52" s="283"/>
-      <c r="F52" s="102"/>
-      <c r="G52" s="99"/>
-      <c r="H52" s="287"/>
-      <c r="I52" s="285"/>
+      <c r="B52" s="99"/>
+      <c r="C52" s="100"/>
+      <c r="D52" s="103"/>
+      <c r="E52" s="103"/>
+      <c r="F52" s="105"/>
+      <c r="G52" s="100"/>
+      <c r="H52" s="107"/>
+      <c r="I52" s="97"/>
       <c r="J52" s="18"/>
       <c r="K52" s="16"/>
       <c r="L52" s="16"/>
@@ -5590,14 +5544,14 @@
       <c r="AA52" s="16"/>
     </row>
     <row r="53" spans="2:28" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B53" s="98"/>
-      <c r="C53" s="99"/>
-      <c r="D53" s="283"/>
-      <c r="E53" s="283"/>
-      <c r="F53" s="102"/>
-      <c r="G53" s="99"/>
-      <c r="H53" s="287"/>
-      <c r="I53" s="285"/>
+      <c r="B53" s="99"/>
+      <c r="C53" s="100"/>
+      <c r="D53" s="103"/>
+      <c r="E53" s="103"/>
+      <c r="F53" s="105"/>
+      <c r="G53" s="100"/>
+      <c r="H53" s="107"/>
+      <c r="I53" s="97"/>
       <c r="J53" s="18"/>
       <c r="K53" s="16"/>
       <c r="L53" s="16"/>
@@ -5618,14 +5572,14 @@
       <c r="AA53" s="16"/>
     </row>
     <row r="54" spans="2:28" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B54" s="98"/>
-      <c r="C54" s="99"/>
-      <c r="D54" s="283"/>
-      <c r="E54" s="283"/>
-      <c r="F54" s="102"/>
-      <c r="G54" s="99"/>
-      <c r="H54" s="287"/>
-      <c r="I54" s="285"/>
+      <c r="B54" s="99"/>
+      <c r="C54" s="100"/>
+      <c r="D54" s="103"/>
+      <c r="E54" s="103"/>
+      <c r="F54" s="105"/>
+      <c r="G54" s="100"/>
+      <c r="H54" s="107"/>
+      <c r="I54" s="97"/>
       <c r="J54" s="18"/>
       <c r="K54" s="16"/>
       <c r="L54" s="16"/>
@@ -5646,14 +5600,14 @@
       <c r="AA54" s="16"/>
     </row>
     <row r="55" spans="2:28" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B55" s="98"/>
-      <c r="C55" s="99"/>
-      <c r="D55" s="283"/>
-      <c r="E55" s="283"/>
-      <c r="F55" s="102"/>
-      <c r="G55" s="99"/>
-      <c r="H55" s="287"/>
-      <c r="I55" s="285"/>
+      <c r="B55" s="99"/>
+      <c r="C55" s="100"/>
+      <c r="D55" s="103"/>
+      <c r="E55" s="103"/>
+      <c r="F55" s="105"/>
+      <c r="G55" s="100"/>
+      <c r="H55" s="107"/>
+      <c r="I55" s="97"/>
       <c r="J55" s="18"/>
       <c r="K55" s="16"/>
       <c r="L55" s="16"/>
@@ -5674,14 +5628,14 @@
       <c r="AA55" s="16"/>
     </row>
     <row r="56" spans="2:28" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B56" s="100"/>
-      <c r="C56" s="101"/>
-      <c r="D56" s="284"/>
-      <c r="E56" s="284"/>
-      <c r="F56" s="103"/>
-      <c r="G56" s="101"/>
-      <c r="H56" s="288"/>
-      <c r="I56" s="286"/>
+      <c r="B56" s="101"/>
+      <c r="C56" s="102"/>
+      <c r="D56" s="104"/>
+      <c r="E56" s="104"/>
+      <c r="F56" s="106"/>
+      <c r="G56" s="102"/>
+      <c r="H56" s="108"/>
+      <c r="I56" s="98"/>
       <c r="J56" s="18"/>
       <c r="K56" s="16"/>
       <c r="L56" s="16"/>
@@ -5707,8 +5661,8 @@
       <c r="D57" s="18"/>
       <c r="E57" s="23"/>
       <c r="F57" s="23"/>
-      <c r="G57" s="113"/>
-      <c r="H57" s="113"/>
+      <c r="G57" s="118"/>
+      <c r="H57" s="118"/>
       <c r="I57" s="18"/>
       <c r="J57" s="18"/>
       <c r="K57" s="16"/>
@@ -5760,16 +5714,16 @@
       <c r="AA58" s="16"/>
     </row>
     <row r="59" spans="2:28" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B59" s="235" t="s">
+      <c r="B59" s="241" t="s">
         <v>55</v>
       </c>
-      <c r="C59" s="236"/>
-      <c r="D59" s="236"/>
-      <c r="E59" s="236"/>
-      <c r="F59" s="236"/>
-      <c r="G59" s="236"/>
-      <c r="H59" s="236"/>
-      <c r="I59" s="237"/>
+      <c r="C59" s="242"/>
+      <c r="D59" s="242"/>
+      <c r="E59" s="242"/>
+      <c r="F59" s="242"/>
+      <c r="G59" s="242"/>
+      <c r="H59" s="242"/>
+      <c r="I59" s="243"/>
       <c r="J59" s="19"/>
       <c r="K59" s="19"/>
       <c r="L59" s="19"/>
@@ -5950,11 +5904,11 @@
         <v>62</v>
       </c>
       <c r="F65" s="86"/>
-      <c r="G65" s="245"/>
+      <c r="G65" s="251"/>
       <c r="H65" s="86" t="s">
         <v>63</v>
       </c>
-      <c r="I65" s="247"/>
+      <c r="I65" s="253"/>
       <c r="J65" s="16"/>
       <c r="K65" s="16"/>
       <c r="L65" s="16"/>
@@ -5981,9 +5935,9 @@
       <c r="D66" s="93"/>
       <c r="E66" s="87"/>
       <c r="F66" s="87"/>
-      <c r="G66" s="246"/>
+      <c r="G66" s="252"/>
       <c r="H66" s="87"/>
-      <c r="I66" s="248"/>
+      <c r="I66" s="254"/>
       <c r="J66" s="16"/>
       <c r="K66" s="16"/>
       <c r="L66" s="16"/>
@@ -6123,10 +6077,10 @@
       <c r="AB70" s="16"/>
     </row>
     <row r="71" spans="2:28" ht="36" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B71" s="241"/>
-      <c r="C71" s="241"/>
-      <c r="D71" s="241"/>
-      <c r="E71" s="241"/>
+      <c r="B71" s="247"/>
+      <c r="C71" s="247"/>
+      <c r="D71" s="247"/>
+      <c r="E71" s="247"/>
       <c r="F71" s="26"/>
       <c r="H71" s="57"/>
       <c r="I71" s="16"/>
@@ -6189,7 +6143,7 @@
       <c r="E73" s="26"/>
       <c r="F73" s="26"/>
       <c r="G73" s="95"/>
-      <c r="H73" s="204"/>
+      <c r="H73" s="210"/>
       <c r="I73" s="16"/>
       <c r="J73" s="16"/>
       <c r="K73" s="16"/>
@@ -6212,13 +6166,13 @@
       <c r="AB73" s="16"/>
     </row>
     <row r="74" spans="2:28" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B74" s="243"/>
-      <c r="C74" s="243"/>
-      <c r="D74" s="243"/>
-      <c r="E74" s="243"/>
+      <c r="B74" s="249"/>
+      <c r="C74" s="249"/>
+      <c r="D74" s="249"/>
+      <c r="E74" s="249"/>
       <c r="F74" s="26"/>
-      <c r="H74" s="112"/>
-      <c r="I74" s="112"/>
+      <c r="H74" s="117"/>
+      <c r="I74" s="117"/>
       <c r="J74" s="16"/>
       <c r="K74" s="16"/>
       <c r="L74" s="16"/>
@@ -6240,13 +6194,13 @@
       <c r="AB74" s="16"/>
     </row>
     <row r="75" spans="2:28" ht="38.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B75" s="244"/>
-      <c r="C75" s="244"/>
-      <c r="D75" s="244"/>
-      <c r="E75" s="244"/>
+      <c r="B75" s="250"/>
+      <c r="C75" s="250"/>
+      <c r="D75" s="250"/>
+      <c r="E75" s="250"/>
       <c r="F75" s="26"/>
-      <c r="H75" s="242"/>
-      <c r="I75" s="242"/>
+      <c r="H75" s="248"/>
+      <c r="I75" s="248"/>
       <c r="J75" s="16"/>
       <c r="K75" s="16"/>
       <c r="L75" s="16"/>
@@ -6419,7 +6373,7 @@
     </row>
     <row r="81" spans="2:28" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B81" s="69" t="s">
-        <v>70</v>
+        <v>160</v>
       </c>
       <c r="C81" s="70"/>
       <c r="D81" s="70"/>
@@ -6450,7 +6404,7 @@
     </row>
     <row r="82" spans="2:28" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B82" s="72" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C82" s="73"/>
       <c r="D82" s="73"/>
@@ -6480,14 +6434,14 @@
       <c r="AB82" s="7"/>
     </row>
     <row r="83" spans="2:28" s="8" customFormat="1" ht="249" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B83" s="238"/>
-      <c r="C83" s="239"/>
-      <c r="D83" s="239"/>
-      <c r="E83" s="239"/>
-      <c r="F83" s="239"/>
-      <c r="G83" s="239"/>
-      <c r="H83" s="239"/>
-      <c r="I83" s="240"/>
+      <c r="B83" s="244"/>
+      <c r="C83" s="245"/>
+      <c r="D83" s="245"/>
+      <c r="E83" s="245"/>
+      <c r="F83" s="245"/>
+      <c r="G83" s="245"/>
+      <c r="H83" s="245"/>
+      <c r="I83" s="246"/>
     </row>
     <row r="84" spans="2:28" hidden="1" x14ac:dyDescent="0.25">
       <c r="G84" s="95"/>
@@ -6803,17 +6757,17 @@
     <mergeCell ref="G80:H80"/>
   </mergeCells>
   <conditionalFormatting sqref="B11:I11 B15:I15 B17:I17 B19:I19 B21:I21 B25:I25 B29:I29 C37:F42 H37:I42 B70:E71 H74:I75 B83:I83">
-    <cfRule type="containsBlanks" dxfId="5" priority="7">
+    <cfRule type="containsBlanks" dxfId="2" priority="7">
       <formula>LEN(TRIM(B11))=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B47:I56">
-    <cfRule type="containsBlanks" dxfId="4" priority="6">
+    <cfRule type="containsBlanks" dxfId="1" priority="6">
       <formula>LEN(TRIM(B47))=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G65:G66 I65:I66 B66:D66 H71">
-    <cfRule type="containsBlanks" dxfId="3" priority="8">
+    <cfRule type="containsBlanks" dxfId="0" priority="8">
       <formula>LEN(TRIM(B65))=0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6892,24 +6846,24 @@
   <sheetData>
     <row r="1" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="58" t="s">
+        <v>105</v>
+      </c>
+      <c r="B1" s="59" t="s">
         <v>106</v>
       </c>
-      <c r="B1" s="59" t="s">
+      <c r="C1" s="60" t="s">
         <v>107</v>
-      </c>
-      <c r="C1" s="60" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="39" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="61" t="s">
+        <v>108</v>
+      </c>
+      <c r="B2" s="62" t="s">
         <v>109</v>
       </c>
-      <c r="B2" s="62" t="s">
-        <v>110</v>
-      </c>
       <c r="C2" s="65" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E2" t="str" cm="1">
         <f t="array" ref="E2:E3">_xlfn.UNIQUE(TablaSena[PROGRAMA])</f>
@@ -6942,13 +6896,13 @@
     </row>
     <row r="3" spans="1:11" ht="39" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="61" t="s">
+        <v>108</v>
+      </c>
+      <c r="B3" s="62" t="s">
         <v>109</v>
       </c>
-      <c r="B3" s="62" t="s">
-        <v>110</v>
-      </c>
       <c r="C3" s="65" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E3" t="str">
         <v>Programación de Software</v>
@@ -6956,398 +6910,398 @@
     </row>
     <row r="4" spans="1:11" ht="39" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="61" t="s">
+        <v>108</v>
+      </c>
+      <c r="B4" s="62" t="s">
         <v>109</v>
       </c>
-      <c r="B4" s="62" t="s">
-        <v>110</v>
-      </c>
       <c r="C4" s="65" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="39" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="61" t="s">
+        <v>108</v>
+      </c>
+      <c r="B5" s="62" t="s">
         <v>109</v>
       </c>
-      <c r="B5" s="62" t="s">
-        <v>110</v>
-      </c>
       <c r="C5" s="65" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="39" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="61" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B6" s="62" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C6" s="65" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="39" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="61" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B7" s="62" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C7" s="65" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="8" spans="1:11" ht="39" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="61" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B8" s="62" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C8" s="65" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="9" spans="1:11" ht="39" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="61" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B9" s="62" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C9" s="65" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="10" spans="1:11" ht="39" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="61" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B10" s="62" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C10" s="65" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="11" spans="1:11" ht="39" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="61" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B11" s="62" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C11" s="65" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="12" spans="1:11" ht="39" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="61" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B12" s="62" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C12" s="65" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="13" spans="1:11" ht="39" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="61" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B13" s="62" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C13" s="65" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="14" spans="1:11" ht="39" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="61" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B14" s="62" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C14" s="65" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="15" spans="1:11" ht="39" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="61" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B15" s="62" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C15" s="65" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="16" spans="1:11" ht="39" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="61" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B16" s="62" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C16" s="65" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="39" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="61" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B17" s="62" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C17" s="65" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="39" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="61" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B18" s="62" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C18" s="65" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="39" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="61" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B19" s="62" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C19" s="65" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="39" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="61" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B20" s="62" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C20" s="65" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="39" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="61" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B21" s="62" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C21" s="65" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="22" spans="1:3" ht="39" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="61" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B22" s="62" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C22" s="65" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="39" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="61" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B23" s="62" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C23" s="65" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="39" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="61" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B24" s="62" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C24" s="65" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="25" spans="1:3" ht="39" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="61" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B25" s="62" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C25" s="65" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="39" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="61" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B26" s="62" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C26" s="65" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="39" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="61" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B27" s="62" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C27" s="65" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="28" spans="1:3" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="61" t="s">
+        <v>116</v>
+      </c>
+      <c r="B28" s="62" t="s">
         <v>117</v>
       </c>
-      <c r="B28" s="62" t="s">
-        <v>118</v>
-      </c>
       <c r="C28" s="65" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="29" spans="1:3" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="61" t="s">
+        <v>116</v>
+      </c>
+      <c r="B29" s="62" t="s">
         <v>117</v>
       </c>
-      <c r="B29" s="62" t="s">
-        <v>118</v>
-      </c>
       <c r="C29" s="65" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="30" spans="1:3" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="61" t="s">
+        <v>116</v>
+      </c>
+      <c r="B30" s="62" t="s">
         <v>117</v>
       </c>
-      <c r="B30" s="62" t="s">
-        <v>118</v>
-      </c>
       <c r="C30" s="65" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="31" spans="1:3" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="61" t="s">
+        <v>116</v>
+      </c>
+      <c r="B31" s="62" t="s">
         <v>117</v>
       </c>
-      <c r="B31" s="62" t="s">
-        <v>118</v>
-      </c>
       <c r="C31" s="65" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="32" spans="1:3" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="61" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B32" s="62" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C32" s="65" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="33" spans="1:3" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="61" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B33" s="62" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C33" s="65" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="61" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B34" s="62" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C34" s="65" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="35" spans="1:3" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="61" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B35" s="62" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C35" s="65" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="36" spans="1:3" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="61" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B36" s="62" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C36" s="65" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="37" spans="1:3" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="61" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B37" s="62" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C37" s="65" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="38" spans="1:3" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="61" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B38" s="62" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C38" s="65" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="39" spans="1:3" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A39" s="63" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B39" s="64" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C39" s="66" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
   </sheetData>
@@ -7439,124 +7393,124 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:24" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A1" s="275" t="s">
+      <c r="A1" s="281" t="s">
+        <v>71</v>
+      </c>
+      <c r="B1" s="281"/>
+      <c r="C1" s="281"/>
+      <c r="D1" s="281"/>
+      <c r="E1" s="281"/>
+      <c r="F1" s="281"/>
+      <c r="G1" s="281"/>
+      <c r="H1" s="281"/>
+      <c r="I1" s="281"/>
+      <c r="J1" s="281"/>
+      <c r="K1" s="281"/>
+      <c r="L1" s="281"/>
+      <c r="M1" s="281"/>
+      <c r="N1" s="281"/>
+      <c r="O1" s="281"/>
+      <c r="P1" s="281"/>
+      <c r="Q1" s="281"/>
+      <c r="R1" s="281"/>
+      <c r="S1" s="281"/>
+      <c r="T1" s="281"/>
+      <c r="U1" s="281" t="s">
         <v>72</v>
       </c>
-      <c r="B1" s="275"/>
-      <c r="C1" s="275"/>
-      <c r="D1" s="275"/>
-      <c r="E1" s="275"/>
-      <c r="F1" s="275"/>
-      <c r="G1" s="275"/>
-      <c r="H1" s="275"/>
-      <c r="I1" s="275"/>
-      <c r="J1" s="275"/>
-      <c r="K1" s="275"/>
-      <c r="L1" s="275"/>
-      <c r="M1" s="275"/>
-      <c r="N1" s="275"/>
-      <c r="O1" s="275"/>
-      <c r="P1" s="275"/>
-      <c r="Q1" s="275"/>
-      <c r="R1" s="275"/>
-      <c r="S1" s="275"/>
-      <c r="T1" s="275"/>
-      <c r="U1" s="275" t="s">
+      <c r="V1" s="281"/>
+      <c r="W1" s="281"/>
+      <c r="X1" s="281"/>
+    </row>
+    <row r="2" spans="1:24" ht="33" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="281"/>
+      <c r="B2" s="281"/>
+      <c r="C2" s="281"/>
+      <c r="D2" s="281"/>
+      <c r="E2" s="281"/>
+      <c r="F2" s="281"/>
+      <c r="G2" s="281"/>
+      <c r="H2" s="281"/>
+      <c r="I2" s="281"/>
+      <c r="J2" s="281"/>
+      <c r="K2" s="281"/>
+      <c r="L2" s="281"/>
+      <c r="M2" s="281"/>
+      <c r="N2" s="281"/>
+      <c r="O2" s="281"/>
+      <c r="P2" s="281"/>
+      <c r="Q2" s="281"/>
+      <c r="R2" s="281"/>
+      <c r="S2" s="281"/>
+      <c r="T2" s="281"/>
+      <c r="U2" s="261" t="s">
         <v>73</v>
       </c>
-      <c r="V1" s="275"/>
-      <c r="W1" s="275"/>
-      <c r="X1" s="275"/>
-    </row>
-    <row r="2" spans="1:24" ht="33" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="275"/>
-      <c r="B2" s="275"/>
-      <c r="C2" s="275"/>
-      <c r="D2" s="275"/>
-      <c r="E2" s="275"/>
-      <c r="F2" s="275"/>
-      <c r="G2" s="275"/>
-      <c r="H2" s="275"/>
-      <c r="I2" s="275"/>
-      <c r="J2" s="275"/>
-      <c r="K2" s="275"/>
-      <c r="L2" s="275"/>
-      <c r="M2" s="275"/>
-      <c r="N2" s="275"/>
-      <c r="O2" s="275"/>
-      <c r="P2" s="275"/>
-      <c r="Q2" s="275"/>
-      <c r="R2" s="275"/>
-      <c r="S2" s="275"/>
-      <c r="T2" s="275"/>
-      <c r="U2" s="255" t="s">
+      <c r="V2" s="261"/>
+      <c r="W2" s="261"/>
+      <c r="X2" s="261"/>
+    </row>
+    <row r="3" spans="1:24" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="U3" s="288"/>
+      <c r="V3" s="288"/>
+      <c r="W3" s="288"/>
+      <c r="X3" s="288"/>
+    </row>
+    <row r="4" spans="1:24" s="2" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="285" t="s">
         <v>74</v>
       </c>
-      <c r="V2" s="255"/>
-      <c r="W2" s="255"/>
-      <c r="X2" s="255"/>
-    </row>
-    <row r="3" spans="1:24" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="U3" s="282"/>
-      <c r="V3" s="282"/>
-      <c r="W3" s="282"/>
-      <c r="X3" s="282"/>
-    </row>
-    <row r="4" spans="1:24" s="2" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="279" t="s">
+      <c r="B4" s="286"/>
+      <c r="C4" s="286"/>
+      <c r="D4" s="286"/>
+      <c r="E4" s="286"/>
+      <c r="F4" s="286"/>
+      <c r="G4" s="286"/>
+      <c r="H4" s="286"/>
+      <c r="I4" s="286"/>
+      <c r="J4" s="286"/>
+      <c r="K4" s="286"/>
+      <c r="L4" s="286"/>
+      <c r="M4" s="287"/>
+      <c r="N4" s="285" t="s">
         <v>75</v>
       </c>
-      <c r="B4" s="280"/>
-      <c r="C4" s="280"/>
-      <c r="D4" s="280"/>
-      <c r="E4" s="280"/>
-      <c r="F4" s="280"/>
-      <c r="G4" s="280"/>
-      <c r="H4" s="280"/>
-      <c r="I4" s="280"/>
-      <c r="J4" s="280"/>
-      <c r="K4" s="280"/>
-      <c r="L4" s="280"/>
-      <c r="M4" s="281"/>
-      <c r="N4" s="279" t="s">
-        <v>76</v>
-      </c>
-      <c r="O4" s="280"/>
-      <c r="P4" s="280"/>
-      <c r="Q4" s="280"/>
-      <c r="R4" s="280"/>
-      <c r="S4" s="280"/>
-      <c r="T4" s="280"/>
-      <c r="U4" s="280"/>
-      <c r="V4" s="280"/>
-      <c r="W4" s="280"/>
-      <c r="X4" s="281"/>
+      <c r="O4" s="286"/>
+      <c r="P4" s="286"/>
+      <c r="Q4" s="286"/>
+      <c r="R4" s="286"/>
+      <c r="S4" s="286"/>
+      <c r="T4" s="286"/>
+      <c r="U4" s="286"/>
+      <c r="V4" s="286"/>
+      <c r="W4" s="286"/>
+      <c r="X4" s="287"/>
     </row>
     <row r="5" spans="1:24" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="276"/>
-      <c r="B5" s="277"/>
-      <c r="C5" s="277"/>
-      <c r="D5" s="277"/>
-      <c r="E5" s="277"/>
-      <c r="F5" s="277"/>
-      <c r="G5" s="277"/>
-      <c r="H5" s="277"/>
-      <c r="I5" s="277"/>
-      <c r="J5" s="277"/>
-      <c r="K5" s="277"/>
-      <c r="L5" s="277"/>
-      <c r="M5" s="278"/>
-      <c r="N5" s="276"/>
-      <c r="O5" s="277"/>
-      <c r="P5" s="277"/>
-      <c r="Q5" s="277"/>
-      <c r="R5" s="277"/>
-      <c r="S5" s="277"/>
-      <c r="T5" s="277"/>
-      <c r="U5" s="277"/>
-      <c r="V5" s="277"/>
-      <c r="W5" s="277"/>
-      <c r="X5" s="278"/>
+      <c r="A5" s="282"/>
+      <c r="B5" s="283"/>
+      <c r="C5" s="283"/>
+      <c r="D5" s="283"/>
+      <c r="E5" s="283"/>
+      <c r="F5" s="283"/>
+      <c r="G5" s="283"/>
+      <c r="H5" s="283"/>
+      <c r="I5" s="283"/>
+      <c r="J5" s="283"/>
+      <c r="K5" s="283"/>
+      <c r="L5" s="283"/>
+      <c r="M5" s="284"/>
+      <c r="N5" s="282"/>
+      <c r="O5" s="283"/>
+      <c r="P5" s="283"/>
+      <c r="Q5" s="283"/>
+      <c r="R5" s="283"/>
+      <c r="S5" s="283"/>
+      <c r="T5" s="283"/>
+      <c r="U5" s="283"/>
+      <c r="V5" s="283"/>
+      <c r="W5" s="283"/>
+      <c r="X5" s="284"/>
     </row>
     <row r="6" spans="1:24" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3"/>
@@ -7585,66 +7539,66 @@
       <c r="X6" s="3"/>
     </row>
     <row r="7" spans="1:24" s="2" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="253" t="s">
+      <c r="A7" s="259" t="s">
+        <v>76</v>
+      </c>
+      <c r="B7" s="259"/>
+      <c r="C7" s="259"/>
+      <c r="D7" s="259"/>
+      <c r="E7" s="259"/>
+      <c r="F7" s="259"/>
+      <c r="G7" s="259"/>
+      <c r="H7" s="259"/>
+      <c r="I7" s="259"/>
+      <c r="J7" s="259" t="s">
         <v>77</v>
       </c>
-      <c r="B7" s="253"/>
-      <c r="C7" s="253"/>
-      <c r="D7" s="253"/>
-      <c r="E7" s="253"/>
-      <c r="F7" s="253"/>
-      <c r="G7" s="253"/>
-      <c r="H7" s="253"/>
-      <c r="I7" s="253"/>
-      <c r="J7" s="253" t="s">
+      <c r="K7" s="259"/>
+      <c r="L7" s="259"/>
+      <c r="M7" s="259"/>
+      <c r="N7" s="259"/>
+      <c r="O7" s="259"/>
+      <c r="P7" s="259" t="s">
         <v>78</v>
       </c>
-      <c r="K7" s="253"/>
-      <c r="L7" s="253"/>
-      <c r="M7" s="253"/>
-      <c r="N7" s="253"/>
-      <c r="O7" s="253"/>
-      <c r="P7" s="253" t="s">
+      <c r="Q7" s="259"/>
+      <c r="R7" s="259"/>
+      <c r="S7" s="259"/>
+      <c r="T7" s="259"/>
+      <c r="U7" s="259"/>
+      <c r="V7" s="259"/>
+      <c r="W7" s="259"/>
+      <c r="X7" s="259"/>
+    </row>
+    <row r="8" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="266"/>
+      <c r="B8" s="266"/>
+      <c r="C8" s="266"/>
+      <c r="D8" s="266"/>
+      <c r="E8" s="266"/>
+      <c r="F8" s="266"/>
+      <c r="G8" s="266"/>
+      <c r="H8" s="266"/>
+      <c r="I8" s="266"/>
+      <c r="J8" s="267" t="s">
         <v>79</v>
       </c>
-      <c r="Q7" s="253"/>
-      <c r="R7" s="253"/>
-      <c r="S7" s="253"/>
-      <c r="T7" s="253"/>
-      <c r="U7" s="253"/>
-      <c r="V7" s="253"/>
-      <c r="W7" s="253"/>
-      <c r="X7" s="253"/>
-    </row>
-    <row r="8" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="260"/>
-      <c r="B8" s="260"/>
-      <c r="C8" s="260"/>
-      <c r="D8" s="260"/>
-      <c r="E8" s="260"/>
-      <c r="F8" s="260"/>
-      <c r="G8" s="260"/>
-      <c r="H8" s="260"/>
-      <c r="I8" s="260"/>
-      <c r="J8" s="261" t="s">
+      <c r="K8" s="268"/>
+      <c r="L8" s="268"/>
+      <c r="M8" s="268"/>
+      <c r="N8" s="268"/>
+      <c r="O8" s="269"/>
+      <c r="P8" s="267" t="s">
         <v>80</v>
       </c>
-      <c r="K8" s="262"/>
-      <c r="L8" s="262"/>
-      <c r="M8" s="262"/>
-      <c r="N8" s="262"/>
-      <c r="O8" s="263"/>
-      <c r="P8" s="261" t="s">
-        <v>81</v>
-      </c>
-      <c r="Q8" s="262"/>
-      <c r="R8" s="262"/>
-      <c r="S8" s="262"/>
-      <c r="T8" s="262"/>
-      <c r="U8" s="262"/>
-      <c r="V8" s="262"/>
-      <c r="W8" s="262"/>
-      <c r="X8" s="263"/>
+      <c r="Q8" s="268"/>
+      <c r="R8" s="268"/>
+      <c r="S8" s="268"/>
+      <c r="T8" s="268"/>
+      <c r="U8" s="268"/>
+      <c r="V8" s="268"/>
+      <c r="W8" s="268"/>
+      <c r="X8" s="269"/>
     </row>
     <row r="9" spans="1:24" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3"/>
@@ -7673,66 +7627,66 @@
       <c r="X9" s="3"/>
     </row>
     <row r="10" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="273" t="s">
+      <c r="A10" s="279" t="s">
+        <v>81</v>
+      </c>
+      <c r="B10" s="279"/>
+      <c r="C10" s="279"/>
+      <c r="D10" s="279"/>
+      <c r="E10" s="279"/>
+      <c r="F10" s="279"/>
+      <c r="G10" s="279"/>
+      <c r="H10" s="279"/>
+      <c r="I10" s="279"/>
+      <c r="J10" s="279"/>
+      <c r="K10" s="279"/>
+      <c r="L10" s="279"/>
+      <c r="M10" s="279"/>
+      <c r="N10" s="279"/>
+      <c r="O10" s="279"/>
+      <c r="P10" s="279"/>
+      <c r="Q10" s="279"/>
+      <c r="R10" s="279"/>
+      <c r="S10" s="279"/>
+      <c r="T10" s="279"/>
+      <c r="U10" s="279"/>
+      <c r="V10" s="279"/>
+      <c r="W10" s="279"/>
+      <c r="X10" s="279"/>
+    </row>
+    <row r="11" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="280" t="s">
         <v>82</v>
       </c>
-      <c r="B10" s="273"/>
-      <c r="C10" s="273"/>
-      <c r="D10" s="273"/>
-      <c r="E10" s="273"/>
-      <c r="F10" s="273"/>
-      <c r="G10" s="273"/>
-      <c r="H10" s="273"/>
-      <c r="I10" s="273"/>
-      <c r="J10" s="273"/>
-      <c r="K10" s="273"/>
-      <c r="L10" s="273"/>
-      <c r="M10" s="273"/>
-      <c r="N10" s="273"/>
-      <c r="O10" s="273"/>
-      <c r="P10" s="273"/>
-      <c r="Q10" s="273"/>
-      <c r="R10" s="273"/>
-      <c r="S10" s="273"/>
-      <c r="T10" s="273"/>
-      <c r="U10" s="273"/>
-      <c r="V10" s="273"/>
-      <c r="W10" s="273"/>
-      <c r="X10" s="273"/>
-    </row>
-    <row r="11" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="274" t="s">
+      <c r="B11" s="280"/>
+      <c r="C11" s="280"/>
+      <c r="D11" s="280"/>
+      <c r="E11" s="280"/>
+      <c r="F11" s="280"/>
+      <c r="G11" s="280" t="s">
         <v>83</v>
       </c>
-      <c r="B11" s="274"/>
-      <c r="C11" s="274"/>
-      <c r="D11" s="274"/>
-      <c r="E11" s="274"/>
-      <c r="F11" s="274"/>
-      <c r="G11" s="274" t="s">
+      <c r="H11" s="280"/>
+      <c r="I11" s="280"/>
+      <c r="J11" s="280"/>
+      <c r="K11" s="280"/>
+      <c r="L11" s="280"/>
+      <c r="M11" s="280" t="s">
         <v>84</v>
       </c>
-      <c r="H11" s="274"/>
-      <c r="I11" s="274"/>
-      <c r="J11" s="274"/>
-      <c r="K11" s="274"/>
-      <c r="L11" s="274"/>
-      <c r="M11" s="274" t="s">
+      <c r="N11" s="280"/>
+      <c r="O11" s="280"/>
+      <c r="P11" s="280"/>
+      <c r="Q11" s="280"/>
+      <c r="R11" s="280"/>
+      <c r="S11" s="280" t="s">
         <v>85</v>
       </c>
-      <c r="N11" s="274"/>
-      <c r="O11" s="274"/>
-      <c r="P11" s="274"/>
-      <c r="Q11" s="274"/>
-      <c r="R11" s="274"/>
-      <c r="S11" s="274" t="s">
-        <v>86</v>
-      </c>
-      <c r="T11" s="274"/>
-      <c r="U11" s="274"/>
-      <c r="V11" s="274"/>
-      <c r="W11" s="274"/>
-      <c r="X11" s="274"/>
+      <c r="T11" s="280"/>
+      <c r="U11" s="280"/>
+      <c r="V11" s="280"/>
+      <c r="W11" s="280"/>
+      <c r="X11" s="280"/>
     </row>
     <row r="12" spans="1:24" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3"/>
@@ -7761,66 +7715,66 @@
       <c r="X12" s="3"/>
     </row>
     <row r="13" spans="1:24" s="2" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="253" t="s">
+      <c r="A13" s="259" t="s">
+        <v>86</v>
+      </c>
+      <c r="B13" s="259"/>
+      <c r="C13" s="259"/>
+      <c r="D13" s="259"/>
+      <c r="E13" s="259"/>
+      <c r="F13" s="259"/>
+      <c r="G13" s="259"/>
+      <c r="H13" s="259"/>
+      <c r="I13" s="259"/>
+      <c r="J13" s="259" t="s">
+        <v>77</v>
+      </c>
+      <c r="K13" s="259"/>
+      <c r="L13" s="259"/>
+      <c r="M13" s="259"/>
+      <c r="N13" s="259"/>
+      <c r="O13" s="259"/>
+      <c r="P13" s="259" t="s">
+        <v>78</v>
+      </c>
+      <c r="Q13" s="259"/>
+      <c r="R13" s="259"/>
+      <c r="S13" s="259"/>
+      <c r="T13" s="259"/>
+      <c r="U13" s="259"/>
+      <c r="V13" s="259"/>
+      <c r="W13" s="259"/>
+      <c r="X13" s="259"/>
+    </row>
+    <row r="14" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="266"/>
+      <c r="B14" s="266"/>
+      <c r="C14" s="266"/>
+      <c r="D14" s="266"/>
+      <c r="E14" s="266"/>
+      <c r="F14" s="266"/>
+      <c r="G14" s="266"/>
+      <c r="H14" s="266"/>
+      <c r="I14" s="266"/>
+      <c r="J14" s="267" t="s">
         <v>87</v>
       </c>
-      <c r="B13" s="253"/>
-      <c r="C13" s="253"/>
-      <c r="D13" s="253"/>
-      <c r="E13" s="253"/>
-      <c r="F13" s="253"/>
-      <c r="G13" s="253"/>
-      <c r="H13" s="253"/>
-      <c r="I13" s="253"/>
-      <c r="J13" s="253" t="s">
-        <v>78</v>
-      </c>
-      <c r="K13" s="253"/>
-      <c r="L13" s="253"/>
-      <c r="M13" s="253"/>
-      <c r="N13" s="253"/>
-      <c r="O13" s="253"/>
-      <c r="P13" s="253" t="s">
-        <v>79</v>
-      </c>
-      <c r="Q13" s="253"/>
-      <c r="R13" s="253"/>
-      <c r="S13" s="253"/>
-      <c r="T13" s="253"/>
-      <c r="U13" s="253"/>
-      <c r="V13" s="253"/>
-      <c r="W13" s="253"/>
-      <c r="X13" s="253"/>
-    </row>
-    <row r="14" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="260"/>
-      <c r="B14" s="260"/>
-      <c r="C14" s="260"/>
-      <c r="D14" s="260"/>
-      <c r="E14" s="260"/>
-      <c r="F14" s="260"/>
-      <c r="G14" s="260"/>
-      <c r="H14" s="260"/>
-      <c r="I14" s="260"/>
-      <c r="J14" s="261" t="s">
+      <c r="K14" s="268"/>
+      <c r="L14" s="268"/>
+      <c r="M14" s="268"/>
+      <c r="N14" s="268"/>
+      <c r="O14" s="269"/>
+      <c r="P14" s="267" t="s">
         <v>88</v>
       </c>
-      <c r="K14" s="262"/>
-      <c r="L14" s="262"/>
-      <c r="M14" s="262"/>
-      <c r="N14" s="262"/>
-      <c r="O14" s="263"/>
-      <c r="P14" s="261" t="s">
-        <v>89</v>
-      </c>
-      <c r="Q14" s="262"/>
-      <c r="R14" s="262"/>
-      <c r="S14" s="262"/>
-      <c r="T14" s="262"/>
-      <c r="U14" s="262"/>
-      <c r="V14" s="262"/>
-      <c r="W14" s="262"/>
-      <c r="X14" s="263"/>
+      <c r="Q14" s="268"/>
+      <c r="R14" s="268"/>
+      <c r="S14" s="268"/>
+      <c r="T14" s="268"/>
+      <c r="U14" s="268"/>
+      <c r="V14" s="268"/>
+      <c r="W14" s="268"/>
+      <c r="X14" s="269"/>
     </row>
     <row r="15" spans="1:24" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3"/>
@@ -7849,162 +7803,162 @@
       <c r="X15" s="3"/>
     </row>
     <row r="16" spans="1:24" s="4" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="264" t="s">
+      <c r="A16" s="270" t="s">
+        <v>89</v>
+      </c>
+      <c r="B16" s="270"/>
+      <c r="C16" s="270"/>
+      <c r="D16" s="270"/>
+      <c r="E16" s="270"/>
+      <c r="F16" s="270"/>
+      <c r="G16" s="270"/>
+      <c r="H16" s="270"/>
+      <c r="I16" s="270"/>
+      <c r="J16" s="271" t="s">
         <v>90</v>
       </c>
-      <c r="B16" s="264"/>
-      <c r="C16" s="264"/>
-      <c r="D16" s="264"/>
-      <c r="E16" s="264"/>
-      <c r="F16" s="264"/>
-      <c r="G16" s="264"/>
-      <c r="H16" s="264"/>
-      <c r="I16" s="264"/>
-      <c r="J16" s="265" t="s">
+      <c r="K16" s="271"/>
+      <c r="L16" s="271"/>
+      <c r="M16" s="271"/>
+      <c r="N16" s="270" t="s">
         <v>91</v>
       </c>
-      <c r="K16" s="265"/>
-      <c r="L16" s="265"/>
-      <c r="M16" s="265"/>
-      <c r="N16" s="264" t="s">
+      <c r="O16" s="270"/>
+      <c r="P16" s="270"/>
+      <c r="Q16" s="270"/>
+      <c r="R16" s="270"/>
+      <c r="S16" s="270"/>
+      <c r="T16" s="272" t="s">
         <v>92</v>
       </c>
-      <c r="O16" s="264"/>
-      <c r="P16" s="264"/>
-      <c r="Q16" s="264"/>
-      <c r="R16" s="264"/>
-      <c r="S16" s="264"/>
-      <c r="T16" s="266" t="s">
+      <c r="U16" s="272"/>
+      <c r="V16" s="272"/>
+      <c r="W16" s="272"/>
+      <c r="X16" s="272"/>
+    </row>
+    <row r="17" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="260" t="s">
         <v>93</v>
       </c>
-      <c r="U16" s="266"/>
-      <c r="V16" s="266"/>
-      <c r="W16" s="266"/>
-      <c r="X16" s="266"/>
-    </row>
-    <row r="17" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="254" t="s">
+      <c r="B17" s="261"/>
+      <c r="C17" s="261"/>
+      <c r="D17" s="261"/>
+      <c r="E17" s="261"/>
+      <c r="F17" s="261"/>
+      <c r="G17" s="261"/>
+      <c r="H17" s="261"/>
+      <c r="I17" s="262"/>
+      <c r="J17" s="273" t="s">
         <v>94</v>
       </c>
-      <c r="B17" s="255"/>
-      <c r="C17" s="255"/>
-      <c r="D17" s="255"/>
-      <c r="E17" s="255"/>
-      <c r="F17" s="255"/>
-      <c r="G17" s="255"/>
-      <c r="H17" s="255"/>
-      <c r="I17" s="256"/>
-      <c r="J17" s="267" t="s">
+      <c r="K17" s="274"/>
+      <c r="L17" s="274"/>
+      <c r="M17" s="275"/>
+      <c r="N17" s="260" t="s">
         <v>95</v>
       </c>
-      <c r="K17" s="268"/>
-      <c r="L17" s="268"/>
-      <c r="M17" s="269"/>
-      <c r="N17" s="254" t="s">
+      <c r="O17" s="261"/>
+      <c r="P17" s="261"/>
+      <c r="Q17" s="261"/>
+      <c r="R17" s="261"/>
+      <c r="S17" s="262"/>
+      <c r="T17" s="260" t="s">
         <v>96</v>
       </c>
-      <c r="O17" s="255"/>
-      <c r="P17" s="255"/>
-      <c r="Q17" s="255"/>
-      <c r="R17" s="255"/>
-      <c r="S17" s="256"/>
-      <c r="T17" s="254" t="s">
-        <v>97</v>
-      </c>
-      <c r="U17" s="255"/>
-      <c r="V17" s="255"/>
-      <c r="W17" s="255"/>
-      <c r="X17" s="256"/>
+      <c r="U17" s="261"/>
+      <c r="V17" s="261"/>
+      <c r="W17" s="261"/>
+      <c r="X17" s="262"/>
     </row>
     <row r="18" spans="1:24" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="257"/>
-      <c r="B18" s="258"/>
-      <c r="C18" s="258"/>
-      <c r="D18" s="258"/>
-      <c r="E18" s="258"/>
-      <c r="F18" s="258"/>
-      <c r="G18" s="258"/>
-      <c r="H18" s="258"/>
-      <c r="I18" s="259"/>
-      <c r="J18" s="270"/>
-      <c r="K18" s="271"/>
-      <c r="L18" s="271"/>
-      <c r="M18" s="272"/>
-      <c r="N18" s="257"/>
-      <c r="O18" s="258"/>
-      <c r="P18" s="258"/>
-      <c r="Q18" s="258"/>
-      <c r="R18" s="258"/>
-      <c r="S18" s="259"/>
-      <c r="T18" s="257"/>
-      <c r="U18" s="258"/>
-      <c r="V18" s="258"/>
-      <c r="W18" s="258"/>
-      <c r="X18" s="259"/>
+      <c r="A18" s="263"/>
+      <c r="B18" s="264"/>
+      <c r="C18" s="264"/>
+      <c r="D18" s="264"/>
+      <c r="E18" s="264"/>
+      <c r="F18" s="264"/>
+      <c r="G18" s="264"/>
+      <c r="H18" s="264"/>
+      <c r="I18" s="265"/>
+      <c r="J18" s="276"/>
+      <c r="K18" s="277"/>
+      <c r="L18" s="277"/>
+      <c r="M18" s="278"/>
+      <c r="N18" s="263"/>
+      <c r="O18" s="264"/>
+      <c r="P18" s="264"/>
+      <c r="Q18" s="264"/>
+      <c r="R18" s="264"/>
+      <c r="S18" s="265"/>
+      <c r="T18" s="263"/>
+      <c r="U18" s="264"/>
+      <c r="V18" s="264"/>
+      <c r="W18" s="264"/>
+      <c r="X18" s="265"/>
     </row>
     <row r="19" spans="1:24" ht="39" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="20" spans="1:24" ht="39" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="21" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A21" s="252" t="s">
+      <c r="A21" s="258" t="s">
+        <v>97</v>
+      </c>
+      <c r="B21" s="258"/>
+      <c r="C21" s="258"/>
+      <c r="D21" s="258"/>
+      <c r="E21" s="258"/>
+      <c r="F21" s="258"/>
+      <c r="G21" s="258"/>
+      <c r="H21" s="258"/>
+      <c r="I21" s="5"/>
+      <c r="J21" s="258" t="s">
+        <v>65</v>
+      </c>
+      <c r="K21" s="258"/>
+      <c r="L21" s="258"/>
+      <c r="M21" s="258"/>
+      <c r="N21" s="258"/>
+      <c r="O21" s="258"/>
+      <c r="P21" s="258"/>
+      <c r="Q21" s="6"/>
+      <c r="R21" s="258" t="s">
         <v>98</v>
       </c>
-      <c r="B21" s="252"/>
-      <c r="C21" s="252"/>
-      <c r="D21" s="252"/>
-      <c r="E21" s="252"/>
-      <c r="F21" s="252"/>
-      <c r="G21" s="252"/>
-      <c r="H21" s="252"/>
-      <c r="I21" s="5"/>
-      <c r="J21" s="252" t="s">
-        <v>65</v>
-      </c>
-      <c r="K21" s="252"/>
-      <c r="L21" s="252"/>
-      <c r="M21" s="252"/>
-      <c r="N21" s="252"/>
-      <c r="O21" s="252"/>
-      <c r="P21" s="252"/>
-      <c r="Q21" s="6"/>
-      <c r="R21" s="252" t="s">
+      <c r="S21" s="258"/>
+      <c r="T21" s="258"/>
+      <c r="U21" s="258"/>
+      <c r="V21" s="258"/>
+      <c r="W21" s="258"/>
+      <c r="X21" s="258"/>
+    </row>
+    <row r="23" spans="1:24" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="P23" s="255" t="s">
         <v>99</v>
       </c>
-      <c r="S21" s="252"/>
-      <c r="T21" s="252"/>
-      <c r="U21" s="252"/>
-      <c r="V21" s="252"/>
-      <c r="W21" s="252"/>
-      <c r="X21" s="252"/>
-    </row>
-    <row r="23" spans="1:24" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="P23" s="249" t="s">
+      <c r="Q23" s="255"/>
+      <c r="R23" s="255"/>
+      <c r="S23" s="255"/>
+      <c r="T23" s="255"/>
+      <c r="U23" s="256" t="s">
         <v>100</v>
       </c>
-      <c r="Q23" s="249"/>
-      <c r="R23" s="249"/>
-      <c r="S23" s="249"/>
-      <c r="T23" s="249"/>
-      <c r="U23" s="250" t="s">
+      <c r="V23" s="256"/>
+      <c r="W23" s="256"/>
+      <c r="X23" s="256"/>
+    </row>
+    <row r="24" spans="1:24" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="P24" s="255" t="s">
         <v>101</v>
       </c>
-      <c r="V23" s="250"/>
-      <c r="W23" s="250"/>
-      <c r="X23" s="250"/>
-    </row>
-    <row r="24" spans="1:24" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="P24" s="249" t="s">
+      <c r="Q24" s="255"/>
+      <c r="R24" s="255"/>
+      <c r="S24" s="255"/>
+      <c r="T24" s="255"/>
+      <c r="U24" s="257" t="s">
         <v>102</v>
       </c>
-      <c r="Q24" s="249"/>
-      <c r="R24" s="249"/>
-      <c r="S24" s="249"/>
-      <c r="T24" s="249"/>
-      <c r="U24" s="251" t="s">
-        <v>103</v>
-      </c>
-      <c r="V24" s="251"/>
-      <c r="W24" s="251"/>
-      <c r="X24" s="251"/>
+      <c r="V24" s="257"/>
+      <c r="W24" s="257"/>
+      <c r="X24" s="257"/>
     </row>
   </sheetData>
   <mergeCells count="40">

</xml_diff>